<commit_message>
Oct 18 11am ET check: +2 parts (Phoenix AZ locker, Chico CA coin-op), +3 business liquidations; no removals
</commit_message>
<xml_diff>
--- a/lot_recon.xlsx
+++ b/lot_recon.xlsx
@@ -16,11 +16,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Removed" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Appliance Parts'!$A$1:$O$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Appliance Parts'!$A$1:$O$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wolf New'!$A$1:$O$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Wolf Used'!$A$1:$O$189</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Wolf Unclear'!$A$1:$O$43</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$69</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -551,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -581,7 +581,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 2026-10-18 08:06 ET</t>
+          <t>Last updated: 2026-10-18 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Active listings: 280 · Removed: 0</t>
+          <t>Active listings: 285 · Removed: 0</t>
         </is>
       </c>
     </row>
@@ -645,10 +645,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>83696</v>
+        <v>84696</v>
       </c>
       <c r="D8" t="n">
         <v>4</v>
@@ -712,13 +712,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13">
@@ -728,10 +728,10 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>900075.08</v>
+        <v>901075.08</v>
       </c>
     </row>
     <row r="15">
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C17" t="n">
         <v>1</v>
@@ -810,7 +810,7 @@
         <v>1</v>
       </c>
       <c r="G17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H17" s="6" t="n">
         <v>4023.69</v>
@@ -960,7 +960,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C22" t="n">
         <v>0</v>
@@ -975,7 +975,7 @@
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H22" s="6" t="n">
         <v>0</v>
@@ -1290,10 +1290,10 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" t="n">
         <v>0</v>
@@ -1308,49 +1308,82 @@
         <v>0</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>40000</v>
+        <v>41000</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2575</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="15" customHeight="1">
+          <t>2575–2629</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Unknown location</t>
+          <t>West / Other</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>75</v>
+        <v>2</v>
       </c>
       <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
         <v>0</v>
       </c>
-      <c r="D33" t="n">
-        <v>14</v>
-      </c>
       <c r="E33" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="F33" t="n">
         <v>0</v>
       </c>
       <c r="G33" t="n">
+        <v>1</v>
+      </c>
+      <c r="H33" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="6" t="n">
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2307</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="15" customHeight="1">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Unknown location</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>75</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" t="n">
+        <v>14</v>
+      </c>
+      <c r="E34" t="n">
+        <v>61</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="6" t="n">
         <v>285195.89</v>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="9" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr">
         <is>
           <t>Price $ (est.) = asking price or current high bid (+ stated shipping); items with no $ figure count as 0.</t>
         </is>
@@ -1367,7 +1400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O38"/>
+  <dimension ref="A1:O42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2917,7 +2950,7 @@
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>▸ California  (1)</t>
+          <t>▸ California  (2)</t>
         </is>
       </c>
       <c r="B36" s="12" t="n"/>
@@ -2996,35 +3029,211 @@
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="17" t="inlineStr">
+    <row r="38" outlineLevel="1">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>California</t>
+        </is>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>Coin-op Whirlpool washer &amp; dryer parts (late 80s–mid 90s) – OEM parts, 40+ coin boxes, consoles, 12 transmissions</t>
+        </is>
+      </c>
+      <c r="C38" s="13" t="inlineStr">
+        <is>
+          <t>bulk lot</t>
+        </is>
+      </c>
+      <c r="D38" s="13" t="inlineStr">
+        <is>
+          <t>Chico</t>
+        </is>
+      </c>
+      <c r="E38" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="F38" s="13" t="n">
+        <v>2629</v>
+      </c>
+      <c r="G38" s="13" t="inlineStr">
+        <is>
+          <t>$1,000</t>
+        </is>
+      </c>
+      <c r="H38" s="15" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I38" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="J38" s="13" t="inlineStr"/>
+      <c r="K38" s="13" t="inlineStr">
+        <is>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L38" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M38" s="13" t="inlineStr"/>
+      <c r="N38" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O38" s="14" t="inlineStr">
+        <is>
+          <t>Retired laundry-route owner (35 yrs). Calls only, no shipping, pickup in Chico. No motors or pumps. Niche older coin-op parts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="17" t="inlineStr">
         <is>
           <t>Subtotal — California</t>
         </is>
       </c>
-      <c r="B38" s="17" t="inlineStr">
+      <c r="B39" s="17" t="inlineStr">
+        <is>
+          <t>2 item(s)</t>
+        </is>
+      </c>
+      <c r="C39" s="18" t="n"/>
+      <c r="D39" s="18" t="n"/>
+      <c r="E39" s="18" t="n"/>
+      <c r="F39" s="18" t="n"/>
+      <c r="G39" s="18" t="n"/>
+      <c r="H39" s="19" t="n">
+        <v>41000</v>
+      </c>
+      <c r="I39" s="18" t="n"/>
+      <c r="J39" s="18" t="n"/>
+      <c r="K39" s="18" t="n"/>
+      <c r="L39" s="18" t="n"/>
+      <c r="M39" s="18" t="n"/>
+      <c r="N39" s="18" t="n"/>
+      <c r="O39" s="18" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>▸ West / Other  (1)</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="n"/>
+      <c r="C40" s="12" t="n"/>
+      <c r="D40" s="12" t="n"/>
+      <c r="E40" s="12" t="n"/>
+      <c r="F40" s="12" t="n"/>
+      <c r="G40" s="12" t="n"/>
+      <c r="H40" s="12" t="n"/>
+      <c r="I40" s="12" t="n"/>
+      <c r="J40" s="12" t="n"/>
+      <c r="K40" s="12" t="n"/>
+      <c r="L40" s="12" t="n"/>
+      <c r="M40" s="12" t="n"/>
+      <c r="N40" s="12" t="n"/>
+      <c r="O40" s="12" t="n"/>
+    </row>
+    <row r="41" outlineLevel="1">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>West / Other</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>Storage locker filled with appliance parts – washer/dryer parts, heating elements, cords, rollers, belts, tools</t>
+        </is>
+      </c>
+      <c r="C41" s="13" t="inlineStr">
+        <is>
+          <t>bulk lot</t>
+        </is>
+      </c>
+      <c r="D41" s="13" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="E41" s="13" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="F41" s="13" t="n">
+        <v>2307</v>
+      </c>
+      <c r="G41" s="13" t="inlineStr">
+        <is>
+          <t>Message for pricing</t>
+        </is>
+      </c>
+      <c r="H41" s="15" t="n"/>
+      <c r="I41" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="J41" s="13" t="inlineStr"/>
+      <c r="K41" s="13" t="inlineStr">
+        <is>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L41" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M41" s="13" t="inlineStr"/>
+      <c r="N41" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O41" s="14" t="inlineStr">
+        <is>
+          <t>Seller is getting out of the appliance business; selling the whole locker (North Phoenix, Deer Valley Rd near 19th Ave). Delivery available per post. Separate from the Phoenix parts-store closing ad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — West / Other</t>
+        </is>
+      </c>
+      <c r="B42" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C38" s="18" t="n"/>
-      <c r="D38" s="18" t="n"/>
-      <c r="E38" s="18" t="n"/>
-      <c r="F38" s="18" t="n"/>
-      <c r="G38" s="18" t="n"/>
-      <c r="H38" s="19" t="n">
-        <v>40000</v>
-      </c>
-      <c r="I38" s="18" t="n"/>
-      <c r="J38" s="18" t="n"/>
-      <c r="K38" s="18" t="n"/>
-      <c r="L38" s="18" t="n"/>
-      <c r="M38" s="18" t="n"/>
-      <c r="N38" s="18" t="n"/>
-      <c r="O38" s="18" t="n"/>
+      <c r="C42" s="18" t="n"/>
+      <c r="D42" s="18" t="n"/>
+      <c r="E42" s="18" t="n"/>
+      <c r="F42" s="18" t="n"/>
+      <c r="G42" s="18" t="n"/>
+      <c r="H42" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="18" t="n"/>
+      <c r="J42" s="18" t="n"/>
+      <c r="K42" s="18" t="n"/>
+      <c r="L42" s="18" t="n"/>
+      <c r="M42" s="18" t="n"/>
+      <c r="N42" s="18" t="n"/>
+      <c r="O42" s="18" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O38"/>
+  <autoFilter ref="A1:O42"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId2"/>
@@ -3043,6 +3252,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N38" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -18521,7 +18732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O64"/>
+  <dimension ref="A1:O69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -18621,7 +18832,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>▸ Greater Boston / South Shore (&lt;50mi)  (4)</t>
+          <t>▸ Greater Boston / South Shore (&lt;50mi)  (5)</t>
         </is>
       </c>
       <c r="B2" s="12" t="n"/>
@@ -18836,17 +19047,17 @@
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>Cannabis facility contents incl. commercial kitchen / stainless</t>
+          <t>Retirement bulk tool lot – 10 tools, sold together</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>facility contents</t>
+          <t>retirement</t>
         </is>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Milford</t>
+          <t>Waltham</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
@@ -18855,23 +19066,23 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="G6" s="13" t="inlineStr">
         <is>
-          <t>Auction, 18% BP</t>
+          <t>$250 all</t>
         </is>
       </c>
       <c r="H6" s="15" t="n"/>
-      <c r="I6" s="13" t="inlineStr"/>
-      <c r="J6" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-03 10:00 AM ET</t>
-        </is>
-      </c>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="J6" s="13" t="inlineStr"/>
       <c r="K6" s="13" t="inlineStr">
         <is>
-          <t>Paul E. Saperstein (PESCO)</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L6" s="13" t="inlineStr">
@@ -18887,120 +19098,120 @@
       </c>
       <c r="O6" s="14" t="inlineStr">
         <is>
+          <t>Small off-category FYI; seller says resell individually.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" outlineLevel="1">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Greater Boston / South Shore (&lt;50mi)</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>Cannabis facility contents incl. commercial kitchen / stainless</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>facility contents</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Milford</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>36</v>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>Auction, 18% BP</t>
+        </is>
+      </c>
+      <c r="H7" s="15" t="n"/>
+      <c r="I7" s="13" t="inlineStr"/>
+      <c r="J7" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-03 10:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K7" s="13" t="inlineStr">
+        <is>
+          <t>Paul E. Saperstein (PESCO)</t>
+        </is>
+      </c>
+      <c r="L7" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M7" s="13" t="inlineStr"/>
+      <c r="N7" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O7" s="14" t="inlineStr">
+        <is>
           <t>Calendar page only (no event page yet). ~45 mi.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Greater Boston / South Shore (&lt;50mi)</t>
         </is>
       </c>
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>4 item(s)</t>
-        </is>
-      </c>
-      <c r="C7" s="18" t="n"/>
-      <c r="D7" s="18" t="n"/>
-      <c r="E7" s="18" t="n"/>
-      <c r="F7" s="18" t="n"/>
-      <c r="G7" s="18" t="n"/>
-      <c r="H7" s="19" t="n">
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>5 item(s)</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="n"/>
+      <c r="D8" s="18" t="n"/>
+      <c r="E8" s="18" t="n"/>
+      <c r="F8" s="18" t="n"/>
+      <c r="G8" s="18" t="n"/>
+      <c r="H8" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I7" s="18" t="n"/>
-      <c r="J7" s="18" t="n"/>
-      <c r="K7" s="18" t="n"/>
-      <c r="L7" s="18" t="n"/>
-      <c r="M7" s="18" t="n"/>
-      <c r="N7" s="18" t="n"/>
-      <c r="O7" s="18" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="I8" s="18" t="n"/>
+      <c r="J8" s="18" t="n"/>
+      <c r="K8" s="18" t="n"/>
+      <c r="L8" s="18" t="n"/>
+      <c r="M8" s="18" t="n"/>
+      <c r="N8" s="18" t="n"/>
+      <c r="O8" s="18" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>▸ North Shore / Merrimack Valley / S. NH  (2)</t>
         </is>
       </c>
-      <c r="B8" s="12" t="n"/>
-      <c r="C8" s="12" t="n"/>
-      <c r="D8" s="12" t="n"/>
-      <c r="E8" s="12" t="n"/>
-      <c r="F8" s="12" t="n"/>
-      <c r="G8" s="12" t="n"/>
-      <c r="H8" s="12" t="n"/>
-      <c r="I8" s="12" t="n"/>
-      <c r="J8" s="12" t="n"/>
-      <c r="K8" s="12" t="n"/>
-      <c r="L8" s="12" t="n"/>
-      <c r="M8" s="12" t="n"/>
-      <c r="N8" s="12" t="n"/>
-      <c r="O8" s="12" t="n"/>
-    </row>
-    <row r="9" outlineLevel="1">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>North Shore / Merrimack Valley / S. NH</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>Commercial mechanical/plumbing/HVAC contractor inventory – multiple pallets of boxed stock, water heater, venting, diffusers</t>
-        </is>
-      </c>
-      <c r="C9" s="13" t="inlineStr">
-        <is>
-          <t>inventory</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>Merrimack</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="inlineStr">
-        <is>
-          <t>NH</t>
-        </is>
-      </c>
-      <c r="F9" s="13" t="n">
-        <v>62</v>
-      </c>
-      <c r="G9" s="13" t="inlineStr">
-        <is>
-          <t>$1 placeholder – make offer on everything</t>
-        </is>
-      </c>
-      <c r="H9" s="15" t="n"/>
-      <c r="I9" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="J9" s="13" t="inlineStr"/>
-      <c r="K9" s="13" t="inlineStr">
-        <is>
-          <t>Craigslist</t>
-        </is>
-      </c>
-      <c r="L9" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M9" s="13" t="inlineStr"/>
-      <c r="N9" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O9" s="14" t="inlineStr">
-        <is>
-          <t>Bulk buyers preferred.</t>
-        </is>
-      </c>
+      <c r="B9" s="12" t="n"/>
+      <c r="C9" s="12" t="n"/>
+      <c r="D9" s="12" t="n"/>
+      <c r="E9" s="12" t="n"/>
+      <c r="F9" s="12" t="n"/>
+      <c r="G9" s="12" t="n"/>
+      <c r="H9" s="12" t="n"/>
+      <c r="I9" s="12" t="n"/>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="12" t="n"/>
+      <c r="L9" s="12" t="n"/>
+      <c r="M9" s="12" t="n"/>
+      <c r="N9" s="12" t="n"/>
+      <c r="O9" s="12" t="n"/>
     </row>
     <row r="10" outlineLevel="1">
       <c r="A10" s="13" t="inlineStr">
@@ -19010,17 +19221,17 @@
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating overstock/returns online auction – 183 lots (fixtures, furnaces, heaters, A/C)</t>
+          <t>Commercial mechanical/plumbing/HVAC contractor inventory – multiple pallets of boxed stock, water heater, venting, diffusers</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>inventory</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>Concord</t>
+          <t>Merrimack</t>
         </is>
       </c>
       <c r="E10" s="13" t="inlineStr">
@@ -19029,27 +19240,23 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>84</v>
+        <v>62</v>
       </c>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>$1 placeholder – make offer on everything</t>
         </is>
       </c>
       <c r="H10" s="15" t="n"/>
       <c r="I10" s="13" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="J10" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-27 07:00 PM ET</t>
-        </is>
-      </c>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="J10" s="13" t="inlineStr"/>
       <c r="K10" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Atlantic Auction Co.)</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L10" s="13" t="inlineStr">
@@ -19065,120 +19272,124 @@
       </c>
       <c r="O10" s="14" t="inlineStr">
         <is>
+          <t>Bulk buyers preferred.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" outlineLevel="1">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>North Shore / Merrimack Valley / S. NH</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>Plumbing &amp; heating overstock/returns online auction – 183 lots (fixtures, furnaces, heaters, A/C)</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>auction</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Concord</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="n">
+        <v>84</v>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>Online auction</t>
+        </is>
+      </c>
+      <c r="H11" s="15" t="n"/>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-27 07:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K11" s="13" t="inlineStr">
+        <is>
+          <t>HiBid (Atlantic Auction Co.)</t>
+        </is>
+      </c>
+      <c r="L11" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M11" s="13" t="inlineStr"/>
+      <c r="N11" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O11" s="14" t="inlineStr">
+        <is>
           <t>Overstock sale, not a closing. Pickup Oct 29–30.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="17" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Subtotal — North Shore / Merrimack Valley / S. NH</t>
         </is>
       </c>
-      <c r="B11" s="17" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>2 item(s)</t>
         </is>
       </c>
-      <c r="C11" s="18" t="n"/>
-      <c r="D11" s="18" t="n"/>
-      <c r="E11" s="18" t="n"/>
-      <c r="F11" s="18" t="n"/>
-      <c r="G11" s="18" t="n"/>
-      <c r="H11" s="19" t="n">
+      <c r="C12" s="18" t="n"/>
+      <c r="D12" s="18" t="n"/>
+      <c r="E12" s="18" t="n"/>
+      <c r="F12" s="18" t="n"/>
+      <c r="G12" s="18" t="n"/>
+      <c r="H12" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I11" s="18" t="n"/>
-      <c r="J11" s="18" t="n"/>
-      <c r="K11" s="18" t="n"/>
-      <c r="L11" s="18" t="n"/>
-      <c r="M11" s="18" t="n"/>
-      <c r="N11" s="18" t="n"/>
-      <c r="O11" s="18" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="I12" s="18" t="n"/>
+      <c r="J12" s="18" t="n"/>
+      <c r="K12" s="18" t="n"/>
+      <c r="L12" s="18" t="n"/>
+      <c r="M12" s="18" t="n"/>
+      <c r="N12" s="18" t="n"/>
+      <c r="O12" s="18" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>▸ Central / Western MA  (3)</t>
         </is>
       </c>
-      <c r="B12" s="12" t="n"/>
-      <c r="C12" s="12" t="n"/>
-      <c r="D12" s="12" t="n"/>
-      <c r="E12" s="12" t="n"/>
-      <c r="F12" s="12" t="n"/>
-      <c r="G12" s="12" t="n"/>
-      <c r="H12" s="12" t="n"/>
-      <c r="I12" s="12" t="n"/>
-      <c r="J12" s="12" t="n"/>
-      <c r="K12" s="12" t="n"/>
-      <c r="L12" s="12" t="n"/>
-      <c r="M12" s="12" t="n"/>
-      <c r="N12" s="12" t="n"/>
-      <c r="O12" s="12" t="n"/>
-    </row>
-    <row r="13" outlineLevel="1">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>Central / Western MA</t>
-        </is>
-      </c>
-      <c r="B13" s="14" t="inlineStr">
-        <is>
-          <t>Gift/souvenir store closing (retirement) – all new stock</t>
-        </is>
-      </c>
-      <c r="C13" s="13" t="inlineStr">
-        <is>
-          <t>store closing</t>
-        </is>
-      </c>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>Thorndike</t>
-        </is>
-      </c>
-      <c r="E13" s="13" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="F13" s="13" t="n">
-        <v>77</v>
-      </c>
-      <c r="G13" s="13" t="inlineStr">
-        <is>
-          <t>By appointment</t>
-        </is>
-      </c>
-      <c r="H13" s="15" t="n"/>
-      <c r="I13" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="J13" s="13" t="inlineStr"/>
-      <c r="K13" s="13" t="inlineStr">
-        <is>
-          <t>Craigslist</t>
-        </is>
-      </c>
-      <c r="L13" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M13" s="13" t="inlineStr"/>
-      <c r="N13" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O13" s="14" t="inlineStr">
-        <is>
-          <t>Updated Oct 8. Off-category FYI.</t>
-        </is>
-      </c>
+      <c r="B13" s="12" t="n"/>
+      <c r="C13" s="12" t="n"/>
+      <c r="D13" s="12" t="n"/>
+      <c r="E13" s="12" t="n"/>
+      <c r="F13" s="12" t="n"/>
+      <c r="G13" s="12" t="n"/>
+      <c r="H13" s="12" t="n"/>
+      <c r="I13" s="12" t="n"/>
+      <c r="J13" s="12" t="n"/>
+      <c r="K13" s="12" t="n"/>
+      <c r="L13" s="12" t="n"/>
+      <c r="M13" s="12" t="n"/>
+      <c r="N13" s="12" t="n"/>
+      <c r="O13" s="12" t="n"/>
     </row>
     <row r="14" outlineLevel="1">
       <c r="A14" s="13" t="inlineStr">
@@ -19188,17 +19399,17 @@
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>UNECO Manufacturing – owners retiring, machine-shop metrology &amp; tooling</t>
+          <t>Gift/souvenir store closing (retirement) – all new stock</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>retirement</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>Chicopee</t>
+          <t>Thorndike</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
@@ -19207,23 +19418,23 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>Online auction, 18% BP</t>
+          <t>By appointment</t>
         </is>
       </c>
       <c r="H14" s="15" t="n"/>
-      <c r="I14" s="13" t="inlineStr"/>
-      <c r="J14" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-04 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="I14" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="J14" s="13" t="inlineStr"/>
       <c r="K14" s="13" t="inlineStr">
         <is>
-          <t>HiBid (DeCosmo Industrial)</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L14" s="13" t="inlineStr">
@@ -19239,7 +19450,7 @@
       </c>
       <c r="O14" s="14" t="inlineStr">
         <is>
-          <t>Niche tooling only. Bidding opens Oct 19.</t>
+          <t>Updated Oct 8. Off-category FYI.</t>
         </is>
       </c>
     </row>
@@ -19251,17 +19462,17 @@
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>Restaurant closing, everything must go – kitchen equipment, stainless, smallwares</t>
+          <t>UNECO Manufacturing – owners retiring, machine-shop metrology &amp; tooling</t>
         </is>
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>restaurant closing</t>
+          <t>retirement</t>
         </is>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
-          <t>Westfield</t>
+          <t>Chicopee</t>
         </is>
       </c>
       <c r="E15" s="13" t="inlineStr">
@@ -19270,23 +19481,23 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t>Make offer</t>
+          <t>Online auction, 18% BP</t>
         </is>
       </c>
       <c r="H15" s="15" t="n"/>
-      <c r="I15" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="J15" s="13" t="inlineStr"/>
+      <c r="I15" s="13" t="inlineStr"/>
+      <c r="J15" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-04 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K15" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>HiBid (DeCosmo Industrial)</t>
         </is>
       </c>
       <c r="L15" s="13" t="inlineStr">
@@ -19302,120 +19513,120 @@
       </c>
       <c r="O15" s="14" t="inlineStr">
         <is>
+          <t>Niche tooling only. Bidding opens Oct 19.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" outlineLevel="1">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Central / Western MA</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>Restaurant closing, everything must go – kitchen equipment, stainless, smallwares</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>restaurant closing</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>Westfield</t>
+        </is>
+      </c>
+      <c r="E16" s="13" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="n">
+        <v>99</v>
+      </c>
+      <c r="G16" s="13" t="inlineStr">
+        <is>
+          <t>Make offer</t>
+        </is>
+      </c>
+      <c r="H16" s="15" t="n"/>
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="J16" s="13" t="inlineStr"/>
+      <c r="K16" s="13" t="inlineStr">
+        <is>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L16" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M16" s="13" t="inlineStr"/>
+      <c r="N16" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O16" s="14" t="inlineStr">
+        <is>
           <t>Related separate post "Complete Restaurant Equipment Package" $3,500 OBO (maybe same restaurant): https://www.craigslist.org/view/d/westfield-complete-restaurant-equipment/9Y5KCdhhgSqEBYbD3wKqVd</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="17" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Central / Western MA</t>
         </is>
       </c>
-      <c r="B16" s="17" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>3 item(s)</t>
         </is>
       </c>
-      <c r="C16" s="18" t="n"/>
-      <c r="D16" s="18" t="n"/>
-      <c r="E16" s="18" t="n"/>
-      <c r="F16" s="18" t="n"/>
-      <c r="G16" s="18" t="n"/>
-      <c r="H16" s="19" t="n">
+      <c r="C17" s="18" t="n"/>
+      <c r="D17" s="18" t="n"/>
+      <c r="E17" s="18" t="n"/>
+      <c r="F17" s="18" t="n"/>
+      <c r="G17" s="18" t="n"/>
+      <c r="H17" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I16" s="18" t="n"/>
-      <c r="J16" s="18" t="n"/>
-      <c r="K16" s="18" t="n"/>
-      <c r="L16" s="18" t="n"/>
-      <c r="M16" s="18" t="n"/>
-      <c r="N16" s="18" t="n"/>
-      <c r="O16" s="18" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="11" t="inlineStr">
-        <is>
-          <t>▸ Maine / VT / Northern NH  (4)</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="n"/>
-      <c r="C17" s="12" t="n"/>
-      <c r="D17" s="12" t="n"/>
-      <c r="E17" s="12" t="n"/>
-      <c r="F17" s="12" t="n"/>
-      <c r="G17" s="12" t="n"/>
-      <c r="H17" s="12" t="n"/>
-      <c r="I17" s="12" t="n"/>
-      <c r="J17" s="12" t="n"/>
-      <c r="K17" s="12" t="n"/>
-      <c r="L17" s="12" t="n"/>
-      <c r="M17" s="12" t="n"/>
-      <c r="N17" s="12" t="n"/>
-      <c r="O17" s="12" t="n"/>
-    </row>
-    <row r="18" outlineLevel="1">
-      <c r="A18" s="13" t="inlineStr">
-        <is>
-          <t>Maine / VT / Northern NH</t>
-        </is>
-      </c>
-      <c r="B18" s="14" t="inlineStr">
-        <is>
-          <t>Oola Bowls secured-party sale – restaurant equipment bought new 2024-25 (Electro Freeze, Scotsman, Atosa)</t>
-        </is>
-      </c>
-      <c r="C18" s="13" t="inlineStr">
-        <is>
-          <t>restaurant</t>
-        </is>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
-        <is>
-          <t>Scarborough</t>
-        </is>
-      </c>
-      <c r="E18" s="13" t="inlineStr">
-        <is>
-          <t>ME</t>
-        </is>
-      </c>
-      <c r="F18" s="13" t="n">
-        <v>104</v>
-      </c>
-      <c r="G18" s="13" t="inlineStr">
-        <is>
-          <t>Online auction (freezers $80–150 when seen)</t>
-        </is>
-      </c>
-      <c r="H18" s="15" t="n"/>
-      <c r="I18" s="13" t="inlineStr"/>
-      <c r="J18" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-19 01:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K18" s="13" t="inlineStr">
-        <is>
-          <t>Keenan Auction / Proxibid</t>
-        </is>
-      </c>
-      <c r="L18" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
-        </is>
-      </c>
-      <c r="M18" s="13" t="inlineStr"/>
-      <c r="N18" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O18" s="14" t="inlineStr">
-        <is>
-          <t>Pickup Oct 21 only.</t>
-        </is>
-      </c>
+      <c r="I17" s="18" t="n"/>
+      <c r="J17" s="18" t="n"/>
+      <c r="K17" s="18" t="n"/>
+      <c r="L17" s="18" t="n"/>
+      <c r="M17" s="18" t="n"/>
+      <c r="N17" s="18" t="n"/>
+      <c r="O17" s="18" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>▸ Maine / VT / Northern NH  (5)</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="n"/>
+      <c r="C18" s="12" t="n"/>
+      <c r="D18" s="12" t="n"/>
+      <c r="E18" s="12" t="n"/>
+      <c r="F18" s="12" t="n"/>
+      <c r="G18" s="12" t="n"/>
+      <c r="H18" s="12" t="n"/>
+      <c r="I18" s="12" t="n"/>
+      <c r="J18" s="12" t="n"/>
+      <c r="K18" s="12" t="n"/>
+      <c r="L18" s="12" t="n"/>
+      <c r="M18" s="12" t="n"/>
+      <c r="N18" s="12" t="n"/>
+      <c r="O18" s="12" t="n"/>
     </row>
     <row r="19" outlineLevel="1">
       <c r="A19" s="13" t="inlineStr">
@@ -19425,17 +19636,17 @@
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>Event-rental business closing – 300+ chairs, 40+ rounds, 1,300+ china, linens (all at once)</t>
+          <t>Oola Bowls secured-party sale – restaurant equipment bought new 2024-25 (Electro Freeze, Scotsman, Atosa)</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>business closing</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>Woolwich</t>
+          <t>Scarborough</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr">
@@ -19444,28 +19655,28 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>135</v>
+        <v>104</v>
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>No price listed</t>
+          <t>Online auction (freezers $80–150 when seen)</t>
         </is>
       </c>
       <c r="H19" s="15" t="n"/>
-      <c r="I19" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="J19" s="13" t="inlineStr"/>
+      <c r="I19" s="13" t="inlineStr"/>
+      <c r="J19" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 01:00 PM ET</t>
+        </is>
+      </c>
       <c r="K19" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
-        </is>
-      </c>
-      <c r="L19" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>Keenan Auction / Proxibid</t>
+        </is>
+      </c>
+      <c r="L19" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M19" s="13" t="inlineStr"/>
@@ -19476,7 +19687,7 @@
       </c>
       <c r="O19" s="14" t="inlineStr">
         <is>
-          <t>Updated Oct 7. Replacement cost &gt;$72K per post.</t>
+          <t>Pickup Oct 21 only.</t>
         </is>
       </c>
     </row>
@@ -19488,42 +19699,42 @@
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>Pellet/wood stoves, heating stock, tools &amp; heavy equipment – "business liquidation", 380 lots</t>
+          <t>Contractor appliance lot – 3 refrigerators, Bosch wall oven, gas range, washer/dryer set</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>contractor lot</t>
         </is>
       </c>
       <c r="D20" s="13" t="inlineStr">
         <is>
-          <t>Lunenburg</t>
+          <t>Scarborough</t>
         </is>
       </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
-          <t>VT</t>
+          <t>ME</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>168</v>
+        <v>104</v>
       </c>
       <c r="G20" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>$200 OBO each, less as a bundle</t>
         </is>
       </c>
       <c r="H20" s="15" t="n"/>
-      <c r="I20" s="13" t="inlineStr"/>
-      <c r="J20" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-04 10:00 AM ET</t>
-        </is>
-      </c>
+      <c r="I20" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="J20" s="13" t="inlineStr"/>
       <c r="K20" s="13" t="inlineStr">
         <is>
-          <t>Thomas Hirchak Co.</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L20" s="13" t="inlineStr">
@@ -19539,7 +19750,7 @@
       </c>
       <c r="O20" s="14" t="inlineStr">
         <is>
-          <t>Closes Wed Nov 4 10 AM, preview Oct 28, removal Nov 9, no shipping.</t>
+          <t>Working units pulled from jobs. Complete appliances, not parts.</t>
         </is>
       </c>
     </row>
@@ -19551,42 +19762,42 @@
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>Bread Loaf Corp wind-down – contractor equipment, staging, telehandler</t>
+          <t>Event-rental business closing – 300+ chairs, 40+ rounds, 1,300+ china, linens (all at once)</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>contractor liquidation</t>
+          <t>business closing</t>
         </is>
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
-          <t>Middlebury</t>
+          <t>Woolwich</t>
         </is>
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>VT</t>
+          <t>ME</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>177</v>
+        <v>135</v>
       </c>
       <c r="G21" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>No price listed</t>
         </is>
       </c>
       <c r="H21" s="15" t="n"/>
-      <c r="I21" s="13" t="inlineStr"/>
-      <c r="J21" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-28 09:00 AM ET</t>
-        </is>
-      </c>
+      <c r="I21" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="J21" s="13" t="inlineStr"/>
       <c r="K21" s="13" t="inlineStr">
         <is>
-          <t>THC Auction</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L21" s="13" t="inlineStr">
@@ -19602,183 +19813,183 @@
       </c>
       <c r="O21" s="14" t="inlineStr">
         <is>
+          <t>Updated Oct 7. Replacement cost &gt;$72K per post.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" outlineLevel="1">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>Maine / VT / Northern NH</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>Pellet/wood stoves, heating stock, tools &amp; heavy equipment – "business liquidation", 380 lots</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>auction</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>Lunenburg</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="inlineStr">
+        <is>
+          <t>VT</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="n">
+        <v>168</v>
+      </c>
+      <c r="G22" s="13" t="inlineStr">
+        <is>
+          <t>Online auction</t>
+        </is>
+      </c>
+      <c r="H22" s="15" t="n"/>
+      <c r="I22" s="13" t="inlineStr"/>
+      <c r="J22" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-04 10:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K22" s="13" t="inlineStr">
+        <is>
+          <t>Thomas Hirchak Co.</t>
+        </is>
+      </c>
+      <c r="L22" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M22" s="13" t="inlineStr"/>
+      <c r="N22" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O22" s="14" t="inlineStr">
+        <is>
+          <t>Closes Wed Nov 4 10 AM, preview Oct 28, removal Nov 9, no shipping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" outlineLevel="1">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>Maine / VT / Northern NH</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Bread Loaf Corp wind-down – contractor equipment, staging, telehandler</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>contractor liquidation</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>Middlebury</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>VT</t>
+        </is>
+      </c>
+      <c r="F23" s="13" t="n">
+        <v>177</v>
+      </c>
+      <c r="G23" s="13" t="inlineStr">
+        <is>
+          <t>Online auction</t>
+        </is>
+      </c>
+      <c r="H23" s="15" t="n"/>
+      <c r="I23" s="13" t="inlineStr"/>
+      <c r="J23" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-28 09:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K23" s="13" t="inlineStr">
+        <is>
+          <t>THC Auction</t>
+        </is>
+      </c>
+      <c r="L23" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M23" s="13" t="inlineStr"/>
+      <c r="N23" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O23" s="14" t="inlineStr">
+        <is>
           <t>Company wind-down.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="17" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Maine / VT / Northern NH</t>
         </is>
       </c>
-      <c r="B22" s="17" t="inlineStr">
-        <is>
-          <t>4 item(s)</t>
-        </is>
-      </c>
-      <c r="C22" s="18" t="n"/>
-      <c r="D22" s="18" t="n"/>
-      <c r="E22" s="18" t="n"/>
-      <c r="F22" s="18" t="n"/>
-      <c r="G22" s="18" t="n"/>
-      <c r="H22" s="19" t="n">
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>5 item(s)</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="n"/>
+      <c r="D24" s="18" t="n"/>
+      <c r="E24" s="18" t="n"/>
+      <c r="F24" s="18" t="n"/>
+      <c r="G24" s="18" t="n"/>
+      <c r="H24" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I22" s="18" t="n"/>
-      <c r="J22" s="18" t="n"/>
-      <c r="K22" s="18" t="n"/>
-      <c r="L22" s="18" t="n"/>
-      <c r="M22" s="18" t="n"/>
-      <c r="N22" s="18" t="n"/>
-      <c r="O22" s="18" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="I24" s="18" t="n"/>
+      <c r="J24" s="18" t="n"/>
+      <c r="K24" s="18" t="n"/>
+      <c r="L24" s="18" t="n"/>
+      <c r="M24" s="18" t="n"/>
+      <c r="N24" s="18" t="n"/>
+      <c r="O24" s="18" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>▸ CT / Hudson Valley  (4)</t>
         </is>
       </c>
-      <c r="B23" s="12" t="n"/>
-      <c r="C23" s="12" t="n"/>
-      <c r="D23" s="12" t="n"/>
-      <c r="E23" s="12" t="n"/>
-      <c r="F23" s="12" t="n"/>
-      <c r="G23" s="12" t="n"/>
-      <c r="H23" s="12" t="n"/>
-      <c r="I23" s="12" t="n"/>
-      <c r="J23" s="12" t="n"/>
-      <c r="K23" s="12" t="n"/>
-      <c r="L23" s="12" t="n"/>
-      <c r="M23" s="12" t="n"/>
-      <c r="N23" s="12" t="n"/>
-      <c r="O23" s="12" t="n"/>
-    </row>
-    <row r="24" outlineLevel="1">
-      <c r="A24" s="13" t="inlineStr">
-        <is>
-          <t>CT / Hudson Valley</t>
-        </is>
-      </c>
-      <c r="B24" s="14" t="inlineStr">
-        <is>
-          <t>Bank-ordered electrical contractor sale – Greenlee/Hilti/Milwaukee tools, GE/Siemens breakers</t>
-        </is>
-      </c>
-      <c r="C24" s="13" t="inlineStr">
-        <is>
-          <t>contractor liquidation</t>
-        </is>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
-        <is>
-          <t>Clinton</t>
-        </is>
-      </c>
-      <c r="E24" s="13" t="inlineStr">
-        <is>
-          <t>CT</t>
-        </is>
-      </c>
-      <c r="F24" s="13" t="n">
-        <v>106</v>
-      </c>
-      <c r="G24" s="13" t="inlineStr">
-        <is>
-          <t>Online auction</t>
-        </is>
-      </c>
-      <c r="H24" s="15" t="n"/>
-      <c r="I24" s="13" t="inlineStr"/>
-      <c r="J24" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-29 05:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K24" s="13" t="inlineStr">
-        <is>
-          <t>Hamilton Group / EstateSales.net</t>
-        </is>
-      </c>
-      <c r="L24" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M24" s="13" t="inlineStr"/>
-      <c r="N24" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O24" s="14" t="inlineStr">
-        <is>
-          <t>Listed "Oct 29 2 PM PST" (= 5 PM ET).</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" outlineLevel="1">
-      <c r="A25" s="13" t="inlineStr">
-        <is>
-          <t>CT / Hudson Valley</t>
-        </is>
-      </c>
-      <c r="B25" s="14" t="inlineStr">
-        <is>
-          <t>Major Intl Chain Surplus – 225 lots commercial refrigeration/kitchen (True, Traulsen, Hobart, Blodgett, Taylor)</t>
-        </is>
-      </c>
-      <c r="C25" s="13" t="inlineStr">
-        <is>
-          <t>commercial surplus</t>
-        </is>
-      </c>
-      <c r="D25" s="13" t="inlineStr">
-        <is>
-          <t>Pleasant Valley</t>
-        </is>
-      </c>
-      <c r="E25" s="13" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="F25" s="13" t="n">
-        <v>157</v>
-      </c>
-      <c r="G25" s="13" t="inlineStr">
-        <is>
-          <t>Online auction</t>
-        </is>
-      </c>
-      <c r="H25" s="15" t="n"/>
-      <c r="I25" s="13" t="inlineStr"/>
-      <c r="J25" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-20 02:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K25" s="13" t="inlineStr">
-        <is>
-          <t>Adams / BidWrangler</t>
-        </is>
-      </c>
-      <c r="L25" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
-        </is>
-      </c>
-      <c r="M25" s="13" t="inlineStr"/>
-      <c r="N25" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O25" s="14" t="inlineStr">
-        <is>
-          <t>Tested and new units.</t>
-        </is>
-      </c>
+      <c r="B25" s="12" t="n"/>
+      <c r="C25" s="12" t="n"/>
+      <c r="D25" s="12" t="n"/>
+      <c r="E25" s="12" t="n"/>
+      <c r="F25" s="12" t="n"/>
+      <c r="G25" s="12" t="n"/>
+      <c r="H25" s="12" t="n"/>
+      <c r="I25" s="12" t="n"/>
+      <c r="J25" s="12" t="n"/>
+      <c r="K25" s="12" t="n"/>
+      <c r="L25" s="12" t="n"/>
+      <c r="M25" s="12" t="n"/>
+      <c r="N25" s="12" t="n"/>
+      <c r="O25" s="12" t="n"/>
     </row>
     <row r="26" outlineLevel="1">
       <c r="A26" s="13" t="inlineStr">
@@ -19788,17 +19999,17 @@
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>Café/bakery liquidation – Traulsen, Vulcan ovens, mixers, Hobart slicer (~74 lots)</t>
+          <t>Bank-ordered electrical contractor sale – Greenlee/Hilti/Milwaukee tools, GE/Siemens breakers</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>contractor liquidation</t>
         </is>
       </c>
       <c r="D26" s="13" t="inlineStr">
         <is>
-          <t>Greenwich</t>
+          <t>Clinton</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
@@ -19807,23 +20018,23 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>164</v>
+        <v>106</v>
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>Live auction + webcast</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H26" s="15" t="n"/>
       <c r="I26" s="13" t="inlineStr"/>
       <c r="J26" s="13" t="inlineStr">
         <is>
-          <t>2026-10-21 06:00 PM ET</t>
+          <t>2026-10-29 05:00 PM ET</t>
         </is>
       </c>
       <c r="K26" s="13" t="inlineStr">
         <is>
-          <t>Best Buy Auctioneers / AuctionGuide</t>
+          <t>Hamilton Group / EstateSales.net</t>
         </is>
       </c>
       <c r="L26" s="13" t="inlineStr">
@@ -19839,7 +20050,7 @@
       </c>
       <c r="O26" s="14" t="inlineStr">
         <is>
-          <t>Oct 21; start time not captured (placeholder 6 PM).</t>
+          <t>Listed "Oct 29 2 PM PST" (= 5 PM ET).</t>
         </is>
       </c>
     </row>
@@ -19851,17 +20062,17 @@
       </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>BJ's Wholesale closeout – racking, forklifts, Hobart</t>
+          <t>Major Intl Chain Surplus – 225 lots commercial refrigeration/kitchen (True, Traulsen, Hobart, Blodgett, Taylor)</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>commercial surplus</t>
         </is>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>Rotterdam</t>
+          <t>Pleasant Valley</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
@@ -19870,7 +20081,7 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="G27" s="13" t="inlineStr">
         <is>
@@ -19881,17 +20092,17 @@
       <c r="I27" s="13" t="inlineStr"/>
       <c r="J27" s="13" t="inlineStr">
         <is>
-          <t>2026-11-10 10:00 AM ET</t>
+          <t>2026-10-20 02:00 PM ET</t>
         </is>
       </c>
       <c r="K27" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
-        </is>
-      </c>
-      <c r="L27" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>Adams / BidWrangler</t>
+        </is>
+      </c>
+      <c r="L27" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M27" s="13" t="inlineStr"/>
@@ -19902,191 +20113,183 @@
       </c>
       <c r="O27" s="14" t="inlineStr">
         <is>
+          <t>Tested and new units.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" outlineLevel="1">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>CT / Hudson Valley</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>Café/bakery liquidation – Traulsen, Vulcan ovens, mixers, Hobart slicer (~74 lots)</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
+        <is>
+          <t>Greenwich</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="n">
+        <v>164</v>
+      </c>
+      <c r="G28" s="13" t="inlineStr">
+        <is>
+          <t>Live auction + webcast</t>
+        </is>
+      </c>
+      <c r="H28" s="15" t="n"/>
+      <c r="I28" s="13" t="inlineStr"/>
+      <c r="J28" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-21 06:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K28" s="13" t="inlineStr">
+        <is>
+          <t>Best Buy Auctioneers / AuctionGuide</t>
+        </is>
+      </c>
+      <c r="L28" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M28" s="13" t="inlineStr"/>
+      <c r="N28" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O28" s="14" t="inlineStr">
+        <is>
+          <t>Oct 21; start time not captured (placeholder 6 PM).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" outlineLevel="1">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>CT / Hudson Valley</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>BJ's Wholesale closeout – racking, forklifts, Hobart</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>store closing</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>Rotterdam</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="F29" s="13" t="n">
+        <v>168</v>
+      </c>
+      <c r="G29" s="13" t="inlineStr">
+        <is>
+          <t>Online auction</t>
+        </is>
+      </c>
+      <c r="H29" s="15" t="n"/>
+      <c r="I29" s="13" t="inlineStr"/>
+      <c r="J29" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-10 10:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K29" s="13" t="inlineStr">
+        <is>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L29" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M29" s="13" t="inlineStr"/>
+      <c r="N29" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O29" s="14" t="inlineStr">
+        <is>
           <t>Closes from Nov 10 10 AM.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="17" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
         <is>
           <t>Subtotal — CT / Hudson Valley</t>
         </is>
       </c>
-      <c r="B28" s="17" t="inlineStr">
+      <c r="B30" s="17" t="inlineStr">
         <is>
           <t>4 item(s)</t>
         </is>
       </c>
-      <c r="C28" s="18" t="n"/>
-      <c r="D28" s="18" t="n"/>
-      <c r="E28" s="18" t="n"/>
-      <c r="F28" s="18" t="n"/>
-      <c r="G28" s="18" t="n"/>
-      <c r="H28" s="19" t="n">
+      <c r="C30" s="18" t="n"/>
+      <c r="D30" s="18" t="n"/>
+      <c r="E30" s="18" t="n"/>
+      <c r="F30" s="18" t="n"/>
+      <c r="G30" s="18" t="n"/>
+      <c r="H30" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I28" s="18" t="n"/>
-      <c r="J28" s="18" t="n"/>
-      <c r="K28" s="18" t="n"/>
-      <c r="L28" s="18" t="n"/>
-      <c r="M28" s="18" t="n"/>
-      <c r="N28" s="18" t="n"/>
-      <c r="O28" s="18" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="11" t="inlineStr">
+      <c r="I30" s="18" t="n"/>
+      <c r="J30" s="18" t="n"/>
+      <c r="K30" s="18" t="n"/>
+      <c r="L30" s="18" t="n"/>
+      <c r="M30" s="18" t="n"/>
+      <c r="N30" s="18" t="n"/>
+      <c r="O30" s="18" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>▸ NYC / Long Island / NJ  (16)</t>
         </is>
       </c>
-      <c r="B29" s="12" t="n"/>
-      <c r="C29" s="12" t="n"/>
-      <c r="D29" s="12" t="n"/>
-      <c r="E29" s="12" t="n"/>
-      <c r="F29" s="12" t="n"/>
-      <c r="G29" s="12" t="n"/>
-      <c r="H29" s="12" t="n"/>
-      <c r="I29" s="12" t="n"/>
-      <c r="J29" s="12" t="n"/>
-      <c r="K29" s="12" t="n"/>
-      <c r="L29" s="12" t="n"/>
-      <c r="M29" s="12" t="n"/>
-      <c r="N29" s="12" t="n"/>
-      <c r="O29" s="12" t="n"/>
-    </row>
-    <row r="30" outlineLevel="1">
-      <c r="A30" s="13" t="inlineStr">
-        <is>
-          <t>NYC / Long Island / NJ</t>
-        </is>
-      </c>
-      <c r="B30" s="14" t="inlineStr">
-        <is>
-          <t>Japanese BBQ &amp; bar – ~47 lots: Turbo Air, Hoshizaki ice machine, Pitco, Beverage-Air</t>
-        </is>
-      </c>
-      <c r="C30" s="13" t="inlineStr">
-        <is>
-          <t>restaurant closing</t>
-        </is>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
-        <is>
-          <t>New York</t>
-        </is>
-      </c>
-      <c r="E30" s="13" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="F30" s="13" t="n">
-        <v>191</v>
-      </c>
-      <c r="G30" s="13" t="inlineStr">
-        <is>
-          <t>Live + webcast, 18% BP + 3%</t>
-        </is>
-      </c>
-      <c r="H30" s="15" t="n"/>
-      <c r="I30" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="J30" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-21 04:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K30" s="13" t="inlineStr">
-        <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
-        </is>
-      </c>
-      <c r="L30" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M30" s="13" t="inlineStr"/>
-      <c r="N30" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O30" s="14" t="inlineStr">
-        <is>
-          <t>Wed Oct 21 4 PM. NYC 10013.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" outlineLevel="1">
-      <c r="A31" s="13" t="inlineStr">
-        <is>
-          <t>NYC / Long Island / NJ</t>
-        </is>
-      </c>
-      <c r="B31" s="14" t="inlineStr">
-        <is>
-          <t>Corporate caterer – Alto-Shaam, new boxed Avantco rice cookers &amp; Cadco oven, Perlick, MerryChef</t>
-        </is>
-      </c>
-      <c r="C31" s="13" t="inlineStr">
-        <is>
-          <t>auction</t>
-        </is>
-      </c>
-      <c r="D31" s="13" t="inlineStr">
-        <is>
-          <t>Jersey City</t>
-        </is>
-      </c>
-      <c r="E31" s="13" t="inlineStr">
-        <is>
-          <t>NJ</t>
-        </is>
-      </c>
-      <c r="F31" s="13" t="n">
-        <v>193</v>
-      </c>
-      <c r="G31" s="13" t="inlineStr">
-        <is>
-          <t>Live + webcast, 18% BP + 3%</t>
-        </is>
-      </c>
-      <c r="H31" s="15" t="n"/>
-      <c r="I31" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="J31" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-22 02:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K31" s="13" t="inlineStr">
-        <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
-        </is>
-      </c>
-      <c r="L31" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M31" s="13" t="inlineStr"/>
-      <c r="N31" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O31" s="14" t="inlineStr">
-        <is>
-          <t>Thu Oct 22 2 PM.</t>
-        </is>
-      </c>
+      <c r="B31" s="12" t="n"/>
+      <c r="C31" s="12" t="n"/>
+      <c r="D31" s="12" t="n"/>
+      <c r="E31" s="12" t="n"/>
+      <c r="F31" s="12" t="n"/>
+      <c r="G31" s="12" t="n"/>
+      <c r="H31" s="12" t="n"/>
+      <c r="I31" s="12" t="n"/>
+      <c r="J31" s="12" t="n"/>
+      <c r="K31" s="12" t="n"/>
+      <c r="L31" s="12" t="n"/>
+      <c r="M31" s="12" t="n"/>
+      <c r="N31" s="12" t="n"/>
+      <c r="O31" s="12" t="n"/>
     </row>
     <row r="32" outlineLevel="1">
       <c r="A32" s="13" t="inlineStr">
@@ -20096,42 +20299,46 @@
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>Tools / plumbing / MRO supply inventory – Hilti/DeWalt/Milwaukee, fittings, heat pumps</t>
+          <t>Japanese BBQ &amp; bar – ~47 lots: Turbo Air, Hoshizaki ice machine, Pitco, Beverage-Air</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>restaurant closing</t>
         </is>
       </c>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>Riverdale</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
         <is>
-          <t>NJ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H32" s="15" t="n"/>
-      <c r="I32" s="13" t="inlineStr"/>
+      <c r="I32" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
       <c r="J32" s="13" t="inlineStr">
         <is>
-          <t>2026-10-30 11:00 AM ET</t>
+          <t>2026-10-21 04:00 PM ET</t>
         </is>
       </c>
       <c r="K32" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
       <c r="L32" s="13" t="inlineStr">
@@ -20147,7 +20354,7 @@
       </c>
       <c r="O32" s="14" t="inlineStr">
         <is>
-          <t>Bulk resale inventory.</t>
+          <t>Wed Oct 21 4 PM. NYC 10013.</t>
         </is>
       </c>
     </row>
@@ -20159,17 +20366,17 @@
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>Ice cream + cookie franchise equipment – Taylor soft-serve, Atosa, Blodgett</t>
+          <t>Corporate caterer – Alto-Shaam, new boxed Avantco rice cookers &amp; Cadco oven, Perlick, MerryChef</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D33" s="13" t="inlineStr">
         <is>
-          <t>Riverdale</t>
+          <t>Jersey City</t>
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr">
@@ -20178,23 +20385,27 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="G33" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H33" s="15" t="n"/>
-      <c r="I33" s="13" t="inlineStr"/>
+      <c r="I33" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="J33" s="13" t="inlineStr">
         <is>
-          <t>2026-11-05 11:00 AM ET</t>
+          <t>2026-10-22 02:00 PM ET</t>
         </is>
       </c>
       <c r="K33" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
       <c r="L33" s="13" t="inlineStr">
@@ -20210,7 +20421,7 @@
       </c>
       <c r="O33" s="14" t="inlineStr">
         <is>
-          <t>Resellable units.</t>
+          <t>Thu Oct 22 2 PM.</t>
         </is>
       </c>
     </row>
@@ -20222,51 +20433,47 @@
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>Like-new restaurant – steam tables, Coldline, Cleveland cook-and-hold, fryers, True freezers</t>
+          <t>Tools / plumbing / MRO supply inventory – Hilti/DeWalt/Milwaukee, fittings, heat pumps</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>inventory</t>
         </is>
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>Staten Island</t>
+          <t>Riverdale</t>
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H34" s="15" t="n"/>
-      <c r="I34" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
+      <c r="I34" s="13" t="inlineStr"/>
       <c r="J34" s="13" t="inlineStr">
         <is>
-          <t>2026-10-19 01:00 PM ET</t>
+          <t>2026-10-30 11:00 AM ET</t>
         </is>
       </c>
       <c r="K34" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
-        </is>
-      </c>
-      <c r="L34" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>A.J. Willner</t>
+        </is>
+      </c>
+      <c r="L34" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M34" s="13" t="inlineStr"/>
@@ -20277,7 +20484,7 @@
       </c>
       <c r="O34" s="14" t="inlineStr">
         <is>
-          <t>"Short notice" auction Mon Oct 19 1 PM.</t>
+          <t>Bulk resale inventory.</t>
         </is>
       </c>
     </row>
@@ -20289,17 +20496,17 @@
       </c>
       <c r="B35" s="14" t="inlineStr">
         <is>
-          <t>Major food-service caterer – new-in-box True reach-ins, Beverage-Air, TurboChef, Resfab ventless fryer</t>
+          <t>Ice cream + cookie franchise equipment – Taylor soft-serve, Atosa, Blodgett</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D35" s="13" t="inlineStr">
         <is>
-          <t>Parsippany</t>
+          <t>Riverdale</t>
         </is>
       </c>
       <c r="E35" s="13" t="inlineStr">
@@ -20308,27 +20515,23 @@
         </is>
       </c>
       <c r="F35" s="13" t="n">
-        <v>206</v>
+        <v>196</v>
       </c>
       <c r="G35" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H35" s="15" t="n"/>
-      <c r="I35" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
+      <c r="I35" s="13" t="inlineStr"/>
       <c r="J35" s="13" t="inlineStr">
         <is>
-          <t>2026-11-03 02:00 PM ET</t>
+          <t>2026-11-05 11:00 AM ET</t>
         </is>
       </c>
       <c r="K35" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>A.J. Willner</t>
         </is>
       </c>
       <c r="L35" s="13" t="inlineStr">
@@ -20344,7 +20547,7 @@
       </c>
       <c r="O35" s="14" t="inlineStr">
         <is>
-          <t>Tue Nov 3 2 PM, checkout Nov 4.</t>
+          <t>Resellable units.</t>
         </is>
       </c>
     </row>
@@ -20356,47 +20559,51 @@
       </c>
       <c r="B36" s="14" t="inlineStr">
         <is>
-          <t>Serpico's Pizzeria (lost lease) – Bari ovens, walk-in, Hobart 60qt, Vulcan range</t>
+          <t>Like-new restaurant – steam tables, Coldline, Cleveland cook-and-hold, fryers, True freezers</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
-          <t>Allenhurst</t>
+          <t>Staten Island</t>
         </is>
       </c>
       <c r="E36" s="13" t="inlineStr">
         <is>
-          <t>NJ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="G36" s="13" t="inlineStr">
         <is>
-          <t>No-reserve online auction</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H36" s="15" t="n"/>
-      <c r="I36" s="13" t="inlineStr"/>
+      <c r="I36" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="J36" s="13" t="inlineStr">
         <is>
-          <t>2026-10-21 11:00 AM ET</t>
+          <t>2026-10-19 01:00 PM ET</t>
         </is>
       </c>
       <c r="K36" s="13" t="inlineStr">
         <is>
-          <t>Peter Costanzo / EstateSales.net</t>
-        </is>
-      </c>
-      <c r="L36" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
+        </is>
+      </c>
+      <c r="L36" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M36" s="13" t="inlineStr"/>
@@ -20407,7 +20614,7 @@
       </c>
       <c r="O36" s="14" t="inlineStr">
         <is>
-          <t>Absolute / no reserve.</t>
+          <t>"Short notice" auction Mon Oct 19 1 PM.</t>
         </is>
       </c>
     </row>
@@ -20419,17 +20626,17 @@
       </c>
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>Altitude Trampoline Park liquidation – partial: Atosa, TurboChef, stainless</t>
+          <t>Major food-service caterer – new-in-box True reach-ins, Beverage-Air, TurboChef, Resfab ventless fryer</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>facility contents</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">
         <is>
-          <t>Iselin</t>
+          <t>Parsippany</t>
         </is>
       </c>
       <c r="E37" s="13" t="inlineStr">
@@ -20438,23 +20645,27 @@
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="G37" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H37" s="15" t="n"/>
-      <c r="I37" s="13" t="inlineStr"/>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
       <c r="J37" s="13" t="inlineStr">
         <is>
-          <t>2026-10-21 11:00 AM ET</t>
+          <t>2026-11-03 02:00 PM ET</t>
         </is>
       </c>
       <c r="K37" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
       <c r="L37" s="13" t="inlineStr">
@@ -20470,7 +20681,7 @@
       </c>
       <c r="O37" s="14" t="inlineStr">
         <is>
-          <t>Some kitchen gear only.</t>
+          <t>Tue Nov 3 2 PM, checkout Nov 4.</t>
         </is>
       </c>
     </row>
@@ -20482,17 +20693,17 @@
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>Restaurant / pizzeria (contents not described)</t>
+          <t>Serpico's Pizzeria (lost lease) – Bari ovens, walk-in, Hobart 60qt, Vulcan range</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>restaurant closing</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
         <is>
-          <t>Berkeley Heights</t>
+          <t>Allenhurst</t>
         </is>
       </c>
       <c r="E38" s="13" t="inlineStr">
@@ -20501,27 +20712,23 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>No-reserve online auction</t>
         </is>
       </c>
       <c r="H38" s="15" t="n"/>
-      <c r="I38" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
+      <c r="I38" s="13" t="inlineStr"/>
       <c r="J38" s="13" t="inlineStr">
         <is>
-          <t>2026-10-20 02:00 PM ET</t>
+          <t>2026-10-21 11:00 AM ET</t>
         </is>
       </c>
       <c r="K38" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>Peter Costanzo / EstateSales.net</t>
         </is>
       </c>
       <c r="L38" s="20" t="inlineStr">
@@ -20537,7 +20744,7 @@
       </c>
       <c r="O38" s="14" t="inlineStr">
         <is>
-          <t>Tue Oct 20 2 PM. No item description on page.</t>
+          <t>Absolute / no reserve.</t>
         </is>
       </c>
     </row>
@@ -20549,17 +20756,17 @@
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>New modular concession kitchens (warehouseman's lien) – 5 units, CaptiveAire hoods, new Ovention/Turbo Air</t>
+          <t>Altitude Trampoline Park liquidation – partial: Atosa, TurboChef, stainless</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>lien sale</t>
+          <t>facility contents</t>
         </is>
       </c>
       <c r="D39" s="13" t="inlineStr">
         <is>
-          <t>Edison</t>
+          <t>Iselin</t>
         </is>
       </c>
       <c r="E39" s="13" t="inlineStr">
@@ -20568,24 +20775,28 @@
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="G39" s="13" t="inlineStr">
         <is>
-          <t>Online auction, $2K load-out fee</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H39" s="15" t="n"/>
       <c r="I39" s="13" t="inlineStr"/>
-      <c r="J39" s="13" t="inlineStr"/>
+      <c r="J39" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-21 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K39" s="13" t="inlineStr">
         <is>
           <t>A.J. Willner</t>
         </is>
       </c>
-      <c r="L39" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+      <c r="L39" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M39" s="13" t="inlineStr"/>
@@ -20596,7 +20807,7 @@
       </c>
       <c r="O39" s="14" t="inlineStr">
         <is>
-          <t>&gt;$100K new. Close date not captured.</t>
+          <t>Some kitchen gear only.</t>
         </is>
       </c>
     </row>
@@ -20608,17 +20819,17 @@
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>Brand-new &amp; scratch-and-dent kitchen/home appliances – ~185 lots (Thermador, GE Café, Miele, Wolf speed oven, Viking, Bosch…)</t>
+          <t>Restaurant / pizzeria (contents not described)</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>restaurant closing</t>
         </is>
       </c>
       <c r="D40" s="13" t="inlineStr">
         <is>
-          <t>Edison</t>
+          <t>Berkeley Heights</t>
         </is>
       </c>
       <c r="E40" s="13" t="inlineStr">
@@ -20627,22 +20838,22 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t>Live + HiBid webcast, 18% BP + 3% card</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H40" s="15" t="n"/>
       <c r="I40" s="13" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="J40" s="13" t="inlineStr">
         <is>
-          <t>2026-10-25 01:00 PM ET</t>
+          <t>2026-10-20 02:00 PM ET</t>
         </is>
       </c>
       <c r="K40" s="13" t="inlineStr">
@@ -20650,16 +20861,12 @@
           <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
-      <c r="L40" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M40" s="21" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
+      <c r="L40" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M40" s="13" t="inlineStr"/>
       <c r="N40" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -20667,7 +20874,7 @@
       </c>
       <c r="O40" s="14" t="inlineStr">
         <is>
-          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale.</t>
+          <t>Tue Oct 20 2 PM. No item description on page.</t>
         </is>
       </c>
     </row>
@@ -20679,17 +20886,17 @@
       </c>
       <c r="B41" s="14" t="inlineStr">
         <is>
-          <t>Party City (Ch. 11) store – fixtures + party merchandise inventory</t>
+          <t>New modular concession kitchens (warehouseman's lien) – 5 units, CaptiveAire hoods, new Ovention/Turbo Air</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>lien sale</t>
         </is>
       </c>
       <c r="D41" s="13" t="inlineStr">
         <is>
-          <t>East Brunswick</t>
+          <t>Edison</t>
         </is>
       </c>
       <c r="E41" s="13" t="inlineStr">
@@ -20698,20 +20905,16 @@
         </is>
       </c>
       <c r="F41" s="13" t="n">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="G41" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Online auction, $2K load-out fee</t>
         </is>
       </c>
       <c r="H41" s="15" t="n"/>
       <c r="I41" s="13" t="inlineStr"/>
-      <c r="J41" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-03 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="J41" s="13" t="inlineStr"/>
       <c r="K41" s="13" t="inlineStr">
         <is>
           <t>A.J. Willner</t>
@@ -20730,7 +20933,7 @@
       </c>
       <c r="O41" s="14" t="inlineStr">
         <is>
-          <t>Store inventory.</t>
+          <t>&gt;$100K new. Close date not captured.</t>
         </is>
       </c>
     </row>
@@ -20742,17 +20945,17 @@
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>High-end deli (contents not described)</t>
+          <t>Brand-new &amp; scratch-and-dent kitchen/home appliances – ~185 lots (Thermador, GE Café, Miele, Wolf speed oven, Viking, Bosch…)</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>restaurant closing</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D42" s="13" t="inlineStr">
         <is>
-          <t>Manalapan Township</t>
+          <t>Edison</t>
         </is>
       </c>
       <c r="E42" s="13" t="inlineStr">
@@ -20761,22 +20964,22 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>Live + HiBid webcast, 18% BP + 3% card</t>
         </is>
       </c>
       <c r="H42" s="15" t="n"/>
       <c r="I42" s="13" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="J42" s="13" t="inlineStr">
         <is>
-          <t>2026-10-19 04:00 PM ET</t>
+          <t>2026-10-25 01:00 PM ET</t>
         </is>
       </c>
       <c r="K42" s="13" t="inlineStr">
@@ -20784,12 +20987,16 @@
           <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
-      <c r="L42" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
-        </is>
-      </c>
-      <c r="M42" s="13" t="inlineStr"/>
+      <c r="L42" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M42" s="21" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
       <c r="N42" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -20797,7 +21004,7 @@
       </c>
       <c r="O42" s="14" t="inlineStr">
         <is>
-          <t>Mon Oct 19 4 PM. No item description on page.</t>
+          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale.</t>
         </is>
       </c>
     </row>
@@ -20809,17 +21016,17 @@
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>Wren Kitchens showroom closing – JennAir/Café/KitchenAid/GE Profile appliances + display kitchens</t>
+          <t>Party City (Ch. 11) store – fixtures + party merchandise inventory</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
         <is>
-          <t>showroom closing</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D43" s="13" t="inlineStr">
         <is>
-          <t>Lawrenceville</t>
+          <t>East Brunswick</t>
         </is>
       </c>
       <c r="E43" s="13" t="inlineStr">
@@ -20828,23 +21035,23 @@
         </is>
       </c>
       <c r="F43" s="13" t="n">
-        <v>239</v>
+        <v>220</v>
       </c>
       <c r="G43" s="13" t="inlineStr">
         <is>
-          <t>Online auction, 18% BP</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H43" s="15" t="n"/>
       <c r="I43" s="13" t="inlineStr"/>
       <c r="J43" s="13" t="inlineStr">
         <is>
-          <t>2026-10-27 09:00 AM ET</t>
+          <t>2026-11-03 11:00 AM ET</t>
         </is>
       </c>
       <c r="K43" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
+          <t>A.J. Willner</t>
         </is>
       </c>
       <c r="L43" s="13" t="inlineStr">
@@ -20860,7 +21067,7 @@
       </c>
       <c r="O43" s="14" t="inlineStr">
         <is>
-          <t>Premium floor-model appliances; lots close from Oct 27 9 AM.</t>
+          <t>Store inventory.</t>
         </is>
       </c>
     </row>
@@ -20872,17 +21079,17 @@
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>Milwaukee / Walmart / hardware store mega auction pt 3</t>
+          <t>High-end deli (contents not described)</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>restaurant closing</t>
         </is>
       </c>
       <c r="D44" s="13" t="inlineStr">
         <is>
-          <t>Mount Holly</t>
+          <t>Manalapan Township</t>
         </is>
       </c>
       <c r="E44" s="13" t="inlineStr">
@@ -20891,23 +21098,27 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>254</v>
+        <v>223</v>
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>HiBid online auction</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H44" s="15" t="n"/>
-      <c r="I44" s="13" t="inlineStr"/>
+      <c r="I44" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="J44" s="13" t="inlineStr">
         <is>
-          <t>2026-10-19 06:00 PM ET</t>
+          <t>2026-10-19 04:00 PM ET</t>
         </is>
       </c>
       <c r="K44" s="13" t="inlineStr">
         <is>
-          <t>HiBid</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
       <c r="L44" s="20" t="inlineStr">
@@ -20923,7 +21134,7 @@
       </c>
       <c r="O44" s="14" t="inlineStr">
         <is>
-          <t>Close Oct 18 or 19 6 PM (later used).</t>
+          <t>Mon Oct 19 4 PM. No item description on page.</t>
         </is>
       </c>
     </row>
@@ -20935,7 +21146,7 @@
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>Wren Kitchens showroom closing – GE/Whirlpool/KitchenAid/Café incl. NIB Café range + 35 kitchens</t>
+          <t>Wren Kitchens showroom closing – JennAir/Café/KitchenAid/GE Profile appliances + display kitchens</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
@@ -20945,7 +21156,7 @@
       </c>
       <c r="D45" s="13" t="inlineStr">
         <is>
-          <t>Cherry Hill</t>
+          <t>Lawrenceville</t>
         </is>
       </c>
       <c r="E45" s="13" t="inlineStr">
@@ -20954,18 +21165,18 @@
         </is>
       </c>
       <c r="F45" s="13" t="n">
-        <v>266</v>
+        <v>239</v>
       </c>
       <c r="G45" s="13" t="inlineStr">
         <is>
-          <t>Online auction, openers ~$0.50</t>
+          <t>Online auction, 18% BP</t>
         </is>
       </c>
       <c r="H45" s="15" t="n"/>
       <c r="I45" s="13" t="inlineStr"/>
       <c r="J45" s="13" t="inlineStr">
         <is>
-          <t>2026-11-02 11:00 AM ET</t>
+          <t>2026-10-27 09:00 AM ET</t>
         </is>
       </c>
       <c r="K45" s="13" t="inlineStr">
@@ -20986,294 +21197,294 @@
       </c>
       <c r="O45" s="14" t="inlineStr">
         <is>
+          <t>Premium floor-model appliances; lots close from Oct 27 9 AM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" outlineLevel="1">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>Milwaukee / Walmart / hardware store mega auction pt 3</t>
+        </is>
+      </c>
+      <c r="C46" s="13" t="inlineStr">
+        <is>
+          <t>inventory</t>
+        </is>
+      </c>
+      <c r="D46" s="13" t="inlineStr">
+        <is>
+          <t>Mount Holly</t>
+        </is>
+      </c>
+      <c r="E46" s="13" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="F46" s="13" t="n">
+        <v>254</v>
+      </c>
+      <c r="G46" s="13" t="inlineStr">
+        <is>
+          <t>HiBid online auction</t>
+        </is>
+      </c>
+      <c r="H46" s="15" t="n"/>
+      <c r="I46" s="13" t="inlineStr"/>
+      <c r="J46" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 06:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K46" s="13" t="inlineStr">
+        <is>
+          <t>HiBid</t>
+        </is>
+      </c>
+      <c r="L46" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M46" s="13" t="inlineStr"/>
+      <c r="N46" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O46" s="14" t="inlineStr">
+        <is>
+          <t>Close Oct 18 or 19 6 PM (later used).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" outlineLevel="1">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>Wren Kitchens showroom closing – GE/Whirlpool/KitchenAid/Café incl. NIB Café range + 35 kitchens</t>
+        </is>
+      </c>
+      <c r="C47" s="13" t="inlineStr">
+        <is>
+          <t>showroom closing</t>
+        </is>
+      </c>
+      <c r="D47" s="13" t="inlineStr">
+        <is>
+          <t>Cherry Hill</t>
+        </is>
+      </c>
+      <c r="E47" s="13" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="F47" s="13" t="n">
+        <v>266</v>
+      </c>
+      <c r="G47" s="13" t="inlineStr">
+        <is>
+          <t>Online auction, openers ~$0.50</t>
+        </is>
+      </c>
+      <c r="H47" s="15" t="n"/>
+      <c r="I47" s="13" t="inlineStr"/>
+      <c r="J47" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-02 11:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K47" s="13" t="inlineStr">
+        <is>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L47" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M47" s="13" t="inlineStr"/>
+      <c r="N47" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O47" s="14" t="inlineStr">
+        <is>
           <t>Lots close from Nov 2 11 AM.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="17" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="17" t="inlineStr">
         <is>
           <t>Subtotal — NYC / Long Island / NJ</t>
         </is>
       </c>
-      <c r="B46" s="17" t="inlineStr">
+      <c r="B48" s="17" t="inlineStr">
         <is>
           <t>16 item(s)</t>
         </is>
       </c>
-      <c r="C46" s="18" t="n"/>
-      <c r="D46" s="18" t="n"/>
-      <c r="E46" s="18" t="n"/>
-      <c r="F46" s="18" t="n"/>
-      <c r="G46" s="18" t="n"/>
-      <c r="H46" s="19" t="n">
+      <c r="C48" s="18" t="n"/>
+      <c r="D48" s="18" t="n"/>
+      <c r="E48" s="18" t="n"/>
+      <c r="F48" s="18" t="n"/>
+      <c r="G48" s="18" t="n"/>
+      <c r="H48" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I46" s="18" t="n"/>
-      <c r="J46" s="18" t="n"/>
-      <c r="K46" s="18" t="n"/>
-      <c r="L46" s="18" t="n"/>
-      <c r="M46" s="18" t="n"/>
-      <c r="N46" s="18" t="n"/>
-      <c r="O46" s="18" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="11" t="inlineStr">
+      <c r="I48" s="18" t="n"/>
+      <c r="J48" s="18" t="n"/>
+      <c r="K48" s="18" t="n"/>
+      <c r="L48" s="18" t="n"/>
+      <c r="M48" s="18" t="n"/>
+      <c r="N48" s="18" t="n"/>
+      <c r="O48" s="18" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="11" t="inlineStr">
         <is>
           <t>▸ Eastern PA / Mid-Atlantic  (1)</t>
         </is>
       </c>
-      <c r="B47" s="12" t="n"/>
-      <c r="C47" s="12" t="n"/>
-      <c r="D47" s="12" t="n"/>
-      <c r="E47" s="12" t="n"/>
-      <c r="F47" s="12" t="n"/>
-      <c r="G47" s="12" t="n"/>
-      <c r="H47" s="12" t="n"/>
-      <c r="I47" s="12" t="n"/>
-      <c r="J47" s="12" t="n"/>
-      <c r="K47" s="12" t="n"/>
-      <c r="L47" s="12" t="n"/>
-      <c r="M47" s="12" t="n"/>
-      <c r="N47" s="12" t="n"/>
-      <c r="O47" s="12" t="n"/>
-    </row>
-    <row r="48" outlineLevel="1">
-      <c r="A48" s="13" t="inlineStr">
+      <c r="B49" s="12" t="n"/>
+      <c r="C49" s="12" t="n"/>
+      <c r="D49" s="12" t="n"/>
+      <c r="E49" s="12" t="n"/>
+      <c r="F49" s="12" t="n"/>
+      <c r="G49" s="12" t="n"/>
+      <c r="H49" s="12" t="n"/>
+      <c r="I49" s="12" t="n"/>
+      <c r="J49" s="12" t="n"/>
+      <c r="K49" s="12" t="n"/>
+      <c r="L49" s="12" t="n"/>
+      <c r="M49" s="12" t="n"/>
+      <c r="N49" s="12" t="n"/>
+      <c r="O49" s="12" t="n"/>
+    </row>
+    <row r="50" outlineLevel="1">
+      <c r="A50" s="13" t="inlineStr">
         <is>
           <t>Eastern PA / Mid-Atlantic</t>
         </is>
       </c>
-      <c r="B48" s="14" t="inlineStr">
+      <c r="B50" s="14" t="inlineStr">
         <is>
           <t>October restaurant consignment – Hobart, Rational, True + NEW scratch-and-dent Migali/Avantco</t>
         </is>
       </c>
-      <c r="C48" s="13" t="inlineStr">
+      <c r="C50" s="13" t="inlineStr">
         <is>
           <t>restaurant</t>
         </is>
       </c>
-      <c r="D48" s="13" t="inlineStr">
+      <c r="D50" s="13" t="inlineStr">
         <is>
           <t>Harrisburg</t>
         </is>
       </c>
-      <c r="E48" s="13" t="inlineStr">
+      <c r="E50" s="13" t="inlineStr">
         <is>
           <t>PA</t>
         </is>
       </c>
-      <c r="F48" s="13" t="n">
+      <c r="F50" s="13" t="n">
         <v>340</v>
       </c>
-      <c r="G48" s="13" t="inlineStr">
+      <c r="G50" s="13" t="inlineStr">
         <is>
           <t>Online auction, 15% BP, ships $55/pallet</t>
         </is>
       </c>
-      <c r="H48" s="15" t="n"/>
-      <c r="I48" s="13" t="inlineStr"/>
-      <c r="J48" s="13" t="inlineStr">
+      <c r="H50" s="15" t="n"/>
+      <c r="I50" s="13" t="inlineStr"/>
+      <c r="J50" s="13" t="inlineStr">
         <is>
           <t>2026-10-21 11:00 AM ET</t>
         </is>
       </c>
-      <c r="K48" s="13" t="inlineStr">
+      <c r="K50" s="13" t="inlineStr">
         <is>
           <t>Restaurant Auction Co</t>
         </is>
       </c>
-      <c r="L48" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M48" s="13" t="inlineStr"/>
-      <c r="N48" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O48" s="14" t="inlineStr">
+      <c r="L50" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M50" s="13" t="inlineStr"/>
+      <c r="N50" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O50" s="14" t="inlineStr">
         <is>
           <t>Closes Oct 21 10 or 11 AM (later used). Shippable.</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="17" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Eastern PA / Mid-Atlantic</t>
         </is>
       </c>
-      <c r="B49" s="17" t="inlineStr">
+      <c r="B51" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C49" s="18" t="n"/>
-      <c r="D49" s="18" t="n"/>
-      <c r="E49" s="18" t="n"/>
-      <c r="F49" s="18" t="n"/>
-      <c r="G49" s="18" t="n"/>
-      <c r="H49" s="19" t="n">
+      <c r="C51" s="18" t="n"/>
+      <c r="D51" s="18" t="n"/>
+      <c r="E51" s="18" t="n"/>
+      <c r="F51" s="18" t="n"/>
+      <c r="G51" s="18" t="n"/>
+      <c r="H51" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I49" s="18" t="n"/>
-      <c r="J49" s="18" t="n"/>
-      <c r="K49" s="18" t="n"/>
-      <c r="L49" s="18" t="n"/>
-      <c r="M49" s="18" t="n"/>
-      <c r="N49" s="18" t="n"/>
-      <c r="O49" s="18" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="11" t="inlineStr">
+      <c r="I51" s="18" t="n"/>
+      <c r="J51" s="18" t="n"/>
+      <c r="K51" s="18" t="n"/>
+      <c r="L51" s="18" t="n"/>
+      <c r="M51" s="18" t="n"/>
+      <c r="N51" s="18" t="n"/>
+      <c r="O51" s="18" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="11" t="inlineStr">
         <is>
           <t>▸ Upstate / Western NY  (3)</t>
         </is>
       </c>
-      <c r="B50" s="12" t="n"/>
-      <c r="C50" s="12" t="n"/>
-      <c r="D50" s="12" t="n"/>
-      <c r="E50" s="12" t="n"/>
-      <c r="F50" s="12" t="n"/>
-      <c r="G50" s="12" t="n"/>
-      <c r="H50" s="12" t="n"/>
-      <c r="I50" s="12" t="n"/>
-      <c r="J50" s="12" t="n"/>
-      <c r="K50" s="12" t="n"/>
-      <c r="L50" s="12" t="n"/>
-      <c r="M50" s="12" t="n"/>
-      <c r="N50" s="12" t="n"/>
-      <c r="O50" s="12" t="n"/>
-    </row>
-    <row r="51" outlineLevel="1">
-      <c r="A51" s="13" t="inlineStr">
-        <is>
-          <t>Upstate / Western NY</t>
-        </is>
-      </c>
-      <c r="B51" s="14" t="inlineStr">
-        <is>
-          <t>Former Taco Del Mar – stainless, warmers, walk-in panels</t>
-        </is>
-      </c>
-      <c r="C51" s="13" t="inlineStr">
-        <is>
-          <t>restaurant</t>
-        </is>
-      </c>
-      <c r="D51" s="13" t="inlineStr">
-        <is>
-          <t>Watson</t>
-        </is>
-      </c>
-      <c r="E51" s="13" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="F51" s="13" t="n">
-        <v>260</v>
-      </c>
-      <c r="G51" s="13" t="inlineStr">
-        <is>
-          <t>HiBid online auction</t>
-        </is>
-      </c>
-      <c r="H51" s="15" t="n"/>
-      <c r="I51" s="13" t="inlineStr"/>
-      <c r="J51" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-20 06:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K51" s="13" t="inlineStr">
-        <is>
-          <t>Adirondack Asset / HiBid</t>
-        </is>
-      </c>
-      <c r="L51" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
-        </is>
-      </c>
-      <c r="M51" s="13" t="inlineStr"/>
-      <c r="N51" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O51" s="14" t="inlineStr">
-        <is>
-          <t>Small lot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" outlineLevel="1">
-      <c r="A52" s="13" t="inlineStr">
-        <is>
-          <t>Upstate / Western NY</t>
-        </is>
-      </c>
-      <c r="B52" s="14" t="inlineStr">
-        <is>
-          <t>Closed restaurant – coolers, fridges, prep tables</t>
-        </is>
-      </c>
-      <c r="C52" s="13" t="inlineStr">
-        <is>
-          <t>restaurant</t>
-        </is>
-      </c>
-      <c r="D52" s="13" t="inlineStr">
-        <is>
-          <t>Palmyra</t>
-        </is>
-      </c>
-      <c r="E52" s="13" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="F52" s="13" t="n">
-        <v>333</v>
-      </c>
-      <c r="G52" s="13" t="inlineStr">
-        <is>
-          <t>HiBid, 15% BP</t>
-        </is>
-      </c>
-      <c r="H52" s="15" t="n"/>
-      <c r="I52" s="13" t="inlineStr"/>
-      <c r="J52" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-19 07:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K52" s="13" t="inlineStr">
-        <is>
-          <t>Reynolds Auction Co / HiBid</t>
-        </is>
-      </c>
-      <c r="L52" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
-        </is>
-      </c>
-      <c r="M52" s="13" t="inlineStr"/>
-      <c r="N52" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O52" s="14" t="inlineStr">
-        <is>
-          <t>No new out-of-state bidders. Small.</t>
-        </is>
-      </c>
+      <c r="B52" s="12" t="n"/>
+      <c r="C52" s="12" t="n"/>
+      <c r="D52" s="12" t="n"/>
+      <c r="E52" s="12" t="n"/>
+      <c r="F52" s="12" t="n"/>
+      <c r="G52" s="12" t="n"/>
+      <c r="H52" s="12" t="n"/>
+      <c r="I52" s="12" t="n"/>
+      <c r="J52" s="12" t="n"/>
+      <c r="K52" s="12" t="n"/>
+      <c r="L52" s="12" t="n"/>
+      <c r="M52" s="12" t="n"/>
+      <c r="N52" s="12" t="n"/>
+      <c r="O52" s="12" t="n"/>
     </row>
     <row r="53" outlineLevel="1">
       <c r="A53" s="13" t="inlineStr">
@@ -21283,7 +21494,7 @@
       </c>
       <c r="B53" s="14" t="inlineStr">
         <is>
-          <t>Restaurant &amp; fitness equipment</t>
+          <t>Former Taco Del Mar – stainless, warmers, walk-in panels</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
@@ -21293,7 +21504,7 @@
       </c>
       <c r="D53" s="13" t="inlineStr">
         <is>
-          <t>Williamsville</t>
+          <t>Watson</t>
         </is>
       </c>
       <c r="E53" s="13" t="inlineStr">
@@ -21302,28 +21513,28 @@
         </is>
       </c>
       <c r="F53" s="13" t="n">
-        <v>408</v>
+        <v>260</v>
       </c>
       <c r="G53" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>HiBid online auction</t>
         </is>
       </c>
       <c r="H53" s="15" t="n"/>
       <c r="I53" s="13" t="inlineStr"/>
       <c r="J53" s="13" t="inlineStr">
         <is>
-          <t>2026-10-26 07:30 PM ET</t>
+          <t>2026-10-20 06:00 PM ET</t>
         </is>
       </c>
       <c r="K53" s="13" t="inlineStr">
         <is>
-          <t>Cash Auctions</t>
-        </is>
-      </c>
-      <c r="L53" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>Adirondack Asset / HiBid</t>
+        </is>
+      </c>
+      <c r="L53" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M53" s="13" t="inlineStr"/>
@@ -21334,455 +21545,692 @@
       </c>
       <c r="O53" s="14" t="inlineStr">
         <is>
+          <t>Small lot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" outlineLevel="1">
+      <c r="A54" s="13" t="inlineStr">
+        <is>
+          <t>Upstate / Western NY</t>
+        </is>
+      </c>
+      <c r="B54" s="14" t="inlineStr">
+        <is>
+          <t>Closed restaurant – coolers, fridges, prep tables</t>
+        </is>
+      </c>
+      <c r="C54" s="13" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D54" s="13" t="inlineStr">
+        <is>
+          <t>Palmyra</t>
+        </is>
+      </c>
+      <c r="E54" s="13" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="F54" s="13" t="n">
+        <v>333</v>
+      </c>
+      <c r="G54" s="13" t="inlineStr">
+        <is>
+          <t>HiBid, 15% BP</t>
+        </is>
+      </c>
+      <c r="H54" s="15" t="n"/>
+      <c r="I54" s="13" t="inlineStr"/>
+      <c r="J54" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K54" s="13" t="inlineStr">
+        <is>
+          <t>Reynolds Auction Co / HiBid</t>
+        </is>
+      </c>
+      <c r="L54" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M54" s="13" t="inlineStr"/>
+      <c r="N54" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O54" s="14" t="inlineStr">
+        <is>
+          <t>No new out-of-state bidders. Small.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" outlineLevel="1">
+      <c r="A55" s="13" t="inlineStr">
+        <is>
+          <t>Upstate / Western NY</t>
+        </is>
+      </c>
+      <c r="B55" s="14" t="inlineStr">
+        <is>
+          <t>Restaurant &amp; fitness equipment</t>
+        </is>
+      </c>
+      <c r="C55" s="13" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D55" s="13" t="inlineStr">
+        <is>
+          <t>Williamsville</t>
+        </is>
+      </c>
+      <c r="E55" s="13" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="F55" s="13" t="n">
+        <v>408</v>
+      </c>
+      <c r="G55" s="13" t="inlineStr">
+        <is>
+          <t>Online auction</t>
+        </is>
+      </c>
+      <c r="H55" s="15" t="n"/>
+      <c r="I55" s="13" t="inlineStr"/>
+      <c r="J55" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-26 07:30 PM ET</t>
+        </is>
+      </c>
+      <c r="K55" s="13" t="inlineStr">
+        <is>
+          <t>Cash Auctions</t>
+        </is>
+      </c>
+      <c r="L55" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M55" s="13" t="inlineStr"/>
+      <c r="N55" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O55" s="14" t="inlineStr">
+        <is>
           <t>Lots not reviewed.</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="17" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Upstate / Western NY</t>
         </is>
       </c>
-      <c r="B54" s="17" t="inlineStr">
+      <c r="B56" s="17" t="inlineStr">
         <is>
           <t>3 item(s)</t>
         </is>
       </c>
-      <c r="C54" s="18" t="n"/>
-      <c r="D54" s="18" t="n"/>
-      <c r="E54" s="18" t="n"/>
-      <c r="F54" s="18" t="n"/>
-      <c r="G54" s="18" t="n"/>
-      <c r="H54" s="19" t="n">
+      <c r="C56" s="18" t="n"/>
+      <c r="D56" s="18" t="n"/>
+      <c r="E56" s="18" t="n"/>
+      <c r="F56" s="18" t="n"/>
+      <c r="G56" s="18" t="n"/>
+      <c r="H56" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I54" s="18" t="n"/>
-      <c r="J54" s="18" t="n"/>
-      <c r="K54" s="18" t="n"/>
-      <c r="L54" s="18" t="n"/>
-      <c r="M54" s="18" t="n"/>
-      <c r="N54" s="18" t="n"/>
-      <c r="O54" s="18" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="11" t="inlineStr">
+      <c r="I56" s="18" t="n"/>
+      <c r="J56" s="18" t="n"/>
+      <c r="K56" s="18" t="n"/>
+      <c r="L56" s="18" t="n"/>
+      <c r="M56" s="18" t="n"/>
+      <c r="N56" s="18" t="n"/>
+      <c r="O56" s="18" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="11" t="inlineStr">
         <is>
           <t>▸ Virginia  (1)</t>
         </is>
       </c>
-      <c r="B55" s="12" t="n"/>
-      <c r="C55" s="12" t="n"/>
-      <c r="D55" s="12" t="n"/>
-      <c r="E55" s="12" t="n"/>
-      <c r="F55" s="12" t="n"/>
-      <c r="G55" s="12" t="n"/>
-      <c r="H55" s="12" t="n"/>
-      <c r="I55" s="12" t="n"/>
-      <c r="J55" s="12" t="n"/>
-      <c r="K55" s="12" t="n"/>
-      <c r="L55" s="12" t="n"/>
-      <c r="M55" s="12" t="n"/>
-      <c r="N55" s="12" t="n"/>
-      <c r="O55" s="12" t="n"/>
-    </row>
-    <row r="56" outlineLevel="1">
-      <c r="A56" s="13" t="inlineStr">
+      <c r="B57" s="12" t="n"/>
+      <c r="C57" s="12" t="n"/>
+      <c r="D57" s="12" t="n"/>
+      <c r="E57" s="12" t="n"/>
+      <c r="F57" s="12" t="n"/>
+      <c r="G57" s="12" t="n"/>
+      <c r="H57" s="12" t="n"/>
+      <c r="I57" s="12" t="n"/>
+      <c r="J57" s="12" t="n"/>
+      <c r="K57" s="12" t="n"/>
+      <c r="L57" s="12" t="n"/>
+      <c r="M57" s="12" t="n"/>
+      <c r="N57" s="12" t="n"/>
+      <c r="O57" s="12" t="n"/>
+    </row>
+    <row r="58" outlineLevel="1">
+      <c r="A58" s="13" t="inlineStr">
         <is>
           <t>Virginia</t>
         </is>
       </c>
-      <c r="B56" s="14" t="inlineStr">
+      <c r="B58" s="14" t="inlineStr">
         <is>
           <t>Haynes Furniture / The Dump – 12 stores closing (furniture, mattresses)</t>
         </is>
       </c>
-      <c r="C56" s="13" t="inlineStr">
+      <c r="C58" s="13" t="inlineStr">
         <is>
           <t>retail GOB</t>
         </is>
       </c>
-      <c r="D56" s="13" t="inlineStr">
+      <c r="D58" s="13" t="inlineStr">
         <is>
           <t>Virginia Beach</t>
         </is>
       </c>
-      <c r="E56" s="13" t="inlineStr">
+      <c r="E58" s="13" t="inlineStr">
         <is>
           <t>VA</t>
         </is>
       </c>
-      <c r="F56" s="13" t="n">
+      <c r="F58" s="13" t="n">
         <v>456</v>
       </c>
-      <c r="G56" s="13" t="inlineStr">
+      <c r="G58" s="13" t="inlineStr">
         <is>
           <t>Retail GOB markdowns</t>
         </is>
       </c>
-      <c r="H56" s="15" t="n"/>
-      <c r="I56" s="13" t="inlineStr">
+      <c r="H58" s="15" t="n"/>
+      <c r="I58" s="13" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>
       </c>
-      <c r="J56" s="13" t="inlineStr"/>
-      <c r="K56" s="13" t="inlineStr">
+      <c r="J58" s="13" t="inlineStr"/>
+      <c r="K58" s="13" t="inlineStr">
         <is>
           <t>SB360 (PR Newswire)</t>
         </is>
       </c>
-      <c r="L56" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M56" s="13" t="inlineStr"/>
-      <c r="N56" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O56" s="14" t="inlineStr">
+      <c r="L58" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M58" s="13" t="inlineStr"/>
+      <c r="N58" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O58" s="14" t="inlineStr">
         <is>
           <t>Posted Oct 8. Multi-state (VA/AZ/GA/IL/TX); pinned at Virginia Beach. Home goods only.</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="17" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Virginia</t>
         </is>
       </c>
-      <c r="B57" s="17" t="inlineStr">
+      <c r="B59" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C57" s="18" t="n"/>
-      <c r="D57" s="18" t="n"/>
-      <c r="E57" s="18" t="n"/>
-      <c r="F57" s="18" t="n"/>
-      <c r="G57" s="18" t="n"/>
-      <c r="H57" s="19" t="n">
+      <c r="C59" s="18" t="n"/>
+      <c r="D59" s="18" t="n"/>
+      <c r="E59" s="18" t="n"/>
+      <c r="F59" s="18" t="n"/>
+      <c r="G59" s="18" t="n"/>
+      <c r="H59" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I57" s="18" t="n"/>
-      <c r="J57" s="18" t="n"/>
-      <c r="K57" s="18" t="n"/>
-      <c r="L57" s="18" t="n"/>
-      <c r="M57" s="18" t="n"/>
-      <c r="N57" s="18" t="n"/>
-      <c r="O57" s="18" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="11" t="inlineStr">
+      <c r="I59" s="18" t="n"/>
+      <c r="J59" s="18" t="n"/>
+      <c r="K59" s="18" t="n"/>
+      <c r="L59" s="18" t="n"/>
+      <c r="M59" s="18" t="n"/>
+      <c r="N59" s="18" t="n"/>
+      <c r="O59" s="18" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
         <is>
           <t>▸ Midwest  (2)</t>
         </is>
       </c>
-      <c r="B58" s="12" t="n"/>
-      <c r="C58" s="12" t="n"/>
-      <c r="D58" s="12" t="n"/>
-      <c r="E58" s="12" t="n"/>
-      <c r="F58" s="12" t="n"/>
-      <c r="G58" s="12" t="n"/>
-      <c r="H58" s="12" t="n"/>
-      <c r="I58" s="12" t="n"/>
-      <c r="J58" s="12" t="n"/>
-      <c r="K58" s="12" t="n"/>
-      <c r="L58" s="12" t="n"/>
-      <c r="M58" s="12" t="n"/>
-      <c r="N58" s="12" t="n"/>
-      <c r="O58" s="12" t="n"/>
-    </row>
-    <row r="59" outlineLevel="1">
-      <c r="A59" s="13" t="inlineStr">
+      <c r="B60" s="12" t="n"/>
+      <c r="C60" s="12" t="n"/>
+      <c r="D60" s="12" t="n"/>
+      <c r="E60" s="12" t="n"/>
+      <c r="F60" s="12" t="n"/>
+      <c r="G60" s="12" t="n"/>
+      <c r="H60" s="12" t="n"/>
+      <c r="I60" s="12" t="n"/>
+      <c r="J60" s="12" t="n"/>
+      <c r="K60" s="12" t="n"/>
+      <c r="L60" s="12" t="n"/>
+      <c r="M60" s="12" t="n"/>
+      <c r="N60" s="12" t="n"/>
+      <c r="O60" s="12" t="n"/>
+    </row>
+    <row r="61" outlineLevel="1">
+      <c r="A61" s="13" t="inlineStr">
         <is>
           <t>Midwest</t>
         </is>
       </c>
-      <c r="B59" s="14" t="inlineStr">
+      <c r="B61" s="14" t="inlineStr">
         <is>
           <t>Freshway Market whole-grocery liquidation – refrigeration racks, cases, walk-ins, generator</t>
         </is>
       </c>
-      <c r="C59" s="13" t="inlineStr">
+      <c r="C61" s="13" t="inlineStr">
         <is>
           <t>store closing</t>
         </is>
       </c>
-      <c r="D59" s="13" t="inlineStr">
+      <c r="D61" s="13" t="inlineStr">
         <is>
           <t>Chicago</t>
         </is>
       </c>
-      <c r="E59" s="13" t="inlineStr">
+      <c r="E61" s="13" t="inlineStr">
         <is>
           <t>IL</t>
         </is>
       </c>
-      <c r="F59" s="13" t="n">
+      <c r="F61" s="13" t="n">
         <v>862</v>
       </c>
-      <c r="G59" s="13" t="inlineStr">
+      <c r="G61" s="13" t="inlineStr">
         <is>
           <t>Online auction</t>
         </is>
       </c>
-      <c r="H59" s="15" t="n"/>
-      <c r="I59" s="13" t="inlineStr"/>
-      <c r="J59" s="13" t="inlineStr">
+      <c r="H61" s="15" t="n"/>
+      <c r="I61" s="13" t="inlineStr"/>
+      <c r="J61" s="13" t="inlineStr">
         <is>
           <t>2026-10-20 11:00 AM ET</t>
         </is>
       </c>
-      <c r="K59" s="13" t="inlineStr">
+      <c r="K61" s="13" t="inlineStr">
         <is>
           <t>Grafe Auction</t>
         </is>
       </c>
-      <c r="L59" s="20" t="inlineStr">
+      <c r="L61" s="20" t="inlineStr">
         <is>
           <t>ENDING SOON</t>
         </is>
       </c>
-      <c r="M59" s="13" t="inlineStr"/>
-      <c r="N59" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O59" s="14" t="inlineStr">
+      <c r="M61" s="13" t="inlineStr"/>
+      <c r="N61" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O61" s="14" t="inlineStr">
         <is>
           <t>Closes from Oct 20 10 AM CDT.</t>
         </is>
       </c>
     </row>
-    <row r="60" outlineLevel="1">
-      <c r="A60" s="13" t="inlineStr">
+    <row r="62" outlineLevel="1">
+      <c r="A62" s="13" t="inlineStr">
         <is>
           <t>Midwest</t>
         </is>
       </c>
-      <c r="B60" s="14" t="inlineStr">
+      <c r="B62" s="14" t="inlineStr">
         <is>
           <t>American Sale – total liquidation, all 7 stores (pools, hot tubs, grills, holiday decor)</t>
         </is>
       </c>
-      <c r="C60" s="13" t="inlineStr">
+      <c r="C62" s="13" t="inlineStr">
         <is>
           <t>retail GOB</t>
         </is>
       </c>
-      <c r="D60" s="13" t="inlineStr">
+      <c r="D62" s="13" t="inlineStr">
         <is>
           <t>Chicagoland</t>
         </is>
       </c>
-      <c r="E60" s="13" t="inlineStr">
+      <c r="E62" s="13" t="inlineStr">
         <is>
           <t>IL</t>
         </is>
       </c>
-      <c r="F60" s="13" t="n">
+      <c r="F62" s="13" t="n">
         <v>876</v>
       </c>
-      <c r="G60" s="13" t="inlineStr">
+      <c r="G62" s="13" t="inlineStr">
         <is>
           <t>Retail GOB, up to 70% off</t>
         </is>
       </c>
-      <c r="H60" s="15" t="n"/>
-      <c r="I60" s="13" t="inlineStr">
+      <c r="H62" s="15" t="n"/>
+      <c r="I62" s="13" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="J60" s="13" t="inlineStr"/>
-      <c r="K60" s="13" t="inlineStr">
+      <c r="J62" s="13" t="inlineStr"/>
+      <c r="K62" s="13" t="inlineStr">
         <is>
           <t>Tiger Group (PR Newswire)</t>
         </is>
       </c>
-      <c r="L60" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M60" s="13" t="inlineStr"/>
-      <c r="N60" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O60" s="14" t="inlineStr">
+      <c r="L62" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M62" s="13" t="inlineStr"/>
+      <c r="N62" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O62" s="14" t="inlineStr">
         <is>
           <t>Posted Oct 15. Watch for a bulk/fixture auction.</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="17" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Midwest</t>
         </is>
       </c>
-      <c r="B61" s="17" t="inlineStr">
+      <c r="B63" s="17" t="inlineStr">
         <is>
           <t>2 item(s)</t>
         </is>
       </c>
-      <c r="C61" s="18" t="n"/>
-      <c r="D61" s="18" t="n"/>
-      <c r="E61" s="18" t="n"/>
-      <c r="F61" s="18" t="n"/>
-      <c r="G61" s="18" t="n"/>
-      <c r="H61" s="19" t="n">
+      <c r="C63" s="18" t="n"/>
+      <c r="D63" s="18" t="n"/>
+      <c r="E63" s="18" t="n"/>
+      <c r="F63" s="18" t="n"/>
+      <c r="G63" s="18" t="n"/>
+      <c r="H63" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I61" s="18" t="n"/>
-      <c r="J61" s="18" t="n"/>
-      <c r="K61" s="18" t="n"/>
-      <c r="L61" s="18" t="n"/>
-      <c r="M61" s="18" t="n"/>
-      <c r="N61" s="18" t="n"/>
-      <c r="O61" s="18" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="11" t="inlineStr">
+      <c r="I63" s="18" t="n"/>
+      <c r="J63" s="18" t="n"/>
+      <c r="K63" s="18" t="n"/>
+      <c r="L63" s="18" t="n"/>
+      <c r="M63" s="18" t="n"/>
+      <c r="N63" s="18" t="n"/>
+      <c r="O63" s="18" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="inlineStr">
         <is>
           <t>▸ Texas / South Central  (1)</t>
         </is>
       </c>
-      <c r="B62" s="12" t="n"/>
-      <c r="C62" s="12" t="n"/>
-      <c r="D62" s="12" t="n"/>
-      <c r="E62" s="12" t="n"/>
-      <c r="F62" s="12" t="n"/>
-      <c r="G62" s="12" t="n"/>
-      <c r="H62" s="12" t="n"/>
-      <c r="I62" s="12" t="n"/>
-      <c r="J62" s="12" t="n"/>
-      <c r="K62" s="12" t="n"/>
-      <c r="L62" s="12" t="n"/>
-      <c r="M62" s="12" t="n"/>
-      <c r="N62" s="12" t="n"/>
-      <c r="O62" s="12" t="n"/>
-    </row>
-    <row r="63" outlineLevel="1">
-      <c r="A63" s="13" t="inlineStr">
+      <c r="B64" s="12" t="n"/>
+      <c r="C64" s="12" t="n"/>
+      <c r="D64" s="12" t="n"/>
+      <c r="E64" s="12" t="n"/>
+      <c r="F64" s="12" t="n"/>
+      <c r="G64" s="12" t="n"/>
+      <c r="H64" s="12" t="n"/>
+      <c r="I64" s="12" t="n"/>
+      <c r="J64" s="12" t="n"/>
+      <c r="K64" s="12" t="n"/>
+      <c r="L64" s="12" t="n"/>
+      <c r="M64" s="12" t="n"/>
+      <c r="N64" s="12" t="n"/>
+      <c r="O64" s="12" t="n"/>
+    </row>
+    <row r="65" outlineLevel="1">
+      <c r="A65" s="13" t="inlineStr">
         <is>
           <t>Texas / South Central</t>
         </is>
       </c>
-      <c r="B63" s="14" t="inlineStr">
+      <c r="B65" s="14" t="inlineStr">
         <is>
           <t>Southwest beverage distributor surplus – mostly unused: 16 True merchandisers, 75 Bunn brewers, 100+ micro-market kiosks</t>
         </is>
       </c>
-      <c r="C63" s="13" t="inlineStr">
+      <c r="C65" s="13" t="inlineStr">
         <is>
           <t>distributor surplus</t>
         </is>
       </c>
-      <c r="D63" s="13" t="inlineStr">
+      <c r="D65" s="13" t="inlineStr">
         <is>
           <t>Mesquite</t>
         </is>
       </c>
-      <c r="E63" s="13" t="inlineStr">
+      <c r="E65" s="13" t="inlineStr">
         <is>
           <t>TX</t>
         </is>
       </c>
-      <c r="F63" s="13" t="n">
+      <c r="F65" s="13" t="n">
         <v>1547</v>
       </c>
-      <c r="G63" s="13" t="inlineStr">
+      <c r="G65" s="13" t="inlineStr">
         <is>
           <t>Online auction</t>
         </is>
       </c>
-      <c r="H63" s="15" t="n"/>
-      <c r="I63" s="13" t="inlineStr"/>
-      <c r="J63" s="13" t="inlineStr">
+      <c r="H65" s="15" t="n"/>
+      <c r="I65" s="13" t="inlineStr"/>
+      <c r="J65" s="13" t="inlineStr">
         <is>
           <t>2026-11-13 11:00 AM ET</t>
         </is>
       </c>
-      <c r="K63" s="13" t="inlineStr">
+      <c r="K65" s="13" t="inlineStr">
         <is>
           <t>Heritage Global Partners</t>
         </is>
       </c>
-      <c r="L63" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M63" s="13" t="inlineStr"/>
-      <c r="N63" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O63" s="14" t="inlineStr">
+      <c r="L65" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M65" s="13" t="inlineStr"/>
+      <c r="N65" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O65" s="14" t="inlineStr">
         <is>
           <t>Near-new appliances, resell by unit. Nov 13 10 AM CST.</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="17" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Texas / South Central</t>
         </is>
       </c>
-      <c r="B64" s="17" t="inlineStr">
+      <c r="B66" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C64" s="18" t="n"/>
-      <c r="D64" s="18" t="n"/>
-      <c r="E64" s="18" t="n"/>
-      <c r="F64" s="18" t="n"/>
-      <c r="G64" s="18" t="n"/>
-      <c r="H64" s="19" t="n">
+      <c r="C66" s="18" t="n"/>
+      <c r="D66" s="18" t="n"/>
+      <c r="E66" s="18" t="n"/>
+      <c r="F66" s="18" t="n"/>
+      <c r="G66" s="18" t="n"/>
+      <c r="H66" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I64" s="18" t="n"/>
-      <c r="J64" s="18" t="n"/>
-      <c r="K64" s="18" t="n"/>
-      <c r="L64" s="18" t="n"/>
-      <c r="M64" s="18" t="n"/>
-      <c r="N64" s="18" t="n"/>
-      <c r="O64" s="18" t="n"/>
+      <c r="I66" s="18" t="n"/>
+      <c r="J66" s="18" t="n"/>
+      <c r="K66" s="18" t="n"/>
+      <c r="L66" s="18" t="n"/>
+      <c r="M66" s="18" t="n"/>
+      <c r="N66" s="18" t="n"/>
+      <c r="O66" s="18" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="11" t="inlineStr">
+        <is>
+          <t>▸ West / Other  (1)</t>
+        </is>
+      </c>
+      <c r="B67" s="12" t="n"/>
+      <c r="C67" s="12" t="n"/>
+      <c r="D67" s="12" t="n"/>
+      <c r="E67" s="12" t="n"/>
+      <c r="F67" s="12" t="n"/>
+      <c r="G67" s="12" t="n"/>
+      <c r="H67" s="12" t="n"/>
+      <c r="I67" s="12" t="n"/>
+      <c r="J67" s="12" t="n"/>
+      <c r="K67" s="12" t="n"/>
+      <c r="L67" s="12" t="n"/>
+      <c r="M67" s="12" t="n"/>
+      <c r="N67" s="12" t="n"/>
+      <c r="O67" s="12" t="n"/>
+    </row>
+    <row r="68" outlineLevel="1">
+      <c r="A68" s="13" t="inlineStr">
+        <is>
+          <t>West / Other</t>
+        </is>
+      </c>
+      <c r="B68" s="14" t="inlineStr">
+        <is>
+          <t>National salad concept liquidation – full contents of 63 fast-casual restaurants (AZ/TX/OK/NV)</t>
+        </is>
+      </c>
+      <c r="C68" s="13" t="inlineStr">
+        <is>
+          <t>restaurant chain liquidation</t>
+        </is>
+      </c>
+      <c r="D68" s="13" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="E68" s="13" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="F68" s="13" t="n">
+        <v>2307</v>
+      </c>
+      <c r="G68" s="13" t="inlineStr">
+        <is>
+          <t>Online auctions, dates TBD</t>
+        </is>
+      </c>
+      <c r="H68" s="15" t="n"/>
+      <c r="I68" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="J68" s="13" t="inlineStr"/>
+      <c r="K68" s="13" t="inlineStr">
+        <is>
+          <t>RestaurantEquipment.bid (TAGeX)</t>
+        </is>
+      </c>
+      <c r="L68" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M68" s="13" t="inlineStr"/>
+      <c r="N68" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O68" s="14" t="inlineStr">
+        <is>
+          <t>Rolling market-by-market auctions, none live yet (Phoenix metro 30 locations, DFW 14, Tucson 6, Houston 5, plus OK/NV). Pickup on site at each restaurant. Pinned at Phoenix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — West / Other</t>
+        </is>
+      </c>
+      <c r="B69" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C69" s="18" t="n"/>
+      <c r="D69" s="18" t="n"/>
+      <c r="E69" s="18" t="n"/>
+      <c r="F69" s="18" t="n"/>
+      <c r="G69" s="18" t="n"/>
+      <c r="H69" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" s="18" t="n"/>
+      <c r="J69" s="18" t="n"/>
+      <c r="K69" s="18" t="n"/>
+      <c r="L69" s="18" t="n"/>
+      <c r="M69" s="18" t="n"/>
+      <c r="N69" s="18" t="n"/>
+      <c r="O69" s="18" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O64"/>
+  <autoFilter ref="A1:O69"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N32" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId22"/>
@@ -21797,14 +22245,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N43" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N44" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N45" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N48" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N51" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N52" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N46" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N47" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N50" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N53" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N56" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N59" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N60" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N63" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N54" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N55" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N58" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N61" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N62" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N65" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N68" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove flower/upholstery shop listings
</commit_message>
<xml_diff>
--- a/lot_recon.xlsx
+++ b/lot_recon.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wolf New'!$A$1:$O$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Wolf Used'!$A$1:$O$188</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Wolf Unclear'!$A$1:$O$40</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$69</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 2026-10-18 13:59 ET</t>
+          <t>Last updated: 2026-10-18 14:02 ET</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Active listings: 286 · Removed: 2</t>
+          <t>Active listings: 284 · Removed: 2</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
         <v>159696</v>
       </c>
       <c r="D8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F8" t="n">
         <v>34</v>
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>0</v>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C13" s="7" t="n">
         <v>975650.08</v>
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C23" t="n">
         <v>1</v>
@@ -1004,7 +1004,7 @@
         <v>4</v>
       </c>
       <c r="G23" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H23" s="6" t="n">
         <v>62163</v>
@@ -2727,9 +2727,9 @@
           <t>HiBid (Auctionfuel)</t>
         </is>
       </c>
-      <c r="L30" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+      <c r="L30" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M30" s="13" t="inlineStr"/>
@@ -18610,7 +18610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O71"/>
+  <dimension ref="A1:O69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -19851,7 +19851,7 @@
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>▸ CT / Hudson Valley  (6)</t>
+          <t>▸ CT / Hudson Valley  (4)</t>
         </is>
       </c>
       <c r="B25" s="12" t="n"/>
@@ -19940,47 +19940,47 @@
       </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>Flower shop liquidation – whole inventory: vases, containers, baskets, ribbon/wrap, floral foam, seasonal decor, gift items</t>
+          <t>Major Intl Chain Surplus – 225 lots commercial refrigeration/kitchen (True, Traulsen, Hobart, Blodgett, Taylor)</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>commercial surplus</t>
         </is>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>Prospect</t>
+          <t>Pleasant Valley</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>119</v>
+        <v>157</v>
       </c>
       <c r="G27" s="13" t="inlineStr">
         <is>
-          <t>$10,000 (whole lot); will split or bundle</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H27" s="15" t="n"/>
-      <c r="I27" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="J27" s="13" t="inlineStr"/>
+      <c r="I27" s="13" t="inlineStr"/>
+      <c r="J27" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-20 02:00 PM ET</t>
+        </is>
+      </c>
       <c r="K27" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
-        </is>
-      </c>
-      <c r="L27" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>Adams / BidWrangler</t>
+        </is>
+      </c>
+      <c r="L27" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M27" s="13" t="inlineStr"/>
@@ -19991,7 +19991,7 @@
       </c>
       <c r="O27" s="14" t="inlineStr">
         <is>
-          <t>Pickup only. Off-category (floral/gift), FYI only.</t>
+          <t>Tested and new units.</t>
         </is>
       </c>
     </row>
@@ -20003,17 +20003,17 @@
       </c>
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>Upholstery shop closing – tools, supplies, Singer 95-1 industrial sewing machine, everything for sale</t>
+          <t>Café/bakery liquidation – Traulsen, Vulcan ovens, mixers, Hobart slicer (~74 lots)</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>West Haven</t>
+          <t>Greenwich</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
@@ -20022,23 +20022,23 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>125</v>
+        <v>164</v>
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>Varies by item ($1 placeholder)</t>
+          <t>Live auction + webcast</t>
         </is>
       </c>
       <c r="H28" s="15" t="n"/>
-      <c r="I28" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="J28" s="13" t="inlineStr"/>
+      <c r="I28" s="13" t="inlineStr"/>
+      <c r="J28" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-21 06:00 PM ET</t>
+        </is>
+      </c>
       <c r="K28" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>Best Buy Auctioneers / AuctionGuide</t>
         </is>
       </c>
       <c r="L28" s="13" t="inlineStr">
@@ -20054,7 +20054,7 @@
       </c>
       <c r="O28" s="14" t="inlineStr">
         <is>
-          <t>Posted 9/13, updated 10/16. Off-category, FYI only.</t>
+          <t>Oct 21; start time not captured (placeholder 6 PM).</t>
         </is>
       </c>
     </row>
@@ -20066,17 +20066,17 @@
       </c>
       <c r="B29" s="14" t="inlineStr">
         <is>
-          <t>Major Intl Chain Surplus – 225 lots commercial refrigeration/kitchen (True, Traulsen, Hobart, Blodgett, Taylor)</t>
+          <t>BJ's Wholesale closeout – racking, forklifts, Hobart</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>commercial surplus</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>Pleasant Valley</t>
+          <t>Rotterdam</t>
         </is>
       </c>
       <c r="E29" s="13" t="inlineStr">
@@ -20085,7 +20085,7 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="G29" s="13" t="inlineStr">
         <is>
@@ -20096,17 +20096,17 @@
       <c r="I29" s="13" t="inlineStr"/>
       <c r="J29" s="13" t="inlineStr">
         <is>
-          <t>2026-10-20 02:00 PM ET</t>
+          <t>2026-11-10 10:00 AM ET</t>
         </is>
       </c>
       <c r="K29" s="13" t="inlineStr">
         <is>
-          <t>Adams / BidWrangler</t>
-        </is>
-      </c>
-      <c r="L29" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L29" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M29" s="13" t="inlineStr"/>
@@ -20117,183 +20117,191 @@
       </c>
       <c r="O29" s="14" t="inlineStr">
         <is>
-          <t>Tested and new units.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" outlineLevel="1">
-      <c r="A30" s="13" t="inlineStr">
-        <is>
-          <t>CT / Hudson Valley</t>
-        </is>
-      </c>
-      <c r="B30" s="14" t="inlineStr">
-        <is>
-          <t>Café/bakery liquidation – Traulsen, Vulcan ovens, mixers, Hobart slicer (~74 lots)</t>
-        </is>
-      </c>
-      <c r="C30" s="13" t="inlineStr">
-        <is>
-          <t>restaurant</t>
-        </is>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
-        <is>
-          <t>Greenwich</t>
-        </is>
-      </c>
-      <c r="E30" s="13" t="inlineStr">
-        <is>
-          <t>CT</t>
-        </is>
-      </c>
-      <c r="F30" s="13" t="n">
-        <v>164</v>
-      </c>
-      <c r="G30" s="13" t="inlineStr">
-        <is>
-          <t>Live auction + webcast</t>
-        </is>
-      </c>
-      <c r="H30" s="15" t="n"/>
-      <c r="I30" s="13" t="inlineStr"/>
-      <c r="J30" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-21 06:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K30" s="13" t="inlineStr">
-        <is>
-          <t>Best Buy Auctioneers / AuctionGuide</t>
-        </is>
-      </c>
-      <c r="L30" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M30" s="13" t="inlineStr"/>
-      <c r="N30" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O30" s="14" t="inlineStr">
-        <is>
-          <t>Oct 21; start time not captured (placeholder 6 PM).</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" outlineLevel="1">
-      <c r="A31" s="13" t="inlineStr">
-        <is>
-          <t>CT / Hudson Valley</t>
-        </is>
-      </c>
-      <c r="B31" s="14" t="inlineStr">
-        <is>
-          <t>BJ's Wholesale closeout – racking, forklifts, Hobart</t>
-        </is>
-      </c>
-      <c r="C31" s="13" t="inlineStr">
-        <is>
-          <t>store closing</t>
-        </is>
-      </c>
-      <c r="D31" s="13" t="inlineStr">
-        <is>
-          <t>Rotterdam</t>
-        </is>
-      </c>
-      <c r="E31" s="13" t="inlineStr">
+          <t>Closes from Nov 10 10 AM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — CT / Hudson Valley</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>4 item(s)</t>
+        </is>
+      </c>
+      <c r="C30" s="18" t="n"/>
+      <c r="D30" s="18" t="n"/>
+      <c r="E30" s="18" t="n"/>
+      <c r="F30" s="18" t="n"/>
+      <c r="G30" s="18" t="n"/>
+      <c r="H30" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="18" t="n"/>
+      <c r="J30" s="18" t="n"/>
+      <c r="K30" s="18" t="n"/>
+      <c r="L30" s="18" t="n"/>
+      <c r="M30" s="18" t="n"/>
+      <c r="N30" s="18" t="n"/>
+      <c r="O30" s="18" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>▸ NYC / Long Island / NJ  (16)</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="n"/>
+      <c r="C31" s="12" t="n"/>
+      <c r="D31" s="12" t="n"/>
+      <c r="E31" s="12" t="n"/>
+      <c r="F31" s="12" t="n"/>
+      <c r="G31" s="12" t="n"/>
+      <c r="H31" s="12" t="n"/>
+      <c r="I31" s="12" t="n"/>
+      <c r="J31" s="12" t="n"/>
+      <c r="K31" s="12" t="n"/>
+      <c r="L31" s="12" t="n"/>
+      <c r="M31" s="12" t="n"/>
+      <c r="N31" s="12" t="n"/>
+      <c r="O31" s="12" t="n"/>
+    </row>
+    <row r="32" outlineLevel="1">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>Japanese BBQ &amp; bar – ~47 lots: Turbo Air, Hoshizaki ice machine, Pitco, Beverage-Air</t>
+        </is>
+      </c>
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>restaurant closing</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="E32" s="13" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
       </c>
-      <c r="F31" s="13" t="n">
-        <v>168</v>
-      </c>
-      <c r="G31" s="13" t="inlineStr">
-        <is>
-          <t>Online auction</t>
-        </is>
-      </c>
-      <c r="H31" s="15" t="n"/>
-      <c r="I31" s="13" t="inlineStr"/>
-      <c r="J31" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-10 10:00 AM ET</t>
-        </is>
-      </c>
-      <c r="K31" s="13" t="inlineStr">
-        <is>
-          <t>Grafe Auction</t>
-        </is>
-      </c>
-      <c r="L31" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M31" s="13" t="inlineStr"/>
-      <c r="N31" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O31" s="14" t="inlineStr">
-        <is>
-          <t>Closes from Nov 10 10 AM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — CT / Hudson Valley</t>
-        </is>
-      </c>
-      <c r="B32" s="17" t="inlineStr">
-        <is>
-          <t>6 item(s)</t>
-        </is>
-      </c>
-      <c r="C32" s="18" t="n"/>
-      <c r="D32" s="18" t="n"/>
-      <c r="E32" s="18" t="n"/>
-      <c r="F32" s="18" t="n"/>
-      <c r="G32" s="18" t="n"/>
-      <c r="H32" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" s="18" t="n"/>
-      <c r="J32" s="18" t="n"/>
-      <c r="K32" s="18" t="n"/>
-      <c r="L32" s="18" t="n"/>
-      <c r="M32" s="18" t="n"/>
-      <c r="N32" s="18" t="n"/>
-      <c r="O32" s="18" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="11" t="inlineStr">
-        <is>
-          <t>▸ NYC / Long Island / NJ  (16)</t>
-        </is>
-      </c>
-      <c r="B33" s="12" t="n"/>
-      <c r="C33" s="12" t="n"/>
-      <c r="D33" s="12" t="n"/>
-      <c r="E33" s="12" t="n"/>
-      <c r="F33" s="12" t="n"/>
-      <c r="G33" s="12" t="n"/>
-      <c r="H33" s="12" t="n"/>
-      <c r="I33" s="12" t="n"/>
-      <c r="J33" s="12" t="n"/>
-      <c r="K33" s="12" t="n"/>
-      <c r="L33" s="12" t="n"/>
-      <c r="M33" s="12" t="n"/>
-      <c r="N33" s="12" t="n"/>
-      <c r="O33" s="12" t="n"/>
+      <c r="F32" s="13" t="n">
+        <v>191</v>
+      </c>
+      <c r="G32" s="13" t="inlineStr">
+        <is>
+          <t>Live + webcast, 18% BP + 3%</t>
+        </is>
+      </c>
+      <c r="H32" s="15" t="n"/>
+      <c r="I32" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J32" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-21 04:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K32" s="13" t="inlineStr">
+        <is>
+          <t>HiBid (Best Buy Auctioneers)</t>
+        </is>
+      </c>
+      <c r="L32" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M32" s="13" t="inlineStr"/>
+      <c r="N32" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O32" s="14" t="inlineStr">
+        <is>
+          <t>Wed Oct 21 4 PM. NYC 10013.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" outlineLevel="1">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Corporate caterer – Alto-Shaam, new boxed Avantco rice cookers &amp; Cadco oven, Perlick, MerryChef</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>auction</t>
+        </is>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t>Jersey City</t>
+        </is>
+      </c>
+      <c r="E33" s="13" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="F33" s="13" t="n">
+        <v>193</v>
+      </c>
+      <c r="G33" s="13" t="inlineStr">
+        <is>
+          <t>Live + webcast, 18% BP + 3%</t>
+        </is>
+      </c>
+      <c r="H33" s="15" t="n"/>
+      <c r="I33" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="J33" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-22 02:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K33" s="13" t="inlineStr">
+        <is>
+          <t>HiBid (Best Buy Auctioneers)</t>
+        </is>
+      </c>
+      <c r="L33" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M33" s="13" t="inlineStr"/>
+      <c r="N33" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O33" s="14" t="inlineStr">
+        <is>
+          <t>Thu Oct 22 2 PM.</t>
+        </is>
+      </c>
     </row>
     <row r="34" outlineLevel="1">
       <c r="A34" s="13" t="inlineStr">
@@ -20303,46 +20311,42 @@
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>Japanese BBQ &amp; bar – ~47 lots: Turbo Air, Hoshizaki ice machine, Pitco, Beverage-Air</t>
+          <t>Tools / plumbing / MRO supply inventory – Hilti/DeWalt/Milwaukee, fittings, heat pumps</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>restaurant closing</t>
+          <t>inventory</t>
         </is>
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Riverdale</t>
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H34" s="15" t="n"/>
-      <c r="I34" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
+      <c r="I34" s="13" t="inlineStr"/>
       <c r="J34" s="13" t="inlineStr">
         <is>
-          <t>2026-10-21 04:00 PM ET</t>
+          <t>2026-10-30 11:00 AM ET</t>
         </is>
       </c>
       <c r="K34" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>A.J. Willner</t>
         </is>
       </c>
       <c r="L34" s="13" t="inlineStr">
@@ -20358,7 +20362,7 @@
       </c>
       <c r="O34" s="14" t="inlineStr">
         <is>
-          <t>Wed Oct 21 4 PM. NYC 10013.</t>
+          <t>Bulk resale inventory.</t>
         </is>
       </c>
     </row>
@@ -20370,17 +20374,17 @@
       </c>
       <c r="B35" s="14" t="inlineStr">
         <is>
-          <t>Corporate caterer – Alto-Shaam, new boxed Avantco rice cookers &amp; Cadco oven, Perlick, MerryChef</t>
+          <t>Ice cream + cookie franchise equipment – Taylor soft-serve, Atosa, Blodgett</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D35" s="13" t="inlineStr">
         <is>
-          <t>Jersey City</t>
+          <t>Riverdale</t>
         </is>
       </c>
       <c r="E35" s="13" t="inlineStr">
@@ -20389,27 +20393,23 @@
         </is>
       </c>
       <c r="F35" s="13" t="n">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="G35" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H35" s="15" t="n"/>
-      <c r="I35" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
+      <c r="I35" s="13" t="inlineStr"/>
       <c r="J35" s="13" t="inlineStr">
         <is>
-          <t>2026-10-22 02:00 PM ET</t>
+          <t>2026-11-05 11:00 AM ET</t>
         </is>
       </c>
       <c r="K35" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>A.J. Willner</t>
         </is>
       </c>
       <c r="L35" s="13" t="inlineStr">
@@ -20425,7 +20425,7 @@
       </c>
       <c r="O35" s="14" t="inlineStr">
         <is>
-          <t>Thu Oct 22 2 PM.</t>
+          <t>Resellable units.</t>
         </is>
       </c>
     </row>
@@ -20437,47 +20437,51 @@
       </c>
       <c r="B36" s="14" t="inlineStr">
         <is>
-          <t>Tools / plumbing / MRO supply inventory – Hilti/DeWalt/Milwaukee, fittings, heat pumps</t>
+          <t>Like-new restaurant – steam tables, Coldline, Cleveland cook-and-hold, fryers, True freezers</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
-          <t>Riverdale</t>
+          <t>Staten Island</t>
         </is>
       </c>
       <c r="E36" s="13" t="inlineStr">
         <is>
-          <t>NJ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="G36" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H36" s="15" t="n"/>
-      <c r="I36" s="13" t="inlineStr"/>
+      <c r="I36" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="J36" s="13" t="inlineStr">
         <is>
-          <t>2026-10-30 11:00 AM ET</t>
+          <t>2026-10-19 01:00 PM ET</t>
         </is>
       </c>
       <c r="K36" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
-        </is>
-      </c>
-      <c r="L36" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
+        </is>
+      </c>
+      <c r="L36" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M36" s="13" t="inlineStr"/>
@@ -20488,7 +20492,7 @@
       </c>
       <c r="O36" s="14" t="inlineStr">
         <is>
-          <t>Bulk resale inventory.</t>
+          <t>"Short notice" auction Mon Oct 19 1 PM.</t>
         </is>
       </c>
     </row>
@@ -20500,17 +20504,17 @@
       </c>
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>Ice cream + cookie franchise equipment – Taylor soft-serve, Atosa, Blodgett</t>
+          <t>Major food-service caterer – new-in-box True reach-ins, Beverage-Air, TurboChef, Resfab ventless fryer</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">
         <is>
-          <t>Riverdale</t>
+          <t>Parsippany</t>
         </is>
       </c>
       <c r="E37" s="13" t="inlineStr">
@@ -20519,23 +20523,27 @@
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>196</v>
+        <v>206</v>
       </c>
       <c r="G37" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H37" s="15" t="n"/>
-      <c r="I37" s="13" t="inlineStr"/>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
       <c r="J37" s="13" t="inlineStr">
         <is>
-          <t>2026-11-05 11:00 AM ET</t>
+          <t>2026-11-03 02:00 PM ET</t>
         </is>
       </c>
       <c r="K37" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
       <c r="L37" s="13" t="inlineStr">
@@ -20551,7 +20559,7 @@
       </c>
       <c r="O37" s="14" t="inlineStr">
         <is>
-          <t>Resellable units.</t>
+          <t>Tue Nov 3 2 PM, checkout Nov 4.</t>
         </is>
       </c>
     </row>
@@ -20563,46 +20571,42 @@
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>Like-new restaurant – steam tables, Coldline, Cleveland cook-and-hold, fryers, True freezers</t>
+          <t>Serpico's Pizzeria (lost lease) – Bari ovens, walk-in, Hobart 60qt, Vulcan range</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
         <is>
-          <t>Staten Island</t>
+          <t>Allenhurst</t>
         </is>
       </c>
       <c r="E38" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>No-reserve online auction</t>
         </is>
       </c>
       <c r="H38" s="15" t="n"/>
-      <c r="I38" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
+      <c r="I38" s="13" t="inlineStr"/>
       <c r="J38" s="13" t="inlineStr">
         <is>
-          <t>2026-10-19 01:00 PM ET</t>
+          <t>2026-10-21 11:00 AM ET</t>
         </is>
       </c>
       <c r="K38" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>Peter Costanzo / EstateSales.net</t>
         </is>
       </c>
       <c r="L38" s="20" t="inlineStr">
@@ -20618,7 +20622,7 @@
       </c>
       <c r="O38" s="14" t="inlineStr">
         <is>
-          <t>"Short notice" auction Mon Oct 19 1 PM.</t>
+          <t>Absolute / no reserve.</t>
         </is>
       </c>
     </row>
@@ -20630,17 +20634,17 @@
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>Major food-service caterer – new-in-box True reach-ins, Beverage-Air, TurboChef, Resfab ventless fryer</t>
+          <t>Altitude Trampoline Park liquidation – partial: Atosa, TurboChef, stainless</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>facility contents</t>
         </is>
       </c>
       <c r="D39" s="13" t="inlineStr">
         <is>
-          <t>Parsippany</t>
+          <t>Iselin</t>
         </is>
       </c>
       <c r="E39" s="13" t="inlineStr">
@@ -20649,32 +20653,28 @@
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="G39" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H39" s="15" t="n"/>
-      <c r="I39" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
+      <c r="I39" s="13" t="inlineStr"/>
       <c r="J39" s="13" t="inlineStr">
         <is>
-          <t>2026-11-03 02:00 PM ET</t>
+          <t>2026-10-21 11:00 AM ET</t>
         </is>
       </c>
       <c r="K39" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
-        </is>
-      </c>
-      <c r="L39" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>A.J. Willner</t>
+        </is>
+      </c>
+      <c r="L39" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M39" s="13" t="inlineStr"/>
@@ -20685,7 +20685,7 @@
       </c>
       <c r="O39" s="14" t="inlineStr">
         <is>
-          <t>Tue Nov 3 2 PM, checkout Nov 4.</t>
+          <t>Some kitchen gear only.</t>
         </is>
       </c>
     </row>
@@ -20697,17 +20697,17 @@
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>Serpico's Pizzeria (lost lease) – Bari ovens, walk-in, Hobart 60qt, Vulcan range</t>
+          <t>Restaurant / pizzeria (contents not described)</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>restaurant closing</t>
         </is>
       </c>
       <c r="D40" s="13" t="inlineStr">
         <is>
-          <t>Allenhurst</t>
+          <t>Berkeley Heights</t>
         </is>
       </c>
       <c r="E40" s="13" t="inlineStr">
@@ -20716,23 +20716,27 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t>No-reserve online auction</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H40" s="15" t="n"/>
-      <c r="I40" s="13" t="inlineStr"/>
+      <c r="I40" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
       <c r="J40" s="13" t="inlineStr">
         <is>
-          <t>2026-10-21 11:00 AM ET</t>
+          <t>2026-10-20 02:00 PM ET</t>
         </is>
       </c>
       <c r="K40" s="13" t="inlineStr">
         <is>
-          <t>Peter Costanzo / EstateSales.net</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
       <c r="L40" s="20" t="inlineStr">
@@ -20748,7 +20752,7 @@
       </c>
       <c r="O40" s="14" t="inlineStr">
         <is>
-          <t>Absolute / no reserve.</t>
+          <t>Tue Oct 20 2 PM. No item description on page.</t>
         </is>
       </c>
     </row>
@@ -20760,17 +20764,17 @@
       </c>
       <c r="B41" s="14" t="inlineStr">
         <is>
-          <t>Altitude Trampoline Park liquidation – partial: Atosa, TurboChef, stainless</t>
+          <t>New modular concession kitchens (warehouseman's lien) – 5 units, CaptiveAire hoods, new Ovention/Turbo Air</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
-          <t>facility contents</t>
+          <t>lien sale</t>
         </is>
       </c>
       <c r="D41" s="13" t="inlineStr">
         <is>
-          <t>Iselin</t>
+          <t>Edison</t>
         </is>
       </c>
       <c r="E41" s="13" t="inlineStr">
@@ -20779,28 +20783,24 @@
         </is>
       </c>
       <c r="F41" s="13" t="n">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="G41" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Online auction, $2K load-out fee</t>
         </is>
       </c>
       <c r="H41" s="15" t="n"/>
       <c r="I41" s="13" t="inlineStr"/>
-      <c r="J41" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-21 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="J41" s="13" t="inlineStr"/>
       <c r="K41" s="13" t="inlineStr">
         <is>
           <t>A.J. Willner</t>
         </is>
       </c>
-      <c r="L41" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+      <c r="L41" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M41" s="13" t="inlineStr"/>
@@ -20811,7 +20811,7 @@
       </c>
       <c r="O41" s="14" t="inlineStr">
         <is>
-          <t>Some kitchen gear only.</t>
+          <t>&gt;$100K new. Close date not captured.</t>
         </is>
       </c>
     </row>
@@ -20823,17 +20823,17 @@
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>Restaurant / pizzeria (contents not described)</t>
+          <t>Brand-new &amp; scratch-and-dent kitchen/home appliances – ~185 lots (Thermador, GE Café, Miele, Wolf speed oven, Viking, Bosch…)</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>restaurant closing</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D42" s="13" t="inlineStr">
         <is>
-          <t>Berkeley Heights</t>
+          <t>Edison</t>
         </is>
       </c>
       <c r="E42" s="13" t="inlineStr">
@@ -20842,22 +20842,22 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>Live + HiBid webcast, 18% BP + 3% card</t>
         </is>
       </c>
       <c r="H42" s="15" t="n"/>
       <c r="I42" s="13" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="J42" s="13" t="inlineStr">
         <is>
-          <t>2026-10-20 02:00 PM ET</t>
+          <t>2026-10-25 01:00 PM ET</t>
         </is>
       </c>
       <c r="K42" s="13" t="inlineStr">
@@ -20865,12 +20865,16 @@
           <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
-      <c r="L42" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
-        </is>
-      </c>
-      <c r="M42" s="13" t="inlineStr"/>
+      <c r="L42" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M42" s="21" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
       <c r="N42" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -20878,7 +20882,7 @@
       </c>
       <c r="O42" s="14" t="inlineStr">
         <is>
-          <t>Tue Oct 20 2 PM. No item description on page.</t>
+          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale.</t>
         </is>
       </c>
     </row>
@@ -20890,17 +20894,17 @@
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>New modular concession kitchens (warehouseman's lien) – 5 units, CaptiveAire hoods, new Ovention/Turbo Air</t>
+          <t>Party City (Ch. 11) store – fixtures + party merchandise inventory</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
         <is>
-          <t>lien sale</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D43" s="13" t="inlineStr">
         <is>
-          <t>Edison</t>
+          <t>East Brunswick</t>
         </is>
       </c>
       <c r="E43" s="13" t="inlineStr">
@@ -20909,16 +20913,20 @@
         </is>
       </c>
       <c r="F43" s="13" t="n">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="G43" s="13" t="inlineStr">
         <is>
-          <t>Online auction, $2K load-out fee</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H43" s="15" t="n"/>
       <c r="I43" s="13" t="inlineStr"/>
-      <c r="J43" s="13" t="inlineStr"/>
+      <c r="J43" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-03 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K43" s="13" t="inlineStr">
         <is>
           <t>A.J. Willner</t>
@@ -20937,7 +20945,7 @@
       </c>
       <c r="O43" s="14" t="inlineStr">
         <is>
-          <t>&gt;$100K new. Close date not captured.</t>
+          <t>Store inventory.</t>
         </is>
       </c>
     </row>
@@ -20949,17 +20957,17 @@
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>Brand-new &amp; scratch-and-dent kitchen/home appliances – ~185 lots (Thermador, GE Café, Miele, Wolf speed oven, Viking, Bosch…)</t>
+          <t>High-end deli (contents not described)</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>restaurant closing</t>
         </is>
       </c>
       <c r="D44" s="13" t="inlineStr">
         <is>
-          <t>Edison</t>
+          <t>Manalapan Township</t>
         </is>
       </c>
       <c r="E44" s="13" t="inlineStr">
@@ -20968,22 +20976,22 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>Live + HiBid webcast, 18% BP + 3% card</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H44" s="15" t="n"/>
       <c r="I44" s="13" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="J44" s="13" t="inlineStr">
         <is>
-          <t>2026-10-25 01:00 PM ET</t>
+          <t>2026-10-19 04:00 PM ET</t>
         </is>
       </c>
       <c r="K44" s="13" t="inlineStr">
@@ -20991,16 +20999,12 @@
           <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
-      <c r="L44" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M44" s="21" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
+      <c r="L44" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M44" s="13" t="inlineStr"/>
       <c r="N44" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -21008,7 +21012,7 @@
       </c>
       <c r="O44" s="14" t="inlineStr">
         <is>
-          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale.</t>
+          <t>Mon Oct 19 4 PM. No item description on page.</t>
         </is>
       </c>
     </row>
@@ -21020,17 +21024,17 @@
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>Party City (Ch. 11) store – fixtures + party merchandise inventory</t>
+          <t>Wren Kitchens showroom closing – JennAir/Café/KitchenAid/GE Profile appliances + display kitchens</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>showroom closing</t>
         </is>
       </c>
       <c r="D45" s="13" t="inlineStr">
         <is>
-          <t>East Brunswick</t>
+          <t>Lawrenceville</t>
         </is>
       </c>
       <c r="E45" s="13" t="inlineStr">
@@ -21039,23 +21043,23 @@
         </is>
       </c>
       <c r="F45" s="13" t="n">
-        <v>220</v>
+        <v>239</v>
       </c>
       <c r="G45" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Online auction, 18% BP</t>
         </is>
       </c>
       <c r="H45" s="15" t="n"/>
       <c r="I45" s="13" t="inlineStr"/>
       <c r="J45" s="13" t="inlineStr">
         <is>
-          <t>2026-11-03 11:00 AM ET</t>
+          <t>2026-10-27 09:00 AM ET</t>
         </is>
       </c>
       <c r="K45" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
+          <t>Grafe Auction</t>
         </is>
       </c>
       <c r="L45" s="13" t="inlineStr">
@@ -21071,7 +21075,7 @@
       </c>
       <c r="O45" s="14" t="inlineStr">
         <is>
-          <t>Store inventory.</t>
+          <t>Premium floor-model appliances; lots close from Oct 27 9 AM.</t>
         </is>
       </c>
     </row>
@@ -21083,17 +21087,17 @@
       </c>
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>High-end deli (contents not described)</t>
+          <t>Milwaukee / Walmart / hardware store mega auction pt 3</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>restaurant closing</t>
+          <t>inventory</t>
         </is>
       </c>
       <c r="D46" s="13" t="inlineStr">
         <is>
-          <t>Manalapan Township</t>
+          <t>Mount Holly</t>
         </is>
       </c>
       <c r="E46" s="13" t="inlineStr">
@@ -21102,27 +21106,23 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>223</v>
+        <v>254</v>
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>HiBid online auction</t>
         </is>
       </c>
       <c r="H46" s="15" t="n"/>
-      <c r="I46" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
+      <c r="I46" s="13" t="inlineStr"/>
       <c r="J46" s="13" t="inlineStr">
         <is>
-          <t>2026-10-19 04:00 PM ET</t>
+          <t>2026-10-19 06:00 PM ET</t>
         </is>
       </c>
       <c r="K46" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>HiBid</t>
         </is>
       </c>
       <c r="L46" s="20" t="inlineStr">
@@ -21138,7 +21138,7 @@
       </c>
       <c r="O46" s="14" t="inlineStr">
         <is>
-          <t>Mon Oct 19 4 PM. No item description on page.</t>
+          <t>Close Oct 18 or 19 6 PM (later used).</t>
         </is>
       </c>
     </row>
@@ -21150,7 +21150,7 @@
       </c>
       <c r="B47" s="14" t="inlineStr">
         <is>
-          <t>Wren Kitchens showroom closing – JennAir/Café/KitchenAid/GE Profile appliances + display kitchens</t>
+          <t>Wren Kitchens showroom closing – GE/Whirlpool/KitchenAid/Café incl. NIB Café range + 35 kitchens</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
@@ -21160,7 +21160,7 @@
       </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>Lawrenceville</t>
+          <t>Cherry Hill</t>
         </is>
       </c>
       <c r="E47" s="13" t="inlineStr">
@@ -21169,18 +21169,18 @@
         </is>
       </c>
       <c r="F47" s="13" t="n">
-        <v>239</v>
+        <v>266</v>
       </c>
       <c r="G47" s="13" t="inlineStr">
         <is>
-          <t>Online auction, 18% BP</t>
+          <t>Online auction, openers ~$0.50</t>
         </is>
       </c>
       <c r="H47" s="15" t="n"/>
       <c r="I47" s="13" t="inlineStr"/>
       <c r="J47" s="13" t="inlineStr">
         <is>
-          <t>2026-10-27 09:00 AM ET</t>
+          <t>2026-11-02 11:00 AM ET</t>
         </is>
       </c>
       <c r="K47" s="13" t="inlineStr">
@@ -21201,294 +21201,294 @@
       </c>
       <c r="O47" s="14" t="inlineStr">
         <is>
-          <t>Premium floor-model appliances; lots close from Oct 27 9 AM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" outlineLevel="1">
-      <c r="A48" s="13" t="inlineStr">
-        <is>
-          <t>NYC / Long Island / NJ</t>
-        </is>
-      </c>
-      <c r="B48" s="14" t="inlineStr">
-        <is>
-          <t>Milwaukee / Walmart / hardware store mega auction pt 3</t>
-        </is>
-      </c>
-      <c r="C48" s="13" t="inlineStr">
-        <is>
-          <t>inventory</t>
-        </is>
-      </c>
-      <c r="D48" s="13" t="inlineStr">
-        <is>
-          <t>Mount Holly</t>
-        </is>
-      </c>
-      <c r="E48" s="13" t="inlineStr">
-        <is>
-          <t>NJ</t>
-        </is>
-      </c>
-      <c r="F48" s="13" t="n">
-        <v>254</v>
-      </c>
-      <c r="G48" s="13" t="inlineStr">
+          <t>Lots close from Nov 2 11 AM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B48" s="17" t="inlineStr">
+        <is>
+          <t>16 item(s)</t>
+        </is>
+      </c>
+      <c r="C48" s="18" t="n"/>
+      <c r="D48" s="18" t="n"/>
+      <c r="E48" s="18" t="n"/>
+      <c r="F48" s="18" t="n"/>
+      <c r="G48" s="18" t="n"/>
+      <c r="H48" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" s="18" t="n"/>
+      <c r="J48" s="18" t="n"/>
+      <c r="K48" s="18" t="n"/>
+      <c r="L48" s="18" t="n"/>
+      <c r="M48" s="18" t="n"/>
+      <c r="N48" s="18" t="n"/>
+      <c r="O48" s="18" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="11" t="inlineStr">
+        <is>
+          <t>▸ Eastern PA / Mid-Atlantic  (1)</t>
+        </is>
+      </c>
+      <c r="B49" s="12" t="n"/>
+      <c r="C49" s="12" t="n"/>
+      <c r="D49" s="12" t="n"/>
+      <c r="E49" s="12" t="n"/>
+      <c r="F49" s="12" t="n"/>
+      <c r="G49" s="12" t="n"/>
+      <c r="H49" s="12" t="n"/>
+      <c r="I49" s="12" t="n"/>
+      <c r="J49" s="12" t="n"/>
+      <c r="K49" s="12" t="n"/>
+      <c r="L49" s="12" t="n"/>
+      <c r="M49" s="12" t="n"/>
+      <c r="N49" s="12" t="n"/>
+      <c r="O49" s="12" t="n"/>
+    </row>
+    <row r="50" outlineLevel="1">
+      <c r="A50" s="13" t="inlineStr">
+        <is>
+          <t>Eastern PA / Mid-Atlantic</t>
+        </is>
+      </c>
+      <c r="B50" s="14" t="inlineStr">
+        <is>
+          <t>October restaurant consignment – Hobart, Rational, True + NEW scratch-and-dent Migali/Avantco</t>
+        </is>
+      </c>
+      <c r="C50" s="13" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D50" s="13" t="inlineStr">
+        <is>
+          <t>Harrisburg</t>
+        </is>
+      </c>
+      <c r="E50" s="13" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="F50" s="13" t="n">
+        <v>340</v>
+      </c>
+      <c r="G50" s="13" t="inlineStr">
+        <is>
+          <t>Online auction, 15% BP, ships $55/pallet</t>
+        </is>
+      </c>
+      <c r="H50" s="15" t="n"/>
+      <c r="I50" s="13" t="inlineStr"/>
+      <c r="J50" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-21 11:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K50" s="13" t="inlineStr">
+        <is>
+          <t>Restaurant Auction Co</t>
+        </is>
+      </c>
+      <c r="L50" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M50" s="13" t="inlineStr"/>
+      <c r="N50" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O50" s="14" t="inlineStr">
+        <is>
+          <t>Closes Oct 21 10 or 11 AM (later used). Shippable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Eastern PA / Mid-Atlantic</t>
+        </is>
+      </c>
+      <c r="B51" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C51" s="18" t="n"/>
+      <c r="D51" s="18" t="n"/>
+      <c r="E51" s="18" t="n"/>
+      <c r="F51" s="18" t="n"/>
+      <c r="G51" s="18" t="n"/>
+      <c r="H51" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" s="18" t="n"/>
+      <c r="J51" s="18" t="n"/>
+      <c r="K51" s="18" t="n"/>
+      <c r="L51" s="18" t="n"/>
+      <c r="M51" s="18" t="n"/>
+      <c r="N51" s="18" t="n"/>
+      <c r="O51" s="18" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="11" t="inlineStr">
+        <is>
+          <t>▸ Upstate / Western NY  (3)</t>
+        </is>
+      </c>
+      <c r="B52" s="12" t="n"/>
+      <c r="C52" s="12" t="n"/>
+      <c r="D52" s="12" t="n"/>
+      <c r="E52" s="12" t="n"/>
+      <c r="F52" s="12" t="n"/>
+      <c r="G52" s="12" t="n"/>
+      <c r="H52" s="12" t="n"/>
+      <c r="I52" s="12" t="n"/>
+      <c r="J52" s="12" t="n"/>
+      <c r="K52" s="12" t="n"/>
+      <c r="L52" s="12" t="n"/>
+      <c r="M52" s="12" t="n"/>
+      <c r="N52" s="12" t="n"/>
+      <c r="O52" s="12" t="n"/>
+    </row>
+    <row r="53" outlineLevel="1">
+      <c r="A53" s="13" t="inlineStr">
+        <is>
+          <t>Upstate / Western NY</t>
+        </is>
+      </c>
+      <c r="B53" s="14" t="inlineStr">
+        <is>
+          <t>Former Taco Del Mar – stainless, warmers, walk-in panels</t>
+        </is>
+      </c>
+      <c r="C53" s="13" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D53" s="13" t="inlineStr">
+        <is>
+          <t>Watson</t>
+        </is>
+      </c>
+      <c r="E53" s="13" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="F53" s="13" t="n">
+        <v>260</v>
+      </c>
+      <c r="G53" s="13" t="inlineStr">
         <is>
           <t>HiBid online auction</t>
         </is>
       </c>
-      <c r="H48" s="15" t="n"/>
-      <c r="I48" s="13" t="inlineStr"/>
-      <c r="J48" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-19 06:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K48" s="13" t="inlineStr">
-        <is>
-          <t>HiBid</t>
-        </is>
-      </c>
-      <c r="L48" s="20" t="inlineStr">
+      <c r="H53" s="15" t="n"/>
+      <c r="I53" s="13" t="inlineStr"/>
+      <c r="J53" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-20 06:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K53" s="13" t="inlineStr">
+        <is>
+          <t>Adirondack Asset / HiBid</t>
+        </is>
+      </c>
+      <c r="L53" s="20" t="inlineStr">
         <is>
           <t>ENDING SOON</t>
         </is>
       </c>
-      <c r="M48" s="13" t="inlineStr"/>
-      <c r="N48" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O48" s="14" t="inlineStr">
-        <is>
-          <t>Close Oct 18 or 19 6 PM (later used).</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" outlineLevel="1">
-      <c r="A49" s="13" t="inlineStr">
-        <is>
-          <t>NYC / Long Island / NJ</t>
-        </is>
-      </c>
-      <c r="B49" s="14" t="inlineStr">
-        <is>
-          <t>Wren Kitchens showroom closing – GE/Whirlpool/KitchenAid/Café incl. NIB Café range + 35 kitchens</t>
-        </is>
-      </c>
-      <c r="C49" s="13" t="inlineStr">
-        <is>
-          <t>showroom closing</t>
-        </is>
-      </c>
-      <c r="D49" s="13" t="inlineStr">
-        <is>
-          <t>Cherry Hill</t>
-        </is>
-      </c>
-      <c r="E49" s="13" t="inlineStr">
-        <is>
-          <t>NJ</t>
-        </is>
-      </c>
-      <c r="F49" s="13" t="n">
-        <v>266</v>
-      </c>
-      <c r="G49" s="13" t="inlineStr">
-        <is>
-          <t>Online auction, openers ~$0.50</t>
-        </is>
-      </c>
-      <c r="H49" s="15" t="n"/>
-      <c r="I49" s="13" t="inlineStr"/>
-      <c r="J49" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-02 11:00 AM ET</t>
-        </is>
-      </c>
-      <c r="K49" s="13" t="inlineStr">
-        <is>
-          <t>Grafe Auction</t>
-        </is>
-      </c>
-      <c r="L49" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M49" s="13" t="inlineStr"/>
-      <c r="N49" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O49" s="14" t="inlineStr">
-        <is>
-          <t>Lots close from Nov 2 11 AM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — NYC / Long Island / NJ</t>
-        </is>
-      </c>
-      <c r="B50" s="17" t="inlineStr">
-        <is>
-          <t>16 item(s)</t>
-        </is>
-      </c>
-      <c r="C50" s="18" t="n"/>
-      <c r="D50" s="18" t="n"/>
-      <c r="E50" s="18" t="n"/>
-      <c r="F50" s="18" t="n"/>
-      <c r="G50" s="18" t="n"/>
-      <c r="H50" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I50" s="18" t="n"/>
-      <c r="J50" s="18" t="n"/>
-      <c r="K50" s="18" t="n"/>
-      <c r="L50" s="18" t="n"/>
-      <c r="M50" s="18" t="n"/>
-      <c r="N50" s="18" t="n"/>
-      <c r="O50" s="18" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="11" t="inlineStr">
-        <is>
-          <t>▸ Eastern PA / Mid-Atlantic  (1)</t>
-        </is>
-      </c>
-      <c r="B51" s="12" t="n"/>
-      <c r="C51" s="12" t="n"/>
-      <c r="D51" s="12" t="n"/>
-      <c r="E51" s="12" t="n"/>
-      <c r="F51" s="12" t="n"/>
-      <c r="G51" s="12" t="n"/>
-      <c r="H51" s="12" t="n"/>
-      <c r="I51" s="12" t="n"/>
-      <c r="J51" s="12" t="n"/>
-      <c r="K51" s="12" t="n"/>
-      <c r="L51" s="12" t="n"/>
-      <c r="M51" s="12" t="n"/>
-      <c r="N51" s="12" t="n"/>
-      <c r="O51" s="12" t="n"/>
-    </row>
-    <row r="52" outlineLevel="1">
-      <c r="A52" s="13" t="inlineStr">
-        <is>
-          <t>Eastern PA / Mid-Atlantic</t>
-        </is>
-      </c>
-      <c r="B52" s="14" t="inlineStr">
-        <is>
-          <t>October restaurant consignment – Hobart, Rational, True + NEW scratch-and-dent Migali/Avantco</t>
-        </is>
-      </c>
-      <c r="C52" s="13" t="inlineStr">
+      <c r="M53" s="13" t="inlineStr"/>
+      <c r="N53" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O53" s="14" t="inlineStr">
+        <is>
+          <t>Small lot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" outlineLevel="1">
+      <c r="A54" s="13" t="inlineStr">
+        <is>
+          <t>Upstate / Western NY</t>
+        </is>
+      </c>
+      <c r="B54" s="14" t="inlineStr">
+        <is>
+          <t>Closed restaurant – coolers, fridges, prep tables</t>
+        </is>
+      </c>
+      <c r="C54" s="13" t="inlineStr">
         <is>
           <t>restaurant</t>
         </is>
       </c>
-      <c r="D52" s="13" t="inlineStr">
-        <is>
-          <t>Harrisburg</t>
-        </is>
-      </c>
-      <c r="E52" s="13" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="F52" s="13" t="n">
-        <v>340</v>
-      </c>
-      <c r="G52" s="13" t="inlineStr">
-        <is>
-          <t>Online auction, 15% BP, ships $55/pallet</t>
-        </is>
-      </c>
-      <c r="H52" s="15" t="n"/>
-      <c r="I52" s="13" t="inlineStr"/>
-      <c r="J52" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-21 11:00 AM ET</t>
-        </is>
-      </c>
-      <c r="K52" s="13" t="inlineStr">
-        <is>
-          <t>Restaurant Auction Co</t>
-        </is>
-      </c>
-      <c r="L52" s="20" t="inlineStr">
+      <c r="D54" s="13" t="inlineStr">
+        <is>
+          <t>Palmyra</t>
+        </is>
+      </c>
+      <c r="E54" s="13" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="F54" s="13" t="n">
+        <v>333</v>
+      </c>
+      <c r="G54" s="13" t="inlineStr">
+        <is>
+          <t>HiBid, 15% BP</t>
+        </is>
+      </c>
+      <c r="H54" s="15" t="n"/>
+      <c r="I54" s="13" t="inlineStr"/>
+      <c r="J54" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K54" s="13" t="inlineStr">
+        <is>
+          <t>Reynolds Auction Co / HiBid</t>
+        </is>
+      </c>
+      <c r="L54" s="20" t="inlineStr">
         <is>
           <t>ENDING SOON</t>
         </is>
       </c>
-      <c r="M52" s="13" t="inlineStr"/>
-      <c r="N52" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O52" s="14" t="inlineStr">
-        <is>
-          <t>Closes Oct 21 10 or 11 AM (later used). Shippable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Eastern PA / Mid-Atlantic</t>
-        </is>
-      </c>
-      <c r="B53" s="17" t="inlineStr">
-        <is>
-          <t>1 item(s)</t>
-        </is>
-      </c>
-      <c r="C53" s="18" t="n"/>
-      <c r="D53" s="18" t="n"/>
-      <c r="E53" s="18" t="n"/>
-      <c r="F53" s="18" t="n"/>
-      <c r="G53" s="18" t="n"/>
-      <c r="H53" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I53" s="18" t="n"/>
-      <c r="J53" s="18" t="n"/>
-      <c r="K53" s="18" t="n"/>
-      <c r="L53" s="18" t="n"/>
-      <c r="M53" s="18" t="n"/>
-      <c r="N53" s="18" t="n"/>
-      <c r="O53" s="18" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="11" t="inlineStr">
-        <is>
-          <t>▸ Upstate / Western NY  (3)</t>
-        </is>
-      </c>
-      <c r="B54" s="12" t="n"/>
-      <c r="C54" s="12" t="n"/>
-      <c r="D54" s="12" t="n"/>
-      <c r="E54" s="12" t="n"/>
-      <c r="F54" s="12" t="n"/>
-      <c r="G54" s="12" t="n"/>
-      <c r="H54" s="12" t="n"/>
-      <c r="I54" s="12" t="n"/>
-      <c r="J54" s="12" t="n"/>
-      <c r="K54" s="12" t="n"/>
-      <c r="L54" s="12" t="n"/>
-      <c r="M54" s="12" t="n"/>
-      <c r="N54" s="12" t="n"/>
-      <c r="O54" s="12" t="n"/>
+      <c r="M54" s="13" t="inlineStr"/>
+      <c r="N54" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O54" s="14" t="inlineStr">
+        <is>
+          <t>No new out-of-state bidders. Small.</t>
+        </is>
+      </c>
     </row>
     <row r="55" outlineLevel="1">
       <c r="A55" s="13" t="inlineStr">
@@ -21498,7 +21498,7 @@
       </c>
       <c r="B55" s="14" t="inlineStr">
         <is>
-          <t>Former Taco Del Mar – stainless, warmers, walk-in panels</t>
+          <t>Restaurant &amp; fitness equipment</t>
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr">
@@ -21508,7 +21508,7 @@
       </c>
       <c r="D55" s="13" t="inlineStr">
         <is>
-          <t>Watson</t>
+          <t>Williamsville</t>
         </is>
       </c>
       <c r="E55" s="13" t="inlineStr">
@@ -21517,28 +21517,28 @@
         </is>
       </c>
       <c r="F55" s="13" t="n">
-        <v>260</v>
+        <v>408</v>
       </c>
       <c r="G55" s="13" t="inlineStr">
         <is>
-          <t>HiBid online auction</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H55" s="15" t="n"/>
       <c r="I55" s="13" t="inlineStr"/>
       <c r="J55" s="13" t="inlineStr">
         <is>
-          <t>2026-10-20 06:00 PM ET</t>
+          <t>2026-10-26 07:30 PM ET</t>
         </is>
       </c>
       <c r="K55" s="13" t="inlineStr">
         <is>
-          <t>Adirondack Asset / HiBid</t>
-        </is>
-      </c>
-      <c r="L55" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>Cash Auctions</t>
+        </is>
+      </c>
+      <c r="L55" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M55" s="13" t="inlineStr"/>
@@ -21549,672 +21549,546 @@
       </c>
       <c r="O55" s="14" t="inlineStr">
         <is>
-          <t>Small lot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" outlineLevel="1">
-      <c r="A56" s="13" t="inlineStr">
-        <is>
-          <t>Upstate / Western NY</t>
-        </is>
-      </c>
-      <c r="B56" s="14" t="inlineStr">
-        <is>
-          <t>Closed restaurant – coolers, fridges, prep tables</t>
-        </is>
-      </c>
-      <c r="C56" s="13" t="inlineStr">
-        <is>
-          <t>restaurant</t>
-        </is>
-      </c>
-      <c r="D56" s="13" t="inlineStr">
-        <is>
-          <t>Palmyra</t>
-        </is>
-      </c>
-      <c r="E56" s="13" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="F56" s="13" t="n">
-        <v>333</v>
-      </c>
-      <c r="G56" s="13" t="inlineStr">
-        <is>
-          <t>HiBid, 15% BP</t>
-        </is>
-      </c>
-      <c r="H56" s="15" t="n"/>
-      <c r="I56" s="13" t="inlineStr"/>
-      <c r="J56" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-19 07:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K56" s="13" t="inlineStr">
-        <is>
-          <t>Reynolds Auction Co / HiBid</t>
-        </is>
-      </c>
-      <c r="L56" s="20" t="inlineStr">
+          <t>Lots not reviewed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Upstate / Western NY</t>
+        </is>
+      </c>
+      <c r="B56" s="17" t="inlineStr">
+        <is>
+          <t>3 item(s)</t>
+        </is>
+      </c>
+      <c r="C56" s="18" t="n"/>
+      <c r="D56" s="18" t="n"/>
+      <c r="E56" s="18" t="n"/>
+      <c r="F56" s="18" t="n"/>
+      <c r="G56" s="18" t="n"/>
+      <c r="H56" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="18" t="n"/>
+      <c r="J56" s="18" t="n"/>
+      <c r="K56" s="18" t="n"/>
+      <c r="L56" s="18" t="n"/>
+      <c r="M56" s="18" t="n"/>
+      <c r="N56" s="18" t="n"/>
+      <c r="O56" s="18" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="11" t="inlineStr">
+        <is>
+          <t>▸ Virginia  (1)</t>
+        </is>
+      </c>
+      <c r="B57" s="12" t="n"/>
+      <c r="C57" s="12" t="n"/>
+      <c r="D57" s="12" t="n"/>
+      <c r="E57" s="12" t="n"/>
+      <c r="F57" s="12" t="n"/>
+      <c r="G57" s="12" t="n"/>
+      <c r="H57" s="12" t="n"/>
+      <c r="I57" s="12" t="n"/>
+      <c r="J57" s="12" t="n"/>
+      <c r="K57" s="12" t="n"/>
+      <c r="L57" s="12" t="n"/>
+      <c r="M57" s="12" t="n"/>
+      <c r="N57" s="12" t="n"/>
+      <c r="O57" s="12" t="n"/>
+    </row>
+    <row r="58" outlineLevel="1">
+      <c r="A58" s="13" t="inlineStr">
+        <is>
+          <t>Virginia</t>
+        </is>
+      </c>
+      <c r="B58" s="14" t="inlineStr">
+        <is>
+          <t>Haynes Furniture / The Dump – 12 stores closing (furniture, mattresses)</t>
+        </is>
+      </c>
+      <c r="C58" s="13" t="inlineStr">
+        <is>
+          <t>retail GOB</t>
+        </is>
+      </c>
+      <c r="D58" s="13" t="inlineStr">
+        <is>
+          <t>Virginia Beach</t>
+        </is>
+      </c>
+      <c r="E58" s="13" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="F58" s="13" t="n">
+        <v>456</v>
+      </c>
+      <c r="G58" s="13" t="inlineStr">
+        <is>
+          <t>Retail GOB markdowns</t>
+        </is>
+      </c>
+      <c r="H58" s="15" t="n"/>
+      <c r="I58" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="J58" s="13" t="inlineStr"/>
+      <c r="K58" s="13" t="inlineStr">
+        <is>
+          <t>SB360 (PR Newswire)</t>
+        </is>
+      </c>
+      <c r="L58" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M58" s="13" t="inlineStr"/>
+      <c r="N58" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O58" s="14" t="inlineStr">
+        <is>
+          <t>Posted Oct 8. Multi-state (VA/AZ/GA/IL/TX); pinned at Virginia Beach. Home goods only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Virginia</t>
+        </is>
+      </c>
+      <c r="B59" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C59" s="18" t="n"/>
+      <c r="D59" s="18" t="n"/>
+      <c r="E59" s="18" t="n"/>
+      <c r="F59" s="18" t="n"/>
+      <c r="G59" s="18" t="n"/>
+      <c r="H59" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" s="18" t="n"/>
+      <c r="J59" s="18" t="n"/>
+      <c r="K59" s="18" t="n"/>
+      <c r="L59" s="18" t="n"/>
+      <c r="M59" s="18" t="n"/>
+      <c r="N59" s="18" t="n"/>
+      <c r="O59" s="18" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t>▸ Midwest  (2)</t>
+        </is>
+      </c>
+      <c r="B60" s="12" t="n"/>
+      <c r="C60" s="12" t="n"/>
+      <c r="D60" s="12" t="n"/>
+      <c r="E60" s="12" t="n"/>
+      <c r="F60" s="12" t="n"/>
+      <c r="G60" s="12" t="n"/>
+      <c r="H60" s="12" t="n"/>
+      <c r="I60" s="12" t="n"/>
+      <c r="J60" s="12" t="n"/>
+      <c r="K60" s="12" t="n"/>
+      <c r="L60" s="12" t="n"/>
+      <c r="M60" s="12" t="n"/>
+      <c r="N60" s="12" t="n"/>
+      <c r="O60" s="12" t="n"/>
+    </row>
+    <row r="61" outlineLevel="1">
+      <c r="A61" s="13" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="B61" s="14" t="inlineStr">
+        <is>
+          <t>Freshway Market whole-grocery liquidation – refrigeration racks, cases, walk-ins, generator</t>
+        </is>
+      </c>
+      <c r="C61" s="13" t="inlineStr">
+        <is>
+          <t>store closing</t>
+        </is>
+      </c>
+      <c r="D61" s="13" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="E61" s="13" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="F61" s="13" t="n">
+        <v>862</v>
+      </c>
+      <c r="G61" s="13" t="inlineStr">
+        <is>
+          <t>Online auction</t>
+        </is>
+      </c>
+      <c r="H61" s="15" t="n"/>
+      <c r="I61" s="13" t="inlineStr"/>
+      <c r="J61" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-20 11:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K61" s="13" t="inlineStr">
+        <is>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L61" s="20" t="inlineStr">
         <is>
           <t>ENDING SOON</t>
         </is>
       </c>
-      <c r="M56" s="13" t="inlineStr"/>
-      <c r="N56" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O56" s="14" t="inlineStr">
-        <is>
-          <t>No new out-of-state bidders. Small.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" outlineLevel="1">
-      <c r="A57" s="13" t="inlineStr">
-        <is>
-          <t>Upstate / Western NY</t>
-        </is>
-      </c>
-      <c r="B57" s="14" t="inlineStr">
-        <is>
-          <t>Restaurant &amp; fitness equipment</t>
-        </is>
-      </c>
-      <c r="C57" s="13" t="inlineStr">
-        <is>
-          <t>restaurant</t>
-        </is>
-      </c>
-      <c r="D57" s="13" t="inlineStr">
-        <is>
-          <t>Williamsville</t>
-        </is>
-      </c>
-      <c r="E57" s="13" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="F57" s="13" t="n">
-        <v>408</v>
-      </c>
-      <c r="G57" s="13" t="inlineStr">
+      <c r="M61" s="13" t="inlineStr"/>
+      <c r="N61" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O61" s="14" t="inlineStr">
+        <is>
+          <t>Closes from Oct 20 10 AM CDT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" outlineLevel="1">
+      <c r="A62" s="13" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="B62" s="14" t="inlineStr">
+        <is>
+          <t>American Sale – total liquidation, all 7 stores (pools, hot tubs, grills, holiday decor)</t>
+        </is>
+      </c>
+      <c r="C62" s="13" t="inlineStr">
+        <is>
+          <t>retail GOB</t>
+        </is>
+      </c>
+      <c r="D62" s="13" t="inlineStr">
+        <is>
+          <t>Chicagoland</t>
+        </is>
+      </c>
+      <c r="E62" s="13" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="F62" s="13" t="n">
+        <v>876</v>
+      </c>
+      <c r="G62" s="13" t="inlineStr">
+        <is>
+          <t>Retail GOB, up to 70% off</t>
+        </is>
+      </c>
+      <c r="H62" s="15" t="n"/>
+      <c r="I62" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="J62" s="13" t="inlineStr"/>
+      <c r="K62" s="13" t="inlineStr">
+        <is>
+          <t>Tiger Group (PR Newswire)</t>
+        </is>
+      </c>
+      <c r="L62" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M62" s="13" t="inlineStr"/>
+      <c r="N62" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O62" s="14" t="inlineStr">
+        <is>
+          <t>Posted Oct 15. Watch for a bulk/fixture auction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Midwest</t>
+        </is>
+      </c>
+      <c r="B63" s="17" t="inlineStr">
+        <is>
+          <t>2 item(s)</t>
+        </is>
+      </c>
+      <c r="C63" s="18" t="n"/>
+      <c r="D63" s="18" t="n"/>
+      <c r="E63" s="18" t="n"/>
+      <c r="F63" s="18" t="n"/>
+      <c r="G63" s="18" t="n"/>
+      <c r="H63" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" s="18" t="n"/>
+      <c r="J63" s="18" t="n"/>
+      <c r="K63" s="18" t="n"/>
+      <c r="L63" s="18" t="n"/>
+      <c r="M63" s="18" t="n"/>
+      <c r="N63" s="18" t="n"/>
+      <c r="O63" s="18" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="inlineStr">
+        <is>
+          <t>▸ Texas / South Central  (1)</t>
+        </is>
+      </c>
+      <c r="B64" s="12" t="n"/>
+      <c r="C64" s="12" t="n"/>
+      <c r="D64" s="12" t="n"/>
+      <c r="E64" s="12" t="n"/>
+      <c r="F64" s="12" t="n"/>
+      <c r="G64" s="12" t="n"/>
+      <c r="H64" s="12" t="n"/>
+      <c r="I64" s="12" t="n"/>
+      <c r="J64" s="12" t="n"/>
+      <c r="K64" s="12" t="n"/>
+      <c r="L64" s="12" t="n"/>
+      <c r="M64" s="12" t="n"/>
+      <c r="N64" s="12" t="n"/>
+      <c r="O64" s="12" t="n"/>
+    </row>
+    <row r="65" outlineLevel="1">
+      <c r="A65" s="13" t="inlineStr">
+        <is>
+          <t>Texas / South Central</t>
+        </is>
+      </c>
+      <c r="B65" s="14" t="inlineStr">
+        <is>
+          <t>Southwest beverage distributor surplus – mostly unused: 16 True merchandisers, 75 Bunn brewers, 100+ micro-market kiosks</t>
+        </is>
+      </c>
+      <c r="C65" s="13" t="inlineStr">
+        <is>
+          <t>distributor surplus</t>
+        </is>
+      </c>
+      <c r="D65" s="13" t="inlineStr">
+        <is>
+          <t>Mesquite</t>
+        </is>
+      </c>
+      <c r="E65" s="13" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="F65" s="13" t="n">
+        <v>1547</v>
+      </c>
+      <c r="G65" s="13" t="inlineStr">
         <is>
           <t>Online auction</t>
         </is>
       </c>
-      <c r="H57" s="15" t="n"/>
-      <c r="I57" s="13" t="inlineStr"/>
-      <c r="J57" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26 07:30 PM ET</t>
-        </is>
-      </c>
-      <c r="K57" s="13" t="inlineStr">
-        <is>
-          <t>Cash Auctions</t>
-        </is>
-      </c>
-      <c r="L57" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M57" s="13" t="inlineStr"/>
-      <c r="N57" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O57" s="14" t="inlineStr">
-        <is>
-          <t>Lots not reviewed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Upstate / Western NY</t>
-        </is>
-      </c>
-      <c r="B58" s="17" t="inlineStr">
-        <is>
-          <t>3 item(s)</t>
-        </is>
-      </c>
-      <c r="C58" s="18" t="n"/>
-      <c r="D58" s="18" t="n"/>
-      <c r="E58" s="18" t="n"/>
-      <c r="F58" s="18" t="n"/>
-      <c r="G58" s="18" t="n"/>
-      <c r="H58" s="19" t="n">
+      <c r="H65" s="15" t="n"/>
+      <c r="I65" s="13" t="inlineStr"/>
+      <c r="J65" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-13 11:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K65" s="13" t="inlineStr">
+        <is>
+          <t>Heritage Global Partners</t>
+        </is>
+      </c>
+      <c r="L65" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M65" s="13" t="inlineStr"/>
+      <c r="N65" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O65" s="14" t="inlineStr">
+        <is>
+          <t>Near-new appliances, resell by unit. Nov 13 10 AM CST.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Texas / South Central</t>
+        </is>
+      </c>
+      <c r="B66" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C66" s="18" t="n"/>
+      <c r="D66" s="18" t="n"/>
+      <c r="E66" s="18" t="n"/>
+      <c r="F66" s="18" t="n"/>
+      <c r="G66" s="18" t="n"/>
+      <c r="H66" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I58" s="18" t="n"/>
-      <c r="J58" s="18" t="n"/>
-      <c r="K58" s="18" t="n"/>
-      <c r="L58" s="18" t="n"/>
-      <c r="M58" s="18" t="n"/>
-      <c r="N58" s="18" t="n"/>
-      <c r="O58" s="18" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="11" t="inlineStr">
-        <is>
-          <t>▸ Virginia  (1)</t>
-        </is>
-      </c>
-      <c r="B59" s="12" t="n"/>
-      <c r="C59" s="12" t="n"/>
-      <c r="D59" s="12" t="n"/>
-      <c r="E59" s="12" t="n"/>
-      <c r="F59" s="12" t="n"/>
-      <c r="G59" s="12" t="n"/>
-      <c r="H59" s="12" t="n"/>
-      <c r="I59" s="12" t="n"/>
-      <c r="J59" s="12" t="n"/>
-      <c r="K59" s="12" t="n"/>
-      <c r="L59" s="12" t="n"/>
-      <c r="M59" s="12" t="n"/>
-      <c r="N59" s="12" t="n"/>
-      <c r="O59" s="12" t="n"/>
-    </row>
-    <row r="60" outlineLevel="1">
-      <c r="A60" s="13" t="inlineStr">
-        <is>
-          <t>Virginia</t>
-        </is>
-      </c>
-      <c r="B60" s="14" t="inlineStr">
-        <is>
-          <t>Haynes Furniture / The Dump – 12 stores closing (furniture, mattresses)</t>
-        </is>
-      </c>
-      <c r="C60" s="13" t="inlineStr">
-        <is>
-          <t>retail GOB</t>
-        </is>
-      </c>
-      <c r="D60" s="13" t="inlineStr">
-        <is>
-          <t>Virginia Beach</t>
-        </is>
-      </c>
-      <c r="E60" s="13" t="inlineStr">
-        <is>
-          <t>VA</t>
-        </is>
-      </c>
-      <c r="F60" s="13" t="n">
-        <v>456</v>
-      </c>
-      <c r="G60" s="13" t="inlineStr">
-        <is>
-          <t>Retail GOB markdowns</t>
-        </is>
-      </c>
-      <c r="H60" s="15" t="n"/>
-      <c r="I60" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="J60" s="13" t="inlineStr"/>
-      <c r="K60" s="13" t="inlineStr">
-        <is>
-          <t>SB360 (PR Newswire)</t>
-        </is>
-      </c>
-      <c r="L60" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M60" s="13" t="inlineStr"/>
-      <c r="N60" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O60" s="14" t="inlineStr">
-        <is>
-          <t>Posted Oct 8. Multi-state (VA/AZ/GA/IL/TX); pinned at Virginia Beach. Home goods only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Virginia</t>
-        </is>
-      </c>
-      <c r="B61" s="17" t="inlineStr">
+      <c r="I66" s="18" t="n"/>
+      <c r="J66" s="18" t="n"/>
+      <c r="K66" s="18" t="n"/>
+      <c r="L66" s="18" t="n"/>
+      <c r="M66" s="18" t="n"/>
+      <c r="N66" s="18" t="n"/>
+      <c r="O66" s="18" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="11" t="inlineStr">
+        <is>
+          <t>▸ West / Other  (1)</t>
+        </is>
+      </c>
+      <c r="B67" s="12" t="n"/>
+      <c r="C67" s="12" t="n"/>
+      <c r="D67" s="12" t="n"/>
+      <c r="E67" s="12" t="n"/>
+      <c r="F67" s="12" t="n"/>
+      <c r="G67" s="12" t="n"/>
+      <c r="H67" s="12" t="n"/>
+      <c r="I67" s="12" t="n"/>
+      <c r="J67" s="12" t="n"/>
+      <c r="K67" s="12" t="n"/>
+      <c r="L67" s="12" t="n"/>
+      <c r="M67" s="12" t="n"/>
+      <c r="N67" s="12" t="n"/>
+      <c r="O67" s="12" t="n"/>
+    </row>
+    <row r="68" outlineLevel="1">
+      <c r="A68" s="13" t="inlineStr">
+        <is>
+          <t>West / Other</t>
+        </is>
+      </c>
+      <c r="B68" s="14" t="inlineStr">
+        <is>
+          <t>National salad concept liquidation – full contents of 63 fast-casual restaurants (AZ/TX/OK/NV)</t>
+        </is>
+      </c>
+      <c r="C68" s="13" t="inlineStr">
+        <is>
+          <t>restaurant chain liquidation</t>
+        </is>
+      </c>
+      <c r="D68" s="13" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="E68" s="13" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="F68" s="13" t="n">
+        <v>2307</v>
+      </c>
+      <c r="G68" s="13" t="inlineStr">
+        <is>
+          <t>Online auctions, dates TBD</t>
+        </is>
+      </c>
+      <c r="H68" s="15" t="n"/>
+      <c r="I68" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="J68" s="13" t="inlineStr"/>
+      <c r="K68" s="13" t="inlineStr">
+        <is>
+          <t>RestaurantEquipment.bid (TAGeX)</t>
+        </is>
+      </c>
+      <c r="L68" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M68" s="13" t="inlineStr"/>
+      <c r="N68" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O68" s="14" t="inlineStr">
+        <is>
+          <t>Rolling market-by-market auctions, none live yet (Phoenix metro 30 locations, DFW 14, Tucson 6, Houston 5, plus OK/NV). Pickup on site at each restaurant. Pinned at Phoenix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — West / Other</t>
+        </is>
+      </c>
+      <c r="B69" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C61" s="18" t="n"/>
-      <c r="D61" s="18" t="n"/>
-      <c r="E61" s="18" t="n"/>
-      <c r="F61" s="18" t="n"/>
-      <c r="G61" s="18" t="n"/>
-      <c r="H61" s="19" t="n">
+      <c r="C69" s="18" t="n"/>
+      <c r="D69" s="18" t="n"/>
+      <c r="E69" s="18" t="n"/>
+      <c r="F69" s="18" t="n"/>
+      <c r="G69" s="18" t="n"/>
+      <c r="H69" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I61" s="18" t="n"/>
-      <c r="J61" s="18" t="n"/>
-      <c r="K61" s="18" t="n"/>
-      <c r="L61" s="18" t="n"/>
-      <c r="M61" s="18" t="n"/>
-      <c r="N61" s="18" t="n"/>
-      <c r="O61" s="18" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="11" t="inlineStr">
-        <is>
-          <t>▸ Midwest  (2)</t>
-        </is>
-      </c>
-      <c r="B62" s="12" t="n"/>
-      <c r="C62" s="12" t="n"/>
-      <c r="D62" s="12" t="n"/>
-      <c r="E62" s="12" t="n"/>
-      <c r="F62" s="12" t="n"/>
-      <c r="G62" s="12" t="n"/>
-      <c r="H62" s="12" t="n"/>
-      <c r="I62" s="12" t="n"/>
-      <c r="J62" s="12" t="n"/>
-      <c r="K62" s="12" t="n"/>
-      <c r="L62" s="12" t="n"/>
-      <c r="M62" s="12" t="n"/>
-      <c r="N62" s="12" t="n"/>
-      <c r="O62" s="12" t="n"/>
-    </row>
-    <row r="63" outlineLevel="1">
-      <c r="A63" s="13" t="inlineStr">
-        <is>
-          <t>Midwest</t>
-        </is>
-      </c>
-      <c r="B63" s="14" t="inlineStr">
-        <is>
-          <t>Freshway Market whole-grocery liquidation – refrigeration racks, cases, walk-ins, generator</t>
-        </is>
-      </c>
-      <c r="C63" s="13" t="inlineStr">
-        <is>
-          <t>store closing</t>
-        </is>
-      </c>
-      <c r="D63" s="13" t="inlineStr">
-        <is>
-          <t>Chicago</t>
-        </is>
-      </c>
-      <c r="E63" s="13" t="inlineStr">
-        <is>
-          <t>IL</t>
-        </is>
-      </c>
-      <c r="F63" s="13" t="n">
-        <v>862</v>
-      </c>
-      <c r="G63" s="13" t="inlineStr">
-        <is>
-          <t>Online auction</t>
-        </is>
-      </c>
-      <c r="H63" s="15" t="n"/>
-      <c r="I63" s="13" t="inlineStr"/>
-      <c r="J63" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-20 11:00 AM ET</t>
-        </is>
-      </c>
-      <c r="K63" s="13" t="inlineStr">
-        <is>
-          <t>Grafe Auction</t>
-        </is>
-      </c>
-      <c r="L63" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
-        </is>
-      </c>
-      <c r="M63" s="13" t="inlineStr"/>
-      <c r="N63" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O63" s="14" t="inlineStr">
-        <is>
-          <t>Closes from Oct 20 10 AM CDT.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" outlineLevel="1">
-      <c r="A64" s="13" t="inlineStr">
-        <is>
-          <t>Midwest</t>
-        </is>
-      </c>
-      <c r="B64" s="14" t="inlineStr">
-        <is>
-          <t>American Sale – total liquidation, all 7 stores (pools, hot tubs, grills, holiday decor)</t>
-        </is>
-      </c>
-      <c r="C64" s="13" t="inlineStr">
-        <is>
-          <t>retail GOB</t>
-        </is>
-      </c>
-      <c r="D64" s="13" t="inlineStr">
-        <is>
-          <t>Chicagoland</t>
-        </is>
-      </c>
-      <c r="E64" s="13" t="inlineStr">
-        <is>
-          <t>IL</t>
-        </is>
-      </c>
-      <c r="F64" s="13" t="n">
-        <v>876</v>
-      </c>
-      <c r="G64" s="13" t="inlineStr">
-        <is>
-          <t>Retail GOB, up to 70% off</t>
-        </is>
-      </c>
-      <c r="H64" s="15" t="n"/>
-      <c r="I64" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="J64" s="13" t="inlineStr"/>
-      <c r="K64" s="13" t="inlineStr">
-        <is>
-          <t>Tiger Group (PR Newswire)</t>
-        </is>
-      </c>
-      <c r="L64" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M64" s="13" t="inlineStr"/>
-      <c r="N64" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O64" s="14" t="inlineStr">
-        <is>
-          <t>Posted Oct 15. Watch for a bulk/fixture auction.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Midwest</t>
-        </is>
-      </c>
-      <c r="B65" s="17" t="inlineStr">
-        <is>
-          <t>2 item(s)</t>
-        </is>
-      </c>
-      <c r="C65" s="18" t="n"/>
-      <c r="D65" s="18" t="n"/>
-      <c r="E65" s="18" t="n"/>
-      <c r="F65" s="18" t="n"/>
-      <c r="G65" s="18" t="n"/>
-      <c r="H65" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I65" s="18" t="n"/>
-      <c r="J65" s="18" t="n"/>
-      <c r="K65" s="18" t="n"/>
-      <c r="L65" s="18" t="n"/>
-      <c r="M65" s="18" t="n"/>
-      <c r="N65" s="18" t="n"/>
-      <c r="O65" s="18" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="11" t="inlineStr">
-        <is>
-          <t>▸ Texas / South Central  (1)</t>
-        </is>
-      </c>
-      <c r="B66" s="12" t="n"/>
-      <c r="C66" s="12" t="n"/>
-      <c r="D66" s="12" t="n"/>
-      <c r="E66" s="12" t="n"/>
-      <c r="F66" s="12" t="n"/>
-      <c r="G66" s="12" t="n"/>
-      <c r="H66" s="12" t="n"/>
-      <c r="I66" s="12" t="n"/>
-      <c r="J66" s="12" t="n"/>
-      <c r="K66" s="12" t="n"/>
-      <c r="L66" s="12" t="n"/>
-      <c r="M66" s="12" t="n"/>
-      <c r="N66" s="12" t="n"/>
-      <c r="O66" s="12" t="n"/>
-    </row>
-    <row r="67" outlineLevel="1">
-      <c r="A67" s="13" t="inlineStr">
-        <is>
-          <t>Texas / South Central</t>
-        </is>
-      </c>
-      <c r="B67" s="14" t="inlineStr">
-        <is>
-          <t>Southwest beverage distributor surplus – mostly unused: 16 True merchandisers, 75 Bunn brewers, 100+ micro-market kiosks</t>
-        </is>
-      </c>
-      <c r="C67" s="13" t="inlineStr">
-        <is>
-          <t>distributor surplus</t>
-        </is>
-      </c>
-      <c r="D67" s="13" t="inlineStr">
-        <is>
-          <t>Mesquite</t>
-        </is>
-      </c>
-      <c r="E67" s="13" t="inlineStr">
-        <is>
-          <t>TX</t>
-        </is>
-      </c>
-      <c r="F67" s="13" t="n">
-        <v>1547</v>
-      </c>
-      <c r="G67" s="13" t="inlineStr">
-        <is>
-          <t>Online auction</t>
-        </is>
-      </c>
-      <c r="H67" s="15" t="n"/>
-      <c r="I67" s="13" t="inlineStr"/>
-      <c r="J67" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-13 11:00 AM ET</t>
-        </is>
-      </c>
-      <c r="K67" s="13" t="inlineStr">
-        <is>
-          <t>Heritage Global Partners</t>
-        </is>
-      </c>
-      <c r="L67" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M67" s="13" t="inlineStr"/>
-      <c r="N67" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O67" s="14" t="inlineStr">
-        <is>
-          <t>Near-new appliances, resell by unit. Nov 13 10 AM CST.</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Texas / South Central</t>
-        </is>
-      </c>
-      <c r="B68" s="17" t="inlineStr">
-        <is>
-          <t>1 item(s)</t>
-        </is>
-      </c>
-      <c r="C68" s="18" t="n"/>
-      <c r="D68" s="18" t="n"/>
-      <c r="E68" s="18" t="n"/>
-      <c r="F68" s="18" t="n"/>
-      <c r="G68" s="18" t="n"/>
-      <c r="H68" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I68" s="18" t="n"/>
-      <c r="J68" s="18" t="n"/>
-      <c r="K68" s="18" t="n"/>
-      <c r="L68" s="18" t="n"/>
-      <c r="M68" s="18" t="n"/>
-      <c r="N68" s="18" t="n"/>
-      <c r="O68" s="18" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="11" t="inlineStr">
-        <is>
-          <t>▸ West / Other  (1)</t>
-        </is>
-      </c>
-      <c r="B69" s="12" t="n"/>
-      <c r="C69" s="12" t="n"/>
-      <c r="D69" s="12" t="n"/>
-      <c r="E69" s="12" t="n"/>
-      <c r="F69" s="12" t="n"/>
-      <c r="G69" s="12" t="n"/>
-      <c r="H69" s="12" t="n"/>
-      <c r="I69" s="12" t="n"/>
-      <c r="J69" s="12" t="n"/>
-      <c r="K69" s="12" t="n"/>
-      <c r="L69" s="12" t="n"/>
-      <c r="M69" s="12" t="n"/>
-      <c r="N69" s="12" t="n"/>
-      <c r="O69" s="12" t="n"/>
-    </row>
-    <row r="70" outlineLevel="1">
-      <c r="A70" s="13" t="inlineStr">
-        <is>
-          <t>West / Other</t>
-        </is>
-      </c>
-      <c r="B70" s="14" t="inlineStr">
-        <is>
-          <t>National salad concept liquidation – full contents of 63 fast-casual restaurants (AZ/TX/OK/NV)</t>
-        </is>
-      </c>
-      <c r="C70" s="13" t="inlineStr">
-        <is>
-          <t>restaurant chain liquidation</t>
-        </is>
-      </c>
-      <c r="D70" s="13" t="inlineStr">
-        <is>
-          <t>Phoenix</t>
-        </is>
-      </c>
-      <c r="E70" s="13" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="F70" s="13" t="n">
-        <v>2307</v>
-      </c>
-      <c r="G70" s="13" t="inlineStr">
-        <is>
-          <t>Online auctions, dates TBD</t>
-        </is>
-      </c>
-      <c r="H70" s="15" t="n"/>
-      <c r="I70" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="J70" s="13" t="inlineStr"/>
-      <c r="K70" s="13" t="inlineStr">
-        <is>
-          <t>RestaurantEquipment.bid (TAGeX)</t>
-        </is>
-      </c>
-      <c r="L70" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M70" s="13" t="inlineStr"/>
-      <c r="N70" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O70" s="14" t="inlineStr">
-        <is>
-          <t>Rolling market-by-market auctions, none live yet (Phoenix metro 30 locations, DFW 14, Tucson 6, Houston 5, plus OK/NV). Pickup on site at each restaurant. Pinned at Phoenix.</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — West / Other</t>
-        </is>
-      </c>
-      <c r="B71" s="17" t="inlineStr">
-        <is>
-          <t>1 item(s)</t>
-        </is>
-      </c>
-      <c r="C71" s="18" t="n"/>
-      <c r="D71" s="18" t="n"/>
-      <c r="E71" s="18" t="n"/>
-      <c r="F71" s="18" t="n"/>
-      <c r="G71" s="18" t="n"/>
-      <c r="H71" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I71" s="18" t="n"/>
-      <c r="J71" s="18" t="n"/>
-      <c r="K71" s="18" t="n"/>
-      <c r="L71" s="18" t="n"/>
-      <c r="M71" s="18" t="n"/>
-      <c r="N71" s="18" t="n"/>
-      <c r="O71" s="18" t="n"/>
+      <c r="I69" s="18" t="n"/>
+      <c r="J69" s="18" t="n"/>
+      <c r="K69" s="18" t="n"/>
+      <c r="L69" s="18" t="n"/>
+      <c r="M69" s="18" t="n"/>
+      <c r="N69" s="18" t="n"/>
+      <c r="O69" s="18" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O71"/>
+  <autoFilter ref="A1:O69"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId2"/>
@@ -22235,8 +22109,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N32" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N35" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N36" r:id="rId24"/>
@@ -22251,17 +22125,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N45" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N46" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N47" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N48" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N49" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N52" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N50" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N53" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N54" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N55" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N56" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N57" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N60" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N63" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N64" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N67" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N70" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N58" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N61" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N62" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N65" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N68" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Lot Recon 2026-10-19 midday: +4 business liquidations, prune Brockton fixtures
Added Somerville NJ bakery/cafe HiBid, Kenilworth NJ Air Systems HVAC shop, Flemington NJ kitchen/store, West Nyack body-shop tools. Removed deleted Brockton Best Buy Outlet racking CL. HiBid Wolf lots already present; bid prices refreshed.
</commit_message>
<xml_diff>
--- a/lot_recon.xlsx
+++ b/lot_recon.xlsx
@@ -20,8 +20,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wolf New'!$A$1:$O$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Wolf Used'!$A$1:$O$189</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Wolf Unclear'!$A$1:$O$40</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$75</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 2026-10-19 08:00 ET</t>
+          <t>Last updated: 2026-10-19 11:11 ET</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Active listings: 291 · Removed: 4</t>
+          <t>Active listings: 294 · Removed: 5</t>
         </is>
       </c>
     </row>
@@ -679,7 +679,7 @@
         <v>164</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>607929.6</v>
+        <v>608011.6</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
@@ -695,7 +695,7 @@
         <v>31</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>137837.5</v>
+        <v>137840</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
@@ -708,13 +708,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13">
@@ -724,10 +724,10 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>980348.08</v>
+        <v>980432.58</v>
       </c>
     </row>
     <row r="15">
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C17" t="n">
         <v>1</v>
@@ -806,7 +806,7 @@
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H17" s="6" t="n">
         <v>5398.69</v>
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C23" t="n">
         <v>1</v>
@@ -1004,10 +1004,10 @@
         <v>4</v>
       </c>
       <c r="G23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>64663</v>
+        <v>64740</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="C24" t="n">
         <v>1</v>
@@ -1037,7 +1037,7 @@
         <v>24</v>
       </c>
       <c r="G24" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H24" s="6" t="n">
         <v>440141</v>
@@ -1073,7 +1073,7 @@
         <v>1</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>1512.5</v>
+        <v>1515</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -1238,7 +1238,7 @@
         <v>2</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -4141,7 +4141,7 @@
       </c>
       <c r="G16" s="13" t="inlineStr">
         <is>
-          <t>$0 current bid + BP</t>
+          <t>$0 / prebids open (live Oct 25)</t>
         </is>
       </c>
       <c r="H16" s="15" t="n">
@@ -7060,11 +7060,11 @@
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>$13 current bid (6 bids) + 18% BP</t>
+          <t>$90 high bid (16 bids)</t>
         </is>
       </c>
       <c r="H34" s="15" t="n">
-        <v>13</v>
+        <v>90</v>
       </c>
       <c r="I34" s="13" t="inlineStr"/>
       <c r="J34" s="13" t="inlineStr">
@@ -7867,7 +7867,7 @@
       <c r="F47" s="18" t="n"/>
       <c r="G47" s="18" t="n"/>
       <c r="H47" s="19" t="n">
-        <v>33063</v>
+        <v>33140</v>
       </c>
       <c r="I47" s="18" t="n"/>
       <c r="J47" s="18" t="n"/>
@@ -12396,7 +12396,7 @@
       </c>
       <c r="G122" s="13" t="inlineStr">
         <is>
-          <t>$0 current bid + BP</t>
+          <t>$0 high bid</t>
         </is>
       </c>
       <c r="H122" s="15" t="n">
@@ -12461,7 +12461,7 @@
       </c>
       <c r="G123" s="13" t="inlineStr">
         <is>
-          <t>$0 current bid + BP</t>
+          <t>$0 high bid</t>
         </is>
       </c>
       <c r="H123" s="15" t="n">
@@ -12574,11 +12574,11 @@
       </c>
       <c r="G126" s="13" t="inlineStr">
         <is>
-          <t>$0 current bid + BP</t>
+          <t>$5 high bid</t>
         </is>
       </c>
       <c r="H126" s="15" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I126" s="13" t="inlineStr"/>
       <c r="J126" s="13" t="inlineStr">
@@ -12629,7 +12629,7 @@
       <c r="F127" s="18" t="n"/>
       <c r="G127" s="18" t="n"/>
       <c r="H127" s="19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I127" s="18" t="n"/>
       <c r="J127" s="18" t="n"/>
@@ -18394,11 +18394,11 @@
       </c>
       <c r="G35" s="13" t="inlineStr">
         <is>
-          <t>$12.50 high bid</t>
+          <t>$15 high bid</t>
         </is>
       </c>
       <c r="H35" s="15" t="n">
-        <v>12.5</v>
+        <v>15</v>
       </c>
       <c r="I35" s="13" t="inlineStr"/>
       <c r="J35" s="13" t="inlineStr">
@@ -18445,7 +18445,7 @@
       <c r="F36" s="18" t="n"/>
       <c r="G36" s="18" t="n"/>
       <c r="H36" s="19" t="n">
-        <v>12.5</v>
+        <v>15</v>
       </c>
       <c r="I36" s="18" t="n"/>
       <c r="J36" s="18" t="n"/>
@@ -18507,7 +18507,7 @@
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>$5 current bid + BP</t>
+          <t>$5 high bid</t>
         </is>
       </c>
       <c r="H38" s="15" t="n">
@@ -18572,7 +18572,7 @@
       </c>
       <c r="G39" s="13" t="inlineStr">
         <is>
-          <t>$0 current bid + BP</t>
+          <t>$0 high bid</t>
         </is>
       </c>
       <c r="H39" s="15" t="n">
@@ -18678,7 +18678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O75"/>
+  <dimension ref="A1:O78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -18778,7 +18778,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>▸ Greater Boston / South Shore (&lt;50mi)  (5)</t>
+          <t>▸ Greater Boston / South Shore (&lt;50mi)  (4)</t>
         </is>
       </c>
       <c r="B2" s="12" t="n"/>
@@ -18804,17 +18804,17 @@
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>Closed Best Buy Outlet – pallet racking, Big Joe order pickers, appliance dollies, carts, cages</t>
+          <t>P&amp;S Mechanical contractor liquidation – plumbing stock, hot water tanks, pumps, tools, 2 ProMaster vans</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
-          <t>store closing fixtures</t>
+          <t>contractor liquidation</t>
         </is>
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>Brockton</t>
+          <t>Plymouth</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
@@ -18823,28 +18823,28 @@
         </is>
       </c>
       <c r="F3" s="13" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G3" s="13" t="inlineStr">
         <is>
-          <t>Racking $40/upright, $80/level; pickers $1,000 OBO</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H3" s="15" t="n"/>
-      <c r="I3" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="J3" s="13" t="inlineStr"/>
+      <c r="I3" s="13" t="inlineStr"/>
+      <c r="J3" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-22 09:00 AM ET</t>
+        </is>
+      </c>
       <c r="K3" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
-        </is>
-      </c>
-      <c r="L3" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>Salvadore Auctions</t>
+        </is>
+      </c>
+      <c r="L3" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M3" s="13" t="inlineStr"/>
@@ -18855,7 +18855,7 @@
       </c>
       <c r="O3" s="14" t="inlineStr">
         <is>
-          <t>200 Westgate Dr. Fixtures/equipment only, no merchandise. On site daily.</t>
+          <t>Page conflicts: Oct 21 or 22 9 AM (later date used). Closest find.</t>
         </is>
       </c>
     </row>
@@ -18867,17 +18867,17 @@
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>P&amp;S Mechanical contractor liquidation – plumbing stock, hot water tanks, pumps, tools, 2 ProMaster vans</t>
+          <t>"Fire sale" former chain restaurant – AccuTemp AccuSteam 36" griddles, Vulcan hot plate, custom stainless stations</t>
         </is>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>contractor liquidation</t>
+          <t>restaurant closing</t>
         </is>
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>Plymouth</t>
+          <t>Cambridge</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -18886,23 +18886,23 @@
         </is>
       </c>
       <c r="F4" s="13" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="G4" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>$9,500 OBO whole lot (or per piece)</t>
         </is>
       </c>
       <c r="H4" s="15" t="n"/>
-      <c r="I4" s="13" t="inlineStr"/>
-      <c r="J4" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-22 09:00 AM ET</t>
-        </is>
-      </c>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="J4" s="13" t="inlineStr"/>
       <c r="K4" s="13" t="inlineStr">
         <is>
-          <t>Salvadore Auctions</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L4" s="13" t="inlineStr">
@@ -18918,7 +18918,7 @@
       </c>
       <c r="O4" s="14" t="inlineStr">
         <is>
-          <t>Page conflicts: Oct 21 or 22 9 AM (later date used). Closest find.</t>
+          <t>Updated Oct 16. Individually priced $13,250 total. Cash/wire/cashier's check.</t>
         </is>
       </c>
     </row>
@@ -18930,17 +18930,17 @@
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>"Fire sale" former chain restaurant – AccuTemp AccuSteam 36" griddles, Vulcan hot plate, custom stainless stations</t>
+          <t>Retirement bulk tool lot – 10 tools, sold together</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>restaurant closing</t>
+          <t>retirement</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Cambridge</t>
+          <t>Waltham</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
@@ -18949,17 +18949,17 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G5" s="13" t="inlineStr">
         <is>
-          <t>$9,500 OBO whole lot (or per piece)</t>
+          <t>$250 all</t>
         </is>
       </c>
       <c r="H5" s="15" t="n"/>
       <c r="I5" s="13" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="J5" s="13" t="inlineStr"/>
@@ -18981,7 +18981,7 @@
       </c>
       <c r="O5" s="14" t="inlineStr">
         <is>
-          <t>Updated Oct 16. Individually priced $13,250 total. Cash/wire/cashier's check.</t>
+          <t>Small off-category FYI; seller says resell individually. Old CL URL deleted; reposted under new URL 2026-10-19 (same $250 / 10 tools).</t>
         </is>
       </c>
     </row>
@@ -18993,17 +18993,17 @@
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>Retirement bulk tool lot – 10 tools, sold together</t>
+          <t>Cannabis facility contents incl. commercial kitchen / stainless</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>retirement</t>
+          <t>facility contents</t>
         </is>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Waltham</t>
+          <t>Milford</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
@@ -19012,23 +19012,23 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="G6" s="13" t="inlineStr">
         <is>
-          <t>$250 all</t>
+          <t>Auction, 18% BP</t>
         </is>
       </c>
       <c r="H6" s="15" t="n"/>
-      <c r="I6" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="J6" s="13" t="inlineStr"/>
+      <c r="I6" s="13" t="inlineStr"/>
+      <c r="J6" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-03 10:00 AM ET</t>
+        </is>
+      </c>
       <c r="K6" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>Paul E. Saperstein (PESCO)</t>
         </is>
       </c>
       <c r="L6" s="13" t="inlineStr">
@@ -19044,120 +19044,120 @@
       </c>
       <c r="O6" s="14" t="inlineStr">
         <is>
-          <t>Small off-category FYI; seller says resell individually. Old CL URL deleted; reposted under new URL 2026-10-19 (same $250 / 10 tools).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" outlineLevel="1">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t>Greater Boston / South Shore (&lt;50mi)</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>Cannabis facility contents incl. commercial kitchen / stainless</t>
-        </is>
-      </c>
-      <c r="C7" s="13" t="inlineStr">
-        <is>
-          <t>facility contents</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>Milford</t>
-        </is>
-      </c>
-      <c r="E7" s="13" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="F7" s="13" t="n">
-        <v>36</v>
-      </c>
-      <c r="G7" s="13" t="inlineStr">
-        <is>
-          <t>Auction, 18% BP</t>
-        </is>
-      </c>
-      <c r="H7" s="15" t="n"/>
-      <c r="I7" s="13" t="inlineStr"/>
-      <c r="J7" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-03 10:00 AM ET</t>
-        </is>
-      </c>
-      <c r="K7" s="13" t="inlineStr">
-        <is>
-          <t>Paul E. Saperstein (PESCO)</t>
-        </is>
-      </c>
-      <c r="L7" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M7" s="13" t="inlineStr"/>
-      <c r="N7" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O7" s="14" t="inlineStr">
-        <is>
           <t>Calendar page only (no event page yet). ~45 mi.</t>
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Greater Boston / South Shore (&lt;50mi)</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>4 item(s)</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="n"/>
+      <c r="D7" s="18" t="n"/>
+      <c r="E7" s="18" t="n"/>
+      <c r="F7" s="18" t="n"/>
+      <c r="G7" s="18" t="n"/>
+      <c r="H7" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="18" t="n"/>
+      <c r="J7" s="18" t="n"/>
+      <c r="K7" s="18" t="n"/>
+      <c r="L7" s="18" t="n"/>
+      <c r="M7" s="18" t="n"/>
+      <c r="N7" s="18" t="n"/>
+      <c r="O7" s="18" t="n"/>
+    </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Greater Boston / South Shore (&lt;50mi)</t>
-        </is>
-      </c>
-      <c r="B8" s="17" t="inlineStr">
-        <is>
-          <t>5 item(s)</t>
-        </is>
-      </c>
-      <c r="C8" s="18" t="n"/>
-      <c r="D8" s="18" t="n"/>
-      <c r="E8" s="18" t="n"/>
-      <c r="F8" s="18" t="n"/>
-      <c r="G8" s="18" t="n"/>
-      <c r="H8" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="18" t="n"/>
-      <c r="J8" s="18" t="n"/>
-      <c r="K8" s="18" t="n"/>
-      <c r="L8" s="18" t="n"/>
-      <c r="M8" s="18" t="n"/>
-      <c r="N8" s="18" t="n"/>
-      <c r="O8" s="18" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>▸ North Shore / Merrimack Valley / S. NH  (2)</t>
         </is>
       </c>
-      <c r="B9" s="12" t="n"/>
-      <c r="C9" s="12" t="n"/>
-      <c r="D9" s="12" t="n"/>
-      <c r="E9" s="12" t="n"/>
-      <c r="F9" s="12" t="n"/>
-      <c r="G9" s="12" t="n"/>
-      <c r="H9" s="12" t="n"/>
-      <c r="I9" s="12" t="n"/>
-      <c r="J9" s="12" t="n"/>
-      <c r="K9" s="12" t="n"/>
-      <c r="L9" s="12" t="n"/>
-      <c r="M9" s="12" t="n"/>
-      <c r="N9" s="12" t="n"/>
-      <c r="O9" s="12" t="n"/>
+      <c r="B8" s="12" t="n"/>
+      <c r="C8" s="12" t="n"/>
+      <c r="D8" s="12" t="n"/>
+      <c r="E8" s="12" t="n"/>
+      <c r="F8" s="12" t="n"/>
+      <c r="G8" s="12" t="n"/>
+      <c r="H8" s="12" t="n"/>
+      <c r="I8" s="12" t="n"/>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="12" t="n"/>
+      <c r="L8" s="12" t="n"/>
+      <c r="M8" s="12" t="n"/>
+      <c r="N8" s="12" t="n"/>
+      <c r="O8" s="12" t="n"/>
+    </row>
+    <row r="9" outlineLevel="1">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>North Shore / Merrimack Valley / S. NH</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>Commercial mechanical/plumbing/HVAC contractor inventory – multiple pallets of boxed stock, water heater, venting, diffusers</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>inventory</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Merrimack</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>62</v>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>$1 placeholder – make offer on everything</t>
+        </is>
+      </c>
+      <c r="H9" s="15" t="n"/>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="inlineStr"/>
+      <c r="K9" s="13" t="inlineStr">
+        <is>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L9" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M9" s="13" t="inlineStr"/>
+      <c r="N9" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O9" s="14" t="inlineStr">
+        <is>
+          <t>Bulk buyers preferred.</t>
+        </is>
+      </c>
     </row>
     <row r="10" outlineLevel="1">
       <c r="A10" s="13" t="inlineStr">
@@ -19167,17 +19167,17 @@
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>Commercial mechanical/plumbing/HVAC contractor inventory – multiple pallets of boxed stock, water heater, venting, diffusers</t>
+          <t>Plumbing &amp; heating overstock/returns online auction – 183 lots (fixtures, furnaces, heaters, A/C)</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>Merrimack</t>
+          <t>Concord</t>
         </is>
       </c>
       <c r="E10" s="13" t="inlineStr">
@@ -19186,23 +19186,27 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>62</v>
+        <v>84</v>
       </c>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t>$1 placeholder – make offer on everything</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H10" s="15" t="n"/>
       <c r="I10" s="13" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="J10" s="13" t="inlineStr"/>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="J10" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-27 07:00 PM ET</t>
+        </is>
+      </c>
       <c r="K10" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>HiBid (Atlantic Auction Co.)</t>
         </is>
       </c>
       <c r="L10" s="13" t="inlineStr">
@@ -19218,124 +19222,120 @@
       </c>
       <c r="O10" s="14" t="inlineStr">
         <is>
-          <t>Bulk buyers preferred.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" outlineLevel="1">
-      <c r="A11" s="13" t="inlineStr">
-        <is>
-          <t>North Shore / Merrimack Valley / S. NH</t>
-        </is>
-      </c>
-      <c r="B11" s="14" t="inlineStr">
-        <is>
-          <t>Plumbing &amp; heating overstock/returns online auction – 183 lots (fixtures, furnaces, heaters, A/C)</t>
-        </is>
-      </c>
-      <c r="C11" s="13" t="inlineStr">
-        <is>
-          <t>auction</t>
-        </is>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>Concord</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="inlineStr">
-        <is>
-          <t>NH</t>
-        </is>
-      </c>
-      <c r="F11" s="13" t="n">
-        <v>84</v>
-      </c>
-      <c r="G11" s="13" t="inlineStr">
-        <is>
-          <t>Online auction</t>
-        </is>
-      </c>
-      <c r="H11" s="15" t="n"/>
-      <c r="I11" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="J11" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-27 07:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K11" s="13" t="inlineStr">
-        <is>
-          <t>HiBid (Atlantic Auction Co.)</t>
-        </is>
-      </c>
-      <c r="L11" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M11" s="13" t="inlineStr"/>
-      <c r="N11" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O11" s="14" t="inlineStr">
-        <is>
           <t>Overstock sale, not a closing. Pickup Oct 29–30.</t>
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — North Shore / Merrimack Valley / S. NH</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>2 item(s)</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="n"/>
+      <c r="D11" s="18" t="n"/>
+      <c r="E11" s="18" t="n"/>
+      <c r="F11" s="18" t="n"/>
+      <c r="G11" s="18" t="n"/>
+      <c r="H11" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="18" t="n"/>
+      <c r="J11" s="18" t="n"/>
+      <c r="K11" s="18" t="n"/>
+      <c r="L11" s="18" t="n"/>
+      <c r="M11" s="18" t="n"/>
+      <c r="N11" s="18" t="n"/>
+      <c r="O11" s="18" t="n"/>
+    </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — North Shore / Merrimack Valley / S. NH</t>
-        </is>
-      </c>
-      <c r="B12" s="17" t="inlineStr">
-        <is>
-          <t>2 item(s)</t>
-        </is>
-      </c>
-      <c r="C12" s="18" t="n"/>
-      <c r="D12" s="18" t="n"/>
-      <c r="E12" s="18" t="n"/>
-      <c r="F12" s="18" t="n"/>
-      <c r="G12" s="18" t="n"/>
-      <c r="H12" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="18" t="n"/>
-      <c r="J12" s="18" t="n"/>
-      <c r="K12" s="18" t="n"/>
-      <c r="L12" s="18" t="n"/>
-      <c r="M12" s="18" t="n"/>
-      <c r="N12" s="18" t="n"/>
-      <c r="O12" s="18" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>▸ Central / Western MA  (3)</t>
         </is>
       </c>
-      <c r="B13" s="12" t="n"/>
-      <c r="C13" s="12" t="n"/>
-      <c r="D13" s="12" t="n"/>
-      <c r="E13" s="12" t="n"/>
-      <c r="F13" s="12" t="n"/>
-      <c r="G13" s="12" t="n"/>
-      <c r="H13" s="12" t="n"/>
-      <c r="I13" s="12" t="n"/>
-      <c r="J13" s="12" t="n"/>
-      <c r="K13" s="12" t="n"/>
-      <c r="L13" s="12" t="n"/>
-      <c r="M13" s="12" t="n"/>
-      <c r="N13" s="12" t="n"/>
-      <c r="O13" s="12" t="n"/>
+      <c r="B12" s="12" t="n"/>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="12" t="n"/>
+      <c r="F12" s="12" t="n"/>
+      <c r="G12" s="12" t="n"/>
+      <c r="H12" s="12" t="n"/>
+      <c r="I12" s="12" t="n"/>
+      <c r="J12" s="12" t="n"/>
+      <c r="K12" s="12" t="n"/>
+      <c r="L12" s="12" t="n"/>
+      <c r="M12" s="12" t="n"/>
+      <c r="N12" s="12" t="n"/>
+      <c r="O12" s="12" t="n"/>
+    </row>
+    <row r="13" outlineLevel="1">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Central / Western MA</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>Gift/souvenir store closing (retirement) – all new stock</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>store closing</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>Thorndike</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="n">
+        <v>77</v>
+      </c>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>By appointment</t>
+        </is>
+      </c>
+      <c r="H13" s="15" t="n"/>
+      <c r="I13" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="J13" s="13" t="inlineStr"/>
+      <c r="K13" s="13" t="inlineStr">
+        <is>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L13" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M13" s="13" t="inlineStr"/>
+      <c r="N13" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O13" s="14" t="inlineStr">
+        <is>
+          <t>Updated Oct 8. Off-category FYI.</t>
+        </is>
+      </c>
     </row>
     <row r="14" outlineLevel="1">
       <c r="A14" s="13" t="inlineStr">
@@ -19345,17 +19345,17 @@
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>Gift/souvenir store closing (retirement) – all new stock</t>
+          <t>UNECO Manufacturing – owners retiring, machine-shop metrology &amp; tooling</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>retirement</t>
         </is>
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>Thorndike</t>
+          <t>Chicopee</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
@@ -19364,23 +19364,23 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>By appointment</t>
+          <t>Online auction, 18% BP</t>
         </is>
       </c>
       <c r="H14" s="15" t="n"/>
-      <c r="I14" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="J14" s="13" t="inlineStr"/>
+      <c r="I14" s="13" t="inlineStr"/>
+      <c r="J14" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-04 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K14" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>HiBid (DeCosmo Industrial)</t>
         </is>
       </c>
       <c r="L14" s="13" t="inlineStr">
@@ -19396,7 +19396,7 @@
       </c>
       <c r="O14" s="14" t="inlineStr">
         <is>
-          <t>Updated Oct 8. Off-category FYI.</t>
+          <t>Niche tooling only. Bidding opens Oct 19.</t>
         </is>
       </c>
     </row>
@@ -19408,17 +19408,17 @@
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>UNECO Manufacturing – owners retiring, machine-shop metrology &amp; tooling</t>
+          <t>Restaurant closing, everything must go – kitchen equipment, stainless, smallwares</t>
         </is>
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>retirement</t>
+          <t>restaurant closing</t>
         </is>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
-          <t>Chicopee</t>
+          <t>Westfield</t>
         </is>
       </c>
       <c r="E15" s="13" t="inlineStr">
@@ -19427,23 +19427,23 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t>Online auction, 18% BP</t>
+          <t>Make offer</t>
         </is>
       </c>
       <c r="H15" s="15" t="n"/>
-      <c r="I15" s="13" t="inlineStr"/>
-      <c r="J15" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-04 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="J15" s="13" t="inlineStr"/>
       <c r="K15" s="13" t="inlineStr">
         <is>
-          <t>HiBid (DeCosmo Industrial)</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L15" s="13" t="inlineStr">
@@ -19459,120 +19459,120 @@
       </c>
       <c r="O15" s="14" t="inlineStr">
         <is>
-          <t>Niche tooling only. Bidding opens Oct 19.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" outlineLevel="1">
-      <c r="A16" s="13" t="inlineStr">
-        <is>
-          <t>Central / Western MA</t>
-        </is>
-      </c>
-      <c r="B16" s="14" t="inlineStr">
-        <is>
-          <t>Restaurant closing, everything must go – kitchen equipment, stainless, smallwares</t>
-        </is>
-      </c>
-      <c r="C16" s="13" t="inlineStr">
-        <is>
-          <t>restaurant closing</t>
-        </is>
-      </c>
-      <c r="D16" s="13" t="inlineStr">
-        <is>
-          <t>Westfield</t>
-        </is>
-      </c>
-      <c r="E16" s="13" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="F16" s="13" t="n">
-        <v>99</v>
-      </c>
-      <c r="G16" s="13" t="inlineStr">
-        <is>
-          <t>Make offer</t>
-        </is>
-      </c>
-      <c r="H16" s="15" t="n"/>
-      <c r="I16" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="J16" s="13" t="inlineStr"/>
-      <c r="K16" s="13" t="inlineStr">
-        <is>
-          <t>Craigslist</t>
-        </is>
-      </c>
-      <c r="L16" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M16" s="13" t="inlineStr"/>
-      <c r="N16" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O16" s="14" t="inlineStr">
-        <is>
           <t>Related separate post "Complete Restaurant Equipment Package" $3,500 OBO (maybe same restaurant): https://www.craigslist.org/view/d/westfield-complete-restaurant-equipment/9Y5KCdhhgSqEBYbD3wKqVd</t>
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Central / Western MA</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>3 item(s)</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="n"/>
+      <c r="D16" s="18" t="n"/>
+      <c r="E16" s="18" t="n"/>
+      <c r="F16" s="18" t="n"/>
+      <c r="G16" s="18" t="n"/>
+      <c r="H16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="18" t="n"/>
+      <c r="J16" s="18" t="n"/>
+      <c r="K16" s="18" t="n"/>
+      <c r="L16" s="18" t="n"/>
+      <c r="M16" s="18" t="n"/>
+      <c r="N16" s="18" t="n"/>
+      <c r="O16" s="18" t="n"/>
+    </row>
     <row r="17">
-      <c r="A17" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Central / Western MA</t>
-        </is>
-      </c>
-      <c r="B17" s="17" t="inlineStr">
-        <is>
-          <t>3 item(s)</t>
-        </is>
-      </c>
-      <c r="C17" s="18" t="n"/>
-      <c r="D17" s="18" t="n"/>
-      <c r="E17" s="18" t="n"/>
-      <c r="F17" s="18" t="n"/>
-      <c r="G17" s="18" t="n"/>
-      <c r="H17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="18" t="n"/>
-      <c r="J17" s="18" t="n"/>
-      <c r="K17" s="18" t="n"/>
-      <c r="L17" s="18" t="n"/>
-      <c r="M17" s="18" t="n"/>
-      <c r="N17" s="18" t="n"/>
-      <c r="O17" s="18" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>▸ Maine / VT / Northern NH  (5)</t>
         </is>
       </c>
-      <c r="B18" s="12" t="n"/>
-      <c r="C18" s="12" t="n"/>
-      <c r="D18" s="12" t="n"/>
-      <c r="E18" s="12" t="n"/>
-      <c r="F18" s="12" t="n"/>
-      <c r="G18" s="12" t="n"/>
-      <c r="H18" s="12" t="n"/>
-      <c r="I18" s="12" t="n"/>
-      <c r="J18" s="12" t="n"/>
-      <c r="K18" s="12" t="n"/>
-      <c r="L18" s="12" t="n"/>
-      <c r="M18" s="12" t="n"/>
-      <c r="N18" s="12" t="n"/>
-      <c r="O18" s="12" t="n"/>
+      <c r="B17" s="12" t="n"/>
+      <c r="C17" s="12" t="n"/>
+      <c r="D17" s="12" t="n"/>
+      <c r="E17" s="12" t="n"/>
+      <c r="F17" s="12" t="n"/>
+      <c r="G17" s="12" t="n"/>
+      <c r="H17" s="12" t="n"/>
+      <c r="I17" s="12" t="n"/>
+      <c r="J17" s="12" t="n"/>
+      <c r="K17" s="12" t="n"/>
+      <c r="L17" s="12" t="n"/>
+      <c r="M17" s="12" t="n"/>
+      <c r="N17" s="12" t="n"/>
+      <c r="O17" s="12" t="n"/>
+    </row>
+    <row r="18" outlineLevel="1">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>Maine / VT / Northern NH</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>Oola Bowls secured-party sale – restaurant equipment bought new 2024-25 (Electro Freeze, Scotsman, Atosa)</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Scarborough</t>
+        </is>
+      </c>
+      <c r="E18" s="13" t="inlineStr">
+        <is>
+          <t>ME</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="n">
+        <v>104</v>
+      </c>
+      <c r="G18" s="13" t="inlineStr">
+        <is>
+          <t>Online auction (freezers $80–150 when seen)</t>
+        </is>
+      </c>
+      <c r="H18" s="15" t="n"/>
+      <c r="I18" s="13" t="inlineStr"/>
+      <c r="J18" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 01:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K18" s="13" t="inlineStr">
+        <is>
+          <t>Keenan Auction / Proxibid</t>
+        </is>
+      </c>
+      <c r="L18" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M18" s="13" t="inlineStr"/>
+      <c r="N18" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O18" s="14" t="inlineStr">
+        <is>
+          <t>Pickup Oct 21 only.</t>
+        </is>
+      </c>
     </row>
     <row r="19" outlineLevel="1">
       <c r="A19" s="13" t="inlineStr">
@@ -19582,12 +19582,12 @@
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>Oola Bowls secured-party sale – restaurant equipment bought new 2024-25 (Electro Freeze, Scotsman, Atosa)</t>
+          <t>Contractor appliance lot – 3 refrigerators, Bosch wall oven, gas range, washer/dryer set</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>contractor lot</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
@@ -19605,24 +19605,24 @@
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>Online auction (freezers $80–150 when seen)</t>
+          <t>$200 OBO each, less as a bundle</t>
         </is>
       </c>
       <c r="H19" s="15" t="n"/>
-      <c r="I19" s="13" t="inlineStr"/>
-      <c r="J19" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-19 01:00 PM ET</t>
-        </is>
-      </c>
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="J19" s="13" t="inlineStr"/>
       <c r="K19" s="13" t="inlineStr">
         <is>
-          <t>Keenan Auction / Proxibid</t>
-        </is>
-      </c>
-      <c r="L19" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L19" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M19" s="13" t="inlineStr"/>
@@ -19633,7 +19633,7 @@
       </c>
       <c r="O19" s="14" t="inlineStr">
         <is>
-          <t>Pickup Oct 21 only.</t>
+          <t>Working units pulled from jobs. Complete appliances, not parts.</t>
         </is>
       </c>
     </row>
@@ -19645,17 +19645,17 @@
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>Contractor appliance lot – 3 refrigerators, Bosch wall oven, gas range, washer/dryer set</t>
+          <t>Event-rental business closing – 300+ chairs, 40+ rounds, 1,300+ china, linens (all at once)</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>contractor lot</t>
+          <t>business closing</t>
         </is>
       </c>
       <c r="D20" s="13" t="inlineStr">
         <is>
-          <t>Scarborough</t>
+          <t>Woolwich</t>
         </is>
       </c>
       <c r="E20" s="13" t="inlineStr">
@@ -19664,17 +19664,17 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>104</v>
+        <v>135</v>
       </c>
       <c r="G20" s="13" t="inlineStr">
         <is>
-          <t>$200 OBO each, less as a bundle</t>
+          <t>No price listed</t>
         </is>
       </c>
       <c r="H20" s="15" t="n"/>
       <c r="I20" s="13" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="J20" s="13" t="inlineStr"/>
@@ -19696,7 +19696,7 @@
       </c>
       <c r="O20" s="14" t="inlineStr">
         <is>
-          <t>Working units pulled from jobs. Complete appliances, not parts.</t>
+          <t>Updated Oct 7. Replacement cost &gt;$72K per post.</t>
         </is>
       </c>
     </row>
@@ -19708,42 +19708,42 @@
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>Event-rental business closing – 300+ chairs, 40+ rounds, 1,300+ china, linens (all at once)</t>
+          <t>Pellet/wood stoves, heating stock, tools &amp; heavy equipment – "business liquidation", 380 lots</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>business closing</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
-          <t>Woolwich</t>
+          <t>Lunenburg</t>
         </is>
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>ME</t>
+          <t>VT</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>135</v>
+        <v>168</v>
       </c>
       <c r="G21" s="13" t="inlineStr">
         <is>
-          <t>No price listed</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H21" s="15" t="n"/>
-      <c r="I21" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="J21" s="13" t="inlineStr"/>
+      <c r="I21" s="13" t="inlineStr"/>
+      <c r="J21" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-04 10:00 AM ET</t>
+        </is>
+      </c>
       <c r="K21" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>Thomas Hirchak Co.</t>
         </is>
       </c>
       <c r="L21" s="13" t="inlineStr">
@@ -19759,7 +19759,7 @@
       </c>
       <c r="O21" s="14" t="inlineStr">
         <is>
-          <t>Updated Oct 7. Replacement cost &gt;$72K per post.</t>
+          <t>Closes Wed Nov 4 10 AM, preview Oct 28, removal Nov 9, no shipping.</t>
         </is>
       </c>
     </row>
@@ -19771,17 +19771,17 @@
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>Pellet/wood stoves, heating stock, tools &amp; heavy equipment – "business liquidation", 380 lots</t>
+          <t>Bread Loaf Corp wind-down – contractor equipment, staging, telehandler</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>contractor liquidation</t>
         </is>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>Lunenburg</t>
+          <t>Middlebury</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
@@ -19790,7 +19790,7 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="G22" s="13" t="inlineStr">
         <is>
@@ -19801,12 +19801,12 @@
       <c r="I22" s="13" t="inlineStr"/>
       <c r="J22" s="13" t="inlineStr">
         <is>
-          <t>2026-11-04 10:00 AM ET</t>
+          <t>2026-10-28 09:00 AM ET</t>
         </is>
       </c>
       <c r="K22" s="13" t="inlineStr">
         <is>
-          <t>Thomas Hirchak Co.</t>
+          <t>THC Auction</t>
         </is>
       </c>
       <c r="L22" s="13" t="inlineStr">
@@ -19822,120 +19822,120 @@
       </c>
       <c r="O22" s="14" t="inlineStr">
         <is>
-          <t>Closes Wed Nov 4 10 AM, preview Oct 28, removal Nov 9, no shipping.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" outlineLevel="1">
-      <c r="A23" s="13" t="inlineStr">
-        <is>
-          <t>Maine / VT / Northern NH</t>
-        </is>
-      </c>
-      <c r="B23" s="14" t="inlineStr">
-        <is>
-          <t>Bread Loaf Corp wind-down – contractor equipment, staging, telehandler</t>
-        </is>
-      </c>
-      <c r="C23" s="13" t="inlineStr">
+          <t>Company wind-down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Maine / VT / Northern NH</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>5 item(s)</t>
+        </is>
+      </c>
+      <c r="C23" s="18" t="n"/>
+      <c r="D23" s="18" t="n"/>
+      <c r="E23" s="18" t="n"/>
+      <c r="F23" s="18" t="n"/>
+      <c r="G23" s="18" t="n"/>
+      <c r="H23" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="18" t="n"/>
+      <c r="J23" s="18" t="n"/>
+      <c r="K23" s="18" t="n"/>
+      <c r="L23" s="18" t="n"/>
+      <c r="M23" s="18" t="n"/>
+      <c r="N23" s="18" t="n"/>
+      <c r="O23" s="18" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>▸ CT / Hudson Valley  (6)</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="n"/>
+      <c r="C24" s="12" t="n"/>
+      <c r="D24" s="12" t="n"/>
+      <c r="E24" s="12" t="n"/>
+      <c r="F24" s="12" t="n"/>
+      <c r="G24" s="12" t="n"/>
+      <c r="H24" s="12" t="n"/>
+      <c r="I24" s="12" t="n"/>
+      <c r="J24" s="12" t="n"/>
+      <c r="K24" s="12" t="n"/>
+      <c r="L24" s="12" t="n"/>
+      <c r="M24" s="12" t="n"/>
+      <c r="N24" s="12" t="n"/>
+      <c r="O24" s="12" t="n"/>
+    </row>
+    <row r="25" outlineLevel="1">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>CT / Hudson Valley</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>Bank-ordered electrical contractor sale – Greenlee/Hilti/Milwaukee tools, GE/Siemens breakers</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
         <is>
           <t>contractor liquidation</t>
         </is>
       </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>Middlebury</t>
-        </is>
-      </c>
-      <c r="E23" s="13" t="inlineStr">
-        <is>
-          <t>VT</t>
-        </is>
-      </c>
-      <c r="F23" s="13" t="n">
-        <v>177</v>
-      </c>
-      <c r="G23" s="13" t="inlineStr">
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>Clinton</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="n">
+        <v>106</v>
+      </c>
+      <c r="G25" s="13" t="inlineStr">
         <is>
           <t>Online auction</t>
         </is>
       </c>
-      <c r="H23" s="15" t="n"/>
-      <c r="I23" s="13" t="inlineStr"/>
-      <c r="J23" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-28 09:00 AM ET</t>
-        </is>
-      </c>
-      <c r="K23" s="13" t="inlineStr">
-        <is>
-          <t>THC Auction</t>
-        </is>
-      </c>
-      <c r="L23" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M23" s="13" t="inlineStr"/>
-      <c r="N23" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O23" s="14" t="inlineStr">
-        <is>
-          <t>Company wind-down.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Maine / VT / Northern NH</t>
-        </is>
-      </c>
-      <c r="B24" s="17" t="inlineStr">
-        <is>
-          <t>5 item(s)</t>
-        </is>
-      </c>
-      <c r="C24" s="18" t="n"/>
-      <c r="D24" s="18" t="n"/>
-      <c r="E24" s="18" t="n"/>
-      <c r="F24" s="18" t="n"/>
-      <c r="G24" s="18" t="n"/>
-      <c r="H24" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="18" t="n"/>
-      <c r="J24" s="18" t="n"/>
-      <c r="K24" s="18" t="n"/>
-      <c r="L24" s="18" t="n"/>
-      <c r="M24" s="18" t="n"/>
-      <c r="N24" s="18" t="n"/>
-      <c r="O24" s="18" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>▸ CT / Hudson Valley  (5)</t>
-        </is>
-      </c>
-      <c r="B25" s="12" t="n"/>
-      <c r="C25" s="12" t="n"/>
-      <c r="D25" s="12" t="n"/>
-      <c r="E25" s="12" t="n"/>
-      <c r="F25" s="12" t="n"/>
-      <c r="G25" s="12" t="n"/>
-      <c r="H25" s="12" t="n"/>
-      <c r="I25" s="12" t="n"/>
-      <c r="J25" s="12" t="n"/>
-      <c r="K25" s="12" t="n"/>
-      <c r="L25" s="12" t="n"/>
-      <c r="M25" s="12" t="n"/>
-      <c r="N25" s="12" t="n"/>
-      <c r="O25" s="12" t="n"/>
+      <c r="H25" s="15" t="n"/>
+      <c r="I25" s="13" t="inlineStr"/>
+      <c r="J25" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-29 05:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K25" s="13" t="inlineStr">
+        <is>
+          <t>Hamilton Group / EstateSales.net</t>
+        </is>
+      </c>
+      <c r="L25" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M25" s="13" t="inlineStr"/>
+      <c r="N25" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O25" s="14" t="inlineStr">
+        <is>
+          <t>Listed "Oct 29 2 PM PST" (= 5 PM ET).</t>
+        </is>
+      </c>
     </row>
     <row r="26" outlineLevel="1">
       <c r="A26" s="13" t="inlineStr">
@@ -19945,26 +19945,26 @@
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>Bank-ordered electrical contractor sale – Greenlee/Hilti/Milwaukee tools, GE/Siemens breakers</t>
+          <t>Major Intl Chain Surplus – 225 lots commercial refrigeration/kitchen (True, Traulsen, Hobart, Blodgett, Taylor)</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>contractor liquidation</t>
+          <t>commercial surplus</t>
         </is>
       </c>
       <c r="D26" s="13" t="inlineStr">
         <is>
-          <t>Clinton</t>
+          <t>Pleasant Valley</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>106</v>
+        <v>157</v>
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
@@ -19975,17 +19975,17 @@
       <c r="I26" s="13" t="inlineStr"/>
       <c r="J26" s="13" t="inlineStr">
         <is>
-          <t>2026-10-29 05:00 PM ET</t>
+          <t>2026-10-20 02:00 PM ET</t>
         </is>
       </c>
       <c r="K26" s="13" t="inlineStr">
         <is>
-          <t>Hamilton Group / EstateSales.net</t>
-        </is>
-      </c>
-      <c r="L26" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>Adams / BidWrangler</t>
+        </is>
+      </c>
+      <c r="L26" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M26" s="13" t="inlineStr"/>
@@ -19996,7 +19996,7 @@
       </c>
       <c r="O26" s="14" t="inlineStr">
         <is>
-          <t>Listed "Oct 29 2 PM PST" (= 5 PM ET).</t>
+          <t>Tested and new units.</t>
         </is>
       </c>
     </row>
@@ -20008,42 +20008,46 @@
       </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>Major Intl Chain Surplus – 225 lots commercial refrigeration/kitchen (True, Traulsen, Hobart, Blodgett, Taylor)</t>
+          <t>The Outlaw Grill Steakhouse – used restaurant equipment auction (PCI Auctions CT, e.g. Vulcan EV60 Endurance 60" range)</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>commercial surplus</t>
+          <t>restaurant auction</t>
         </is>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>Pleasant Valley</t>
+          <t>Stamford</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="G27" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Online auction, current bids</t>
         </is>
       </c>
       <c r="H27" s="15" t="n"/>
-      <c r="I27" s="13" t="inlineStr"/>
+      <c r="I27" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
       <c r="J27" s="13" t="inlineStr">
         <is>
-          <t>2026-10-20 02:00 PM ET</t>
+          <t>2026-10-21 08:30 PM ET</t>
         </is>
       </c>
       <c r="K27" s="13" t="inlineStr">
         <is>
-          <t>Adams / BidWrangler</t>
+          <t>PCI Auctions</t>
         </is>
       </c>
       <c r="L27" s="20" t="inlineStr">
@@ -20059,7 +20063,7 @@
       </c>
       <c r="O27" s="14" t="inlineStr">
         <is>
-          <t>Tested and new units.</t>
+          <t>Ends Wed Oct 21 8:30 PM EDT. PCI warehouse, 36 Ludlow St, Stamford CT. Page lists preview Oct 28 and removal Thu Oct 29 11-3 (after close). Shipping/delivery available; payment due on pickup day. Items still being added.</t>
         </is>
       </c>
     </row>
@@ -20071,17 +20075,17 @@
       </c>
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>The Outlaw Grill Steakhouse – used restaurant equipment auction (PCI Auctions CT, e.g. Vulcan EV60 Endurance 60" range)</t>
+          <t>Café/bakery liquidation – Traulsen, Vulcan ovens, mixers, Hobart slicer (~74 lots)</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>restaurant auction</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>Stamford</t>
+          <t>Greenwich</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
@@ -20090,27 +20094,23 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>Online auction, current bids</t>
+          <t>Live auction + webcast</t>
         </is>
       </c>
       <c r="H28" s="15" t="n"/>
-      <c r="I28" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
+      <c r="I28" s="13" t="inlineStr"/>
       <c r="J28" s="13" t="inlineStr">
         <is>
-          <t>2026-10-21 08:30 PM ET</t>
+          <t>2026-10-21 06:00 PM ET</t>
         </is>
       </c>
       <c r="K28" s="13" t="inlineStr">
         <is>
-          <t>PCI Auctions</t>
+          <t>Best Buy Auctioneers / AuctionGuide</t>
         </is>
       </c>
       <c r="L28" s="20" t="inlineStr">
@@ -20126,7 +20126,7 @@
       </c>
       <c r="O28" s="14" t="inlineStr">
         <is>
-          <t>Ends Wed Oct 21 8:30 PM EDT. PCI warehouse, 36 Ludlow St, Stamford CT. Page lists preview Oct 28 and removal Thu Oct 29 11-3 (after close). Shipping/delivery available; payment due on pickup day. Items still being added.</t>
+          <t>Oct 21; start time not captured (placeholder 6 PM).</t>
         </is>
       </c>
     </row>
@@ -20138,47 +20138,47 @@
       </c>
       <c r="B29" s="14" t="inlineStr">
         <is>
-          <t>Café/bakery liquidation – Traulsen, Vulcan ovens, mixers, Hobart slicer (~74 lots)</t>
+          <t>BJ's Wholesale closeout – racking, forklifts, Hobart</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>Greenwich</t>
+          <t>Rotterdam</t>
         </is>
       </c>
       <c r="E29" s="13" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="G29" s="13" t="inlineStr">
         <is>
-          <t>Live auction + webcast</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H29" s="15" t="n"/>
       <c r="I29" s="13" t="inlineStr"/>
       <c r="J29" s="13" t="inlineStr">
         <is>
-          <t>2026-10-21 06:00 PM ET</t>
+          <t>2026-11-10 10:00 AM ET</t>
         </is>
       </c>
       <c r="K29" s="13" t="inlineStr">
         <is>
-          <t>Best Buy Auctioneers / AuctionGuide</t>
-        </is>
-      </c>
-      <c r="L29" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L29" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M29" s="13" t="inlineStr"/>
@@ -20189,7 +20189,7 @@
       </c>
       <c r="O29" s="14" t="inlineStr">
         <is>
-          <t>Oct 21; start time not captured (placeholder 6 PM).</t>
+          <t>Closes from Nov 10 10 AM.</t>
         </is>
       </c>
     </row>
@@ -20201,17 +20201,17 @@
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>BJ's Wholesale closeout – racking, forklifts, Hobart</t>
+          <t>Body shop closing after 50 years – tools, welder, generators, plasma</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>tools liquidation</t>
         </is>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>Rotterdam</t>
+          <t>West Nyack</t>
         </is>
       </c>
       <c r="E30" s="13" t="inlineStr">
@@ -20220,23 +20220,23 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Make offer / lot</t>
         </is>
       </c>
       <c r="H30" s="15" t="n"/>
-      <c r="I30" s="13" t="inlineStr"/>
-      <c r="J30" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-10 10:00 AM ET</t>
-        </is>
-      </c>
+      <c r="I30" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="J30" s="13" t="inlineStr"/>
       <c r="K30" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L30" s="13" t="inlineStr">
@@ -20252,7 +20252,7 @@
       </c>
       <c r="O30" s="14" t="inlineStr">
         <is>
-          <t>Closes from Nov 10 10 AM.</t>
+          <t>One-man auto body shop closing/retirement (Park Ridge / West Nyack NY-NJ border). Heat lamps, Kansas jack pullers, Miller 200 welder, generators, sheet-metal brake, hydraulic press, plasma cutter, engine hoist. Posted Aug 16; still open 2026-10-19.</t>
         </is>
       </c>
     </row>
@@ -20264,7 +20264,7 @@
       </c>
       <c r="B31" s="17" t="inlineStr">
         <is>
-          <t>5 item(s)</t>
+          <t>6 item(s)</t>
         </is>
       </c>
       <c r="C31" s="18" t="n"/>
@@ -20286,7 +20286,7 @@
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>▸ NYC / Long Island / NJ  (21)</t>
+          <t>▸ NYC / Long Island / NJ  (24)</t>
         </is>
       </c>
       <c r="B32" s="12" t="n"/>
@@ -21021,17 +21021,17 @@
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>Serpico's Pizzeria (lost lease) – Bari ovens, walk-in, Hobart 60qt, Vulcan range</t>
+          <t>Air Systems Inc – sheet metal / HVAC fabrication shop liquidation</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>HVAC shop liquidation</t>
         </is>
       </c>
       <c r="D44" s="13" t="inlineStr">
         <is>
-          <t>Allenhurst</t>
+          <t>Kenilworth</t>
         </is>
       </c>
       <c r="E44" s="13" t="inlineStr">
@@ -21040,28 +21040,28 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>No-reserve online auction</t>
+          <t>Timed online (15% BP)</t>
         </is>
       </c>
       <c r="H44" s="15" t="n"/>
       <c r="I44" s="13" t="inlineStr"/>
       <c r="J44" s="13" t="inlineStr">
         <is>
-          <t>2026-10-21 11:00 AM ET</t>
+          <t>2026-10-29 11:00 AM ET</t>
         </is>
       </c>
       <c r="K44" s="13" t="inlineStr">
         <is>
-          <t>Peter Costanzo / EstateSales.net</t>
-        </is>
-      </c>
-      <c r="L44" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>A.J. Willner Auctions</t>
+        </is>
+      </c>
+      <c r="L44" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M44" s="13" t="inlineStr"/>
@@ -21072,7 +21072,7 @@
       </c>
       <c r="O44" s="14" t="inlineStr">
         <is>
-          <t>Absolute / no reserve.</t>
+          <t>Vicon HVAC plasma; Flagler/Lockformer/Roto-Die/Engel fab; welders; Clark forklift; Genie Superlift; Ridgid/Milwaukee/DeWalt/Bosch/Hilti/Makita tools; AeroVent/Carnes exhaust fans; racking/scaffolding. Preview Oct 28–29 AM; pickup Oct 29 PM–Nov 4. Same town as Carnes fan CL lot.</t>
         </is>
       </c>
     </row>
@@ -21084,17 +21084,17 @@
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>Altitude Trampoline Park liquidation – partial: Atosa, TurboChef, stainless</t>
+          <t>Serpico's Pizzeria (lost lease) – Bari ovens, walk-in, Hobart 60qt, Vulcan range</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
         <is>
-          <t>facility contents</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D45" s="13" t="inlineStr">
         <is>
-          <t>Iselin</t>
+          <t>Allenhurst</t>
         </is>
       </c>
       <c r="E45" s="13" t="inlineStr">
@@ -21103,11 +21103,11 @@
         </is>
       </c>
       <c r="F45" s="13" t="n">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G45" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>No-reserve online auction</t>
         </is>
       </c>
       <c r="H45" s="15" t="n"/>
@@ -21119,7 +21119,7 @@
       </c>
       <c r="K45" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
+          <t>Peter Costanzo / EstateSales.net</t>
         </is>
       </c>
       <c r="L45" s="20" t="inlineStr">
@@ -21135,7 +21135,7 @@
       </c>
       <c r="O45" s="14" t="inlineStr">
         <is>
-          <t>Some kitchen gear only.</t>
+          <t>Absolute / no reserve.</t>
         </is>
       </c>
     </row>
@@ -21147,17 +21147,17 @@
       </c>
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>Restaurant / pizzeria (contents not described)</t>
+          <t>Altitude Trampoline Park liquidation – partial: Atosa, TurboChef, stainless</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>restaurant closing</t>
+          <t>facility contents</t>
         </is>
       </c>
       <c r="D46" s="13" t="inlineStr">
         <is>
-          <t>Berkeley Heights</t>
+          <t>Iselin</t>
         </is>
       </c>
       <c r="E46" s="13" t="inlineStr">
@@ -21166,27 +21166,23 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H46" s="15" t="n"/>
-      <c r="I46" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
+      <c r="I46" s="13" t="inlineStr"/>
       <c r="J46" s="13" t="inlineStr">
         <is>
-          <t>2026-10-20 02:00 PM ET</t>
+          <t>2026-10-21 11:00 AM ET</t>
         </is>
       </c>
       <c r="K46" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>A.J. Willner</t>
         </is>
       </c>
       <c r="L46" s="20" t="inlineStr">
@@ -21202,7 +21198,7 @@
       </c>
       <c r="O46" s="14" t="inlineStr">
         <is>
-          <t>Tue Oct 20 2 PM. No item description on page.</t>
+          <t>Some kitchen gear only.</t>
         </is>
       </c>
     </row>
@@ -21214,17 +21210,17 @@
       </c>
       <c r="B47" s="14" t="inlineStr">
         <is>
-          <t>New modular concession kitchens (warehouseman's lien) – 5 units, CaptiveAire hoods, new Ovention/Turbo Air</t>
+          <t>Restaurant / pizzeria (contents not described)</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
         <is>
-          <t>lien sale</t>
+          <t>restaurant closing</t>
         </is>
       </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>Edison</t>
+          <t>Berkeley Heights</t>
         </is>
       </c>
       <c r="E47" s="13" t="inlineStr">
@@ -21233,24 +21229,32 @@
         </is>
       </c>
       <c r="F47" s="13" t="n">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="G47" s="13" t="inlineStr">
         <is>
-          <t>Online auction, $2K load-out fee</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H47" s="15" t="n"/>
-      <c r="I47" s="13" t="inlineStr"/>
-      <c r="J47" s="13" t="inlineStr"/>
+      <c r="I47" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J47" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-20 02:00 PM ET</t>
+        </is>
+      </c>
       <c r="K47" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
-        </is>
-      </c>
-      <c r="L47" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
+        </is>
+      </c>
+      <c r="L47" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M47" s="13" t="inlineStr"/>
@@ -21261,7 +21265,7 @@
       </c>
       <c r="O47" s="14" t="inlineStr">
         <is>
-          <t>&gt;$100K new. Close date not captured.</t>
+          <t>Tue Oct 20 2 PM. No item description on page.</t>
         </is>
       </c>
     </row>
@@ -21273,12 +21277,12 @@
       </c>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>Brand-new &amp; scratch-and-dent kitchen/home appliances – ~185 lots (Thermador, GE Café, Miele, Wolf speed oven, Viking, Bosch…)</t>
+          <t>New modular concession kitchens (warehouseman's lien) – 5 units, CaptiveAire hoods, new Ovention/Turbo Air</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>lien sale</t>
         </is>
       </c>
       <c r="D48" s="13" t="inlineStr">
@@ -21296,23 +21300,15 @@
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>Live + HiBid webcast, 18% BP + 3% card</t>
+          <t>Online auction, $2K load-out fee</t>
         </is>
       </c>
       <c r="H48" s="15" t="n"/>
-      <c r="I48" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="J48" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-25 01:00 PM ET</t>
-        </is>
-      </c>
+      <c r="I48" s="13" t="inlineStr"/>
+      <c r="J48" s="13" t="inlineStr"/>
       <c r="K48" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>A.J. Willner</t>
         </is>
       </c>
       <c r="L48" s="13" t="inlineStr">
@@ -21320,11 +21316,7 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M48" s="21" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
+      <c r="M48" s="13" t="inlineStr"/>
       <c r="N48" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -21332,7 +21324,7 @@
       </c>
       <c r="O48" s="14" t="inlineStr">
         <is>
-          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale.</t>
+          <t>&gt;$100K new. Close date not captured.</t>
         </is>
       </c>
     </row>
@@ -21344,17 +21336,17 @@
       </c>
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>Party City (Ch. 11) store – fixtures + party merchandise inventory</t>
+          <t>Brand-new &amp; scratch-and-dent kitchen/home appliances – ~185 lots (Thermador, GE Café, Miele, Wolf speed oven, Viking, Bosch…)</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D49" s="13" t="inlineStr">
         <is>
-          <t>East Brunswick</t>
+          <t>Edison</t>
         </is>
       </c>
       <c r="E49" s="13" t="inlineStr">
@@ -21363,23 +21355,27 @@
         </is>
       </c>
       <c r="F49" s="13" t="n">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="G49" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Live + HiBid webcast, 18% BP + 3% card</t>
         </is>
       </c>
       <c r="H49" s="15" t="n"/>
-      <c r="I49" s="13" t="inlineStr"/>
+      <c r="I49" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
       <c r="J49" s="13" t="inlineStr">
         <is>
-          <t>2026-11-03 11:00 AM ET</t>
+          <t>2026-10-25 01:00 PM ET</t>
         </is>
       </c>
       <c r="K49" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
       <c r="L49" s="13" t="inlineStr">
@@ -21387,7 +21383,11 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M49" s="13" t="inlineStr"/>
+      <c r="M49" s="21" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
       <c r="N49" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -21395,7 +21395,7 @@
       </c>
       <c r="O49" s="14" t="inlineStr">
         <is>
-          <t>Store inventory.</t>
+          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale.</t>
         </is>
       </c>
     </row>
@@ -21407,17 +21407,17 @@
       </c>
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>High-end deli (contents not described)</t>
+          <t>Party City (Ch. 11) store – fixtures + party merchandise inventory</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>restaurant closing</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D50" s="13" t="inlineStr">
         <is>
-          <t>Manalapan Township</t>
+          <t>East Brunswick</t>
         </is>
       </c>
       <c r="E50" s="13" t="inlineStr">
@@ -21426,32 +21426,28 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H50" s="15" t="n"/>
-      <c r="I50" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
+      <c r="I50" s="13" t="inlineStr"/>
       <c r="J50" s="13" t="inlineStr">
         <is>
-          <t>2026-10-19 04:00 PM ET</t>
+          <t>2026-11-03 11:00 AM ET</t>
         </is>
       </c>
       <c r="K50" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
-        </is>
-      </c>
-      <c r="L50" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>A.J. Willner</t>
+        </is>
+      </c>
+      <c r="L50" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M50" s="13" t="inlineStr"/>
@@ -21462,7 +21458,7 @@
       </c>
       <c r="O50" s="14" t="inlineStr">
         <is>
-          <t>Mon Oct 19 4 PM. No item description on page.</t>
+          <t>Store inventory.</t>
         </is>
       </c>
     </row>
@@ -21474,17 +21470,17 @@
       </c>
       <c r="B51" s="14" t="inlineStr">
         <is>
-          <t>Wren Kitchens showroom closing – JennAir/Café/KitchenAid/GE Profile appliances + display kitchens</t>
+          <t>High-end deli (contents not described)</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
-          <t>showroom closing</t>
+          <t>restaurant closing</t>
         </is>
       </c>
       <c r="D51" s="13" t="inlineStr">
         <is>
-          <t>Lawrenceville</t>
+          <t>Manalapan Township</t>
         </is>
       </c>
       <c r="E51" s="13" t="inlineStr">
@@ -21493,28 +21489,32 @@
         </is>
       </c>
       <c r="F51" s="13" t="n">
-        <v>239</v>
+        <v>223</v>
       </c>
       <c r="G51" s="13" t="inlineStr">
         <is>
-          <t>Online auction, 18% BP</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H51" s="15" t="n"/>
-      <c r="I51" s="13" t="inlineStr"/>
+      <c r="I51" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="J51" s="13" t="inlineStr">
         <is>
-          <t>2026-10-27 09:00 AM ET</t>
+          <t>2026-10-19 04:00 PM ET</t>
         </is>
       </c>
       <c r="K51" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
-        </is>
-      </c>
-      <c r="L51" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
+        </is>
+      </c>
+      <c r="L51" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M51" s="13" t="inlineStr"/>
@@ -21525,7 +21525,7 @@
       </c>
       <c r="O51" s="14" t="inlineStr">
         <is>
-          <t>Premium floor-model appliances; lots close from Oct 27 9 AM.</t>
+          <t>Mon Oct 19 4 PM. No item description on page.</t>
         </is>
       </c>
     </row>
@@ -21537,17 +21537,17 @@
       </c>
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>Milwaukee / Walmart / hardware store mega auction pt 3</t>
+          <t>Bakery/Cafe Somerville NJ – rack ovens, La Marzocco, food truck (~76 lots)</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D52" s="13" t="inlineStr">
         <is>
-          <t>Mount Holly</t>
+          <t>Somerville</t>
         </is>
       </c>
       <c r="E52" s="13" t="inlineStr">
@@ -21556,28 +21556,32 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>254</v>
+        <v>224</v>
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>HiBid online auction</t>
+          <t>Live webcast + online (18% BP online)</t>
         </is>
       </c>
       <c r="H52" s="15" t="n"/>
-      <c r="I52" s="13" t="inlineStr"/>
+      <c r="I52" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
       <c r="J52" s="13" t="inlineStr">
         <is>
-          <t>2026-10-19 06:00 PM ET</t>
+          <t>2026-10-26 02:00 PM ET</t>
         </is>
       </c>
       <c r="K52" s="13" t="inlineStr">
         <is>
-          <t>HiBid</t>
-        </is>
-      </c>
-      <c r="L52" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>HiBid / Best Buy Auctioneers</t>
+        </is>
+      </c>
+      <c r="L52" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M52" s="13" t="inlineStr"/>
@@ -21588,7 +21592,7 @@
       </c>
       <c r="O52" s="14" t="inlineStr">
         <is>
-          <t>Close Oct 18 or 19 6 PM (later used).</t>
+          <t>Full bakery/cafe commercial kitchen: food truck w/ pizza oven, La Marzocco espresso, Mazzer, Baxter + Empire Logiudice rack ovens, dough depositor, Globe floor mixer, Artic Air / SS refrigeration, fryers, Vitamix, Robot Coupe, display cases, dining furniture. Preview 11 AM sale day; checkout Tue 10/27.</t>
         </is>
       </c>
     </row>
@@ -21600,17 +21604,17 @@
       </c>
       <c r="B53" s="14" t="inlineStr">
         <is>
-          <t>Wren Kitchens showroom closing – GE/Whirlpool/KitchenAid/Café incl. NIB Café range + 35 kitchens</t>
+          <t>Ability to Work kitchen and store – commercial kitchen + store fixtures (~135 lots)</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>showroom closing</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D53" s="13" t="inlineStr">
         <is>
-          <t>Cherry Hill</t>
+          <t>Flemington</t>
         </is>
       </c>
       <c r="E53" s="13" t="inlineStr">
@@ -21619,23 +21623,23 @@
         </is>
       </c>
       <c r="F53" s="13" t="n">
-        <v>266</v>
+        <v>237</v>
       </c>
       <c r="G53" s="13" t="inlineStr">
         <is>
-          <t>Online auction, openers ~$0.50</t>
+          <t>Timed online (15% BP)</t>
         </is>
       </c>
       <c r="H53" s="15" t="n"/>
       <c r="I53" s="13" t="inlineStr"/>
       <c r="J53" s="13" t="inlineStr">
         <is>
-          <t>2026-11-02 11:00 AM ET</t>
+          <t>2026-10-27 11:02 AM ET</t>
         </is>
       </c>
       <c r="K53" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
+          <t>HiBid</t>
         </is>
       </c>
       <c r="L53" s="13" t="inlineStr">
@@ -21651,107 +21655,185 @@
       </c>
       <c r="O53" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Nov 2 11 AM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — NYC / Long Island / NJ</t>
-        </is>
-      </c>
-      <c r="B54" s="17" t="inlineStr">
-        <is>
-          <t>21 item(s)</t>
-        </is>
-      </c>
-      <c r="C54" s="18" t="n"/>
-      <c r="D54" s="18" t="n"/>
-      <c r="E54" s="18" t="n"/>
-      <c r="F54" s="18" t="n"/>
-      <c r="G54" s="18" t="n"/>
-      <c r="H54" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I54" s="18" t="n"/>
-      <c r="J54" s="18" t="n"/>
-      <c r="K54" s="18" t="n"/>
-      <c r="L54" s="18" t="n"/>
-      <c r="M54" s="18" t="n"/>
-      <c r="N54" s="18" t="n"/>
-      <c r="O54" s="18" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="11" t="inlineStr">
-        <is>
-          <t>▸ Eastern PA / Mid-Atlantic  (1)</t>
-        </is>
-      </c>
-      <c r="B55" s="12" t="n"/>
-      <c r="C55" s="12" t="n"/>
-      <c r="D55" s="12" t="n"/>
-      <c r="E55" s="12" t="n"/>
-      <c r="F55" s="12" t="n"/>
-      <c r="G55" s="12" t="n"/>
-      <c r="H55" s="12" t="n"/>
-      <c r="I55" s="12" t="n"/>
-      <c r="J55" s="12" t="n"/>
-      <c r="K55" s="12" t="n"/>
-      <c r="L55" s="12" t="n"/>
-      <c r="M55" s="12" t="n"/>
-      <c r="N55" s="12" t="n"/>
-      <c r="O55" s="12" t="n"/>
+          <t>Apprentice/hospitality training cafe-kitchen and store dispersal. Preview 9–11 AM sale day; removal Oct 27 noon–Oct 29.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" outlineLevel="1">
+      <c r="A54" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B54" s="14" t="inlineStr">
+        <is>
+          <t>Wren Kitchens showroom closing – JennAir/Café/KitchenAid/GE Profile appliances + display kitchens</t>
+        </is>
+      </c>
+      <c r="C54" s="13" t="inlineStr">
+        <is>
+          <t>showroom closing</t>
+        </is>
+      </c>
+      <c r="D54" s="13" t="inlineStr">
+        <is>
+          <t>Lawrenceville</t>
+        </is>
+      </c>
+      <c r="E54" s="13" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="F54" s="13" t="n">
+        <v>239</v>
+      </c>
+      <c r="G54" s="13" t="inlineStr">
+        <is>
+          <t>Online auction, 18% BP</t>
+        </is>
+      </c>
+      <c r="H54" s="15" t="n"/>
+      <c r="I54" s="13" t="inlineStr"/>
+      <c r="J54" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-27 09:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K54" s="13" t="inlineStr">
+        <is>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L54" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M54" s="13" t="inlineStr"/>
+      <c r="N54" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O54" s="14" t="inlineStr">
+        <is>
+          <t>Premium floor-model appliances; lots close from Oct 27 9 AM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" outlineLevel="1">
+      <c r="A55" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B55" s="14" t="inlineStr">
+        <is>
+          <t>Milwaukee / Walmart / hardware store mega auction pt 3</t>
+        </is>
+      </c>
+      <c r="C55" s="13" t="inlineStr">
+        <is>
+          <t>inventory</t>
+        </is>
+      </c>
+      <c r="D55" s="13" t="inlineStr">
+        <is>
+          <t>Mount Holly</t>
+        </is>
+      </c>
+      <c r="E55" s="13" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="F55" s="13" t="n">
+        <v>254</v>
+      </c>
+      <c r="G55" s="13" t="inlineStr">
+        <is>
+          <t>HiBid online auction</t>
+        </is>
+      </c>
+      <c r="H55" s="15" t="n"/>
+      <c r="I55" s="13" t="inlineStr"/>
+      <c r="J55" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 06:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K55" s="13" t="inlineStr">
+        <is>
+          <t>HiBid</t>
+        </is>
+      </c>
+      <c r="L55" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M55" s="13" t="inlineStr"/>
+      <c r="N55" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O55" s="14" t="inlineStr">
+        <is>
+          <t>Close Oct 18 or 19 6 PM (later used).</t>
+        </is>
+      </c>
     </row>
     <row r="56" outlineLevel="1">
       <c r="A56" s="13" t="inlineStr">
         <is>
-          <t>Eastern PA / Mid-Atlantic</t>
+          <t>NYC / Long Island / NJ</t>
         </is>
       </c>
       <c r="B56" s="14" t="inlineStr">
         <is>
-          <t>October restaurant consignment – Hobart, Rational, True + NEW scratch-and-dent Migali/Avantco</t>
+          <t>Wren Kitchens showroom closing – GE/Whirlpool/KitchenAid/Café incl. NIB Café range + 35 kitchens</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>showroom closing</t>
         </is>
       </c>
       <c r="D56" s="13" t="inlineStr">
         <is>
-          <t>Harrisburg</t>
+          <t>Cherry Hill</t>
         </is>
       </c>
       <c r="E56" s="13" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>340</v>
+        <v>266</v>
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>Online auction, 15% BP, ships $55/pallet</t>
+          <t>Online auction, openers ~$0.50</t>
         </is>
       </c>
       <c r="H56" s="15" t="n"/>
       <c r="I56" s="13" t="inlineStr"/>
       <c r="J56" s="13" t="inlineStr">
         <is>
-          <t>2026-10-21 11:00 AM ET</t>
+          <t>2026-11-02 11:00 AM ET</t>
         </is>
       </c>
       <c r="K56" s="13" t="inlineStr">
         <is>
-          <t>Restaurant Auction Co</t>
-        </is>
-      </c>
-      <c r="L56" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L56" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M56" s="13" t="inlineStr"/>
@@ -21762,19 +21844,19 @@
       </c>
       <c r="O56" s="14" t="inlineStr">
         <is>
-          <t>Closes Oct 21 10 or 11 AM (later used). Shippable.</t>
+          <t>Lots close from Nov 2 11 AM.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="17" t="inlineStr">
         <is>
-          <t>Subtotal — Eastern PA / Mid-Atlantic</t>
+          <t>Subtotal — NYC / Long Island / NJ</t>
         </is>
       </c>
       <c r="B57" s="17" t="inlineStr">
         <is>
-          <t>1 item(s)</t>
+          <t>24 item(s)</t>
         </is>
       </c>
       <c r="C57" s="18" t="n"/>
@@ -21796,7 +21878,7 @@
     <row r="58">
       <c r="A58" s="11" t="inlineStr">
         <is>
-          <t>▸ Upstate / Western NY  (3)</t>
+          <t>▸ Eastern PA / Mid-Atlantic  (1)</t>
         </is>
       </c>
       <c r="B58" s="12" t="n"/>
@@ -21817,12 +21899,12 @@
     <row r="59" outlineLevel="1">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>Upstate / Western NY</t>
+          <t>Eastern PA / Mid-Atlantic</t>
         </is>
       </c>
       <c r="B59" s="14" t="inlineStr">
         <is>
-          <t>Former Taco Del Mar – stainless, warmers, walk-in panels</t>
+          <t>October restaurant consignment – Hobart, Rational, True + NEW scratch-and-dent Migali/Avantco</t>
         </is>
       </c>
       <c r="C59" s="13" t="inlineStr">
@@ -21832,32 +21914,32 @@
       </c>
       <c r="D59" s="13" t="inlineStr">
         <is>
-          <t>Watson</t>
+          <t>Harrisburg</t>
         </is>
       </c>
       <c r="E59" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="F59" s="13" t="n">
-        <v>260</v>
+        <v>340</v>
       </c>
       <c r="G59" s="13" t="inlineStr">
         <is>
-          <t>HiBid online auction</t>
+          <t>Online auction, 15% BP, ships $55/pallet</t>
         </is>
       </c>
       <c r="H59" s="15" t="n"/>
       <c r="I59" s="13" t="inlineStr"/>
       <c r="J59" s="13" t="inlineStr">
         <is>
-          <t>2026-10-20 06:00 PM ET</t>
+          <t>2026-10-21 11:00 AM ET</t>
         </is>
       </c>
       <c r="K59" s="13" t="inlineStr">
         <is>
-          <t>Adirondack Asset / HiBid</t>
+          <t>Restaurant Auction Co</t>
         </is>
       </c>
       <c r="L59" s="20" t="inlineStr">
@@ -21873,228 +21955,228 @@
       </c>
       <c r="O59" s="14" t="inlineStr">
         <is>
+          <t>Closes Oct 21 10 or 11 AM (later used). Shippable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Eastern PA / Mid-Atlantic</t>
+        </is>
+      </c>
+      <c r="B60" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C60" s="18" t="n"/>
+      <c r="D60" s="18" t="n"/>
+      <c r="E60" s="18" t="n"/>
+      <c r="F60" s="18" t="n"/>
+      <c r="G60" s="18" t="n"/>
+      <c r="H60" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" s="18" t="n"/>
+      <c r="J60" s="18" t="n"/>
+      <c r="K60" s="18" t="n"/>
+      <c r="L60" s="18" t="n"/>
+      <c r="M60" s="18" t="n"/>
+      <c r="N60" s="18" t="n"/>
+      <c r="O60" s="18" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="11" t="inlineStr">
+        <is>
+          <t>▸ Upstate / Western NY  (3)</t>
+        </is>
+      </c>
+      <c r="B61" s="12" t="n"/>
+      <c r="C61" s="12" t="n"/>
+      <c r="D61" s="12" t="n"/>
+      <c r="E61" s="12" t="n"/>
+      <c r="F61" s="12" t="n"/>
+      <c r="G61" s="12" t="n"/>
+      <c r="H61" s="12" t="n"/>
+      <c r="I61" s="12" t="n"/>
+      <c r="J61" s="12" t="n"/>
+      <c r="K61" s="12" t="n"/>
+      <c r="L61" s="12" t="n"/>
+      <c r="M61" s="12" t="n"/>
+      <c r="N61" s="12" t="n"/>
+      <c r="O61" s="12" t="n"/>
+    </row>
+    <row r="62" outlineLevel="1">
+      <c r="A62" s="13" t="inlineStr">
+        <is>
+          <t>Upstate / Western NY</t>
+        </is>
+      </c>
+      <c r="B62" s="14" t="inlineStr">
+        <is>
+          <t>Former Taco Del Mar – stainless, warmers, walk-in panels</t>
+        </is>
+      </c>
+      <c r="C62" s="13" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D62" s="13" t="inlineStr">
+        <is>
+          <t>Watson</t>
+        </is>
+      </c>
+      <c r="E62" s="13" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="F62" s="13" t="n">
+        <v>260</v>
+      </c>
+      <c r="G62" s="13" t="inlineStr">
+        <is>
+          <t>HiBid online auction</t>
+        </is>
+      </c>
+      <c r="H62" s="15" t="n"/>
+      <c r="I62" s="13" t="inlineStr"/>
+      <c r="J62" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-20 06:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K62" s="13" t="inlineStr">
+        <is>
+          <t>Adirondack Asset / HiBid</t>
+        </is>
+      </c>
+      <c r="L62" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M62" s="13" t="inlineStr"/>
+      <c r="N62" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O62" s="14" t="inlineStr">
+        <is>
           <t>Small lot.</t>
         </is>
       </c>
     </row>
-    <row r="60" outlineLevel="1">
-      <c r="A60" s="13" t="inlineStr">
+    <row r="63" outlineLevel="1">
+      <c r="A63" s="13" t="inlineStr">
         <is>
           <t>Upstate / Western NY</t>
         </is>
       </c>
-      <c r="B60" s="14" t="inlineStr">
+      <c r="B63" s="14" t="inlineStr">
         <is>
           <t>Closed restaurant – coolers, fridges, prep tables</t>
         </is>
       </c>
-      <c r="C60" s="13" t="inlineStr">
+      <c r="C63" s="13" t="inlineStr">
         <is>
           <t>restaurant</t>
         </is>
       </c>
-      <c r="D60" s="13" t="inlineStr">
+      <c r="D63" s="13" t="inlineStr">
         <is>
           <t>Palmyra</t>
         </is>
       </c>
-      <c r="E60" s="13" t="inlineStr">
+      <c r="E63" s="13" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
       </c>
-      <c r="F60" s="13" t="n">
+      <c r="F63" s="13" t="n">
         <v>333</v>
       </c>
-      <c r="G60" s="13" t="inlineStr">
+      <c r="G63" s="13" t="inlineStr">
         <is>
           <t>HiBid, 15% BP</t>
         </is>
       </c>
-      <c r="H60" s="15" t="n"/>
-      <c r="I60" s="13" t="inlineStr"/>
-      <c r="J60" s="13" t="inlineStr">
+      <c r="H63" s="15" t="n"/>
+      <c r="I63" s="13" t="inlineStr"/>
+      <c r="J63" s="13" t="inlineStr">
         <is>
           <t>2026-10-19 07:00 PM ET</t>
         </is>
       </c>
-      <c r="K60" s="13" t="inlineStr">
+      <c r="K63" s="13" t="inlineStr">
         <is>
           <t>Reynolds Auction Co / HiBid</t>
         </is>
       </c>
-      <c r="L60" s="20" t="inlineStr">
+      <c r="L63" s="20" t="inlineStr">
         <is>
           <t>ENDING SOON</t>
         </is>
       </c>
-      <c r="M60" s="13" t="inlineStr"/>
-      <c r="N60" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O60" s="14" t="inlineStr">
+      <c r="M63" s="13" t="inlineStr"/>
+      <c r="N63" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O63" s="14" t="inlineStr">
         <is>
           <t>No new out-of-state bidders. Small.</t>
         </is>
       </c>
-    </row>
-    <row r="61" outlineLevel="1">
-      <c r="A61" s="13" t="inlineStr">
-        <is>
-          <t>Upstate / Western NY</t>
-        </is>
-      </c>
-      <c r="B61" s="14" t="inlineStr">
-        <is>
-          <t>Restaurant &amp; fitness equipment</t>
-        </is>
-      </c>
-      <c r="C61" s="13" t="inlineStr">
-        <is>
-          <t>restaurant</t>
-        </is>
-      </c>
-      <c r="D61" s="13" t="inlineStr">
-        <is>
-          <t>Williamsville</t>
-        </is>
-      </c>
-      <c r="E61" s="13" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="F61" s="13" t="n">
-        <v>408</v>
-      </c>
-      <c r="G61" s="13" t="inlineStr">
-        <is>
-          <t>Online auction</t>
-        </is>
-      </c>
-      <c r="H61" s="15" t="n"/>
-      <c r="I61" s="13" t="inlineStr"/>
-      <c r="J61" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26 07:30 PM ET</t>
-        </is>
-      </c>
-      <c r="K61" s="13" t="inlineStr">
-        <is>
-          <t>Cash Auctions</t>
-        </is>
-      </c>
-      <c r="L61" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M61" s="13" t="inlineStr"/>
-      <c r="N61" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O61" s="14" t="inlineStr">
-        <is>
-          <t>Lots not reviewed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Upstate / Western NY</t>
-        </is>
-      </c>
-      <c r="B62" s="17" t="inlineStr">
-        <is>
-          <t>3 item(s)</t>
-        </is>
-      </c>
-      <c r="C62" s="18" t="n"/>
-      <c r="D62" s="18" t="n"/>
-      <c r="E62" s="18" t="n"/>
-      <c r="F62" s="18" t="n"/>
-      <c r="G62" s="18" t="n"/>
-      <c r="H62" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I62" s="18" t="n"/>
-      <c r="J62" s="18" t="n"/>
-      <c r="K62" s="18" t="n"/>
-      <c r="L62" s="18" t="n"/>
-      <c r="M62" s="18" t="n"/>
-      <c r="N62" s="18" t="n"/>
-      <c r="O62" s="18" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="11" t="inlineStr">
-        <is>
-          <t>▸ Virginia  (1)</t>
-        </is>
-      </c>
-      <c r="B63" s="12" t="n"/>
-      <c r="C63" s="12" t="n"/>
-      <c r="D63" s="12" t="n"/>
-      <c r="E63" s="12" t="n"/>
-      <c r="F63" s="12" t="n"/>
-      <c r="G63" s="12" t="n"/>
-      <c r="H63" s="12" t="n"/>
-      <c r="I63" s="12" t="n"/>
-      <c r="J63" s="12" t="n"/>
-      <c r="K63" s="12" t="n"/>
-      <c r="L63" s="12" t="n"/>
-      <c r="M63" s="12" t="n"/>
-      <c r="N63" s="12" t="n"/>
-      <c r="O63" s="12" t="n"/>
     </row>
     <row r="64" outlineLevel="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>Virginia</t>
+          <t>Upstate / Western NY</t>
         </is>
       </c>
       <c r="B64" s="14" t="inlineStr">
         <is>
-          <t>Haynes Furniture / The Dump – 12 stores closing (furniture, mattresses)</t>
+          <t>Restaurant &amp; fitness equipment</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>retail GOB</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D64" s="13" t="inlineStr">
         <is>
-          <t>Virginia Beach</t>
+          <t>Williamsville</t>
         </is>
       </c>
       <c r="E64" s="13" t="inlineStr">
         <is>
-          <t>VA</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F64" s="13" t="n">
-        <v>456</v>
+        <v>408</v>
       </c>
       <c r="G64" s="13" t="inlineStr">
         <is>
-          <t>Retail GOB markdowns</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H64" s="15" t="n"/>
-      <c r="I64" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="J64" s="13" t="inlineStr"/>
+      <c r="I64" s="13" t="inlineStr"/>
+      <c r="J64" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-26 07:30 PM ET</t>
+        </is>
+      </c>
       <c r="K64" s="13" t="inlineStr">
         <is>
-          <t>SB360 (PR Newswire)</t>
+          <t>Cash Auctions</t>
         </is>
       </c>
       <c r="L64" s="13" t="inlineStr">
@@ -22110,19 +22192,19 @@
       </c>
       <c r="O64" s="14" t="inlineStr">
         <is>
-          <t>Posted Oct 8. Multi-state (VA/AZ/GA/IL/TX); pinned at Virginia Beach. Home goods only.</t>
+          <t>Lots not reviewed.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="17" t="inlineStr">
         <is>
-          <t>Subtotal — Virginia</t>
+          <t>Subtotal — Upstate / Western NY</t>
         </is>
       </c>
       <c r="B65" s="17" t="inlineStr">
         <is>
-          <t>1 item(s)</t>
+          <t>3 item(s)</t>
         </is>
       </c>
       <c r="C65" s="18" t="n"/>
@@ -22144,7 +22226,7 @@
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
         <is>
-          <t>▸ Midwest  (2)</t>
+          <t>▸ Virginia  (1)</t>
         </is>
       </c>
       <c r="B66" s="12" t="n"/>
@@ -22165,52 +22247,52 @@
     <row r="67" outlineLevel="1">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>Virginia</t>
         </is>
       </c>
       <c r="B67" s="14" t="inlineStr">
         <is>
-          <t>Freshway Market whole-grocery liquidation – refrigeration racks, cases, walk-ins, generator</t>
+          <t>Haynes Furniture / The Dump – 12 stores closing (furniture, mattresses)</t>
         </is>
       </c>
       <c r="C67" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>retail GOB</t>
         </is>
       </c>
       <c r="D67" s="13" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Virginia Beach</t>
         </is>
       </c>
       <c r="E67" s="13" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>VA</t>
         </is>
       </c>
       <c r="F67" s="13" t="n">
-        <v>862</v>
+        <v>456</v>
       </c>
       <c r="G67" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Retail GOB markdowns</t>
         </is>
       </c>
       <c r="H67" s="15" t="n"/>
-      <c r="I67" s="13" t="inlineStr"/>
-      <c r="J67" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-20 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="I67" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="J67" s="13" t="inlineStr"/>
       <c r="K67" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
-        </is>
-      </c>
-      <c r="L67" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>SB360 (PR Newswire)</t>
+        </is>
+      </c>
+      <c r="L67" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M67" s="13" t="inlineStr"/>
@@ -22221,165 +22303,165 @@
       </c>
       <c r="O67" s="14" t="inlineStr">
         <is>
+          <t>Posted Oct 8. Multi-state (VA/AZ/GA/IL/TX); pinned at Virginia Beach. Home goods only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Virginia</t>
+        </is>
+      </c>
+      <c r="B68" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C68" s="18" t="n"/>
+      <c r="D68" s="18" t="n"/>
+      <c r="E68" s="18" t="n"/>
+      <c r="F68" s="18" t="n"/>
+      <c r="G68" s="18" t="n"/>
+      <c r="H68" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" s="18" t="n"/>
+      <c r="J68" s="18" t="n"/>
+      <c r="K68" s="18" t="n"/>
+      <c r="L68" s="18" t="n"/>
+      <c r="M68" s="18" t="n"/>
+      <c r="N68" s="18" t="n"/>
+      <c r="O68" s="18" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="11" t="inlineStr">
+        <is>
+          <t>▸ Midwest  (2)</t>
+        </is>
+      </c>
+      <c r="B69" s="12" t="n"/>
+      <c r="C69" s="12" t="n"/>
+      <c r="D69" s="12" t="n"/>
+      <c r="E69" s="12" t="n"/>
+      <c r="F69" s="12" t="n"/>
+      <c r="G69" s="12" t="n"/>
+      <c r="H69" s="12" t="n"/>
+      <c r="I69" s="12" t="n"/>
+      <c r="J69" s="12" t="n"/>
+      <c r="K69" s="12" t="n"/>
+      <c r="L69" s="12" t="n"/>
+      <c r="M69" s="12" t="n"/>
+      <c r="N69" s="12" t="n"/>
+      <c r="O69" s="12" t="n"/>
+    </row>
+    <row r="70" outlineLevel="1">
+      <c r="A70" s="13" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="B70" s="14" t="inlineStr">
+        <is>
+          <t>Freshway Market whole-grocery liquidation – refrigeration racks, cases, walk-ins, generator</t>
+        </is>
+      </c>
+      <c r="C70" s="13" t="inlineStr">
+        <is>
+          <t>store closing</t>
+        </is>
+      </c>
+      <c r="D70" s="13" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="E70" s="13" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="F70" s="13" t="n">
+        <v>862</v>
+      </c>
+      <c r="G70" s="13" t="inlineStr">
+        <is>
+          <t>Online auction</t>
+        </is>
+      </c>
+      <c r="H70" s="15" t="n"/>
+      <c r="I70" s="13" t="inlineStr"/>
+      <c r="J70" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-20 11:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K70" s="13" t="inlineStr">
+        <is>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L70" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M70" s="13" t="inlineStr"/>
+      <c r="N70" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O70" s="14" t="inlineStr">
+        <is>
           <t>Closes from Oct 20 10 AM CDT.</t>
         </is>
       </c>
-    </row>
-    <row r="68" outlineLevel="1">
-      <c r="A68" s="13" t="inlineStr">
-        <is>
-          <t>Midwest</t>
-        </is>
-      </c>
-      <c r="B68" s="14" t="inlineStr">
-        <is>
-          <t>American Sale – total liquidation, all 7 stores (pools, hot tubs, grills, holiday decor)</t>
-        </is>
-      </c>
-      <c r="C68" s="13" t="inlineStr">
-        <is>
-          <t>retail GOB</t>
-        </is>
-      </c>
-      <c r="D68" s="13" t="inlineStr">
-        <is>
-          <t>Chicagoland</t>
-        </is>
-      </c>
-      <c r="E68" s="13" t="inlineStr">
-        <is>
-          <t>IL</t>
-        </is>
-      </c>
-      <c r="F68" s="13" t="n">
-        <v>876</v>
-      </c>
-      <c r="G68" s="13" t="inlineStr">
-        <is>
-          <t>Retail GOB, up to 70% off</t>
-        </is>
-      </c>
-      <c r="H68" s="15" t="n"/>
-      <c r="I68" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="J68" s="13" t="inlineStr"/>
-      <c r="K68" s="13" t="inlineStr">
-        <is>
-          <t>Tiger Group (PR Newswire)</t>
-        </is>
-      </c>
-      <c r="L68" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M68" s="13" t="inlineStr"/>
-      <c r="N68" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O68" s="14" t="inlineStr">
-        <is>
-          <t>Posted Oct 15. Watch for a bulk/fixture auction.</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Midwest</t>
-        </is>
-      </c>
-      <c r="B69" s="17" t="inlineStr">
-        <is>
-          <t>2 item(s)</t>
-        </is>
-      </c>
-      <c r="C69" s="18" t="n"/>
-      <c r="D69" s="18" t="n"/>
-      <c r="E69" s="18" t="n"/>
-      <c r="F69" s="18" t="n"/>
-      <c r="G69" s="18" t="n"/>
-      <c r="H69" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I69" s="18" t="n"/>
-      <c r="J69" s="18" t="n"/>
-      <c r="K69" s="18" t="n"/>
-      <c r="L69" s="18" t="n"/>
-      <c r="M69" s="18" t="n"/>
-      <c r="N69" s="18" t="n"/>
-      <c r="O69" s="18" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="11" t="inlineStr">
-        <is>
-          <t>▸ Texas / South Central  (1)</t>
-        </is>
-      </c>
-      <c r="B70" s="12" t="n"/>
-      <c r="C70" s="12" t="n"/>
-      <c r="D70" s="12" t="n"/>
-      <c r="E70" s="12" t="n"/>
-      <c r="F70" s="12" t="n"/>
-      <c r="G70" s="12" t="n"/>
-      <c r="H70" s="12" t="n"/>
-      <c r="I70" s="12" t="n"/>
-      <c r="J70" s="12" t="n"/>
-      <c r="K70" s="12" t="n"/>
-      <c r="L70" s="12" t="n"/>
-      <c r="M70" s="12" t="n"/>
-      <c r="N70" s="12" t="n"/>
-      <c r="O70" s="12" t="n"/>
     </row>
     <row r="71" outlineLevel="1">
       <c r="A71" s="13" t="inlineStr">
         <is>
-          <t>Texas / South Central</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="B71" s="14" t="inlineStr">
         <is>
-          <t>Southwest beverage distributor surplus – mostly unused: 16 True merchandisers, 75 Bunn brewers, 100+ micro-market kiosks</t>
+          <t>American Sale – total liquidation, all 7 stores (pools, hot tubs, grills, holiday decor)</t>
         </is>
       </c>
       <c r="C71" s="13" t="inlineStr">
         <is>
-          <t>distributor surplus</t>
+          <t>retail GOB</t>
         </is>
       </c>
       <c r="D71" s="13" t="inlineStr">
         <is>
-          <t>Mesquite</t>
+          <t>Chicagoland</t>
         </is>
       </c>
       <c r="E71" s="13" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="F71" s="13" t="n">
-        <v>1547</v>
+        <v>876</v>
       </c>
       <c r="G71" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Retail GOB, up to 70% off</t>
         </is>
       </c>
       <c r="H71" s="15" t="n"/>
-      <c r="I71" s="13" t="inlineStr"/>
-      <c r="J71" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-13 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="I71" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="J71" s="13" t="inlineStr"/>
       <c r="K71" s="13" t="inlineStr">
         <is>
-          <t>Heritage Global Partners</t>
+          <t>Tiger Group (PR Newswire)</t>
         </is>
       </c>
       <c r="L71" s="13" t="inlineStr">
@@ -22395,19 +22477,19 @@
       </c>
       <c r="O71" s="14" t="inlineStr">
         <is>
-          <t>Near-new appliances, resell by unit. Nov 13 10 AM CST.</t>
+          <t>Posted Oct 15. Watch for a bulk/fixture auction.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="17" t="inlineStr">
         <is>
-          <t>Subtotal — Texas / South Central</t>
+          <t>Subtotal — Midwest</t>
         </is>
       </c>
       <c r="B72" s="17" t="inlineStr">
         <is>
-          <t>1 item(s)</t>
+          <t>2 item(s)</t>
         </is>
       </c>
       <c r="C72" s="18" t="n"/>
@@ -22429,7 +22511,7 @@
     <row r="73">
       <c r="A73" s="11" t="inlineStr">
         <is>
-          <t>▸ West / Other  (1)</t>
+          <t>▸ Texas / South Central  (1)</t>
         </is>
       </c>
       <c r="B73" s="12" t="n"/>
@@ -22450,47 +22532,47 @@
     <row r="74" outlineLevel="1">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>West / Other</t>
+          <t>Texas / South Central</t>
         </is>
       </c>
       <c r="B74" s="14" t="inlineStr">
         <is>
-          <t>National salad concept liquidation – full contents of 63 fast-casual restaurants (AZ/TX/OK/NV)</t>
+          <t>Southwest beverage distributor surplus – mostly unused: 16 True merchandisers, 75 Bunn brewers, 100+ micro-market kiosks</t>
         </is>
       </c>
       <c r="C74" s="13" t="inlineStr">
         <is>
-          <t>restaurant chain liquidation</t>
+          <t>distributor surplus</t>
         </is>
       </c>
       <c r="D74" s="13" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Mesquite</t>
         </is>
       </c>
       <c r="E74" s="13" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="F74" s="13" t="n">
-        <v>2307</v>
+        <v>1547</v>
       </c>
       <c r="G74" s="13" t="inlineStr">
         <is>
-          <t>Online auctions, dates TBD</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H74" s="15" t="n"/>
-      <c r="I74" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="J74" s="13" t="inlineStr"/>
+      <c r="I74" s="13" t="inlineStr"/>
+      <c r="J74" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-13 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K74" s="13" t="inlineStr">
         <is>
-          <t>RestaurantEquipment.bid (TAGeX)</t>
+          <t>Heritage Global Partners</t>
         </is>
       </c>
       <c r="L74" s="13" t="inlineStr">
@@ -22506,14 +22588,14 @@
       </c>
       <c r="O74" s="14" t="inlineStr">
         <is>
-          <t>Rolling market-by-market auctions, none live yet (Phoenix metro 30 locations, DFW 14, Tucson 6, Houston 5, plus OK/NV). Pickup on site at each restaurant. Pinned at Phoenix.</t>
+          <t>Near-new appliances, resell by unit. Nov 13 10 AM CST.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="17" t="inlineStr">
         <is>
-          <t>Subtotal — West / Other</t>
+          <t>Subtotal — Texas / South Central</t>
         </is>
       </c>
       <c r="B75" s="17" t="inlineStr">
@@ -22537,24 +22619,135 @@
       <c r="N75" s="18" t="n"/>
       <c r="O75" s="18" t="n"/>
     </row>
+    <row r="76">
+      <c r="A76" s="11" t="inlineStr">
+        <is>
+          <t>▸ West / Other  (1)</t>
+        </is>
+      </c>
+      <c r="B76" s="12" t="n"/>
+      <c r="C76" s="12" t="n"/>
+      <c r="D76" s="12" t="n"/>
+      <c r="E76" s="12" t="n"/>
+      <c r="F76" s="12" t="n"/>
+      <c r="G76" s="12" t="n"/>
+      <c r="H76" s="12" t="n"/>
+      <c r="I76" s="12" t="n"/>
+      <c r="J76" s="12" t="n"/>
+      <c r="K76" s="12" t="n"/>
+      <c r="L76" s="12" t="n"/>
+      <c r="M76" s="12" t="n"/>
+      <c r="N76" s="12" t="n"/>
+      <c r="O76" s="12" t="n"/>
+    </row>
+    <row r="77" outlineLevel="1">
+      <c r="A77" s="13" t="inlineStr">
+        <is>
+          <t>West / Other</t>
+        </is>
+      </c>
+      <c r="B77" s="14" t="inlineStr">
+        <is>
+          <t>National salad concept liquidation – full contents of 63 fast-casual restaurants (AZ/TX/OK/NV)</t>
+        </is>
+      </c>
+      <c r="C77" s="13" t="inlineStr">
+        <is>
+          <t>restaurant chain liquidation</t>
+        </is>
+      </c>
+      <c r="D77" s="13" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="E77" s="13" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="F77" s="13" t="n">
+        <v>2307</v>
+      </c>
+      <c r="G77" s="13" t="inlineStr">
+        <is>
+          <t>Online auctions, dates TBD</t>
+        </is>
+      </c>
+      <c r="H77" s="15" t="n"/>
+      <c r="I77" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="J77" s="13" t="inlineStr"/>
+      <c r="K77" s="13" t="inlineStr">
+        <is>
+          <t>RestaurantEquipment.bid (TAGeX)</t>
+        </is>
+      </c>
+      <c r="L77" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M77" s="13" t="inlineStr"/>
+      <c r="N77" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O77" s="14" t="inlineStr">
+        <is>
+          <t>Rolling market-by-market auctions, none live yet (Phoenix metro 30 locations, DFW 14, Tucson 6, Houston 5, plus OK/NV). Pickup on site at each restaurant. Pinned at Phoenix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — West / Other</t>
+        </is>
+      </c>
+      <c r="B78" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C78" s="18" t="n"/>
+      <c r="D78" s="18" t="n"/>
+      <c r="E78" s="18" t="n"/>
+      <c r="F78" s="18" t="n"/>
+      <c r="G78" s="18" t="n"/>
+      <c r="H78" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I78" s="18" t="n"/>
+      <c r="J78" s="18" t="n"/>
+      <c r="K78" s="18" t="n"/>
+      <c r="L78" s="18" t="n"/>
+      <c r="M78" s="18" t="n"/>
+      <c r="N78" s="18" t="n"/>
+      <c r="O78" s="18" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O75"/>
+  <autoFilter ref="A1:O78"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId18"/>
@@ -22581,15 +22774,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N51" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N52" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N53" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N56" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N59" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N60" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N61" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N64" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N67" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N68" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N71" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N74" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N54" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N55" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N56" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N59" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N62" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N63" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N64" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N67" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N70" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N71" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N74" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N77" r:id="rId53"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -22601,7 +22797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -22895,7 +23091,7 @@
       </c>
       <c r="O4" s="14" t="inlineStr">
         <is>
-          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed]</t>
+          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -22960,17 +23156,81 @@
       </c>
       <c r="O5" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Greater Boston / South Shore (&lt;50mi)</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Closed Best Buy Outlet – pallet racking, Big Joe order pickers, appliance dollies, carts, cages</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>store closing fixtures</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Brockton</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>Racking $40/upright, $80/level; pickers $1,000 OBO</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="n"/>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="J6" s="13" t="inlineStr"/>
+      <c r="K6" s="13" t="inlineStr">
+        <is>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L6" s="13" t="inlineStr">
+        <is>
+          <t>REMOVED</t>
+        </is>
+      </c>
+      <c r="M6" s="13" t="inlineStr"/>
+      <c r="N6" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O6" s="14" t="inlineStr">
+        <is>
+          <t>200 Westgate Dr. Fixtures/equipment only, no merchandise. On site daily. CL deleted by author (HTTP 410) as of 2026-10-19 midday recheck.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O5"/>
+  <autoFilter ref="A1:O6"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Lot Recon 2026-10-19 2pm ET: +2 business liquidations (Bridgeport CT fab shop, St. Louis Straub's), prune ended Oola Bowls + Auctionfuel 785897
</commit_message>
<xml_diff>
--- a/lot_recon.xlsx
+++ b/lot_recon.xlsx
@@ -16,12 +16,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Removed" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Appliance Parts'!$A$1:$O$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Appliance Parts'!$A$1:$O$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wolf New'!$A$1:$O$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Wolf Used'!$A$1:$O$189</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Wolf Unclear'!$A$1:$O$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$78</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 2026-10-19 11:11 ET</t>
+          <t>Last updated: 2026-10-19 14:04 ET</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Active listings: 294 · Removed: 5</t>
+          <t>Active listings: 293 · Removed: 8</t>
         </is>
       </c>
     </row>
@@ -641,13 +641,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>159696</v>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F8" t="n">
         <v>34</v>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C13" s="7" t="n">
         <v>980432.58</v>
@@ -956,7 +956,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C22" t="n">
         <v>0</v>
@@ -971,7 +971,7 @@
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H22" s="6" t="n">
         <v>0</v>
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C23" t="n">
         <v>1</v>
@@ -1004,7 +1004,7 @@
         <v>4</v>
       </c>
       <c r="G23" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H23" s="6" t="n">
         <v>64740</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C24" t="n">
         <v>1</v>
@@ -1037,7 +1037,7 @@
         <v>24</v>
       </c>
       <c r="G24" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H24" s="6" t="n">
         <v>440141</v>
@@ -1187,10 +1187,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C30" t="n">
         <v>2</v>
@@ -1235,14 +1235,14 @@
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H30" s="6" t="n">
         <v>5</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>743–876</t>
+          <t>743–1046</t>
         </is>
       </c>
     </row>
@@ -1396,7 +1396,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O43"/>
+  <dimension ref="A1:O42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2227,7 +2227,7 @@
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>▸ Southeast  (5)</t>
+          <t>▸ Southeast  (4)</t>
         </is>
       </c>
       <c r="B21" s="12" t="n"/>
@@ -2318,12 +2318,12 @@
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>Auctionfuel returns catalog – 100+ single appliance-part lots (Louisville)</t>
+          <t>[SMALL] Whirlpool parts assortment</t>
         </is>
       </c>
       <c r="C23" s="13" t="inlineStr">
         <is>
-          <t>auction catalog</t>
+          <t>small lot</t>
         </is>
       </c>
       <c r="D23" s="13" t="inlineStr">
@@ -2341,26 +2341,20 @@
       </c>
       <c r="G23" s="13" t="inlineStr">
         <is>
-          <t>$0–1 openers + 15% BP + $1/lot</t>
-        </is>
-      </c>
-      <c r="H23" s="15" t="n">
-        <v>0</v>
-      </c>
+          <t>Price n/a</t>
+        </is>
+      </c>
+      <c r="H23" s="15" t="n"/>
       <c r="I23" s="13" t="inlineStr"/>
-      <c r="J23" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-19 02:00 PM ET</t>
-        </is>
-      </c>
+      <c r="J23" s="13" t="inlineStr"/>
       <c r="K23" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Auctionfuel)</t>
-        </is>
-      </c>
-      <c r="L23" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L23" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M23" s="13" t="inlineStr"/>
@@ -2371,7 +2365,7 @@
       </c>
       <c r="O23" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 19 2 PM ET.</t>
+          <t>Small lead.</t>
         </is>
       </c>
     </row>
@@ -2383,43 +2377,53 @@
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>[SMALL] Whirlpool parts assortment</t>
+          <t>Misc. appliance parts pallet (parts only)</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>small lot</t>
+          <t>auction pallet</t>
         </is>
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>Dalton</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>832</v>
+        <v>917</v>
       </c>
       <c r="G24" s="13" t="inlineStr">
         <is>
-          <t>Price n/a</t>
-        </is>
-      </c>
-      <c r="H24" s="15" t="n"/>
-      <c r="I24" s="13" t="inlineStr"/>
-      <c r="J24" s="13" t="inlineStr"/>
+          <t>$50 high bid + 15% BP</t>
+        </is>
+      </c>
+      <c r="H24" s="15" t="n">
+        <v>50</v>
+      </c>
+      <c r="I24" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="J24" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 09:18 PM ET</t>
+        </is>
+      </c>
       <c r="K24" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
-        </is>
-      </c>
-      <c r="L24" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>HiBid</t>
+        </is>
+      </c>
+      <c r="L24" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M24" s="13" t="inlineStr"/>
@@ -2430,7 +2434,7 @@
       </c>
       <c r="O24" s="14" t="inlineStr">
         <is>
-          <t>Small lead.</t>
+          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18.</t>
         </is>
       </c>
     </row>
@@ -2442,53 +2446,47 @@
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>Misc. appliance parts pallet (parts only)</t>
+          <t>Established appliance sales / parts / service business</t>
         </is>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>auction pallet</t>
+          <t>business sale</t>
         </is>
       </c>
       <c r="D25" s="13" t="inlineStr">
         <is>
-          <t>Dalton</t>
+          <t>Oakland Park</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>917</v>
+        <v>1222</v>
       </c>
       <c r="G25" s="13" t="inlineStr">
         <is>
-          <t>$50 high bid + 15% BP</t>
-        </is>
-      </c>
-      <c r="H25" s="15" t="n">
-        <v>50</v>
-      </c>
+          <t>Price n/a</t>
+        </is>
+      </c>
+      <c r="H25" s="15" t="n"/>
       <c r="I25" s="13" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="J25" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-19 09:18 PM ET</t>
-        </is>
-      </c>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="J25" s="13" t="inlineStr"/>
       <c r="K25" s="13" t="inlineStr">
         <is>
-          <t>HiBid</t>
-        </is>
-      </c>
-      <c r="L25" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L25" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M25" s="13" t="inlineStr"/>
@@ -2499,120 +2497,122 @@
       </c>
       <c r="O25" s="14" t="inlineStr">
         <is>
-          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" outlineLevel="1">
-      <c r="A26" s="13" t="inlineStr">
-        <is>
-          <t>Southeast</t>
-        </is>
-      </c>
-      <c r="B26" s="14" t="inlineStr">
-        <is>
-          <t>Established appliance sales / parts / service business</t>
-        </is>
-      </c>
-      <c r="C26" s="13" t="inlineStr">
-        <is>
-          <t>business sale</t>
-        </is>
-      </c>
-      <c r="D26" s="13" t="inlineStr">
-        <is>
-          <t>Oakland Park</t>
-        </is>
-      </c>
-      <c r="E26" s="13" t="inlineStr">
-        <is>
-          <t>FL</t>
-        </is>
-      </c>
-      <c r="F26" s="13" t="n">
-        <v>1222</v>
-      </c>
-      <c r="G26" s="13" t="inlineStr">
-        <is>
-          <t>Price n/a</t>
-        </is>
-      </c>
-      <c r="H26" s="15" t="n"/>
-      <c r="I26" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="J26" s="13" t="inlineStr"/>
-      <c r="K26" s="13" t="inlineStr">
-        <is>
-          <t>Craigslist</t>
-        </is>
-      </c>
-      <c r="L26" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M26" s="13" t="inlineStr"/>
-      <c r="N26" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O26" s="14" t="inlineStr">
-        <is>
           <t>Whole business sale (Fort Lauderdale area).</t>
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Southeast</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>4 item(s)</t>
+        </is>
+      </c>
+      <c r="C26" s="18" t="n"/>
+      <c r="D26" s="18" t="n"/>
+      <c r="E26" s="18" t="n"/>
+      <c r="F26" s="18" t="n"/>
+      <c r="G26" s="18" t="n"/>
+      <c r="H26" s="19" t="n">
+        <v>36050</v>
+      </c>
+      <c r="I26" s="18" t="n"/>
+      <c r="J26" s="18" t="n"/>
+      <c r="K26" s="18" t="n"/>
+      <c r="L26" s="18" t="n"/>
+      <c r="M26" s="18" t="n"/>
+      <c r="N26" s="18" t="n"/>
+      <c r="O26" s="18" t="n"/>
+    </row>
     <row r="27">
-      <c r="A27" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Southeast</t>
-        </is>
-      </c>
-      <c r="B27" s="17" t="inlineStr">
-        <is>
-          <t>5 item(s)</t>
-        </is>
-      </c>
-      <c r="C27" s="18" t="n"/>
-      <c r="D27" s="18" t="n"/>
-      <c r="E27" s="18" t="n"/>
-      <c r="F27" s="18" t="n"/>
-      <c r="G27" s="18" t="n"/>
-      <c r="H27" s="19" t="n">
-        <v>36050</v>
-      </c>
-      <c r="I27" s="18" t="n"/>
-      <c r="J27" s="18" t="n"/>
-      <c r="K27" s="18" t="n"/>
-      <c r="L27" s="18" t="n"/>
-      <c r="M27" s="18" t="n"/>
-      <c r="N27" s="18" t="n"/>
-      <c r="O27" s="18" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="11" t="inlineStr">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>▸ Midwest  (2)</t>
         </is>
       </c>
-      <c r="B28" s="12" t="n"/>
-      <c r="C28" s="12" t="n"/>
-      <c r="D28" s="12" t="n"/>
-      <c r="E28" s="12" t="n"/>
-      <c r="F28" s="12" t="n"/>
-      <c r="G28" s="12" t="n"/>
-      <c r="H28" s="12" t="n"/>
-      <c r="I28" s="12" t="n"/>
-      <c r="J28" s="12" t="n"/>
-      <c r="K28" s="12" t="n"/>
-      <c r="L28" s="12" t="n"/>
-      <c r="M28" s="12" t="n"/>
-      <c r="N28" s="12" t="n"/>
-      <c r="O28" s="12" t="n"/>
+      <c r="B27" s="12" t="n"/>
+      <c r="C27" s="12" t="n"/>
+      <c r="D27" s="12" t="n"/>
+      <c r="E27" s="12" t="n"/>
+      <c r="F27" s="12" t="n"/>
+      <c r="G27" s="12" t="n"/>
+      <c r="H27" s="12" t="n"/>
+      <c r="I27" s="12" t="n"/>
+      <c r="J27" s="12" t="n"/>
+      <c r="K27" s="12" t="n"/>
+      <c r="L27" s="12" t="n"/>
+      <c r="M27" s="12" t="n"/>
+      <c r="N27" s="12" t="n"/>
+      <c r="O27" s="12" t="n"/>
+    </row>
+    <row r="28" outlineLevel="1">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>Auctionfuel returns catalog – 100+ single appliance-part lots (Fort Wayne)</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>auction catalog</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
+        <is>
+          <t>Fort Wayne</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="n">
+        <v>743</v>
+      </c>
+      <c r="G28" s="13" t="inlineStr">
+        <is>
+          <t>$0–1 openers + 15% BP + $1/lot</t>
+        </is>
+      </c>
+      <c r="H28" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="13" t="inlineStr"/>
+      <c r="J28" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-20 02:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K28" s="13" t="inlineStr">
+        <is>
+          <t>HiBid (Auctionfuel)</t>
+        </is>
+      </c>
+      <c r="L28" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M28" s="13" t="inlineStr"/>
+      <c r="N28" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O28" s="14" t="inlineStr">
+        <is>
+          <t>Lots close from Oct 20 2 PM ET.</t>
+        </is>
+      </c>
     </row>
     <row r="29" outlineLevel="1">
       <c r="A29" s="13" t="inlineStr">
@@ -2622,7 +2622,7 @@
       </c>
       <c r="B29" s="14" t="inlineStr">
         <is>
-          <t>Auctionfuel returns catalog – 100+ single appliance-part lots (Fort Wayne)</t>
+          <t>Auctionfuel returns catalog – 100+ single appliance-part lots (Indianapolis)</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
@@ -2632,7 +2632,7 @@
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>Fort Wayne</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="E29" s="13" t="inlineStr">
@@ -2641,7 +2641,7 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>743</v>
+        <v>816</v>
       </c>
       <c r="G29" s="13" t="inlineStr">
         <is>
@@ -2654,7 +2654,7 @@
       <c r="I29" s="13" t="inlineStr"/>
       <c r="J29" s="13" t="inlineStr">
         <is>
-          <t>2026-10-20 02:00 PM ET</t>
+          <t>2026-10-21 02:00 PM ET</t>
         </is>
       </c>
       <c r="K29" s="13" t="inlineStr">
@@ -2675,122 +2675,120 @@
       </c>
       <c r="O29" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 20 2 PM ET.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" outlineLevel="1">
-      <c r="A30" s="13" t="inlineStr">
-        <is>
-          <t>Midwest</t>
-        </is>
-      </c>
-      <c r="B30" s="14" t="inlineStr">
-        <is>
-          <t>Auctionfuel returns catalog – 100+ single appliance-part lots (Indianapolis)</t>
-        </is>
-      </c>
-      <c r="C30" s="13" t="inlineStr">
-        <is>
-          <t>auction catalog</t>
-        </is>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
-        <is>
-          <t>Indianapolis</t>
-        </is>
-      </c>
-      <c r="E30" s="13" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="F30" s="13" t="n">
-        <v>816</v>
-      </c>
-      <c r="G30" s="13" t="inlineStr">
-        <is>
-          <t>$0–1 openers + 15% BP + $1/lot</t>
-        </is>
-      </c>
-      <c r="H30" s="15" t="n">
+          <t>Lots close in sequence from Oct 21 2 PM ET.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Midwest</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>2 item(s)</t>
+        </is>
+      </c>
+      <c r="C30" s="18" t="n"/>
+      <c r="D30" s="18" t="n"/>
+      <c r="E30" s="18" t="n"/>
+      <c r="F30" s="18" t="n"/>
+      <c r="G30" s="18" t="n"/>
+      <c r="H30" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I30" s="13" t="inlineStr"/>
-      <c r="J30" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-21 02:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K30" s="13" t="inlineStr">
-        <is>
-          <t>HiBid (Auctionfuel)</t>
-        </is>
-      </c>
-      <c r="L30" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
-        </is>
-      </c>
-      <c r="M30" s="13" t="inlineStr"/>
-      <c r="N30" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O30" s="14" t="inlineStr">
-        <is>
-          <t>Lots close in sequence from Oct 21 2 PM ET.</t>
-        </is>
-      </c>
+      <c r="I30" s="18" t="n"/>
+      <c r="J30" s="18" t="n"/>
+      <c r="K30" s="18" t="n"/>
+      <c r="L30" s="18" t="n"/>
+      <c r="M30" s="18" t="n"/>
+      <c r="N30" s="18" t="n"/>
+      <c r="O30" s="18" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Midwest</t>
-        </is>
-      </c>
-      <c r="B31" s="17" t="inlineStr">
-        <is>
-          <t>2 item(s)</t>
-        </is>
-      </c>
-      <c r="C31" s="18" t="n"/>
-      <c r="D31" s="18" t="n"/>
-      <c r="E31" s="18" t="n"/>
-      <c r="F31" s="18" t="n"/>
-      <c r="G31" s="18" t="n"/>
-      <c r="H31" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" s="18" t="n"/>
-      <c r="J31" s="18" t="n"/>
-      <c r="K31" s="18" t="n"/>
-      <c r="L31" s="18" t="n"/>
-      <c r="M31" s="18" t="n"/>
-      <c r="N31" s="18" t="n"/>
-      <c r="O31" s="18" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="11" t="inlineStr">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>▸ Texas / South Central  (2)</t>
         </is>
       </c>
-      <c r="B32" s="12" t="n"/>
-      <c r="C32" s="12" t="n"/>
-      <c r="D32" s="12" t="n"/>
-      <c r="E32" s="12" t="n"/>
-      <c r="F32" s="12" t="n"/>
-      <c r="G32" s="12" t="n"/>
-      <c r="H32" s="12" t="n"/>
-      <c r="I32" s="12" t="n"/>
-      <c r="J32" s="12" t="n"/>
-      <c r="K32" s="12" t="n"/>
-      <c r="L32" s="12" t="n"/>
-      <c r="M32" s="12" t="n"/>
-      <c r="N32" s="12" t="n"/>
-      <c r="O32" s="12" t="n"/>
+      <c r="B31" s="12" t="n"/>
+      <c r="C31" s="12" t="n"/>
+      <c r="D31" s="12" t="n"/>
+      <c r="E31" s="12" t="n"/>
+      <c r="F31" s="12" t="n"/>
+      <c r="G31" s="12" t="n"/>
+      <c r="H31" s="12" t="n"/>
+      <c r="I31" s="12" t="n"/>
+      <c r="J31" s="12" t="n"/>
+      <c r="K31" s="12" t="n"/>
+      <c r="L31" s="12" t="n"/>
+      <c r="M31" s="12" t="n"/>
+      <c r="N31" s="12" t="n"/>
+      <c r="O31" s="12" t="n"/>
+    </row>
+    <row r="32" outlineLevel="1">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>Texas / South Central</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>Wholesale Hisense appliance parts – stove &amp; refrigerator parts</t>
+        </is>
+      </c>
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>bulk lot</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="inlineStr">
+        <is>
+          <t>Owasso</t>
+        </is>
+      </c>
+      <c r="E32" s="13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F32" s="13" t="n">
+        <v>1395</v>
+      </c>
+      <c r="G32" s="13" t="inlineStr">
+        <is>
+          <t>Wholesale (price at sale)</t>
+        </is>
+      </c>
+      <c r="H32" s="15" t="n"/>
+      <c r="I32" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="J32" s="13" t="inlineStr"/>
+      <c r="K32" s="13" t="inlineStr">
+        <is>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L32" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M32" s="13" t="inlineStr"/>
+      <c r="N32" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O32" s="14" t="inlineStr">
+        <is>
+          <t>Updated 2026-10-12. Seller says LOCAL BUYERS ONLY, out-of-area excluded, cash pickup.</t>
+        </is>
+      </c>
     </row>
     <row r="33" outlineLevel="1">
       <c r="A33" s="13" t="inlineStr">
@@ -2800,7 +2798,7 @@
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>Wholesale Hisense appliance parts – stove &amp; refrigerator parts</t>
+          <t>Huge bulk lot appliance parts – ~2 trailer loads, GE/Whirlpool/Maytag</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
@@ -2810,32 +2808,30 @@
       </c>
       <c r="D33" s="13" t="inlineStr">
         <is>
-          <t>Owasso</t>
+          <t>Abilene</t>
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>1395</v>
+        <v>1714</v>
       </c>
       <c r="G33" s="13" t="inlineStr">
         <is>
-          <t>Wholesale (price at sale)</t>
-        </is>
-      </c>
-      <c r="H33" s="15" t="n"/>
-      <c r="I33" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
+          <t>$5,001</t>
+        </is>
+      </c>
+      <c r="H33" s="15" t="n">
+        <v>5001</v>
+      </c>
+      <c r="I33" s="13" t="inlineStr"/>
       <c r="J33" s="13" t="inlineStr"/>
       <c r="K33" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>Geebo</t>
         </is>
       </c>
       <c r="L33" s="13" t="inlineStr">
@@ -2851,118 +2847,118 @@
       </c>
       <c r="O33" s="14" t="inlineStr">
         <is>
-          <t>Updated 2026-10-12. Seller says LOCAL BUYERS ONLY, out-of-area excluded, cash pickup.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" outlineLevel="1">
-      <c r="A34" s="13" t="inlineStr">
-        <is>
-          <t>Texas / South Central</t>
-        </is>
-      </c>
-      <c r="B34" s="14" t="inlineStr">
-        <is>
-          <t>Huge bulk lot appliance parts – ~2 trailer loads, GE/Whirlpool/Maytag</t>
-        </is>
-      </c>
-      <c r="C34" s="13" t="inlineStr">
-        <is>
-          <t>bulk lot</t>
-        </is>
-      </c>
-      <c r="D34" s="13" t="inlineStr">
-        <is>
-          <t>Abilene</t>
-        </is>
-      </c>
-      <c r="E34" s="13" t="inlineStr">
-        <is>
-          <t>TX</t>
-        </is>
-      </c>
-      <c r="F34" s="13" t="n">
-        <v>1714</v>
-      </c>
-      <c r="G34" s="13" t="inlineStr">
-        <is>
-          <t>$5,001</t>
-        </is>
-      </c>
-      <c r="H34" s="15" t="n">
+          <t>Post date unclear (may be older). Pickup only. User already messaged seller.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Texas / South Central</t>
+        </is>
+      </c>
+      <c r="B34" s="17" t="inlineStr">
+        <is>
+          <t>2 item(s)</t>
+        </is>
+      </c>
+      <c r="C34" s="18" t="n"/>
+      <c r="D34" s="18" t="n"/>
+      <c r="E34" s="18" t="n"/>
+      <c r="F34" s="18" t="n"/>
+      <c r="G34" s="18" t="n"/>
+      <c r="H34" s="19" t="n">
         <v>5001</v>
       </c>
-      <c r="I34" s="13" t="inlineStr"/>
-      <c r="J34" s="13" t="inlineStr"/>
-      <c r="K34" s="13" t="inlineStr">
-        <is>
-          <t>Geebo</t>
-        </is>
-      </c>
-      <c r="L34" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M34" s="13" t="inlineStr"/>
-      <c r="N34" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O34" s="14" t="inlineStr">
-        <is>
-          <t>Post date unclear (may be older). Pickup only. User already messaged seller.</t>
-        </is>
-      </c>
+      <c r="I34" s="18" t="n"/>
+      <c r="J34" s="18" t="n"/>
+      <c r="K34" s="18" t="n"/>
+      <c r="L34" s="18" t="n"/>
+      <c r="M34" s="18" t="n"/>
+      <c r="N34" s="18" t="n"/>
+      <c r="O34" s="18" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Texas / South Central</t>
-        </is>
-      </c>
-      <c r="B35" s="17" t="inlineStr">
-        <is>
-          <t>2 item(s)</t>
-        </is>
-      </c>
-      <c r="C35" s="18" t="n"/>
-      <c r="D35" s="18" t="n"/>
-      <c r="E35" s="18" t="n"/>
-      <c r="F35" s="18" t="n"/>
-      <c r="G35" s="18" t="n"/>
-      <c r="H35" s="19" t="n">
-        <v>5001</v>
-      </c>
-      <c r="I35" s="18" t="n"/>
-      <c r="J35" s="18" t="n"/>
-      <c r="K35" s="18" t="n"/>
-      <c r="L35" s="18" t="n"/>
-      <c r="M35" s="18" t="n"/>
-      <c r="N35" s="18" t="n"/>
-      <c r="O35" s="18" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="11" t="inlineStr">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>▸ California  (2)</t>
         </is>
       </c>
-      <c r="B36" s="12" t="n"/>
-      <c r="C36" s="12" t="n"/>
-      <c r="D36" s="12" t="n"/>
-      <c r="E36" s="12" t="n"/>
-      <c r="F36" s="12" t="n"/>
-      <c r="G36" s="12" t="n"/>
-      <c r="H36" s="12" t="n"/>
-      <c r="I36" s="12" t="n"/>
-      <c r="J36" s="12" t="n"/>
-      <c r="K36" s="12" t="n"/>
-      <c r="L36" s="12" t="n"/>
-      <c r="M36" s="12" t="n"/>
-      <c r="N36" s="12" t="n"/>
-      <c r="O36" s="12" t="n"/>
+      <c r="B35" s="12" t="n"/>
+      <c r="C35" s="12" t="n"/>
+      <c r="D35" s="12" t="n"/>
+      <c r="E35" s="12" t="n"/>
+      <c r="F35" s="12" t="n"/>
+      <c r="G35" s="12" t="n"/>
+      <c r="H35" s="12" t="n"/>
+      <c r="I35" s="12" t="n"/>
+      <c r="J35" s="12" t="n"/>
+      <c r="K35" s="12" t="n"/>
+      <c r="L35" s="12" t="n"/>
+      <c r="M35" s="12" t="n"/>
+      <c r="N35" s="12" t="n"/>
+      <c r="O35" s="12" t="n"/>
+    </row>
+    <row r="36" outlineLevel="1">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>California</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>Appliance repair company for sale (incl. parts inventory)</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>business sale</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>Escondido</t>
+        </is>
+      </c>
+      <c r="E36" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="n">
+        <v>2575</v>
+      </c>
+      <c r="G36" s="13" t="inlineStr">
+        <is>
+          <t>$40,000</t>
+        </is>
+      </c>
+      <c r="H36" s="15" t="n">
+        <v>40000</v>
+      </c>
+      <c r="I36" s="13" t="inlineStr"/>
+      <c r="J36" s="13" t="inlineStr"/>
+      <c r="K36" s="13" t="inlineStr">
+        <is>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L36" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M36" s="13" t="inlineStr"/>
+      <c r="N36" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O36" s="14" t="inlineStr">
+        <is>
+          <t>Whole business sale.</t>
+        </is>
+      </c>
     </row>
     <row r="37" outlineLevel="1">
       <c r="A37" s="13" t="inlineStr">
@@ -2972,17 +2968,17 @@
       </c>
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>Appliance repair company for sale (incl. parts inventory)</t>
+          <t>Coin-op Whirlpool washer &amp; dryer parts (late 80s–mid 90s) – OEM parts, 40+ coin boxes, consoles, 12 transmissions</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>business sale</t>
+          <t>bulk lot</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">
         <is>
-          <t>Escondido</t>
+          <t>Chico</t>
         </is>
       </c>
       <c r="E37" s="13" t="inlineStr">
@@ -2991,17 +2987,21 @@
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>2575</v>
+        <v>2629</v>
       </c>
       <c r="G37" s="13" t="inlineStr">
         <is>
-          <t>$40,000</t>
+          <t>$1,000</t>
         </is>
       </c>
       <c r="H37" s="15" t="n">
-        <v>40000</v>
-      </c>
-      <c r="I37" s="13" t="inlineStr"/>
+        <v>1000</v>
+      </c>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
       <c r="J37" s="13" t="inlineStr"/>
       <c r="K37" s="13" t="inlineStr">
         <is>
@@ -3021,122 +3021,120 @@
       </c>
       <c r="O37" s="14" t="inlineStr">
         <is>
-          <t>Whole business sale.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" outlineLevel="1">
-      <c r="A38" s="13" t="inlineStr">
-        <is>
-          <t>California</t>
-        </is>
-      </c>
-      <c r="B38" s="14" t="inlineStr">
-        <is>
-          <t>Coin-op Whirlpool washer &amp; dryer parts (late 80s–mid 90s) – OEM parts, 40+ coin boxes, consoles, 12 transmissions</t>
-        </is>
-      </c>
-      <c r="C38" s="13" t="inlineStr">
+          <t>Retired laundry-route owner (35 yrs). Calls only, no shipping, pickup in Chico. No motors or pumps. Niche older coin-op parts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — California</t>
+        </is>
+      </c>
+      <c r="B38" s="17" t="inlineStr">
+        <is>
+          <t>2 item(s)</t>
+        </is>
+      </c>
+      <c r="C38" s="18" t="n"/>
+      <c r="D38" s="18" t="n"/>
+      <c r="E38" s="18" t="n"/>
+      <c r="F38" s="18" t="n"/>
+      <c r="G38" s="18" t="n"/>
+      <c r="H38" s="19" t="n">
+        <v>41000</v>
+      </c>
+      <c r="I38" s="18" t="n"/>
+      <c r="J38" s="18" t="n"/>
+      <c r="K38" s="18" t="n"/>
+      <c r="L38" s="18" t="n"/>
+      <c r="M38" s="18" t="n"/>
+      <c r="N38" s="18" t="n"/>
+      <c r="O38" s="18" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>▸ West / Other  (2)</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="n"/>
+      <c r="C39" s="12" t="n"/>
+      <c r="D39" s="12" t="n"/>
+      <c r="E39" s="12" t="n"/>
+      <c r="F39" s="12" t="n"/>
+      <c r="G39" s="12" t="n"/>
+      <c r="H39" s="12" t="n"/>
+      <c r="I39" s="12" t="n"/>
+      <c r="J39" s="12" t="n"/>
+      <c r="K39" s="12" t="n"/>
+      <c r="L39" s="12" t="n"/>
+      <c r="M39" s="12" t="n"/>
+      <c r="N39" s="12" t="n"/>
+      <c r="O39" s="12" t="n"/>
+    </row>
+    <row r="40" outlineLevel="1">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>West / Other</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>Storage locker filled with appliance parts – washer/dryer parts, heating elements, cords, rollers, belts, tools</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr">
         <is>
           <t>bulk lot</t>
         </is>
       </c>
-      <c r="D38" s="13" t="inlineStr">
-        <is>
-          <t>Chico</t>
-        </is>
-      </c>
-      <c r="E38" s="13" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-      <c r="F38" s="13" t="n">
-        <v>2629</v>
-      </c>
-      <c r="G38" s="13" t="inlineStr">
-        <is>
-          <t>$1,000</t>
-        </is>
-      </c>
-      <c r="H38" s="15" t="n">
-        <v>1000</v>
-      </c>
-      <c r="I38" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="J38" s="13" t="inlineStr"/>
-      <c r="K38" s="13" t="inlineStr">
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="E40" s="13" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="F40" s="13" t="n">
+        <v>2307</v>
+      </c>
+      <c r="G40" s="13" t="inlineStr">
+        <is>
+          <t>Message for pricing</t>
+        </is>
+      </c>
+      <c r="H40" s="15" t="n"/>
+      <c r="I40" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="J40" s="13" t="inlineStr"/>
+      <c r="K40" s="13" t="inlineStr">
         <is>
           <t>Craigslist</t>
         </is>
       </c>
-      <c r="L38" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M38" s="13" t="inlineStr"/>
-      <c r="N38" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O38" s="14" t="inlineStr">
-        <is>
-          <t>Retired laundry-route owner (35 yrs). Calls only, no shipping, pickup in Chico. No motors or pumps. Niche older coin-op parts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — California</t>
-        </is>
-      </c>
-      <c r="B39" s="17" t="inlineStr">
-        <is>
-          <t>2 item(s)</t>
-        </is>
-      </c>
-      <c r="C39" s="18" t="n"/>
-      <c r="D39" s="18" t="n"/>
-      <c r="E39" s="18" t="n"/>
-      <c r="F39" s="18" t="n"/>
-      <c r="G39" s="18" t="n"/>
-      <c r="H39" s="19" t="n">
-        <v>41000</v>
-      </c>
-      <c r="I39" s="18" t="n"/>
-      <c r="J39" s="18" t="n"/>
-      <c r="K39" s="18" t="n"/>
-      <c r="L39" s="18" t="n"/>
-      <c r="M39" s="18" t="n"/>
-      <c r="N39" s="18" t="n"/>
-      <c r="O39" s="18" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="11" t="inlineStr">
-        <is>
-          <t>▸ West / Other  (2)</t>
-        </is>
-      </c>
-      <c r="B40" s="12" t="n"/>
-      <c r="C40" s="12" t="n"/>
-      <c r="D40" s="12" t="n"/>
-      <c r="E40" s="12" t="n"/>
-      <c r="F40" s="12" t="n"/>
-      <c r="G40" s="12" t="n"/>
-      <c r="H40" s="12" t="n"/>
-      <c r="I40" s="12" t="n"/>
-      <c r="J40" s="12" t="n"/>
-      <c r="K40" s="12" t="n"/>
-      <c r="L40" s="12" t="n"/>
-      <c r="M40" s="12" t="n"/>
-      <c r="N40" s="12" t="n"/>
-      <c r="O40" s="12" t="n"/>
+      <c r="L40" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M40" s="13" t="inlineStr"/>
+      <c r="N40" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O40" s="14" t="inlineStr">
+        <is>
+          <t>Seller is getting out of the appliance business; selling the whole locker (North Phoenix, Deer Valley Rd near 19th Ave). Delivery available per post. Separate from the Phoenix parts-store closing ad.</t>
+        </is>
+      </c>
     </row>
     <row r="41" outlineLevel="1">
       <c r="A41" s="13" t="inlineStr">
@@ -3146,17 +3144,17 @@
       </c>
       <c r="B41" s="14" t="inlineStr">
         <is>
-          <t>Storage locker filled with appliance parts – washer/dryer parts, heating elements, cords, rollers, belts, tools</t>
+          <t>Appliance repair &amp; sales business for sale – 100+ appliances (~90% new), liftgate truck, large powered storage unit</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
-          <t>bulk lot</t>
+          <t>business for sale</t>
         </is>
       </c>
       <c r="D41" s="13" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Surprise</t>
         </is>
       </c>
       <c r="E41" s="13" t="inlineStr">
@@ -3165,17 +3163,19 @@
         </is>
       </c>
       <c r="F41" s="13" t="n">
-        <v>2307</v>
+        <v>2317</v>
       </c>
       <c r="G41" s="13" t="inlineStr">
         <is>
-          <t>Message for pricing</t>
-        </is>
-      </c>
-      <c r="H41" s="15" t="n"/>
+          <t>$75,000</t>
+        </is>
+      </c>
+      <c r="H41" s="15" t="n">
+        <v>75000</v>
+      </c>
       <c r="I41" s="13" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="J41" s="13" t="inlineStr"/>
@@ -3197,104 +3197,39 @@
       </c>
       <c r="O41" s="14" t="inlineStr">
         <is>
-          <t>Seller is getting out of the appliance business; selling the whole locker (North Phoenix, Deer Valley Rd near 19th Ave). Delivery available per post. Separate from the Phoenix parts-store closing ad.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" outlineLevel="1">
-      <c r="A42" s="13" t="inlineStr">
-        <is>
-          <t>West / Other</t>
-        </is>
-      </c>
-      <c r="B42" s="14" t="inlineStr">
-        <is>
-          <t>Appliance repair &amp; sales business for sale – 100+ appliances (~90% new), liftgate truck, large powered storage unit</t>
-        </is>
-      </c>
-      <c r="C42" s="13" t="inlineStr">
-        <is>
-          <t>business for sale</t>
-        </is>
-      </c>
-      <c r="D42" s="13" t="inlineStr">
-        <is>
-          <t>Surprise</t>
-        </is>
-      </c>
-      <c r="E42" s="13" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="F42" s="13" t="n">
-        <v>2317</v>
-      </c>
-      <c r="G42" s="13" t="inlineStr">
-        <is>
-          <t>$75,000</t>
-        </is>
-      </c>
-      <c r="H42" s="15" t="n">
+          <t>Retiring owner of 14-year business serving rental-property owners. Whole appliances (fridges, stoves, microwaves, dishwashers, W/D), not a parts inventory. Storage unit near Dysart &amp; Bell Rd. By appointment only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — West / Other</t>
+        </is>
+      </c>
+      <c r="B42" s="17" t="inlineStr">
+        <is>
+          <t>2 item(s)</t>
+        </is>
+      </c>
+      <c r="C42" s="18" t="n"/>
+      <c r="D42" s="18" t="n"/>
+      <c r="E42" s="18" t="n"/>
+      <c r="F42" s="18" t="n"/>
+      <c r="G42" s="18" t="n"/>
+      <c r="H42" s="19" t="n">
         <v>75000</v>
       </c>
-      <c r="I42" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="J42" s="13" t="inlineStr"/>
-      <c r="K42" s="13" t="inlineStr">
-        <is>
-          <t>Craigslist</t>
-        </is>
-      </c>
-      <c r="L42" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M42" s="13" t="inlineStr"/>
-      <c r="N42" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O42" s="14" t="inlineStr">
-        <is>
-          <t>Retiring owner of 14-year business serving rental-property owners. Whole appliances (fridges, stoves, microwaves, dishwashers, W/D), not a parts inventory. Storage unit near Dysart &amp; Bell Rd. By appointment only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — West / Other</t>
-        </is>
-      </c>
-      <c r="B43" s="17" t="inlineStr">
-        <is>
-          <t>2 item(s)</t>
-        </is>
-      </c>
-      <c r="C43" s="18" t="n"/>
-      <c r="D43" s="18" t="n"/>
-      <c r="E43" s="18" t="n"/>
-      <c r="F43" s="18" t="n"/>
-      <c r="G43" s="18" t="n"/>
-      <c r="H43" s="19" t="n">
-        <v>75000</v>
-      </c>
-      <c r="I43" s="18" t="n"/>
-      <c r="J43" s="18" t="n"/>
-      <c r="K43" s="18" t="n"/>
-      <c r="L43" s="18" t="n"/>
-      <c r="M43" s="18" t="n"/>
-      <c r="N43" s="18" t="n"/>
-      <c r="O43" s="18" t="n"/>
+      <c r="I42" s="18" t="n"/>
+      <c r="J42" s="18" t="n"/>
+      <c r="K42" s="18" t="n"/>
+      <c r="L42" s="18" t="n"/>
+      <c r="M42" s="18" t="n"/>
+      <c r="N42" s="18" t="n"/>
+      <c r="O42" s="18" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O43"/>
+  <autoFilter ref="A1:O42"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId2"/>
@@ -3307,15 +3242,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N32" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N36" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N38" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N40" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -19493,7 +19427,7 @@
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>▸ Maine / VT / Northern NH  (5)</t>
+          <t>▸ Maine / VT / Northern NH  (4)</t>
         </is>
       </c>
       <c r="B17" s="12" t="n"/>
@@ -19519,12 +19453,12 @@
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>Oola Bowls secured-party sale – restaurant equipment bought new 2024-25 (Electro Freeze, Scotsman, Atosa)</t>
+          <t>Contractor appliance lot – 3 refrigerators, Bosch wall oven, gas range, washer/dryer set</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>contractor lot</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr">
@@ -19542,24 +19476,24 @@
       </c>
       <c r="G18" s="13" t="inlineStr">
         <is>
-          <t>Online auction (freezers $80–150 when seen)</t>
+          <t>$200 OBO each, less as a bundle</t>
         </is>
       </c>
       <c r="H18" s="15" t="n"/>
-      <c r="I18" s="13" t="inlineStr"/>
-      <c r="J18" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-19 01:00 PM ET</t>
-        </is>
-      </c>
+      <c r="I18" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="J18" s="13" t="inlineStr"/>
       <c r="K18" s="13" t="inlineStr">
         <is>
-          <t>Keenan Auction / Proxibid</t>
-        </is>
-      </c>
-      <c r="L18" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L18" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M18" s="13" t="inlineStr"/>
@@ -19570,7 +19504,7 @@
       </c>
       <c r="O18" s="14" t="inlineStr">
         <is>
-          <t>Pickup Oct 21 only.</t>
+          <t>Working units pulled from jobs. Complete appliances, not parts.</t>
         </is>
       </c>
     </row>
@@ -19582,17 +19516,17 @@
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>Contractor appliance lot – 3 refrigerators, Bosch wall oven, gas range, washer/dryer set</t>
+          <t>Event-rental business closing – 300+ chairs, 40+ rounds, 1,300+ china, linens (all at once)</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>contractor lot</t>
+          <t>business closing</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>Scarborough</t>
+          <t>Woolwich</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr">
@@ -19601,17 +19535,17 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>104</v>
+        <v>135</v>
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>$200 OBO each, less as a bundle</t>
+          <t>No price listed</t>
         </is>
       </c>
       <c r="H19" s="15" t="n"/>
       <c r="I19" s="13" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="J19" s="13" t="inlineStr"/>
@@ -19633,7 +19567,7 @@
       </c>
       <c r="O19" s="14" t="inlineStr">
         <is>
-          <t>Working units pulled from jobs. Complete appliances, not parts.</t>
+          <t>Updated Oct 7. Replacement cost &gt;$72K per post.</t>
         </is>
       </c>
     </row>
@@ -19645,42 +19579,42 @@
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>Event-rental business closing – 300+ chairs, 40+ rounds, 1,300+ china, linens (all at once)</t>
+          <t>Pellet/wood stoves, heating stock, tools &amp; heavy equipment – "business liquidation", 380 lots</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>business closing</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D20" s="13" t="inlineStr">
         <is>
-          <t>Woolwich</t>
+          <t>Lunenburg</t>
         </is>
       </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
-          <t>ME</t>
+          <t>VT</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>135</v>
+        <v>168</v>
       </c>
       <c r="G20" s="13" t="inlineStr">
         <is>
-          <t>No price listed</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H20" s="15" t="n"/>
-      <c r="I20" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="J20" s="13" t="inlineStr"/>
+      <c r="I20" s="13" t="inlineStr"/>
+      <c r="J20" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-04 10:00 AM ET</t>
+        </is>
+      </c>
       <c r="K20" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>Thomas Hirchak Co.</t>
         </is>
       </c>
       <c r="L20" s="13" t="inlineStr">
@@ -19696,7 +19630,7 @@
       </c>
       <c r="O20" s="14" t="inlineStr">
         <is>
-          <t>Updated Oct 7. Replacement cost &gt;$72K per post.</t>
+          <t>Closes Wed Nov 4 10 AM, preview Oct 28, removal Nov 9, no shipping.</t>
         </is>
       </c>
     </row>
@@ -19708,17 +19642,17 @@
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>Pellet/wood stoves, heating stock, tools &amp; heavy equipment – "business liquidation", 380 lots</t>
+          <t>Bread Loaf Corp wind-down – contractor equipment, staging, telehandler</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>contractor liquidation</t>
         </is>
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
-          <t>Lunenburg</t>
+          <t>Middlebury</t>
         </is>
       </c>
       <c r="E21" s="13" t="inlineStr">
@@ -19727,7 +19661,7 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="G21" s="13" t="inlineStr">
         <is>
@@ -19738,12 +19672,12 @@
       <c r="I21" s="13" t="inlineStr"/>
       <c r="J21" s="13" t="inlineStr">
         <is>
-          <t>2026-11-04 10:00 AM ET</t>
+          <t>2026-10-28 09:00 AM ET</t>
         </is>
       </c>
       <c r="K21" s="13" t="inlineStr">
         <is>
-          <t>Thomas Hirchak Co.</t>
+          <t>THC Auction</t>
         </is>
       </c>
       <c r="L21" s="13" t="inlineStr">
@@ -19759,120 +19693,120 @@
       </c>
       <c r="O21" s="14" t="inlineStr">
         <is>
-          <t>Closes Wed Nov 4 10 AM, preview Oct 28, removal Nov 9, no shipping.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" outlineLevel="1">
-      <c r="A22" s="13" t="inlineStr">
-        <is>
-          <t>Maine / VT / Northern NH</t>
-        </is>
-      </c>
-      <c r="B22" s="14" t="inlineStr">
-        <is>
-          <t>Bread Loaf Corp wind-down – contractor equipment, staging, telehandler</t>
-        </is>
-      </c>
-      <c r="C22" s="13" t="inlineStr">
+          <t>Company wind-down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Maine / VT / Northern NH</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>4 item(s)</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="n"/>
+      <c r="D22" s="18" t="n"/>
+      <c r="E22" s="18" t="n"/>
+      <c r="F22" s="18" t="n"/>
+      <c r="G22" s="18" t="n"/>
+      <c r="H22" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="18" t="n"/>
+      <c r="J22" s="18" t="n"/>
+      <c r="K22" s="18" t="n"/>
+      <c r="L22" s="18" t="n"/>
+      <c r="M22" s="18" t="n"/>
+      <c r="N22" s="18" t="n"/>
+      <c r="O22" s="18" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>▸ CT / Hudson Valley  (7)</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="n"/>
+      <c r="C23" s="12" t="n"/>
+      <c r="D23" s="12" t="n"/>
+      <c r="E23" s="12" t="n"/>
+      <c r="F23" s="12" t="n"/>
+      <c r="G23" s="12" t="n"/>
+      <c r="H23" s="12" t="n"/>
+      <c r="I23" s="12" t="n"/>
+      <c r="J23" s="12" t="n"/>
+      <c r="K23" s="12" t="n"/>
+      <c r="L23" s="12" t="n"/>
+      <c r="M23" s="12" t="n"/>
+      <c r="N23" s="12" t="n"/>
+      <c r="O23" s="12" t="n"/>
+    </row>
+    <row r="24" outlineLevel="1">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>CT / Hudson Valley</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>Bank-ordered electrical contractor sale – Greenlee/Hilti/Milwaukee tools, GE/Siemens breakers</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
         <is>
           <t>contractor liquidation</t>
         </is>
       </c>
-      <c r="D22" s="13" t="inlineStr">
-        <is>
-          <t>Middlebury</t>
-        </is>
-      </c>
-      <c r="E22" s="13" t="inlineStr">
-        <is>
-          <t>VT</t>
-        </is>
-      </c>
-      <c r="F22" s="13" t="n">
-        <v>177</v>
-      </c>
-      <c r="G22" s="13" t="inlineStr">
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>Clinton</t>
+        </is>
+      </c>
+      <c r="E24" s="13" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="n">
+        <v>106</v>
+      </c>
+      <c r="G24" s="13" t="inlineStr">
         <is>
           <t>Online auction</t>
         </is>
       </c>
-      <c r="H22" s="15" t="n"/>
-      <c r="I22" s="13" t="inlineStr"/>
-      <c r="J22" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-28 09:00 AM ET</t>
-        </is>
-      </c>
-      <c r="K22" s="13" t="inlineStr">
-        <is>
-          <t>THC Auction</t>
-        </is>
-      </c>
-      <c r="L22" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M22" s="13" t="inlineStr"/>
-      <c r="N22" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O22" s="14" t="inlineStr">
-        <is>
-          <t>Company wind-down.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Maine / VT / Northern NH</t>
-        </is>
-      </c>
-      <c r="B23" s="17" t="inlineStr">
-        <is>
-          <t>5 item(s)</t>
-        </is>
-      </c>
-      <c r="C23" s="18" t="n"/>
-      <c r="D23" s="18" t="n"/>
-      <c r="E23" s="18" t="n"/>
-      <c r="F23" s="18" t="n"/>
-      <c r="G23" s="18" t="n"/>
-      <c r="H23" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="18" t="n"/>
-      <c r="J23" s="18" t="n"/>
-      <c r="K23" s="18" t="n"/>
-      <c r="L23" s="18" t="n"/>
-      <c r="M23" s="18" t="n"/>
-      <c r="N23" s="18" t="n"/>
-      <c r="O23" s="18" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t>▸ CT / Hudson Valley  (6)</t>
-        </is>
-      </c>
-      <c r="B24" s="12" t="n"/>
-      <c r="C24" s="12" t="n"/>
-      <c r="D24" s="12" t="n"/>
-      <c r="E24" s="12" t="n"/>
-      <c r="F24" s="12" t="n"/>
-      <c r="G24" s="12" t="n"/>
-      <c r="H24" s="12" t="n"/>
-      <c r="I24" s="12" t="n"/>
-      <c r="J24" s="12" t="n"/>
-      <c r="K24" s="12" t="n"/>
-      <c r="L24" s="12" t="n"/>
-      <c r="M24" s="12" t="n"/>
-      <c r="N24" s="12" t="n"/>
-      <c r="O24" s="12" t="n"/>
+      <c r="H24" s="15" t="n"/>
+      <c r="I24" s="13" t="inlineStr"/>
+      <c r="J24" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-29 05:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K24" s="13" t="inlineStr">
+        <is>
+          <t>Hamilton Group / EstateSales.net</t>
+        </is>
+      </c>
+      <c r="L24" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M24" s="13" t="inlineStr"/>
+      <c r="N24" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O24" s="14" t="inlineStr">
+        <is>
+          <t>Listed "Oct 29 2 PM PST" (= 5 PM ET).</t>
+        </is>
+      </c>
     </row>
     <row r="25" outlineLevel="1">
       <c r="A25" s="13" t="inlineStr">
@@ -19882,17 +19816,17 @@
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>Bank-ordered electrical contractor sale – Greenlee/Hilti/Milwaukee tools, GE/Siemens breakers</t>
+          <t>Fabrication &amp; welding shop liquidation – everything must be sold</t>
         </is>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>contractor liquidation</t>
+          <t>machine shop liquidation</t>
         </is>
       </c>
       <c r="D25" s="13" t="inlineStr">
         <is>
-          <t>Clinton</t>
+          <t>Bridgeport</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
@@ -19901,23 +19835,23 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>106</v>
+        <v>139</v>
       </c>
       <c r="G25" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Priced per machine (e.g. W.A. Whitney punch press $4,950; DoAll bandsaw $950)</t>
         </is>
       </c>
       <c r="H25" s="15" t="n"/>
-      <c r="I25" s="13" t="inlineStr"/>
-      <c r="J25" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-29 05:00 PM ET</t>
-        </is>
-      </c>
+      <c r="I25" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="J25" s="13" t="inlineStr"/>
       <c r="K25" s="13" t="inlineStr">
         <is>
-          <t>Hamilton Group / EstateSales.net</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L25" s="13" t="inlineStr">
@@ -19933,7 +19867,7 @@
       </c>
       <c r="O25" s="14" t="inlineStr">
         <is>
-          <t>Listed "Oct 29 2 PM PST" (= 5 PM ET).</t>
+          <t>All assets/equipment/tools of a fab &amp; welding shop; machines under power, inspection by appointment, buyer removes (small forklift on site). Several big items already SOLD (Cincinnati brake/shear, plasma table, Lown roll). Remaining: Whitney + Roper Whitney punch presses, DoAll V36 bandsaw, Thompson spot welder, George Ohl 120" brake, Bridgeport mill, etc. Mostly 220V. Posted May 15, updated Oct 19.</t>
         </is>
       </c>
     </row>
@@ -20264,7 +20198,7 @@
       </c>
       <c r="B31" s="17" t="inlineStr">
         <is>
-          <t>6 item(s)</t>
+          <t>7 item(s)</t>
         </is>
       </c>
       <c r="C31" s="18" t="n"/>
@@ -20286,7 +20220,7 @@
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>▸ NYC / Long Island / NJ  (24)</t>
+          <t>▸ NYC / Long Island / NJ  (23)</t>
         </is>
       </c>
       <c r="B32" s="12" t="n"/>
@@ -20547,9 +20481,9 @@
           <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
-      <c r="L36" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+      <c r="L36" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M36" s="13" t="inlineStr"/>
@@ -20824,7 +20758,7 @@
       </c>
       <c r="B41" s="14" t="inlineStr">
         <is>
-          <t>Like-new restaurant – steam tables, Coldline, Cleveland cook-and-hold, fryers, True freezers</t>
+          <t>Major food-service caterer – new-in-box True reach-ins, Beverage-Air, TurboChef, Resfab ventless fryer</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
@@ -20834,16 +20768,16 @@
       </c>
       <c r="D41" s="13" t="inlineStr">
         <is>
-          <t>Staten Island</t>
+          <t>Parsippany</t>
         </is>
       </c>
       <c r="E41" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="F41" s="13" t="n">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="G41" s="13" t="inlineStr">
         <is>
@@ -20853,12 +20787,12 @@
       <c r="H41" s="15" t="n"/>
       <c r="I41" s="13" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="J41" s="13" t="inlineStr">
         <is>
-          <t>2026-10-19 01:00 PM ET</t>
+          <t>2026-11-03 02:00 PM ET</t>
         </is>
       </c>
       <c r="K41" s="13" t="inlineStr">
@@ -20866,9 +20800,9 @@
           <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
-      <c r="L41" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+      <c r="L41" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M41" s="13" t="inlineStr"/>
@@ -20879,7 +20813,7 @@
       </c>
       <c r="O41" s="14" t="inlineStr">
         <is>
-          <t>"Short notice" auction Mon Oct 19 1 PM.</t>
+          <t>Tue Nov 3 2 PM, checkout Nov 4.</t>
         </is>
       </c>
     </row>
@@ -20891,17 +20825,17 @@
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>Major food-service caterer – new-in-box True reach-ins, Beverage-Air, TurboChef, Resfab ventless fryer</t>
+          <t>Business closing – 160 new Carnes exhaust fans</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>HVAC inventory</t>
         </is>
       </c>
       <c r="D42" s="13" t="inlineStr">
         <is>
-          <t>Parsippany</t>
+          <t>Kenilworth</t>
         </is>
       </c>
       <c r="E42" s="13" t="inlineStr">
@@ -20914,23 +20848,19 @@
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>$40 each or $5,000 all OBO</t>
         </is>
       </c>
       <c r="H42" s="15" t="n"/>
       <c r="I42" s="13" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="J42" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-03 02:00 PM ET</t>
-        </is>
-      </c>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="J42" s="13" t="inlineStr"/>
       <c r="K42" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L42" s="13" t="inlineStr">
@@ -20946,7 +20876,7 @@
       </c>
       <c r="O42" s="14" t="inlineStr">
         <is>
-          <t>Tue Nov 3 2 PM, checkout Nov 4.</t>
+          <t>160 new Carnes 80CFM 1.0 sone exhaust fans. $40 each or $5,000 for all OBO. Business closing HVAC inventory.</t>
         </is>
       </c>
     </row>
@@ -20958,12 +20888,12 @@
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>Business closing – 160 new Carnes exhaust fans</t>
+          <t>Air Systems Inc – sheet metal / HVAC fabrication shop liquidation</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
         <is>
-          <t>HVAC inventory</t>
+          <t>HVAC shop liquidation</t>
         </is>
       </c>
       <c r="D43" s="13" t="inlineStr">
@@ -20981,19 +20911,19 @@
       </c>
       <c r="G43" s="13" t="inlineStr">
         <is>
-          <t>$40 each or $5,000 all OBO</t>
+          <t>Timed online (15% BP)</t>
         </is>
       </c>
       <c r="H43" s="15" t="n"/>
-      <c r="I43" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="J43" s="13" t="inlineStr"/>
+      <c r="I43" s="13" t="inlineStr"/>
+      <c r="J43" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-29 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K43" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>A.J. Willner Auctions</t>
         </is>
       </c>
       <c r="L43" s="13" t="inlineStr">
@@ -21009,7 +20939,7 @@
       </c>
       <c r="O43" s="14" t="inlineStr">
         <is>
-          <t>160 new Carnes 80CFM 1.0 sone exhaust fans. $40 each or $5,000 for all OBO. Business closing HVAC inventory.</t>
+          <t>Vicon HVAC plasma; Flagler/Lockformer/Roto-Die/Engel fab; welders; Clark forklift; Genie Superlift; Ridgid/Milwaukee/DeWalt/Bosch/Hilti/Makita tools; AeroVent/Carnes exhaust fans; racking/scaffolding. Preview Oct 28–29 AM; pickup Oct 29 PM–Nov 4. Same town as Carnes fan CL lot.</t>
         </is>
       </c>
     </row>
@@ -21021,17 +20951,17 @@
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>Air Systems Inc – sheet metal / HVAC fabrication shop liquidation</t>
+          <t>Serpico's Pizzeria (lost lease) – Bari ovens, walk-in, Hobart 60qt, Vulcan range</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>HVAC shop liquidation</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D44" s="13" t="inlineStr">
         <is>
-          <t>Kenilworth</t>
+          <t>Allenhurst</t>
         </is>
       </c>
       <c r="E44" s="13" t="inlineStr">
@@ -21040,28 +20970,28 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>Timed online (15% BP)</t>
+          <t>No-reserve online auction</t>
         </is>
       </c>
       <c r="H44" s="15" t="n"/>
       <c r="I44" s="13" t="inlineStr"/>
       <c r="J44" s="13" t="inlineStr">
         <is>
-          <t>2026-10-29 11:00 AM ET</t>
+          <t>2026-10-21 11:00 AM ET</t>
         </is>
       </c>
       <c r="K44" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner Auctions</t>
-        </is>
-      </c>
-      <c r="L44" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>Peter Costanzo / EstateSales.net</t>
+        </is>
+      </c>
+      <c r="L44" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M44" s="13" t="inlineStr"/>
@@ -21072,7 +21002,7 @@
       </c>
       <c r="O44" s="14" t="inlineStr">
         <is>
-          <t>Vicon HVAC plasma; Flagler/Lockformer/Roto-Die/Engel fab; welders; Clark forklift; Genie Superlift; Ridgid/Milwaukee/DeWalt/Bosch/Hilti/Makita tools; AeroVent/Carnes exhaust fans; racking/scaffolding. Preview Oct 28–29 AM; pickup Oct 29 PM–Nov 4. Same town as Carnes fan CL lot.</t>
+          <t>Absolute / no reserve.</t>
         </is>
       </c>
     </row>
@@ -21084,17 +21014,17 @@
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>Serpico's Pizzeria (lost lease) – Bari ovens, walk-in, Hobart 60qt, Vulcan range</t>
+          <t>Altitude Trampoline Park liquidation – partial: Atosa, TurboChef, stainless</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>facility contents</t>
         </is>
       </c>
       <c r="D45" s="13" t="inlineStr">
         <is>
-          <t>Allenhurst</t>
+          <t>Iselin</t>
         </is>
       </c>
       <c r="E45" s="13" t="inlineStr">
@@ -21103,11 +21033,11 @@
         </is>
       </c>
       <c r="F45" s="13" t="n">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G45" s="13" t="inlineStr">
         <is>
-          <t>No-reserve online auction</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H45" s="15" t="n"/>
@@ -21119,7 +21049,7 @@
       </c>
       <c r="K45" s="13" t="inlineStr">
         <is>
-          <t>Peter Costanzo / EstateSales.net</t>
+          <t>A.J. Willner</t>
         </is>
       </c>
       <c r="L45" s="20" t="inlineStr">
@@ -21135,7 +21065,7 @@
       </c>
       <c r="O45" s="14" t="inlineStr">
         <is>
-          <t>Absolute / no reserve.</t>
+          <t>Some kitchen gear only.</t>
         </is>
       </c>
     </row>
@@ -21147,17 +21077,17 @@
       </c>
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>Altitude Trampoline Park liquidation – partial: Atosa, TurboChef, stainless</t>
+          <t>Restaurant / pizzeria (contents not described)</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>facility contents</t>
+          <t>restaurant closing</t>
         </is>
       </c>
       <c r="D46" s="13" t="inlineStr">
         <is>
-          <t>Iselin</t>
+          <t>Berkeley Heights</t>
         </is>
       </c>
       <c r="E46" s="13" t="inlineStr">
@@ -21166,23 +21096,27 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H46" s="15" t="n"/>
-      <c r="I46" s="13" t="inlineStr"/>
+      <c r="I46" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
       <c r="J46" s="13" t="inlineStr">
         <is>
-          <t>2026-10-21 11:00 AM ET</t>
+          <t>2026-10-20 02:00 PM ET</t>
         </is>
       </c>
       <c r="K46" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
       <c r="L46" s="20" t="inlineStr">
@@ -21198,7 +21132,7 @@
       </c>
       <c r="O46" s="14" t="inlineStr">
         <is>
-          <t>Some kitchen gear only.</t>
+          <t>Tue Oct 20 2 PM. No item description on page.</t>
         </is>
       </c>
     </row>
@@ -21210,17 +21144,17 @@
       </c>
       <c r="B47" s="14" t="inlineStr">
         <is>
-          <t>Restaurant / pizzeria (contents not described)</t>
+          <t>New modular concession kitchens (warehouseman's lien) – 5 units, CaptiveAire hoods, new Ovention/Turbo Air</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
         <is>
-          <t>restaurant closing</t>
+          <t>lien sale</t>
         </is>
       </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>Berkeley Heights</t>
+          <t>Edison</t>
         </is>
       </c>
       <c r="E47" s="13" t="inlineStr">
@@ -21229,32 +21163,24 @@
         </is>
       </c>
       <c r="F47" s="13" t="n">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="G47" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>Online auction, $2K load-out fee</t>
         </is>
       </c>
       <c r="H47" s="15" t="n"/>
-      <c r="I47" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="J47" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-20 02:00 PM ET</t>
-        </is>
-      </c>
+      <c r="I47" s="13" t="inlineStr"/>
+      <c r="J47" s="13" t="inlineStr"/>
       <c r="K47" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
-        </is>
-      </c>
-      <c r="L47" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>A.J. Willner</t>
+        </is>
+      </c>
+      <c r="L47" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M47" s="13" t="inlineStr"/>
@@ -21265,7 +21191,7 @@
       </c>
       <c r="O47" s="14" t="inlineStr">
         <is>
-          <t>Tue Oct 20 2 PM. No item description on page.</t>
+          <t>&gt;$100K new. Close date not captured.</t>
         </is>
       </c>
     </row>
@@ -21277,12 +21203,12 @@
       </c>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>New modular concession kitchens (warehouseman's lien) – 5 units, CaptiveAire hoods, new Ovention/Turbo Air</t>
+          <t>Brand-new &amp; scratch-and-dent kitchen/home appliances – ~185 lots (Thermador, GE Café, Miele, Wolf speed oven, Viking, Bosch…)</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>lien sale</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D48" s="13" t="inlineStr">
@@ -21300,15 +21226,23 @@
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>Online auction, $2K load-out fee</t>
+          <t>Live + HiBid webcast, 18% BP + 3% card</t>
         </is>
       </c>
       <c r="H48" s="15" t="n"/>
-      <c r="I48" s="13" t="inlineStr"/>
-      <c r="J48" s="13" t="inlineStr"/>
+      <c r="I48" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="J48" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-25 01:00 PM ET</t>
+        </is>
+      </c>
       <c r="K48" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
       <c r="L48" s="13" t="inlineStr">
@@ -21316,7 +21250,11 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M48" s="13" t="inlineStr"/>
+      <c r="M48" s="21" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
       <c r="N48" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -21324,7 +21262,7 @@
       </c>
       <c r="O48" s="14" t="inlineStr">
         <is>
-          <t>&gt;$100K new. Close date not captured.</t>
+          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale.</t>
         </is>
       </c>
     </row>
@@ -21336,17 +21274,17 @@
       </c>
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>Brand-new &amp; scratch-and-dent kitchen/home appliances – ~185 lots (Thermador, GE Café, Miele, Wolf speed oven, Viking, Bosch…)</t>
+          <t>Party City (Ch. 11) store – fixtures + party merchandise inventory</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D49" s="13" t="inlineStr">
         <is>
-          <t>Edison</t>
+          <t>East Brunswick</t>
         </is>
       </c>
       <c r="E49" s="13" t="inlineStr">
@@ -21355,27 +21293,23 @@
         </is>
       </c>
       <c r="F49" s="13" t="n">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="G49" s="13" t="inlineStr">
         <is>
-          <t>Live + HiBid webcast, 18% BP + 3% card</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H49" s="15" t="n"/>
-      <c r="I49" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
+      <c r="I49" s="13" t="inlineStr"/>
       <c r="J49" s="13" t="inlineStr">
         <is>
-          <t>2026-10-25 01:00 PM ET</t>
+          <t>2026-11-03 11:00 AM ET</t>
         </is>
       </c>
       <c r="K49" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>A.J. Willner</t>
         </is>
       </c>
       <c r="L49" s="13" t="inlineStr">
@@ -21383,11 +21317,7 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M49" s="21" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
+      <c r="M49" s="13" t="inlineStr"/>
       <c r="N49" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -21395,7 +21325,7 @@
       </c>
       <c r="O49" s="14" t="inlineStr">
         <is>
-          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale.</t>
+          <t>Store inventory.</t>
         </is>
       </c>
     </row>
@@ -21407,17 +21337,17 @@
       </c>
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>Party City (Ch. 11) store – fixtures + party merchandise inventory</t>
+          <t>High-end deli (contents not described)</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>restaurant closing</t>
         </is>
       </c>
       <c r="D50" s="13" t="inlineStr">
         <is>
-          <t>East Brunswick</t>
+          <t>Manalapan Township</t>
         </is>
       </c>
       <c r="E50" s="13" t="inlineStr">
@@ -21426,28 +21356,32 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H50" s="15" t="n"/>
-      <c r="I50" s="13" t="inlineStr"/>
+      <c r="I50" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="J50" s="13" t="inlineStr">
         <is>
-          <t>2026-11-03 11:00 AM ET</t>
+          <t>2026-10-19 04:00 PM ET</t>
         </is>
       </c>
       <c r="K50" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
-        </is>
-      </c>
-      <c r="L50" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
+        </is>
+      </c>
+      <c r="L50" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M50" s="13" t="inlineStr"/>
@@ -21458,7 +21392,7 @@
       </c>
       <c r="O50" s="14" t="inlineStr">
         <is>
-          <t>Store inventory.</t>
+          <t>Mon Oct 19 4 PM. No item description on page.</t>
         </is>
       </c>
     </row>
@@ -21470,17 +21404,17 @@
       </c>
       <c r="B51" s="14" t="inlineStr">
         <is>
-          <t>High-end deli (contents not described)</t>
+          <t>Bakery/Cafe Somerville NJ – rack ovens, La Marzocco, food truck (~76 lots)</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
-          <t>restaurant closing</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D51" s="13" t="inlineStr">
         <is>
-          <t>Manalapan Township</t>
+          <t>Somerville</t>
         </is>
       </c>
       <c r="E51" s="13" t="inlineStr">
@@ -21489,32 +21423,32 @@
         </is>
       </c>
       <c r="F51" s="13" t="n">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="G51" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>Live webcast + online (18% BP online)</t>
         </is>
       </c>
       <c r="H51" s="15" t="n"/>
       <c r="I51" s="13" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="J51" s="13" t="inlineStr">
         <is>
-          <t>2026-10-19 04:00 PM ET</t>
+          <t>2026-10-26 02:00 PM ET</t>
         </is>
       </c>
       <c r="K51" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
-        </is>
-      </c>
-      <c r="L51" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>HiBid / Best Buy Auctioneers</t>
+        </is>
+      </c>
+      <c r="L51" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M51" s="13" t="inlineStr"/>
@@ -21525,7 +21459,7 @@
       </c>
       <c r="O51" s="14" t="inlineStr">
         <is>
-          <t>Mon Oct 19 4 PM. No item description on page.</t>
+          <t>Full bakery/cafe commercial kitchen: food truck w/ pizza oven, La Marzocco espresso, Mazzer, Baxter + Empire Logiudice rack ovens, dough depositor, Globe floor mixer, Artic Air / SS refrigeration, fryers, Vitamix, Robot Coupe, display cases, dining furniture. Preview 11 AM sale day; checkout Tue 10/27.</t>
         </is>
       </c>
     </row>
@@ -21537,7 +21471,7 @@
       </c>
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>Bakery/Cafe Somerville NJ – rack ovens, La Marzocco, food truck (~76 lots)</t>
+          <t>Ability to Work kitchen and store – commercial kitchen + store fixtures (~135 lots)</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
@@ -21547,7 +21481,7 @@
       </c>
       <c r="D52" s="13" t="inlineStr">
         <is>
-          <t>Somerville</t>
+          <t>Flemington</t>
         </is>
       </c>
       <c r="E52" s="13" t="inlineStr">
@@ -21556,27 +21490,23 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>Live webcast + online (18% BP online)</t>
+          <t>Timed online (15% BP)</t>
         </is>
       </c>
       <c r="H52" s="15" t="n"/>
-      <c r="I52" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
+      <c r="I52" s="13" t="inlineStr"/>
       <c r="J52" s="13" t="inlineStr">
         <is>
-          <t>2026-10-26 02:00 PM ET</t>
+          <t>2026-10-27 11:02 AM ET</t>
         </is>
       </c>
       <c r="K52" s="13" t="inlineStr">
         <is>
-          <t>HiBid / Best Buy Auctioneers</t>
+          <t>HiBid</t>
         </is>
       </c>
       <c r="L52" s="13" t="inlineStr">
@@ -21592,7 +21522,7 @@
       </c>
       <c r="O52" s="14" t="inlineStr">
         <is>
-          <t>Full bakery/cafe commercial kitchen: food truck w/ pizza oven, La Marzocco espresso, Mazzer, Baxter + Empire Logiudice rack ovens, dough depositor, Globe floor mixer, Artic Air / SS refrigeration, fryers, Vitamix, Robot Coupe, display cases, dining furniture. Preview 11 AM sale day; checkout Tue 10/27.</t>
+          <t>Apprentice/hospitality training cafe-kitchen and store dispersal. Preview 9–11 AM sale day; removal Oct 27 noon–Oct 29.</t>
         </is>
       </c>
     </row>
@@ -21604,17 +21534,17 @@
       </c>
       <c r="B53" s="14" t="inlineStr">
         <is>
-          <t>Ability to Work kitchen and store – commercial kitchen + store fixtures (~135 lots)</t>
+          <t>Wren Kitchens showroom closing – JennAir/Café/KitchenAid/GE Profile appliances + display kitchens</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>showroom closing</t>
         </is>
       </c>
       <c r="D53" s="13" t="inlineStr">
         <is>
-          <t>Flemington</t>
+          <t>Lawrenceville</t>
         </is>
       </c>
       <c r="E53" s="13" t="inlineStr">
@@ -21623,23 +21553,23 @@
         </is>
       </c>
       <c r="F53" s="13" t="n">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="G53" s="13" t="inlineStr">
         <is>
-          <t>Timed online (15% BP)</t>
+          <t>Online auction, 18% BP</t>
         </is>
       </c>
       <c r="H53" s="15" t="n"/>
       <c r="I53" s="13" t="inlineStr"/>
       <c r="J53" s="13" t="inlineStr">
         <is>
-          <t>2026-10-27 11:02 AM ET</t>
+          <t>2026-10-27 09:00 AM ET</t>
         </is>
       </c>
       <c r="K53" s="13" t="inlineStr">
         <is>
-          <t>HiBid</t>
+          <t>Grafe Auction</t>
         </is>
       </c>
       <c r="L53" s="13" t="inlineStr">
@@ -21655,7 +21585,7 @@
       </c>
       <c r="O53" s="14" t="inlineStr">
         <is>
-          <t>Apprentice/hospitality training cafe-kitchen and store dispersal. Preview 9–11 AM sale day; removal Oct 27 noon–Oct 29.</t>
+          <t>Premium floor-model appliances; lots close from Oct 27 9 AM.</t>
         </is>
       </c>
     </row>
@@ -21667,17 +21597,17 @@
       </c>
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>Wren Kitchens showroom closing – JennAir/Café/KitchenAid/GE Profile appliances + display kitchens</t>
+          <t>Milwaukee / Walmart / hardware store mega auction pt 3</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>showroom closing</t>
+          <t>inventory</t>
         </is>
       </c>
       <c r="D54" s="13" t="inlineStr">
         <is>
-          <t>Lawrenceville</t>
+          <t>Mount Holly</t>
         </is>
       </c>
       <c r="E54" s="13" t="inlineStr">
@@ -21686,28 +21616,28 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>239</v>
+        <v>254</v>
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>Online auction, 18% BP</t>
+          <t>HiBid online auction</t>
         </is>
       </c>
       <c r="H54" s="15" t="n"/>
       <c r="I54" s="13" t="inlineStr"/>
       <c r="J54" s="13" t="inlineStr">
         <is>
-          <t>2026-10-27 09:00 AM ET</t>
+          <t>2026-10-19 06:00 PM ET</t>
         </is>
       </c>
       <c r="K54" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
-        </is>
-      </c>
-      <c r="L54" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>HiBid</t>
+        </is>
+      </c>
+      <c r="L54" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M54" s="13" t="inlineStr"/>
@@ -21718,7 +21648,7 @@
       </c>
       <c r="O54" s="14" t="inlineStr">
         <is>
-          <t>Premium floor-model appliances; lots close from Oct 27 9 AM.</t>
+          <t>Close Oct 18 or 19 6 PM (later used).</t>
         </is>
       </c>
     </row>
@@ -21730,17 +21660,17 @@
       </c>
       <c r="B55" s="14" t="inlineStr">
         <is>
-          <t>Milwaukee / Walmart / hardware store mega auction pt 3</t>
+          <t>Wren Kitchens showroom closing – GE/Whirlpool/KitchenAid/Café incl. NIB Café range + 35 kitchens</t>
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>showroom closing</t>
         </is>
       </c>
       <c r="D55" s="13" t="inlineStr">
         <is>
-          <t>Mount Holly</t>
+          <t>Cherry Hill</t>
         </is>
       </c>
       <c r="E55" s="13" t="inlineStr">
@@ -21749,28 +21679,28 @@
         </is>
       </c>
       <c r="F55" s="13" t="n">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="G55" s="13" t="inlineStr">
         <is>
-          <t>HiBid online auction</t>
+          <t>Online auction, openers ~$0.50</t>
         </is>
       </c>
       <c r="H55" s="15" t="n"/>
       <c r="I55" s="13" t="inlineStr"/>
       <c r="J55" s="13" t="inlineStr">
         <is>
-          <t>2026-10-19 06:00 PM ET</t>
+          <t>2026-11-02 11:00 AM ET</t>
         </is>
       </c>
       <c r="K55" s="13" t="inlineStr">
         <is>
-          <t>HiBid</t>
-        </is>
-      </c>
-      <c r="L55" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L55" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M55" s="13" t="inlineStr"/>
@@ -21781,231 +21711,231 @@
       </c>
       <c r="O55" s="14" t="inlineStr">
         <is>
-          <t>Close Oct 18 or 19 6 PM (later used).</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" outlineLevel="1">
-      <c r="A56" s="13" t="inlineStr">
-        <is>
-          <t>NYC / Long Island / NJ</t>
-        </is>
-      </c>
-      <c r="B56" s="14" t="inlineStr">
-        <is>
-          <t>Wren Kitchens showroom closing – GE/Whirlpool/KitchenAid/Café incl. NIB Café range + 35 kitchens</t>
-        </is>
-      </c>
-      <c r="C56" s="13" t="inlineStr">
-        <is>
-          <t>showroom closing</t>
-        </is>
-      </c>
-      <c r="D56" s="13" t="inlineStr">
-        <is>
-          <t>Cherry Hill</t>
-        </is>
-      </c>
-      <c r="E56" s="13" t="inlineStr">
-        <is>
-          <t>NJ</t>
-        </is>
-      </c>
-      <c r="F56" s="13" t="n">
-        <v>266</v>
-      </c>
-      <c r="G56" s="13" t="inlineStr">
-        <is>
-          <t>Online auction, openers ~$0.50</t>
-        </is>
-      </c>
-      <c r="H56" s="15" t="n"/>
-      <c r="I56" s="13" t="inlineStr"/>
-      <c r="J56" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-02 11:00 AM ET</t>
-        </is>
-      </c>
-      <c r="K56" s="13" t="inlineStr">
-        <is>
-          <t>Grafe Auction</t>
-        </is>
-      </c>
-      <c r="L56" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M56" s="13" t="inlineStr"/>
-      <c r="N56" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O56" s="14" t="inlineStr">
-        <is>
           <t>Lots close from Nov 2 11 AM.</t>
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B56" s="17" t="inlineStr">
+        <is>
+          <t>23 item(s)</t>
+        </is>
+      </c>
+      <c r="C56" s="18" t="n"/>
+      <c r="D56" s="18" t="n"/>
+      <c r="E56" s="18" t="n"/>
+      <c r="F56" s="18" t="n"/>
+      <c r="G56" s="18" t="n"/>
+      <c r="H56" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="18" t="n"/>
+      <c r="J56" s="18" t="n"/>
+      <c r="K56" s="18" t="n"/>
+      <c r="L56" s="18" t="n"/>
+      <c r="M56" s="18" t="n"/>
+      <c r="N56" s="18" t="n"/>
+      <c r="O56" s="18" t="n"/>
+    </row>
     <row r="57">
-      <c r="A57" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — NYC / Long Island / NJ</t>
-        </is>
-      </c>
-      <c r="B57" s="17" t="inlineStr">
-        <is>
-          <t>24 item(s)</t>
-        </is>
-      </c>
-      <c r="C57" s="18" t="n"/>
-      <c r="D57" s="18" t="n"/>
-      <c r="E57" s="18" t="n"/>
-      <c r="F57" s="18" t="n"/>
-      <c r="G57" s="18" t="n"/>
-      <c r="H57" s="19" t="n">
+      <c r="A57" s="11" t="inlineStr">
+        <is>
+          <t>▸ Eastern PA / Mid-Atlantic  (1)</t>
+        </is>
+      </c>
+      <c r="B57" s="12" t="n"/>
+      <c r="C57" s="12" t="n"/>
+      <c r="D57" s="12" t="n"/>
+      <c r="E57" s="12" t="n"/>
+      <c r="F57" s="12" t="n"/>
+      <c r="G57" s="12" t="n"/>
+      <c r="H57" s="12" t="n"/>
+      <c r="I57" s="12" t="n"/>
+      <c r="J57" s="12" t="n"/>
+      <c r="K57" s="12" t="n"/>
+      <c r="L57" s="12" t="n"/>
+      <c r="M57" s="12" t="n"/>
+      <c r="N57" s="12" t="n"/>
+      <c r="O57" s="12" t="n"/>
+    </row>
+    <row r="58" outlineLevel="1">
+      <c r="A58" s="13" t="inlineStr">
+        <is>
+          <t>Eastern PA / Mid-Atlantic</t>
+        </is>
+      </c>
+      <c r="B58" s="14" t="inlineStr">
+        <is>
+          <t>October restaurant consignment – Hobart, Rational, True + NEW scratch-and-dent Migali/Avantco</t>
+        </is>
+      </c>
+      <c r="C58" s="13" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D58" s="13" t="inlineStr">
+        <is>
+          <t>Harrisburg</t>
+        </is>
+      </c>
+      <c r="E58" s="13" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="F58" s="13" t="n">
+        <v>340</v>
+      </c>
+      <c r="G58" s="13" t="inlineStr">
+        <is>
+          <t>Online auction, 15% BP, ships $55/pallet</t>
+        </is>
+      </c>
+      <c r="H58" s="15" t="n"/>
+      <c r="I58" s="13" t="inlineStr"/>
+      <c r="J58" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-21 11:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K58" s="13" t="inlineStr">
+        <is>
+          <t>Restaurant Auction Co</t>
+        </is>
+      </c>
+      <c r="L58" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M58" s="13" t="inlineStr"/>
+      <c r="N58" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O58" s="14" t="inlineStr">
+        <is>
+          <t>Closes Oct 21 10 or 11 AM (later used). Shippable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Eastern PA / Mid-Atlantic</t>
+        </is>
+      </c>
+      <c r="B59" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C59" s="18" t="n"/>
+      <c r="D59" s="18" t="n"/>
+      <c r="E59" s="18" t="n"/>
+      <c r="F59" s="18" t="n"/>
+      <c r="G59" s="18" t="n"/>
+      <c r="H59" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I57" s="18" t="n"/>
-      <c r="J57" s="18" t="n"/>
-      <c r="K57" s="18" t="n"/>
-      <c r="L57" s="18" t="n"/>
-      <c r="M57" s="18" t="n"/>
-      <c r="N57" s="18" t="n"/>
-      <c r="O57" s="18" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="11" t="inlineStr">
-        <is>
-          <t>▸ Eastern PA / Mid-Atlantic  (1)</t>
-        </is>
-      </c>
-      <c r="B58" s="12" t="n"/>
-      <c r="C58" s="12" t="n"/>
-      <c r="D58" s="12" t="n"/>
-      <c r="E58" s="12" t="n"/>
-      <c r="F58" s="12" t="n"/>
-      <c r="G58" s="12" t="n"/>
-      <c r="H58" s="12" t="n"/>
-      <c r="I58" s="12" t="n"/>
-      <c r="J58" s="12" t="n"/>
-      <c r="K58" s="12" t="n"/>
-      <c r="L58" s="12" t="n"/>
-      <c r="M58" s="12" t="n"/>
-      <c r="N58" s="12" t="n"/>
-      <c r="O58" s="12" t="n"/>
-    </row>
-    <row r="59" outlineLevel="1">
-      <c r="A59" s="13" t="inlineStr">
-        <is>
-          <t>Eastern PA / Mid-Atlantic</t>
-        </is>
-      </c>
-      <c r="B59" s="14" t="inlineStr">
-        <is>
-          <t>October restaurant consignment – Hobart, Rational, True + NEW scratch-and-dent Migali/Avantco</t>
-        </is>
-      </c>
-      <c r="C59" s="13" t="inlineStr">
+      <c r="I59" s="18" t="n"/>
+      <c r="J59" s="18" t="n"/>
+      <c r="K59" s="18" t="n"/>
+      <c r="L59" s="18" t="n"/>
+      <c r="M59" s="18" t="n"/>
+      <c r="N59" s="18" t="n"/>
+      <c r="O59" s="18" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t>▸ Upstate / Western NY  (3)</t>
+        </is>
+      </c>
+      <c r="B60" s="12" t="n"/>
+      <c r="C60" s="12" t="n"/>
+      <c r="D60" s="12" t="n"/>
+      <c r="E60" s="12" t="n"/>
+      <c r="F60" s="12" t="n"/>
+      <c r="G60" s="12" t="n"/>
+      <c r="H60" s="12" t="n"/>
+      <c r="I60" s="12" t="n"/>
+      <c r="J60" s="12" t="n"/>
+      <c r="K60" s="12" t="n"/>
+      <c r="L60" s="12" t="n"/>
+      <c r="M60" s="12" t="n"/>
+      <c r="N60" s="12" t="n"/>
+      <c r="O60" s="12" t="n"/>
+    </row>
+    <row r="61" outlineLevel="1">
+      <c r="A61" s="13" t="inlineStr">
+        <is>
+          <t>Upstate / Western NY</t>
+        </is>
+      </c>
+      <c r="B61" s="14" t="inlineStr">
+        <is>
+          <t>Former Taco Del Mar – stainless, warmers, walk-in panels</t>
+        </is>
+      </c>
+      <c r="C61" s="13" t="inlineStr">
         <is>
           <t>restaurant</t>
         </is>
       </c>
-      <c r="D59" s="13" t="inlineStr">
-        <is>
-          <t>Harrisburg</t>
-        </is>
-      </c>
-      <c r="E59" s="13" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="F59" s="13" t="n">
-        <v>340</v>
-      </c>
-      <c r="G59" s="13" t="inlineStr">
-        <is>
-          <t>Online auction, 15% BP, ships $55/pallet</t>
-        </is>
-      </c>
-      <c r="H59" s="15" t="n"/>
-      <c r="I59" s="13" t="inlineStr"/>
-      <c r="J59" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-21 11:00 AM ET</t>
-        </is>
-      </c>
-      <c r="K59" s="13" t="inlineStr">
-        <is>
-          <t>Restaurant Auction Co</t>
-        </is>
-      </c>
-      <c r="L59" s="20" t="inlineStr">
+      <c r="D61" s="13" t="inlineStr">
+        <is>
+          <t>Watson</t>
+        </is>
+      </c>
+      <c r="E61" s="13" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="F61" s="13" t="n">
+        <v>260</v>
+      </c>
+      <c r="G61" s="13" t="inlineStr">
+        <is>
+          <t>HiBid online auction</t>
+        </is>
+      </c>
+      <c r="H61" s="15" t="n"/>
+      <c r="I61" s="13" t="inlineStr"/>
+      <c r="J61" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-20 06:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K61" s="13" t="inlineStr">
+        <is>
+          <t>Adirondack Asset / HiBid</t>
+        </is>
+      </c>
+      <c r="L61" s="20" t="inlineStr">
         <is>
           <t>ENDING SOON</t>
         </is>
       </c>
-      <c r="M59" s="13" t="inlineStr"/>
-      <c r="N59" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O59" s="14" t="inlineStr">
-        <is>
-          <t>Closes Oct 21 10 or 11 AM (later used). Shippable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Eastern PA / Mid-Atlantic</t>
-        </is>
-      </c>
-      <c r="B60" s="17" t="inlineStr">
-        <is>
-          <t>1 item(s)</t>
-        </is>
-      </c>
-      <c r="C60" s="18" t="n"/>
-      <c r="D60" s="18" t="n"/>
-      <c r="E60" s="18" t="n"/>
-      <c r="F60" s="18" t="n"/>
-      <c r="G60" s="18" t="n"/>
-      <c r="H60" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I60" s="18" t="n"/>
-      <c r="J60" s="18" t="n"/>
-      <c r="K60" s="18" t="n"/>
-      <c r="L60" s="18" t="n"/>
-      <c r="M60" s="18" t="n"/>
-      <c r="N60" s="18" t="n"/>
-      <c r="O60" s="18" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="11" t="inlineStr">
-        <is>
-          <t>▸ Upstate / Western NY  (3)</t>
-        </is>
-      </c>
-      <c r="B61" s="12" t="n"/>
-      <c r="C61" s="12" t="n"/>
-      <c r="D61" s="12" t="n"/>
-      <c r="E61" s="12" t="n"/>
-      <c r="F61" s="12" t="n"/>
-      <c r="G61" s="12" t="n"/>
-      <c r="H61" s="12" t="n"/>
-      <c r="I61" s="12" t="n"/>
-      <c r="J61" s="12" t="n"/>
-      <c r="K61" s="12" t="n"/>
-      <c r="L61" s="12" t="n"/>
-      <c r="M61" s="12" t="n"/>
-      <c r="N61" s="12" t="n"/>
-      <c r="O61" s="12" t="n"/>
+      <c r="M61" s="13" t="inlineStr"/>
+      <c r="N61" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O61" s="14" t="inlineStr">
+        <is>
+          <t>Small lot.</t>
+        </is>
+      </c>
     </row>
     <row r="62" outlineLevel="1">
       <c r="A62" s="13" t="inlineStr">
@@ -22015,7 +21945,7 @@
       </c>
       <c r="B62" s="14" t="inlineStr">
         <is>
-          <t>Former Taco Del Mar – stainless, warmers, walk-in panels</t>
+          <t>Closed restaurant – coolers, fridges, prep tables</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
@@ -22025,7 +21955,7 @@
       </c>
       <c r="D62" s="13" t="inlineStr">
         <is>
-          <t>Watson</t>
+          <t>Palmyra</t>
         </is>
       </c>
       <c r="E62" s="13" t="inlineStr">
@@ -22034,23 +21964,23 @@
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>260</v>
+        <v>333</v>
       </c>
       <c r="G62" s="13" t="inlineStr">
         <is>
-          <t>HiBid online auction</t>
+          <t>HiBid, 15% BP</t>
         </is>
       </c>
       <c r="H62" s="15" t="n"/>
       <c r="I62" s="13" t="inlineStr"/>
       <c r="J62" s="13" t="inlineStr">
         <is>
-          <t>2026-10-20 06:00 PM ET</t>
+          <t>2026-10-19 07:00 PM ET</t>
         </is>
       </c>
       <c r="K62" s="13" t="inlineStr">
         <is>
-          <t>Adirondack Asset / HiBid</t>
+          <t>Reynolds Auction Co / HiBid</t>
         </is>
       </c>
       <c r="L62" s="20" t="inlineStr">
@@ -22066,7 +21996,7 @@
       </c>
       <c r="O62" s="14" t="inlineStr">
         <is>
-          <t>Small lot.</t>
+          <t>No new out-of-state bidders. Small.</t>
         </is>
       </c>
     </row>
@@ -22078,7 +22008,7 @@
       </c>
       <c r="B63" s="14" t="inlineStr">
         <is>
-          <t>Closed restaurant – coolers, fridges, prep tables</t>
+          <t>Restaurant &amp; fitness equipment</t>
         </is>
       </c>
       <c r="C63" s="13" t="inlineStr">
@@ -22088,7 +22018,7 @@
       </c>
       <c r="D63" s="13" t="inlineStr">
         <is>
-          <t>Palmyra</t>
+          <t>Williamsville</t>
         </is>
       </c>
       <c r="E63" s="13" t="inlineStr">
@@ -22097,28 +22027,28 @@
         </is>
       </c>
       <c r="F63" s="13" t="n">
-        <v>333</v>
+        <v>408</v>
       </c>
       <c r="G63" s="13" t="inlineStr">
         <is>
-          <t>HiBid, 15% BP</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H63" s="15" t="n"/>
       <c r="I63" s="13" t="inlineStr"/>
       <c r="J63" s="13" t="inlineStr">
         <is>
-          <t>2026-10-19 07:00 PM ET</t>
+          <t>2026-10-26 07:30 PM ET</t>
         </is>
       </c>
       <c r="K63" s="13" t="inlineStr">
         <is>
-          <t>Reynolds Auction Co / HiBid</t>
-        </is>
-      </c>
-      <c r="L63" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>Cash Auctions</t>
+        </is>
+      </c>
+      <c r="L63" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M63" s="13" t="inlineStr"/>
@@ -22129,231 +22059,231 @@
       </c>
       <c r="O63" s="14" t="inlineStr">
         <is>
-          <t>No new out-of-state bidders. Small.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" outlineLevel="1">
-      <c r="A64" s="13" t="inlineStr">
-        <is>
-          <t>Upstate / Western NY</t>
-        </is>
-      </c>
-      <c r="B64" s="14" t="inlineStr">
-        <is>
-          <t>Restaurant &amp; fitness equipment</t>
-        </is>
-      </c>
-      <c r="C64" s="13" t="inlineStr">
-        <is>
-          <t>restaurant</t>
-        </is>
-      </c>
-      <c r="D64" s="13" t="inlineStr">
-        <is>
-          <t>Williamsville</t>
-        </is>
-      </c>
-      <c r="E64" s="13" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="F64" s="13" t="n">
-        <v>408</v>
-      </c>
-      <c r="G64" s="13" t="inlineStr">
+          <t>Lots not reviewed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Upstate / Western NY</t>
+        </is>
+      </c>
+      <c r="B64" s="17" t="inlineStr">
+        <is>
+          <t>3 item(s)</t>
+        </is>
+      </c>
+      <c r="C64" s="18" t="n"/>
+      <c r="D64" s="18" t="n"/>
+      <c r="E64" s="18" t="n"/>
+      <c r="F64" s="18" t="n"/>
+      <c r="G64" s="18" t="n"/>
+      <c r="H64" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I64" s="18" t="n"/>
+      <c r="J64" s="18" t="n"/>
+      <c r="K64" s="18" t="n"/>
+      <c r="L64" s="18" t="n"/>
+      <c r="M64" s="18" t="n"/>
+      <c r="N64" s="18" t="n"/>
+      <c r="O64" s="18" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="11" t="inlineStr">
+        <is>
+          <t>▸ Virginia  (1)</t>
+        </is>
+      </c>
+      <c r="B65" s="12" t="n"/>
+      <c r="C65" s="12" t="n"/>
+      <c r="D65" s="12" t="n"/>
+      <c r="E65" s="12" t="n"/>
+      <c r="F65" s="12" t="n"/>
+      <c r="G65" s="12" t="n"/>
+      <c r="H65" s="12" t="n"/>
+      <c r="I65" s="12" t="n"/>
+      <c r="J65" s="12" t="n"/>
+      <c r="K65" s="12" t="n"/>
+      <c r="L65" s="12" t="n"/>
+      <c r="M65" s="12" t="n"/>
+      <c r="N65" s="12" t="n"/>
+      <c r="O65" s="12" t="n"/>
+    </row>
+    <row r="66" outlineLevel="1">
+      <c r="A66" s="13" t="inlineStr">
+        <is>
+          <t>Virginia</t>
+        </is>
+      </c>
+      <c r="B66" s="14" t="inlineStr">
+        <is>
+          <t>Haynes Furniture / The Dump – 12 stores closing (furniture, mattresses)</t>
+        </is>
+      </c>
+      <c r="C66" s="13" t="inlineStr">
+        <is>
+          <t>retail GOB</t>
+        </is>
+      </c>
+      <c r="D66" s="13" t="inlineStr">
+        <is>
+          <t>Virginia Beach</t>
+        </is>
+      </c>
+      <c r="E66" s="13" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="F66" s="13" t="n">
+        <v>456</v>
+      </c>
+      <c r="G66" s="13" t="inlineStr">
+        <is>
+          <t>Retail GOB markdowns</t>
+        </is>
+      </c>
+      <c r="H66" s="15" t="n"/>
+      <c r="I66" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="J66" s="13" t="inlineStr"/>
+      <c r="K66" s="13" t="inlineStr">
+        <is>
+          <t>SB360 (PR Newswire)</t>
+        </is>
+      </c>
+      <c r="L66" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M66" s="13" t="inlineStr"/>
+      <c r="N66" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O66" s="14" t="inlineStr">
+        <is>
+          <t>Posted Oct 8. Multi-state (VA/AZ/GA/IL/TX); pinned at Virginia Beach. Home goods only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Virginia</t>
+        </is>
+      </c>
+      <c r="B67" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C67" s="18" t="n"/>
+      <c r="D67" s="18" t="n"/>
+      <c r="E67" s="18" t="n"/>
+      <c r="F67" s="18" t="n"/>
+      <c r="G67" s="18" t="n"/>
+      <c r="H67" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" s="18" t="n"/>
+      <c r="J67" s="18" t="n"/>
+      <c r="K67" s="18" t="n"/>
+      <c r="L67" s="18" t="n"/>
+      <c r="M67" s="18" t="n"/>
+      <c r="N67" s="18" t="n"/>
+      <c r="O67" s="18" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="inlineStr">
+        <is>
+          <t>▸ Midwest  (3)</t>
+        </is>
+      </c>
+      <c r="B68" s="12" t="n"/>
+      <c r="C68" s="12" t="n"/>
+      <c r="D68" s="12" t="n"/>
+      <c r="E68" s="12" t="n"/>
+      <c r="F68" s="12" t="n"/>
+      <c r="G68" s="12" t="n"/>
+      <c r="H68" s="12" t="n"/>
+      <c r="I68" s="12" t="n"/>
+      <c r="J68" s="12" t="n"/>
+      <c r="K68" s="12" t="n"/>
+      <c r="L68" s="12" t="n"/>
+      <c r="M68" s="12" t="n"/>
+      <c r="N68" s="12" t="n"/>
+      <c r="O68" s="12" t="n"/>
+    </row>
+    <row r="69" outlineLevel="1">
+      <c r="A69" s="13" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="B69" s="14" t="inlineStr">
+        <is>
+          <t>Freshway Market whole-grocery liquidation – refrigeration racks, cases, walk-ins, generator</t>
+        </is>
+      </c>
+      <c r="C69" s="13" t="inlineStr">
+        <is>
+          <t>store closing</t>
+        </is>
+      </c>
+      <c r="D69" s="13" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="E69" s="13" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="F69" s="13" t="n">
+        <v>862</v>
+      </c>
+      <c r="G69" s="13" t="inlineStr">
         <is>
           <t>Online auction</t>
         </is>
       </c>
-      <c r="H64" s="15" t="n"/>
-      <c r="I64" s="13" t="inlineStr"/>
-      <c r="J64" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26 07:30 PM ET</t>
-        </is>
-      </c>
-      <c r="K64" s="13" t="inlineStr">
-        <is>
-          <t>Cash Auctions</t>
-        </is>
-      </c>
-      <c r="L64" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M64" s="13" t="inlineStr"/>
-      <c r="N64" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O64" s="14" t="inlineStr">
-        <is>
-          <t>Lots not reviewed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Upstate / Western NY</t>
-        </is>
-      </c>
-      <c r="B65" s="17" t="inlineStr">
-        <is>
-          <t>3 item(s)</t>
-        </is>
-      </c>
-      <c r="C65" s="18" t="n"/>
-      <c r="D65" s="18" t="n"/>
-      <c r="E65" s="18" t="n"/>
-      <c r="F65" s="18" t="n"/>
-      <c r="G65" s="18" t="n"/>
-      <c r="H65" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I65" s="18" t="n"/>
-      <c r="J65" s="18" t="n"/>
-      <c r="K65" s="18" t="n"/>
-      <c r="L65" s="18" t="n"/>
-      <c r="M65" s="18" t="n"/>
-      <c r="N65" s="18" t="n"/>
-      <c r="O65" s="18" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="11" t="inlineStr">
-        <is>
-          <t>▸ Virginia  (1)</t>
-        </is>
-      </c>
-      <c r="B66" s="12" t="n"/>
-      <c r="C66" s="12" t="n"/>
-      <c r="D66" s="12" t="n"/>
-      <c r="E66" s="12" t="n"/>
-      <c r="F66" s="12" t="n"/>
-      <c r="G66" s="12" t="n"/>
-      <c r="H66" s="12" t="n"/>
-      <c r="I66" s="12" t="n"/>
-      <c r="J66" s="12" t="n"/>
-      <c r="K66" s="12" t="n"/>
-      <c r="L66" s="12" t="n"/>
-      <c r="M66" s="12" t="n"/>
-      <c r="N66" s="12" t="n"/>
-      <c r="O66" s="12" t="n"/>
-    </row>
-    <row r="67" outlineLevel="1">
-      <c r="A67" s="13" t="inlineStr">
-        <is>
-          <t>Virginia</t>
-        </is>
-      </c>
-      <c r="B67" s="14" t="inlineStr">
-        <is>
-          <t>Haynes Furniture / The Dump – 12 stores closing (furniture, mattresses)</t>
-        </is>
-      </c>
-      <c r="C67" s="13" t="inlineStr">
-        <is>
-          <t>retail GOB</t>
-        </is>
-      </c>
-      <c r="D67" s="13" t="inlineStr">
-        <is>
-          <t>Virginia Beach</t>
-        </is>
-      </c>
-      <c r="E67" s="13" t="inlineStr">
-        <is>
-          <t>VA</t>
-        </is>
-      </c>
-      <c r="F67" s="13" t="n">
-        <v>456</v>
-      </c>
-      <c r="G67" s="13" t="inlineStr">
-        <is>
-          <t>Retail GOB markdowns</t>
-        </is>
-      </c>
-      <c r="H67" s="15" t="n"/>
-      <c r="I67" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="J67" s="13" t="inlineStr"/>
-      <c r="K67" s="13" t="inlineStr">
-        <is>
-          <t>SB360 (PR Newswire)</t>
-        </is>
-      </c>
-      <c r="L67" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M67" s="13" t="inlineStr"/>
-      <c r="N67" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O67" s="14" t="inlineStr">
-        <is>
-          <t>Posted Oct 8. Multi-state (VA/AZ/GA/IL/TX); pinned at Virginia Beach. Home goods only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Virginia</t>
-        </is>
-      </c>
-      <c r="B68" s="17" t="inlineStr">
-        <is>
-          <t>1 item(s)</t>
-        </is>
-      </c>
-      <c r="C68" s="18" t="n"/>
-      <c r="D68" s="18" t="n"/>
-      <c r="E68" s="18" t="n"/>
-      <c r="F68" s="18" t="n"/>
-      <c r="G68" s="18" t="n"/>
-      <c r="H68" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I68" s="18" t="n"/>
-      <c r="J68" s="18" t="n"/>
-      <c r="K68" s="18" t="n"/>
-      <c r="L68" s="18" t="n"/>
-      <c r="M68" s="18" t="n"/>
-      <c r="N68" s="18" t="n"/>
-      <c r="O68" s="18" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="11" t="inlineStr">
-        <is>
-          <t>▸ Midwest  (2)</t>
-        </is>
-      </c>
-      <c r="B69" s="12" t="n"/>
-      <c r="C69" s="12" t="n"/>
-      <c r="D69" s="12" t="n"/>
-      <c r="E69" s="12" t="n"/>
-      <c r="F69" s="12" t="n"/>
-      <c r="G69" s="12" t="n"/>
-      <c r="H69" s="12" t="n"/>
-      <c r="I69" s="12" t="n"/>
-      <c r="J69" s="12" t="n"/>
-      <c r="K69" s="12" t="n"/>
-      <c r="L69" s="12" t="n"/>
-      <c r="M69" s="12" t="n"/>
-      <c r="N69" s="12" t="n"/>
-      <c r="O69" s="12" t="n"/>
+      <c r="H69" s="15" t="n"/>
+      <c r="I69" s="13" t="inlineStr"/>
+      <c r="J69" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-20 11:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K69" s="13" t="inlineStr">
+        <is>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L69" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M69" s="13" t="inlineStr"/>
+      <c r="N69" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O69" s="14" t="inlineStr">
+        <is>
+          <t>Closes from Oct 20 10 AM CDT.</t>
+        </is>
+      </c>
     </row>
     <row r="70" outlineLevel="1">
       <c r="A70" s="13" t="inlineStr">
@@ -22363,17 +22293,17 @@
       </c>
       <c r="B70" s="14" t="inlineStr">
         <is>
-          <t>Freshway Market whole-grocery liquidation – refrigeration racks, cases, walk-ins, generator</t>
+          <t>American Sale – total liquidation, all 7 stores (pools, hot tubs, grills, holiday decor)</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>retail GOB</t>
         </is>
       </c>
       <c r="D70" s="13" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Chicagoland</t>
         </is>
       </c>
       <c r="E70" s="13" t="inlineStr">
@@ -22382,28 +22312,28 @@
         </is>
       </c>
       <c r="F70" s="13" t="n">
-        <v>862</v>
+        <v>876</v>
       </c>
       <c r="G70" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Retail GOB, up to 70% off</t>
         </is>
       </c>
       <c r="H70" s="15" t="n"/>
-      <c r="I70" s="13" t="inlineStr"/>
-      <c r="J70" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-20 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="I70" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="J70" s="13" t="inlineStr"/>
       <c r="K70" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
-        </is>
-      </c>
-      <c r="L70" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>Tiger Group (PR Newswire)</t>
+        </is>
+      </c>
+      <c r="L70" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M70" s="13" t="inlineStr"/>
@@ -22414,7 +22344,7 @@
       </c>
       <c r="O70" s="14" t="inlineStr">
         <is>
-          <t>Closes from Oct 20 10 AM CDT.</t>
+          <t>Posted Oct 15. Watch for a bulk/fixture auction.</t>
         </is>
       </c>
     </row>
@@ -22426,47 +22356,47 @@
       </c>
       <c r="B71" s="14" t="inlineStr">
         <is>
-          <t>American Sale – total liquidation, all 7 stores (pools, hot tubs, grills, holiday decor)</t>
+          <t>Straub's Fine Foods store equipment – bakery, kitchen, meat room, Hussmann refrigeration</t>
         </is>
       </c>
       <c r="C71" s="13" t="inlineStr">
         <is>
-          <t>retail GOB</t>
+          <t>grocery/restaurant</t>
         </is>
       </c>
       <c r="D71" s="13" t="inlineStr">
         <is>
-          <t>Chicagoland</t>
+          <t>St. Louis</t>
         </is>
       </c>
       <c r="E71" s="13" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="F71" s="13" t="n">
-        <v>876</v>
+        <v>1046</v>
       </c>
       <c r="G71" s="13" t="inlineStr">
         <is>
-          <t>Retail GOB, up to 70% off</t>
+          <t>Online auction (18% BP)</t>
         </is>
       </c>
       <c r="H71" s="15" t="n"/>
-      <c r="I71" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="J71" s="13" t="inlineStr"/>
+      <c r="I71" s="13" t="inlineStr"/>
+      <c r="J71" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-21 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K71" s="13" t="inlineStr">
         <is>
-          <t>Tiger Group (PR Newswire)</t>
-        </is>
-      </c>
-      <c r="L71" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L71" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M71" s="13" t="inlineStr"/>
@@ -22477,7 +22407,7 @@
       </c>
       <c r="O71" s="14" t="inlineStr">
         <is>
-          <t>Posted Oct 15. Watch for a bulk/fixture auction.</t>
+          <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis.</t>
         </is>
       </c>
     </row>
@@ -22489,7 +22419,7 @@
       </c>
       <c r="B72" s="17" t="inlineStr">
         <is>
-          <t>2 item(s)</t>
+          <t>3 item(s)</t>
         </is>
       </c>
       <c r="C72" s="18" t="n"/>
@@ -22746,7 +22676,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId17"/>
@@ -22776,12 +22706,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N53" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N54" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N55" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N56" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N59" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N58" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N61" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N62" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N63" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N64" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N67" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N66" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N69" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N70" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N71" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N74" r:id="rId52"/>
@@ -22797,7 +22727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -23091,7 +23021,7 @@
       </c>
       <c r="O4" s="14" t="inlineStr">
         <is>
-          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed]</t>
+          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23156,59 +23086,61 @@
       </c>
       <c r="O5" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed]</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>Greater Boston / South Shore (&lt;50mi)</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>Closed Best Buy Outlet – pallet racking, Big Joe order pickers, appliance dollies, carts, cages</t>
+          <t>Auctionfuel returns catalog – 100+ single appliance-part lots (Louisville)</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>store closing fixtures</t>
+          <t>auction catalog</t>
         </is>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Brockton</t>
+          <t>Louisville</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>KY</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>11</v>
+        <v>832</v>
       </c>
       <c r="G6" s="13" t="inlineStr">
         <is>
-          <t>Racking $40/upright, $80/level; pickers $1,000 OBO</t>
-        </is>
-      </c>
-      <c r="H6" s="15" t="n"/>
-      <c r="I6" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="J6" s="13" t="inlineStr"/>
+          <t>$0–1 openers + 15% BP + $1/lot</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="13" t="inlineStr"/>
+      <c r="J6" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 02:00 PM ET</t>
+        </is>
+      </c>
       <c r="K6" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>HiBid (Auctionfuel)</t>
         </is>
       </c>
       <c r="L6" s="13" t="inlineStr">
         <is>
-          <t>REMOVED</t>
+          <t>EXPIRED (2026-10-19 02:00 PM ET)</t>
         </is>
       </c>
       <c r="M6" s="13" t="inlineStr"/>
@@ -23219,18 +23151,214 @@
       </c>
       <c r="O6" s="14" t="inlineStr">
         <is>
+          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Maine / VT / Northern NH</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>Oola Bowls secured-party sale – restaurant equipment bought new 2024-25 (Electro Freeze, Scotsman, Atosa)</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Scarborough</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>ME</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>104</v>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>Online auction (freezers $80–150 when seen)</t>
+        </is>
+      </c>
+      <c r="H7" s="15" t="n"/>
+      <c r="I7" s="13" t="inlineStr"/>
+      <c r="J7" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 01:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K7" s="13" t="inlineStr">
+        <is>
+          <t>Keenan Auction / Proxibid</t>
+        </is>
+      </c>
+      <c r="L7" s="13" t="inlineStr">
+        <is>
+          <t>EXPIRED (2026-10-19 01:00 PM ET)</t>
+        </is>
+      </c>
+      <c r="M7" s="13" t="inlineStr"/>
+      <c r="N7" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O7" s="14" t="inlineStr">
+        <is>
+          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed]</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Greater Boston / South Shore (&lt;50mi)</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Closed Best Buy Outlet – pallet racking, Big Joe order pickers, appliance dollies, carts, cages</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>store closing fixtures</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>Brockton</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>Racking $40/upright, $80/level; pickers $1,000 OBO</t>
+        </is>
+      </c>
+      <c r="H8" s="15" t="n"/>
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="J8" s="13" t="inlineStr"/>
+      <c r="K8" s="13" t="inlineStr">
+        <is>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L8" s="13" t="inlineStr">
+        <is>
+          <t>REMOVED</t>
+        </is>
+      </c>
+      <c r="M8" s="13" t="inlineStr"/>
+      <c r="N8" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O8" s="14" t="inlineStr">
+        <is>
           <t>200 Westgate Dr. Fixtures/equipment only, no merchandise. On site daily. CL deleted by author (HTTP 410) as of 2026-10-19 midday recheck.</t>
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>Like-new restaurant – steam tables, Coldline, Cleveland cook-and-hold, fryers, True freezers</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>auction</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Staten Island</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>203</v>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>Live + webcast, 18% BP + 3%</t>
+        </is>
+      </c>
+      <c r="H9" s="15" t="n"/>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 01:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K9" s="13" t="inlineStr">
+        <is>
+          <t>HiBid (Best Buy Auctioneers)</t>
+        </is>
+      </c>
+      <c r="L9" s="13" t="inlineStr">
+        <is>
+          <t>EXPIRED (2026-10-19 01:00 PM ET)</t>
+        </is>
+      </c>
+      <c r="M9" s="13" t="inlineStr"/>
+      <c r="N9" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O9" s="14" t="inlineStr">
+        <is>
+          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O6"/>
+  <autoFilter ref="A1:O9"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Lot Recon 2026-10-20 11am ET: +3 business liquidations (U.S. Vision Montclair NJ, Baonanas Jersey City NJ, Rush Bowls Westfield NJ), prune closed Freshway Market Chicago
</commit_message>
<xml_diff>
--- a/lot_recon.xlsx
+++ b/lot_recon.xlsx
@@ -20,8 +20,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wolf New'!$A$1:$O$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Wolf Used'!$A$1:$O$189</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Wolf Unclear'!$A$1:$O$40</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$82</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 2026-10-20 08:03 ET</t>
+          <t>Last updated: 2026-10-20 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Active listings: 293 · Removed: 13</t>
+          <t>Active listings: 295 · Removed: 14</t>
         </is>
       </c>
     </row>
@@ -679,7 +679,7 @@
         <v>164</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>608011.6</v>
+        <v>608022.6</v>
       </c>
       <c r="D10" t="n">
         <v>3</v>
@@ -695,7 +695,7 @@
         <v>31</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>137840</v>
+        <v>137850</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
@@ -708,13 +708,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13">
@@ -724,10 +724,10 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>980382.58</v>
+        <v>980403.58</v>
       </c>
     </row>
     <row r="15">
@@ -1007,7 +1007,7 @@
         <v>9</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>64740</v>
+        <v>64751</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C24" t="n">
         <v>1</v>
@@ -1037,7 +1037,7 @@
         <v>24</v>
       </c>
       <c r="G24" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="H24" s="6" t="n">
         <v>440141</v>
@@ -1073,7 +1073,7 @@
         <v>1</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>1515</v>
+        <v>1525</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C30" t="n">
         <v>2</v>
@@ -1235,7 +1235,7 @@
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H30" s="6" t="n">
         <v>5</v>
@@ -6860,11 +6860,11 @@
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>$90 high bid (16 bids)</t>
+          <t>$101 high bid (17 bids)</t>
         </is>
       </c>
       <c r="H34" s="15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="I34" s="13" t="inlineStr"/>
       <c r="J34" s="13" t="inlineStr">
@@ -7667,7 +7667,7 @@
       <c r="F47" s="18" t="n"/>
       <c r="G47" s="18" t="n"/>
       <c r="H47" s="19" t="n">
-        <v>33140</v>
+        <v>33151</v>
       </c>
       <c r="I47" s="18" t="n"/>
       <c r="J47" s="18" t="n"/>
@@ -18194,11 +18194,11 @@
       </c>
       <c r="G35" s="13" t="inlineStr">
         <is>
-          <t>$15 high bid</t>
+          <t>$25 high bid (9 bids)</t>
         </is>
       </c>
       <c r="H35" s="15" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="I35" s="13" t="inlineStr"/>
       <c r="J35" s="13" t="inlineStr">
@@ -18245,7 +18245,7 @@
       <c r="F36" s="18" t="n"/>
       <c r="G36" s="18" t="n"/>
       <c r="H36" s="19" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="I36" s="18" t="n"/>
       <c r="J36" s="18" t="n"/>
@@ -18478,7 +18478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O82"/>
+  <dimension ref="A1:O84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -20275,7 +20275,7 @@
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>▸ NYC / Long Island / NJ  (22)</t>
+          <t>▸ NYC / Long Island / NJ  (25)</t>
         </is>
       </c>
       <c r="B35" s="12" t="n"/>
@@ -20687,17 +20687,17 @@
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>Tools / plumbing / MRO supply inventory – Hilti/DeWalt/Milwaukee, fittings, heat pumps</t>
+          <t>Baonanas LLC ABC sale: turnkey ice cream / gelato / dessert shop equipment</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>restaurant / commercial kitchen contents</t>
         </is>
       </c>
       <c r="D42" s="13" t="inlineStr">
         <is>
-          <t>Riverdale</t>
+          <t>Jersey City</t>
         </is>
       </c>
       <c r="E42" s="13" t="inlineStr">
@@ -20706,23 +20706,19 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Accepting offers</t>
         </is>
       </c>
       <c r="H42" s="15" t="n"/>
       <c r="I42" s="13" t="inlineStr"/>
-      <c r="J42" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-30 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="J42" s="13" t="inlineStr"/>
       <c r="K42" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
+          <t>AuctionAdvisors</t>
         </is>
       </c>
       <c r="L42" s="13" t="inlineStr">
@@ -20738,7 +20734,7 @@
       </c>
       <c r="O42" s="14" t="inlineStr">
         <is>
-          <t>Bulk resale inventory.</t>
+          <t>181 Monticello Ave. Assignment for the benefit of creditors. IFI Panorama gelato display cases, refrigerated topping stations, commercial mixers, refrigerators/freezers, stainless worktables, ice machine, POS, smallwares, gelato carts, catering gear, FF&amp;E.</t>
         </is>
       </c>
     </row>
@@ -20750,12 +20746,12 @@
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>Ice cream + cookie franchise equipment – Taylor soft-serve, Atosa, Blodgett</t>
+          <t>Tools / plumbing / MRO supply inventory – Hilti/DeWalt/Milwaukee, fittings, heat pumps</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>inventory</t>
         </is>
       </c>
       <c r="D43" s="13" t="inlineStr">
@@ -20780,7 +20776,7 @@
       <c r="I43" s="13" t="inlineStr"/>
       <c r="J43" s="13" t="inlineStr">
         <is>
-          <t>2026-11-05 11:00 AM ET</t>
+          <t>2026-10-30 11:00 AM ET</t>
         </is>
       </c>
       <c r="K43" s="13" t="inlineStr">
@@ -20801,7 +20797,7 @@
       </c>
       <c r="O43" s="14" t="inlineStr">
         <is>
-          <t>Resellable units.</t>
+          <t>Bulk resale inventory.</t>
         </is>
       </c>
     </row>
@@ -20813,17 +20809,17 @@
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>Wascomat commercial washers liquidation (22× W105, 6× W185, dryer panels)</t>
+          <t>Ice cream + cookie franchise equipment – Taylor soft-serve, Atosa, Blodgett</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>commercial laundry</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D44" s="13" t="inlineStr">
         <is>
-          <t>Newark</t>
+          <t>Riverdale</t>
         </is>
       </c>
       <c r="E44" s="13" t="inlineStr">
@@ -20832,23 +20828,23 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>$500–$800 each / panels $150</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H44" s="15" t="n"/>
-      <c r="I44" s="13" t="inlineStr">
-        <is>
-          <t>2026-07-12</t>
-        </is>
-      </c>
-      <c r="J44" s="13" t="inlineStr"/>
+      <c r="I44" s="13" t="inlineStr"/>
+      <c r="J44" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-05 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K44" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>A.J. Willner</t>
         </is>
       </c>
       <c r="L44" s="13" t="inlineStr">
@@ -20864,7 +20860,7 @@
       </c>
       <c r="O44" s="14" t="inlineStr">
         <is>
-          <t>22× W105 @ $500, 6× W185 @ $800, 20 dryer panels $150. Commercial laundry liquidation.</t>
+          <t>Resellable units.</t>
         </is>
       </c>
     </row>
@@ -20876,17 +20872,17 @@
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>Major food-service caterer – new-in-box True reach-ins, Beverage-Air, TurboChef, Resfab ventless fryer</t>
+          <t>U.S. Vision court-ordered liquidation: ~70,000 designer eyeglass/sunglass frames + optical/optometry equipment at ~80 former stores + IP</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>court-ordered retail chain liquidation</t>
         </is>
       </c>
       <c r="D45" s="13" t="inlineStr">
         <is>
-          <t>Parsippany</t>
+          <t>Montclair</t>
         </is>
       </c>
       <c r="E45" s="13" t="inlineStr">
@@ -20895,27 +20891,19 @@
         </is>
       </c>
       <c r="F45" s="13" t="n">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="G45" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>Accepting offers (terms in offering memo, NDA required)</t>
         </is>
       </c>
       <c r="H45" s="15" t="n"/>
-      <c r="I45" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="J45" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-03 02:00 PM ET</t>
-        </is>
-      </c>
+      <c r="I45" s="13" t="inlineStr"/>
+      <c r="J45" s="13" t="inlineStr"/>
       <c r="K45" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>AuctionAdvisors</t>
         </is>
       </c>
       <c r="L45" s="13" t="inlineStr">
@@ -20931,7 +20919,7 @@
       </c>
       <c r="O45" s="14" t="inlineStr">
         <is>
-          <t>Tue Nov 3 2 PM, checkout Nov 4.</t>
+          <t>Three-lot sale pursuant to court order; bids accepted for individual lots, combinations, or substantially all assets. Equipment is spread across ~80 former store locations. Not appliance-related; big-ticket bulk inventory play.</t>
         </is>
       </c>
     </row>
@@ -20943,17 +20931,17 @@
       </c>
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>Business closing – 160 new Carnes exhaust fans</t>
+          <t>Wascomat commercial washers liquidation (22× W105, 6× W185, dryer panels)</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>HVAC inventory</t>
+          <t>commercial laundry</t>
         </is>
       </c>
       <c r="D46" s="13" t="inlineStr">
         <is>
-          <t>Kenilworth</t>
+          <t>Newark</t>
         </is>
       </c>
       <c r="E46" s="13" t="inlineStr">
@@ -20962,17 +20950,17 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>$40 each or $5,000 all OBO</t>
+          <t>$500–$800 each / panels $150</t>
         </is>
       </c>
       <c r="H46" s="15" t="n"/>
       <c r="I46" s="13" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="J46" s="13" t="inlineStr"/>
@@ -20994,7 +20982,7 @@
       </c>
       <c r="O46" s="14" t="inlineStr">
         <is>
-          <t>160 new Carnes 80CFM 1.0 sone exhaust fans. $40 each or $5,000 for all OBO. Business closing HVAC inventory.</t>
+          <t>22× W105 @ $500, 6× W185 @ $800, 20 dryer panels $150. Commercial laundry liquidation.</t>
         </is>
       </c>
     </row>
@@ -21006,17 +20994,17 @@
       </c>
       <c r="B47" s="14" t="inlineStr">
         <is>
-          <t>Air Systems Inc – sheet metal / HVAC fabrication shop liquidation</t>
+          <t>Major food-service caterer – new-in-box True reach-ins, Beverage-Air, TurboChef, Resfab ventless fryer</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
         <is>
-          <t>HVAC shop liquidation</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>Kenilworth</t>
+          <t>Parsippany</t>
         </is>
       </c>
       <c r="E47" s="13" t="inlineStr">
@@ -21029,19 +21017,23 @@
       </c>
       <c r="G47" s="13" t="inlineStr">
         <is>
-          <t>Timed online (15% BP)</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H47" s="15" t="n"/>
-      <c r="I47" s="13" t="inlineStr"/>
+      <c r="I47" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
       <c r="J47" s="13" t="inlineStr">
         <is>
-          <t>2026-10-29 11:00 AM ET</t>
+          <t>2026-11-03 02:00 PM ET</t>
         </is>
       </c>
       <c r="K47" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner Auctions</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
       <c r="L47" s="13" t="inlineStr">
@@ -21057,7 +21049,7 @@
       </c>
       <c r="O47" s="14" t="inlineStr">
         <is>
-          <t>Vicon HVAC plasma; Flagler/Lockformer/Roto-Die/Engel fab; welders; Clark forklift; Genie Superlift; Ridgid/Milwaukee/DeWalt/Bosch/Hilti/Makita tools; AeroVent/Carnes exhaust fans; racking/scaffolding. Preview Oct 28–29 AM; pickup Oct 29 PM–Nov 4. Same town as Carnes fan CL lot.</t>
+          <t>Tue Nov 3 2 PM, checkout Nov 4.</t>
         </is>
       </c>
     </row>
@@ -21069,17 +21061,17 @@
       </c>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>Serpico's Pizzeria (lost lease) – Bari ovens, walk-in, Hobart 60qt, Vulcan range</t>
+          <t>Business closing – 160 new Carnes exhaust fans</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>HVAC inventory</t>
         </is>
       </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>Allenhurst</t>
+          <t>Kenilworth</t>
         </is>
       </c>
       <c r="E48" s="13" t="inlineStr">
@@ -21088,28 +21080,28 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>No-reserve online auction</t>
+          <t>$40 each or $5,000 all OBO</t>
         </is>
       </c>
       <c r="H48" s="15" t="n"/>
-      <c r="I48" s="13" t="inlineStr"/>
-      <c r="J48" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-21 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="I48" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="J48" s="13" t="inlineStr"/>
       <c r="K48" s="13" t="inlineStr">
         <is>
-          <t>Peter Costanzo / EstateSales.net</t>
-        </is>
-      </c>
-      <c r="L48" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L48" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M48" s="13" t="inlineStr"/>
@@ -21120,7 +21112,7 @@
       </c>
       <c r="O48" s="14" t="inlineStr">
         <is>
-          <t>Absolute / no reserve.</t>
+          <t>160 new Carnes 80CFM 1.0 sone exhaust fans. $40 each or $5,000 for all OBO. Business closing HVAC inventory.</t>
         </is>
       </c>
     </row>
@@ -21132,17 +21124,17 @@
       </c>
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>Altitude Trampoline Park liquidation – partial: Atosa, TurboChef, stainless</t>
+          <t>Air Systems Inc – sheet metal / HVAC fabrication shop liquidation</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
         <is>
-          <t>facility contents</t>
+          <t>HVAC shop liquidation</t>
         </is>
       </c>
       <c r="D49" s="13" t="inlineStr">
         <is>
-          <t>Iselin</t>
+          <t>Kenilworth</t>
         </is>
       </c>
       <c r="E49" s="13" t="inlineStr">
@@ -21151,28 +21143,28 @@
         </is>
       </c>
       <c r="F49" s="13" t="n">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="G49" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Timed online (15% BP)</t>
         </is>
       </c>
       <c r="H49" s="15" t="n"/>
       <c r="I49" s="13" t="inlineStr"/>
       <c r="J49" s="13" t="inlineStr">
         <is>
-          <t>2026-10-21 11:00 AM ET</t>
+          <t>2026-10-29 11:00 AM ET</t>
         </is>
       </c>
       <c r="K49" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
-        </is>
-      </c>
-      <c r="L49" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>A.J. Willner Auctions</t>
+        </is>
+      </c>
+      <c r="L49" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M49" s="13" t="inlineStr"/>
@@ -21183,7 +21175,7 @@
       </c>
       <c r="O49" s="14" t="inlineStr">
         <is>
-          <t>Some kitchen gear only.</t>
+          <t>Vicon HVAC plasma; Flagler/Lockformer/Roto-Die/Engel fab; welders; Clark forklift; Genie Superlift; Ridgid/Milwaukee/DeWalt/Bosch/Hilti/Makita tools; AeroVent/Carnes exhaust fans; racking/scaffolding. Preview Oct 28–29 AM; pickup Oct 29 PM–Nov 4. Same town as Carnes fan CL lot.</t>
         </is>
       </c>
     </row>
@@ -21195,17 +21187,17 @@
       </c>
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>Restaurant / pizzeria (contents not described)</t>
+          <t>Former Rush Bowls franchise ABC sale: commercial refrigeration, Vitamix blenders, ice &amp; beverage equipment</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>restaurant closing</t>
+          <t>restaurant / commercial kitchen contents</t>
         </is>
       </c>
       <c r="D50" s="13" t="inlineStr">
         <is>
-          <t>Berkeley Heights</t>
+          <t>Westfield</t>
         </is>
       </c>
       <c r="E50" s="13" t="inlineStr">
@@ -21214,32 +21206,24 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>Accepting offers</t>
         </is>
       </c>
       <c r="H50" s="15" t="n"/>
-      <c r="I50" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="J50" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-20 02:00 PM ET</t>
-        </is>
-      </c>
+      <c r="I50" s="13" t="inlineStr"/>
+      <c r="J50" s="13" t="inlineStr"/>
       <c r="K50" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
-        </is>
-      </c>
-      <c r="L50" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>AuctionAdvisors</t>
+        </is>
+      </c>
+      <c r="L50" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M50" s="13" t="inlineStr"/>
@@ -21250,7 +21234,7 @@
       </c>
       <c r="O50" s="14" t="inlineStr">
         <is>
-          <t>Tue Oct 20 2 PM. No item description on page.</t>
+          <t>27 East Broad St. Assignment for the benefit of creditors of 333 Star Enterprises (d/b/a Rush Bowls). Commercial refrigeration/freezers, Vitamix blenders, stainless workstations/sinks, ice and beverage equipment, POS, shelving. Inspection by contacting the auctioneer.</t>
         </is>
       </c>
     </row>
@@ -21262,17 +21246,17 @@
       </c>
       <c r="B51" s="14" t="inlineStr">
         <is>
-          <t>New modular concession kitchens (warehouseman's lien) – 5 units, CaptiveAire hoods, new Ovention/Turbo Air</t>
+          <t>Serpico's Pizzeria (lost lease) – Bari ovens, walk-in, Hobart 60qt, Vulcan range</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
-          <t>lien sale</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D51" s="13" t="inlineStr">
         <is>
-          <t>Edison</t>
+          <t>Allenhurst</t>
         </is>
       </c>
       <c r="E51" s="13" t="inlineStr">
@@ -21281,24 +21265,28 @@
         </is>
       </c>
       <c r="F51" s="13" t="n">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="G51" s="13" t="inlineStr">
         <is>
-          <t>Online auction, $2K load-out fee</t>
+          <t>No-reserve online auction</t>
         </is>
       </c>
       <c r="H51" s="15" t="n"/>
       <c r="I51" s="13" t="inlineStr"/>
-      <c r="J51" s="13" t="inlineStr"/>
+      <c r="J51" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-21 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K51" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
-        </is>
-      </c>
-      <c r="L51" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>Peter Costanzo / EstateSales.net</t>
+        </is>
+      </c>
+      <c r="L51" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M51" s="13" t="inlineStr"/>
@@ -21309,7 +21297,7 @@
       </c>
       <c r="O51" s="14" t="inlineStr">
         <is>
-          <t>&gt;$100K new. Close date not captured.</t>
+          <t>Absolute / no reserve.</t>
         </is>
       </c>
     </row>
@@ -21321,17 +21309,17 @@
       </c>
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>Brand-new &amp; scratch-and-dent kitchen/home appliances – ~185 lots (Thermador, GE Café, Miele, Wolf speed oven, Viking, Bosch…)</t>
+          <t>Altitude Trampoline Park liquidation – partial: Atosa, TurboChef, stainless</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>facility contents</t>
         </is>
       </c>
       <c r="D52" s="13" t="inlineStr">
         <is>
-          <t>Edison</t>
+          <t>Iselin</t>
         </is>
       </c>
       <c r="E52" s="13" t="inlineStr">
@@ -21340,39 +21328,31 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>Live + HiBid webcast, 18% BP + 3% card</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H52" s="15" t="n"/>
-      <c r="I52" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
+      <c r="I52" s="13" t="inlineStr"/>
       <c r="J52" s="13" t="inlineStr">
         <is>
-          <t>2026-10-25 01:00 PM ET</t>
+          <t>2026-10-21 11:00 AM ET</t>
         </is>
       </c>
       <c r="K52" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
-        </is>
-      </c>
-      <c r="L52" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M52" s="21" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
+          <t>A.J. Willner</t>
+        </is>
+      </c>
+      <c r="L52" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M52" s="13" t="inlineStr"/>
       <c r="N52" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -21380,7 +21360,7 @@
       </c>
       <c r="O52" s="14" t="inlineStr">
         <is>
-          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale.</t>
+          <t>Some kitchen gear only.</t>
         </is>
       </c>
     </row>
@@ -21392,17 +21372,17 @@
       </c>
       <c r="B53" s="14" t="inlineStr">
         <is>
-          <t>Party City (Ch. 11) store – fixtures + party merchandise inventory</t>
+          <t>Restaurant / pizzeria (contents not described)</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>restaurant closing</t>
         </is>
       </c>
       <c r="D53" s="13" t="inlineStr">
         <is>
-          <t>East Brunswick</t>
+          <t>Berkeley Heights</t>
         </is>
       </c>
       <c r="E53" s="13" t="inlineStr">
@@ -21411,28 +21391,32 @@
         </is>
       </c>
       <c r="F53" s="13" t="n">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="G53" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H53" s="15" t="n"/>
-      <c r="I53" s="13" t="inlineStr"/>
+      <c r="I53" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
       <c r="J53" s="13" t="inlineStr">
         <is>
-          <t>2026-11-03 11:00 AM ET</t>
+          <t>2026-10-20 02:00 PM ET</t>
         </is>
       </c>
       <c r="K53" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
-        </is>
-      </c>
-      <c r="L53" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
+        </is>
+      </c>
+      <c r="L53" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M53" s="13" t="inlineStr"/>
@@ -21443,7 +21427,7 @@
       </c>
       <c r="O53" s="14" t="inlineStr">
         <is>
-          <t>Store inventory.</t>
+          <t>Tue Oct 20 2 PM. No item description on page.</t>
         </is>
       </c>
     </row>
@@ -21455,17 +21439,17 @@
       </c>
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>Bakery/Cafe Somerville NJ – rack ovens, La Marzocco, food truck (~76 lots)</t>
+          <t>New modular concession kitchens (warehouseman's lien) – 5 units, CaptiveAire hoods, new Ovention/Turbo Air</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>lien sale</t>
         </is>
       </c>
       <c r="D54" s="13" t="inlineStr">
         <is>
-          <t>Somerville</t>
+          <t>Edison</t>
         </is>
       </c>
       <c r="E54" s="13" t="inlineStr">
@@ -21474,27 +21458,19 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>Live webcast + online (18% BP online)</t>
+          <t>Online auction, $2K load-out fee</t>
         </is>
       </c>
       <c r="H54" s="15" t="n"/>
-      <c r="I54" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="J54" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26 02:00 PM ET</t>
-        </is>
-      </c>
+      <c r="I54" s="13" t="inlineStr"/>
+      <c r="J54" s="13" t="inlineStr"/>
       <c r="K54" s="13" t="inlineStr">
         <is>
-          <t>HiBid / Best Buy Auctioneers</t>
+          <t>A.J. Willner</t>
         </is>
       </c>
       <c r="L54" s="13" t="inlineStr">
@@ -21510,7 +21486,7 @@
       </c>
       <c r="O54" s="14" t="inlineStr">
         <is>
-          <t>Full bakery/cafe commercial kitchen: food truck w/ pizza oven, La Marzocco espresso, Mazzer, Baxter + Empire Logiudice rack ovens, dough depositor, Globe floor mixer, Artic Air / SS refrigeration, fryers, Vitamix, Robot Coupe, display cases, dining furniture. Preview 11 AM sale day; checkout Tue 10/27.</t>
+          <t>&gt;$100K new. Close date not captured.</t>
         </is>
       </c>
     </row>
@@ -21522,17 +21498,17 @@
       </c>
       <c r="B55" s="14" t="inlineStr">
         <is>
-          <t>Ability to Work kitchen and store – commercial kitchen + store fixtures (~135 lots)</t>
+          <t>Brand-new &amp; scratch-and-dent kitchen/home appliances – ~185 lots (Thermador, GE Café, Miele, Wolf speed oven, Viking, Bosch…)</t>
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D55" s="13" t="inlineStr">
         <is>
-          <t>Flemington</t>
+          <t>Edison</t>
         </is>
       </c>
       <c r="E55" s="13" t="inlineStr">
@@ -21541,23 +21517,27 @@
         </is>
       </c>
       <c r="F55" s="13" t="n">
-        <v>237</v>
+        <v>217</v>
       </c>
       <c r="G55" s="13" t="inlineStr">
         <is>
-          <t>Timed online (15% BP)</t>
+          <t>Live + HiBid webcast, 18% BP + 3% card</t>
         </is>
       </c>
       <c r="H55" s="15" t="n"/>
-      <c r="I55" s="13" t="inlineStr"/>
+      <c r="I55" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
       <c r="J55" s="13" t="inlineStr">
         <is>
-          <t>2026-10-27 11:02 AM ET</t>
+          <t>2026-10-25 01:00 PM ET</t>
         </is>
       </c>
       <c r="K55" s="13" t="inlineStr">
         <is>
-          <t>HiBid</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
       <c r="L55" s="13" t="inlineStr">
@@ -21565,7 +21545,11 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M55" s="13" t="inlineStr"/>
+      <c r="M55" s="21" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
       <c r="N55" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -21573,7 +21557,7 @@
       </c>
       <c r="O55" s="14" t="inlineStr">
         <is>
-          <t>Apprentice/hospitality training cafe-kitchen and store dispersal. Preview 9–11 AM sale day; removal Oct 27 noon–Oct 29.</t>
+          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale.</t>
         </is>
       </c>
     </row>
@@ -21585,17 +21569,17 @@
       </c>
       <c r="B56" s="14" t="inlineStr">
         <is>
-          <t>Wren Kitchens showroom closing – JennAir/Café/KitchenAid/GE Profile appliances + display kitchens</t>
+          <t>Party City (Ch. 11) store – fixtures + party merchandise inventory</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>showroom closing</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D56" s="13" t="inlineStr">
         <is>
-          <t>Lawrenceville</t>
+          <t>East Brunswick</t>
         </is>
       </c>
       <c r="E56" s="13" t="inlineStr">
@@ -21604,23 +21588,23 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>239</v>
+        <v>220</v>
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>Online auction, 18% BP</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H56" s="15" t="n"/>
       <c r="I56" s="13" t="inlineStr"/>
       <c r="J56" s="13" t="inlineStr">
         <is>
-          <t>2026-10-27 09:00 AM ET</t>
+          <t>2026-11-03 11:00 AM ET</t>
         </is>
       </c>
       <c r="K56" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
+          <t>A.J. Willner</t>
         </is>
       </c>
       <c r="L56" s="13" t="inlineStr">
@@ -21636,7 +21620,7 @@
       </c>
       <c r="O56" s="14" t="inlineStr">
         <is>
-          <t>Premium floor-model appliances; lots close from Oct 27 9 AM.</t>
+          <t>Store inventory.</t>
         </is>
       </c>
     </row>
@@ -21648,17 +21632,17 @@
       </c>
       <c r="B57" s="14" t="inlineStr">
         <is>
-          <t>Wren Kitchens showroom closing – GE/Whirlpool/KitchenAid/Café incl. NIB Café range + 35 kitchens</t>
+          <t>Bakery/Cafe Somerville NJ – rack ovens, La Marzocco, food truck (~76 lots)</t>
         </is>
       </c>
       <c r="C57" s="13" t="inlineStr">
         <is>
-          <t>showroom closing</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D57" s="13" t="inlineStr">
         <is>
-          <t>Cherry Hill</t>
+          <t>Somerville</t>
         </is>
       </c>
       <c r="E57" s="13" t="inlineStr">
@@ -21667,23 +21651,27 @@
         </is>
       </c>
       <c r="F57" s="13" t="n">
-        <v>266</v>
+        <v>224</v>
       </c>
       <c r="G57" s="13" t="inlineStr">
         <is>
-          <t>Online auction, openers ~$0.50</t>
+          <t>Live webcast + online (18% BP online)</t>
         </is>
       </c>
       <c r="H57" s="15" t="n"/>
-      <c r="I57" s="13" t="inlineStr"/>
+      <c r="I57" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
       <c r="J57" s="13" t="inlineStr">
         <is>
-          <t>2026-11-02 11:00 AM ET</t>
+          <t>2026-10-26 02:00 PM ET</t>
         </is>
       </c>
       <c r="K57" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
+          <t>HiBid / Best Buy Auctioneers</t>
         </is>
       </c>
       <c r="L57" s="13" t="inlineStr">
@@ -21699,107 +21687,185 @@
       </c>
       <c r="O57" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Nov 2 11 AM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — NYC / Long Island / NJ</t>
-        </is>
-      </c>
-      <c r="B58" s="17" t="inlineStr">
-        <is>
-          <t>22 item(s)</t>
-        </is>
-      </c>
-      <c r="C58" s="18" t="n"/>
-      <c r="D58" s="18" t="n"/>
-      <c r="E58" s="18" t="n"/>
-      <c r="F58" s="18" t="n"/>
-      <c r="G58" s="18" t="n"/>
-      <c r="H58" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I58" s="18" t="n"/>
-      <c r="J58" s="18" t="n"/>
-      <c r="K58" s="18" t="n"/>
-      <c r="L58" s="18" t="n"/>
-      <c r="M58" s="18" t="n"/>
-      <c r="N58" s="18" t="n"/>
-      <c r="O58" s="18" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="11" t="inlineStr">
-        <is>
-          <t>▸ Eastern PA / Mid-Atlantic  (1)</t>
-        </is>
-      </c>
-      <c r="B59" s="12" t="n"/>
-      <c r="C59" s="12" t="n"/>
-      <c r="D59" s="12" t="n"/>
-      <c r="E59" s="12" t="n"/>
-      <c r="F59" s="12" t="n"/>
-      <c r="G59" s="12" t="n"/>
-      <c r="H59" s="12" t="n"/>
-      <c r="I59" s="12" t="n"/>
-      <c r="J59" s="12" t="n"/>
-      <c r="K59" s="12" t="n"/>
-      <c r="L59" s="12" t="n"/>
-      <c r="M59" s="12" t="n"/>
-      <c r="N59" s="12" t="n"/>
-      <c r="O59" s="12" t="n"/>
+          <t>Full bakery/cafe commercial kitchen: food truck w/ pizza oven, La Marzocco espresso, Mazzer, Baxter + Empire Logiudice rack ovens, dough depositor, Globe floor mixer, Artic Air / SS refrigeration, fryers, Vitamix, Robot Coupe, display cases, dining furniture. Preview 11 AM sale day; checkout Tue 10/27.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" outlineLevel="1">
+      <c r="A58" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B58" s="14" t="inlineStr">
+        <is>
+          <t>Ability to Work kitchen and store – commercial kitchen + store fixtures (~135 lots)</t>
+        </is>
+      </c>
+      <c r="C58" s="13" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D58" s="13" t="inlineStr">
+        <is>
+          <t>Flemington</t>
+        </is>
+      </c>
+      <c r="E58" s="13" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="F58" s="13" t="n">
+        <v>237</v>
+      </c>
+      <c r="G58" s="13" t="inlineStr">
+        <is>
+          <t>Timed online (15% BP)</t>
+        </is>
+      </c>
+      <c r="H58" s="15" t="n"/>
+      <c r="I58" s="13" t="inlineStr"/>
+      <c r="J58" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-27 11:02 AM ET</t>
+        </is>
+      </c>
+      <c r="K58" s="13" t="inlineStr">
+        <is>
+          <t>HiBid</t>
+        </is>
+      </c>
+      <c r="L58" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M58" s="13" t="inlineStr"/>
+      <c r="N58" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O58" s="14" t="inlineStr">
+        <is>
+          <t>Apprentice/hospitality training cafe-kitchen and store dispersal. Preview 9–11 AM sale day; removal Oct 27 noon–Oct 29.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" outlineLevel="1">
+      <c r="A59" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B59" s="14" t="inlineStr">
+        <is>
+          <t>Wren Kitchens showroom closing – JennAir/Café/KitchenAid/GE Profile appliances + display kitchens</t>
+        </is>
+      </c>
+      <c r="C59" s="13" t="inlineStr">
+        <is>
+          <t>showroom closing</t>
+        </is>
+      </c>
+      <c r="D59" s="13" t="inlineStr">
+        <is>
+          <t>Lawrenceville</t>
+        </is>
+      </c>
+      <c r="E59" s="13" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="F59" s="13" t="n">
+        <v>239</v>
+      </c>
+      <c r="G59" s="13" t="inlineStr">
+        <is>
+          <t>Online auction, 18% BP</t>
+        </is>
+      </c>
+      <c r="H59" s="15" t="n"/>
+      <c r="I59" s="13" t="inlineStr"/>
+      <c r="J59" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-27 09:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K59" s="13" t="inlineStr">
+        <is>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L59" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M59" s="13" t="inlineStr"/>
+      <c r="N59" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O59" s="14" t="inlineStr">
+        <is>
+          <t>Premium floor-model appliances; lots close from Oct 27 9 AM.</t>
+        </is>
+      </c>
     </row>
     <row r="60" outlineLevel="1">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>Eastern PA / Mid-Atlantic</t>
+          <t>NYC / Long Island / NJ</t>
         </is>
       </c>
       <c r="B60" s="14" t="inlineStr">
         <is>
-          <t>October restaurant consignment – Hobart, Rational, True + NEW scratch-and-dent Migali/Avantco</t>
+          <t>Wren Kitchens showroom closing – GE/Whirlpool/KitchenAid/Café incl. NIB Café range + 35 kitchens</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>showroom closing</t>
         </is>
       </c>
       <c r="D60" s="13" t="inlineStr">
         <is>
-          <t>Harrisburg</t>
+          <t>Cherry Hill</t>
         </is>
       </c>
       <c r="E60" s="13" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>340</v>
+        <v>266</v>
       </c>
       <c r="G60" s="13" t="inlineStr">
         <is>
-          <t>Online auction, 15% BP, ships $55/pallet</t>
+          <t>Online auction, openers ~$0.50</t>
         </is>
       </c>
       <c r="H60" s="15" t="n"/>
       <c r="I60" s="13" t="inlineStr"/>
       <c r="J60" s="13" t="inlineStr">
         <is>
-          <t>2026-10-21 11:00 AM ET</t>
+          <t>2026-11-02 11:00 AM ET</t>
         </is>
       </c>
       <c r="K60" s="13" t="inlineStr">
         <is>
-          <t>Restaurant Auction Co</t>
-        </is>
-      </c>
-      <c r="L60" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L60" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M60" s="13" t="inlineStr"/>
@@ -21810,19 +21876,19 @@
       </c>
       <c r="O60" s="14" t="inlineStr">
         <is>
-          <t>Closes Oct 21 10 or 11 AM (later used). Shippable.</t>
+          <t>Lots close from Nov 2 11 AM.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="17" t="inlineStr">
         <is>
-          <t>Subtotal — Eastern PA / Mid-Atlantic</t>
+          <t>Subtotal — NYC / Long Island / NJ</t>
         </is>
       </c>
       <c r="B61" s="17" t="inlineStr">
         <is>
-          <t>1 item(s)</t>
+          <t>25 item(s)</t>
         </is>
       </c>
       <c r="C61" s="18" t="n"/>
@@ -21844,7 +21910,7 @@
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
         <is>
-          <t>▸ Western PA / Ohio Valley  (1)</t>
+          <t>▸ Eastern PA / Mid-Atlantic  (1)</t>
         </is>
       </c>
       <c r="B62" s="12" t="n"/>
@@ -21865,22 +21931,22 @@
     <row r="63" outlineLevel="1">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>Western PA / Ohio Valley</t>
+          <t>Eastern PA / Mid-Atlantic</t>
         </is>
       </c>
       <c r="B63" s="14" t="inlineStr">
         <is>
-          <t>Millers Pizza &amp; More – pizza business, commercial kitchen &amp; event space contents (362 lots)</t>
+          <t>October restaurant consignment – Hobart, Rational, True + NEW scratch-and-dent Migali/Avantco</t>
         </is>
       </c>
       <c r="C63" s="13" t="inlineStr">
         <is>
-          <t>restaurant / commercial kitchen contents</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D63" s="13" t="inlineStr">
         <is>
-          <t>Everson</t>
+          <t>Harrisburg</t>
         </is>
       </c>
       <c r="E63" s="13" t="inlineStr">
@@ -21889,28 +21955,28 @@
         </is>
       </c>
       <c r="F63" s="13" t="n">
-        <v>478</v>
+        <v>340</v>
       </c>
       <c r="G63" s="13" t="inlineStr">
         <is>
-          <t>Online auction, 15% buyer premium</t>
+          <t>Online auction, 15% BP, ships $55/pallet</t>
         </is>
       </c>
       <c r="H63" s="15" t="n"/>
       <c r="I63" s="13" t="inlineStr"/>
       <c r="J63" s="13" t="inlineStr">
         <is>
-          <t>2026-10-25 07:00 PM ET</t>
+          <t>2026-10-21 11:00 AM ET</t>
         </is>
       </c>
       <c r="K63" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Bid Local LLC)</t>
-        </is>
-      </c>
-      <c r="L63" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>Restaurant Auction Co</t>
+        </is>
+      </c>
+      <c r="L63" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M63" s="13" t="inlineStr"/>
@@ -21921,14 +21987,14 @@
       </c>
       <c r="O63" s="14" t="inlineStr">
         <is>
-          <t>Property of Millers Pizza and More LLC; online-only, 362 lots, lots begin closing Oct 25 7 PM. Pickup Everson PA by appointment Tue 10/27 and Wed 10/28. Building (4,500 sq ft) to be auctioned separately.</t>
+          <t>Closes Oct 21 10 or 11 AM (later used). Shippable.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="17" t="inlineStr">
         <is>
-          <t>Subtotal — Western PA / Ohio Valley</t>
+          <t>Subtotal — Eastern PA / Mid-Atlantic</t>
         </is>
       </c>
       <c r="B64" s="17" t="inlineStr">
@@ -21955,7 +22021,7 @@
     <row r="65">
       <c r="A65" s="11" t="inlineStr">
         <is>
-          <t>▸ Upstate / Western NY  (2)</t>
+          <t>▸ Western PA / Ohio Valley  (1)</t>
         </is>
       </c>
       <c r="B65" s="12" t="n"/>
@@ -21976,52 +22042,52 @@
     <row r="66" outlineLevel="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>Upstate / Western NY</t>
+          <t>Western PA / Ohio Valley</t>
         </is>
       </c>
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>Former Taco Del Mar – stainless, warmers, walk-in panels</t>
+          <t>Millers Pizza &amp; More – pizza business, commercial kitchen &amp; event space contents (362 lots)</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>restaurant / commercial kitchen contents</t>
         </is>
       </c>
       <c r="D66" s="13" t="inlineStr">
         <is>
-          <t>Watson</t>
+          <t>Everson</t>
         </is>
       </c>
       <c r="E66" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="F66" s="13" t="n">
-        <v>260</v>
+        <v>478</v>
       </c>
       <c r="G66" s="13" t="inlineStr">
         <is>
-          <t>HiBid online auction</t>
+          <t>Online auction, 15% buyer premium</t>
         </is>
       </c>
       <c r="H66" s="15" t="n"/>
       <c r="I66" s="13" t="inlineStr"/>
       <c r="J66" s="13" t="inlineStr">
         <is>
-          <t>2026-10-20 06:00 PM ET</t>
+          <t>2026-10-25 07:00 PM ET</t>
         </is>
       </c>
       <c r="K66" s="13" t="inlineStr">
         <is>
-          <t>Adirondack Asset / HiBid</t>
-        </is>
-      </c>
-      <c r="L66" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>HiBid (Bid Local LLC)</t>
+        </is>
+      </c>
+      <c r="L66" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M66" s="13" t="inlineStr"/>
@@ -22032,165 +22098,165 @@
       </c>
       <c r="O66" s="14" t="inlineStr">
         <is>
+          <t>Property of Millers Pizza and More LLC; online-only, 362 lots, lots begin closing Oct 25 7 PM. Pickup Everson PA by appointment Tue 10/27 and Wed 10/28. Building (4,500 sq ft) to be auctioned separately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Western PA / Ohio Valley</t>
+        </is>
+      </c>
+      <c r="B67" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C67" s="18" t="n"/>
+      <c r="D67" s="18" t="n"/>
+      <c r="E67" s="18" t="n"/>
+      <c r="F67" s="18" t="n"/>
+      <c r="G67" s="18" t="n"/>
+      <c r="H67" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" s="18" t="n"/>
+      <c r="J67" s="18" t="n"/>
+      <c r="K67" s="18" t="n"/>
+      <c r="L67" s="18" t="n"/>
+      <c r="M67" s="18" t="n"/>
+      <c r="N67" s="18" t="n"/>
+      <c r="O67" s="18" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="inlineStr">
+        <is>
+          <t>▸ Upstate / Western NY  (2)</t>
+        </is>
+      </c>
+      <c r="B68" s="12" t="n"/>
+      <c r="C68" s="12" t="n"/>
+      <c r="D68" s="12" t="n"/>
+      <c r="E68" s="12" t="n"/>
+      <c r="F68" s="12" t="n"/>
+      <c r="G68" s="12" t="n"/>
+      <c r="H68" s="12" t="n"/>
+      <c r="I68" s="12" t="n"/>
+      <c r="J68" s="12" t="n"/>
+      <c r="K68" s="12" t="n"/>
+      <c r="L68" s="12" t="n"/>
+      <c r="M68" s="12" t="n"/>
+      <c r="N68" s="12" t="n"/>
+      <c r="O68" s="12" t="n"/>
+    </row>
+    <row r="69" outlineLevel="1">
+      <c r="A69" s="13" t="inlineStr">
+        <is>
+          <t>Upstate / Western NY</t>
+        </is>
+      </c>
+      <c r="B69" s="14" t="inlineStr">
+        <is>
+          <t>Former Taco Del Mar – stainless, warmers, walk-in panels</t>
+        </is>
+      </c>
+      <c r="C69" s="13" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D69" s="13" t="inlineStr">
+        <is>
+          <t>Watson</t>
+        </is>
+      </c>
+      <c r="E69" s="13" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="F69" s="13" t="n">
+        <v>260</v>
+      </c>
+      <c r="G69" s="13" t="inlineStr">
+        <is>
+          <t>HiBid online auction</t>
+        </is>
+      </c>
+      <c r="H69" s="15" t="n"/>
+      <c r="I69" s="13" t="inlineStr"/>
+      <c r="J69" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-20 06:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K69" s="13" t="inlineStr">
+        <is>
+          <t>Adirondack Asset / HiBid</t>
+        </is>
+      </c>
+      <c r="L69" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M69" s="13" t="inlineStr"/>
+      <c r="N69" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O69" s="14" t="inlineStr">
+        <is>
           <t>Small lot.</t>
         </is>
       </c>
-    </row>
-    <row r="67" outlineLevel="1">
-      <c r="A67" s="13" t="inlineStr">
-        <is>
-          <t>Upstate / Western NY</t>
-        </is>
-      </c>
-      <c r="B67" s="14" t="inlineStr">
-        <is>
-          <t>Restaurant &amp; fitness equipment</t>
-        </is>
-      </c>
-      <c r="C67" s="13" t="inlineStr">
-        <is>
-          <t>restaurant</t>
-        </is>
-      </c>
-      <c r="D67" s="13" t="inlineStr">
-        <is>
-          <t>Williamsville</t>
-        </is>
-      </c>
-      <c r="E67" s="13" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="F67" s="13" t="n">
-        <v>408</v>
-      </c>
-      <c r="G67" s="13" t="inlineStr">
-        <is>
-          <t>Online auction</t>
-        </is>
-      </c>
-      <c r="H67" s="15" t="n"/>
-      <c r="I67" s="13" t="inlineStr"/>
-      <c r="J67" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26 07:30 PM ET</t>
-        </is>
-      </c>
-      <c r="K67" s="13" t="inlineStr">
-        <is>
-          <t>Cash Auctions</t>
-        </is>
-      </c>
-      <c r="L67" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M67" s="13" t="inlineStr"/>
-      <c r="N67" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O67" s="14" t="inlineStr">
-        <is>
-          <t>Lots not reviewed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Upstate / Western NY</t>
-        </is>
-      </c>
-      <c r="B68" s="17" t="inlineStr">
-        <is>
-          <t>2 item(s)</t>
-        </is>
-      </c>
-      <c r="C68" s="18" t="n"/>
-      <c r="D68" s="18" t="n"/>
-      <c r="E68" s="18" t="n"/>
-      <c r="F68" s="18" t="n"/>
-      <c r="G68" s="18" t="n"/>
-      <c r="H68" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I68" s="18" t="n"/>
-      <c r="J68" s="18" t="n"/>
-      <c r="K68" s="18" t="n"/>
-      <c r="L68" s="18" t="n"/>
-      <c r="M68" s="18" t="n"/>
-      <c r="N68" s="18" t="n"/>
-      <c r="O68" s="18" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="11" t="inlineStr">
-        <is>
-          <t>▸ Virginia  (1)</t>
-        </is>
-      </c>
-      <c r="B69" s="12" t="n"/>
-      <c r="C69" s="12" t="n"/>
-      <c r="D69" s="12" t="n"/>
-      <c r="E69" s="12" t="n"/>
-      <c r="F69" s="12" t="n"/>
-      <c r="G69" s="12" t="n"/>
-      <c r="H69" s="12" t="n"/>
-      <c r="I69" s="12" t="n"/>
-      <c r="J69" s="12" t="n"/>
-      <c r="K69" s="12" t="n"/>
-      <c r="L69" s="12" t="n"/>
-      <c r="M69" s="12" t="n"/>
-      <c r="N69" s="12" t="n"/>
-      <c r="O69" s="12" t="n"/>
     </row>
     <row r="70" outlineLevel="1">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>Virginia</t>
+          <t>Upstate / Western NY</t>
         </is>
       </c>
       <c r="B70" s="14" t="inlineStr">
         <is>
-          <t>Haynes Furniture / The Dump – 12 stores closing (furniture, mattresses)</t>
+          <t>Restaurant &amp; fitness equipment</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>retail GOB</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D70" s="13" t="inlineStr">
         <is>
-          <t>Virginia Beach</t>
+          <t>Williamsville</t>
         </is>
       </c>
       <c r="E70" s="13" t="inlineStr">
         <is>
-          <t>VA</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F70" s="13" t="n">
-        <v>456</v>
+        <v>408</v>
       </c>
       <c r="G70" s="13" t="inlineStr">
         <is>
-          <t>Retail GOB markdowns</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H70" s="15" t="n"/>
-      <c r="I70" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="J70" s="13" t="inlineStr"/>
+      <c r="I70" s="13" t="inlineStr"/>
+      <c r="J70" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-26 07:30 PM ET</t>
+        </is>
+      </c>
       <c r="K70" s="13" t="inlineStr">
         <is>
-          <t>SB360 (PR Newswire)</t>
+          <t>Cash Auctions</t>
         </is>
       </c>
       <c r="L70" s="13" t="inlineStr">
@@ -22206,19 +22272,19 @@
       </c>
       <c r="O70" s="14" t="inlineStr">
         <is>
-          <t>Posted Oct 8. Multi-state (VA/AZ/GA/IL/TX); pinned at Virginia Beach. Home goods only.</t>
+          <t>Lots not reviewed.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="17" t="inlineStr">
         <is>
-          <t>Subtotal — Virginia</t>
+          <t>Subtotal — Upstate / Western NY</t>
         </is>
       </c>
       <c r="B71" s="17" t="inlineStr">
         <is>
-          <t>1 item(s)</t>
+          <t>2 item(s)</t>
         </is>
       </c>
       <c r="C71" s="18" t="n"/>
@@ -22240,7 +22306,7 @@
     <row r="72">
       <c r="A72" s="11" t="inlineStr">
         <is>
-          <t>▸ Midwest  (3)</t>
+          <t>▸ Virginia  (1)</t>
         </is>
       </c>
       <c r="B72" s="12" t="n"/>
@@ -22261,52 +22327,52 @@
     <row r="73" outlineLevel="1">
       <c r="A73" s="13" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>Virginia</t>
         </is>
       </c>
       <c r="B73" s="14" t="inlineStr">
         <is>
-          <t>Freshway Market whole-grocery liquidation – refrigeration racks, cases, walk-ins, generator</t>
+          <t>Haynes Furniture / The Dump – 12 stores closing (furniture, mattresses)</t>
         </is>
       </c>
       <c r="C73" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>retail GOB</t>
         </is>
       </c>
       <c r="D73" s="13" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Virginia Beach</t>
         </is>
       </c>
       <c r="E73" s="13" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>VA</t>
         </is>
       </c>
       <c r="F73" s="13" t="n">
-        <v>862</v>
+        <v>456</v>
       </c>
       <c r="G73" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Retail GOB markdowns</t>
         </is>
       </c>
       <c r="H73" s="15" t="n"/>
-      <c r="I73" s="13" t="inlineStr"/>
-      <c r="J73" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-20 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="I73" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="J73" s="13" t="inlineStr"/>
       <c r="K73" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
-        </is>
-      </c>
-      <c r="L73" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>SB360 (PR Newswire)</t>
+        </is>
+      </c>
+      <c r="L73" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M73" s="13" t="inlineStr"/>
@@ -22317,387 +22383,435 @@
       </c>
       <c r="O73" s="14" t="inlineStr">
         <is>
-          <t>Closes from Oct 20 10 AM CDT.</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" outlineLevel="1">
-      <c r="A74" s="13" t="inlineStr">
+          <t>Posted Oct 8. Multi-state (VA/AZ/GA/IL/TX); pinned at Virginia Beach. Home goods only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Virginia</t>
+        </is>
+      </c>
+      <c r="B74" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C74" s="18" t="n"/>
+      <c r="D74" s="18" t="n"/>
+      <c r="E74" s="18" t="n"/>
+      <c r="F74" s="18" t="n"/>
+      <c r="G74" s="18" t="n"/>
+      <c r="H74" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I74" s="18" t="n"/>
+      <c r="J74" s="18" t="n"/>
+      <c r="K74" s="18" t="n"/>
+      <c r="L74" s="18" t="n"/>
+      <c r="M74" s="18" t="n"/>
+      <c r="N74" s="18" t="n"/>
+      <c r="O74" s="18" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="11" t="inlineStr">
+        <is>
+          <t>▸ Midwest  (2)</t>
+        </is>
+      </c>
+      <c r="B75" s="12" t="n"/>
+      <c r="C75" s="12" t="n"/>
+      <c r="D75" s="12" t="n"/>
+      <c r="E75" s="12" t="n"/>
+      <c r="F75" s="12" t="n"/>
+      <c r="G75" s="12" t="n"/>
+      <c r="H75" s="12" t="n"/>
+      <c r="I75" s="12" t="n"/>
+      <c r="J75" s="12" t="n"/>
+      <c r="K75" s="12" t="n"/>
+      <c r="L75" s="12" t="n"/>
+      <c r="M75" s="12" t="n"/>
+      <c r="N75" s="12" t="n"/>
+      <c r="O75" s="12" t="n"/>
+    </row>
+    <row r="76" outlineLevel="1">
+      <c r="A76" s="13" t="inlineStr">
         <is>
           <t>Midwest</t>
         </is>
       </c>
-      <c r="B74" s="14" t="inlineStr">
+      <c r="B76" s="14" t="inlineStr">
         <is>
           <t>American Sale – total liquidation, all 7 stores (pools, hot tubs, grills, holiday decor)</t>
         </is>
       </c>
-      <c r="C74" s="13" t="inlineStr">
+      <c r="C76" s="13" t="inlineStr">
         <is>
           <t>retail GOB</t>
         </is>
       </c>
-      <c r="D74" s="13" t="inlineStr">
+      <c r="D76" s="13" t="inlineStr">
         <is>
           <t>Chicagoland</t>
         </is>
       </c>
-      <c r="E74" s="13" t="inlineStr">
+      <c r="E76" s="13" t="inlineStr">
         <is>
           <t>IL</t>
         </is>
       </c>
-      <c r="F74" s="13" t="n">
+      <c r="F76" s="13" t="n">
         <v>876</v>
       </c>
-      <c r="G74" s="13" t="inlineStr">
+      <c r="G76" s="13" t="inlineStr">
         <is>
           <t>Retail GOB, up to 70% off</t>
         </is>
       </c>
-      <c r="H74" s="15" t="n"/>
-      <c r="I74" s="13" t="inlineStr">
+      <c r="H76" s="15" t="n"/>
+      <c r="I76" s="13" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="J74" s="13" t="inlineStr"/>
-      <c r="K74" s="13" t="inlineStr">
+      <c r="J76" s="13" t="inlineStr"/>
+      <c r="K76" s="13" t="inlineStr">
         <is>
           <t>Tiger Group (PR Newswire)</t>
         </is>
       </c>
-      <c r="L74" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M74" s="13" t="inlineStr"/>
-      <c r="N74" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O74" s="14" t="inlineStr">
+      <c r="L76" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M76" s="13" t="inlineStr"/>
+      <c r="N76" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O76" s="14" t="inlineStr">
         <is>
           <t>Posted Oct 15. Watch for a bulk/fixture auction.</t>
         </is>
       </c>
     </row>
-    <row r="75" outlineLevel="1">
-      <c r="A75" s="13" t="inlineStr">
+    <row r="77" outlineLevel="1">
+      <c r="A77" s="13" t="inlineStr">
         <is>
           <t>Midwest</t>
         </is>
       </c>
-      <c r="B75" s="14" t="inlineStr">
+      <c r="B77" s="14" t="inlineStr">
         <is>
           <t>Straub's Fine Foods store equipment – bakery, kitchen, meat room, Hussmann refrigeration</t>
         </is>
       </c>
-      <c r="C75" s="13" t="inlineStr">
+      <c r="C77" s="13" t="inlineStr">
         <is>
           <t>grocery/restaurant</t>
         </is>
       </c>
-      <c r="D75" s="13" t="inlineStr">
+      <c r="D77" s="13" t="inlineStr">
         <is>
           <t>St. Louis</t>
         </is>
       </c>
-      <c r="E75" s="13" t="inlineStr">
+      <c r="E77" s="13" t="inlineStr">
         <is>
           <t>MO</t>
         </is>
       </c>
-      <c r="F75" s="13" t="n">
+      <c r="F77" s="13" t="n">
         <v>1046</v>
       </c>
-      <c r="G75" s="13" t="inlineStr">
+      <c r="G77" s="13" t="inlineStr">
         <is>
           <t>Online auction (18% BP)</t>
         </is>
       </c>
-      <c r="H75" s="15" t="n"/>
-      <c r="I75" s="13" t="inlineStr"/>
-      <c r="J75" s="13" t="inlineStr">
+      <c r="H77" s="15" t="n"/>
+      <c r="I77" s="13" t="inlineStr"/>
+      <c r="J77" s="13" t="inlineStr">
         <is>
           <t>2026-10-21 11:00 AM ET</t>
         </is>
       </c>
-      <c r="K75" s="13" t="inlineStr">
+      <c r="K77" s="13" t="inlineStr">
         <is>
           <t>Grafe Auction</t>
         </is>
       </c>
-      <c r="L75" s="20" t="inlineStr">
+      <c r="L77" s="20" t="inlineStr">
         <is>
           <t>ENDING SOON</t>
         </is>
       </c>
-      <c r="M75" s="13" t="inlineStr"/>
-      <c r="N75" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O75" s="14" t="inlineStr">
+      <c r="M77" s="13" t="inlineStr"/>
+      <c r="N77" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O77" s="14" t="inlineStr">
         <is>
           <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis.</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="17" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Midwest</t>
         </is>
       </c>
-      <c r="B76" s="17" t="inlineStr">
-        <is>
-          <t>3 item(s)</t>
-        </is>
-      </c>
-      <c r="C76" s="18" t="n"/>
-      <c r="D76" s="18" t="n"/>
-      <c r="E76" s="18" t="n"/>
-      <c r="F76" s="18" t="n"/>
-      <c r="G76" s="18" t="n"/>
-      <c r="H76" s="19" t="n">
+      <c r="B78" s="17" t="inlineStr">
+        <is>
+          <t>2 item(s)</t>
+        </is>
+      </c>
+      <c r="C78" s="18" t="n"/>
+      <c r="D78" s="18" t="n"/>
+      <c r="E78" s="18" t="n"/>
+      <c r="F78" s="18" t="n"/>
+      <c r="G78" s="18" t="n"/>
+      <c r="H78" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I76" s="18" t="n"/>
-      <c r="J76" s="18" t="n"/>
-      <c r="K76" s="18" t="n"/>
-      <c r="L76" s="18" t="n"/>
-      <c r="M76" s="18" t="n"/>
-      <c r="N76" s="18" t="n"/>
-      <c r="O76" s="18" t="n"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="11" t="inlineStr">
+      <c r="I78" s="18" t="n"/>
+      <c r="J78" s="18" t="n"/>
+      <c r="K78" s="18" t="n"/>
+      <c r="L78" s="18" t="n"/>
+      <c r="M78" s="18" t="n"/>
+      <c r="N78" s="18" t="n"/>
+      <c r="O78" s="18" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="11" t="inlineStr">
         <is>
           <t>▸ Texas / South Central  (1)</t>
         </is>
       </c>
-      <c r="B77" s="12" t="n"/>
-      <c r="C77" s="12" t="n"/>
-      <c r="D77" s="12" t="n"/>
-      <c r="E77" s="12" t="n"/>
-      <c r="F77" s="12" t="n"/>
-      <c r="G77" s="12" t="n"/>
-      <c r="H77" s="12" t="n"/>
-      <c r="I77" s="12" t="n"/>
-      <c r="J77" s="12" t="n"/>
-      <c r="K77" s="12" t="n"/>
-      <c r="L77" s="12" t="n"/>
-      <c r="M77" s="12" t="n"/>
-      <c r="N77" s="12" t="n"/>
-      <c r="O77" s="12" t="n"/>
-    </row>
-    <row r="78" outlineLevel="1">
-      <c r="A78" s="13" t="inlineStr">
+      <c r="B79" s="12" t="n"/>
+      <c r="C79" s="12" t="n"/>
+      <c r="D79" s="12" t="n"/>
+      <c r="E79" s="12" t="n"/>
+      <c r="F79" s="12" t="n"/>
+      <c r="G79" s="12" t="n"/>
+      <c r="H79" s="12" t="n"/>
+      <c r="I79" s="12" t="n"/>
+      <c r="J79" s="12" t="n"/>
+      <c r="K79" s="12" t="n"/>
+      <c r="L79" s="12" t="n"/>
+      <c r="M79" s="12" t="n"/>
+      <c r="N79" s="12" t="n"/>
+      <c r="O79" s="12" t="n"/>
+    </row>
+    <row r="80" outlineLevel="1">
+      <c r="A80" s="13" t="inlineStr">
         <is>
           <t>Texas / South Central</t>
         </is>
       </c>
-      <c r="B78" s="14" t="inlineStr">
+      <c r="B80" s="14" t="inlineStr">
         <is>
           <t>Southwest beverage distributor surplus – mostly unused: 16 True merchandisers, 75 Bunn brewers, 100+ micro-market kiosks</t>
         </is>
       </c>
-      <c r="C78" s="13" t="inlineStr">
+      <c r="C80" s="13" t="inlineStr">
         <is>
           <t>distributor surplus</t>
         </is>
       </c>
-      <c r="D78" s="13" t="inlineStr">
+      <c r="D80" s="13" t="inlineStr">
         <is>
           <t>Mesquite</t>
         </is>
       </c>
-      <c r="E78" s="13" t="inlineStr">
+      <c r="E80" s="13" t="inlineStr">
         <is>
           <t>TX</t>
         </is>
       </c>
-      <c r="F78" s="13" t="n">
+      <c r="F80" s="13" t="n">
         <v>1547</v>
       </c>
-      <c r="G78" s="13" t="inlineStr">
+      <c r="G80" s="13" t="inlineStr">
         <is>
           <t>Online auction</t>
         </is>
       </c>
-      <c r="H78" s="15" t="n"/>
-      <c r="I78" s="13" t="inlineStr"/>
-      <c r="J78" s="13" t="inlineStr">
+      <c r="H80" s="15" t="n"/>
+      <c r="I80" s="13" t="inlineStr"/>
+      <c r="J80" s="13" t="inlineStr">
         <is>
           <t>2026-11-13 11:00 AM ET</t>
         </is>
       </c>
-      <c r="K78" s="13" t="inlineStr">
+      <c r="K80" s="13" t="inlineStr">
         <is>
           <t>Heritage Global Partners</t>
         </is>
       </c>
-      <c r="L78" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M78" s="13" t="inlineStr"/>
-      <c r="N78" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O78" s="14" t="inlineStr">
+      <c r="L80" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M80" s="13" t="inlineStr"/>
+      <c r="N80" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O80" s="14" t="inlineStr">
         <is>
           <t>Near-new appliances, resell by unit. Nov 13 10 AM CST.</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="17" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Texas / South Central</t>
         </is>
       </c>
-      <c r="B79" s="17" t="inlineStr">
+      <c r="B81" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C79" s="18" t="n"/>
-      <c r="D79" s="18" t="n"/>
-      <c r="E79" s="18" t="n"/>
-      <c r="F79" s="18" t="n"/>
-      <c r="G79" s="18" t="n"/>
-      <c r="H79" s="19" t="n">
+      <c r="C81" s="18" t="n"/>
+      <c r="D81" s="18" t="n"/>
+      <c r="E81" s="18" t="n"/>
+      <c r="F81" s="18" t="n"/>
+      <c r="G81" s="18" t="n"/>
+      <c r="H81" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I79" s="18" t="n"/>
-      <c r="J79" s="18" t="n"/>
-      <c r="K79" s="18" t="n"/>
-      <c r="L79" s="18" t="n"/>
-      <c r="M79" s="18" t="n"/>
-      <c r="N79" s="18" t="n"/>
-      <c r="O79" s="18" t="n"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="11" t="inlineStr">
+      <c r="I81" s="18" t="n"/>
+      <c r="J81" s="18" t="n"/>
+      <c r="K81" s="18" t="n"/>
+      <c r="L81" s="18" t="n"/>
+      <c r="M81" s="18" t="n"/>
+      <c r="N81" s="18" t="n"/>
+      <c r="O81" s="18" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="inlineStr">
         <is>
           <t>▸ West / Other  (1)</t>
         </is>
       </c>
-      <c r="B80" s="12" t="n"/>
-      <c r="C80" s="12" t="n"/>
-      <c r="D80" s="12" t="n"/>
-      <c r="E80" s="12" t="n"/>
-      <c r="F80" s="12" t="n"/>
-      <c r="G80" s="12" t="n"/>
-      <c r="H80" s="12" t="n"/>
-      <c r="I80" s="12" t="n"/>
-      <c r="J80" s="12" t="n"/>
-      <c r="K80" s="12" t="n"/>
-      <c r="L80" s="12" t="n"/>
-      <c r="M80" s="12" t="n"/>
-      <c r="N80" s="12" t="n"/>
-      <c r="O80" s="12" t="n"/>
-    </row>
-    <row r="81" outlineLevel="1">
-      <c r="A81" s="13" t="inlineStr">
+      <c r="B82" s="12" t="n"/>
+      <c r="C82" s="12" t="n"/>
+      <c r="D82" s="12" t="n"/>
+      <c r="E82" s="12" t="n"/>
+      <c r="F82" s="12" t="n"/>
+      <c r="G82" s="12" t="n"/>
+      <c r="H82" s="12" t="n"/>
+      <c r="I82" s="12" t="n"/>
+      <c r="J82" s="12" t="n"/>
+      <c r="K82" s="12" t="n"/>
+      <c r="L82" s="12" t="n"/>
+      <c r="M82" s="12" t="n"/>
+      <c r="N82" s="12" t="n"/>
+      <c r="O82" s="12" t="n"/>
+    </row>
+    <row r="83" outlineLevel="1">
+      <c r="A83" s="13" t="inlineStr">
         <is>
           <t>West / Other</t>
         </is>
       </c>
-      <c r="B81" s="14" t="inlineStr">
+      <c r="B83" s="14" t="inlineStr">
         <is>
           <t>National salad concept liquidation – full contents of 63 fast-casual restaurants (AZ/TX/OK/NV)</t>
         </is>
       </c>
-      <c r="C81" s="13" t="inlineStr">
+      <c r="C83" s="13" t="inlineStr">
         <is>
           <t>restaurant chain liquidation</t>
         </is>
       </c>
-      <c r="D81" s="13" t="inlineStr">
+      <c r="D83" s="13" t="inlineStr">
         <is>
           <t>Phoenix</t>
         </is>
       </c>
-      <c r="E81" s="13" t="inlineStr">
+      <c r="E83" s="13" t="inlineStr">
         <is>
           <t>AZ</t>
         </is>
       </c>
-      <c r="F81" s="13" t="n">
+      <c r="F83" s="13" t="n">
         <v>2307</v>
       </c>
-      <c r="G81" s="13" t="inlineStr">
+      <c r="G83" s="13" t="inlineStr">
         <is>
           <t>Online auctions, dates TBD</t>
         </is>
       </c>
-      <c r="H81" s="15" t="n"/>
-      <c r="I81" s="13" t="inlineStr">
+      <c r="H83" s="15" t="n"/>
+      <c r="I83" s="13" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="J81" s="13" t="inlineStr"/>
-      <c r="K81" s="13" t="inlineStr">
+      <c r="J83" s="13" t="inlineStr"/>
+      <c r="K83" s="13" t="inlineStr">
         <is>
           <t>RestaurantEquipment.bid (TAGeX)</t>
         </is>
       </c>
-      <c r="L81" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M81" s="13" t="inlineStr"/>
-      <c r="N81" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O81" s="14" t="inlineStr">
+      <c r="L83" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M83" s="13" t="inlineStr"/>
+      <c r="N83" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O83" s="14" t="inlineStr">
         <is>
           <t>Rolling market-by-market auctions, none live yet (Phoenix metro 30 locations, DFW 14, Tucson 6, Houston 5, plus OK/NV). Pickup on site at each restaurant. Pinned at Phoenix.</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="17" t="inlineStr">
+    <row r="84">
+      <c r="A84" s="17" t="inlineStr">
         <is>
           <t>Subtotal — West / Other</t>
         </is>
       </c>
-      <c r="B82" s="17" t="inlineStr">
+      <c r="B84" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C82" s="18" t="n"/>
-      <c r="D82" s="18" t="n"/>
-      <c r="E82" s="18" t="n"/>
-      <c r="F82" s="18" t="n"/>
-      <c r="G82" s="18" t="n"/>
-      <c r="H82" s="19" t="n">
+      <c r="C84" s="18" t="n"/>
+      <c r="D84" s="18" t="n"/>
+      <c r="E84" s="18" t="n"/>
+      <c r="F84" s="18" t="n"/>
+      <c r="G84" s="18" t="n"/>
+      <c r="H84" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I82" s="18" t="n"/>
-      <c r="J82" s="18" t="n"/>
-      <c r="K82" s="18" t="n"/>
-      <c r="L82" s="18" t="n"/>
-      <c r="M82" s="18" t="n"/>
-      <c r="N82" s="18" t="n"/>
-      <c r="O82" s="18" t="n"/>
+      <c r="I84" s="18" t="n"/>
+      <c r="J84" s="18" t="n"/>
+      <c r="K84" s="18" t="n"/>
+      <c r="L84" s="18" t="n"/>
+      <c r="M84" s="18" t="n"/>
+      <c r="N84" s="18" t="n"/>
+      <c r="O84" s="18" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O82"/>
+  <autoFilter ref="A1:O84"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId2"/>
@@ -22744,16 +22858,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N55" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N56" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N57" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N60" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N63" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N66" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N67" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N70" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N73" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N74" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N75" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N78" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N81" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N58" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N59" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N60" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N63" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N66" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N69" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N70" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N73" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N76" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N77" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N80" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N83" r:id="rId57"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -22765,7 +22881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -22927,7 +23043,7 @@
       </c>
       <c r="O2" s="14" t="inlineStr">
         <is>
-          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -22990,7 +23106,7 @@
       </c>
       <c r="O3" s="14" t="inlineStr">
         <is>
-          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23191,7 +23307,7 @@
       </c>
       <c r="O6" s="14" t="inlineStr">
         <is>
-          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23256,7 +23372,7 @@
       </c>
       <c r="O7" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23321,7 +23437,7 @@
       </c>
       <c r="O8" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23384,7 +23500,7 @@
       </c>
       <c r="O9" s="14" t="inlineStr">
         <is>
-          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23447,7 +23563,7 @@
       </c>
       <c r="O10" s="14" t="inlineStr">
         <is>
-          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23510,59 +23626,59 @@
       </c>
       <c r="O11" s="14" t="inlineStr">
         <is>
-          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>Greater Boston / South Shore (&lt;50mi)</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>Closed Best Buy Outlet – pallet racking, Big Joe order pickers, appliance dollies, carts, cages</t>
+          <t>Freshway Market whole-grocery liquidation – refrigeration racks, cases, walk-ins, generator</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>store closing fixtures</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Brockton</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E12" s="13" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>11</v>
+        <v>862</v>
       </c>
       <c r="G12" s="13" t="inlineStr">
         <is>
-          <t>Racking $40/upright, $80/level; pickers $1,000 OBO</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H12" s="15" t="n"/>
-      <c r="I12" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="J12" s="13" t="inlineStr"/>
+      <c r="I12" s="13" t="inlineStr"/>
+      <c r="J12" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-20 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K12" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>Grafe Auction</t>
         </is>
       </c>
       <c r="L12" s="13" t="inlineStr">
         <is>
-          <t>REMOVED</t>
+          <t>EXPIRED (2026-10-20 11:00 AM ET)</t>
         </is>
       </c>
       <c r="M12" s="13" t="inlineStr"/>
@@ -23573,63 +23689,59 @@
       </c>
       <c r="O12" s="14" t="inlineStr">
         <is>
-          <t>200 Westgate Dr. Fixtures/equipment only, no merchandise. On site daily. CL deleted by author (HTTP 410) as of 2026-10-19 midday recheck.</t>
+          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>NYC / Long Island / NJ</t>
+          <t>Greater Boston / South Shore (&lt;50mi)</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>Like-new restaurant – steam tables, Coldline, Cleveland cook-and-hold, fryers, True freezers</t>
+          <t>Closed Best Buy Outlet – pallet racking, Big Joe order pickers, appliance dollies, carts, cages</t>
         </is>
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>store closing fixtures</t>
         </is>
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>Staten Island</t>
+          <t>Brockton</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>203</v>
+        <v>11</v>
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>Racking $40/upright, $80/level; pickers $1,000 OBO</t>
         </is>
       </c>
       <c r="H13" s="15" t="n"/>
       <c r="I13" s="13" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="J13" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-19 01:00 PM ET</t>
-        </is>
-      </c>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="J13" s="13" t="inlineStr"/>
       <c r="K13" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L13" s="13" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-10-19 01:00 PM ET)</t>
+          <t>REMOVED</t>
         </is>
       </c>
       <c r="M13" s="13" t="inlineStr"/>
@@ -23640,7 +23752,7 @@
       </c>
       <c r="O13" s="14" t="inlineStr">
         <is>
-          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>200 Westgate Dr. Fixtures/equipment only, no merchandise. On site daily. CL deleted by author (HTTP 410) as of 2026-10-19 midday recheck.</t>
         </is>
       </c>
     </row>
@@ -23652,26 +23764,26 @@
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>High-end deli (contents not described)</t>
+          <t>Like-new restaurant – steam tables, Coldline, Cleveland cook-and-hold, fryers, True freezers</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>restaurant closing</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>Manalapan Township</t>
+          <t>Staten Island</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>NJ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>223</v>
+        <v>203</v>
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
@@ -23686,7 +23798,7 @@
       </c>
       <c r="J14" s="13" t="inlineStr">
         <is>
-          <t>2026-10-19 04:00 PM ET</t>
+          <t>2026-10-19 01:00 PM ET</t>
         </is>
       </c>
       <c r="K14" s="13" t="inlineStr">
@@ -23696,7 +23808,7 @@
       </c>
       <c r="L14" s="13" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-10-19 04:00 PM ET)</t>
+          <t>EXPIRED (2026-10-19 01:00 PM ET)</t>
         </is>
       </c>
       <c r="M14" s="13" t="inlineStr"/>
@@ -23707,12 +23819,79 @@
       </c>
       <c r="O14" s="14" t="inlineStr">
         <is>
-          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>High-end deli (contents not described)</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>restaurant closing</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Manalapan Township</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="n">
+        <v>223</v>
+      </c>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>Live + webcast, 18% BP + 3%</t>
+        </is>
+      </c>
+      <c r="H15" s="15" t="n"/>
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="J15" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 04:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K15" s="13" t="inlineStr">
+        <is>
+          <t>HiBid (Best Buy Auctioneers)</t>
+        </is>
+      </c>
+      <c r="L15" s="13" t="inlineStr">
+        <is>
+          <t>EXPIRED (2026-10-19 04:00 PM ET)</t>
+        </is>
+      </c>
+      <c r="M15" s="13" t="inlineStr"/>
+      <c r="N15" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O15" s="14" t="inlineStr">
+        <is>
+          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O14"/>
+  <autoFilter ref="A1:O15"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
@@ -23727,6 +23906,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Watch update 2026-10-20 6pm ET: remove ended bl-019 ADK Taco Del Mar auction; recheck 144 URLs
</commit_message>
<xml_diff>
--- a/lot_recon.xlsx
+++ b/lot_recon.xlsx
@@ -20,8 +20,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wolf New'!$A$1:$O$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Wolf Used'!$A$1:$O$189</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Wolf Unclear'!$A$1:$O$40</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$85</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 2026-10-20 14:01 ET</t>
+          <t>Last updated: 2026-10-20 18:00 ET</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Active listings: 295 · Removed: 17</t>
+          <t>Active listings: 294 · Removed: 18</t>
         </is>
       </c>
     </row>
@@ -708,13 +708,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13">
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C13" s="7" t="n">
         <v>980438.58</v>
@@ -1121,7 +1121,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C27" t="n">
         <v>0</v>
@@ -1136,7 +1136,7 @@
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H27" s="6" t="n">
         <v>2250</v>
@@ -18412,7 +18412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O85"/>
+  <dimension ref="A1:O84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -22137,7 +22137,7 @@
     <row r="69">
       <c r="A69" s="11" t="inlineStr">
         <is>
-          <t>▸ Upstate / Western NY  (2)</t>
+          <t>▸ Upstate / Western NY  (1)</t>
         </is>
       </c>
       <c r="B69" s="12" t="n"/>
@@ -22163,7 +22163,7 @@
       </c>
       <c r="B70" s="14" t="inlineStr">
         <is>
-          <t>Former Taco Del Mar – stainless, warmers, walk-in panels</t>
+          <t>Restaurant &amp; fitness equipment</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
@@ -22173,7 +22173,7 @@
       </c>
       <c r="D70" s="13" t="inlineStr">
         <is>
-          <t>Watson</t>
+          <t>Williamsville</t>
         </is>
       </c>
       <c r="E70" s="13" t="inlineStr">
@@ -22182,28 +22182,28 @@
         </is>
       </c>
       <c r="F70" s="13" t="n">
-        <v>260</v>
+        <v>408</v>
       </c>
       <c r="G70" s="13" t="inlineStr">
         <is>
-          <t>HiBid online auction</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H70" s="15" t="n"/>
       <c r="I70" s="13" t="inlineStr"/>
       <c r="J70" s="13" t="inlineStr">
         <is>
-          <t>2026-10-20 06:00 PM ET</t>
+          <t>2026-10-26 07:30 PM ET</t>
         </is>
       </c>
       <c r="K70" s="13" t="inlineStr">
         <is>
-          <t>Adirondack Asset / HiBid</t>
-        </is>
-      </c>
-      <c r="L70" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>Cash Auctions</t>
+        </is>
+      </c>
+      <c r="L70" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M70" s="13" t="inlineStr"/>
@@ -22214,231 +22214,231 @@
       </c>
       <c r="O70" s="14" t="inlineStr">
         <is>
-          <t>Small lot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" outlineLevel="1">
-      <c r="A71" s="13" t="inlineStr">
-        <is>
-          <t>Upstate / Western NY</t>
-        </is>
-      </c>
-      <c r="B71" s="14" t="inlineStr">
-        <is>
-          <t>Restaurant &amp; fitness equipment</t>
-        </is>
-      </c>
-      <c r="C71" s="13" t="inlineStr">
-        <is>
-          <t>restaurant</t>
-        </is>
-      </c>
-      <c r="D71" s="13" t="inlineStr">
-        <is>
-          <t>Williamsville</t>
-        </is>
-      </c>
-      <c r="E71" s="13" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="F71" s="13" t="n">
-        <v>408</v>
-      </c>
-      <c r="G71" s="13" t="inlineStr">
-        <is>
-          <t>Online auction</t>
-        </is>
-      </c>
-      <c r="H71" s="15" t="n"/>
-      <c r="I71" s="13" t="inlineStr"/>
-      <c r="J71" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26 07:30 PM ET</t>
-        </is>
-      </c>
-      <c r="K71" s="13" t="inlineStr">
-        <is>
-          <t>Cash Auctions</t>
-        </is>
-      </c>
-      <c r="L71" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M71" s="13" t="inlineStr"/>
-      <c r="N71" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O71" s="14" t="inlineStr">
-        <is>
           <t>Lots not reviewed.</t>
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Upstate / Western NY</t>
+        </is>
+      </c>
+      <c r="B71" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C71" s="18" t="n"/>
+      <c r="D71" s="18" t="n"/>
+      <c r="E71" s="18" t="n"/>
+      <c r="F71" s="18" t="n"/>
+      <c r="G71" s="18" t="n"/>
+      <c r="H71" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I71" s="18" t="n"/>
+      <c r="J71" s="18" t="n"/>
+      <c r="K71" s="18" t="n"/>
+      <c r="L71" s="18" t="n"/>
+      <c r="M71" s="18" t="n"/>
+      <c r="N71" s="18" t="n"/>
+      <c r="O71" s="18" t="n"/>
+    </row>
     <row r="72">
-      <c r="A72" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Upstate / Western NY</t>
-        </is>
-      </c>
-      <c r="B72" s="17" t="inlineStr">
-        <is>
-          <t>2 item(s)</t>
-        </is>
-      </c>
-      <c r="C72" s="18" t="n"/>
-      <c r="D72" s="18" t="n"/>
-      <c r="E72" s="18" t="n"/>
-      <c r="F72" s="18" t="n"/>
-      <c r="G72" s="18" t="n"/>
-      <c r="H72" s="19" t="n">
+      <c r="A72" s="11" t="inlineStr">
+        <is>
+          <t>▸ Virginia  (1)</t>
+        </is>
+      </c>
+      <c r="B72" s="12" t="n"/>
+      <c r="C72" s="12" t="n"/>
+      <c r="D72" s="12" t="n"/>
+      <c r="E72" s="12" t="n"/>
+      <c r="F72" s="12" t="n"/>
+      <c r="G72" s="12" t="n"/>
+      <c r="H72" s="12" t="n"/>
+      <c r="I72" s="12" t="n"/>
+      <c r="J72" s="12" t="n"/>
+      <c r="K72" s="12" t="n"/>
+      <c r="L72" s="12" t="n"/>
+      <c r="M72" s="12" t="n"/>
+      <c r="N72" s="12" t="n"/>
+      <c r="O72" s="12" t="n"/>
+    </row>
+    <row r="73" outlineLevel="1">
+      <c r="A73" s="13" t="inlineStr">
+        <is>
+          <t>Virginia</t>
+        </is>
+      </c>
+      <c r="B73" s="14" t="inlineStr">
+        <is>
+          <t>Haynes Furniture / The Dump – 12 stores closing (furniture, mattresses)</t>
+        </is>
+      </c>
+      <c r="C73" s="13" t="inlineStr">
+        <is>
+          <t>retail GOB</t>
+        </is>
+      </c>
+      <c r="D73" s="13" t="inlineStr">
+        <is>
+          <t>Virginia Beach</t>
+        </is>
+      </c>
+      <c r="E73" s="13" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="F73" s="13" t="n">
+        <v>456</v>
+      </c>
+      <c r="G73" s="13" t="inlineStr">
+        <is>
+          <t>Retail GOB markdowns</t>
+        </is>
+      </c>
+      <c r="H73" s="15" t="n"/>
+      <c r="I73" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="J73" s="13" t="inlineStr"/>
+      <c r="K73" s="13" t="inlineStr">
+        <is>
+          <t>SB360 (PR Newswire)</t>
+        </is>
+      </c>
+      <c r="L73" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M73" s="13" t="inlineStr"/>
+      <c r="N73" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O73" s="14" t="inlineStr">
+        <is>
+          <t>Posted Oct 8. Multi-state (VA/AZ/GA/IL/TX); pinned at Virginia Beach. Home goods only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Virginia</t>
+        </is>
+      </c>
+      <c r="B74" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C74" s="18" t="n"/>
+      <c r="D74" s="18" t="n"/>
+      <c r="E74" s="18" t="n"/>
+      <c r="F74" s="18" t="n"/>
+      <c r="G74" s="18" t="n"/>
+      <c r="H74" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I72" s="18" t="n"/>
-      <c r="J72" s="18" t="n"/>
-      <c r="K72" s="18" t="n"/>
-      <c r="L72" s="18" t="n"/>
-      <c r="M72" s="18" t="n"/>
-      <c r="N72" s="18" t="n"/>
-      <c r="O72" s="18" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="11" t="inlineStr">
-        <is>
-          <t>▸ Virginia  (1)</t>
-        </is>
-      </c>
-      <c r="B73" s="12" t="n"/>
-      <c r="C73" s="12" t="n"/>
-      <c r="D73" s="12" t="n"/>
-      <c r="E73" s="12" t="n"/>
-      <c r="F73" s="12" t="n"/>
-      <c r="G73" s="12" t="n"/>
-      <c r="H73" s="12" t="n"/>
-      <c r="I73" s="12" t="n"/>
-      <c r="J73" s="12" t="n"/>
-      <c r="K73" s="12" t="n"/>
-      <c r="L73" s="12" t="n"/>
-      <c r="M73" s="12" t="n"/>
-      <c r="N73" s="12" t="n"/>
-      <c r="O73" s="12" t="n"/>
-    </row>
-    <row r="74" outlineLevel="1">
-      <c r="A74" s="13" t="inlineStr">
-        <is>
-          <t>Virginia</t>
-        </is>
-      </c>
-      <c r="B74" s="14" t="inlineStr">
-        <is>
-          <t>Haynes Furniture / The Dump – 12 stores closing (furniture, mattresses)</t>
-        </is>
-      </c>
-      <c r="C74" s="13" t="inlineStr">
+      <c r="I74" s="18" t="n"/>
+      <c r="J74" s="18" t="n"/>
+      <c r="K74" s="18" t="n"/>
+      <c r="L74" s="18" t="n"/>
+      <c r="M74" s="18" t="n"/>
+      <c r="N74" s="18" t="n"/>
+      <c r="O74" s="18" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="11" t="inlineStr">
+        <is>
+          <t>▸ Midwest  (2)</t>
+        </is>
+      </c>
+      <c r="B75" s="12" t="n"/>
+      <c r="C75" s="12" t="n"/>
+      <c r="D75" s="12" t="n"/>
+      <c r="E75" s="12" t="n"/>
+      <c r="F75" s="12" t="n"/>
+      <c r="G75" s="12" t="n"/>
+      <c r="H75" s="12" t="n"/>
+      <c r="I75" s="12" t="n"/>
+      <c r="J75" s="12" t="n"/>
+      <c r="K75" s="12" t="n"/>
+      <c r="L75" s="12" t="n"/>
+      <c r="M75" s="12" t="n"/>
+      <c r="N75" s="12" t="n"/>
+      <c r="O75" s="12" t="n"/>
+    </row>
+    <row r="76" outlineLevel="1">
+      <c r="A76" s="13" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="B76" s="14" t="inlineStr">
+        <is>
+          <t>American Sale – total liquidation, all 7 stores (pools, hot tubs, grills, holiday decor)</t>
+        </is>
+      </c>
+      <c r="C76" s="13" t="inlineStr">
         <is>
           <t>retail GOB</t>
         </is>
       </c>
-      <c r="D74" s="13" t="inlineStr">
-        <is>
-          <t>Virginia Beach</t>
-        </is>
-      </c>
-      <c r="E74" s="13" t="inlineStr">
-        <is>
-          <t>VA</t>
-        </is>
-      </c>
-      <c r="F74" s="13" t="n">
-        <v>456</v>
-      </c>
-      <c r="G74" s="13" t="inlineStr">
-        <is>
-          <t>Retail GOB markdowns</t>
-        </is>
-      </c>
-      <c r="H74" s="15" t="n"/>
-      <c r="I74" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="J74" s="13" t="inlineStr"/>
-      <c r="K74" s="13" t="inlineStr">
-        <is>
-          <t>SB360 (PR Newswire)</t>
-        </is>
-      </c>
-      <c r="L74" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M74" s="13" t="inlineStr"/>
-      <c r="N74" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O74" s="14" t="inlineStr">
-        <is>
-          <t>Posted Oct 8. Multi-state (VA/AZ/GA/IL/TX); pinned at Virginia Beach. Home goods only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Virginia</t>
-        </is>
-      </c>
-      <c r="B75" s="17" t="inlineStr">
-        <is>
-          <t>1 item(s)</t>
-        </is>
-      </c>
-      <c r="C75" s="18" t="n"/>
-      <c r="D75" s="18" t="n"/>
-      <c r="E75" s="18" t="n"/>
-      <c r="F75" s="18" t="n"/>
-      <c r="G75" s="18" t="n"/>
-      <c r="H75" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I75" s="18" t="n"/>
-      <c r="J75" s="18" t="n"/>
-      <c r="K75" s="18" t="n"/>
-      <c r="L75" s="18" t="n"/>
-      <c r="M75" s="18" t="n"/>
-      <c r="N75" s="18" t="n"/>
-      <c r="O75" s="18" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="11" t="inlineStr">
-        <is>
-          <t>▸ Midwest  (2)</t>
-        </is>
-      </c>
-      <c r="B76" s="12" t="n"/>
-      <c r="C76" s="12" t="n"/>
-      <c r="D76" s="12" t="n"/>
-      <c r="E76" s="12" t="n"/>
-      <c r="F76" s="12" t="n"/>
-      <c r="G76" s="12" t="n"/>
-      <c r="H76" s="12" t="n"/>
-      <c r="I76" s="12" t="n"/>
-      <c r="J76" s="12" t="n"/>
-      <c r="K76" s="12" t="n"/>
-      <c r="L76" s="12" t="n"/>
-      <c r="M76" s="12" t="n"/>
-      <c r="N76" s="12" t="n"/>
-      <c r="O76" s="12" t="n"/>
+      <c r="D76" s="13" t="inlineStr">
+        <is>
+          <t>Chicagoland</t>
+        </is>
+      </c>
+      <c r="E76" s="13" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="F76" s="13" t="n">
+        <v>876</v>
+      </c>
+      <c r="G76" s="13" t="inlineStr">
+        <is>
+          <t>Retail GOB, up to 70% off</t>
+        </is>
+      </c>
+      <c r="H76" s="15" t="n"/>
+      <c r="I76" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="J76" s="13" t="inlineStr"/>
+      <c r="K76" s="13" t="inlineStr">
+        <is>
+          <t>Tiger Group (PR Newswire)</t>
+        </is>
+      </c>
+      <c r="L76" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M76" s="13" t="inlineStr"/>
+      <c r="N76" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O76" s="14" t="inlineStr">
+        <is>
+          <t>Posted Oct 15. Watch for a bulk/fixture auction.</t>
+        </is>
+      </c>
     </row>
     <row r="77" outlineLevel="1">
       <c r="A77" s="13" t="inlineStr">
@@ -22448,47 +22448,47 @@
       </c>
       <c r="B77" s="14" t="inlineStr">
         <is>
-          <t>American Sale – total liquidation, all 7 stores (pools, hot tubs, grills, holiday decor)</t>
+          <t>Straub's Fine Foods store equipment – bakery, kitchen, meat room, Hussmann refrigeration</t>
         </is>
       </c>
       <c r="C77" s="13" t="inlineStr">
         <is>
-          <t>retail GOB</t>
+          <t>grocery/restaurant</t>
         </is>
       </c>
       <c r="D77" s="13" t="inlineStr">
         <is>
-          <t>Chicagoland</t>
+          <t>St. Louis</t>
         </is>
       </c>
       <c r="E77" s="13" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="F77" s="13" t="n">
-        <v>876</v>
+        <v>1046</v>
       </c>
       <c r="G77" s="13" t="inlineStr">
         <is>
-          <t>Retail GOB, up to 70% off</t>
+          <t>Online auction (18% BP)</t>
         </is>
       </c>
       <c r="H77" s="15" t="n"/>
-      <c r="I77" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="J77" s="13" t="inlineStr"/>
+      <c r="I77" s="13" t="inlineStr"/>
+      <c r="J77" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-21 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K77" s="13" t="inlineStr">
         <is>
-          <t>Tiger Group (PR Newswire)</t>
-        </is>
-      </c>
-      <c r="L77" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L77" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M77" s="13" t="inlineStr"/>
@@ -22499,324 +22499,261 @@
       </c>
       <c r="O77" s="14" t="inlineStr">
         <is>
-          <t>Posted Oct 15. Watch for a bulk/fixture auction.</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" outlineLevel="1">
-      <c r="A78" s="13" t="inlineStr">
-        <is>
-          <t>Midwest</t>
-        </is>
-      </c>
-      <c r="B78" s="14" t="inlineStr">
-        <is>
-          <t>Straub's Fine Foods store equipment – bakery, kitchen, meat room, Hussmann refrigeration</t>
-        </is>
-      </c>
-      <c r="C78" s="13" t="inlineStr">
-        <is>
-          <t>grocery/restaurant</t>
-        </is>
-      </c>
-      <c r="D78" s="13" t="inlineStr">
-        <is>
-          <t>St. Louis</t>
-        </is>
-      </c>
-      <c r="E78" s="13" t="inlineStr">
-        <is>
-          <t>MO</t>
-        </is>
-      </c>
-      <c r="F78" s="13" t="n">
-        <v>1046</v>
-      </c>
-      <c r="G78" s="13" t="inlineStr">
-        <is>
-          <t>Online auction (18% BP)</t>
-        </is>
-      </c>
-      <c r="H78" s="15" t="n"/>
-      <c r="I78" s="13" t="inlineStr"/>
-      <c r="J78" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-21 11:00 AM ET</t>
-        </is>
-      </c>
-      <c r="K78" s="13" t="inlineStr">
-        <is>
-          <t>Grafe Auction</t>
-        </is>
-      </c>
-      <c r="L78" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
-        </is>
-      </c>
-      <c r="M78" s="13" t="inlineStr"/>
-      <c r="N78" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O78" s="14" t="inlineStr">
-        <is>
           <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis.</t>
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Midwest</t>
+        </is>
+      </c>
+      <c r="B78" s="17" t="inlineStr">
+        <is>
+          <t>2 item(s)</t>
+        </is>
+      </c>
+      <c r="C78" s="18" t="n"/>
+      <c r="D78" s="18" t="n"/>
+      <c r="E78" s="18" t="n"/>
+      <c r="F78" s="18" t="n"/>
+      <c r="G78" s="18" t="n"/>
+      <c r="H78" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I78" s="18" t="n"/>
+      <c r="J78" s="18" t="n"/>
+      <c r="K78" s="18" t="n"/>
+      <c r="L78" s="18" t="n"/>
+      <c r="M78" s="18" t="n"/>
+      <c r="N78" s="18" t="n"/>
+      <c r="O78" s="18" t="n"/>
+    </row>
     <row r="79">
-      <c r="A79" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Midwest</t>
-        </is>
-      </c>
-      <c r="B79" s="17" t="inlineStr">
-        <is>
-          <t>2 item(s)</t>
-        </is>
-      </c>
-      <c r="C79" s="18" t="n"/>
-      <c r="D79" s="18" t="n"/>
-      <c r="E79" s="18" t="n"/>
-      <c r="F79" s="18" t="n"/>
-      <c r="G79" s="18" t="n"/>
-      <c r="H79" s="19" t="n">
+      <c r="A79" s="11" t="inlineStr">
+        <is>
+          <t>▸ Texas / South Central  (1)</t>
+        </is>
+      </c>
+      <c r="B79" s="12" t="n"/>
+      <c r="C79" s="12" t="n"/>
+      <c r="D79" s="12" t="n"/>
+      <c r="E79" s="12" t="n"/>
+      <c r="F79" s="12" t="n"/>
+      <c r="G79" s="12" t="n"/>
+      <c r="H79" s="12" t="n"/>
+      <c r="I79" s="12" t="n"/>
+      <c r="J79" s="12" t="n"/>
+      <c r="K79" s="12" t="n"/>
+      <c r="L79" s="12" t="n"/>
+      <c r="M79" s="12" t="n"/>
+      <c r="N79" s="12" t="n"/>
+      <c r="O79" s="12" t="n"/>
+    </row>
+    <row r="80" outlineLevel="1">
+      <c r="A80" s="13" t="inlineStr">
+        <is>
+          <t>Texas / South Central</t>
+        </is>
+      </c>
+      <c r="B80" s="14" t="inlineStr">
+        <is>
+          <t>Southwest beverage distributor surplus – mostly unused: 16 True merchandisers, 75 Bunn brewers, 100+ micro-market kiosks</t>
+        </is>
+      </c>
+      <c r="C80" s="13" t="inlineStr">
+        <is>
+          <t>distributor surplus</t>
+        </is>
+      </c>
+      <c r="D80" s="13" t="inlineStr">
+        <is>
+          <t>Mesquite</t>
+        </is>
+      </c>
+      <c r="E80" s="13" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="F80" s="13" t="n">
+        <v>1547</v>
+      </c>
+      <c r="G80" s="13" t="inlineStr">
+        <is>
+          <t>Online auction</t>
+        </is>
+      </c>
+      <c r="H80" s="15" t="n"/>
+      <c r="I80" s="13" t="inlineStr"/>
+      <c r="J80" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-13 11:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K80" s="13" t="inlineStr">
+        <is>
+          <t>Heritage Global Partners</t>
+        </is>
+      </c>
+      <c r="L80" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M80" s="13" t="inlineStr"/>
+      <c r="N80" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O80" s="14" t="inlineStr">
+        <is>
+          <t>Near-new appliances, resell by unit. Nov 13 10 AM CST.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Texas / South Central</t>
+        </is>
+      </c>
+      <c r="B81" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C81" s="18" t="n"/>
+      <c r="D81" s="18" t="n"/>
+      <c r="E81" s="18" t="n"/>
+      <c r="F81" s="18" t="n"/>
+      <c r="G81" s="18" t="n"/>
+      <c r="H81" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I79" s="18" t="n"/>
-      <c r="J79" s="18" t="n"/>
-      <c r="K79" s="18" t="n"/>
-      <c r="L79" s="18" t="n"/>
-      <c r="M79" s="18" t="n"/>
-      <c r="N79" s="18" t="n"/>
-      <c r="O79" s="18" t="n"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="11" t="inlineStr">
-        <is>
-          <t>▸ Texas / South Central  (1)</t>
-        </is>
-      </c>
-      <c r="B80" s="12" t="n"/>
-      <c r="C80" s="12" t="n"/>
-      <c r="D80" s="12" t="n"/>
-      <c r="E80" s="12" t="n"/>
-      <c r="F80" s="12" t="n"/>
-      <c r="G80" s="12" t="n"/>
-      <c r="H80" s="12" t="n"/>
-      <c r="I80" s="12" t="n"/>
-      <c r="J80" s="12" t="n"/>
-      <c r="K80" s="12" t="n"/>
-      <c r="L80" s="12" t="n"/>
-      <c r="M80" s="12" t="n"/>
-      <c r="N80" s="12" t="n"/>
-      <c r="O80" s="12" t="n"/>
-    </row>
-    <row r="81" outlineLevel="1">
-      <c r="A81" s="13" t="inlineStr">
-        <is>
-          <t>Texas / South Central</t>
-        </is>
-      </c>
-      <c r="B81" s="14" t="inlineStr">
-        <is>
-          <t>Southwest beverage distributor surplus – mostly unused: 16 True merchandisers, 75 Bunn brewers, 100+ micro-market kiosks</t>
-        </is>
-      </c>
-      <c r="C81" s="13" t="inlineStr">
-        <is>
-          <t>distributor surplus</t>
-        </is>
-      </c>
-      <c r="D81" s="13" t="inlineStr">
-        <is>
-          <t>Mesquite</t>
-        </is>
-      </c>
-      <c r="E81" s="13" t="inlineStr">
-        <is>
-          <t>TX</t>
-        </is>
-      </c>
-      <c r="F81" s="13" t="n">
-        <v>1547</v>
-      </c>
-      <c r="G81" s="13" t="inlineStr">
-        <is>
-          <t>Online auction</t>
-        </is>
-      </c>
-      <c r="H81" s="15" t="n"/>
-      <c r="I81" s="13" t="inlineStr"/>
-      <c r="J81" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-13 11:00 AM ET</t>
-        </is>
-      </c>
-      <c r="K81" s="13" t="inlineStr">
-        <is>
-          <t>Heritage Global Partners</t>
-        </is>
-      </c>
-      <c r="L81" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M81" s="13" t="inlineStr"/>
-      <c r="N81" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O81" s="14" t="inlineStr">
-        <is>
-          <t>Near-new appliances, resell by unit. Nov 13 10 AM CST.</t>
-        </is>
-      </c>
+      <c r="I81" s="18" t="n"/>
+      <c r="J81" s="18" t="n"/>
+      <c r="K81" s="18" t="n"/>
+      <c r="L81" s="18" t="n"/>
+      <c r="M81" s="18" t="n"/>
+      <c r="N81" s="18" t="n"/>
+      <c r="O81" s="18" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Texas / South Central</t>
-        </is>
-      </c>
-      <c r="B82" s="17" t="inlineStr">
+      <c r="A82" s="11" t="inlineStr">
+        <is>
+          <t>▸ West / Other  (1)</t>
+        </is>
+      </c>
+      <c r="B82" s="12" t="n"/>
+      <c r="C82" s="12" t="n"/>
+      <c r="D82" s="12" t="n"/>
+      <c r="E82" s="12" t="n"/>
+      <c r="F82" s="12" t="n"/>
+      <c r="G82" s="12" t="n"/>
+      <c r="H82" s="12" t="n"/>
+      <c r="I82" s="12" t="n"/>
+      <c r="J82" s="12" t="n"/>
+      <c r="K82" s="12" t="n"/>
+      <c r="L82" s="12" t="n"/>
+      <c r="M82" s="12" t="n"/>
+      <c r="N82" s="12" t="n"/>
+      <c r="O82" s="12" t="n"/>
+    </row>
+    <row r="83" outlineLevel="1">
+      <c r="A83" s="13" t="inlineStr">
+        <is>
+          <t>West / Other</t>
+        </is>
+      </c>
+      <c r="B83" s="14" t="inlineStr">
+        <is>
+          <t>National salad concept liquidation – full contents of 63 fast-casual restaurants (AZ/TX/OK/NV)</t>
+        </is>
+      </c>
+      <c r="C83" s="13" t="inlineStr">
+        <is>
+          <t>restaurant chain liquidation</t>
+        </is>
+      </c>
+      <c r="D83" s="13" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="E83" s="13" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="F83" s="13" t="n">
+        <v>2307</v>
+      </c>
+      <c r="G83" s="13" t="inlineStr">
+        <is>
+          <t>Online auctions, dates TBD</t>
+        </is>
+      </c>
+      <c r="H83" s="15" t="n"/>
+      <c r="I83" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="J83" s="13" t="inlineStr"/>
+      <c r="K83" s="13" t="inlineStr">
+        <is>
+          <t>RestaurantEquipment.bid (TAGeX)</t>
+        </is>
+      </c>
+      <c r="L83" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M83" s="13" t="inlineStr"/>
+      <c r="N83" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O83" s="14" t="inlineStr">
+        <is>
+          <t>Rolling market-by-market auctions, none live yet (Phoenix metro 30 locations, DFW 14, Tucson 6, Houston 5, plus OK/NV). Pickup on site at each restaurant. Pinned at Phoenix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — West / Other</t>
+        </is>
+      </c>
+      <c r="B84" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C82" s="18" t="n"/>
-      <c r="D82" s="18" t="n"/>
-      <c r="E82" s="18" t="n"/>
-      <c r="F82" s="18" t="n"/>
-      <c r="G82" s="18" t="n"/>
-      <c r="H82" s="19" t="n">
+      <c r="C84" s="18" t="n"/>
+      <c r="D84" s="18" t="n"/>
+      <c r="E84" s="18" t="n"/>
+      <c r="F84" s="18" t="n"/>
+      <c r="G84" s="18" t="n"/>
+      <c r="H84" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I82" s="18" t="n"/>
-      <c r="J82" s="18" t="n"/>
-      <c r="K82" s="18" t="n"/>
-      <c r="L82" s="18" t="n"/>
-      <c r="M82" s="18" t="n"/>
-      <c r="N82" s="18" t="n"/>
-      <c r="O82" s="18" t="n"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="11" t="inlineStr">
-        <is>
-          <t>▸ West / Other  (1)</t>
-        </is>
-      </c>
-      <c r="B83" s="12" t="n"/>
-      <c r="C83" s="12" t="n"/>
-      <c r="D83" s="12" t="n"/>
-      <c r="E83" s="12" t="n"/>
-      <c r="F83" s="12" t="n"/>
-      <c r="G83" s="12" t="n"/>
-      <c r="H83" s="12" t="n"/>
-      <c r="I83" s="12" t="n"/>
-      <c r="J83" s="12" t="n"/>
-      <c r="K83" s="12" t="n"/>
-      <c r="L83" s="12" t="n"/>
-      <c r="M83" s="12" t="n"/>
-      <c r="N83" s="12" t="n"/>
-      <c r="O83" s="12" t="n"/>
-    </row>
-    <row r="84" outlineLevel="1">
-      <c r="A84" s="13" t="inlineStr">
-        <is>
-          <t>West / Other</t>
-        </is>
-      </c>
-      <c r="B84" s="14" t="inlineStr">
-        <is>
-          <t>National salad concept liquidation – full contents of 63 fast-casual restaurants (AZ/TX/OK/NV)</t>
-        </is>
-      </c>
-      <c r="C84" s="13" t="inlineStr">
-        <is>
-          <t>restaurant chain liquidation</t>
-        </is>
-      </c>
-      <c r="D84" s="13" t="inlineStr">
-        <is>
-          <t>Phoenix</t>
-        </is>
-      </c>
-      <c r="E84" s="13" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="F84" s="13" t="n">
-        <v>2307</v>
-      </c>
-      <c r="G84" s="13" t="inlineStr">
-        <is>
-          <t>Online auctions, dates TBD</t>
-        </is>
-      </c>
-      <c r="H84" s="15" t="n"/>
-      <c r="I84" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="J84" s="13" t="inlineStr"/>
-      <c r="K84" s="13" t="inlineStr">
-        <is>
-          <t>RestaurantEquipment.bid (TAGeX)</t>
-        </is>
-      </c>
-      <c r="L84" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M84" s="13" t="inlineStr"/>
-      <c r="N84" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O84" s="14" t="inlineStr">
-        <is>
-          <t>Rolling market-by-market auctions, none live yet (Phoenix metro 30 locations, DFW 14, Tucson 6, Houston 5, plus OK/NV). Pickup on site at each restaurant. Pinned at Phoenix.</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — West / Other</t>
-        </is>
-      </c>
-      <c r="B85" s="17" t="inlineStr">
-        <is>
-          <t>1 item(s)</t>
-        </is>
-      </c>
-      <c r="C85" s="18" t="n"/>
-      <c r="D85" s="18" t="n"/>
-      <c r="E85" s="18" t="n"/>
-      <c r="F85" s="18" t="n"/>
-      <c r="G85" s="18" t="n"/>
-      <c r="H85" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I85" s="18" t="n"/>
-      <c r="J85" s="18" t="n"/>
-      <c r="K85" s="18" t="n"/>
-      <c r="L85" s="18" t="n"/>
-      <c r="M85" s="18" t="n"/>
-      <c r="N85" s="18" t="n"/>
-      <c r="O85" s="18" t="n"/>
+      <c r="I84" s="18" t="n"/>
+      <c r="J84" s="18" t="n"/>
+      <c r="K84" s="18" t="n"/>
+      <c r="L84" s="18" t="n"/>
+      <c r="M84" s="18" t="n"/>
+      <c r="N84" s="18" t="n"/>
+      <c r="O84" s="18" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O85"/>
+  <autoFilter ref="A1:O84"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId2"/>
@@ -22870,12 +22807,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N66" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N67" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N70" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N71" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N74" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N73" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N76" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N77" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N78" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N81" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N84" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N80" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N83" r:id="rId57"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -22887,7 +22823,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O18"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -23049,7 +22985,7 @@
       </c>
       <c r="O2" s="14" t="inlineStr">
         <is>
-          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23112,7 +23048,7 @@
       </c>
       <c r="O3" s="14" t="inlineStr">
         <is>
-          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23313,7 +23249,7 @@
       </c>
       <c r="O6" s="14" t="inlineStr">
         <is>
-          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23378,7 +23314,7 @@
       </c>
       <c r="O7" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23443,7 +23379,7 @@
       </c>
       <c r="O8" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23508,7 +23444,7 @@
       </c>
       <c r="O9" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23571,7 +23507,7 @@
       </c>
       <c r="O10" s="14" t="inlineStr">
         <is>
-          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23634,7 +23570,7 @@
       </c>
       <c r="O11" s="14" t="inlineStr">
         <is>
-          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23697,7 +23633,7 @@
       </c>
       <c r="O12" s="14" t="inlineStr">
         <is>
-          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23760,59 +23696,59 @@
       </c>
       <c r="O13" s="14" t="inlineStr">
         <is>
-          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>Upstate / Western NY</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>Freshway Market whole-grocery liquidation – refrigeration racks, cases, walk-ins, generator</t>
+          <t>Former Taco Del Mar – stainless, warmers, walk-in panels</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Watson</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>862</v>
+        <v>260</v>
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>HiBid online auction</t>
         </is>
       </c>
       <c r="H14" s="15" t="n"/>
       <c r="I14" s="13" t="inlineStr"/>
       <c r="J14" s="13" t="inlineStr">
         <is>
-          <t>2026-10-20 11:00 AM ET</t>
+          <t>2026-10-20 06:00 PM ET</t>
         </is>
       </c>
       <c r="K14" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
+          <t>Adirondack Asset / HiBid</t>
         </is>
       </c>
       <c r="L14" s="13" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-10-20 11:00 AM ET)</t>
+          <t>EXPIRED (2026-10-20 06:00 PM ET)</t>
         </is>
       </c>
       <c r="M14" s="13" t="inlineStr"/>
@@ -23823,59 +23759,59 @@
       </c>
       <c r="O14" s="14" t="inlineStr">
         <is>
-          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Small lot. [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>Greater Boston / South Shore (&lt;50mi)</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>Closed Best Buy Outlet – pallet racking, Big Joe order pickers, appliance dollies, carts, cages</t>
+          <t>Freshway Market whole-grocery liquidation – refrigeration racks, cases, walk-ins, generator</t>
         </is>
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>store closing fixtures</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
-          <t>Brockton</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>11</v>
+        <v>862</v>
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t>Racking $40/upright, $80/level; pickers $1,000 OBO</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H15" s="15" t="n"/>
-      <c r="I15" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="J15" s="13" t="inlineStr"/>
+      <c r="I15" s="13" t="inlineStr"/>
+      <c r="J15" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-20 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K15" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>Grafe Auction</t>
         </is>
       </c>
       <c r="L15" s="13" t="inlineStr">
         <is>
-          <t>REMOVED</t>
+          <t>EXPIRED (2026-10-20 11:00 AM ET)</t>
         </is>
       </c>
       <c r="M15" s="13" t="inlineStr"/>
@@ -23886,63 +23822,59 @@
       </c>
       <c r="O15" s="14" t="inlineStr">
         <is>
-          <t>200 Westgate Dr. Fixtures/equipment only, no merchandise. On site daily. CL deleted by author (HTTP 410) as of 2026-10-19 midday recheck.</t>
+          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>NYC / Long Island / NJ</t>
+          <t>Greater Boston / South Shore (&lt;50mi)</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>Like-new restaurant – steam tables, Coldline, Cleveland cook-and-hold, fryers, True freezers</t>
+          <t>Closed Best Buy Outlet – pallet racking, Big Joe order pickers, appliance dollies, carts, cages</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>store closing fixtures</t>
         </is>
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
-          <t>Staten Island</t>
+          <t>Brockton</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>203</v>
+        <v>11</v>
       </c>
       <c r="G16" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>Racking $40/upright, $80/level; pickers $1,000 OBO</t>
         </is>
       </c>
       <c r="H16" s="15" t="n"/>
       <c r="I16" s="13" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="J16" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-19 01:00 PM ET</t>
-        </is>
-      </c>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="J16" s="13" t="inlineStr"/>
       <c r="K16" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L16" s="13" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-10-19 01:00 PM ET)</t>
+          <t>REMOVED</t>
         </is>
       </c>
       <c r="M16" s="13" t="inlineStr"/>
@@ -23953,7 +23885,7 @@
       </c>
       <c r="O16" s="14" t="inlineStr">
         <is>
-          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>200 Westgate Dr. Fixtures/equipment only, no merchandise. On site daily. CL deleted by author (HTTP 410) as of 2026-10-19 midday recheck.</t>
         </is>
       </c>
     </row>
@@ -23965,26 +23897,26 @@
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>Restaurant / pizzeria (contents not described)</t>
+          <t>Like-new restaurant – steam tables, Coldline, Cleveland cook-and-hold, fryers, True freezers</t>
         </is>
       </c>
       <c r="C17" s="13" t="inlineStr">
         <is>
-          <t>restaurant closing</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>Berkeley Heights</t>
+          <t>Staten Island</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>NJ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
@@ -23994,12 +23926,12 @@
       <c r="H17" s="15" t="n"/>
       <c r="I17" s="13" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="J17" s="13" t="inlineStr">
         <is>
-          <t>2026-10-20 02:00 PM ET</t>
+          <t>2026-10-19 01:00 PM ET</t>
         </is>
       </c>
       <c r="K17" s="13" t="inlineStr">
@@ -24009,7 +23941,7 @@
       </c>
       <c r="L17" s="13" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-10-20 02:00 PM ET)</t>
+          <t>EXPIRED (2026-10-19 01:00 PM ET)</t>
         </is>
       </c>
       <c r="M17" s="13" t="inlineStr"/>
@@ -24020,7 +23952,7 @@
       </c>
       <c r="O17" s="14" t="inlineStr">
         <is>
-          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed]</t>
+          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24032,7 +23964,7 @@
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>High-end deli (contents not described)</t>
+          <t>Restaurant / pizzeria (contents not described)</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
@@ -24042,7 +23974,7 @@
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>Manalapan Township</t>
+          <t>Berkeley Heights</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
@@ -24051,7 +23983,7 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="G18" s="13" t="inlineStr">
         <is>
@@ -24061,12 +23993,12 @@
       <c r="H18" s="15" t="n"/>
       <c r="I18" s="13" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="J18" s="13" t="inlineStr">
         <is>
-          <t>2026-10-19 04:00 PM ET</t>
+          <t>2026-10-20 02:00 PM ET</t>
         </is>
       </c>
       <c r="K18" s="13" t="inlineStr">
@@ -24076,7 +24008,7 @@
       </c>
       <c r="L18" s="13" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-10-19 04:00 PM ET)</t>
+          <t>EXPIRED (2026-10-20 02:00 PM ET)</t>
         </is>
       </c>
       <c r="M18" s="13" t="inlineStr"/>
@@ -24087,12 +24019,79 @@
       </c>
       <c r="O18" s="14" t="inlineStr">
         <is>
-          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>High-end deli (contents not described)</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>restaurant closing</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>Manalapan Township</t>
+        </is>
+      </c>
+      <c r="E19" s="13" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="n">
+        <v>223</v>
+      </c>
+      <c r="G19" s="13" t="inlineStr">
+        <is>
+          <t>Live + webcast, 18% BP + 3%</t>
+        </is>
+      </c>
+      <c r="H19" s="15" t="n"/>
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="J19" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 04:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K19" s="13" t="inlineStr">
+        <is>
+          <t>HiBid (Best Buy Auctioneers)</t>
+        </is>
+      </c>
+      <c r="L19" s="13" t="inlineStr">
+        <is>
+          <t>EXPIRED (2026-10-19 04:00 PM ET)</t>
+        </is>
+      </c>
+      <c r="M19" s="13" t="inlineStr"/>
+      <c r="N19" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O19" s="14" t="inlineStr">
+        <is>
+          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O18"/>
+  <autoFilter ref="A1:O19"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
@@ -24111,6 +24110,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Watch update 2026-10-21 8am ET: +2 parts (Montrose CO, SLC UT businesses), +2 liquidations (South Amboy NJ, Austin MN); Waltham repost URL
</commit_message>
<xml_diff>
--- a/lot_recon.xlsx
+++ b/lot_recon.xlsx
@@ -16,11 +16,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Removed" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Appliance Parts'!$A$1:$O$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Appliance Parts'!$A$1:$O$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wolf New'!$A$1:$O$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Wolf Used'!$A$1:$O$189</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Wolf Unclear'!$A$1:$O$40</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$86</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 2026-10-20 18:00 ET</t>
+          <t>Last updated: 2026-10-21 08:05 ET</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Active listings: 294 · Removed: 18</t>
+          <t>Active listings: 298 · Removed: 18</t>
         </is>
       </c>
     </row>
@@ -641,10 +641,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>159646</v>
+        <v>454646</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
@@ -679,7 +679,7 @@
         <v>164</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>608027.6</v>
+        <v>608029.6</v>
       </c>
       <c r="D10" t="n">
         <v>3</v>
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>0</v>
@@ -724,10 +724,10 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>980438.58</v>
+        <v>1275440.58</v>
       </c>
     </row>
     <row r="15">
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C24" t="n">
         <v>1</v>
@@ -1037,7 +1037,7 @@
         <v>24</v>
       </c>
       <c r="G24" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H24" s="6" t="n">
         <v>440141</v>
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C30" t="n">
         <v>1</v>
@@ -1235,14 +1235,14 @@
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>807–1046</t>
+          <t>807–1124</t>
         </is>
       </c>
     </row>
@@ -1319,10 +1319,10 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C33" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
@@ -1337,11 +1337,11 @@
         <v>1</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>75000</v>
+        <v>370000</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2307–2317</t>
+          <t>1954–2317</t>
         </is>
       </c>
     </row>
@@ -1396,7 +1396,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O39"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2858,7 +2858,7 @@
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>▸ West / Other  (2)</t>
+          <t>▸ West / Other  (4)</t>
         </is>
       </c>
       <c r="B36" s="12" t="n"/>
@@ -2884,36 +2884,38 @@
       </c>
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>Storage locker filled with appliance parts – washer/dryer parts, heating elements, cords, rollers, belts, tools</t>
+          <t>Appliance service business for sale (Western Slope) - established warranty-servicer setups with many manufacturers</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>bulk lot</t>
+          <t>business for sale</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Montrose</t>
         </is>
       </c>
       <c r="E37" s="13" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>2307</v>
+        <v>1954</v>
       </c>
       <c r="G37" s="13" t="inlineStr">
         <is>
-          <t>Message for pricing</t>
-        </is>
-      </c>
-      <c r="H37" s="15" t="n"/>
+          <t>$110,000</t>
+        </is>
+      </c>
+      <c r="H37" s="15" t="n">
+        <v>110000</v>
+      </c>
       <c r="I37" s="13" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="J37" s="13" t="inlineStr"/>
@@ -2935,7 +2937,7 @@
       </c>
       <c r="O37" s="14" t="inlineStr">
         <is>
-          <t>Seller is getting out of the appliance business; selling the whole locker (North Phoenix, Deer Valley Rd near 19th Ave). Delivery available per post. Separate from the Phoenix parts-store closing ad.</t>
+          <t>Going-concern service business; possible seller financing; no parts inventory mentioned. Updated 2026-10-17.</t>
         </is>
       </c>
     </row>
@@ -2947,7 +2949,7 @@
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>Appliance repair &amp; sales business for sale – 100+ appliances (~90% new), liftgate truck, large powered storage unit</t>
+          <t>Appliance Repair Technicians: Own the Business - $65K parts inventory/stock + $25K FF&amp;E + 2022 Promaster van</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
@@ -2957,34 +2959,30 @@
       </c>
       <c r="D38" s="13" t="inlineStr">
         <is>
-          <t>Surprise</t>
+          <t>Salt Lake City</t>
         </is>
       </c>
       <c r="E38" s="13" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>UT</t>
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>2317</v>
+        <v>2109</v>
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>$75,000</t>
+          <t>$185,000 (price reduced)</t>
         </is>
       </c>
       <c r="H38" s="15" t="n">
-        <v>75000</v>
-      </c>
-      <c r="I38" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
+        <v>185000</v>
+      </c>
+      <c r="I38" s="13" t="inlineStr"/>
       <c r="J38" s="13" t="inlineStr"/>
       <c r="K38" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>BusinessesForSale (First Choice Business Brokers #3924670)</t>
         </is>
       </c>
       <c r="L38" s="13" t="inlineStr">
@@ -3000,39 +2998,167 @@
       </c>
       <c r="O38" s="14" t="inlineStr">
         <is>
+          <t>Home-based, est. March 2020, Salt Lake County UT. Includes ~$65K inventory/stock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" outlineLevel="1">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>West / Other</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>Storage locker filled with appliance parts – washer/dryer parts, heating elements, cords, rollers, belts, tools</t>
+        </is>
+      </c>
+      <c r="C39" s="13" t="inlineStr">
+        <is>
+          <t>bulk lot</t>
+        </is>
+      </c>
+      <c r="D39" s="13" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="E39" s="13" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="F39" s="13" t="n">
+        <v>2307</v>
+      </c>
+      <c r="G39" s="13" t="inlineStr">
+        <is>
+          <t>Message for pricing</t>
+        </is>
+      </c>
+      <c r="H39" s="15" t="n"/>
+      <c r="I39" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="J39" s="13" t="inlineStr"/>
+      <c r="K39" s="13" t="inlineStr">
+        <is>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L39" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M39" s="13" t="inlineStr"/>
+      <c r="N39" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O39" s="14" t="inlineStr">
+        <is>
+          <t>Seller is getting out of the appliance business; selling the whole locker (North Phoenix, Deer Valley Rd near 19th Ave). Delivery available per post. Separate from the Phoenix parts-store closing ad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" outlineLevel="1">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>West / Other</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>Appliance repair &amp; sales business for sale – 100+ appliances (~90% new), liftgate truck, large powered storage unit</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr">
+        <is>
+          <t>business for sale</t>
+        </is>
+      </c>
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>Surprise</t>
+        </is>
+      </c>
+      <c r="E40" s="13" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="F40" s="13" t="n">
+        <v>2317</v>
+      </c>
+      <c r="G40" s="13" t="inlineStr">
+        <is>
+          <t>$75,000</t>
+        </is>
+      </c>
+      <c r="H40" s="15" t="n">
+        <v>75000</v>
+      </c>
+      <c r="I40" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="J40" s="13" t="inlineStr"/>
+      <c r="K40" s="13" t="inlineStr">
+        <is>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L40" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M40" s="13" t="inlineStr"/>
+      <c r="N40" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O40" s="14" t="inlineStr">
+        <is>
           <t>Retiring owner of 14-year business serving rental-property owners. Whole appliances (fridges, stoves, microwaves, dishwashers, W/D), not a parts inventory. Storage unit near Dysart &amp; Bell Rd. By appointment only.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="17" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="17" t="inlineStr">
         <is>
           <t>Subtotal — West / Other</t>
         </is>
       </c>
-      <c r="B39" s="17" t="inlineStr">
-        <is>
-          <t>2 item(s)</t>
-        </is>
-      </c>
-      <c r="C39" s="18" t="n"/>
-      <c r="D39" s="18" t="n"/>
-      <c r="E39" s="18" t="n"/>
-      <c r="F39" s="18" t="n"/>
-      <c r="G39" s="18" t="n"/>
-      <c r="H39" s="19" t="n">
-        <v>75000</v>
-      </c>
-      <c r="I39" s="18" t="n"/>
-      <c r="J39" s="18" t="n"/>
-      <c r="K39" s="18" t="n"/>
-      <c r="L39" s="18" t="n"/>
-      <c r="M39" s="18" t="n"/>
-      <c r="N39" s="18" t="n"/>
-      <c r="O39" s="18" t="n"/>
+      <c r="B41" s="17" t="inlineStr">
+        <is>
+          <t>4 item(s)</t>
+        </is>
+      </c>
+      <c r="C41" s="18" t="n"/>
+      <c r="D41" s="18" t="n"/>
+      <c r="E41" s="18" t="n"/>
+      <c r="F41" s="18" t="n"/>
+      <c r="G41" s="18" t="n"/>
+      <c r="H41" s="19" t="n">
+        <v>370000</v>
+      </c>
+      <c r="I41" s="18" t="n"/>
+      <c r="J41" s="18" t="n"/>
+      <c r="K41" s="18" t="n"/>
+      <c r="L41" s="18" t="n"/>
+      <c r="M41" s="18" t="n"/>
+      <c r="N41" s="18" t="n"/>
+      <c r="O41" s="18" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O39"/>
+  <autoFilter ref="A1:O41"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId2"/>
@@ -3050,6 +3176,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N38" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N39" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N40" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12308,11 +12436,11 @@
       </c>
       <c r="G126" s="13" t="inlineStr">
         <is>
-          <t>$5 high bid</t>
+          <t>$7 high bid (3 bids)</t>
         </is>
       </c>
       <c r="H126" s="15" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I126" s="13" t="inlineStr"/>
       <c r="J126" s="13" t="inlineStr">
@@ -12363,7 +12491,7 @@
       <c r="F127" s="18" t="n"/>
       <c r="G127" s="18" t="n"/>
       <c r="H127" s="19" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I127" s="18" t="n"/>
       <c r="J127" s="18" t="n"/>
@@ -18412,7 +18540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O84"/>
+  <dimension ref="A1:O86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -18715,7 +18843,7 @@
       </c>
       <c r="O5" s="14" t="inlineStr">
         <is>
-          <t>Small off-category FYI; seller says resell individually. Old CL URL deleted; reposted under new URL 2026-10-19 (same $250 / 10 tools).</t>
+          <t>Small off-category FYI; seller says resell individually. Old CL URL deleted; reposted under new URL 2026-10-19 (same $250 / 10 tools). Reposted again 2026-10-21 under new URL (same $250 / 10 tools).</t>
         </is>
       </c>
     </row>
@@ -20146,7 +20274,7 @@
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>▸ NYC / Long Island / NJ  (24)</t>
+          <t>▸ NYC / Long Island / NJ  (25)</t>
         </is>
       </c>
       <c r="B34" s="12" t="n"/>
@@ -21243,17 +21371,17 @@
       </c>
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>New modular concession kitchens (warehouseman's lien) – 5 units, CaptiveAire hoods, new Ovention/Turbo Air</t>
+          <t>Bimmer Clinic business liquidation (BMW repair shop): vehicle lifts, forklift, skid steer, refrigerant recovery, shop tools &amp; equipment</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>lien sale</t>
+          <t>business liquidation auction</t>
         </is>
       </c>
       <c r="D52" s="13" t="inlineStr">
         <is>
-          <t>Edison</t>
+          <t>South Amboy</t>
         </is>
       </c>
       <c r="E52" s="13" t="inlineStr">
@@ -21262,19 +21390,23 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>Online auction, $2K load-out fee</t>
+          <t>Timed online auction</t>
         </is>
       </c>
       <c r="H52" s="15" t="n"/>
       <c r="I52" s="13" t="inlineStr"/>
-      <c r="J52" s="13" t="inlineStr"/>
+      <c r="J52" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-12 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K52" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
+          <t>AJ Willner Auctions</t>
         </is>
       </c>
       <c r="L52" s="13" t="inlineStr">
@@ -21290,7 +21422,7 @@
       </c>
       <c r="O52" s="14" t="inlineStr">
         <is>
-          <t>&gt;$100K new. Close date not captured.</t>
+          <t>Ends Nov 12 11 AM EST.</t>
         </is>
       </c>
     </row>
@@ -21302,12 +21434,12 @@
       </c>
       <c r="B53" s="14" t="inlineStr">
         <is>
-          <t>Brand-new &amp; scratch-and-dent kitchen/home appliances – ~185 lots (Thermador, GE Café, Miele, Wolf speed oven, Viking, Bosch…)</t>
+          <t>New modular concession kitchens (warehouseman's lien) – 5 units, CaptiveAire hoods, new Ovention/Turbo Air</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>lien sale</t>
         </is>
       </c>
       <c r="D53" s="13" t="inlineStr">
@@ -21325,23 +21457,15 @@
       </c>
       <c r="G53" s="13" t="inlineStr">
         <is>
-          <t>Live + HiBid webcast, 18% BP + 3% card</t>
+          <t>Online auction, $2K load-out fee</t>
         </is>
       </c>
       <c r="H53" s="15" t="n"/>
-      <c r="I53" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="J53" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-25 01:00 PM ET</t>
-        </is>
-      </c>
+      <c r="I53" s="13" t="inlineStr"/>
+      <c r="J53" s="13" t="inlineStr"/>
       <c r="K53" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>A.J. Willner</t>
         </is>
       </c>
       <c r="L53" s="13" t="inlineStr">
@@ -21349,11 +21473,7 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M53" s="21" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
+      <c r="M53" s="13" t="inlineStr"/>
       <c r="N53" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -21361,7 +21481,7 @@
       </c>
       <c r="O53" s="14" t="inlineStr">
         <is>
-          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale.</t>
+          <t>&gt;$100K new. Close date not captured.</t>
         </is>
       </c>
     </row>
@@ -21373,17 +21493,17 @@
       </c>
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>Party City (Ch. 11) store – fixtures + party merchandise inventory</t>
+          <t>Brand-new &amp; scratch-and-dent kitchen/home appliances – ~185 lots (Thermador, GE Café, Miele, Wolf speed oven, Viking, Bosch…)</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D54" s="13" t="inlineStr">
         <is>
-          <t>East Brunswick</t>
+          <t>Edison</t>
         </is>
       </c>
       <c r="E54" s="13" t="inlineStr">
@@ -21392,23 +21512,27 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Live + HiBid webcast, 18% BP + 3% card</t>
         </is>
       </c>
       <c r="H54" s="15" t="n"/>
-      <c r="I54" s="13" t="inlineStr"/>
+      <c r="I54" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
       <c r="J54" s="13" t="inlineStr">
         <is>
-          <t>2026-11-03 11:00 AM ET</t>
+          <t>2026-10-25 01:00 PM ET</t>
         </is>
       </c>
       <c r="K54" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
       <c r="L54" s="13" t="inlineStr">
@@ -21416,7 +21540,11 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M54" s="13" t="inlineStr"/>
+      <c r="M54" s="21" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
       <c r="N54" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -21424,7 +21552,7 @@
       </c>
       <c r="O54" s="14" t="inlineStr">
         <is>
-          <t>Store inventory.</t>
+          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale.</t>
         </is>
       </c>
     </row>
@@ -21436,17 +21564,17 @@
       </c>
       <c r="B55" s="14" t="inlineStr">
         <is>
-          <t>Bakery/Cafe Somerville NJ – rack ovens, La Marzocco, food truck (~76 lots)</t>
+          <t>Party City (Ch. 11) store – fixtures + party merchandise inventory</t>
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D55" s="13" t="inlineStr">
         <is>
-          <t>Somerville</t>
+          <t>East Brunswick</t>
         </is>
       </c>
       <c r="E55" s="13" t="inlineStr">
@@ -21455,27 +21583,23 @@
         </is>
       </c>
       <c r="F55" s="13" t="n">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="G55" s="13" t="inlineStr">
         <is>
-          <t>Live webcast + online (18% BP online)</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H55" s="15" t="n"/>
-      <c r="I55" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
+      <c r="I55" s="13" t="inlineStr"/>
       <c r="J55" s="13" t="inlineStr">
         <is>
-          <t>2026-10-26 02:00 PM ET</t>
+          <t>2026-11-03 11:00 AM ET</t>
         </is>
       </c>
       <c r="K55" s="13" t="inlineStr">
         <is>
-          <t>HiBid / Best Buy Auctioneers</t>
+          <t>A.J. Willner</t>
         </is>
       </c>
       <c r="L55" s="13" t="inlineStr">
@@ -21491,7 +21615,7 @@
       </c>
       <c r="O55" s="14" t="inlineStr">
         <is>
-          <t>Full bakery/cafe commercial kitchen: food truck w/ pizza oven, La Marzocco espresso, Mazzer, Baxter + Empire Logiudice rack ovens, dough depositor, Globe floor mixer, Artic Air / SS refrigeration, fryers, Vitamix, Robot Coupe, display cases, dining furniture. Preview 11 AM sale day; checkout Tue 10/27.</t>
+          <t>Store inventory.</t>
         </is>
       </c>
     </row>
@@ -21503,7 +21627,7 @@
       </c>
       <c r="B56" s="14" t="inlineStr">
         <is>
-          <t>Ability to Work kitchen and store – commercial kitchen + store fixtures (~135 lots)</t>
+          <t>Bakery/Cafe Somerville NJ – rack ovens, La Marzocco, food truck (~76 lots)</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
@@ -21513,7 +21637,7 @@
       </c>
       <c r="D56" s="13" t="inlineStr">
         <is>
-          <t>Flemington</t>
+          <t>Somerville</t>
         </is>
       </c>
       <c r="E56" s="13" t="inlineStr">
@@ -21522,23 +21646,27 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>237</v>
+        <v>224</v>
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>Timed online (15% BP)</t>
+          <t>Live webcast + online (18% BP online)</t>
         </is>
       </c>
       <c r="H56" s="15" t="n"/>
-      <c r="I56" s="13" t="inlineStr"/>
+      <c r="I56" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
       <c r="J56" s="13" t="inlineStr">
         <is>
-          <t>2026-10-27 11:02 AM ET</t>
+          <t>2026-10-26 02:00 PM ET</t>
         </is>
       </c>
       <c r="K56" s="13" t="inlineStr">
         <is>
-          <t>HiBid</t>
+          <t>HiBid / Best Buy Auctioneers</t>
         </is>
       </c>
       <c r="L56" s="13" t="inlineStr">
@@ -21554,7 +21682,7 @@
       </c>
       <c r="O56" s="14" t="inlineStr">
         <is>
-          <t>Apprentice/hospitality training cafe-kitchen and store dispersal. Preview 9–11 AM sale day; removal Oct 27 noon–Oct 29.</t>
+          <t>Full bakery/cafe commercial kitchen: food truck w/ pizza oven, La Marzocco espresso, Mazzer, Baxter + Empire Logiudice rack ovens, dough depositor, Globe floor mixer, Artic Air / SS refrigeration, fryers, Vitamix, Robot Coupe, display cases, dining furniture. Preview 11 AM sale day; checkout Tue 10/27.</t>
         </is>
       </c>
     </row>
@@ -21566,17 +21694,17 @@
       </c>
       <c r="B57" s="14" t="inlineStr">
         <is>
-          <t>Wren Kitchens showroom closing – JennAir/Café/KitchenAid/GE Profile appliances + display kitchens</t>
+          <t>Ability to Work kitchen and store – commercial kitchen + store fixtures (~135 lots)</t>
         </is>
       </c>
       <c r="C57" s="13" t="inlineStr">
         <is>
-          <t>showroom closing</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D57" s="13" t="inlineStr">
         <is>
-          <t>Lawrenceville</t>
+          <t>Flemington</t>
         </is>
       </c>
       <c r="E57" s="13" t="inlineStr">
@@ -21585,23 +21713,23 @@
         </is>
       </c>
       <c r="F57" s="13" t="n">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="G57" s="13" t="inlineStr">
         <is>
-          <t>Online auction, 18% BP</t>
+          <t>Timed online (15% BP)</t>
         </is>
       </c>
       <c r="H57" s="15" t="n"/>
       <c r="I57" s="13" t="inlineStr"/>
       <c r="J57" s="13" t="inlineStr">
         <is>
-          <t>2026-10-27 09:00 AM ET</t>
+          <t>2026-10-27 11:02 AM ET</t>
         </is>
       </c>
       <c r="K57" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
+          <t>HiBid</t>
         </is>
       </c>
       <c r="L57" s="13" t="inlineStr">
@@ -21617,7 +21745,7 @@
       </c>
       <c r="O57" s="14" t="inlineStr">
         <is>
-          <t>Premium floor-model appliances; lots close from Oct 27 9 AM.</t>
+          <t>Apprentice/hospitality training cafe-kitchen and store dispersal. Preview 9–11 AM sale day; removal Oct 27 noon–Oct 29.</t>
         </is>
       </c>
     </row>
@@ -21629,7 +21757,7 @@
       </c>
       <c r="B58" s="14" t="inlineStr">
         <is>
-          <t>Wren Kitchens showroom closing – GE/Whirlpool/KitchenAid/Café incl. NIB Café range + 35 kitchens</t>
+          <t>Wren Kitchens showroom closing – JennAir/Café/KitchenAid/GE Profile appliances + display kitchens</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
@@ -21639,7 +21767,7 @@
       </c>
       <c r="D58" s="13" t="inlineStr">
         <is>
-          <t>Cherry Hill</t>
+          <t>Lawrenceville</t>
         </is>
       </c>
       <c r="E58" s="13" t="inlineStr">
@@ -21648,18 +21776,18 @@
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>266</v>
+        <v>239</v>
       </c>
       <c r="G58" s="13" t="inlineStr">
         <is>
-          <t>Online auction, openers ~$0.50</t>
+          <t>Online auction, 18% BP</t>
         </is>
       </c>
       <c r="H58" s="15" t="n"/>
       <c r="I58" s="13" t="inlineStr"/>
       <c r="J58" s="13" t="inlineStr">
         <is>
-          <t>2026-11-02 11:00 AM ET</t>
+          <t>2026-10-27 09:00 AM ET</t>
         </is>
       </c>
       <c r="K58" s="13" t="inlineStr">
@@ -21680,124 +21808,120 @@
       </c>
       <c r="O58" s="14" t="inlineStr">
         <is>
+          <t>Premium floor-model appliances; lots close from Oct 27 9 AM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" outlineLevel="1">
+      <c r="A59" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B59" s="14" t="inlineStr">
+        <is>
+          <t>Wren Kitchens showroom closing – GE/Whirlpool/KitchenAid/Café incl. NIB Café range + 35 kitchens</t>
+        </is>
+      </c>
+      <c r="C59" s="13" t="inlineStr">
+        <is>
+          <t>showroom closing</t>
+        </is>
+      </c>
+      <c r="D59" s="13" t="inlineStr">
+        <is>
+          <t>Cherry Hill</t>
+        </is>
+      </c>
+      <c r="E59" s="13" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="F59" s="13" t="n">
+        <v>266</v>
+      </c>
+      <c r="G59" s="13" t="inlineStr">
+        <is>
+          <t>Online auction, openers ~$0.50</t>
+        </is>
+      </c>
+      <c r="H59" s="15" t="n"/>
+      <c r="I59" s="13" t="inlineStr"/>
+      <c r="J59" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-02 11:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K59" s="13" t="inlineStr">
+        <is>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L59" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M59" s="13" t="inlineStr"/>
+      <c r="N59" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O59" s="14" t="inlineStr">
+        <is>
           <t>Lots close from Nov 2 11 AM.</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="17" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="17" t="inlineStr">
         <is>
           <t>Subtotal — NYC / Long Island / NJ</t>
         </is>
       </c>
-      <c r="B59" s="17" t="inlineStr">
-        <is>
-          <t>24 item(s)</t>
-        </is>
-      </c>
-      <c r="C59" s="18" t="n"/>
-      <c r="D59" s="18" t="n"/>
-      <c r="E59" s="18" t="n"/>
-      <c r="F59" s="18" t="n"/>
-      <c r="G59" s="18" t="n"/>
-      <c r="H59" s="19" t="n">
+      <c r="B60" s="17" t="inlineStr">
+        <is>
+          <t>25 item(s)</t>
+        </is>
+      </c>
+      <c r="C60" s="18" t="n"/>
+      <c r="D60" s="18" t="n"/>
+      <c r="E60" s="18" t="n"/>
+      <c r="F60" s="18" t="n"/>
+      <c r="G60" s="18" t="n"/>
+      <c r="H60" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I59" s="18" t="n"/>
-      <c r="J59" s="18" t="n"/>
-      <c r="K59" s="18" t="n"/>
-      <c r="L59" s="18" t="n"/>
-      <c r="M59" s="18" t="n"/>
-      <c r="N59" s="18" t="n"/>
-      <c r="O59" s="18" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="11" t="inlineStr">
+      <c r="I60" s="18" t="n"/>
+      <c r="J60" s="18" t="n"/>
+      <c r="K60" s="18" t="n"/>
+      <c r="L60" s="18" t="n"/>
+      <c r="M60" s="18" t="n"/>
+      <c r="N60" s="18" t="n"/>
+      <c r="O60" s="18" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="11" t="inlineStr">
         <is>
           <t>▸ Eastern PA / Mid-Atlantic  (2)</t>
         </is>
       </c>
-      <c r="B60" s="12" t="n"/>
-      <c r="C60" s="12" t="n"/>
-      <c r="D60" s="12" t="n"/>
-      <c r="E60" s="12" t="n"/>
-      <c r="F60" s="12" t="n"/>
-      <c r="G60" s="12" t="n"/>
-      <c r="H60" s="12" t="n"/>
-      <c r="I60" s="12" t="n"/>
-      <c r="J60" s="12" t="n"/>
-      <c r="K60" s="12" t="n"/>
-      <c r="L60" s="12" t="n"/>
-      <c r="M60" s="12" t="n"/>
-      <c r="N60" s="12" t="n"/>
-      <c r="O60" s="12" t="n"/>
-    </row>
-    <row r="61" outlineLevel="1">
-      <c r="A61" s="13" t="inlineStr">
-        <is>
-          <t>Eastern PA / Mid-Atlantic</t>
-        </is>
-      </c>
-      <c r="B61" s="14" t="inlineStr">
-        <is>
-          <t>Piscitello's Home Center closing after 68 years: storewide 20% off liquidation (hardware, lumber, doors, windows, kitchen/bath)</t>
-        </is>
-      </c>
-      <c r="C61" s="13" t="inlineStr">
-        <is>
-          <t>store closing</t>
-        </is>
-      </c>
-      <c r="D61" s="13" t="inlineStr">
-        <is>
-          <t>Wilson</t>
-        </is>
-      </c>
-      <c r="E61" s="13" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="F61" s="13" t="n">
-        <v>250</v>
-      </c>
-      <c r="G61" s="13" t="inlineStr">
-        <is>
-          <t>20% off storewide (all sales final)</t>
-        </is>
-      </c>
-      <c r="H61" s="15" t="n"/>
-      <c r="I61" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="J61" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-30 06:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K61" s="13" t="inlineStr">
-        <is>
-          <t>LehighValley.com article</t>
-        </is>
-      </c>
-      <c r="L61" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M61" s="13" t="inlineStr"/>
-      <c r="N61" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O61" s="14" t="inlineStr">
-        <is>
-          <t>2300 Wood Ave, Wilson Borough (Easton area). Final day Oct 30. Retail-floor sale, not a bulk lot; ask in person about buying remaining stock outright.</t>
-        </is>
-      </c>
+      <c r="B61" s="12" t="n"/>
+      <c r="C61" s="12" t="n"/>
+      <c r="D61" s="12" t="n"/>
+      <c r="E61" s="12" t="n"/>
+      <c r="F61" s="12" t="n"/>
+      <c r="G61" s="12" t="n"/>
+      <c r="H61" s="12" t="n"/>
+      <c r="I61" s="12" t="n"/>
+      <c r="J61" s="12" t="n"/>
+      <c r="K61" s="12" t="n"/>
+      <c r="L61" s="12" t="n"/>
+      <c r="M61" s="12" t="n"/>
+      <c r="N61" s="12" t="n"/>
+      <c r="O61" s="12" t="n"/>
     </row>
     <row r="62" outlineLevel="1">
       <c r="A62" s="13" t="inlineStr">
@@ -21807,17 +21931,17 @@
       </c>
       <c r="B62" s="14" t="inlineStr">
         <is>
-          <t>October restaurant consignment – Hobart, Rational, True + NEW scratch-and-dent Migali/Avantco</t>
+          <t>Piscitello's Home Center closing after 68 years: storewide 20% off liquidation (hardware, lumber, doors, windows, kitchen/bath)</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D62" s="13" t="inlineStr">
         <is>
-          <t>Harrisburg</t>
+          <t>Wilson</t>
         </is>
       </c>
       <c r="E62" s="13" t="inlineStr">
@@ -21826,28 +21950,32 @@
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>340</v>
+        <v>250</v>
       </c>
       <c r="G62" s="13" t="inlineStr">
         <is>
-          <t>Online auction, 15% BP, ships $55/pallet</t>
+          <t>20% off storewide (all sales final)</t>
         </is>
       </c>
       <c r="H62" s="15" t="n"/>
-      <c r="I62" s="13" t="inlineStr"/>
+      <c r="I62" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
       <c r="J62" s="13" t="inlineStr">
         <is>
-          <t>2026-10-21 11:00 AM ET</t>
+          <t>2026-10-30 06:00 PM ET</t>
         </is>
       </c>
       <c r="K62" s="13" t="inlineStr">
         <is>
-          <t>Restaurant Auction Co</t>
-        </is>
-      </c>
-      <c r="L62" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>LehighValley.com article</t>
+        </is>
+      </c>
+      <c r="L62" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M62" s="13" t="inlineStr"/>
@@ -21858,124 +21986,120 @@
       </c>
       <c r="O62" s="14" t="inlineStr">
         <is>
+          <t>2300 Wood Ave, Wilson Borough (Easton area). Final day Oct 30. Retail-floor sale, not a bulk lot; ask in person about buying remaining stock outright.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" outlineLevel="1">
+      <c r="A63" s="13" t="inlineStr">
+        <is>
+          <t>Eastern PA / Mid-Atlantic</t>
+        </is>
+      </c>
+      <c r="B63" s="14" t="inlineStr">
+        <is>
+          <t>October restaurant consignment – Hobart, Rational, True + NEW scratch-and-dent Migali/Avantco</t>
+        </is>
+      </c>
+      <c r="C63" s="13" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D63" s="13" t="inlineStr">
+        <is>
+          <t>Harrisburg</t>
+        </is>
+      </c>
+      <c r="E63" s="13" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="F63" s="13" t="n">
+        <v>340</v>
+      </c>
+      <c r="G63" s="13" t="inlineStr">
+        <is>
+          <t>Online auction, 15% BP, ships $55/pallet</t>
+        </is>
+      </c>
+      <c r="H63" s="15" t="n"/>
+      <c r="I63" s="13" t="inlineStr"/>
+      <c r="J63" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-21 11:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K63" s="13" t="inlineStr">
+        <is>
+          <t>Restaurant Auction Co</t>
+        </is>
+      </c>
+      <c r="L63" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M63" s="13" t="inlineStr"/>
+      <c r="N63" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O63" s="14" t="inlineStr">
+        <is>
           <t>Closes Oct 21 10 or 11 AM (later used). Shippable.</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="17" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Eastern PA / Mid-Atlantic</t>
         </is>
       </c>
-      <c r="B63" s="17" t="inlineStr">
+      <c r="B64" s="17" t="inlineStr">
         <is>
           <t>2 item(s)</t>
         </is>
       </c>
-      <c r="C63" s="18" t="n"/>
-      <c r="D63" s="18" t="n"/>
-      <c r="E63" s="18" t="n"/>
-      <c r="F63" s="18" t="n"/>
-      <c r="G63" s="18" t="n"/>
-      <c r="H63" s="19" t="n">
+      <c r="C64" s="18" t="n"/>
+      <c r="D64" s="18" t="n"/>
+      <c r="E64" s="18" t="n"/>
+      <c r="F64" s="18" t="n"/>
+      <c r="G64" s="18" t="n"/>
+      <c r="H64" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I63" s="18" t="n"/>
-      <c r="J63" s="18" t="n"/>
-      <c r="K63" s="18" t="n"/>
-      <c r="L63" s="18" t="n"/>
-      <c r="M63" s="18" t="n"/>
-      <c r="N63" s="18" t="n"/>
-      <c r="O63" s="18" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="11" t="inlineStr">
+      <c r="I64" s="18" t="n"/>
+      <c r="J64" s="18" t="n"/>
+      <c r="K64" s="18" t="n"/>
+      <c r="L64" s="18" t="n"/>
+      <c r="M64" s="18" t="n"/>
+      <c r="N64" s="18" t="n"/>
+      <c r="O64" s="18" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="11" t="inlineStr">
         <is>
           <t>▸ Western PA / Ohio Valley  (3)</t>
         </is>
       </c>
-      <c r="B64" s="12" t="n"/>
-      <c r="C64" s="12" t="n"/>
-      <c r="D64" s="12" t="n"/>
-      <c r="E64" s="12" t="n"/>
-      <c r="F64" s="12" t="n"/>
-      <c r="G64" s="12" t="n"/>
-      <c r="H64" s="12" t="n"/>
-      <c r="I64" s="12" t="n"/>
-      <c r="J64" s="12" t="n"/>
-      <c r="K64" s="12" t="n"/>
-      <c r="L64" s="12" t="n"/>
-      <c r="M64" s="12" t="n"/>
-      <c r="N64" s="12" t="n"/>
-      <c r="O64" s="12" t="n"/>
-    </row>
-    <row r="65" outlineLevel="1">
-      <c r="A65" s="13" t="inlineStr">
-        <is>
-          <t>Western PA / Ohio Valley</t>
-        </is>
-      </c>
-      <c r="B65" s="14" t="inlineStr">
-        <is>
-          <t>Petrunak's Hardware Store liquidation Day 1 (530 lots: doors, hardware, tools, building supplies)</t>
-        </is>
-      </c>
-      <c r="C65" s="13" t="inlineStr">
-        <is>
-          <t>store closing auction</t>
-        </is>
-      </c>
-      <c r="D65" s="13" t="inlineStr">
-        <is>
-          <t>Windber</t>
-        </is>
-      </c>
-      <c r="E65" s="13" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="F65" s="13" t="n">
-        <v>437</v>
-      </c>
-      <c r="G65" s="13" t="inlineStr">
-        <is>
-          <t>Timed online auction (530 lots)</t>
-        </is>
-      </c>
-      <c r="H65" s="15" t="n"/>
-      <c r="I65" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="J65" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-21 08:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K65" s="13" t="inlineStr">
-        <is>
-          <t>Carey Auctions</t>
-        </is>
-      </c>
-      <c r="L65" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
-        </is>
-      </c>
-      <c r="M65" s="13" t="inlineStr"/>
-      <c r="N65" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O65" s="14" t="inlineStr">
-        <is>
-          <t>Ends Oct 21 7 PM CDT (8 PM ET). 1500 Somerset Ave, Windber PA. Pickups Oct 24-28. Hardware store, not appliance parts.</t>
-        </is>
-      </c>
+      <c r="B65" s="12" t="n"/>
+      <c r="C65" s="12" t="n"/>
+      <c r="D65" s="12" t="n"/>
+      <c r="E65" s="12" t="n"/>
+      <c r="F65" s="12" t="n"/>
+      <c r="G65" s="12" t="n"/>
+      <c r="H65" s="12" t="n"/>
+      <c r="I65" s="12" t="n"/>
+      <c r="J65" s="12" t="n"/>
+      <c r="K65" s="12" t="n"/>
+      <c r="L65" s="12" t="n"/>
+      <c r="M65" s="12" t="n"/>
+      <c r="N65" s="12" t="n"/>
+      <c r="O65" s="12" t="n"/>
     </row>
     <row r="66" outlineLevel="1">
       <c r="A66" s="13" t="inlineStr">
@@ -21985,7 +22109,7 @@
       </c>
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>Petrunak's Hardware Store liquidation Day 2 (433 lots)</t>
+          <t>Petrunak's Hardware Store liquidation Day 1 (530 lots: doors, hardware, tools, building supplies)</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
@@ -22008,7 +22132,7 @@
       </c>
       <c r="G66" s="13" t="inlineStr">
         <is>
-          <t>Timed online auction (433 lots)</t>
+          <t>Timed online auction (530 lots)</t>
         </is>
       </c>
       <c r="H66" s="15" t="n"/>
@@ -22019,7 +22143,7 @@
       </c>
       <c r="J66" s="13" t="inlineStr">
         <is>
-          <t>2026-10-22 08:00 PM ET</t>
+          <t>2026-10-21 08:00 PM ET</t>
         </is>
       </c>
       <c r="K66" s="13" t="inlineStr">
@@ -22040,7 +22164,7 @@
       </c>
       <c r="O66" s="14" t="inlineStr">
         <is>
-          <t>Ends Oct 22 7 PM CDT (8 PM ET). Same store as Day 1; pickups Oct 24-28.</t>
+          <t>Ends Oct 21 7 PM CDT (8 PM ET). 1500 Somerset Ave, Windber PA. Pickups Oct 24-28. Hardware store, not appliance parts.</t>
         </is>
       </c>
     </row>
@@ -22052,17 +22176,17 @@
       </c>
       <c r="B67" s="14" t="inlineStr">
         <is>
-          <t>Millers Pizza &amp; More – pizza business, commercial kitchen &amp; event space contents (362 lots)</t>
+          <t>Petrunak's Hardware Store liquidation Day 2 (433 lots)</t>
         </is>
       </c>
       <c r="C67" s="13" t="inlineStr">
         <is>
-          <t>restaurant / commercial kitchen contents</t>
+          <t>store closing auction</t>
         </is>
       </c>
       <c r="D67" s="13" t="inlineStr">
         <is>
-          <t>Everson</t>
+          <t>Windber</t>
         </is>
       </c>
       <c r="E67" s="13" t="inlineStr">
@@ -22071,28 +22195,32 @@
         </is>
       </c>
       <c r="F67" s="13" t="n">
-        <v>478</v>
+        <v>437</v>
       </c>
       <c r="G67" s="13" t="inlineStr">
         <is>
-          <t>Online auction, 15% buyer premium</t>
+          <t>Timed online auction (433 lots)</t>
         </is>
       </c>
       <c r="H67" s="15" t="n"/>
-      <c r="I67" s="13" t="inlineStr"/>
+      <c r="I67" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
       <c r="J67" s="13" t="inlineStr">
         <is>
-          <t>2026-10-25 07:00 PM ET</t>
+          <t>2026-10-22 08:00 PM ET</t>
         </is>
       </c>
       <c r="K67" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Bid Local LLC)</t>
-        </is>
-      </c>
-      <c r="L67" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>Carey Auctions</t>
+        </is>
+      </c>
+      <c r="L67" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M67" s="13" t="inlineStr"/>
@@ -22103,342 +22231,342 @@
       </c>
       <c r="O67" s="14" t="inlineStr">
         <is>
+          <t>Ends Oct 22 7 PM CDT (8 PM ET). Same store as Day 1; pickups Oct 24-28.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" outlineLevel="1">
+      <c r="A68" s="13" t="inlineStr">
+        <is>
+          <t>Western PA / Ohio Valley</t>
+        </is>
+      </c>
+      <c r="B68" s="14" t="inlineStr">
+        <is>
+          <t>Millers Pizza &amp; More – pizza business, commercial kitchen &amp; event space contents (362 lots)</t>
+        </is>
+      </c>
+      <c r="C68" s="13" t="inlineStr">
+        <is>
+          <t>restaurant / commercial kitchen contents</t>
+        </is>
+      </c>
+      <c r="D68" s="13" t="inlineStr">
+        <is>
+          <t>Everson</t>
+        </is>
+      </c>
+      <c r="E68" s="13" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="F68" s="13" t="n">
+        <v>478</v>
+      </c>
+      <c r="G68" s="13" t="inlineStr">
+        <is>
+          <t>Online auction, 15% buyer premium</t>
+        </is>
+      </c>
+      <c r="H68" s="15" t="n"/>
+      <c r="I68" s="13" t="inlineStr"/>
+      <c r="J68" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-25 07:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K68" s="13" t="inlineStr">
+        <is>
+          <t>HiBid (Bid Local LLC)</t>
+        </is>
+      </c>
+      <c r="L68" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M68" s="13" t="inlineStr"/>
+      <c r="N68" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O68" s="14" t="inlineStr">
+        <is>
           <t>Property of Millers Pizza and More LLC; online-only, 362 lots, lots begin closing Oct 25 7 PM. Pickup Everson PA by appointment Tue 10/27 and Wed 10/28. Building (4,500 sq ft) to be auctioned separately.</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="17" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Western PA / Ohio Valley</t>
         </is>
       </c>
-      <c r="B68" s="17" t="inlineStr">
+      <c r="B69" s="17" t="inlineStr">
         <is>
           <t>3 item(s)</t>
         </is>
       </c>
-      <c r="C68" s="18" t="n"/>
-      <c r="D68" s="18" t="n"/>
-      <c r="E68" s="18" t="n"/>
-      <c r="F68" s="18" t="n"/>
-      <c r="G68" s="18" t="n"/>
-      <c r="H68" s="19" t="n">
+      <c r="C69" s="18" t="n"/>
+      <c r="D69" s="18" t="n"/>
+      <c r="E69" s="18" t="n"/>
+      <c r="F69" s="18" t="n"/>
+      <c r="G69" s="18" t="n"/>
+      <c r="H69" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I68" s="18" t="n"/>
-      <c r="J68" s="18" t="n"/>
-      <c r="K68" s="18" t="n"/>
-      <c r="L68" s="18" t="n"/>
-      <c r="M68" s="18" t="n"/>
-      <c r="N68" s="18" t="n"/>
-      <c r="O68" s="18" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="11" t="inlineStr">
+      <c r="I69" s="18" t="n"/>
+      <c r="J69" s="18" t="n"/>
+      <c r="K69" s="18" t="n"/>
+      <c r="L69" s="18" t="n"/>
+      <c r="M69" s="18" t="n"/>
+      <c r="N69" s="18" t="n"/>
+      <c r="O69" s="18" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="inlineStr">
         <is>
           <t>▸ Upstate / Western NY  (1)</t>
         </is>
       </c>
-      <c r="B69" s="12" t="n"/>
-      <c r="C69" s="12" t="n"/>
-      <c r="D69" s="12" t="n"/>
-      <c r="E69" s="12" t="n"/>
-      <c r="F69" s="12" t="n"/>
-      <c r="G69" s="12" t="n"/>
-      <c r="H69" s="12" t="n"/>
-      <c r="I69" s="12" t="n"/>
-      <c r="J69" s="12" t="n"/>
-      <c r="K69" s="12" t="n"/>
-      <c r="L69" s="12" t="n"/>
-      <c r="M69" s="12" t="n"/>
-      <c r="N69" s="12" t="n"/>
-      <c r="O69" s="12" t="n"/>
-    </row>
-    <row r="70" outlineLevel="1">
-      <c r="A70" s="13" t="inlineStr">
+      <c r="B70" s="12" t="n"/>
+      <c r="C70" s="12" t="n"/>
+      <c r="D70" s="12" t="n"/>
+      <c r="E70" s="12" t="n"/>
+      <c r="F70" s="12" t="n"/>
+      <c r="G70" s="12" t="n"/>
+      <c r="H70" s="12" t="n"/>
+      <c r="I70" s="12" t="n"/>
+      <c r="J70" s="12" t="n"/>
+      <c r="K70" s="12" t="n"/>
+      <c r="L70" s="12" t="n"/>
+      <c r="M70" s="12" t="n"/>
+      <c r="N70" s="12" t="n"/>
+      <c r="O70" s="12" t="n"/>
+    </row>
+    <row r="71" outlineLevel="1">
+      <c r="A71" s="13" t="inlineStr">
         <is>
           <t>Upstate / Western NY</t>
         </is>
       </c>
-      <c r="B70" s="14" t="inlineStr">
+      <c r="B71" s="14" t="inlineStr">
         <is>
           <t>Restaurant &amp; fitness equipment</t>
         </is>
       </c>
-      <c r="C70" s="13" t="inlineStr">
+      <c r="C71" s="13" t="inlineStr">
         <is>
           <t>restaurant</t>
         </is>
       </c>
-      <c r="D70" s="13" t="inlineStr">
+      <c r="D71" s="13" t="inlineStr">
         <is>
           <t>Williamsville</t>
         </is>
       </c>
-      <c r="E70" s="13" t="inlineStr">
+      <c r="E71" s="13" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
       </c>
-      <c r="F70" s="13" t="n">
+      <c r="F71" s="13" t="n">
         <v>408</v>
       </c>
-      <c r="G70" s="13" t="inlineStr">
+      <c r="G71" s="13" t="inlineStr">
         <is>
           <t>Online auction</t>
         </is>
       </c>
-      <c r="H70" s="15" t="n"/>
-      <c r="I70" s="13" t="inlineStr"/>
-      <c r="J70" s="13" t="inlineStr">
+      <c r="H71" s="15" t="n"/>
+      <c r="I71" s="13" t="inlineStr"/>
+      <c r="J71" s="13" t="inlineStr">
         <is>
           <t>2026-10-26 07:30 PM ET</t>
         </is>
       </c>
-      <c r="K70" s="13" t="inlineStr">
+      <c r="K71" s="13" t="inlineStr">
         <is>
           <t>Cash Auctions</t>
         </is>
       </c>
-      <c r="L70" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M70" s="13" t="inlineStr"/>
-      <c r="N70" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O70" s="14" t="inlineStr">
+      <c r="L71" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M71" s="13" t="inlineStr"/>
+      <c r="N71" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O71" s="14" t="inlineStr">
         <is>
           <t>Lots not reviewed.</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="17" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Upstate / Western NY</t>
         </is>
       </c>
-      <c r="B71" s="17" t="inlineStr">
+      <c r="B72" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C71" s="18" t="n"/>
-      <c r="D71" s="18" t="n"/>
-      <c r="E71" s="18" t="n"/>
-      <c r="F71" s="18" t="n"/>
-      <c r="G71" s="18" t="n"/>
-      <c r="H71" s="19" t="n">
+      <c r="C72" s="18" t="n"/>
+      <c r="D72" s="18" t="n"/>
+      <c r="E72" s="18" t="n"/>
+      <c r="F72" s="18" t="n"/>
+      <c r="G72" s="18" t="n"/>
+      <c r="H72" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I71" s="18" t="n"/>
-      <c r="J71" s="18" t="n"/>
-      <c r="K71" s="18" t="n"/>
-      <c r="L71" s="18" t="n"/>
-      <c r="M71" s="18" t="n"/>
-      <c r="N71" s="18" t="n"/>
-      <c r="O71" s="18" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="11" t="inlineStr">
+      <c r="I72" s="18" t="n"/>
+      <c r="J72" s="18" t="n"/>
+      <c r="K72" s="18" t="n"/>
+      <c r="L72" s="18" t="n"/>
+      <c r="M72" s="18" t="n"/>
+      <c r="N72" s="18" t="n"/>
+      <c r="O72" s="18" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="11" t="inlineStr">
         <is>
           <t>▸ Virginia  (1)</t>
         </is>
       </c>
-      <c r="B72" s="12" t="n"/>
-      <c r="C72" s="12" t="n"/>
-      <c r="D72" s="12" t="n"/>
-      <c r="E72" s="12" t="n"/>
-      <c r="F72" s="12" t="n"/>
-      <c r="G72" s="12" t="n"/>
-      <c r="H72" s="12" t="n"/>
-      <c r="I72" s="12" t="n"/>
-      <c r="J72" s="12" t="n"/>
-      <c r="K72" s="12" t="n"/>
-      <c r="L72" s="12" t="n"/>
-      <c r="M72" s="12" t="n"/>
-      <c r="N72" s="12" t="n"/>
-      <c r="O72" s="12" t="n"/>
-    </row>
-    <row r="73" outlineLevel="1">
-      <c r="A73" s="13" t="inlineStr">
+      <c r="B73" s="12" t="n"/>
+      <c r="C73" s="12" t="n"/>
+      <c r="D73" s="12" t="n"/>
+      <c r="E73" s="12" t="n"/>
+      <c r="F73" s="12" t="n"/>
+      <c r="G73" s="12" t="n"/>
+      <c r="H73" s="12" t="n"/>
+      <c r="I73" s="12" t="n"/>
+      <c r="J73" s="12" t="n"/>
+      <c r="K73" s="12" t="n"/>
+      <c r="L73" s="12" t="n"/>
+      <c r="M73" s="12" t="n"/>
+      <c r="N73" s="12" t="n"/>
+      <c r="O73" s="12" t="n"/>
+    </row>
+    <row r="74" outlineLevel="1">
+      <c r="A74" s="13" t="inlineStr">
         <is>
           <t>Virginia</t>
         </is>
       </c>
-      <c r="B73" s="14" t="inlineStr">
+      <c r="B74" s="14" t="inlineStr">
         <is>
           <t>Haynes Furniture / The Dump – 12 stores closing (furniture, mattresses)</t>
         </is>
       </c>
-      <c r="C73" s="13" t="inlineStr">
+      <c r="C74" s="13" t="inlineStr">
         <is>
           <t>retail GOB</t>
         </is>
       </c>
-      <c r="D73" s="13" t="inlineStr">
+      <c r="D74" s="13" t="inlineStr">
         <is>
           <t>Virginia Beach</t>
         </is>
       </c>
-      <c r="E73" s="13" t="inlineStr">
+      <c r="E74" s="13" t="inlineStr">
         <is>
           <t>VA</t>
         </is>
       </c>
-      <c r="F73" s="13" t="n">
+      <c r="F74" s="13" t="n">
         <v>456</v>
       </c>
-      <c r="G73" s="13" t="inlineStr">
+      <c r="G74" s="13" t="inlineStr">
         <is>
           <t>Retail GOB markdowns</t>
         </is>
       </c>
-      <c r="H73" s="15" t="n"/>
-      <c r="I73" s="13" t="inlineStr">
+      <c r="H74" s="15" t="n"/>
+      <c r="I74" s="13" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>
       </c>
-      <c r="J73" s="13" t="inlineStr"/>
-      <c r="K73" s="13" t="inlineStr">
+      <c r="J74" s="13" t="inlineStr"/>
+      <c r="K74" s="13" t="inlineStr">
         <is>
           <t>SB360 (PR Newswire)</t>
         </is>
       </c>
-      <c r="L73" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M73" s="13" t="inlineStr"/>
-      <c r="N73" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O73" s="14" t="inlineStr">
+      <c r="L74" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M74" s="13" t="inlineStr"/>
+      <c r="N74" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O74" s="14" t="inlineStr">
         <is>
           <t>Posted Oct 8. Multi-state (VA/AZ/GA/IL/TX); pinned at Virginia Beach. Home goods only.</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="17" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Virginia</t>
         </is>
       </c>
-      <c r="B74" s="17" t="inlineStr">
+      <c r="B75" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C74" s="18" t="n"/>
-      <c r="D74" s="18" t="n"/>
-      <c r="E74" s="18" t="n"/>
-      <c r="F74" s="18" t="n"/>
-      <c r="G74" s="18" t="n"/>
-      <c r="H74" s="19" t="n">
+      <c r="C75" s="18" t="n"/>
+      <c r="D75" s="18" t="n"/>
+      <c r="E75" s="18" t="n"/>
+      <c r="F75" s="18" t="n"/>
+      <c r="G75" s="18" t="n"/>
+      <c r="H75" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I74" s="18" t="n"/>
-      <c r="J74" s="18" t="n"/>
-      <c r="K74" s="18" t="n"/>
-      <c r="L74" s="18" t="n"/>
-      <c r="M74" s="18" t="n"/>
-      <c r="N74" s="18" t="n"/>
-      <c r="O74" s="18" t="n"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="11" t="inlineStr">
-        <is>
-          <t>▸ Midwest  (2)</t>
-        </is>
-      </c>
-      <c r="B75" s="12" t="n"/>
-      <c r="C75" s="12" t="n"/>
-      <c r="D75" s="12" t="n"/>
-      <c r="E75" s="12" t="n"/>
-      <c r="F75" s="12" t="n"/>
-      <c r="G75" s="12" t="n"/>
-      <c r="H75" s="12" t="n"/>
-      <c r="I75" s="12" t="n"/>
-      <c r="J75" s="12" t="n"/>
-      <c r="K75" s="12" t="n"/>
-      <c r="L75" s="12" t="n"/>
-      <c r="M75" s="12" t="n"/>
-      <c r="N75" s="12" t="n"/>
-      <c r="O75" s="12" t="n"/>
-    </row>
-    <row r="76" outlineLevel="1">
-      <c r="A76" s="13" t="inlineStr">
-        <is>
-          <t>Midwest</t>
-        </is>
-      </c>
-      <c r="B76" s="14" t="inlineStr">
-        <is>
-          <t>American Sale – total liquidation, all 7 stores (pools, hot tubs, grills, holiday decor)</t>
-        </is>
-      </c>
-      <c r="C76" s="13" t="inlineStr">
-        <is>
-          <t>retail GOB</t>
-        </is>
-      </c>
-      <c r="D76" s="13" t="inlineStr">
-        <is>
-          <t>Chicagoland</t>
-        </is>
-      </c>
-      <c r="E76" s="13" t="inlineStr">
-        <is>
-          <t>IL</t>
-        </is>
-      </c>
-      <c r="F76" s="13" t="n">
-        <v>876</v>
-      </c>
-      <c r="G76" s="13" t="inlineStr">
-        <is>
-          <t>Retail GOB, up to 70% off</t>
-        </is>
-      </c>
-      <c r="H76" s="15" t="n"/>
-      <c r="I76" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="J76" s="13" t="inlineStr"/>
-      <c r="K76" s="13" t="inlineStr">
-        <is>
-          <t>Tiger Group (PR Newswire)</t>
-        </is>
-      </c>
-      <c r="L76" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M76" s="13" t="inlineStr"/>
-      <c r="N76" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O76" s="14" t="inlineStr">
-        <is>
-          <t>Posted Oct 15. Watch for a bulk/fixture auction.</t>
-        </is>
-      </c>
+      <c r="I75" s="18" t="n"/>
+      <c r="J75" s="18" t="n"/>
+      <c r="K75" s="18" t="n"/>
+      <c r="L75" s="18" t="n"/>
+      <c r="M75" s="18" t="n"/>
+      <c r="N75" s="18" t="n"/>
+      <c r="O75" s="18" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="11" t="inlineStr">
+        <is>
+          <t>▸ Midwest  (3)</t>
+        </is>
+      </c>
+      <c r="B76" s="12" t="n"/>
+      <c r="C76" s="12" t="n"/>
+      <c r="D76" s="12" t="n"/>
+      <c r="E76" s="12" t="n"/>
+      <c r="F76" s="12" t="n"/>
+      <c r="G76" s="12" t="n"/>
+      <c r="H76" s="12" t="n"/>
+      <c r="I76" s="12" t="n"/>
+      <c r="J76" s="12" t="n"/>
+      <c r="K76" s="12" t="n"/>
+      <c r="L76" s="12" t="n"/>
+      <c r="M76" s="12" t="n"/>
+      <c r="N76" s="12" t="n"/>
+      <c r="O76" s="12" t="n"/>
     </row>
     <row r="77" outlineLevel="1">
       <c r="A77" s="13" t="inlineStr">
@@ -22448,47 +22576,47 @@
       </c>
       <c r="B77" s="14" t="inlineStr">
         <is>
-          <t>Straub's Fine Foods store equipment – bakery, kitchen, meat room, Hussmann refrigeration</t>
+          <t>American Sale – total liquidation, all 7 stores (pools, hot tubs, grills, holiday decor)</t>
         </is>
       </c>
       <c r="C77" s="13" t="inlineStr">
         <is>
-          <t>grocery/restaurant</t>
+          <t>retail GOB</t>
         </is>
       </c>
       <c r="D77" s="13" t="inlineStr">
         <is>
-          <t>St. Louis</t>
+          <t>Chicagoland</t>
         </is>
       </c>
       <c r="E77" s="13" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="F77" s="13" t="n">
-        <v>1046</v>
+        <v>876</v>
       </c>
       <c r="G77" s="13" t="inlineStr">
         <is>
-          <t>Online auction (18% BP)</t>
+          <t>Retail GOB, up to 70% off</t>
         </is>
       </c>
       <c r="H77" s="15" t="n"/>
-      <c r="I77" s="13" t="inlineStr"/>
-      <c r="J77" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-21 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="I77" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="J77" s="13" t="inlineStr"/>
       <c r="K77" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
-        </is>
-      </c>
-      <c r="L77" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>Tiger Group (PR Newswire)</t>
+        </is>
+      </c>
+      <c r="L77" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M77" s="13" t="inlineStr"/>
@@ -22499,261 +22627,387 @@
       </c>
       <c r="O77" s="14" t="inlineStr">
         <is>
+          <t>Posted Oct 15. Watch for a bulk/fixture auction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" outlineLevel="1">
+      <c r="A78" s="13" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="B78" s="14" t="inlineStr">
+        <is>
+          <t>Straub's Fine Foods store equipment – bakery, kitchen, meat room, Hussmann refrigeration</t>
+        </is>
+      </c>
+      <c r="C78" s="13" t="inlineStr">
+        <is>
+          <t>grocery/restaurant</t>
+        </is>
+      </c>
+      <c r="D78" s="13" t="inlineStr">
+        <is>
+          <t>St. Louis</t>
+        </is>
+      </c>
+      <c r="E78" s="13" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="F78" s="13" t="n">
+        <v>1046</v>
+      </c>
+      <c r="G78" s="13" t="inlineStr">
+        <is>
+          <t>Online auction (18% BP)</t>
+        </is>
+      </c>
+      <c r="H78" s="15" t="n"/>
+      <c r="I78" s="13" t="inlineStr"/>
+      <c r="J78" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-21 11:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K78" s="13" t="inlineStr">
+        <is>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L78" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M78" s="13" t="inlineStr"/>
+      <c r="N78" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O78" s="14" t="inlineStr">
+        <is>
           <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis.</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="17" t="inlineStr">
+    <row r="79" outlineLevel="1">
+      <c r="A79" s="13" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="B79" s="14" t="inlineStr">
+        <is>
+          <t>Restaurant, Bar &amp; DJ Equipment Liquidation: Alto-Shaam combi, Southbend/Blodgett ovens, True refrigeration, Manitowoc, Hobart saw, DJ/AV gear</t>
+        </is>
+      </c>
+      <c r="C79" s="13" t="inlineStr">
+        <is>
+          <t>restaurant liquidation auction</t>
+        </is>
+      </c>
+      <c r="D79" s="13" t="inlineStr">
+        <is>
+          <t>Austin</t>
+        </is>
+      </c>
+      <c r="E79" s="13" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="F79" s="13" t="n">
+        <v>1124</v>
+      </c>
+      <c r="G79" s="13" t="inlineStr">
+        <is>
+          <t>Timed online auction</t>
+        </is>
+      </c>
+      <c r="H79" s="15" t="n"/>
+      <c r="I79" s="13" t="inlineStr"/>
+      <c r="J79" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-26 02:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K79" s="13" t="inlineStr">
+        <is>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L79" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M79" s="13" t="inlineStr"/>
+      <c r="N79" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O79" s="14" t="inlineStr">
+        <is>
+          <t>Begins closing Oct 26 1 PM CDT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Midwest</t>
         </is>
       </c>
-      <c r="B78" s="17" t="inlineStr">
-        <is>
-          <t>2 item(s)</t>
-        </is>
-      </c>
-      <c r="C78" s="18" t="n"/>
-      <c r="D78" s="18" t="n"/>
-      <c r="E78" s="18" t="n"/>
-      <c r="F78" s="18" t="n"/>
-      <c r="G78" s="18" t="n"/>
-      <c r="H78" s="19" t="n">
+      <c r="B80" s="17" t="inlineStr">
+        <is>
+          <t>3 item(s)</t>
+        </is>
+      </c>
+      <c r="C80" s="18" t="n"/>
+      <c r="D80" s="18" t="n"/>
+      <c r="E80" s="18" t="n"/>
+      <c r="F80" s="18" t="n"/>
+      <c r="G80" s="18" t="n"/>
+      <c r="H80" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I78" s="18" t="n"/>
-      <c r="J78" s="18" t="n"/>
-      <c r="K78" s="18" t="n"/>
-      <c r="L78" s="18" t="n"/>
-      <c r="M78" s="18" t="n"/>
-      <c r="N78" s="18" t="n"/>
-      <c r="O78" s="18" t="n"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="11" t="inlineStr">
+      <c r="I80" s="18" t="n"/>
+      <c r="J80" s="18" t="n"/>
+      <c r="K80" s="18" t="n"/>
+      <c r="L80" s="18" t="n"/>
+      <c r="M80" s="18" t="n"/>
+      <c r="N80" s="18" t="n"/>
+      <c r="O80" s="18" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="11" t="inlineStr">
         <is>
           <t>▸ Texas / South Central  (1)</t>
         </is>
       </c>
-      <c r="B79" s="12" t="n"/>
-      <c r="C79" s="12" t="n"/>
-      <c r="D79" s="12" t="n"/>
-      <c r="E79" s="12" t="n"/>
-      <c r="F79" s="12" t="n"/>
-      <c r="G79" s="12" t="n"/>
-      <c r="H79" s="12" t="n"/>
-      <c r="I79" s="12" t="n"/>
-      <c r="J79" s="12" t="n"/>
-      <c r="K79" s="12" t="n"/>
-      <c r="L79" s="12" t="n"/>
-      <c r="M79" s="12" t="n"/>
-      <c r="N79" s="12" t="n"/>
-      <c r="O79" s="12" t="n"/>
-    </row>
-    <row r="80" outlineLevel="1">
-      <c r="A80" s="13" t="inlineStr">
+      <c r="B81" s="12" t="n"/>
+      <c r="C81" s="12" t="n"/>
+      <c r="D81" s="12" t="n"/>
+      <c r="E81" s="12" t="n"/>
+      <c r="F81" s="12" t="n"/>
+      <c r="G81" s="12" t="n"/>
+      <c r="H81" s="12" t="n"/>
+      <c r="I81" s="12" t="n"/>
+      <c r="J81" s="12" t="n"/>
+      <c r="K81" s="12" t="n"/>
+      <c r="L81" s="12" t="n"/>
+      <c r="M81" s="12" t="n"/>
+      <c r="N81" s="12" t="n"/>
+      <c r="O81" s="12" t="n"/>
+    </row>
+    <row r="82" outlineLevel="1">
+      <c r="A82" s="13" t="inlineStr">
         <is>
           <t>Texas / South Central</t>
         </is>
       </c>
-      <c r="B80" s="14" t="inlineStr">
+      <c r="B82" s="14" t="inlineStr">
         <is>
           <t>Southwest beverage distributor surplus – mostly unused: 16 True merchandisers, 75 Bunn brewers, 100+ micro-market kiosks</t>
         </is>
       </c>
-      <c r="C80" s="13" t="inlineStr">
+      <c r="C82" s="13" t="inlineStr">
         <is>
           <t>distributor surplus</t>
         </is>
       </c>
-      <c r="D80" s="13" t="inlineStr">
+      <c r="D82" s="13" t="inlineStr">
         <is>
           <t>Mesquite</t>
         </is>
       </c>
-      <c r="E80" s="13" t="inlineStr">
+      <c r="E82" s="13" t="inlineStr">
         <is>
           <t>TX</t>
         </is>
       </c>
-      <c r="F80" s="13" t="n">
+      <c r="F82" s="13" t="n">
         <v>1547</v>
       </c>
-      <c r="G80" s="13" t="inlineStr">
+      <c r="G82" s="13" t="inlineStr">
         <is>
           <t>Online auction</t>
         </is>
       </c>
-      <c r="H80" s="15" t="n"/>
-      <c r="I80" s="13" t="inlineStr"/>
-      <c r="J80" s="13" t="inlineStr">
+      <c r="H82" s="15" t="n"/>
+      <c r="I82" s="13" t="inlineStr"/>
+      <c r="J82" s="13" t="inlineStr">
         <is>
           <t>2026-11-13 11:00 AM ET</t>
         </is>
       </c>
-      <c r="K80" s="13" t="inlineStr">
+      <c r="K82" s="13" t="inlineStr">
         <is>
           <t>Heritage Global Partners</t>
         </is>
       </c>
-      <c r="L80" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M80" s="13" t="inlineStr"/>
-      <c r="N80" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O80" s="14" t="inlineStr">
+      <c r="L82" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M82" s="13" t="inlineStr"/>
+      <c r="N82" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O82" s="14" t="inlineStr">
         <is>
           <t>Near-new appliances, resell by unit. Nov 13 10 AM CST.</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="17" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Texas / South Central</t>
         </is>
       </c>
-      <c r="B81" s="17" t="inlineStr">
+      <c r="B83" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C81" s="18" t="n"/>
-      <c r="D81" s="18" t="n"/>
-      <c r="E81" s="18" t="n"/>
-      <c r="F81" s="18" t="n"/>
-      <c r="G81" s="18" t="n"/>
-      <c r="H81" s="19" t="n">
+      <c r="C83" s="18" t="n"/>
+      <c r="D83" s="18" t="n"/>
+      <c r="E83" s="18" t="n"/>
+      <c r="F83" s="18" t="n"/>
+      <c r="G83" s="18" t="n"/>
+      <c r="H83" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I81" s="18" t="n"/>
-      <c r="J81" s="18" t="n"/>
-      <c r="K81" s="18" t="n"/>
-      <c r="L81" s="18" t="n"/>
-      <c r="M81" s="18" t="n"/>
-      <c r="N81" s="18" t="n"/>
-      <c r="O81" s="18" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="11" t="inlineStr">
+      <c r="I83" s="18" t="n"/>
+      <c r="J83" s="18" t="n"/>
+      <c r="K83" s="18" t="n"/>
+      <c r="L83" s="18" t="n"/>
+      <c r="M83" s="18" t="n"/>
+      <c r="N83" s="18" t="n"/>
+      <c r="O83" s="18" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="11" t="inlineStr">
         <is>
           <t>▸ West / Other  (1)</t>
         </is>
       </c>
-      <c r="B82" s="12" t="n"/>
-      <c r="C82" s="12" t="n"/>
-      <c r="D82" s="12" t="n"/>
-      <c r="E82" s="12" t="n"/>
-      <c r="F82" s="12" t="n"/>
-      <c r="G82" s="12" t="n"/>
-      <c r="H82" s="12" t="n"/>
-      <c r="I82" s="12" t="n"/>
-      <c r="J82" s="12" t="n"/>
-      <c r="K82" s="12" t="n"/>
-      <c r="L82" s="12" t="n"/>
-      <c r="M82" s="12" t="n"/>
-      <c r="N82" s="12" t="n"/>
-      <c r="O82" s="12" t="n"/>
-    </row>
-    <row r="83" outlineLevel="1">
-      <c r="A83" s="13" t="inlineStr">
+      <c r="B84" s="12" t="n"/>
+      <c r="C84" s="12" t="n"/>
+      <c r="D84" s="12" t="n"/>
+      <c r="E84" s="12" t="n"/>
+      <c r="F84" s="12" t="n"/>
+      <c r="G84" s="12" t="n"/>
+      <c r="H84" s="12" t="n"/>
+      <c r="I84" s="12" t="n"/>
+      <c r="J84" s="12" t="n"/>
+      <c r="K84" s="12" t="n"/>
+      <c r="L84" s="12" t="n"/>
+      <c r="M84" s="12" t="n"/>
+      <c r="N84" s="12" t="n"/>
+      <c r="O84" s="12" t="n"/>
+    </row>
+    <row r="85" outlineLevel="1">
+      <c r="A85" s="13" t="inlineStr">
         <is>
           <t>West / Other</t>
         </is>
       </c>
-      <c r="B83" s="14" t="inlineStr">
+      <c r="B85" s="14" t="inlineStr">
         <is>
           <t>National salad concept liquidation – full contents of 63 fast-casual restaurants (AZ/TX/OK/NV)</t>
         </is>
       </c>
-      <c r="C83" s="13" t="inlineStr">
+      <c r="C85" s="13" t="inlineStr">
         <is>
           <t>restaurant chain liquidation</t>
         </is>
       </c>
-      <c r="D83" s="13" t="inlineStr">
+      <c r="D85" s="13" t="inlineStr">
         <is>
           <t>Phoenix</t>
         </is>
       </c>
-      <c r="E83" s="13" t="inlineStr">
+      <c r="E85" s="13" t="inlineStr">
         <is>
           <t>AZ</t>
         </is>
       </c>
-      <c r="F83" s="13" t="n">
+      <c r="F85" s="13" t="n">
         <v>2307</v>
       </c>
-      <c r="G83" s="13" t="inlineStr">
+      <c r="G85" s="13" t="inlineStr">
         <is>
           <t>Online auctions, dates TBD</t>
         </is>
       </c>
-      <c r="H83" s="15" t="n"/>
-      <c r="I83" s="13" t="inlineStr">
+      <c r="H85" s="15" t="n"/>
+      <c r="I85" s="13" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="J83" s="13" t="inlineStr"/>
-      <c r="K83" s="13" t="inlineStr">
+      <c r="J85" s="13" t="inlineStr"/>
+      <c r="K85" s="13" t="inlineStr">
         <is>
           <t>RestaurantEquipment.bid (TAGeX)</t>
         </is>
       </c>
-      <c r="L83" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M83" s="13" t="inlineStr"/>
-      <c r="N83" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O83" s="14" t="inlineStr">
+      <c r="L85" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M85" s="13" t="inlineStr"/>
+      <c r="N85" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O85" s="14" t="inlineStr">
         <is>
           <t>Rolling market-by-market auctions, none live yet (Phoenix metro 30 locations, DFW 14, Tucson 6, Houston 5, plus OK/NV). Pickup on site at each restaurant. Pinned at Phoenix.</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="17" t="inlineStr">
+    <row r="86">
+      <c r="A86" s="17" t="inlineStr">
         <is>
           <t>Subtotal — West / Other</t>
         </is>
       </c>
-      <c r="B84" s="17" t="inlineStr">
+      <c r="B86" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C84" s="18" t="n"/>
-      <c r="D84" s="18" t="n"/>
-      <c r="E84" s="18" t="n"/>
-      <c r="F84" s="18" t="n"/>
-      <c r="G84" s="18" t="n"/>
-      <c r="H84" s="19" t="n">
+      <c r="C86" s="18" t="n"/>
+      <c r="D86" s="18" t="n"/>
+      <c r="E86" s="18" t="n"/>
+      <c r="F86" s="18" t="n"/>
+      <c r="G86" s="18" t="n"/>
+      <c r="H86" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I84" s="18" t="n"/>
-      <c r="J84" s="18" t="n"/>
-      <c r="K84" s="18" t="n"/>
-      <c r="L84" s="18" t="n"/>
-      <c r="M84" s="18" t="n"/>
-      <c r="N84" s="18" t="n"/>
-      <c r="O84" s="18" t="n"/>
+      <c r="I86" s="18" t="n"/>
+      <c r="J86" s="18" t="n"/>
+      <c r="K86" s="18" t="n"/>
+      <c r="L86" s="18" t="n"/>
+      <c r="M86" s="18" t="n"/>
+      <c r="N86" s="18" t="n"/>
+      <c r="O86" s="18" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O84"/>
+  <autoFilter ref="A1:O86"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId2"/>
@@ -22801,17 +23055,19 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N56" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N57" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N58" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N61" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N59" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N62" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N65" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N63" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N66" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N67" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N70" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N73" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N76" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N68" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N71" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N74" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N77" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N80" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N83" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N78" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N79" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N82" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N85" r:id="rId59"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -22985,7 +23241,7 @@
       </c>
       <c r="O2" s="14" t="inlineStr">
         <is>
-          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23048,7 +23304,7 @@
       </c>
       <c r="O3" s="14" t="inlineStr">
         <is>
-          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23249,7 +23505,7 @@
       </c>
       <c r="O6" s="14" t="inlineStr">
         <is>
-          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23314,7 +23570,7 @@
       </c>
       <c r="O7" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23379,7 +23635,7 @@
       </c>
       <c r="O8" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23444,7 +23700,7 @@
       </c>
       <c r="O9" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23507,7 +23763,7 @@
       </c>
       <c r="O10" s="14" t="inlineStr">
         <is>
-          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23570,7 +23826,7 @@
       </c>
       <c r="O11" s="14" t="inlineStr">
         <is>
-          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23633,7 +23889,7 @@
       </c>
       <c r="O12" s="14" t="inlineStr">
         <is>
-          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23696,7 +23952,7 @@
       </c>
       <c r="O13" s="14" t="inlineStr">
         <is>
-          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23759,7 +24015,7 @@
       </c>
       <c r="O14" s="14" t="inlineStr">
         <is>
-          <t>Small lot. [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Small lot. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23822,7 +24078,7 @@
       </c>
       <c r="O15" s="14" t="inlineStr">
         <is>
-          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23952,7 +24208,7 @@
       </c>
       <c r="O17" s="14" t="inlineStr">
         <is>
-          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24019,7 +24275,7 @@
       </c>
       <c r="O18" s="14" t="inlineStr">
         <is>
-          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24086,7 +24342,7 @@
       </c>
       <c r="O19" s="14" t="inlineStr">
         <is>
-          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed]</t>
+          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Watch update 2026-10-21 11am ET: no new finds, nothing removed; rechecked active listings
</commit_message>
<xml_diff>
--- a/lot_recon.xlsx
+++ b/lot_recon.xlsx
@@ -20,8 +20,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wolf New'!$A$1:$O$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Wolf Used'!$A$1:$O$189</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Wolf Unclear'!$A$1:$O$40</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$86</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 2026-10-21 08:05 ET</t>
+          <t>Last updated: 2026-10-21 11:02 ET</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Active listings: 298 · Removed: 18</t>
+          <t>Active listings: 294 · Removed: 22</t>
         </is>
       </c>
     </row>
@@ -708,13 +708,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="C13" s="7" t="n">
         <v>1275440.58</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C24" t="n">
         <v>1</v>
@@ -1037,7 +1037,7 @@
         <v>24</v>
       </c>
       <c r="G24" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H24" s="6" t="n">
         <v>440141</v>
@@ -1055,7 +1055,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C25" t="n">
         <v>1</v>
@@ -1070,7 +1070,7 @@
         <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H25" s="6" t="n">
         <v>1555</v>
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C30" t="n">
         <v>1</v>
@@ -1235,7 +1235,7 @@
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H30" s="6" t="n">
         <v>7</v>
@@ -18540,7 +18540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O86"/>
+  <dimension ref="A1:O82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -20274,7 +20274,7 @@
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>▸ NYC / Long Island / NJ  (25)</t>
+          <t>▸ NYC / Long Island / NJ  (23)</t>
         </is>
       </c>
       <c r="B34" s="12" t="n"/>
@@ -21245,17 +21245,17 @@
       </c>
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>Serpico's Pizzeria (lost lease) – Bari ovens, walk-in, Hobart 60qt, Vulcan range</t>
+          <t>Bimmer Clinic business liquidation (BMW repair shop): vehicle lifts, forklift, skid steer, refrigerant recovery, shop tools &amp; equipment</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>business liquidation auction</t>
         </is>
       </c>
       <c r="D50" s="13" t="inlineStr">
         <is>
-          <t>Allenhurst</t>
+          <t>South Amboy</t>
         </is>
       </c>
       <c r="E50" s="13" t="inlineStr">
@@ -21264,28 +21264,28 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>No-reserve online auction</t>
+          <t>Timed online auction</t>
         </is>
       </c>
       <c r="H50" s="15" t="n"/>
       <c r="I50" s="13" t="inlineStr"/>
       <c r="J50" s="13" t="inlineStr">
         <is>
-          <t>2026-10-21 11:00 AM ET</t>
+          <t>2026-11-12 11:00 AM ET</t>
         </is>
       </c>
       <c r="K50" s="13" t="inlineStr">
         <is>
-          <t>Peter Costanzo / EstateSales.net</t>
-        </is>
-      </c>
-      <c r="L50" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>AJ Willner Auctions</t>
+        </is>
+      </c>
+      <c r="L50" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M50" s="13" t="inlineStr"/>
@@ -21296,7 +21296,7 @@
       </c>
       <c r="O50" s="14" t="inlineStr">
         <is>
-          <t>Absolute / no reserve.</t>
+          <t>Ends Nov 12 11 AM EST.</t>
         </is>
       </c>
     </row>
@@ -21308,17 +21308,17 @@
       </c>
       <c r="B51" s="14" t="inlineStr">
         <is>
-          <t>Altitude Trampoline Park liquidation – partial: Atosa, TurboChef, stainless</t>
+          <t>New modular concession kitchens (warehouseman's lien) – 5 units, CaptiveAire hoods, new Ovention/Turbo Air</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
-          <t>facility contents</t>
+          <t>lien sale</t>
         </is>
       </c>
       <c r="D51" s="13" t="inlineStr">
         <is>
-          <t>Iselin</t>
+          <t>Edison</t>
         </is>
       </c>
       <c r="E51" s="13" t="inlineStr">
@@ -21327,28 +21327,24 @@
         </is>
       </c>
       <c r="F51" s="13" t="n">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="G51" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Online auction, $2K load-out fee</t>
         </is>
       </c>
       <c r="H51" s="15" t="n"/>
       <c r="I51" s="13" t="inlineStr"/>
-      <c r="J51" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-21 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="J51" s="13" t="inlineStr"/>
       <c r="K51" s="13" t="inlineStr">
         <is>
           <t>A.J. Willner</t>
         </is>
       </c>
-      <c r="L51" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+      <c r="L51" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M51" s="13" t="inlineStr"/>
@@ -21359,7 +21355,7 @@
       </c>
       <c r="O51" s="14" t="inlineStr">
         <is>
-          <t>Some kitchen gear only.</t>
+          <t>&gt;$100K new. Close date not captured.</t>
         </is>
       </c>
     </row>
@@ -21371,17 +21367,17 @@
       </c>
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>Bimmer Clinic business liquidation (BMW repair shop): vehicle lifts, forklift, skid steer, refrigerant recovery, shop tools &amp; equipment</t>
+          <t>Brand-new &amp; scratch-and-dent kitchen/home appliances – ~185 lots (Thermador, GE Café, Miele, Wolf speed oven, Viking, Bosch…)</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>business liquidation auction</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D52" s="13" t="inlineStr">
         <is>
-          <t>South Amboy</t>
+          <t>Edison</t>
         </is>
       </c>
       <c r="E52" s="13" t="inlineStr">
@@ -21390,23 +21386,27 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>Timed online auction</t>
+          <t>Live + HiBid webcast, 18% BP + 3% card</t>
         </is>
       </c>
       <c r="H52" s="15" t="n"/>
-      <c r="I52" s="13" t="inlineStr"/>
+      <c r="I52" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
       <c r="J52" s="13" t="inlineStr">
         <is>
-          <t>2026-11-12 11:00 AM ET</t>
+          <t>2026-10-25 01:00 PM ET</t>
         </is>
       </c>
       <c r="K52" s="13" t="inlineStr">
         <is>
-          <t>AJ Willner Auctions</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
       <c r="L52" s="13" t="inlineStr">
@@ -21414,7 +21414,11 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M52" s="13" t="inlineStr"/>
+      <c r="M52" s="21" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
       <c r="N52" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -21422,7 +21426,7 @@
       </c>
       <c r="O52" s="14" t="inlineStr">
         <is>
-          <t>Ends Nov 12 11 AM EST.</t>
+          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale.</t>
         </is>
       </c>
     </row>
@@ -21434,17 +21438,17 @@
       </c>
       <c r="B53" s="14" t="inlineStr">
         <is>
-          <t>New modular concession kitchens (warehouseman's lien) – 5 units, CaptiveAire hoods, new Ovention/Turbo Air</t>
+          <t>Party City (Ch. 11) store – fixtures + party merchandise inventory</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>lien sale</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D53" s="13" t="inlineStr">
         <is>
-          <t>Edison</t>
+          <t>East Brunswick</t>
         </is>
       </c>
       <c r="E53" s="13" t="inlineStr">
@@ -21453,16 +21457,20 @@
         </is>
       </c>
       <c r="F53" s="13" t="n">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="G53" s="13" t="inlineStr">
         <is>
-          <t>Online auction, $2K load-out fee</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H53" s="15" t="n"/>
       <c r="I53" s="13" t="inlineStr"/>
-      <c r="J53" s="13" t="inlineStr"/>
+      <c r="J53" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-03 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K53" s="13" t="inlineStr">
         <is>
           <t>A.J. Willner</t>
@@ -21481,7 +21489,7 @@
       </c>
       <c r="O53" s="14" t="inlineStr">
         <is>
-          <t>&gt;$100K new. Close date not captured.</t>
+          <t>Store inventory.</t>
         </is>
       </c>
     </row>
@@ -21493,17 +21501,17 @@
       </c>
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>Brand-new &amp; scratch-and-dent kitchen/home appliances – ~185 lots (Thermador, GE Café, Miele, Wolf speed oven, Viking, Bosch…)</t>
+          <t>Bakery/Cafe Somerville NJ – rack ovens, La Marzocco, food truck (~76 lots)</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D54" s="13" t="inlineStr">
         <is>
-          <t>Edison</t>
+          <t>Somerville</t>
         </is>
       </c>
       <c r="E54" s="13" t="inlineStr">
@@ -21512,27 +21520,27 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>Live + HiBid webcast, 18% BP + 3% card</t>
+          <t>Live webcast + online (18% BP online)</t>
         </is>
       </c>
       <c r="H54" s="15" t="n"/>
       <c r="I54" s="13" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="J54" s="13" t="inlineStr">
         <is>
-          <t>2026-10-25 01:00 PM ET</t>
+          <t>2026-10-26 02:00 PM ET</t>
         </is>
       </c>
       <c r="K54" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>HiBid / Best Buy Auctioneers</t>
         </is>
       </c>
       <c r="L54" s="13" t="inlineStr">
@@ -21540,11 +21548,7 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M54" s="21" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
+      <c r="M54" s="13" t="inlineStr"/>
       <c r="N54" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -21552,7 +21556,7 @@
       </c>
       <c r="O54" s="14" t="inlineStr">
         <is>
-          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale.</t>
+          <t>Full bakery/cafe commercial kitchen: food truck w/ pizza oven, La Marzocco espresso, Mazzer, Baxter + Empire Logiudice rack ovens, dough depositor, Globe floor mixer, Artic Air / SS refrigeration, fryers, Vitamix, Robot Coupe, display cases, dining furniture. Preview 11 AM sale day; checkout Tue 10/27.</t>
         </is>
       </c>
     </row>
@@ -21564,17 +21568,17 @@
       </c>
       <c r="B55" s="14" t="inlineStr">
         <is>
-          <t>Party City (Ch. 11) store – fixtures + party merchandise inventory</t>
+          <t>Ability to Work kitchen and store – commercial kitchen + store fixtures (~135 lots)</t>
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D55" s="13" t="inlineStr">
         <is>
-          <t>East Brunswick</t>
+          <t>Flemington</t>
         </is>
       </c>
       <c r="E55" s="13" t="inlineStr">
@@ -21583,23 +21587,23 @@
         </is>
       </c>
       <c r="F55" s="13" t="n">
-        <v>220</v>
+        <v>237</v>
       </c>
       <c r="G55" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Timed online (15% BP)</t>
         </is>
       </c>
       <c r="H55" s="15" t="n"/>
       <c r="I55" s="13" t="inlineStr"/>
       <c r="J55" s="13" t="inlineStr">
         <is>
-          <t>2026-11-03 11:00 AM ET</t>
+          <t>2026-10-27 11:02 AM ET</t>
         </is>
       </c>
       <c r="K55" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
+          <t>HiBid</t>
         </is>
       </c>
       <c r="L55" s="13" t="inlineStr">
@@ -21615,7 +21619,7 @@
       </c>
       <c r="O55" s="14" t="inlineStr">
         <is>
-          <t>Store inventory.</t>
+          <t>Apprentice/hospitality training cafe-kitchen and store dispersal. Preview 9–11 AM sale day; removal Oct 27 noon–Oct 29.</t>
         </is>
       </c>
     </row>
@@ -21627,17 +21631,17 @@
       </c>
       <c r="B56" s="14" t="inlineStr">
         <is>
-          <t>Bakery/Cafe Somerville NJ – rack ovens, La Marzocco, food truck (~76 lots)</t>
+          <t>Wren Kitchens showroom closing – JennAir/Café/KitchenAid/GE Profile appliances + display kitchens</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>showroom closing</t>
         </is>
       </c>
       <c r="D56" s="13" t="inlineStr">
         <is>
-          <t>Somerville</t>
+          <t>Lawrenceville</t>
         </is>
       </c>
       <c r="E56" s="13" t="inlineStr">
@@ -21646,27 +21650,23 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>224</v>
+        <v>239</v>
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>Live webcast + online (18% BP online)</t>
+          <t>Online auction, 18% BP</t>
         </is>
       </c>
       <c r="H56" s="15" t="n"/>
-      <c r="I56" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
+      <c r="I56" s="13" t="inlineStr"/>
       <c r="J56" s="13" t="inlineStr">
         <is>
-          <t>2026-10-26 02:00 PM ET</t>
+          <t>2026-10-27 09:00 AM ET</t>
         </is>
       </c>
       <c r="K56" s="13" t="inlineStr">
         <is>
-          <t>HiBid / Best Buy Auctioneers</t>
+          <t>Grafe Auction</t>
         </is>
       </c>
       <c r="L56" s="13" t="inlineStr">
@@ -21682,7 +21682,7 @@
       </c>
       <c r="O56" s="14" t="inlineStr">
         <is>
-          <t>Full bakery/cafe commercial kitchen: food truck w/ pizza oven, La Marzocco espresso, Mazzer, Baxter + Empire Logiudice rack ovens, dough depositor, Globe floor mixer, Artic Air / SS refrigeration, fryers, Vitamix, Robot Coupe, display cases, dining furniture. Preview 11 AM sale day; checkout Tue 10/27.</t>
+          <t>Premium floor-model appliances; lots close from Oct 27 9 AM.</t>
         </is>
       </c>
     </row>
@@ -21694,17 +21694,17 @@
       </c>
       <c r="B57" s="14" t="inlineStr">
         <is>
-          <t>Ability to Work kitchen and store – commercial kitchen + store fixtures (~135 lots)</t>
+          <t>Wren Kitchens showroom closing – GE/Whirlpool/KitchenAid/Café incl. NIB Café range + 35 kitchens</t>
         </is>
       </c>
       <c r="C57" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>showroom closing</t>
         </is>
       </c>
       <c r="D57" s="13" t="inlineStr">
         <is>
-          <t>Flemington</t>
+          <t>Cherry Hill</t>
         </is>
       </c>
       <c r="E57" s="13" t="inlineStr">
@@ -21713,23 +21713,23 @@
         </is>
       </c>
       <c r="F57" s="13" t="n">
-        <v>237</v>
+        <v>266</v>
       </c>
       <c r="G57" s="13" t="inlineStr">
         <is>
-          <t>Timed online (15% BP)</t>
+          <t>Online auction, openers ~$0.50</t>
         </is>
       </c>
       <c r="H57" s="15" t="n"/>
       <c r="I57" s="13" t="inlineStr"/>
       <c r="J57" s="13" t="inlineStr">
         <is>
-          <t>2026-10-27 11:02 AM ET</t>
+          <t>2026-11-02 11:00 AM ET</t>
         </is>
       </c>
       <c r="K57" s="13" t="inlineStr">
         <is>
-          <t>HiBid</t>
+          <t>Grafe Auction</t>
         </is>
       </c>
       <c r="L57" s="13" t="inlineStr">
@@ -21745,270 +21745,192 @@
       </c>
       <c r="O57" s="14" t="inlineStr">
         <is>
-          <t>Apprentice/hospitality training cafe-kitchen and store dispersal. Preview 9–11 AM sale day; removal Oct 27 noon–Oct 29.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" outlineLevel="1">
-      <c r="A58" s="13" t="inlineStr">
-        <is>
-          <t>NYC / Long Island / NJ</t>
-        </is>
-      </c>
-      <c r="B58" s="14" t="inlineStr">
-        <is>
-          <t>Wren Kitchens showroom closing – JennAir/Café/KitchenAid/GE Profile appliances + display kitchens</t>
-        </is>
-      </c>
-      <c r="C58" s="13" t="inlineStr">
-        <is>
-          <t>showroom closing</t>
-        </is>
-      </c>
-      <c r="D58" s="13" t="inlineStr">
-        <is>
-          <t>Lawrenceville</t>
-        </is>
-      </c>
-      <c r="E58" s="13" t="inlineStr">
-        <is>
-          <t>NJ</t>
-        </is>
-      </c>
-      <c r="F58" s="13" t="n">
-        <v>239</v>
-      </c>
-      <c r="G58" s="13" t="inlineStr">
-        <is>
-          <t>Online auction, 18% BP</t>
-        </is>
-      </c>
-      <c r="H58" s="15" t="n"/>
-      <c r="I58" s="13" t="inlineStr"/>
-      <c r="J58" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-27 09:00 AM ET</t>
-        </is>
-      </c>
-      <c r="K58" s="13" t="inlineStr">
-        <is>
-          <t>Grafe Auction</t>
-        </is>
-      </c>
-      <c r="L58" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M58" s="13" t="inlineStr"/>
-      <c r="N58" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O58" s="14" t="inlineStr">
-        <is>
-          <t>Premium floor-model appliances; lots close from Oct 27 9 AM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" outlineLevel="1">
-      <c r="A59" s="13" t="inlineStr">
-        <is>
-          <t>NYC / Long Island / NJ</t>
-        </is>
-      </c>
-      <c r="B59" s="14" t="inlineStr">
-        <is>
-          <t>Wren Kitchens showroom closing – GE/Whirlpool/KitchenAid/Café incl. NIB Café range + 35 kitchens</t>
-        </is>
-      </c>
-      <c r="C59" s="13" t="inlineStr">
-        <is>
-          <t>showroom closing</t>
-        </is>
-      </c>
-      <c r="D59" s="13" t="inlineStr">
-        <is>
-          <t>Cherry Hill</t>
-        </is>
-      </c>
-      <c r="E59" s="13" t="inlineStr">
-        <is>
-          <t>NJ</t>
-        </is>
-      </c>
-      <c r="F59" s="13" t="n">
-        <v>266</v>
-      </c>
-      <c r="G59" s="13" t="inlineStr">
-        <is>
-          <t>Online auction, openers ~$0.50</t>
-        </is>
-      </c>
-      <c r="H59" s="15" t="n"/>
-      <c r="I59" s="13" t="inlineStr"/>
-      <c r="J59" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-02 11:00 AM ET</t>
-        </is>
-      </c>
-      <c r="K59" s="13" t="inlineStr">
-        <is>
-          <t>Grafe Auction</t>
-        </is>
-      </c>
-      <c r="L59" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M59" s="13" t="inlineStr"/>
-      <c r="N59" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O59" s="14" t="inlineStr">
-        <is>
           <t>Lots close from Nov 2 11 AM.</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="17" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="17" t="inlineStr">
         <is>
           <t>Subtotal — NYC / Long Island / NJ</t>
         </is>
       </c>
-      <c r="B60" s="17" t="inlineStr">
-        <is>
-          <t>25 item(s)</t>
-        </is>
-      </c>
-      <c r="C60" s="18" t="n"/>
-      <c r="D60" s="18" t="n"/>
-      <c r="E60" s="18" t="n"/>
-      <c r="F60" s="18" t="n"/>
-      <c r="G60" s="18" t="n"/>
-      <c r="H60" s="19" t="n">
+      <c r="B58" s="17" t="inlineStr">
+        <is>
+          <t>23 item(s)</t>
+        </is>
+      </c>
+      <c r="C58" s="18" t="n"/>
+      <c r="D58" s="18" t="n"/>
+      <c r="E58" s="18" t="n"/>
+      <c r="F58" s="18" t="n"/>
+      <c r="G58" s="18" t="n"/>
+      <c r="H58" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I60" s="18" t="n"/>
-      <c r="J60" s="18" t="n"/>
-      <c r="K60" s="18" t="n"/>
-      <c r="L60" s="18" t="n"/>
-      <c r="M60" s="18" t="n"/>
-      <c r="N60" s="18" t="n"/>
-      <c r="O60" s="18" t="n"/>
+      <c r="I58" s="18" t="n"/>
+      <c r="J58" s="18" t="n"/>
+      <c r="K58" s="18" t="n"/>
+      <c r="L58" s="18" t="n"/>
+      <c r="M58" s="18" t="n"/>
+      <c r="N58" s="18" t="n"/>
+      <c r="O58" s="18" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="11" t="inlineStr">
+        <is>
+          <t>▸ Eastern PA / Mid-Atlantic  (1)</t>
+        </is>
+      </c>
+      <c r="B59" s="12" t="n"/>
+      <c r="C59" s="12" t="n"/>
+      <c r="D59" s="12" t="n"/>
+      <c r="E59" s="12" t="n"/>
+      <c r="F59" s="12" t="n"/>
+      <c r="G59" s="12" t="n"/>
+      <c r="H59" s="12" t="n"/>
+      <c r="I59" s="12" t="n"/>
+      <c r="J59" s="12" t="n"/>
+      <c r="K59" s="12" t="n"/>
+      <c r="L59" s="12" t="n"/>
+      <c r="M59" s="12" t="n"/>
+      <c r="N59" s="12" t="n"/>
+      <c r="O59" s="12" t="n"/>
+    </row>
+    <row r="60" outlineLevel="1">
+      <c r="A60" s="13" t="inlineStr">
+        <is>
+          <t>Eastern PA / Mid-Atlantic</t>
+        </is>
+      </c>
+      <c r="B60" s="14" t="inlineStr">
+        <is>
+          <t>Piscitello's Home Center closing after 68 years: storewide 20% off liquidation (hardware, lumber, doors, windows, kitchen/bath)</t>
+        </is>
+      </c>
+      <c r="C60" s="13" t="inlineStr">
+        <is>
+          <t>store closing</t>
+        </is>
+      </c>
+      <c r="D60" s="13" t="inlineStr">
+        <is>
+          <t>Wilson</t>
+        </is>
+      </c>
+      <c r="E60" s="13" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="F60" s="13" t="n">
+        <v>250</v>
+      </c>
+      <c r="G60" s="13" t="inlineStr">
+        <is>
+          <t>20% off storewide (all sales final)</t>
+        </is>
+      </c>
+      <c r="H60" s="15" t="n"/>
+      <c r="I60" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="J60" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-30 06:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K60" s="13" t="inlineStr">
+        <is>
+          <t>LehighValley.com article</t>
+        </is>
+      </c>
+      <c r="L60" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M60" s="13" t="inlineStr"/>
+      <c r="N60" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O60" s="14" t="inlineStr">
+        <is>
+          <t>2300 Wood Ave, Wilson Borough (Easton area). Final day Oct 30. Retail-floor sale, not a bulk lot; ask in person about buying remaining stock outright.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
-      <c r="A61" s="11" t="inlineStr">
-        <is>
-          <t>▸ Eastern PA / Mid-Atlantic  (2)</t>
-        </is>
-      </c>
-      <c r="B61" s="12" t="n"/>
-      <c r="C61" s="12" t="n"/>
-      <c r="D61" s="12" t="n"/>
-      <c r="E61" s="12" t="n"/>
-      <c r="F61" s="12" t="n"/>
-      <c r="G61" s="12" t="n"/>
-      <c r="H61" s="12" t="n"/>
-      <c r="I61" s="12" t="n"/>
-      <c r="J61" s="12" t="n"/>
-      <c r="K61" s="12" t="n"/>
-      <c r="L61" s="12" t="n"/>
-      <c r="M61" s="12" t="n"/>
-      <c r="N61" s="12" t="n"/>
-      <c r="O61" s="12" t="n"/>
-    </row>
-    <row r="62" outlineLevel="1">
-      <c r="A62" s="13" t="inlineStr">
-        <is>
-          <t>Eastern PA / Mid-Atlantic</t>
-        </is>
-      </c>
-      <c r="B62" s="14" t="inlineStr">
-        <is>
-          <t>Piscitello's Home Center closing after 68 years: storewide 20% off liquidation (hardware, lumber, doors, windows, kitchen/bath)</t>
-        </is>
-      </c>
-      <c r="C62" s="13" t="inlineStr">
-        <is>
-          <t>store closing</t>
-        </is>
-      </c>
-      <c r="D62" s="13" t="inlineStr">
-        <is>
-          <t>Wilson</t>
-        </is>
-      </c>
-      <c r="E62" s="13" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="F62" s="13" t="n">
-        <v>250</v>
-      </c>
-      <c r="G62" s="13" t="inlineStr">
-        <is>
-          <t>20% off storewide (all sales final)</t>
-        </is>
-      </c>
-      <c r="H62" s="15" t="n"/>
-      <c r="I62" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="J62" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-30 06:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K62" s="13" t="inlineStr">
-        <is>
-          <t>LehighValley.com article</t>
-        </is>
-      </c>
-      <c r="L62" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M62" s="13" t="inlineStr"/>
-      <c r="N62" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O62" s="14" t="inlineStr">
-        <is>
-          <t>2300 Wood Ave, Wilson Borough (Easton area). Final day Oct 30. Retail-floor sale, not a bulk lot; ask in person about buying remaining stock outright.</t>
-        </is>
-      </c>
+      <c r="A61" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Eastern PA / Mid-Atlantic</t>
+        </is>
+      </c>
+      <c r="B61" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C61" s="18" t="n"/>
+      <c r="D61" s="18" t="n"/>
+      <c r="E61" s="18" t="n"/>
+      <c r="F61" s="18" t="n"/>
+      <c r="G61" s="18" t="n"/>
+      <c r="H61" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" s="18" t="n"/>
+      <c r="J61" s="18" t="n"/>
+      <c r="K61" s="18" t="n"/>
+      <c r="L61" s="18" t="n"/>
+      <c r="M61" s="18" t="n"/>
+      <c r="N61" s="18" t="n"/>
+      <c r="O61" s="18" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
+          <t>▸ Western PA / Ohio Valley  (3)</t>
+        </is>
+      </c>
+      <c r="B62" s="12" t="n"/>
+      <c r="C62" s="12" t="n"/>
+      <c r="D62" s="12" t="n"/>
+      <c r="E62" s="12" t="n"/>
+      <c r="F62" s="12" t="n"/>
+      <c r="G62" s="12" t="n"/>
+      <c r="H62" s="12" t="n"/>
+      <c r="I62" s="12" t="n"/>
+      <c r="J62" s="12" t="n"/>
+      <c r="K62" s="12" t="n"/>
+      <c r="L62" s="12" t="n"/>
+      <c r="M62" s="12" t="n"/>
+      <c r="N62" s="12" t="n"/>
+      <c r="O62" s="12" t="n"/>
     </row>
     <row r="63" outlineLevel="1">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>Eastern PA / Mid-Atlantic</t>
+          <t>Western PA / Ohio Valley</t>
         </is>
       </c>
       <c r="B63" s="14" t="inlineStr">
         <is>
-          <t>October restaurant consignment – Hobart, Rational, True + NEW scratch-and-dent Migali/Avantco</t>
+          <t>Petrunak's Hardware Store liquidation Day 1 (530 lots: doors, hardware, tools, building supplies)</t>
         </is>
       </c>
       <c r="C63" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>store closing auction</t>
         </is>
       </c>
       <c r="D63" s="13" t="inlineStr">
         <is>
-          <t>Harrisburg</t>
+          <t>Windber</t>
         </is>
       </c>
       <c r="E63" s="13" t="inlineStr">
@@ -22017,23 +21939,27 @@
         </is>
       </c>
       <c r="F63" s="13" t="n">
-        <v>340</v>
+        <v>437</v>
       </c>
       <c r="G63" s="13" t="inlineStr">
         <is>
-          <t>Online auction, 15% BP, ships $55/pallet</t>
+          <t>Timed online auction (530 lots)</t>
         </is>
       </c>
       <c r="H63" s="15" t="n"/>
-      <c r="I63" s="13" t="inlineStr"/>
+      <c r="I63" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
       <c r="J63" s="13" t="inlineStr">
         <is>
-          <t>2026-10-21 11:00 AM ET</t>
+          <t>2026-10-21 08:00 PM ET</t>
         </is>
       </c>
       <c r="K63" s="13" t="inlineStr">
         <is>
-          <t>Restaurant Auction Co</t>
+          <t>Carey Auctions</t>
         </is>
       </c>
       <c r="L63" s="20" t="inlineStr">
@@ -22049,236 +21975,232 @@
       </c>
       <c r="O63" s="14" t="inlineStr">
         <is>
-          <t>Closes Oct 21 10 or 11 AM (later used). Shippable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Eastern PA / Mid-Atlantic</t>
-        </is>
-      </c>
-      <c r="B64" s="17" t="inlineStr">
-        <is>
-          <t>2 item(s)</t>
-        </is>
-      </c>
-      <c r="C64" s="18" t="n"/>
-      <c r="D64" s="18" t="n"/>
-      <c r="E64" s="18" t="n"/>
-      <c r="F64" s="18" t="n"/>
-      <c r="G64" s="18" t="n"/>
-      <c r="H64" s="19" t="n">
+          <t>Ends Oct 21 7 PM CDT (8 PM ET). 1500 Somerset Ave, Windber PA. Pickups Oct 24-28. Hardware store, not appliance parts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" outlineLevel="1">
+      <c r="A64" s="13" t="inlineStr">
+        <is>
+          <t>Western PA / Ohio Valley</t>
+        </is>
+      </c>
+      <c r="B64" s="14" t="inlineStr">
+        <is>
+          <t>Petrunak's Hardware Store liquidation Day 2 (433 lots)</t>
+        </is>
+      </c>
+      <c r="C64" s="13" t="inlineStr">
+        <is>
+          <t>store closing auction</t>
+        </is>
+      </c>
+      <c r="D64" s="13" t="inlineStr">
+        <is>
+          <t>Windber</t>
+        </is>
+      </c>
+      <c r="E64" s="13" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="F64" s="13" t="n">
+        <v>437</v>
+      </c>
+      <c r="G64" s="13" t="inlineStr">
+        <is>
+          <t>Timed online auction (433 lots)</t>
+        </is>
+      </c>
+      <c r="H64" s="15" t="n"/>
+      <c r="I64" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="J64" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K64" s="13" t="inlineStr">
+        <is>
+          <t>Carey Auctions</t>
+        </is>
+      </c>
+      <c r="L64" s="20" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M64" s="13" t="inlineStr"/>
+      <c r="N64" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O64" s="14" t="inlineStr">
+        <is>
+          <t>Ends Oct 22 7 PM CDT (8 PM ET). Same store as Day 1; pickups Oct 24-28.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" outlineLevel="1">
+      <c r="A65" s="13" t="inlineStr">
+        <is>
+          <t>Western PA / Ohio Valley</t>
+        </is>
+      </c>
+      <c r="B65" s="14" t="inlineStr">
+        <is>
+          <t>Millers Pizza &amp; More – pizza business, commercial kitchen &amp; event space contents (362 lots)</t>
+        </is>
+      </c>
+      <c r="C65" s="13" t="inlineStr">
+        <is>
+          <t>restaurant / commercial kitchen contents</t>
+        </is>
+      </c>
+      <c r="D65" s="13" t="inlineStr">
+        <is>
+          <t>Everson</t>
+        </is>
+      </c>
+      <c r="E65" s="13" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="F65" s="13" t="n">
+        <v>478</v>
+      </c>
+      <c r="G65" s="13" t="inlineStr">
+        <is>
+          <t>Online auction, 15% buyer premium</t>
+        </is>
+      </c>
+      <c r="H65" s="15" t="n"/>
+      <c r="I65" s="13" t="inlineStr"/>
+      <c r="J65" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-25 07:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K65" s="13" t="inlineStr">
+        <is>
+          <t>HiBid (Bid Local LLC)</t>
+        </is>
+      </c>
+      <c r="L65" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M65" s="13" t="inlineStr"/>
+      <c r="N65" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O65" s="14" t="inlineStr">
+        <is>
+          <t>Property of Millers Pizza and More LLC; online-only, 362 lots, lots begin closing Oct 25 7 PM. Pickup Everson PA by appointment Tue 10/27 and Wed 10/28. Building (4,500 sq ft) to be auctioned separately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Western PA / Ohio Valley</t>
+        </is>
+      </c>
+      <c r="B66" s="17" t="inlineStr">
+        <is>
+          <t>3 item(s)</t>
+        </is>
+      </c>
+      <c r="C66" s="18" t="n"/>
+      <c r="D66" s="18" t="n"/>
+      <c r="E66" s="18" t="n"/>
+      <c r="F66" s="18" t="n"/>
+      <c r="G66" s="18" t="n"/>
+      <c r="H66" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I64" s="18" t="n"/>
-      <c r="J64" s="18" t="n"/>
-      <c r="K64" s="18" t="n"/>
-      <c r="L64" s="18" t="n"/>
-      <c r="M64" s="18" t="n"/>
-      <c r="N64" s="18" t="n"/>
-      <c r="O64" s="18" t="n"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="11" t="inlineStr">
-        <is>
-          <t>▸ Western PA / Ohio Valley  (3)</t>
-        </is>
-      </c>
-      <c r="B65" s="12" t="n"/>
-      <c r="C65" s="12" t="n"/>
-      <c r="D65" s="12" t="n"/>
-      <c r="E65" s="12" t="n"/>
-      <c r="F65" s="12" t="n"/>
-      <c r="G65" s="12" t="n"/>
-      <c r="H65" s="12" t="n"/>
-      <c r="I65" s="12" t="n"/>
-      <c r="J65" s="12" t="n"/>
-      <c r="K65" s="12" t="n"/>
-      <c r="L65" s="12" t="n"/>
-      <c r="M65" s="12" t="n"/>
-      <c r="N65" s="12" t="n"/>
-      <c r="O65" s="12" t="n"/>
-    </row>
-    <row r="66" outlineLevel="1">
-      <c r="A66" s="13" t="inlineStr">
-        <is>
-          <t>Western PA / Ohio Valley</t>
-        </is>
-      </c>
-      <c r="B66" s="14" t="inlineStr">
-        <is>
-          <t>Petrunak's Hardware Store liquidation Day 1 (530 lots: doors, hardware, tools, building supplies)</t>
-        </is>
-      </c>
-      <c r="C66" s="13" t="inlineStr">
-        <is>
-          <t>store closing auction</t>
-        </is>
-      </c>
-      <c r="D66" s="13" t="inlineStr">
-        <is>
-          <t>Windber</t>
-        </is>
-      </c>
-      <c r="E66" s="13" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="F66" s="13" t="n">
-        <v>437</v>
-      </c>
-      <c r="G66" s="13" t="inlineStr">
-        <is>
-          <t>Timed online auction (530 lots)</t>
-        </is>
-      </c>
-      <c r="H66" s="15" t="n"/>
-      <c r="I66" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="J66" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-21 08:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K66" s="13" t="inlineStr">
-        <is>
-          <t>Carey Auctions</t>
-        </is>
-      </c>
-      <c r="L66" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
-        </is>
-      </c>
-      <c r="M66" s="13" t="inlineStr"/>
-      <c r="N66" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O66" s="14" t="inlineStr">
-        <is>
-          <t>Ends Oct 21 7 PM CDT (8 PM ET). 1500 Somerset Ave, Windber PA. Pickups Oct 24-28. Hardware store, not appliance parts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" outlineLevel="1">
-      <c r="A67" s="13" t="inlineStr">
-        <is>
-          <t>Western PA / Ohio Valley</t>
-        </is>
-      </c>
-      <c r="B67" s="14" t="inlineStr">
-        <is>
-          <t>Petrunak's Hardware Store liquidation Day 2 (433 lots)</t>
-        </is>
-      </c>
-      <c r="C67" s="13" t="inlineStr">
-        <is>
-          <t>store closing auction</t>
-        </is>
-      </c>
-      <c r="D67" s="13" t="inlineStr">
-        <is>
-          <t>Windber</t>
-        </is>
-      </c>
-      <c r="E67" s="13" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="F67" s="13" t="n">
-        <v>437</v>
-      </c>
-      <c r="G67" s="13" t="inlineStr">
-        <is>
-          <t>Timed online auction (433 lots)</t>
-        </is>
-      </c>
-      <c r="H67" s="15" t="n"/>
-      <c r="I67" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="J67" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-22 08:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K67" s="13" t="inlineStr">
-        <is>
-          <t>Carey Auctions</t>
-        </is>
-      </c>
-      <c r="L67" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
-        </is>
-      </c>
-      <c r="M67" s="13" t="inlineStr"/>
-      <c r="N67" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O67" s="14" t="inlineStr">
-        <is>
-          <t>Ends Oct 22 7 PM CDT (8 PM ET). Same store as Day 1; pickups Oct 24-28.</t>
-        </is>
-      </c>
+      <c r="I66" s="18" t="n"/>
+      <c r="J66" s="18" t="n"/>
+      <c r="K66" s="18" t="n"/>
+      <c r="L66" s="18" t="n"/>
+      <c r="M66" s="18" t="n"/>
+      <c r="N66" s="18" t="n"/>
+      <c r="O66" s="18" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="11" t="inlineStr">
+        <is>
+          <t>▸ Upstate / Western NY  (1)</t>
+        </is>
+      </c>
+      <c r="B67" s="12" t="n"/>
+      <c r="C67" s="12" t="n"/>
+      <c r="D67" s="12" t="n"/>
+      <c r="E67" s="12" t="n"/>
+      <c r="F67" s="12" t="n"/>
+      <c r="G67" s="12" t="n"/>
+      <c r="H67" s="12" t="n"/>
+      <c r="I67" s="12" t="n"/>
+      <c r="J67" s="12" t="n"/>
+      <c r="K67" s="12" t="n"/>
+      <c r="L67" s="12" t="n"/>
+      <c r="M67" s="12" t="n"/>
+      <c r="N67" s="12" t="n"/>
+      <c r="O67" s="12" t="n"/>
     </row>
     <row r="68" outlineLevel="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>Western PA / Ohio Valley</t>
+          <t>Upstate / Western NY</t>
         </is>
       </c>
       <c r="B68" s="14" t="inlineStr">
         <is>
-          <t>Millers Pizza &amp; More – pizza business, commercial kitchen &amp; event space contents (362 lots)</t>
+          <t>Restaurant &amp; fitness equipment</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>restaurant / commercial kitchen contents</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D68" s="13" t="inlineStr">
         <is>
-          <t>Everson</t>
+          <t>Williamsville</t>
         </is>
       </c>
       <c r="E68" s="13" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F68" s="13" t="n">
-        <v>478</v>
+        <v>408</v>
       </c>
       <c r="G68" s="13" t="inlineStr">
         <is>
-          <t>Online auction, 15% buyer premium</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H68" s="15" t="n"/>
       <c r="I68" s="13" t="inlineStr"/>
       <c r="J68" s="13" t="inlineStr">
         <is>
-          <t>2026-10-25 07:00 PM ET</t>
+          <t>2026-10-26 07:30 PM ET</t>
         </is>
       </c>
       <c r="K68" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Bid Local LLC)</t>
+          <t>Cash Auctions</t>
         </is>
       </c>
       <c r="L68" s="13" t="inlineStr">
@@ -22294,19 +22216,19 @@
       </c>
       <c r="O68" s="14" t="inlineStr">
         <is>
-          <t>Property of Millers Pizza and More LLC; online-only, 362 lots, lots begin closing Oct 25 7 PM. Pickup Everson PA by appointment Tue 10/27 and Wed 10/28. Building (4,500 sq ft) to be auctioned separately.</t>
+          <t>Lots not reviewed.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="17" t="inlineStr">
         <is>
-          <t>Subtotal — Western PA / Ohio Valley</t>
+          <t>Subtotal — Upstate / Western NY</t>
         </is>
       </c>
       <c r="B69" s="17" t="inlineStr">
         <is>
-          <t>3 item(s)</t>
+          <t>1 item(s)</t>
         </is>
       </c>
       <c r="C69" s="18" t="n"/>
@@ -22328,7 +22250,7 @@
     <row r="70">
       <c r="A70" s="11" t="inlineStr">
         <is>
-          <t>▸ Upstate / Western NY  (1)</t>
+          <t>▸ Virginia  (1)</t>
         </is>
       </c>
       <c r="B70" s="12" t="n"/>
@@ -22349,47 +22271,47 @@
     <row r="71" outlineLevel="1">
       <c r="A71" s="13" t="inlineStr">
         <is>
-          <t>Upstate / Western NY</t>
+          <t>Virginia</t>
         </is>
       </c>
       <c r="B71" s="14" t="inlineStr">
         <is>
-          <t>Restaurant &amp; fitness equipment</t>
+          <t>Haynes Furniture / The Dump – 12 stores closing (furniture, mattresses)</t>
         </is>
       </c>
       <c r="C71" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>retail GOB</t>
         </is>
       </c>
       <c r="D71" s="13" t="inlineStr">
         <is>
-          <t>Williamsville</t>
+          <t>Virginia Beach</t>
         </is>
       </c>
       <c r="E71" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>VA</t>
         </is>
       </c>
       <c r="F71" s="13" t="n">
-        <v>408</v>
+        <v>456</v>
       </c>
       <c r="G71" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Retail GOB markdowns</t>
         </is>
       </c>
       <c r="H71" s="15" t="n"/>
-      <c r="I71" s="13" t="inlineStr"/>
-      <c r="J71" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26 07:30 PM ET</t>
-        </is>
-      </c>
+      <c r="I71" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="J71" s="13" t="inlineStr"/>
       <c r="K71" s="13" t="inlineStr">
         <is>
-          <t>Cash Auctions</t>
+          <t>SB360 (PR Newswire)</t>
         </is>
       </c>
       <c r="L71" s="13" t="inlineStr">
@@ -22405,14 +22327,14 @@
       </c>
       <c r="O71" s="14" t="inlineStr">
         <is>
-          <t>Lots not reviewed.</t>
+          <t>Posted Oct 8. Multi-state (VA/AZ/GA/IL/TX); pinned at Virginia Beach. Home goods only.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="17" t="inlineStr">
         <is>
-          <t>Subtotal — Upstate / Western NY</t>
+          <t>Subtotal — Virginia</t>
         </is>
       </c>
       <c r="B72" s="17" t="inlineStr">
@@ -22439,7 +22361,7 @@
     <row r="73">
       <c r="A73" s="11" t="inlineStr">
         <is>
-          <t>▸ Virginia  (1)</t>
+          <t>▸ Midwest  (2)</t>
         </is>
       </c>
       <c r="B73" s="12" t="n"/>
@@ -22460,12 +22382,12 @@
     <row r="74" outlineLevel="1">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>Virginia</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="B74" s="14" t="inlineStr">
         <is>
-          <t>Haynes Furniture / The Dump – 12 stores closing (furniture, mattresses)</t>
+          <t>American Sale – total liquidation, all 7 stores (pools, hot tubs, grills, holiday decor)</t>
         </is>
       </c>
       <c r="C74" s="13" t="inlineStr">
@@ -22475,32 +22397,32 @@
       </c>
       <c r="D74" s="13" t="inlineStr">
         <is>
-          <t>Virginia Beach</t>
+          <t>Chicagoland</t>
         </is>
       </c>
       <c r="E74" s="13" t="inlineStr">
         <is>
-          <t>VA</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="F74" s="13" t="n">
-        <v>456</v>
+        <v>876</v>
       </c>
       <c r="G74" s="13" t="inlineStr">
         <is>
-          <t>Retail GOB markdowns</t>
+          <t>Retail GOB, up to 70% off</t>
         </is>
       </c>
       <c r="H74" s="15" t="n"/>
       <c r="I74" s="13" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="J74" s="13" t="inlineStr"/>
       <c r="K74" s="13" t="inlineStr">
         <is>
-          <t>SB360 (PR Newswire)</t>
+          <t>Tiger Group (PR Newswire)</t>
         </is>
       </c>
       <c r="L74" s="13" t="inlineStr">
@@ -22516,170 +22438,170 @@
       </c>
       <c r="O74" s="14" t="inlineStr">
         <is>
-          <t>Posted Oct 8. Multi-state (VA/AZ/GA/IL/TX); pinned at Virginia Beach. Home goods only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Virginia</t>
-        </is>
-      </c>
-      <c r="B75" s="17" t="inlineStr">
-        <is>
-          <t>1 item(s)</t>
-        </is>
-      </c>
-      <c r="C75" s="18" t="n"/>
-      <c r="D75" s="18" t="n"/>
-      <c r="E75" s="18" t="n"/>
-      <c r="F75" s="18" t="n"/>
-      <c r="G75" s="18" t="n"/>
-      <c r="H75" s="19" t="n">
+          <t>Posted Oct 15. Watch for a bulk/fixture auction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" outlineLevel="1">
+      <c r="A75" s="13" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="B75" s="14" t="inlineStr">
+        <is>
+          <t>Restaurant, Bar &amp; DJ Equipment Liquidation: Alto-Shaam combi, Southbend/Blodgett ovens, True refrigeration, Manitowoc, Hobart saw, DJ/AV gear</t>
+        </is>
+      </c>
+      <c r="C75" s="13" t="inlineStr">
+        <is>
+          <t>restaurant liquidation auction</t>
+        </is>
+      </c>
+      <c r="D75" s="13" t="inlineStr">
+        <is>
+          <t>Austin</t>
+        </is>
+      </c>
+      <c r="E75" s="13" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="F75" s="13" t="n">
+        <v>1124</v>
+      </c>
+      <c r="G75" s="13" t="inlineStr">
+        <is>
+          <t>Timed online auction</t>
+        </is>
+      </c>
+      <c r="H75" s="15" t="n"/>
+      <c r="I75" s="13" t="inlineStr"/>
+      <c r="J75" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-26 02:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K75" s="13" t="inlineStr">
+        <is>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L75" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M75" s="13" t="inlineStr"/>
+      <c r="N75" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O75" s="14" t="inlineStr">
+        <is>
+          <t>Begins closing Oct 26 1 PM CDT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Midwest</t>
+        </is>
+      </c>
+      <c r="B76" s="17" t="inlineStr">
+        <is>
+          <t>2 item(s)</t>
+        </is>
+      </c>
+      <c r="C76" s="18" t="n"/>
+      <c r="D76" s="18" t="n"/>
+      <c r="E76" s="18" t="n"/>
+      <c r="F76" s="18" t="n"/>
+      <c r="G76" s="18" t="n"/>
+      <c r="H76" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I75" s="18" t="n"/>
-      <c r="J75" s="18" t="n"/>
-      <c r="K75" s="18" t="n"/>
-      <c r="L75" s="18" t="n"/>
-      <c r="M75" s="18" t="n"/>
-      <c r="N75" s="18" t="n"/>
-      <c r="O75" s="18" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="11" t="inlineStr">
-        <is>
-          <t>▸ Midwest  (3)</t>
-        </is>
-      </c>
-      <c r="B76" s="12" t="n"/>
-      <c r="C76" s="12" t="n"/>
-      <c r="D76" s="12" t="n"/>
-      <c r="E76" s="12" t="n"/>
-      <c r="F76" s="12" t="n"/>
-      <c r="G76" s="12" t="n"/>
-      <c r="H76" s="12" t="n"/>
-      <c r="I76" s="12" t="n"/>
-      <c r="J76" s="12" t="n"/>
-      <c r="K76" s="12" t="n"/>
-      <c r="L76" s="12" t="n"/>
-      <c r="M76" s="12" t="n"/>
-      <c r="N76" s="12" t="n"/>
-      <c r="O76" s="12" t="n"/>
-    </row>
-    <row r="77" outlineLevel="1">
-      <c r="A77" s="13" t="inlineStr">
-        <is>
-          <t>Midwest</t>
-        </is>
-      </c>
-      <c r="B77" s="14" t="inlineStr">
-        <is>
-          <t>American Sale – total liquidation, all 7 stores (pools, hot tubs, grills, holiday decor)</t>
-        </is>
-      </c>
-      <c r="C77" s="13" t="inlineStr">
-        <is>
-          <t>retail GOB</t>
-        </is>
-      </c>
-      <c r="D77" s="13" t="inlineStr">
-        <is>
-          <t>Chicagoland</t>
-        </is>
-      </c>
-      <c r="E77" s="13" t="inlineStr">
-        <is>
-          <t>IL</t>
-        </is>
-      </c>
-      <c r="F77" s="13" t="n">
-        <v>876</v>
-      </c>
-      <c r="G77" s="13" t="inlineStr">
-        <is>
-          <t>Retail GOB, up to 70% off</t>
-        </is>
-      </c>
-      <c r="H77" s="15" t="n"/>
-      <c r="I77" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="J77" s="13" t="inlineStr"/>
-      <c r="K77" s="13" t="inlineStr">
-        <is>
-          <t>Tiger Group (PR Newswire)</t>
-        </is>
-      </c>
-      <c r="L77" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M77" s="13" t="inlineStr"/>
-      <c r="N77" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O77" s="14" t="inlineStr">
-        <is>
-          <t>Posted Oct 15. Watch for a bulk/fixture auction.</t>
-        </is>
-      </c>
+      <c r="I76" s="18" t="n"/>
+      <c r="J76" s="18" t="n"/>
+      <c r="K76" s="18" t="n"/>
+      <c r="L76" s="18" t="n"/>
+      <c r="M76" s="18" t="n"/>
+      <c r="N76" s="18" t="n"/>
+      <c r="O76" s="18" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="11" t="inlineStr">
+        <is>
+          <t>▸ Texas / South Central  (1)</t>
+        </is>
+      </c>
+      <c r="B77" s="12" t="n"/>
+      <c r="C77" s="12" t="n"/>
+      <c r="D77" s="12" t="n"/>
+      <c r="E77" s="12" t="n"/>
+      <c r="F77" s="12" t="n"/>
+      <c r="G77" s="12" t="n"/>
+      <c r="H77" s="12" t="n"/>
+      <c r="I77" s="12" t="n"/>
+      <c r="J77" s="12" t="n"/>
+      <c r="K77" s="12" t="n"/>
+      <c r="L77" s="12" t="n"/>
+      <c r="M77" s="12" t="n"/>
+      <c r="N77" s="12" t="n"/>
+      <c r="O77" s="12" t="n"/>
     </row>
     <row r="78" outlineLevel="1">
       <c r="A78" s="13" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>Texas / South Central</t>
         </is>
       </c>
       <c r="B78" s="14" t="inlineStr">
         <is>
-          <t>Straub's Fine Foods store equipment – bakery, kitchen, meat room, Hussmann refrigeration</t>
+          <t>Southwest beverage distributor surplus – mostly unused: 16 True merchandisers, 75 Bunn brewers, 100+ micro-market kiosks</t>
         </is>
       </c>
       <c r="C78" s="13" t="inlineStr">
         <is>
-          <t>grocery/restaurant</t>
+          <t>distributor surplus</t>
         </is>
       </c>
       <c r="D78" s="13" t="inlineStr">
         <is>
-          <t>St. Louis</t>
+          <t>Mesquite</t>
         </is>
       </c>
       <c r="E78" s="13" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="F78" s="13" t="n">
-        <v>1046</v>
+        <v>1547</v>
       </c>
       <c r="G78" s="13" t="inlineStr">
         <is>
-          <t>Online auction (18% BP)</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H78" s="15" t="n"/>
       <c r="I78" s="13" t="inlineStr"/>
       <c r="J78" s="13" t="inlineStr">
         <is>
-          <t>2026-10-21 11:00 AM ET</t>
+          <t>2026-11-13 11:00 AM ET</t>
         </is>
       </c>
       <c r="K78" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
-        </is>
-      </c>
-      <c r="L78" s="20" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>Heritage Global Partners</t>
+        </is>
+      </c>
+      <c r="L78" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M78" s="13" t="inlineStr"/>
@@ -22690,324 +22612,150 @@
       </c>
       <c r="O78" s="14" t="inlineStr">
         <is>
-          <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis.</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" outlineLevel="1">
-      <c r="A79" s="13" t="inlineStr">
-        <is>
-          <t>Midwest</t>
-        </is>
-      </c>
-      <c r="B79" s="14" t="inlineStr">
-        <is>
-          <t>Restaurant, Bar &amp; DJ Equipment Liquidation: Alto-Shaam combi, Southbend/Blodgett ovens, True refrigeration, Manitowoc, Hobart saw, DJ/AV gear</t>
-        </is>
-      </c>
-      <c r="C79" s="13" t="inlineStr">
-        <is>
-          <t>restaurant liquidation auction</t>
-        </is>
-      </c>
-      <c r="D79" s="13" t="inlineStr">
-        <is>
-          <t>Austin</t>
-        </is>
-      </c>
-      <c r="E79" s="13" t="inlineStr">
-        <is>
-          <t>MN</t>
-        </is>
-      </c>
-      <c r="F79" s="13" t="n">
-        <v>1124</v>
-      </c>
-      <c r="G79" s="13" t="inlineStr">
-        <is>
-          <t>Timed online auction</t>
-        </is>
-      </c>
-      <c r="H79" s="15" t="n"/>
-      <c r="I79" s="13" t="inlineStr"/>
-      <c r="J79" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26 02:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K79" s="13" t="inlineStr">
-        <is>
-          <t>Grafe Auction</t>
-        </is>
-      </c>
-      <c r="L79" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M79" s="13" t="inlineStr"/>
-      <c r="N79" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O79" s="14" t="inlineStr">
-        <is>
-          <t>Begins closing Oct 26 1 PM CDT.</t>
-        </is>
-      </c>
+          <t>Near-new appliances, resell by unit. Nov 13 10 AM CST.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Texas / South Central</t>
+        </is>
+      </c>
+      <c r="B79" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C79" s="18" t="n"/>
+      <c r="D79" s="18" t="n"/>
+      <c r="E79" s="18" t="n"/>
+      <c r="F79" s="18" t="n"/>
+      <c r="G79" s="18" t="n"/>
+      <c r="H79" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I79" s="18" t="n"/>
+      <c r="J79" s="18" t="n"/>
+      <c r="K79" s="18" t="n"/>
+      <c r="L79" s="18" t="n"/>
+      <c r="M79" s="18" t="n"/>
+      <c r="N79" s="18" t="n"/>
+      <c r="O79" s="18" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Midwest</t>
-        </is>
-      </c>
-      <c r="B80" s="17" t="inlineStr">
-        <is>
-          <t>3 item(s)</t>
-        </is>
-      </c>
-      <c r="C80" s="18" t="n"/>
-      <c r="D80" s="18" t="n"/>
-      <c r="E80" s="18" t="n"/>
-      <c r="F80" s="18" t="n"/>
-      <c r="G80" s="18" t="n"/>
-      <c r="H80" s="19" t="n">
+      <c r="A80" s="11" t="inlineStr">
+        <is>
+          <t>▸ West / Other  (1)</t>
+        </is>
+      </c>
+      <c r="B80" s="12" t="n"/>
+      <c r="C80" s="12" t="n"/>
+      <c r="D80" s="12" t="n"/>
+      <c r="E80" s="12" t="n"/>
+      <c r="F80" s="12" t="n"/>
+      <c r="G80" s="12" t="n"/>
+      <c r="H80" s="12" t="n"/>
+      <c r="I80" s="12" t="n"/>
+      <c r="J80" s="12" t="n"/>
+      <c r="K80" s="12" t="n"/>
+      <c r="L80" s="12" t="n"/>
+      <c r="M80" s="12" t="n"/>
+      <c r="N80" s="12" t="n"/>
+      <c r="O80" s="12" t="n"/>
+    </row>
+    <row r="81" outlineLevel="1">
+      <c r="A81" s="13" t="inlineStr">
+        <is>
+          <t>West / Other</t>
+        </is>
+      </c>
+      <c r="B81" s="14" t="inlineStr">
+        <is>
+          <t>National salad concept liquidation – full contents of 63 fast-casual restaurants (AZ/TX/OK/NV)</t>
+        </is>
+      </c>
+      <c r="C81" s="13" t="inlineStr">
+        <is>
+          <t>restaurant chain liquidation</t>
+        </is>
+      </c>
+      <c r="D81" s="13" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="E81" s="13" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="F81" s="13" t="n">
+        <v>2307</v>
+      </c>
+      <c r="G81" s="13" t="inlineStr">
+        <is>
+          <t>Online auctions, dates TBD</t>
+        </is>
+      </c>
+      <c r="H81" s="15" t="n"/>
+      <c r="I81" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="J81" s="13" t="inlineStr"/>
+      <c r="K81" s="13" t="inlineStr">
+        <is>
+          <t>RestaurantEquipment.bid (TAGeX)</t>
+        </is>
+      </c>
+      <c r="L81" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M81" s="13" t="inlineStr"/>
+      <c r="N81" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O81" s="14" t="inlineStr">
+        <is>
+          <t>Rolling market-by-market auctions, none live yet (Phoenix metro 30 locations, DFW 14, Tucson 6, Houston 5, plus OK/NV). Pickup on site at each restaurant. Pinned at Phoenix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — West / Other</t>
+        </is>
+      </c>
+      <c r="B82" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C82" s="18" t="n"/>
+      <c r="D82" s="18" t="n"/>
+      <c r="E82" s="18" t="n"/>
+      <c r="F82" s="18" t="n"/>
+      <c r="G82" s="18" t="n"/>
+      <c r="H82" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I80" s="18" t="n"/>
-      <c r="J80" s="18" t="n"/>
-      <c r="K80" s="18" t="n"/>
-      <c r="L80" s="18" t="n"/>
-      <c r="M80" s="18" t="n"/>
-      <c r="N80" s="18" t="n"/>
-      <c r="O80" s="18" t="n"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="11" t="inlineStr">
-        <is>
-          <t>▸ Texas / South Central  (1)</t>
-        </is>
-      </c>
-      <c r="B81" s="12" t="n"/>
-      <c r="C81" s="12" t="n"/>
-      <c r="D81" s="12" t="n"/>
-      <c r="E81" s="12" t="n"/>
-      <c r="F81" s="12" t="n"/>
-      <c r="G81" s="12" t="n"/>
-      <c r="H81" s="12" t="n"/>
-      <c r="I81" s="12" t="n"/>
-      <c r="J81" s="12" t="n"/>
-      <c r="K81" s="12" t="n"/>
-      <c r="L81" s="12" t="n"/>
-      <c r="M81" s="12" t="n"/>
-      <c r="N81" s="12" t="n"/>
-      <c r="O81" s="12" t="n"/>
-    </row>
-    <row r="82" outlineLevel="1">
-      <c r="A82" s="13" t="inlineStr">
-        <is>
-          <t>Texas / South Central</t>
-        </is>
-      </c>
-      <c r="B82" s="14" t="inlineStr">
-        <is>
-          <t>Southwest beverage distributor surplus – mostly unused: 16 True merchandisers, 75 Bunn brewers, 100+ micro-market kiosks</t>
-        </is>
-      </c>
-      <c r="C82" s="13" t="inlineStr">
-        <is>
-          <t>distributor surplus</t>
-        </is>
-      </c>
-      <c r="D82" s="13" t="inlineStr">
-        <is>
-          <t>Mesquite</t>
-        </is>
-      </c>
-      <c r="E82" s="13" t="inlineStr">
-        <is>
-          <t>TX</t>
-        </is>
-      </c>
-      <c r="F82" s="13" t="n">
-        <v>1547</v>
-      </c>
-      <c r="G82" s="13" t="inlineStr">
-        <is>
-          <t>Online auction</t>
-        </is>
-      </c>
-      <c r="H82" s="15" t="n"/>
-      <c r="I82" s="13" t="inlineStr"/>
-      <c r="J82" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-13 11:00 AM ET</t>
-        </is>
-      </c>
-      <c r="K82" s="13" t="inlineStr">
-        <is>
-          <t>Heritage Global Partners</t>
-        </is>
-      </c>
-      <c r="L82" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M82" s="13" t="inlineStr"/>
-      <c r="N82" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O82" s="14" t="inlineStr">
-        <is>
-          <t>Near-new appliances, resell by unit. Nov 13 10 AM CST.</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Texas / South Central</t>
-        </is>
-      </c>
-      <c r="B83" s="17" t="inlineStr">
-        <is>
-          <t>1 item(s)</t>
-        </is>
-      </c>
-      <c r="C83" s="18" t="n"/>
-      <c r="D83" s="18" t="n"/>
-      <c r="E83" s="18" t="n"/>
-      <c r="F83" s="18" t="n"/>
-      <c r="G83" s="18" t="n"/>
-      <c r="H83" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I83" s="18" t="n"/>
-      <c r="J83" s="18" t="n"/>
-      <c r="K83" s="18" t="n"/>
-      <c r="L83" s="18" t="n"/>
-      <c r="M83" s="18" t="n"/>
-      <c r="N83" s="18" t="n"/>
-      <c r="O83" s="18" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="11" t="inlineStr">
-        <is>
-          <t>▸ West / Other  (1)</t>
-        </is>
-      </c>
-      <c r="B84" s="12" t="n"/>
-      <c r="C84" s="12" t="n"/>
-      <c r="D84" s="12" t="n"/>
-      <c r="E84" s="12" t="n"/>
-      <c r="F84" s="12" t="n"/>
-      <c r="G84" s="12" t="n"/>
-      <c r="H84" s="12" t="n"/>
-      <c r="I84" s="12" t="n"/>
-      <c r="J84" s="12" t="n"/>
-      <c r="K84" s="12" t="n"/>
-      <c r="L84" s="12" t="n"/>
-      <c r="M84" s="12" t="n"/>
-      <c r="N84" s="12" t="n"/>
-      <c r="O84" s="12" t="n"/>
-    </row>
-    <row r="85" outlineLevel="1">
-      <c r="A85" s="13" t="inlineStr">
-        <is>
-          <t>West / Other</t>
-        </is>
-      </c>
-      <c r="B85" s="14" t="inlineStr">
-        <is>
-          <t>National salad concept liquidation – full contents of 63 fast-casual restaurants (AZ/TX/OK/NV)</t>
-        </is>
-      </c>
-      <c r="C85" s="13" t="inlineStr">
-        <is>
-          <t>restaurant chain liquidation</t>
-        </is>
-      </c>
-      <c r="D85" s="13" t="inlineStr">
-        <is>
-          <t>Phoenix</t>
-        </is>
-      </c>
-      <c r="E85" s="13" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="F85" s="13" t="n">
-        <v>2307</v>
-      </c>
-      <c r="G85" s="13" t="inlineStr">
-        <is>
-          <t>Online auctions, dates TBD</t>
-        </is>
-      </c>
-      <c r="H85" s="15" t="n"/>
-      <c r="I85" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="J85" s="13" t="inlineStr"/>
-      <c r="K85" s="13" t="inlineStr">
-        <is>
-          <t>RestaurantEquipment.bid (TAGeX)</t>
-        </is>
-      </c>
-      <c r="L85" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M85" s="13" t="inlineStr"/>
-      <c r="N85" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O85" s="14" t="inlineStr">
-        <is>
-          <t>Rolling market-by-market auctions, none live yet (Phoenix metro 30 locations, DFW 14, Tucson 6, Houston 5, plus OK/NV). Pickup on site at each restaurant. Pinned at Phoenix.</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — West / Other</t>
-        </is>
-      </c>
-      <c r="B86" s="17" t="inlineStr">
-        <is>
-          <t>1 item(s)</t>
-        </is>
-      </c>
-      <c r="C86" s="18" t="n"/>
-      <c r="D86" s="18" t="n"/>
-      <c r="E86" s="18" t="n"/>
-      <c r="F86" s="18" t="n"/>
-      <c r="G86" s="18" t="n"/>
-      <c r="H86" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I86" s="18" t="n"/>
-      <c r="J86" s="18" t="n"/>
-      <c r="K86" s="18" t="n"/>
-      <c r="L86" s="18" t="n"/>
-      <c r="M86" s="18" t="n"/>
-      <c r="N86" s="18" t="n"/>
-      <c r="O86" s="18" t="n"/>
+      <c r="I82" s="18" t="n"/>
+      <c r="J82" s="18" t="n"/>
+      <c r="K82" s="18" t="n"/>
+      <c r="L82" s="18" t="n"/>
+      <c r="M82" s="18" t="n"/>
+      <c r="N82" s="18" t="n"/>
+      <c r="O82" s="18" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O86"/>
+  <autoFilter ref="A1:O82"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId2"/>
@@ -23054,20 +22802,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N55" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N56" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N57" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N58" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N59" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N62" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N63" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N66" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N67" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N68" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N71" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N74" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N77" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N78" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N79" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N82" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N85" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N60" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N63" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N64" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N65" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N68" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N71" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N74" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N75" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N78" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N81" r:id="rId55"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -23079,7 +22823,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:O23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -23241,7 +22985,7 @@
       </c>
       <c r="O2" s="14" t="inlineStr">
         <is>
-          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
+          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23304,7 +23048,7 @@
       </c>
       <c r="O3" s="14" t="inlineStr">
         <is>
-          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
+          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23505,7 +23249,7 @@
       </c>
       <c r="O6" s="14" t="inlineStr">
         <is>
-          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
+          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23570,7 +23314,7 @@
       </c>
       <c r="O7" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23635,7 +23379,7 @@
       </c>
       <c r="O8" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
+          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23700,7 +23444,7 @@
       </c>
       <c r="O9" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
+          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23763,7 +23507,7 @@
       </c>
       <c r="O10" s="14" t="inlineStr">
         <is>
-          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
+          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23826,59 +23570,59 @@
       </c>
       <c r="O11" s="14" t="inlineStr">
         <is>
-          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
+          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>NYC / Long Island / NJ</t>
+          <t>Eastern PA / Mid-Atlantic</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>Milwaukee / Walmart / hardware store mega auction pt 3</t>
+          <t>October restaurant consignment – Hobart, Rational, True + NEW scratch-and-dent Migali/Avantco</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Mount Holly</t>
+          <t>Harrisburg</t>
         </is>
       </c>
       <c r="E12" s="13" t="inlineStr">
         <is>
-          <t>NJ</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>254</v>
+        <v>340</v>
       </c>
       <c r="G12" s="13" t="inlineStr">
         <is>
-          <t>HiBid online auction</t>
+          <t>Online auction, 15% BP, ships $55/pallet</t>
         </is>
       </c>
       <c r="H12" s="15" t="n"/>
       <c r="I12" s="13" t="inlineStr"/>
       <c r="J12" s="13" t="inlineStr">
         <is>
-          <t>2026-10-19 06:00 PM ET</t>
+          <t>2026-10-21 11:00 AM ET</t>
         </is>
       </c>
       <c r="K12" s="13" t="inlineStr">
         <is>
-          <t>HiBid</t>
+          <t>Restaurant Auction Co</t>
         </is>
       </c>
       <c r="L12" s="13" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-10-19 06:00 PM ET)</t>
+          <t>EXPIRED (2026-10-21 11:00 AM ET)</t>
         </is>
       </c>
       <c r="M12" s="13" t="inlineStr"/>
@@ -23889,19 +23633,19 @@
       </c>
       <c r="O12" s="14" t="inlineStr">
         <is>
-          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
+          <t>Closes Oct 21 10 or 11 AM (later used). Shippable. [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>Upstate / Western NY</t>
+          <t>NYC / Long Island / NJ</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>Closed restaurant – coolers, fridges, prep tables</t>
+          <t>Serpico's Pizzeria (lost lease) – Bari ovens, walk-in, Hobart 60qt, Vulcan range</t>
         </is>
       </c>
       <c r="C13" s="13" t="inlineStr">
@@ -23911,37 +23655,37 @@
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>Palmyra</t>
+          <t>Allenhurst</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>333</v>
+        <v>210</v>
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>HiBid, 15% BP</t>
+          <t>No-reserve online auction</t>
         </is>
       </c>
       <c r="H13" s="15" t="n"/>
       <c r="I13" s="13" t="inlineStr"/>
       <c r="J13" s="13" t="inlineStr">
         <is>
-          <t>2026-10-19 07:00 PM ET</t>
+          <t>2026-10-21 11:00 AM ET</t>
         </is>
       </c>
       <c r="K13" s="13" t="inlineStr">
         <is>
-          <t>Reynolds Auction Co / HiBid</t>
+          <t>Peter Costanzo / EstateSales.net</t>
         </is>
       </c>
       <c r="L13" s="13" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-10-19 07:00 PM ET)</t>
+          <t>EXPIRED (2026-10-21 11:00 AM ET)</t>
         </is>
       </c>
       <c r="M13" s="13" t="inlineStr"/>
@@ -23952,38 +23696,38 @@
       </c>
       <c r="O13" s="14" t="inlineStr">
         <is>
-          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
+          <t>Absolute / no reserve. [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>Upstate / Western NY</t>
+          <t>NYC / Long Island / NJ</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>Former Taco Del Mar – stainless, warmers, walk-in panels</t>
+          <t>Milwaukee / Walmart / hardware store mega auction pt 3</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>inventory</t>
         </is>
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>Watson</t>
+          <t>Mount Holly</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
@@ -23994,17 +23738,17 @@
       <c r="I14" s="13" t="inlineStr"/>
       <c r="J14" s="13" t="inlineStr">
         <is>
-          <t>2026-10-20 06:00 PM ET</t>
+          <t>2026-10-19 06:00 PM ET</t>
         </is>
       </c>
       <c r="K14" s="13" t="inlineStr">
         <is>
-          <t>Adirondack Asset / HiBid</t>
+          <t>HiBid</t>
         </is>
       </c>
       <c r="L14" s="13" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-10-20 06:00 PM ET)</t>
+          <t>EXPIRED (2026-10-19 06:00 PM ET)</t>
         </is>
       </c>
       <c r="M14" s="13" t="inlineStr"/>
@@ -24015,38 +23759,38 @@
       </c>
       <c r="O14" s="14" t="inlineStr">
         <is>
-          <t>Small lot. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
+          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>NYC / Long Island / NJ</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>Freshway Market whole-grocery liquidation – refrigeration racks, cases, walk-ins, generator</t>
+          <t>Altitude Trampoline Park liquidation – partial: Atosa, TurboChef, stainless</t>
         </is>
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>facility contents</t>
         </is>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Iselin</t>
         </is>
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>862</v>
+        <v>211</v>
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
@@ -24057,17 +23801,17 @@
       <c r="I15" s="13" t="inlineStr"/>
       <c r="J15" s="13" t="inlineStr">
         <is>
-          <t>2026-10-20 11:00 AM ET</t>
+          <t>2026-10-21 11:00 AM ET</t>
         </is>
       </c>
       <c r="K15" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
+          <t>A.J. Willner</t>
         </is>
       </c>
       <c r="L15" s="13" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-10-20 11:00 AM ET)</t>
+          <t>EXPIRED (2026-10-21 11:00 AM ET)</t>
         </is>
       </c>
       <c r="M15" s="13" t="inlineStr"/>
@@ -24078,59 +23822,59 @@
       </c>
       <c r="O15" s="14" t="inlineStr">
         <is>
-          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
+          <t>Some kitchen gear only. [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>Greater Boston / South Shore (&lt;50mi)</t>
+          <t>Upstate / Western NY</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>Closed Best Buy Outlet – pallet racking, Big Joe order pickers, appliance dollies, carts, cages</t>
+          <t>Closed restaurant – coolers, fridges, prep tables</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>store closing fixtures</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
-          <t>Brockton</t>
+          <t>Palmyra</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>11</v>
+        <v>333</v>
       </c>
       <c r="G16" s="13" t="inlineStr">
         <is>
-          <t>Racking $40/upright, $80/level; pickers $1,000 OBO</t>
+          <t>HiBid, 15% BP</t>
         </is>
       </c>
       <c r="H16" s="15" t="n"/>
-      <c r="I16" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="J16" s="13" t="inlineStr"/>
+      <c r="I16" s="13" t="inlineStr"/>
+      <c r="J16" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:00 PM ET</t>
+        </is>
+      </c>
       <c r="K16" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>Reynolds Auction Co / HiBid</t>
         </is>
       </c>
       <c r="L16" s="13" t="inlineStr">
         <is>
-          <t>REMOVED</t>
+          <t>EXPIRED (2026-10-19 07:00 PM ET)</t>
         </is>
       </c>
       <c r="M16" s="13" t="inlineStr"/>
@@ -24141,29 +23885,29 @@
       </c>
       <c r="O16" s="14" t="inlineStr">
         <is>
-          <t>200 Westgate Dr. Fixtures/equipment only, no merchandise. On site daily. CL deleted by author (HTTP 410) as of 2026-10-19 midday recheck.</t>
+          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>NYC / Long Island / NJ</t>
+          <t>Upstate / Western NY</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>Like-new restaurant – steam tables, Coldline, Cleveland cook-and-hold, fryers, True freezers</t>
+          <t>Former Taco Del Mar – stainless, warmers, walk-in panels</t>
         </is>
       </c>
       <c r="C17" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>Staten Island</t>
+          <t>Watson</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
@@ -24172,32 +23916,28 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>203</v>
+        <v>260</v>
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>HiBid online auction</t>
         </is>
       </c>
       <c r="H17" s="15" t="n"/>
-      <c r="I17" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
+      <c r="I17" s="13" t="inlineStr"/>
       <c r="J17" s="13" t="inlineStr">
         <is>
-          <t>2026-10-19 01:00 PM ET</t>
+          <t>2026-10-20 06:00 PM ET</t>
         </is>
       </c>
       <c r="K17" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>Adirondack Asset / HiBid</t>
         </is>
       </c>
       <c r="L17" s="13" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-10-19 01:00 PM ET)</t>
+          <t>EXPIRED (2026-10-20 06:00 PM ET)</t>
         </is>
       </c>
       <c r="M17" s="13" t="inlineStr"/>
@@ -24208,63 +23948,59 @@
       </c>
       <c r="O17" s="14" t="inlineStr">
         <is>
-          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
+          <t>Small lot. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>NYC / Long Island / NJ</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>Restaurant / pizzeria (contents not described)</t>
+          <t>Freshway Market whole-grocery liquidation – refrigeration racks, cases, walk-ins, generator</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>restaurant closing</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>Berkeley Heights</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>NJ</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>213</v>
+        <v>862</v>
       </c>
       <c r="G18" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H18" s="15" t="n"/>
-      <c r="I18" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
+      <c r="I18" s="13" t="inlineStr"/>
       <c r="J18" s="13" t="inlineStr">
         <is>
-          <t>2026-10-20 02:00 PM ET</t>
+          <t>2026-10-20 11:00 AM ET</t>
         </is>
       </c>
       <c r="K18" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>Grafe Auction</t>
         </is>
       </c>
       <c r="L18" s="13" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-10-20 02:00 PM ET)</t>
+          <t>EXPIRED (2026-10-20 11:00 AM ET)</t>
         </is>
       </c>
       <c r="M18" s="13" t="inlineStr"/>
@@ -24275,63 +24011,59 @@
       </c>
       <c r="O18" s="14" t="inlineStr">
         <is>
-          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
+          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>NYC / Long Island / NJ</t>
+          <t>Greater Boston / South Shore (&lt;50mi)</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>High-end deli (contents not described)</t>
+          <t>Closed Best Buy Outlet – pallet racking, Big Joe order pickers, appliance dollies, carts, cages</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>restaurant closing</t>
+          <t>store closing fixtures</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>Manalapan Township</t>
+          <t>Brockton</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>NJ</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>223</v>
+        <v>11</v>
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>Racking $40/upright, $80/level; pickers $1,000 OBO</t>
         </is>
       </c>
       <c r="H19" s="15" t="n"/>
       <c r="I19" s="13" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="J19" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-19 04:00 PM ET</t>
-        </is>
-      </c>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="J19" s="13" t="inlineStr"/>
       <c r="K19" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L19" s="13" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-10-19 04:00 PM ET)</t>
+          <t>REMOVED</t>
         </is>
       </c>
       <c r="M19" s="13" t="inlineStr"/>
@@ -24342,12 +24074,276 @@
       </c>
       <c r="O19" s="14" t="inlineStr">
         <is>
-          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
+          <t>200 Westgate Dr. Fixtures/equipment only, no merchandise. On site daily. CL deleted by author (HTTP 410) as of 2026-10-19 midday recheck.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>Like-new restaurant – steam tables, Coldline, Cleveland cook-and-hold, fryers, True freezers</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>auction</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>Staten Island</t>
+        </is>
+      </c>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="n">
+        <v>203</v>
+      </c>
+      <c r="G20" s="13" t="inlineStr">
+        <is>
+          <t>Live + webcast, 18% BP + 3%</t>
+        </is>
+      </c>
+      <c r="H20" s="15" t="n"/>
+      <c r="I20" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="J20" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 01:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K20" s="13" t="inlineStr">
+        <is>
+          <t>HiBid (Best Buy Auctioneers)</t>
+        </is>
+      </c>
+      <c r="L20" s="13" t="inlineStr">
+        <is>
+          <t>EXPIRED (2026-10-19 01:00 PM ET)</t>
+        </is>
+      </c>
+      <c r="M20" s="13" t="inlineStr"/>
+      <c r="N20" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O20" s="14" t="inlineStr">
+        <is>
+          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>Restaurant / pizzeria (contents not described)</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>restaurant closing</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>Berkeley Heights</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="F21" s="13" t="n">
+        <v>213</v>
+      </c>
+      <c r="G21" s="13" t="inlineStr">
+        <is>
+          <t>Live + webcast, 18% BP + 3%</t>
+        </is>
+      </c>
+      <c r="H21" s="15" t="n"/>
+      <c r="I21" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J21" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-20 02:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K21" s="13" t="inlineStr">
+        <is>
+          <t>HiBid (Best Buy Auctioneers)</t>
+        </is>
+      </c>
+      <c r="L21" s="13" t="inlineStr">
+        <is>
+          <t>EXPIRED (2026-10-20 02:00 PM ET)</t>
+        </is>
+      </c>
+      <c r="M21" s="13" t="inlineStr"/>
+      <c r="N21" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O21" s="14" t="inlineStr">
+        <is>
+          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>High-end deli (contents not described)</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>restaurant closing</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>Manalapan Township</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="n">
+        <v>223</v>
+      </c>
+      <c r="G22" s="13" t="inlineStr">
+        <is>
+          <t>Live + webcast, 18% BP + 3%</t>
+        </is>
+      </c>
+      <c r="H22" s="15" t="n"/>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="J22" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 04:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K22" s="13" t="inlineStr">
+        <is>
+          <t>HiBid (Best Buy Auctioneers)</t>
+        </is>
+      </c>
+      <c r="L22" s="13" t="inlineStr">
+        <is>
+          <t>EXPIRED (2026-10-19 04:00 PM ET)</t>
+        </is>
+      </c>
+      <c r="M22" s="13" t="inlineStr"/>
+      <c r="N22" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O22" s="14" t="inlineStr">
+        <is>
+          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Straub's Fine Foods store equipment – bakery, kitchen, meat room, Hussmann refrigeration</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>grocery/restaurant</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>St. Louis</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="F23" s="13" t="n">
+        <v>1046</v>
+      </c>
+      <c r="G23" s="13" t="inlineStr">
+        <is>
+          <t>Online auction (18% BP)</t>
+        </is>
+      </c>
+      <c r="H23" s="15" t="n"/>
+      <c r="I23" s="13" t="inlineStr"/>
+      <c r="J23" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-21 11:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K23" s="13" t="inlineStr">
+        <is>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L23" s="13" t="inlineStr">
+        <is>
+          <t>EXPIRED (2026-10-21 11:00 AM ET)</t>
+        </is>
+      </c>
+      <c r="M23" s="13" t="inlineStr"/>
+      <c r="N23" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O23" s="14" t="inlineStr">
+        <is>
+          <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis. [auto-removed 2026-10-21: closing date passed]</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O19"/>
+  <autoFilter ref="A1:O23"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
@@ -24367,6 +24363,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Lot Recon update 2026-10-23 11am ET: +Limerick Hardware liquidation PA, +Nyack NY consignment shop bulk inventory
</commit_message>
<xml_diff>
--- a/lot_recon.xlsx
+++ b/lot_recon.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wolf New'!$A$1:$O$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Wolf Used'!$A$1:$O$188</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Wolf Unclear'!$A$1:$O$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$96</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 2026-10-23 08:02 ET</t>
+          <t>Last updated: 2026-10-23 11:06 ET</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Active listings: 301 · Removed: 35</t>
+          <t>Active listings: 303 · Removed: 35</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>0</v>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="C13" s="7" t="n">
         <v>1441929.58</v>
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C23" t="n">
         <v>1</v>
@@ -1004,7 +1004,7 @@
         <v>4</v>
       </c>
       <c r="G23" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H23" s="6" t="n">
         <v>64650</v>
@@ -1055,7 +1055,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C25" t="n">
         <v>1</v>
@@ -1070,7 +1070,7 @@
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H25" s="6" t="n">
         <v>1500</v>
@@ -18342,7 +18342,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O94"/>
+  <dimension ref="A1:O96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -19887,7 +19887,7 @@
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>▸ CT / Hudson Valley  (8)</t>
+          <t>▸ CT / Hudson Valley  (9)</t>
         </is>
       </c>
       <c r="B31" s="12" t="n"/>
@@ -20291,17 +20291,17 @@
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>Body shop closing after 50 years – tools, welder, generators, plasma</t>
+          <t>Consignment shop remaining inventory, bulk buyer wanted</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>tools liquidation</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
         <is>
-          <t>West Nyack</t>
+          <t>Nyack</t>
         </is>
       </c>
       <c r="E38" s="13" t="inlineStr">
@@ -20310,17 +20310,17 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>Make offer / lot</t>
+          <t>Best offer</t>
         </is>
       </c>
       <c r="H38" s="15" t="n"/>
       <c r="I38" s="13" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="J38" s="13" t="inlineStr"/>
@@ -20342,7 +20342,7 @@
       </c>
       <c r="O38" s="14" t="inlineStr">
         <is>
-          <t>One-man auto body shop closing/retirement (Park Ridge / West Nyack NY-NJ border). Heat lamps, Kansas jack pullers, Miller 200 welder, generators, sheet-metal brake, hydraulic press, plasma cutter, engine hoist. Posted Aug 16; still open 2026-10-19.</t>
+          <t>Assorted secondhand consignment merchandise; one buyer preferred for most/all; pricing negotiable; buyer arranges pickup.</t>
         </is>
       </c>
     </row>
@@ -20354,17 +20354,17 @@
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>Woodworkers shop closing sale – shop tools &amp; hand tools</t>
+          <t>Body shop closing after 50 years – tools, welder, generators, plasma</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>woodworking shop closing</t>
+          <t>tools liquidation</t>
         </is>
       </c>
       <c r="D39" s="13" t="inlineStr">
         <is>
-          <t>Tappan</t>
+          <t>West Nyack</t>
         </is>
       </c>
       <c r="E39" s="13" t="inlineStr">
@@ -20373,17 +20373,17 @@
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G39" s="13" t="inlineStr">
         <is>
-          <t>Priced individually (some free)</t>
+          <t>Make offer / lot</t>
         </is>
       </c>
       <c r="H39" s="15" t="n"/>
       <c r="I39" s="13" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="J39" s="13" t="inlineStr"/>
@@ -20405,120 +20405,120 @@
       </c>
       <c r="O39" s="14" t="inlineStr">
         <is>
+          <t>One-man auto body shop closing/retirement (Park Ridge / West Nyack NY-NJ border). Heat lamps, Kansas jack pullers, Miller 200 welder, generators, sheet-metal brake, hydraulic press, plasma cutter, engine hoist. Posted Aug 16; still open 2026-10-19.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" outlineLevel="1">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>CT / Hudson Valley</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>Woodworkers shop closing sale – shop tools &amp; hand tools</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr">
+        <is>
+          <t>woodworking shop closing</t>
+        </is>
+      </c>
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>Tappan</t>
+        </is>
+      </c>
+      <c r="E40" s="13" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="F40" s="13" t="n">
+        <v>179</v>
+      </c>
+      <c r="G40" s="13" t="inlineStr">
+        <is>
+          <t>Priced individually (some free)</t>
+        </is>
+      </c>
+      <c r="H40" s="15" t="n"/>
+      <c r="I40" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="J40" s="13" t="inlineStr"/>
+      <c r="K40" s="13" t="inlineStr">
+        <is>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L40" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M40" s="13" t="inlineStr"/>
+      <c r="N40" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O40" s="14" t="inlineStr">
+        <is>
           <t>Ongoing shop-closing sale at 61 Main St, Tappan; many shop and hand tools, schedule a visit. Near the West Nyack body-shop sale (bl-054) for one trip.</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="17" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="17" t="inlineStr">
         <is>
           <t>Subtotal — CT / Hudson Valley</t>
         </is>
       </c>
-      <c r="B40" s="17" t="inlineStr">
-        <is>
-          <t>8 item(s)</t>
-        </is>
-      </c>
-      <c r="C40" s="18" t="n"/>
-      <c r="D40" s="18" t="n"/>
-      <c r="E40" s="18" t="n"/>
-      <c r="F40" s="18" t="n"/>
-      <c r="G40" s="18" t="n"/>
-      <c r="H40" s="19" t="n">
+      <c r="B41" s="17" t="inlineStr">
+        <is>
+          <t>9 item(s)</t>
+        </is>
+      </c>
+      <c r="C41" s="18" t="n"/>
+      <c r="D41" s="18" t="n"/>
+      <c r="E41" s="18" t="n"/>
+      <c r="F41" s="18" t="n"/>
+      <c r="G41" s="18" t="n"/>
+      <c r="H41" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I40" s="18" t="n"/>
-      <c r="J40" s="18" t="n"/>
-      <c r="K40" s="18" t="n"/>
-      <c r="L40" s="18" t="n"/>
-      <c r="M40" s="18" t="n"/>
-      <c r="N40" s="18" t="n"/>
-      <c r="O40" s="18" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="11" t="inlineStr">
+      <c r="I41" s="18" t="n"/>
+      <c r="J41" s="18" t="n"/>
+      <c r="K41" s="18" t="n"/>
+      <c r="L41" s="18" t="n"/>
+      <c r="M41" s="18" t="n"/>
+      <c r="N41" s="18" t="n"/>
+      <c r="O41" s="18" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="11" t="inlineStr">
         <is>
           <t>▸ NYC / Long Island / NJ  (26)</t>
         </is>
       </c>
-      <c r="B41" s="12" t="n"/>
-      <c r="C41" s="12" t="n"/>
-      <c r="D41" s="12" t="n"/>
-      <c r="E41" s="12" t="n"/>
-      <c r="F41" s="12" t="n"/>
-      <c r="G41" s="12" t="n"/>
-      <c r="H41" s="12" t="n"/>
-      <c r="I41" s="12" t="n"/>
-      <c r="J41" s="12" t="n"/>
-      <c r="K41" s="12" t="n"/>
-      <c r="L41" s="12" t="n"/>
-      <c r="M41" s="12" t="n"/>
-      <c r="N41" s="12" t="n"/>
-      <c r="O41" s="12" t="n"/>
-    </row>
-    <row r="42" outlineLevel="1">
-      <c r="A42" s="13" t="inlineStr">
-        <is>
-          <t>NYC / Long Island / NJ</t>
-        </is>
-      </c>
-      <c r="B42" s="14" t="inlineStr">
-        <is>
-          <t>Viva Margherita restaurant complete contents (building torn down)</t>
-        </is>
-      </c>
-      <c r="C42" s="13" t="inlineStr">
-        <is>
-          <t>restaurant closing</t>
-        </is>
-      </c>
-      <c r="D42" s="13" t="inlineStr">
-        <is>
-          <t>Edgewater</t>
-        </is>
-      </c>
-      <c r="E42" s="13" t="inlineStr">
-        <is>
-          <t>NJ</t>
-        </is>
-      </c>
-      <c r="F42" s="13" t="n">
-        <v>186</v>
-      </c>
-      <c r="G42" s="13" t="inlineStr">
-        <is>
-          <t>Complete contents / make offer</t>
-        </is>
-      </c>
-      <c r="H42" s="15" t="n"/>
-      <c r="I42" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-      <c r="J42" s="13" t="inlineStr"/>
-      <c r="K42" s="13" t="inlineStr">
-        <is>
-          <t>Craigslist</t>
-        </is>
-      </c>
-      <c r="L42" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M42" s="13" t="inlineStr"/>
-      <c r="N42" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O42" s="14" t="inlineStr">
-        <is>
-          <t>Address 163 Old River Road, Edgewater NJ. Building being torn down; complete restaurant contents for sale / make offer.</t>
-        </is>
-      </c>
+      <c r="B42" s="12" t="n"/>
+      <c r="C42" s="12" t="n"/>
+      <c r="D42" s="12" t="n"/>
+      <c r="E42" s="12" t="n"/>
+      <c r="F42" s="12" t="n"/>
+      <c r="G42" s="12" t="n"/>
+      <c r="H42" s="12" t="n"/>
+      <c r="I42" s="12" t="n"/>
+      <c r="J42" s="12" t="n"/>
+      <c r="K42" s="12" t="n"/>
+      <c r="L42" s="12" t="n"/>
+      <c r="M42" s="12" t="n"/>
+      <c r="N42" s="12" t="n"/>
+      <c r="O42" s="12" t="n"/>
     </row>
     <row r="43" outlineLevel="1">
       <c r="A43" s="13" t="inlineStr">
@@ -20528,7 +20528,7 @@
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>Gourmet Deli/Caterer, 100-yr Madison Ave deli liquidation (51 lots: Alto-Shaam ovens, Globe slicer, refrigerated deli cases/merchandisers, walk-in box, Metro racking)</t>
+          <t>Viva Margherita restaurant complete contents (building torn down)</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
@@ -20538,36 +20538,32 @@
       </c>
       <c r="D43" s="13" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Edgewater</t>
         </is>
       </c>
       <c r="E43" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="F43" s="13" t="n">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="G43" s="13" t="inlineStr">
         <is>
-          <t>Live/online auction, prebidding open; 18% BP online</t>
+          <t>Complete contents / make offer</t>
         </is>
       </c>
       <c r="H43" s="15" t="n"/>
       <c r="I43" s="13" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="J43" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-27 02:00 PM ET</t>
-        </is>
-      </c>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="J43" s="13" t="inlineStr"/>
       <c r="K43" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L43" s="13" t="inlineStr">
@@ -20583,7 +20579,7 @@
       </c>
       <c r="O43" s="14" t="inlineStr">
         <is>
-          <t>Live webcast starts Tue Oct 27 2 PM ET; preview Oct 27 11 AM; checkout Wed Oct 28 10-5. Address released before auction. Shipping can be arranged at buyer's cost.</t>
+          <t>Address 163 Old River Road, Edgewater NJ. Building being torn down; complete restaurant contents for sale / make offer.</t>
         </is>
       </c>
     </row>
@@ -20595,17 +20591,17 @@
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>Daycare/preschool closing: entire inventory of 4 classrooms (tables, cubbies, indoor playground, toys; $40K invested)</t>
+          <t>Gourmet Deli/Caterer, 100-yr Madison Ave deli liquidation (51 lots: Alto-Shaam ovens, Globe slicer, refrigerated deli cases/merchandisers, walk-in box, Metro racking)</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>business closing</t>
+          <t>restaurant closing</t>
         </is>
       </c>
       <c r="D44" s="13" t="inlineStr">
         <is>
-          <t>Long Island City</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="E44" s="13" t="inlineStr">
@@ -20614,23 +20610,27 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>$8,000 all</t>
+          <t>Live/online auction, prebidding open; 18% BP online</t>
         </is>
       </c>
       <c r="H44" s="15" t="n"/>
       <c r="I44" s="13" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="J44" s="13" t="inlineStr"/>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J44" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-27 02:00 PM ET</t>
+        </is>
+      </c>
       <c r="K44" s="13" t="inlineStr">
         <is>
-          <t>Craigslist (by owner)</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
       <c r="L44" s="13" t="inlineStr">
@@ -20646,7 +20646,7 @@
       </c>
       <c r="O44" s="14" t="inlineStr">
         <is>
-          <t>Off-category FYI; bulky, needs a truck.</t>
+          <t>Live webcast starts Tue Oct 27 2 PM ET; preview Oct 27 11 AM; checkout Wed Oct 28 10-5. Address released before auction. Shipping can be arranged at buyer's cost.</t>
         </is>
       </c>
     </row>
@@ -20658,17 +20658,17 @@
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>Kitchen store closing: sinks, faucets, hoods, vanities, counters, office stuff (mostly new in box)</t>
+          <t>Daycare/preschool closing: entire inventory of 4 classrooms (tables, cubbies, indoor playground, toys; $40K invested)</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>business closing</t>
         </is>
       </c>
       <c r="D45" s="13" t="inlineStr">
         <is>
-          <t>Brooklyn</t>
+          <t>Long Island City</t>
         </is>
       </c>
       <c r="E45" s="13" t="inlineStr">
@@ -20677,11 +20677,11 @@
         </is>
       </c>
       <c r="F45" s="13" t="n">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="G45" s="13" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>$8,000 all</t>
         </is>
       </c>
       <c r="H45" s="15" t="n"/>
@@ -20709,7 +20709,7 @@
       </c>
       <c r="O45" s="14" t="inlineStr">
         <is>
-          <t>Sheepshead Bay. Mostly new-in-box kitchen/bath fixtures; delivery available for large purchases. No prices posted.</t>
+          <t>Off-category FYI; bulky, needs a truck.</t>
         </is>
       </c>
     </row>
@@ -20721,17 +20721,17 @@
       </c>
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>Flooring company closed – pro tool package</t>
+          <t>Kitchen store closing: sinks, faucets, hoods, vanities, counters, office stuff (mostly new in box)</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>tools liquidation</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D46" s="13" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Brooklyn</t>
         </is>
       </c>
       <c r="E46" s="13" t="inlineStr">
@@ -20740,23 +20740,23 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>$1,000</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H46" s="15" t="n"/>
       <c r="I46" s="13" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J46" s="13" t="inlineStr"/>
       <c r="K46" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>Craigslist (by owner)</t>
         </is>
       </c>
       <c r="L46" s="13" t="inlineStr">
@@ -20772,7 +20772,7 @@
       </c>
       <c r="O46" s="14" t="inlineStr">
         <is>
-          <t>Flooring/construction company closed; pro tool package $1,000.</t>
+          <t>Sheepshead Bay. Mostly new-in-box kitchen/bath fixtures; delivery available for large purchases. No prices posted.</t>
         </is>
       </c>
     </row>
@@ -20784,12 +20784,12 @@
       </c>
       <c r="B47" s="14" t="inlineStr">
         <is>
-          <t>New-in-box commercial refrigeration lot – 10 Beverage-Air &amp; Perlick units (bar never opened)</t>
+          <t>Flooring company closed – pro tool package</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
         <is>
-          <t>commercial refrigeration lot</t>
+          <t>tools liquidation</t>
         </is>
       </c>
       <c r="D47" s="13" t="inlineStr">
@@ -20807,13 +20807,13 @@
       </c>
       <c r="G47" s="13" t="inlineStr">
         <is>
-          <t>$27,500 all 10 (or per unit $2,800–$4,150)</t>
+          <t>$1,000</t>
         </is>
       </c>
       <c r="H47" s="15" t="n"/>
       <c r="I47" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="J47" s="13" t="inlineStr"/>
@@ -20835,7 +20835,7 @@
       </c>
       <c r="O47" s="14" t="inlineStr">
         <is>
-          <t>Financial District. Never installed, factory packaging: 2 Beverage-Air HBF23HC-1-HS reach-in freezers ($4,150 ea), 3 HBR23HC-1-HS reach-in fridges ($3,550 ea), 1 UCR48AHC 48" undercounter ($2,800), 3 Perlick HC24FS4 glass frosters + 1 HC24RS4 beverage fridge ($2,850 ea). Seller says full retail $47,463 (about 42% off as a bundle). Updated Oct 14.</t>
+          <t>Flooring/construction company closed; pro tool package $1,000.</t>
         </is>
       </c>
     </row>
@@ -20847,46 +20847,42 @@
       </c>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>Corporate caterer – Alto-Shaam, new boxed Avantco rice cookers &amp; Cadco oven, Perlick, MerryChef</t>
+          <t>New-in-box commercial refrigeration lot – 10 Beverage-Air &amp; Perlick units (bar never opened)</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>commercial refrigeration lot</t>
         </is>
       </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>Jersey City</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="E48" s="13" t="inlineStr">
         <is>
-          <t>NJ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>$27,500 all 10 (or per unit $2,800–$4,150)</t>
         </is>
       </c>
       <c r="H48" s="15" t="n"/>
       <c r="I48" s="13" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="J48" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-05 07:00 PM ET</t>
-        </is>
-      </c>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="J48" s="13" t="inlineStr"/>
       <c r="K48" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L48" s="13" t="inlineStr">
@@ -20902,7 +20898,7 @@
       </c>
       <c r="O48" s="14" t="inlineStr">
         <is>
-          <t>Thu Oct 22 2 PM. [auto-removed 2026-10-22: closing date passed] | Rescheduled: live &amp; online Nov 5 (preview 11 AM, bidding closes 7 PM ET), 19 lots.</t>
+          <t>Financial District. Never installed, factory packaging: 2 Beverage-Air HBF23HC-1-HS reach-in freezers ($4,150 ea), 3 HBR23HC-1-HS reach-in fridges ($3,550 ea), 1 UCR48AHC 48" undercounter ($2,800), 3 Perlick HC24FS4 glass frosters + 1 HC24RS4 beverage fridge ($2,850 ea). Seller says full retail $47,463 (about 42% off as a bundle). Updated Oct 14.</t>
         </is>
       </c>
     </row>
@@ -20914,12 +20910,12 @@
       </c>
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>Lighting store closing – lease ended, up to 70% off showroom</t>
+          <t>Corporate caterer – Alto-Shaam, new boxed Avantco rice cookers &amp; Cadco oven, Perlick, MerryChef</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D49" s="13" t="inlineStr">
@@ -20937,19 +20933,23 @@
       </c>
       <c r="G49" s="13" t="inlineStr">
         <is>
-          <t>up to 70% off</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H49" s="15" t="n"/>
       <c r="I49" s="13" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="J49" s="13" t="inlineStr"/>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="J49" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-05 07:00 PM ET</t>
+        </is>
+      </c>
       <c r="K49" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
       <c r="L49" s="13" t="inlineStr">
@@ -20965,7 +20965,7 @@
       </c>
       <c r="O49" s="14" t="inlineStr">
         <is>
-          <t>Lighting store closing, lease ended. Showroom inventory up to 70% off.</t>
+          <t>Thu Oct 22 2 PM. [auto-removed 2026-10-22: closing date passed] | Rescheduled: live &amp; online Nov 5 (preview 11 AM, bidding closes 7 PM ET), 19 lots.</t>
         </is>
       </c>
     </row>
@@ -20977,12 +20977,12 @@
       </c>
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>Baonanas LLC ABC sale: turnkey ice cream / gelato / dessert shop equipment</t>
+          <t>Lighting store closing – lease ended, up to 70% off showroom</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>restaurant / commercial kitchen contents</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D50" s="13" t="inlineStr">
@@ -21000,15 +21000,19 @@
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>Accepting offers</t>
+          <t>up to 70% off</t>
         </is>
       </c>
       <c r="H50" s="15" t="n"/>
-      <c r="I50" s="13" t="inlineStr"/>
+      <c r="I50" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
       <c r="J50" s="13" t="inlineStr"/>
       <c r="K50" s="13" t="inlineStr">
         <is>
-          <t>AuctionAdvisors</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L50" s="13" t="inlineStr">
@@ -21024,7 +21028,7 @@
       </c>
       <c r="O50" s="14" t="inlineStr">
         <is>
-          <t>181 Monticello Ave. Assignment for the benefit of creditors. IFI Panorama gelato display cases, refrigerated topping stations, commercial mixers, refrigerators/freezers, stainless worktables, ice machine, POS, smallwares, gelato carts, catering gear, FF&amp;E.</t>
+          <t>Lighting store closing, lease ended. Showroom inventory up to 70% off.</t>
         </is>
       </c>
     </row>
@@ -21036,17 +21040,17 @@
       </c>
       <c r="B51" s="14" t="inlineStr">
         <is>
-          <t>Tools / plumbing / MRO supply inventory – Hilti/DeWalt/Milwaukee, fittings, heat pumps</t>
+          <t>Baonanas LLC ABC sale: turnkey ice cream / gelato / dessert shop equipment</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>restaurant / commercial kitchen contents</t>
         </is>
       </c>
       <c r="D51" s="13" t="inlineStr">
         <is>
-          <t>Riverdale</t>
+          <t>Jersey City</t>
         </is>
       </c>
       <c r="E51" s="13" t="inlineStr">
@@ -21055,23 +21059,19 @@
         </is>
       </c>
       <c r="F51" s="13" t="n">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="G51" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Accepting offers</t>
         </is>
       </c>
       <c r="H51" s="15" t="n"/>
       <c r="I51" s="13" t="inlineStr"/>
-      <c r="J51" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-30 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="J51" s="13" t="inlineStr"/>
       <c r="K51" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
+          <t>AuctionAdvisors</t>
         </is>
       </c>
       <c r="L51" s="13" t="inlineStr">
@@ -21087,7 +21087,7 @@
       </c>
       <c r="O51" s="14" t="inlineStr">
         <is>
-          <t>Bulk resale inventory.</t>
+          <t>181 Monticello Ave. Assignment for the benefit of creditors. IFI Panorama gelato display cases, refrigerated topping stations, commercial mixers, refrigerators/freezers, stainless worktables, ice machine, POS, smallwares, gelato carts, catering gear, FF&amp;E.</t>
         </is>
       </c>
     </row>
@@ -21099,12 +21099,12 @@
       </c>
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>Ice cream + cookie franchise equipment – Taylor soft-serve, Atosa, Blodgett</t>
+          <t>Tools / plumbing / MRO supply inventory – Hilti/DeWalt/Milwaukee, fittings, heat pumps</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>inventory</t>
         </is>
       </c>
       <c r="D52" s="13" t="inlineStr">
@@ -21129,7 +21129,7 @@
       <c r="I52" s="13" t="inlineStr"/>
       <c r="J52" s="13" t="inlineStr">
         <is>
-          <t>2026-11-05 11:00 AM ET</t>
+          <t>2026-10-30 11:00 AM ET</t>
         </is>
       </c>
       <c r="K52" s="13" t="inlineStr">
@@ -21150,7 +21150,7 @@
       </c>
       <c r="O52" s="14" t="inlineStr">
         <is>
-          <t>Resellable units.</t>
+          <t>Bulk resale inventory.</t>
         </is>
       </c>
     </row>
@@ -21162,17 +21162,17 @@
       </c>
       <c r="B53" s="14" t="inlineStr">
         <is>
-          <t>U.S. Vision court-ordered liquidation: ~70,000 designer eyeglass/sunglass frames + optical/optometry equipment at ~80 former stores + IP</t>
+          <t>Ice cream + cookie franchise equipment – Taylor soft-serve, Atosa, Blodgett</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>court-ordered retail chain liquidation</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D53" s="13" t="inlineStr">
         <is>
-          <t>Montclair</t>
+          <t>Riverdale</t>
         </is>
       </c>
       <c r="E53" s="13" t="inlineStr">
@@ -21181,19 +21181,23 @@
         </is>
       </c>
       <c r="F53" s="13" t="n">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G53" s="13" t="inlineStr">
         <is>
-          <t>Accepting offers (terms in offering memo, NDA required)</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H53" s="15" t="n"/>
       <c r="I53" s="13" t="inlineStr"/>
-      <c r="J53" s="13" t="inlineStr"/>
+      <c r="J53" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-05 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K53" s="13" t="inlineStr">
         <is>
-          <t>AuctionAdvisors</t>
+          <t>A.J. Willner</t>
         </is>
       </c>
       <c r="L53" s="13" t="inlineStr">
@@ -21209,7 +21213,7 @@
       </c>
       <c r="O53" s="14" t="inlineStr">
         <is>
-          <t>Three-lot sale pursuant to court order; bids accepted for individual lots, combinations, or substantially all assets. Equipment is spread across ~80 former store locations. Not appliance-related; big-ticket bulk inventory play.</t>
+          <t>Resellable units.</t>
         </is>
       </c>
     </row>
@@ -21221,17 +21225,17 @@
       </c>
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>Wascomat commercial washers liquidation (22× W105, 6× W185, dryer panels)</t>
+          <t>U.S. Vision court-ordered liquidation: ~70,000 designer eyeglass/sunglass frames + optical/optometry equipment at ~80 former stores + IP</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>commercial laundry</t>
+          <t>court-ordered retail chain liquidation</t>
         </is>
       </c>
       <c r="D54" s="13" t="inlineStr">
         <is>
-          <t>Newark</t>
+          <t>Montclair</t>
         </is>
       </c>
       <c r="E54" s="13" t="inlineStr">
@@ -21240,23 +21244,19 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>$500–$800 each / panels $150</t>
+          <t>Accepting offers (terms in offering memo, NDA required)</t>
         </is>
       </c>
       <c r="H54" s="15" t="n"/>
-      <c r="I54" s="13" t="inlineStr">
-        <is>
-          <t>2026-07-12</t>
-        </is>
-      </c>
+      <c r="I54" s="13" t="inlineStr"/>
       <c r="J54" s="13" t="inlineStr"/>
       <c r="K54" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>AuctionAdvisors</t>
         </is>
       </c>
       <c r="L54" s="13" t="inlineStr">
@@ -21272,7 +21272,7 @@
       </c>
       <c r="O54" s="14" t="inlineStr">
         <is>
-          <t>22× W105 @ $500, 6× W185 @ $800, 20 dryer panels $150. Commercial laundry liquidation.</t>
+          <t>Three-lot sale pursuant to court order; bids accepted for individual lots, combinations, or substantially all assets. Equipment is spread across ~80 former store locations. Not appliance-related; big-ticket bulk inventory play.</t>
         </is>
       </c>
     </row>
@@ -21284,17 +21284,17 @@
       </c>
       <c r="B55" s="14" t="inlineStr">
         <is>
-          <t>Major food-service caterer – new-in-box True reach-ins, Beverage-Air, TurboChef, Resfab ventless fryer</t>
+          <t>Wascomat commercial washers liquidation (22× W105, 6× W185, dryer panels)</t>
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>commercial laundry</t>
         </is>
       </c>
       <c r="D55" s="13" t="inlineStr">
         <is>
-          <t>Parsippany</t>
+          <t>Newark</t>
         </is>
       </c>
       <c r="E55" s="13" t="inlineStr">
@@ -21303,27 +21303,23 @@
         </is>
       </c>
       <c r="F55" s="13" t="n">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="G55" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>$500–$800 each / panels $150</t>
         </is>
       </c>
       <c r="H55" s="15" t="n"/>
       <c r="I55" s="13" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="J55" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-03 02:00 PM ET</t>
-        </is>
-      </c>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="J55" s="13" t="inlineStr"/>
       <c r="K55" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L55" s="13" t="inlineStr">
@@ -21339,7 +21335,7 @@
       </c>
       <c r="O55" s="14" t="inlineStr">
         <is>
-          <t>Tue Nov 3 2 PM, checkout Nov 4.</t>
+          <t>22× W105 @ $500, 6× W185 @ $800, 20 dryer panels $150. Commercial laundry liquidation.</t>
         </is>
       </c>
     </row>
@@ -21351,17 +21347,17 @@
       </c>
       <c r="B56" s="14" t="inlineStr">
         <is>
-          <t>Business closing – 160 new Carnes exhaust fans</t>
+          <t>Major food-service caterer – new-in-box True reach-ins, Beverage-Air, TurboChef, Resfab ventless fryer</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>HVAC inventory</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D56" s="13" t="inlineStr">
         <is>
-          <t>Kenilworth</t>
+          <t>Parsippany</t>
         </is>
       </c>
       <c r="E56" s="13" t="inlineStr">
@@ -21374,19 +21370,23 @@
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>$40 each or $5,000 all OBO</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H56" s="15" t="n"/>
       <c r="I56" s="13" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="J56" s="13" t="inlineStr"/>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="J56" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-03 02:00 PM ET</t>
+        </is>
+      </c>
       <c r="K56" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
       <c r="L56" s="13" t="inlineStr">
@@ -21402,7 +21402,7 @@
       </c>
       <c r="O56" s="14" t="inlineStr">
         <is>
-          <t>160 new Carnes 80CFM 1.0 sone exhaust fans. $40 each or $5,000 for all OBO. Business closing HVAC inventory.</t>
+          <t>Tue Nov 3 2 PM, checkout Nov 4.</t>
         </is>
       </c>
     </row>
@@ -21414,12 +21414,12 @@
       </c>
       <c r="B57" s="14" t="inlineStr">
         <is>
-          <t>Air Systems Inc – sheet metal / HVAC fabrication shop liquidation</t>
+          <t>Business closing – 160 new Carnes exhaust fans</t>
         </is>
       </c>
       <c r="C57" s="13" t="inlineStr">
         <is>
-          <t>HVAC shop liquidation</t>
+          <t>HVAC inventory</t>
         </is>
       </c>
       <c r="D57" s="13" t="inlineStr">
@@ -21437,19 +21437,19 @@
       </c>
       <c r="G57" s="13" t="inlineStr">
         <is>
-          <t>Timed online (15% BP)</t>
+          <t>$40 each or $5,000 all OBO</t>
         </is>
       </c>
       <c r="H57" s="15" t="n"/>
-      <c r="I57" s="13" t="inlineStr"/>
-      <c r="J57" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-29 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="I57" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="J57" s="13" t="inlineStr"/>
       <c r="K57" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner Auctions</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L57" s="13" t="inlineStr">
@@ -21465,7 +21465,7 @@
       </c>
       <c r="O57" s="14" t="inlineStr">
         <is>
-          <t>Vicon HVAC plasma; Flagler/Lockformer/Roto-Die/Engel fab; welders; Clark forklift; Genie Superlift; Ridgid/Milwaukee/DeWalt/Bosch/Hilti/Makita tools; AeroVent/Carnes exhaust fans; racking/scaffolding. Preview Oct 28–29 AM; pickup Oct 29 PM–Nov 4. Same town as Carnes fan CL lot.</t>
+          <t>160 new Carnes 80CFM 1.0 sone exhaust fans. $40 each or $5,000 for all OBO. Business closing HVAC inventory.</t>
         </is>
       </c>
     </row>
@@ -21477,17 +21477,17 @@
       </c>
       <c r="B58" s="14" t="inlineStr">
         <is>
-          <t>Former Rush Bowls franchise ABC sale: commercial refrigeration, Vitamix blenders, ice &amp; beverage equipment</t>
+          <t>Air Systems Inc – sheet metal / HVAC fabrication shop liquidation</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>restaurant / commercial kitchen contents</t>
+          <t>HVAC shop liquidation</t>
         </is>
       </c>
       <c r="D58" s="13" t="inlineStr">
         <is>
-          <t>Westfield</t>
+          <t>Kenilworth</t>
         </is>
       </c>
       <c r="E58" s="13" t="inlineStr">
@@ -21496,19 +21496,23 @@
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="G58" s="13" t="inlineStr">
         <is>
-          <t>Accepting offers</t>
+          <t>Timed online (15% BP)</t>
         </is>
       </c>
       <c r="H58" s="15" t="n"/>
       <c r="I58" s="13" t="inlineStr"/>
-      <c r="J58" s="13" t="inlineStr"/>
+      <c r="J58" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-29 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K58" s="13" t="inlineStr">
         <is>
-          <t>AuctionAdvisors</t>
+          <t>A.J. Willner Auctions</t>
         </is>
       </c>
       <c r="L58" s="13" t="inlineStr">
@@ -21524,7 +21528,7 @@
       </c>
       <c r="O58" s="14" t="inlineStr">
         <is>
-          <t>27 East Broad St. Assignment for the benefit of creditors of 333 Star Enterprises (d/b/a Rush Bowls). Commercial refrigeration/freezers, Vitamix blenders, stainless workstations/sinks, ice and beverage equipment, POS, shelving. Inspection by contacting the auctioneer.</t>
+          <t>Vicon HVAC plasma; Flagler/Lockformer/Roto-Die/Engel fab; welders; Clark forklift; Genie Superlift; Ridgid/Milwaukee/DeWalt/Bosch/Hilti/Makita tools; AeroVent/Carnes exhaust fans; racking/scaffolding. Preview Oct 28–29 AM; pickup Oct 29 PM–Nov 4. Same town as Carnes fan CL lot.</t>
         </is>
       </c>
     </row>
@@ -21536,17 +21540,17 @@
       </c>
       <c r="B59" s="14" t="inlineStr">
         <is>
-          <t>Bimmer Clinic business liquidation (BMW repair shop): vehicle lifts, forklift, skid steer, refrigerant recovery, shop tools &amp; equipment</t>
+          <t>Former Rush Bowls franchise ABC sale: commercial refrigeration, Vitamix blenders, ice &amp; beverage equipment</t>
         </is>
       </c>
       <c r="C59" s="13" t="inlineStr">
         <is>
-          <t>business liquidation auction</t>
+          <t>restaurant / commercial kitchen contents</t>
         </is>
       </c>
       <c r="D59" s="13" t="inlineStr">
         <is>
-          <t>South Amboy</t>
+          <t>Westfield</t>
         </is>
       </c>
       <c r="E59" s="13" t="inlineStr">
@@ -21555,23 +21559,19 @@
         </is>
       </c>
       <c r="F59" s="13" t="n">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="G59" s="13" t="inlineStr">
         <is>
-          <t>Timed online auction</t>
+          <t>Accepting offers</t>
         </is>
       </c>
       <c r="H59" s="15" t="n"/>
       <c r="I59" s="13" t="inlineStr"/>
-      <c r="J59" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-12 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="J59" s="13" t="inlineStr"/>
       <c r="K59" s="13" t="inlineStr">
         <is>
-          <t>AJ Willner Auctions</t>
+          <t>AuctionAdvisors</t>
         </is>
       </c>
       <c r="L59" s="13" t="inlineStr">
@@ -21587,7 +21587,7 @@
       </c>
       <c r="O59" s="14" t="inlineStr">
         <is>
-          <t>Ends Nov 12 11 AM EST.</t>
+          <t>27 East Broad St. Assignment for the benefit of creditors of 333 Star Enterprises (d/b/a Rush Bowls). Commercial refrigeration/freezers, Vitamix blenders, stainless workstations/sinks, ice and beverage equipment, POS, shelving. Inspection by contacting the auctioneer.</t>
         </is>
       </c>
     </row>
@@ -21599,17 +21599,17 @@
       </c>
       <c r="B60" s="14" t="inlineStr">
         <is>
-          <t>Drywall &amp; Acoustical Contractor 2: Hilti tools, material handling, supplies (Ideal Trading Corp)</t>
+          <t>Bimmer Clinic business liquidation (BMW repair shop): vehicle lifts, forklift, skid steer, refrigerant recovery, shop tools &amp; equipment</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>business liquidation auction</t>
         </is>
       </c>
       <c r="D60" s="13" t="inlineStr">
         <is>
-          <t>Randolph</t>
+          <t>South Amboy</t>
         </is>
       </c>
       <c r="E60" s="13" t="inlineStr">
@@ -21618,23 +21618,23 @@
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G60" s="13" t="inlineStr">
         <is>
-          <t>Online auction (HiBid terms)</t>
+          <t>Timed online auction</t>
         </is>
       </c>
       <c r="H60" s="15" t="n"/>
       <c r="I60" s="13" t="inlineStr"/>
       <c r="J60" s="13" t="inlineStr">
         <is>
-          <t>2026-10-28 11:00 AM ET</t>
+          <t>2026-11-12 11:00 AM ET</t>
         </is>
       </c>
       <c r="K60" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Ideal Trading Corp)</t>
+          <t>AJ Willner Auctions</t>
         </is>
       </c>
       <c r="L60" s="13" t="inlineStr">
@@ -21650,7 +21650,7 @@
       </c>
       <c r="O60" s="14" t="inlineStr">
         <is>
-          <t>Contractor contents; closes Oct 28 11 AM. Hilti tools resell well on eBay.</t>
+          <t>Ends Nov 12 11 AM EST.</t>
         </is>
       </c>
     </row>
@@ -21662,17 +21662,17 @@
       </c>
       <c r="B61" s="14" t="inlineStr">
         <is>
-          <t>New modular concession kitchens (warehouseman's lien) – 5 units, CaptiveAire hoods, new Ovention/Turbo Air</t>
+          <t>Drywall &amp; Acoustical Contractor 2: Hilti tools, material handling, supplies (Ideal Trading Corp)</t>
         </is>
       </c>
       <c r="C61" s="13" t="inlineStr">
         <is>
-          <t>lien sale</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D61" s="13" t="inlineStr">
         <is>
-          <t>Edison</t>
+          <t>Randolph</t>
         </is>
       </c>
       <c r="E61" s="13" t="inlineStr">
@@ -21681,19 +21681,23 @@
         </is>
       </c>
       <c r="F61" s="13" t="n">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="G61" s="13" t="inlineStr">
         <is>
-          <t>Online auction, $2K load-out fee</t>
+          <t>Online auction (HiBid terms)</t>
         </is>
       </c>
       <c r="H61" s="15" t="n"/>
       <c r="I61" s="13" t="inlineStr"/>
-      <c r="J61" s="13" t="inlineStr"/>
+      <c r="J61" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-28 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K61" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
+          <t>HiBid (Ideal Trading Corp)</t>
         </is>
       </c>
       <c r="L61" s="13" t="inlineStr">
@@ -21709,7 +21713,7 @@
       </c>
       <c r="O61" s="14" t="inlineStr">
         <is>
-          <t>&gt;$100K new. Close date not captured.</t>
+          <t>Contractor contents; closes Oct 28 11 AM. Hilti tools resell well on eBay.</t>
         </is>
       </c>
     </row>
@@ -21721,12 +21725,12 @@
       </c>
       <c r="B62" s="14" t="inlineStr">
         <is>
-          <t>Brand-new &amp; scratch-and-dent kitchen/home appliances – ~185 lots (Thermador, GE Café, Miele, Wolf speed oven, Viking, Bosch…)</t>
+          <t>New modular concession kitchens (warehouseman's lien) – 5 units, CaptiveAire hoods, new Ovention/Turbo Air</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>lien sale</t>
         </is>
       </c>
       <c r="D62" s="13" t="inlineStr">
@@ -21744,35 +21748,23 @@
       </c>
       <c r="G62" s="13" t="inlineStr">
         <is>
-          <t>Live + HiBid webcast, 18% BP + 3% card</t>
+          <t>Online auction, $2K load-out fee</t>
         </is>
       </c>
       <c r="H62" s="15" t="n"/>
-      <c r="I62" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="J62" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-25 01:00 PM ET</t>
-        </is>
-      </c>
+      <c r="I62" s="13" t="inlineStr"/>
+      <c r="J62" s="13" t="inlineStr"/>
       <c r="K62" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
-        </is>
-      </c>
-      <c r="L62" s="21" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
-        </is>
-      </c>
-      <c r="M62" s="20" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
+          <t>A.J. Willner</t>
+        </is>
+      </c>
+      <c r="L62" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M62" s="13" t="inlineStr"/>
       <c r="N62" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -21780,7 +21772,7 @@
       </c>
       <c r="O62" s="14" t="inlineStr">
         <is>
-          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale.</t>
+          <t>&gt;$100K new. Close date not captured.</t>
         </is>
       </c>
     </row>
@@ -21792,17 +21784,17 @@
       </c>
       <c r="B63" s="14" t="inlineStr">
         <is>
-          <t>Party City (Ch. 11) store – fixtures + party merchandise inventory</t>
+          <t>Brand-new &amp; scratch-and-dent kitchen/home appliances – ~185 lots (Thermador, GE Café, Miele, Wolf speed oven, Viking, Bosch…)</t>
         </is>
       </c>
       <c r="C63" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D63" s="13" t="inlineStr">
         <is>
-          <t>East Brunswick</t>
+          <t>Edison</t>
         </is>
       </c>
       <c r="E63" s="13" t="inlineStr">
@@ -21811,31 +21803,39 @@
         </is>
       </c>
       <c r="F63" s="13" t="n">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="G63" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Live + HiBid webcast, 18% BP + 3% card</t>
         </is>
       </c>
       <c r="H63" s="15" t="n"/>
-      <c r="I63" s="13" t="inlineStr"/>
+      <c r="I63" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
       <c r="J63" s="13" t="inlineStr">
         <is>
-          <t>2026-11-03 11:00 AM ET</t>
+          <t>2026-10-25 01:00 PM ET</t>
         </is>
       </c>
       <c r="K63" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
-        </is>
-      </c>
-      <c r="L63" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M63" s="13" t="inlineStr"/>
+          <t>HiBid (Best Buy Auctioneers)</t>
+        </is>
+      </c>
+      <c r="L63" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M63" s="20" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
       <c r="N63" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -21843,7 +21843,7 @@
       </c>
       <c r="O63" s="14" t="inlineStr">
         <is>
-          <t>Store inventory.</t>
+          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale.</t>
         </is>
       </c>
     </row>
@@ -21855,17 +21855,17 @@
       </c>
       <c r="B64" s="14" t="inlineStr">
         <is>
-          <t>Bakery/Cafe Somerville NJ – rack ovens, La Marzocco, food truck (~76 lots)</t>
+          <t>Party City (Ch. 11) store – fixtures + party merchandise inventory</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D64" s="13" t="inlineStr">
         <is>
-          <t>Somerville</t>
+          <t>East Brunswick</t>
         </is>
       </c>
       <c r="E64" s="13" t="inlineStr">
@@ -21874,27 +21874,23 @@
         </is>
       </c>
       <c r="F64" s="13" t="n">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="G64" s="13" t="inlineStr">
         <is>
-          <t>Live webcast + online (18% BP online)</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H64" s="15" t="n"/>
-      <c r="I64" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
+      <c r="I64" s="13" t="inlineStr"/>
       <c r="J64" s="13" t="inlineStr">
         <is>
-          <t>2026-10-26 02:00 PM ET</t>
+          <t>2026-11-03 11:00 AM ET</t>
         </is>
       </c>
       <c r="K64" s="13" t="inlineStr">
         <is>
-          <t>HiBid / Best Buy Auctioneers</t>
+          <t>A.J. Willner</t>
         </is>
       </c>
       <c r="L64" s="13" t="inlineStr">
@@ -21910,7 +21906,7 @@
       </c>
       <c r="O64" s="14" t="inlineStr">
         <is>
-          <t>Full bakery/cafe commercial kitchen: food truck w/ pizza oven, La Marzocco espresso, Mazzer, Baxter + Empire Logiudice rack ovens, dough depositor, Globe floor mixer, Artic Air / SS refrigeration, fryers, Vitamix, Robot Coupe, display cases, dining furniture. Preview 11 AM sale day; checkout Tue 10/27.</t>
+          <t>Store inventory.</t>
         </is>
       </c>
     </row>
@@ -21922,7 +21918,7 @@
       </c>
       <c r="B65" s="14" t="inlineStr">
         <is>
-          <t>Ability to Work kitchen and store – commercial kitchen + store fixtures (~135 lots)</t>
+          <t>Bakery/Cafe Somerville NJ – rack ovens, La Marzocco, food truck (~76 lots)</t>
         </is>
       </c>
       <c r="C65" s="13" t="inlineStr">
@@ -21932,7 +21928,7 @@
       </c>
       <c r="D65" s="13" t="inlineStr">
         <is>
-          <t>Flemington</t>
+          <t>Somerville</t>
         </is>
       </c>
       <c r="E65" s="13" t="inlineStr">
@@ -21941,23 +21937,27 @@
         </is>
       </c>
       <c r="F65" s="13" t="n">
-        <v>237</v>
+        <v>224</v>
       </c>
       <c r="G65" s="13" t="inlineStr">
         <is>
-          <t>Timed online (15% BP)</t>
+          <t>Live webcast + online (18% BP online)</t>
         </is>
       </c>
       <c r="H65" s="15" t="n"/>
-      <c r="I65" s="13" t="inlineStr"/>
+      <c r="I65" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
       <c r="J65" s="13" t="inlineStr">
         <is>
-          <t>2026-10-27 11:02 AM ET</t>
+          <t>2026-10-26 02:00 PM ET</t>
         </is>
       </c>
       <c r="K65" s="13" t="inlineStr">
         <is>
-          <t>HiBid</t>
+          <t>HiBid / Best Buy Auctioneers</t>
         </is>
       </c>
       <c r="L65" s="13" t="inlineStr">
@@ -21973,7 +21973,7 @@
       </c>
       <c r="O65" s="14" t="inlineStr">
         <is>
-          <t>Apprentice/hospitality training cafe-kitchen and store dispersal. Preview 9–11 AM sale day; removal Oct 27 noon–Oct 29.</t>
+          <t>Full bakery/cafe commercial kitchen: food truck w/ pizza oven, La Marzocco espresso, Mazzer, Baxter + Empire Logiudice rack ovens, dough depositor, Globe floor mixer, Artic Air / SS refrigeration, fryers, Vitamix, Robot Coupe, display cases, dining furniture. Preview 11 AM sale day; checkout Tue 10/27.</t>
         </is>
       </c>
     </row>
@@ -21985,17 +21985,17 @@
       </c>
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>Wren Kitchens showroom closing – JennAir/Café/KitchenAid/GE Profile appliances + display kitchens</t>
+          <t>Ability to Work kitchen and store – commercial kitchen + store fixtures (~135 lots)</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>showroom closing</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D66" s="13" t="inlineStr">
         <is>
-          <t>Lawrenceville</t>
+          <t>Flemington</t>
         </is>
       </c>
       <c r="E66" s="13" t="inlineStr">
@@ -22004,23 +22004,23 @@
         </is>
       </c>
       <c r="F66" s="13" t="n">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="G66" s="13" t="inlineStr">
         <is>
-          <t>Online auction, 18% BP</t>
+          <t>Timed online (15% BP)</t>
         </is>
       </c>
       <c r="H66" s="15" t="n"/>
       <c r="I66" s="13" t="inlineStr"/>
       <c r="J66" s="13" t="inlineStr">
         <is>
-          <t>2026-10-27 09:00 AM ET</t>
+          <t>2026-10-27 11:02 AM ET</t>
         </is>
       </c>
       <c r="K66" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
+          <t>HiBid</t>
         </is>
       </c>
       <c r="L66" s="13" t="inlineStr">
@@ -22036,7 +22036,7 @@
       </c>
       <c r="O66" s="14" t="inlineStr">
         <is>
-          <t>Premium floor-model appliances; lots close from Oct 27 9 AM.</t>
+          <t>Apprentice/hospitality training cafe-kitchen and store dispersal. Preview 9–11 AM sale day; removal Oct 27 noon–Oct 29.</t>
         </is>
       </c>
     </row>
@@ -22048,7 +22048,7 @@
       </c>
       <c r="B67" s="14" t="inlineStr">
         <is>
-          <t>Wren Kitchens showroom closing – GE/Whirlpool/KitchenAid/Café incl. NIB Café range + 35 kitchens</t>
+          <t>Wren Kitchens showroom closing – JennAir/Café/KitchenAid/GE Profile appliances + display kitchens</t>
         </is>
       </c>
       <c r="C67" s="13" t="inlineStr">
@@ -22058,7 +22058,7 @@
       </c>
       <c r="D67" s="13" t="inlineStr">
         <is>
-          <t>Cherry Hill</t>
+          <t>Lawrenceville</t>
         </is>
       </c>
       <c r="E67" s="13" t="inlineStr">
@@ -22067,18 +22067,18 @@
         </is>
       </c>
       <c r="F67" s="13" t="n">
-        <v>266</v>
+        <v>239</v>
       </c>
       <c r="G67" s="13" t="inlineStr">
         <is>
-          <t>Online auction, openers ~$0.50</t>
+          <t>Online auction, 18% BP</t>
         </is>
       </c>
       <c r="H67" s="15" t="n"/>
       <c r="I67" s="13" t="inlineStr"/>
       <c r="J67" s="13" t="inlineStr">
         <is>
-          <t>2026-11-02 11:00 AM ET</t>
+          <t>2026-10-27 09:00 AM ET</t>
         </is>
       </c>
       <c r="K67" s="13" t="inlineStr">
@@ -22099,124 +22099,120 @@
       </c>
       <c r="O67" s="14" t="inlineStr">
         <is>
+          <t>Premium floor-model appliances; lots close from Oct 27 9 AM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" outlineLevel="1">
+      <c r="A68" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B68" s="14" t="inlineStr">
+        <is>
+          <t>Wren Kitchens showroom closing – GE/Whirlpool/KitchenAid/Café incl. NIB Café range + 35 kitchens</t>
+        </is>
+      </c>
+      <c r="C68" s="13" t="inlineStr">
+        <is>
+          <t>showroom closing</t>
+        </is>
+      </c>
+      <c r="D68" s="13" t="inlineStr">
+        <is>
+          <t>Cherry Hill</t>
+        </is>
+      </c>
+      <c r="E68" s="13" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="F68" s="13" t="n">
+        <v>266</v>
+      </c>
+      <c r="G68" s="13" t="inlineStr">
+        <is>
+          <t>Online auction, openers ~$0.50</t>
+        </is>
+      </c>
+      <c r="H68" s="15" t="n"/>
+      <c r="I68" s="13" t="inlineStr"/>
+      <c r="J68" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-02 11:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K68" s="13" t="inlineStr">
+        <is>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L68" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M68" s="13" t="inlineStr"/>
+      <c r="N68" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O68" s="14" t="inlineStr">
+        <is>
           <t>Lots close from Nov 2 11 AM.</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="17" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="17" t="inlineStr">
         <is>
           <t>Subtotal — NYC / Long Island / NJ</t>
         </is>
       </c>
-      <c r="B68" s="17" t="inlineStr">
+      <c r="B69" s="17" t="inlineStr">
         <is>
           <t>26 item(s)</t>
         </is>
       </c>
-      <c r="C68" s="18" t="n"/>
-      <c r="D68" s="18" t="n"/>
-      <c r="E68" s="18" t="n"/>
-      <c r="F68" s="18" t="n"/>
-      <c r="G68" s="18" t="n"/>
-      <c r="H68" s="19" t="n">
+      <c r="C69" s="18" t="n"/>
+      <c r="D69" s="18" t="n"/>
+      <c r="E69" s="18" t="n"/>
+      <c r="F69" s="18" t="n"/>
+      <c r="G69" s="18" t="n"/>
+      <c r="H69" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I68" s="18" t="n"/>
-      <c r="J68" s="18" t="n"/>
-      <c r="K68" s="18" t="n"/>
-      <c r="L68" s="18" t="n"/>
-      <c r="M68" s="18" t="n"/>
-      <c r="N68" s="18" t="n"/>
-      <c r="O68" s="18" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="11" t="inlineStr">
-        <is>
-          <t>▸ Eastern PA / Mid-Atlantic  (2)</t>
-        </is>
-      </c>
-      <c r="B69" s="12" t="n"/>
-      <c r="C69" s="12" t="n"/>
-      <c r="D69" s="12" t="n"/>
-      <c r="E69" s="12" t="n"/>
-      <c r="F69" s="12" t="n"/>
-      <c r="G69" s="12" t="n"/>
-      <c r="H69" s="12" t="n"/>
-      <c r="I69" s="12" t="n"/>
-      <c r="J69" s="12" t="n"/>
-      <c r="K69" s="12" t="n"/>
-      <c r="L69" s="12" t="n"/>
-      <c r="M69" s="12" t="n"/>
-      <c r="N69" s="12" t="n"/>
-      <c r="O69" s="12" t="n"/>
-    </row>
-    <row r="70" outlineLevel="1">
-      <c r="A70" s="13" t="inlineStr">
-        <is>
-          <t>Eastern PA / Mid-Atlantic</t>
-        </is>
-      </c>
-      <c r="B70" s="14" t="inlineStr">
-        <is>
-          <t>Piscitello's Home Center closing after 68 years: storewide 20% off liquidation (hardware, lumber, doors, windows, kitchen/bath)</t>
-        </is>
-      </c>
-      <c r="C70" s="13" t="inlineStr">
-        <is>
-          <t>store closing</t>
-        </is>
-      </c>
-      <c r="D70" s="13" t="inlineStr">
-        <is>
-          <t>Wilson</t>
-        </is>
-      </c>
-      <c r="E70" s="13" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="F70" s="13" t="n">
-        <v>250</v>
-      </c>
-      <c r="G70" s="13" t="inlineStr">
-        <is>
-          <t>20% off storewide (all sales final)</t>
-        </is>
-      </c>
-      <c r="H70" s="15" t="n"/>
-      <c r="I70" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="J70" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-30 06:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K70" s="13" t="inlineStr">
-        <is>
-          <t>LehighValley.com article</t>
-        </is>
-      </c>
-      <c r="L70" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M70" s="13" t="inlineStr"/>
-      <c r="N70" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O70" s="14" t="inlineStr">
-        <is>
-          <t>2300 Wood Ave, Wilson Borough (Easton area). Final day Oct 30. Retail-floor sale, not a bulk lot; ask in person about buying remaining stock outright.</t>
-        </is>
-      </c>
+      <c r="I69" s="18" t="n"/>
+      <c r="J69" s="18" t="n"/>
+      <c r="K69" s="18" t="n"/>
+      <c r="L69" s="18" t="n"/>
+      <c r="M69" s="18" t="n"/>
+      <c r="N69" s="18" t="n"/>
+      <c r="O69" s="18" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="inlineStr">
+        <is>
+          <t>▸ Eastern PA / Mid-Atlantic  (3)</t>
+        </is>
+      </c>
+      <c r="B70" s="12" t="n"/>
+      <c r="C70" s="12" t="n"/>
+      <c r="D70" s="12" t="n"/>
+      <c r="E70" s="12" t="n"/>
+      <c r="F70" s="12" t="n"/>
+      <c r="G70" s="12" t="n"/>
+      <c r="H70" s="12" t="n"/>
+      <c r="I70" s="12" t="n"/>
+      <c r="J70" s="12" t="n"/>
+      <c r="K70" s="12" t="n"/>
+      <c r="L70" s="12" t="n"/>
+      <c r="M70" s="12" t="n"/>
+      <c r="N70" s="12" t="n"/>
+      <c r="O70" s="12" t="n"/>
     </row>
     <row r="71" outlineLevel="1">
       <c r="A71" s="13" t="inlineStr">
@@ -22226,17 +22222,17 @@
       </c>
       <c r="B71" s="14" t="inlineStr">
         <is>
-          <t>Victorino's Pizzeria + Subway sub shop + brand-new scratch &amp; dent restaurant equipment (Marsal pizza oven, True merchandisers, Vulcan/Migali fryers, Stoelting soft-serve)</t>
+          <t>Piscitello's Home Center closing after 68 years: storewide 20% off liquidation (hardware, lumber, doors, windows, kitchen/bath)</t>
         </is>
       </c>
       <c r="C71" s="13" t="inlineStr">
         <is>
-          <t>restaurant closing</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D71" s="13" t="inlineStr">
         <is>
-          <t>Manheim</t>
+          <t>Wilson</t>
         </is>
       </c>
       <c r="E71" s="13" t="inlineStr">
@@ -22245,27 +22241,27 @@
         </is>
       </c>
       <c r="F71" s="13" t="n">
-        <v>320</v>
+        <v>250</v>
       </c>
       <c r="G71" s="13" t="inlineStr">
         <is>
-          <t>Online auction, items being added</t>
+          <t>20% off storewide (all sales final)</t>
         </is>
       </c>
       <c r="H71" s="15" t="n"/>
       <c r="I71" s="13" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="J71" s="13" t="inlineStr">
         <is>
-          <t>2026-11-05 08:00 PM ET</t>
+          <t>2026-10-30 06:00 PM ET</t>
         </is>
       </c>
       <c r="K71" s="13" t="inlineStr">
         <is>
-          <t>PCI Auctions East Coast</t>
+          <t>LehighValley.com article</t>
         </is>
       </c>
       <c r="L71" s="13" t="inlineStr">
@@ -22281,879 +22277,1013 @@
       </c>
       <c r="O71" s="14" t="inlineStr">
         <is>
+          <t>2300 Wood Ave, Wilson Borough (Easton area). Final day Oct 30. Retail-floor sale, not a bulk lot; ask in person about buying remaining stock outright.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" outlineLevel="1">
+      <c r="A72" s="13" t="inlineStr">
+        <is>
+          <t>Eastern PA / Mid-Atlantic</t>
+        </is>
+      </c>
+      <c r="B72" s="14" t="inlineStr">
+        <is>
+          <t>Limerick Hardware inventory liquidation (Alderfer, online-only)</t>
+        </is>
+      </c>
+      <c r="C72" s="13" t="inlineStr">
+        <is>
+          <t>store closing</t>
+        </is>
+      </c>
+      <c r="D72" s="13" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="E72" s="13" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="F72" s="13" t="n">
+        <v>277</v>
+      </c>
+      <c r="G72" s="13" t="inlineStr">
+        <is>
+          <t>Online auction, no reserve info</t>
+        </is>
+      </c>
+      <c r="H72" s="15" t="n"/>
+      <c r="I72" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="J72" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-02 08:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K72" s="13" t="inlineStr">
+        <is>
+          <t>Alderfer Auction</t>
+        </is>
+      </c>
+      <c r="L72" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M72" s="13" t="inlineStr"/>
+      <c r="N72" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O72" s="14" t="inlineStr">
+        <is>
+          <t>Hardware store inventory: Hillman fasteners/cabinets, DeWalt/Paslode tools, plumbing/electrical (Moen, Watts), Traeger/Weber/Broil King grills, Toro TimeCutter zero-turn, Wesco pallet jack, Lozier shelving, checkouts. Preview by appointment Fri Oct 30 1-3PM. Begins closing Nov 2 8PM EST.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" outlineLevel="1">
+      <c r="A73" s="13" t="inlineStr">
+        <is>
+          <t>Eastern PA / Mid-Atlantic</t>
+        </is>
+      </c>
+      <c r="B73" s="14" t="inlineStr">
+        <is>
+          <t>Victorino's Pizzeria + Subway sub shop + brand-new scratch &amp; dent restaurant equipment (Marsal pizza oven, True merchandisers, Vulcan/Migali fryers, Stoelting soft-serve)</t>
+        </is>
+      </c>
+      <c r="C73" s="13" t="inlineStr">
+        <is>
+          <t>restaurant closing</t>
+        </is>
+      </c>
+      <c r="D73" s="13" t="inlineStr">
+        <is>
+          <t>Manheim</t>
+        </is>
+      </c>
+      <c r="E73" s="13" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="F73" s="13" t="n">
+        <v>320</v>
+      </c>
+      <c r="G73" s="13" t="inlineStr">
+        <is>
+          <t>Online auction, items being added</t>
+        </is>
+      </c>
+      <c r="H73" s="15" t="n"/>
+      <c r="I73" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="J73" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-05 08:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K73" s="13" t="inlineStr">
+        <is>
+          <t>PCI Auctions East Coast</t>
+        </is>
+      </c>
+      <c r="L73" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M73" s="13" t="inlineStr"/>
+      <c r="N73" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O73" s="14" t="inlineStr">
+        <is>
           <t>Ends Thu Nov 5 8 PM EST. PCI East Coast warehouse, 141 W End Dr, Manheim PA. Preview Wed Nov 4 10-2; removal Fri Nov 6 10-4. Shipping/delivery available.</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="17" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Eastern PA / Mid-Atlantic</t>
         </is>
       </c>
-      <c r="B72" s="17" t="inlineStr">
+      <c r="B74" s="17" t="inlineStr">
+        <is>
+          <t>3 item(s)</t>
+        </is>
+      </c>
+      <c r="C74" s="18" t="n"/>
+      <c r="D74" s="18" t="n"/>
+      <c r="E74" s="18" t="n"/>
+      <c r="F74" s="18" t="n"/>
+      <c r="G74" s="18" t="n"/>
+      <c r="H74" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I74" s="18" t="n"/>
+      <c r="J74" s="18" t="n"/>
+      <c r="K74" s="18" t="n"/>
+      <c r="L74" s="18" t="n"/>
+      <c r="M74" s="18" t="n"/>
+      <c r="N74" s="18" t="n"/>
+      <c r="O74" s="18" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="11" t="inlineStr">
+        <is>
+          <t>▸ Western PA / Ohio Valley  (1)</t>
+        </is>
+      </c>
+      <c r="B75" s="12" t="n"/>
+      <c r="C75" s="12" t="n"/>
+      <c r="D75" s="12" t="n"/>
+      <c r="E75" s="12" t="n"/>
+      <c r="F75" s="12" t="n"/>
+      <c r="G75" s="12" t="n"/>
+      <c r="H75" s="12" t="n"/>
+      <c r="I75" s="12" t="n"/>
+      <c r="J75" s="12" t="n"/>
+      <c r="K75" s="12" t="n"/>
+      <c r="L75" s="12" t="n"/>
+      <c r="M75" s="12" t="n"/>
+      <c r="N75" s="12" t="n"/>
+      <c r="O75" s="12" t="n"/>
+    </row>
+    <row r="76" outlineLevel="1">
+      <c r="A76" s="13" t="inlineStr">
+        <is>
+          <t>Western PA / Ohio Valley</t>
+        </is>
+      </c>
+      <c r="B76" s="14" t="inlineStr">
+        <is>
+          <t>Millers Pizza &amp; More – pizza business, commercial kitchen &amp; event space contents (362 lots)</t>
+        </is>
+      </c>
+      <c r="C76" s="13" t="inlineStr">
+        <is>
+          <t>restaurant / commercial kitchen contents</t>
+        </is>
+      </c>
+      <c r="D76" s="13" t="inlineStr">
+        <is>
+          <t>Everson</t>
+        </is>
+      </c>
+      <c r="E76" s="13" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="F76" s="13" t="n">
+        <v>478</v>
+      </c>
+      <c r="G76" s="13" t="inlineStr">
+        <is>
+          <t>Online auction, 15% buyer premium</t>
+        </is>
+      </c>
+      <c r="H76" s="15" t="n"/>
+      <c r="I76" s="13" t="inlineStr"/>
+      <c r="J76" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-25 07:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K76" s="13" t="inlineStr">
+        <is>
+          <t>HiBid (Bid Local LLC)</t>
+        </is>
+      </c>
+      <c r="L76" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M76" s="13" t="inlineStr"/>
+      <c r="N76" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O76" s="14" t="inlineStr">
+        <is>
+          <t>Property of Millers Pizza and More LLC; online-only, 362 lots, lots begin closing Oct 25 7 PM. Pickup Everson PA by appointment Tue 10/27 and Wed 10/28. Building (4,500 sq ft) to be auctioned separately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Western PA / Ohio Valley</t>
+        </is>
+      </c>
+      <c r="B77" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C77" s="18" t="n"/>
+      <c r="D77" s="18" t="n"/>
+      <c r="E77" s="18" t="n"/>
+      <c r="F77" s="18" t="n"/>
+      <c r="G77" s="18" t="n"/>
+      <c r="H77" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I77" s="18" t="n"/>
+      <c r="J77" s="18" t="n"/>
+      <c r="K77" s="18" t="n"/>
+      <c r="L77" s="18" t="n"/>
+      <c r="M77" s="18" t="n"/>
+      <c r="N77" s="18" t="n"/>
+      <c r="O77" s="18" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="11" t="inlineStr">
+        <is>
+          <t>▸ Upstate / Western NY  (1)</t>
+        </is>
+      </c>
+      <c r="B78" s="12" t="n"/>
+      <c r="C78" s="12" t="n"/>
+      <c r="D78" s="12" t="n"/>
+      <c r="E78" s="12" t="n"/>
+      <c r="F78" s="12" t="n"/>
+      <c r="G78" s="12" t="n"/>
+      <c r="H78" s="12" t="n"/>
+      <c r="I78" s="12" t="n"/>
+      <c r="J78" s="12" t="n"/>
+      <c r="K78" s="12" t="n"/>
+      <c r="L78" s="12" t="n"/>
+      <c r="M78" s="12" t="n"/>
+      <c r="N78" s="12" t="n"/>
+      <c r="O78" s="12" t="n"/>
+    </row>
+    <row r="79" outlineLevel="1">
+      <c r="A79" s="13" t="inlineStr">
+        <is>
+          <t>Upstate / Western NY</t>
+        </is>
+      </c>
+      <c r="B79" s="14" t="inlineStr">
+        <is>
+          <t>Restaurant &amp; fitness equipment</t>
+        </is>
+      </c>
+      <c r="C79" s="13" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D79" s="13" t="inlineStr">
+        <is>
+          <t>Williamsville</t>
+        </is>
+      </c>
+      <c r="E79" s="13" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="F79" s="13" t="n">
+        <v>408</v>
+      </c>
+      <c r="G79" s="13" t="inlineStr">
+        <is>
+          <t>Online auction</t>
+        </is>
+      </c>
+      <c r="H79" s="15" t="n"/>
+      <c r="I79" s="13" t="inlineStr"/>
+      <c r="J79" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-26 07:30 PM ET</t>
+        </is>
+      </c>
+      <c r="K79" s="13" t="inlineStr">
+        <is>
+          <t>Cash Auctions</t>
+        </is>
+      </c>
+      <c r="L79" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M79" s="13" t="inlineStr"/>
+      <c r="N79" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O79" s="14" t="inlineStr">
+        <is>
+          <t>Lots not reviewed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Upstate / Western NY</t>
+        </is>
+      </c>
+      <c r="B80" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C80" s="18" t="n"/>
+      <c r="D80" s="18" t="n"/>
+      <c r="E80" s="18" t="n"/>
+      <c r="F80" s="18" t="n"/>
+      <c r="G80" s="18" t="n"/>
+      <c r="H80" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I80" s="18" t="n"/>
+      <c r="J80" s="18" t="n"/>
+      <c r="K80" s="18" t="n"/>
+      <c r="L80" s="18" t="n"/>
+      <c r="M80" s="18" t="n"/>
+      <c r="N80" s="18" t="n"/>
+      <c r="O80" s="18" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="11" t="inlineStr">
+        <is>
+          <t>▸ Virginia  (1)</t>
+        </is>
+      </c>
+      <c r="B81" s="12" t="n"/>
+      <c r="C81" s="12" t="n"/>
+      <c r="D81" s="12" t="n"/>
+      <c r="E81" s="12" t="n"/>
+      <c r="F81" s="12" t="n"/>
+      <c r="G81" s="12" t="n"/>
+      <c r="H81" s="12" t="n"/>
+      <c r="I81" s="12" t="n"/>
+      <c r="J81" s="12" t="n"/>
+      <c r="K81" s="12" t="n"/>
+      <c r="L81" s="12" t="n"/>
+      <c r="M81" s="12" t="n"/>
+      <c r="N81" s="12" t="n"/>
+      <c r="O81" s="12" t="n"/>
+    </row>
+    <row r="82" outlineLevel="1">
+      <c r="A82" s="13" t="inlineStr">
+        <is>
+          <t>Virginia</t>
+        </is>
+      </c>
+      <c r="B82" s="14" t="inlineStr">
+        <is>
+          <t>Haynes Furniture / The Dump – 12 stores closing (furniture, mattresses)</t>
+        </is>
+      </c>
+      <c r="C82" s="13" t="inlineStr">
+        <is>
+          <t>retail GOB</t>
+        </is>
+      </c>
+      <c r="D82" s="13" t="inlineStr">
+        <is>
+          <t>Virginia Beach</t>
+        </is>
+      </c>
+      <c r="E82" s="13" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="F82" s="13" t="n">
+        <v>456</v>
+      </c>
+      <c r="G82" s="13" t="inlineStr">
+        <is>
+          <t>Retail GOB markdowns</t>
+        </is>
+      </c>
+      <c r="H82" s="15" t="n"/>
+      <c r="I82" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="J82" s="13" t="inlineStr"/>
+      <c r="K82" s="13" t="inlineStr">
+        <is>
+          <t>SB360 (PR Newswire)</t>
+        </is>
+      </c>
+      <c r="L82" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M82" s="13" t="inlineStr"/>
+      <c r="N82" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O82" s="14" t="inlineStr">
+        <is>
+          <t>Posted Oct 8. Multi-state (VA/AZ/GA/IL/TX); pinned at Virginia Beach. Home goods only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Virginia</t>
+        </is>
+      </c>
+      <c r="B83" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C83" s="18" t="n"/>
+      <c r="D83" s="18" t="n"/>
+      <c r="E83" s="18" t="n"/>
+      <c r="F83" s="18" t="n"/>
+      <c r="G83" s="18" t="n"/>
+      <c r="H83" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I83" s="18" t="n"/>
+      <c r="J83" s="18" t="n"/>
+      <c r="K83" s="18" t="n"/>
+      <c r="L83" s="18" t="n"/>
+      <c r="M83" s="18" t="n"/>
+      <c r="N83" s="18" t="n"/>
+      <c r="O83" s="18" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="11" t="inlineStr">
+        <is>
+          <t>▸ Southeast  (1)</t>
+        </is>
+      </c>
+      <c r="B84" s="12" t="n"/>
+      <c r="C84" s="12" t="n"/>
+      <c r="D84" s="12" t="n"/>
+      <c r="E84" s="12" t="n"/>
+      <c r="F84" s="12" t="n"/>
+      <c r="G84" s="12" t="n"/>
+      <c r="H84" s="12" t="n"/>
+      <c r="I84" s="12" t="n"/>
+      <c r="J84" s="12" t="n"/>
+      <c r="K84" s="12" t="n"/>
+      <c r="L84" s="12" t="n"/>
+      <c r="M84" s="12" t="n"/>
+      <c r="N84" s="12" t="n"/>
+      <c r="O84" s="12" t="n"/>
+    </row>
+    <row r="85" outlineLevel="1">
+      <c r="A85" s="13" t="inlineStr">
+        <is>
+          <t>Southeast</t>
+        </is>
+      </c>
+      <c r="B85" s="14" t="inlineStr">
+        <is>
+          <t>Carter Control Systems Inc. bankruptcy Day 2: fabrication equipment + $5MM+ inventory (conveyor systems maker)</t>
+        </is>
+      </c>
+      <c r="C85" s="13" t="inlineStr">
+        <is>
+          <t>bankruptcy auction</t>
+        </is>
+      </c>
+      <c r="D85" s="13" t="inlineStr">
+        <is>
+          <t>Savannah</t>
+        </is>
+      </c>
+      <c r="E85" s="13" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="F85" s="13" t="n">
+        <v>894</v>
+      </c>
+      <c r="G85" s="13" t="inlineStr">
+        <is>
+          <t>Timed online auction</t>
+        </is>
+      </c>
+      <c r="H85" s="15" t="n"/>
+      <c r="I85" s="13" t="inlineStr"/>
+      <c r="J85" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-28 10:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K85" s="13" t="inlineStr">
+        <is>
+          <t>PPL Group</t>
+        </is>
+      </c>
+      <c r="L85" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M85" s="13" t="inlineStr"/>
+      <c r="N85" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O85" s="14" t="inlineStr">
+        <is>
+          <t>Ends Oct 28 10 AM ET; preview Oct 26-27; removal Oct 29-Nov 13.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Southeast</t>
+        </is>
+      </c>
+      <c r="B86" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C86" s="18" t="n"/>
+      <c r="D86" s="18" t="n"/>
+      <c r="E86" s="18" t="n"/>
+      <c r="F86" s="18" t="n"/>
+      <c r="G86" s="18" t="n"/>
+      <c r="H86" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" s="18" t="n"/>
+      <c r="J86" s="18" t="n"/>
+      <c r="K86" s="18" t="n"/>
+      <c r="L86" s="18" t="n"/>
+      <c r="M86" s="18" t="n"/>
+      <c r="N86" s="18" t="n"/>
+      <c r="O86" s="18" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="11" t="inlineStr">
+        <is>
+          <t>▸ Midwest  (2)</t>
+        </is>
+      </c>
+      <c r="B87" s="12" t="n"/>
+      <c r="C87" s="12" t="n"/>
+      <c r="D87" s="12" t="n"/>
+      <c r="E87" s="12" t="n"/>
+      <c r="F87" s="12" t="n"/>
+      <c r="G87" s="12" t="n"/>
+      <c r="H87" s="12" t="n"/>
+      <c r="I87" s="12" t="n"/>
+      <c r="J87" s="12" t="n"/>
+      <c r="K87" s="12" t="n"/>
+      <c r="L87" s="12" t="n"/>
+      <c r="M87" s="12" t="n"/>
+      <c r="N87" s="12" t="n"/>
+      <c r="O87" s="12" t="n"/>
+    </row>
+    <row r="88" outlineLevel="1">
+      <c r="A88" s="13" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="B88" s="14" t="inlineStr">
+        <is>
+          <t>American Sale – total liquidation, all 7 stores (pools, hot tubs, grills, holiday decor)</t>
+        </is>
+      </c>
+      <c r="C88" s="13" t="inlineStr">
+        <is>
+          <t>retail GOB</t>
+        </is>
+      </c>
+      <c r="D88" s="13" t="inlineStr">
+        <is>
+          <t>Chicagoland</t>
+        </is>
+      </c>
+      <c r="E88" s="13" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="F88" s="13" t="n">
+        <v>876</v>
+      </c>
+      <c r="G88" s="13" t="inlineStr">
+        <is>
+          <t>Retail GOB, up to 70% off</t>
+        </is>
+      </c>
+      <c r="H88" s="15" t="n"/>
+      <c r="I88" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="J88" s="13" t="inlineStr"/>
+      <c r="K88" s="13" t="inlineStr">
+        <is>
+          <t>Tiger Group (PR Newswire)</t>
+        </is>
+      </c>
+      <c r="L88" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M88" s="13" t="inlineStr"/>
+      <c r="N88" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O88" s="14" t="inlineStr">
+        <is>
+          <t>Posted Oct 15. Watch for a bulk/fixture auction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" outlineLevel="1">
+      <c r="A89" s="13" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="B89" s="14" t="inlineStr">
+        <is>
+          <t>Restaurant, Bar &amp; DJ Equipment Liquidation: Alto-Shaam combi, Southbend/Blodgett ovens, True refrigeration, Manitowoc, Hobart saw, DJ/AV gear</t>
+        </is>
+      </c>
+      <c r="C89" s="13" t="inlineStr">
+        <is>
+          <t>restaurant liquidation auction</t>
+        </is>
+      </c>
+      <c r="D89" s="13" t="inlineStr">
+        <is>
+          <t>Austin</t>
+        </is>
+      </c>
+      <c r="E89" s="13" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="F89" s="13" t="n">
+        <v>1124</v>
+      </c>
+      <c r="G89" s="13" t="inlineStr">
+        <is>
+          <t>Timed online auction</t>
+        </is>
+      </c>
+      <c r="H89" s="15" t="n"/>
+      <c r="I89" s="13" t="inlineStr"/>
+      <c r="J89" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-26 02:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K89" s="13" t="inlineStr">
+        <is>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L89" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M89" s="13" t="inlineStr"/>
+      <c r="N89" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O89" s="14" t="inlineStr">
+        <is>
+          <t>Begins closing Oct 26 1 PM CDT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Midwest</t>
+        </is>
+      </c>
+      <c r="B90" s="17" t="inlineStr">
         <is>
           <t>2 item(s)</t>
         </is>
       </c>
-      <c r="C72" s="18" t="n"/>
-      <c r="D72" s="18" t="n"/>
-      <c r="E72" s="18" t="n"/>
-      <c r="F72" s="18" t="n"/>
-      <c r="G72" s="18" t="n"/>
-      <c r="H72" s="19" t="n">
+      <c r="C90" s="18" t="n"/>
+      <c r="D90" s="18" t="n"/>
+      <c r="E90" s="18" t="n"/>
+      <c r="F90" s="18" t="n"/>
+      <c r="G90" s="18" t="n"/>
+      <c r="H90" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I72" s="18" t="n"/>
-      <c r="J72" s="18" t="n"/>
-      <c r="K72" s="18" t="n"/>
-      <c r="L72" s="18" t="n"/>
-      <c r="M72" s="18" t="n"/>
-      <c r="N72" s="18" t="n"/>
-      <c r="O72" s="18" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="11" t="inlineStr">
-        <is>
-          <t>▸ Western PA / Ohio Valley  (1)</t>
-        </is>
-      </c>
-      <c r="B73" s="12" t="n"/>
-      <c r="C73" s="12" t="n"/>
-      <c r="D73" s="12" t="n"/>
-      <c r="E73" s="12" t="n"/>
-      <c r="F73" s="12" t="n"/>
-      <c r="G73" s="12" t="n"/>
-      <c r="H73" s="12" t="n"/>
-      <c r="I73" s="12" t="n"/>
-      <c r="J73" s="12" t="n"/>
-      <c r="K73" s="12" t="n"/>
-      <c r="L73" s="12" t="n"/>
-      <c r="M73" s="12" t="n"/>
-      <c r="N73" s="12" t="n"/>
-      <c r="O73" s="12" t="n"/>
-    </row>
-    <row r="74" outlineLevel="1">
-      <c r="A74" s="13" t="inlineStr">
-        <is>
-          <t>Western PA / Ohio Valley</t>
-        </is>
-      </c>
-      <c r="B74" s="14" t="inlineStr">
-        <is>
-          <t>Millers Pizza &amp; More – pizza business, commercial kitchen &amp; event space contents (362 lots)</t>
-        </is>
-      </c>
-      <c r="C74" s="13" t="inlineStr">
-        <is>
-          <t>restaurant / commercial kitchen contents</t>
-        </is>
-      </c>
-      <c r="D74" s="13" t="inlineStr">
-        <is>
-          <t>Everson</t>
-        </is>
-      </c>
-      <c r="E74" s="13" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="F74" s="13" t="n">
-        <v>478</v>
-      </c>
-      <c r="G74" s="13" t="inlineStr">
-        <is>
-          <t>Online auction, 15% buyer premium</t>
-        </is>
-      </c>
-      <c r="H74" s="15" t="n"/>
-      <c r="I74" s="13" t="inlineStr"/>
-      <c r="J74" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-25 07:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K74" s="13" t="inlineStr">
-        <is>
-          <t>HiBid (Bid Local LLC)</t>
-        </is>
-      </c>
-      <c r="L74" s="21" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
-        </is>
-      </c>
-      <c r="M74" s="13" t="inlineStr"/>
-      <c r="N74" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O74" s="14" t="inlineStr">
-        <is>
-          <t>Property of Millers Pizza and More LLC; online-only, 362 lots, lots begin closing Oct 25 7 PM. Pickup Everson PA by appointment Tue 10/27 and Wed 10/28. Building (4,500 sq ft) to be auctioned separately.</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Western PA / Ohio Valley</t>
-        </is>
-      </c>
-      <c r="B75" s="17" t="inlineStr">
+      <c r="I90" s="18" t="n"/>
+      <c r="J90" s="18" t="n"/>
+      <c r="K90" s="18" t="n"/>
+      <c r="L90" s="18" t="n"/>
+      <c r="M90" s="18" t="n"/>
+      <c r="N90" s="18" t="n"/>
+      <c r="O90" s="18" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="11" t="inlineStr">
+        <is>
+          <t>▸ Texas / South Central  (1)</t>
+        </is>
+      </c>
+      <c r="B91" s="12" t="n"/>
+      <c r="C91" s="12" t="n"/>
+      <c r="D91" s="12" t="n"/>
+      <c r="E91" s="12" t="n"/>
+      <c r="F91" s="12" t="n"/>
+      <c r="G91" s="12" t="n"/>
+      <c r="H91" s="12" t="n"/>
+      <c r="I91" s="12" t="n"/>
+      <c r="J91" s="12" t="n"/>
+      <c r="K91" s="12" t="n"/>
+      <c r="L91" s="12" t="n"/>
+      <c r="M91" s="12" t="n"/>
+      <c r="N91" s="12" t="n"/>
+      <c r="O91" s="12" t="n"/>
+    </row>
+    <row r="92" outlineLevel="1">
+      <c r="A92" s="13" t="inlineStr">
+        <is>
+          <t>Texas / South Central</t>
+        </is>
+      </c>
+      <c r="B92" s="14" t="inlineStr">
+        <is>
+          <t>Southwest beverage distributor surplus – mostly unused: 16 True merchandisers, 75 Bunn brewers, 100+ micro-market kiosks</t>
+        </is>
+      </c>
+      <c r="C92" s="13" t="inlineStr">
+        <is>
+          <t>distributor surplus</t>
+        </is>
+      </c>
+      <c r="D92" s="13" t="inlineStr">
+        <is>
+          <t>Mesquite</t>
+        </is>
+      </c>
+      <c r="E92" s="13" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="F92" s="13" t="n">
+        <v>1547</v>
+      </c>
+      <c r="G92" s="13" t="inlineStr">
+        <is>
+          <t>Online auction</t>
+        </is>
+      </c>
+      <c r="H92" s="15" t="n"/>
+      <c r="I92" s="13" t="inlineStr"/>
+      <c r="J92" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-13 11:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K92" s="13" t="inlineStr">
+        <is>
+          <t>Heritage Global Partners</t>
+        </is>
+      </c>
+      <c r="L92" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M92" s="13" t="inlineStr"/>
+      <c r="N92" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O92" s="14" t="inlineStr">
+        <is>
+          <t>Near-new appliances, resell by unit. Nov 13 10 AM CST.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Texas / South Central</t>
+        </is>
+      </c>
+      <c r="B93" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C75" s="18" t="n"/>
-      <c r="D75" s="18" t="n"/>
-      <c r="E75" s="18" t="n"/>
-      <c r="F75" s="18" t="n"/>
-      <c r="G75" s="18" t="n"/>
-      <c r="H75" s="19" t="n">
+      <c r="C93" s="18" t="n"/>
+      <c r="D93" s="18" t="n"/>
+      <c r="E93" s="18" t="n"/>
+      <c r="F93" s="18" t="n"/>
+      <c r="G93" s="18" t="n"/>
+      <c r="H93" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I75" s="18" t="n"/>
-      <c r="J75" s="18" t="n"/>
-      <c r="K75" s="18" t="n"/>
-      <c r="L75" s="18" t="n"/>
-      <c r="M75" s="18" t="n"/>
-      <c r="N75" s="18" t="n"/>
-      <c r="O75" s="18" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="11" t="inlineStr">
-        <is>
-          <t>▸ Upstate / Western NY  (1)</t>
-        </is>
-      </c>
-      <c r="B76" s="12" t="n"/>
-      <c r="C76" s="12" t="n"/>
-      <c r="D76" s="12" t="n"/>
-      <c r="E76" s="12" t="n"/>
-      <c r="F76" s="12" t="n"/>
-      <c r="G76" s="12" t="n"/>
-      <c r="H76" s="12" t="n"/>
-      <c r="I76" s="12" t="n"/>
-      <c r="J76" s="12" t="n"/>
-      <c r="K76" s="12" t="n"/>
-      <c r="L76" s="12" t="n"/>
-      <c r="M76" s="12" t="n"/>
-      <c r="N76" s="12" t="n"/>
-      <c r="O76" s="12" t="n"/>
-    </row>
-    <row r="77" outlineLevel="1">
-      <c r="A77" s="13" t="inlineStr">
-        <is>
-          <t>Upstate / Western NY</t>
-        </is>
-      </c>
-      <c r="B77" s="14" t="inlineStr">
-        <is>
-          <t>Restaurant &amp; fitness equipment</t>
-        </is>
-      </c>
-      <c r="C77" s="13" t="inlineStr">
-        <is>
-          <t>restaurant</t>
-        </is>
-      </c>
-      <c r="D77" s="13" t="inlineStr">
-        <is>
-          <t>Williamsville</t>
-        </is>
-      </c>
-      <c r="E77" s="13" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="F77" s="13" t="n">
-        <v>408</v>
-      </c>
-      <c r="G77" s="13" t="inlineStr">
-        <is>
-          <t>Online auction</t>
-        </is>
-      </c>
-      <c r="H77" s="15" t="n"/>
-      <c r="I77" s="13" t="inlineStr"/>
-      <c r="J77" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26 07:30 PM ET</t>
-        </is>
-      </c>
-      <c r="K77" s="13" t="inlineStr">
-        <is>
-          <t>Cash Auctions</t>
-        </is>
-      </c>
-      <c r="L77" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M77" s="13" t="inlineStr"/>
-      <c r="N77" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O77" s="14" t="inlineStr">
-        <is>
-          <t>Lots not reviewed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Upstate / Western NY</t>
-        </is>
-      </c>
-      <c r="B78" s="17" t="inlineStr">
+      <c r="I93" s="18" t="n"/>
+      <c r="J93" s="18" t="n"/>
+      <c r="K93" s="18" t="n"/>
+      <c r="L93" s="18" t="n"/>
+      <c r="M93" s="18" t="n"/>
+      <c r="N93" s="18" t="n"/>
+      <c r="O93" s="18" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="11" t="inlineStr">
+        <is>
+          <t>▸ West / Other  (1)</t>
+        </is>
+      </c>
+      <c r="B94" s="12" t="n"/>
+      <c r="C94" s="12" t="n"/>
+      <c r="D94" s="12" t="n"/>
+      <c r="E94" s="12" t="n"/>
+      <c r="F94" s="12" t="n"/>
+      <c r="G94" s="12" t="n"/>
+      <c r="H94" s="12" t="n"/>
+      <c r="I94" s="12" t="n"/>
+      <c r="J94" s="12" t="n"/>
+      <c r="K94" s="12" t="n"/>
+      <c r="L94" s="12" t="n"/>
+      <c r="M94" s="12" t="n"/>
+      <c r="N94" s="12" t="n"/>
+      <c r="O94" s="12" t="n"/>
+    </row>
+    <row r="95" outlineLevel="1">
+      <c r="A95" s="13" t="inlineStr">
+        <is>
+          <t>West / Other</t>
+        </is>
+      </c>
+      <c r="B95" s="14" t="inlineStr">
+        <is>
+          <t>National salad concept liquidation – full contents of 63 fast-casual restaurants (AZ/TX/OK/NV)</t>
+        </is>
+      </c>
+      <c r="C95" s="13" t="inlineStr">
+        <is>
+          <t>restaurant chain liquidation</t>
+        </is>
+      </c>
+      <c r="D95" s="13" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="E95" s="13" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="F95" s="13" t="n">
+        <v>2307</v>
+      </c>
+      <c r="G95" s="13" t="inlineStr">
+        <is>
+          <t>Online auctions, dates TBD</t>
+        </is>
+      </c>
+      <c r="H95" s="15" t="n"/>
+      <c r="I95" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="J95" s="13" t="inlineStr"/>
+      <c r="K95" s="13" t="inlineStr">
+        <is>
+          <t>RestaurantEquipment.bid (TAGeX)</t>
+        </is>
+      </c>
+      <c r="L95" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M95" s="13" t="inlineStr"/>
+      <c r="N95" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O95" s="14" t="inlineStr">
+        <is>
+          <t>Rolling market-by-market auctions, none live yet (Phoenix metro 30 locations, DFW 14, Tucson 6, Houston 5, plus OK/NV). Pickup on site at each restaurant. Pinned at Phoenix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — West / Other</t>
+        </is>
+      </c>
+      <c r="B96" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C78" s="18" t="n"/>
-      <c r="D78" s="18" t="n"/>
-      <c r="E78" s="18" t="n"/>
-      <c r="F78" s="18" t="n"/>
-      <c r="G78" s="18" t="n"/>
-      <c r="H78" s="19" t="n">
+      <c r="C96" s="18" t="n"/>
+      <c r="D96" s="18" t="n"/>
+      <c r="E96" s="18" t="n"/>
+      <c r="F96" s="18" t="n"/>
+      <c r="G96" s="18" t="n"/>
+      <c r="H96" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I78" s="18" t="n"/>
-      <c r="J78" s="18" t="n"/>
-      <c r="K78" s="18" t="n"/>
-      <c r="L78" s="18" t="n"/>
-      <c r="M78" s="18" t="n"/>
-      <c r="N78" s="18" t="n"/>
-      <c r="O78" s="18" t="n"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="11" t="inlineStr">
-        <is>
-          <t>▸ Virginia  (1)</t>
-        </is>
-      </c>
-      <c r="B79" s="12" t="n"/>
-      <c r="C79" s="12" t="n"/>
-      <c r="D79" s="12" t="n"/>
-      <c r="E79" s="12" t="n"/>
-      <c r="F79" s="12" t="n"/>
-      <c r="G79" s="12" t="n"/>
-      <c r="H79" s="12" t="n"/>
-      <c r="I79" s="12" t="n"/>
-      <c r="J79" s="12" t="n"/>
-      <c r="K79" s="12" t="n"/>
-      <c r="L79" s="12" t="n"/>
-      <c r="M79" s="12" t="n"/>
-      <c r="N79" s="12" t="n"/>
-      <c r="O79" s="12" t="n"/>
-    </row>
-    <row r="80" outlineLevel="1">
-      <c r="A80" s="13" t="inlineStr">
-        <is>
-          <t>Virginia</t>
-        </is>
-      </c>
-      <c r="B80" s="14" t="inlineStr">
-        <is>
-          <t>Haynes Furniture / The Dump – 12 stores closing (furniture, mattresses)</t>
-        </is>
-      </c>
-      <c r="C80" s="13" t="inlineStr">
-        <is>
-          <t>retail GOB</t>
-        </is>
-      </c>
-      <c r="D80" s="13" t="inlineStr">
-        <is>
-          <t>Virginia Beach</t>
-        </is>
-      </c>
-      <c r="E80" s="13" t="inlineStr">
-        <is>
-          <t>VA</t>
-        </is>
-      </c>
-      <c r="F80" s="13" t="n">
-        <v>456</v>
-      </c>
-      <c r="G80" s="13" t="inlineStr">
-        <is>
-          <t>Retail GOB markdowns</t>
-        </is>
-      </c>
-      <c r="H80" s="15" t="n"/>
-      <c r="I80" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="J80" s="13" t="inlineStr"/>
-      <c r="K80" s="13" t="inlineStr">
-        <is>
-          <t>SB360 (PR Newswire)</t>
-        </is>
-      </c>
-      <c r="L80" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M80" s="13" t="inlineStr"/>
-      <c r="N80" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O80" s="14" t="inlineStr">
-        <is>
-          <t>Posted Oct 8. Multi-state (VA/AZ/GA/IL/TX); pinned at Virginia Beach. Home goods only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Virginia</t>
-        </is>
-      </c>
-      <c r="B81" s="17" t="inlineStr">
-        <is>
-          <t>1 item(s)</t>
-        </is>
-      </c>
-      <c r="C81" s="18" t="n"/>
-      <c r="D81" s="18" t="n"/>
-      <c r="E81" s="18" t="n"/>
-      <c r="F81" s="18" t="n"/>
-      <c r="G81" s="18" t="n"/>
-      <c r="H81" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I81" s="18" t="n"/>
-      <c r="J81" s="18" t="n"/>
-      <c r="K81" s="18" t="n"/>
-      <c r="L81" s="18" t="n"/>
-      <c r="M81" s="18" t="n"/>
-      <c r="N81" s="18" t="n"/>
-      <c r="O81" s="18" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="11" t="inlineStr">
-        <is>
-          <t>▸ Southeast  (1)</t>
-        </is>
-      </c>
-      <c r="B82" s="12" t="n"/>
-      <c r="C82" s="12" t="n"/>
-      <c r="D82" s="12" t="n"/>
-      <c r="E82" s="12" t="n"/>
-      <c r="F82" s="12" t="n"/>
-      <c r="G82" s="12" t="n"/>
-      <c r="H82" s="12" t="n"/>
-      <c r="I82" s="12" t="n"/>
-      <c r="J82" s="12" t="n"/>
-      <c r="K82" s="12" t="n"/>
-      <c r="L82" s="12" t="n"/>
-      <c r="M82" s="12" t="n"/>
-      <c r="N82" s="12" t="n"/>
-      <c r="O82" s="12" t="n"/>
-    </row>
-    <row r="83" outlineLevel="1">
-      <c r="A83" s="13" t="inlineStr">
-        <is>
-          <t>Southeast</t>
-        </is>
-      </c>
-      <c r="B83" s="14" t="inlineStr">
-        <is>
-          <t>Carter Control Systems Inc. bankruptcy Day 2: fabrication equipment + $5MM+ inventory (conveyor systems maker)</t>
-        </is>
-      </c>
-      <c r="C83" s="13" t="inlineStr">
-        <is>
-          <t>bankruptcy auction</t>
-        </is>
-      </c>
-      <c r="D83" s="13" t="inlineStr">
-        <is>
-          <t>Savannah</t>
-        </is>
-      </c>
-      <c r="E83" s="13" t="inlineStr">
-        <is>
-          <t>GA</t>
-        </is>
-      </c>
-      <c r="F83" s="13" t="n">
-        <v>894</v>
-      </c>
-      <c r="G83" s="13" t="inlineStr">
-        <is>
-          <t>Timed online auction</t>
-        </is>
-      </c>
-      <c r="H83" s="15" t="n"/>
-      <c r="I83" s="13" t="inlineStr"/>
-      <c r="J83" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-28 10:00 AM ET</t>
-        </is>
-      </c>
-      <c r="K83" s="13" t="inlineStr">
-        <is>
-          <t>PPL Group</t>
-        </is>
-      </c>
-      <c r="L83" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M83" s="13" t="inlineStr"/>
-      <c r="N83" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O83" s="14" t="inlineStr">
-        <is>
-          <t>Ends Oct 28 10 AM ET; preview Oct 26-27; removal Oct 29-Nov 13.</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Southeast</t>
-        </is>
-      </c>
-      <c r="B84" s="17" t="inlineStr">
-        <is>
-          <t>1 item(s)</t>
-        </is>
-      </c>
-      <c r="C84" s="18" t="n"/>
-      <c r="D84" s="18" t="n"/>
-      <c r="E84" s="18" t="n"/>
-      <c r="F84" s="18" t="n"/>
-      <c r="G84" s="18" t="n"/>
-      <c r="H84" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I84" s="18" t="n"/>
-      <c r="J84" s="18" t="n"/>
-      <c r="K84" s="18" t="n"/>
-      <c r="L84" s="18" t="n"/>
-      <c r="M84" s="18" t="n"/>
-      <c r="N84" s="18" t="n"/>
-      <c r="O84" s="18" t="n"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="11" t="inlineStr">
-        <is>
-          <t>▸ Midwest  (2)</t>
-        </is>
-      </c>
-      <c r="B85" s="12" t="n"/>
-      <c r="C85" s="12" t="n"/>
-      <c r="D85" s="12" t="n"/>
-      <c r="E85" s="12" t="n"/>
-      <c r="F85" s="12" t="n"/>
-      <c r="G85" s="12" t="n"/>
-      <c r="H85" s="12" t="n"/>
-      <c r="I85" s="12" t="n"/>
-      <c r="J85" s="12" t="n"/>
-      <c r="K85" s="12" t="n"/>
-      <c r="L85" s="12" t="n"/>
-      <c r="M85" s="12" t="n"/>
-      <c r="N85" s="12" t="n"/>
-      <c r="O85" s="12" t="n"/>
-    </row>
-    <row r="86" outlineLevel="1">
-      <c r="A86" s="13" t="inlineStr">
-        <is>
-          <t>Midwest</t>
-        </is>
-      </c>
-      <c r="B86" s="14" t="inlineStr">
-        <is>
-          <t>American Sale – total liquidation, all 7 stores (pools, hot tubs, grills, holiday decor)</t>
-        </is>
-      </c>
-      <c r="C86" s="13" t="inlineStr">
-        <is>
-          <t>retail GOB</t>
-        </is>
-      </c>
-      <c r="D86" s="13" t="inlineStr">
-        <is>
-          <t>Chicagoland</t>
-        </is>
-      </c>
-      <c r="E86" s="13" t="inlineStr">
-        <is>
-          <t>IL</t>
-        </is>
-      </c>
-      <c r="F86" s="13" t="n">
-        <v>876</v>
-      </c>
-      <c r="G86" s="13" t="inlineStr">
-        <is>
-          <t>Retail GOB, up to 70% off</t>
-        </is>
-      </c>
-      <c r="H86" s="15" t="n"/>
-      <c r="I86" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="J86" s="13" t="inlineStr"/>
-      <c r="K86" s="13" t="inlineStr">
-        <is>
-          <t>Tiger Group (PR Newswire)</t>
-        </is>
-      </c>
-      <c r="L86" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M86" s="13" t="inlineStr"/>
-      <c r="N86" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O86" s="14" t="inlineStr">
-        <is>
-          <t>Posted Oct 15. Watch for a bulk/fixture auction.</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" outlineLevel="1">
-      <c r="A87" s="13" t="inlineStr">
-        <is>
-          <t>Midwest</t>
-        </is>
-      </c>
-      <c r="B87" s="14" t="inlineStr">
-        <is>
-          <t>Restaurant, Bar &amp; DJ Equipment Liquidation: Alto-Shaam combi, Southbend/Blodgett ovens, True refrigeration, Manitowoc, Hobart saw, DJ/AV gear</t>
-        </is>
-      </c>
-      <c r="C87" s="13" t="inlineStr">
-        <is>
-          <t>restaurant liquidation auction</t>
-        </is>
-      </c>
-      <c r="D87" s="13" t="inlineStr">
-        <is>
-          <t>Austin</t>
-        </is>
-      </c>
-      <c r="E87" s="13" t="inlineStr">
-        <is>
-          <t>MN</t>
-        </is>
-      </c>
-      <c r="F87" s="13" t="n">
-        <v>1124</v>
-      </c>
-      <c r="G87" s="13" t="inlineStr">
-        <is>
-          <t>Timed online auction</t>
-        </is>
-      </c>
-      <c r="H87" s="15" t="n"/>
-      <c r="I87" s="13" t="inlineStr"/>
-      <c r="J87" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26 02:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K87" s="13" t="inlineStr">
-        <is>
-          <t>Grafe Auction</t>
-        </is>
-      </c>
-      <c r="L87" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M87" s="13" t="inlineStr"/>
-      <c r="N87" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O87" s="14" t="inlineStr">
-        <is>
-          <t>Begins closing Oct 26 1 PM CDT.</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Midwest</t>
-        </is>
-      </c>
-      <c r="B88" s="17" t="inlineStr">
-        <is>
-          <t>2 item(s)</t>
-        </is>
-      </c>
-      <c r="C88" s="18" t="n"/>
-      <c r="D88" s="18" t="n"/>
-      <c r="E88" s="18" t="n"/>
-      <c r="F88" s="18" t="n"/>
-      <c r="G88" s="18" t="n"/>
-      <c r="H88" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I88" s="18" t="n"/>
-      <c r="J88" s="18" t="n"/>
-      <c r="K88" s="18" t="n"/>
-      <c r="L88" s="18" t="n"/>
-      <c r="M88" s="18" t="n"/>
-      <c r="N88" s="18" t="n"/>
-      <c r="O88" s="18" t="n"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="11" t="inlineStr">
-        <is>
-          <t>▸ Texas / South Central  (1)</t>
-        </is>
-      </c>
-      <c r="B89" s="12" t="n"/>
-      <c r="C89" s="12" t="n"/>
-      <c r="D89" s="12" t="n"/>
-      <c r="E89" s="12" t="n"/>
-      <c r="F89" s="12" t="n"/>
-      <c r="G89" s="12" t="n"/>
-      <c r="H89" s="12" t="n"/>
-      <c r="I89" s="12" t="n"/>
-      <c r="J89" s="12" t="n"/>
-      <c r="K89" s="12" t="n"/>
-      <c r="L89" s="12" t="n"/>
-      <c r="M89" s="12" t="n"/>
-      <c r="N89" s="12" t="n"/>
-      <c r="O89" s="12" t="n"/>
-    </row>
-    <row r="90" outlineLevel="1">
-      <c r="A90" s="13" t="inlineStr">
-        <is>
-          <t>Texas / South Central</t>
-        </is>
-      </c>
-      <c r="B90" s="14" t="inlineStr">
-        <is>
-          <t>Southwest beverage distributor surplus – mostly unused: 16 True merchandisers, 75 Bunn brewers, 100+ micro-market kiosks</t>
-        </is>
-      </c>
-      <c r="C90" s="13" t="inlineStr">
-        <is>
-          <t>distributor surplus</t>
-        </is>
-      </c>
-      <c r="D90" s="13" t="inlineStr">
-        <is>
-          <t>Mesquite</t>
-        </is>
-      </c>
-      <c r="E90" s="13" t="inlineStr">
-        <is>
-          <t>TX</t>
-        </is>
-      </c>
-      <c r="F90" s="13" t="n">
-        <v>1547</v>
-      </c>
-      <c r="G90" s="13" t="inlineStr">
-        <is>
-          <t>Online auction</t>
-        </is>
-      </c>
-      <c r="H90" s="15" t="n"/>
-      <c r="I90" s="13" t="inlineStr"/>
-      <c r="J90" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-13 11:00 AM ET</t>
-        </is>
-      </c>
-      <c r="K90" s="13" t="inlineStr">
-        <is>
-          <t>Heritage Global Partners</t>
-        </is>
-      </c>
-      <c r="L90" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M90" s="13" t="inlineStr"/>
-      <c r="N90" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O90" s="14" t="inlineStr">
-        <is>
-          <t>Near-new appliances, resell by unit. Nov 13 10 AM CST.</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Texas / South Central</t>
-        </is>
-      </c>
-      <c r="B91" s="17" t="inlineStr">
-        <is>
-          <t>1 item(s)</t>
-        </is>
-      </c>
-      <c r="C91" s="18" t="n"/>
-      <c r="D91" s="18" t="n"/>
-      <c r="E91" s="18" t="n"/>
-      <c r="F91" s="18" t="n"/>
-      <c r="G91" s="18" t="n"/>
-      <c r="H91" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I91" s="18" t="n"/>
-      <c r="J91" s="18" t="n"/>
-      <c r="K91" s="18" t="n"/>
-      <c r="L91" s="18" t="n"/>
-      <c r="M91" s="18" t="n"/>
-      <c r="N91" s="18" t="n"/>
-      <c r="O91" s="18" t="n"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="11" t="inlineStr">
-        <is>
-          <t>▸ West / Other  (1)</t>
-        </is>
-      </c>
-      <c r="B92" s="12" t="n"/>
-      <c r="C92" s="12" t="n"/>
-      <c r="D92" s="12" t="n"/>
-      <c r="E92" s="12" t="n"/>
-      <c r="F92" s="12" t="n"/>
-      <c r="G92" s="12" t="n"/>
-      <c r="H92" s="12" t="n"/>
-      <c r="I92" s="12" t="n"/>
-      <c r="J92" s="12" t="n"/>
-      <c r="K92" s="12" t="n"/>
-      <c r="L92" s="12" t="n"/>
-      <c r="M92" s="12" t="n"/>
-      <c r="N92" s="12" t="n"/>
-      <c r="O92" s="12" t="n"/>
-    </row>
-    <row r="93" outlineLevel="1">
-      <c r="A93" s="13" t="inlineStr">
-        <is>
-          <t>West / Other</t>
-        </is>
-      </c>
-      <c r="B93" s="14" t="inlineStr">
-        <is>
-          <t>National salad concept liquidation – full contents of 63 fast-casual restaurants (AZ/TX/OK/NV)</t>
-        </is>
-      </c>
-      <c r="C93" s="13" t="inlineStr">
-        <is>
-          <t>restaurant chain liquidation</t>
-        </is>
-      </c>
-      <c r="D93" s="13" t="inlineStr">
-        <is>
-          <t>Phoenix</t>
-        </is>
-      </c>
-      <c r="E93" s="13" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="F93" s="13" t="n">
-        <v>2307</v>
-      </c>
-      <c r="G93" s="13" t="inlineStr">
-        <is>
-          <t>Online auctions, dates TBD</t>
-        </is>
-      </c>
-      <c r="H93" s="15" t="n"/>
-      <c r="I93" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="J93" s="13" t="inlineStr"/>
-      <c r="K93" s="13" t="inlineStr">
-        <is>
-          <t>RestaurantEquipment.bid (TAGeX)</t>
-        </is>
-      </c>
-      <c r="L93" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M93" s="13" t="inlineStr"/>
-      <c r="N93" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O93" s="14" t="inlineStr">
-        <is>
-          <t>Rolling market-by-market auctions, none live yet (Phoenix metro 30 locations, DFW 14, Tucson 6, Houston 5, plus OK/NV). Pickup on site at each restaurant. Pinned at Phoenix.</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — West / Other</t>
-        </is>
-      </c>
-      <c r="B94" s="17" t="inlineStr">
-        <is>
-          <t>1 item(s)</t>
-        </is>
-      </c>
-      <c r="C94" s="18" t="n"/>
-      <c r="D94" s="18" t="n"/>
-      <c r="E94" s="18" t="n"/>
-      <c r="F94" s="18" t="n"/>
-      <c r="G94" s="18" t="n"/>
-      <c r="H94" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I94" s="18" t="n"/>
-      <c r="J94" s="18" t="n"/>
-      <c r="K94" s="18" t="n"/>
-      <c r="L94" s="18" t="n"/>
-      <c r="M94" s="18" t="n"/>
-      <c r="N94" s="18" t="n"/>
-      <c r="O94" s="18" t="n"/>
+      <c r="I96" s="18" t="n"/>
+      <c r="J96" s="18" t="n"/>
+      <c r="K96" s="18" t="n"/>
+      <c r="L96" s="18" t="n"/>
+      <c r="M96" s="18" t="n"/>
+      <c r="N96" s="18" t="n"/>
+      <c r="O96" s="18" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O94"/>
+  <autoFilter ref="A1:O96"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId2"/>
@@ -23182,7 +23312,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N38" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N39" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N40" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N43" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N44" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N45" r:id="rId31"/>
@@ -23208,16 +23338,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N65" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N66" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N67" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N70" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N68" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N71" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N74" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N77" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N80" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N83" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N86" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N87" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N90" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N93" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N72" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N73" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N76" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N79" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N82" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N85" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N88" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N89" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N92" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N95" r:id="rId65"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -23391,7 +23523,7 @@
       </c>
       <c r="O2" s="14" t="inlineStr">
         <is>
-          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23454,7 +23586,7 @@
       </c>
       <c r="O3" s="14" t="inlineStr">
         <is>
-          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23584,7 +23716,7 @@
       </c>
       <c r="O5" s="14" t="inlineStr">
         <is>
-          <t>Online auction, closes Thu Oct 22 8:37 PM ET. $12.50 high bid (4 bids) as of 2026-10-18. [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Online auction, closes Thu Oct 22 8:37 PM ET. $12.50 high bid (4 bids) as of 2026-10-18. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23789,7 +23921,7 @@
       </c>
       <c r="O8" s="14" t="inlineStr">
         <is>
-          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23854,7 +23986,7 @@
       </c>
       <c r="O9" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23919,7 +24051,7 @@
       </c>
       <c r="O10" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23984,7 +24116,7 @@
       </c>
       <c r="O11" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24114,7 +24246,7 @@
       </c>
       <c r="O13" s="14" t="inlineStr">
         <is>
-          <t>Lots close in sequence from Oct 21 2 PM ET. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Lots close in sequence from Oct 21 2 PM ET. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24179,7 +24311,7 @@
       </c>
       <c r="O14" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24244,7 +24376,7 @@
       </c>
       <c r="O15" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24307,7 +24439,7 @@
       </c>
       <c r="O16" s="14" t="inlineStr">
         <is>
-          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24370,7 +24502,7 @@
       </c>
       <c r="O17" s="14" t="inlineStr">
         <is>
-          <t>Page conflicts: Oct 21 or 22 9 AM (later date used). Closest find. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Page conflicts: Oct 21 or 22 9 AM (later date used). Closest find. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24433,7 +24565,7 @@
       </c>
       <c r="O18" s="14" t="inlineStr">
         <is>
-          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24496,7 +24628,7 @@
       </c>
       <c r="O19" s="14" t="inlineStr">
         <is>
-          <t>Closes Oct 21 10 or 11 AM (later used). Shippable. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Closes Oct 21 10 or 11 AM (later used). Shippable. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24559,7 +24691,7 @@
       </c>
       <c r="O20" s="14" t="inlineStr">
         <is>
-          <t>Oct 21; start time not captured (placeholder 6 PM). [removed 2026-10-21: live webcast auction held Oct 21; listing page now HTTP 503] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Oct 21; start time not captured (placeholder 6 PM). [removed 2026-10-21: live webcast auction held Oct 21; listing page now HTTP 503] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24622,7 +24754,7 @@
       </c>
       <c r="O21" s="14" t="inlineStr">
         <is>
-          <t>Absolute / no reserve. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Absolute / no reserve. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24685,7 +24817,7 @@
       </c>
       <c r="O22" s="14" t="inlineStr">
         <is>
-          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24748,7 +24880,7 @@
       </c>
       <c r="O23" s="14" t="inlineStr">
         <is>
-          <t>Some kitchen gear only. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Some kitchen gear only. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24811,7 +24943,7 @@
       </c>
       <c r="O24" s="14" t="inlineStr">
         <is>
-          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24874,7 +25006,7 @@
       </c>
       <c r="O25" s="14" t="inlineStr">
         <is>
-          <t>Small lot. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Small lot. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24937,7 +25069,7 @@
       </c>
       <c r="O26" s="14" t="inlineStr">
         <is>
-          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25006,7 +25138,7 @@
       </c>
       <c r="O27" s="14" t="inlineStr">
         <is>
-          <t>About 3 days left as of Oct 18 (~Oct 21; exact time not captured). Pickup Sat Oct 24 12–4 PM by appointment. Used, minor wear. eBay asks $200–420; rough resale $150–250. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>About 3 days left as of Oct 18 (~Oct 21; exact time not captured). Pickup Sat Oct 24 12–4 PM by appointment. Used, minor wear. eBay asks $200–420; rough resale $150–250. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25136,7 +25268,7 @@
       </c>
       <c r="O29" s="14" t="inlineStr">
         <is>
-          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25203,7 +25335,7 @@
       </c>
       <c r="O30" s="14" t="inlineStr">
         <is>
-          <t>Wed Oct 21 4 PM. NYC 10013. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Wed Oct 21 4 PM. NYC 10013. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25270,7 +25402,7 @@
       </c>
       <c r="O31" s="14" t="inlineStr">
         <is>
-          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25337,7 +25469,7 @@
       </c>
       <c r="O32" s="14" t="inlineStr">
         <is>
-          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25404,7 +25536,7 @@
       </c>
       <c r="O33" s="14" t="inlineStr">
         <is>
-          <t>Ends Wed Oct 21 8:30 PM EDT. PCI warehouse, 36 Ludlow St, Stamford CT. Page lists preview Oct 28 and removal Thu Oct 29 11-3 (after close). Shipping/delivery available; payment due on pickup day. Items still being added. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Ends Wed Oct 21 8:30 PM EDT. PCI warehouse, 36 Ludlow St, Stamford CT. Page lists preview Oct 28 and removal Thu Oct 29 11-3 (after close). Shipping/delivery available; payment due on pickup day. Items still being added. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25467,7 +25599,7 @@
       </c>
       <c r="O34" s="14" t="inlineStr">
         <is>
-          <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25534,7 +25666,7 @@
       </c>
       <c r="O35" s="14" t="inlineStr">
         <is>
-          <t>Ends Oct 21 7 PM CDT (8 PM ET). 1500 Somerset Ave, Windber PA. Pickups Oct 24-28. Hardware store, not appliance parts. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Ends Oct 21 7 PM CDT (8 PM ET). 1500 Somerset Ave, Windber PA. Pickups Oct 24-28. Hardware store, not appliance parts. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25601,7 +25733,7 @@
       </c>
       <c r="O36" s="14" t="inlineStr">
         <is>
-          <t>Ends Oct 22 7 PM CDT (8 PM ET). Same store as Day 1; pickups Oct 24-28. [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Ends Oct 22 7 PM CDT (8 PM ET). Same store as Day 1; pickups Oct 24-28. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lot Recon update 2026-10-23 night: +Met Foodmarkets Bronx; -Nyack consignment
</commit_message>
<xml_diff>
--- a/lot_recon.xlsx
+++ b/lot_recon.xlsx
@@ -21,7 +21,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Wolf Used'!$A$1:$O$188</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Wolf Unclear'!$A$1:$O$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$97</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 2026-10-23 14:02 ET</t>
+          <t>Last updated: 2026-10-23 18:05 ET</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Active listings: 304 · Removed: 35</t>
+          <t>Active listings: 304 · Removed: 36</t>
         </is>
       </c>
     </row>
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C23" t="n">
         <v>1</v>
@@ -1004,7 +1004,7 @@
         <v>4</v>
       </c>
       <c r="G23" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H23" s="6" t="n">
         <v>64650</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C24" t="n">
         <v>1</v>
@@ -1037,7 +1037,7 @@
         <v>24</v>
       </c>
       <c r="G24" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H24" s="6" t="n">
         <v>439991</v>
@@ -19954,7 +19954,7 @@
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>▸ CT / Hudson Valley  (9)</t>
+          <t>▸ CT / Hudson Valley  (8)</t>
         </is>
       </c>
       <c r="B32" s="12" t="n"/>
@@ -20358,17 +20358,17 @@
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>Consignment shop remaining inventory, bulk buyer wanted</t>
+          <t>Body shop closing after 50 years – tools, welder, generators, plasma</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>tools liquidation</t>
         </is>
       </c>
       <c r="D39" s="13" t="inlineStr">
         <is>
-          <t>Nyack</t>
+          <t>West Nyack</t>
         </is>
       </c>
       <c r="E39" s="13" t="inlineStr">
@@ -20377,17 +20377,17 @@
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="G39" s="13" t="inlineStr">
         <is>
-          <t>Best offer</t>
+          <t>Make offer / lot</t>
         </is>
       </c>
       <c r="H39" s="15" t="n"/>
       <c r="I39" s="13" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="J39" s="13" t="inlineStr"/>
@@ -20409,7 +20409,7 @@
       </c>
       <c r="O39" s="14" t="inlineStr">
         <is>
-          <t>Assorted secondhand consignment merchandise; one buyer preferred for most/all; pricing negotiable; buyer arranges pickup.</t>
+          <t>One-man auto body shop closing/retirement (Park Ridge / West Nyack NY-NJ border). Heat lamps, Kansas jack pullers, Miller 200 welder, generators, sheet-metal brake, hydraulic press, plasma cutter, engine hoist. Posted Aug 16; still open 2026-10-19.</t>
         </is>
       </c>
     </row>
@@ -20421,17 +20421,17 @@
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>Body shop closing after 50 years – tools, welder, generators, plasma</t>
+          <t>Woodworkers shop closing sale – shop tools &amp; hand tools</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>tools liquidation</t>
+          <t>woodworking shop closing</t>
         </is>
       </c>
       <c r="D40" s="13" t="inlineStr">
         <is>
-          <t>West Nyack</t>
+          <t>Tappan</t>
         </is>
       </c>
       <c r="E40" s="13" t="inlineStr">
@@ -20440,17 +20440,17 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t>Make offer / lot</t>
+          <t>Priced individually (some free)</t>
         </is>
       </c>
       <c r="H40" s="15" t="n"/>
       <c r="I40" s="13" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="J40" s="13" t="inlineStr"/>
@@ -20472,120 +20472,124 @@
       </c>
       <c r="O40" s="14" t="inlineStr">
         <is>
-          <t>One-man auto body shop closing/retirement (Park Ridge / West Nyack NY-NJ border). Heat lamps, Kansas jack pullers, Miller 200 welder, generators, sheet-metal brake, hydraulic press, plasma cutter, engine hoist. Posted Aug 16; still open 2026-10-19.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" outlineLevel="1">
-      <c r="A41" s="13" t="inlineStr">
-        <is>
-          <t>CT / Hudson Valley</t>
-        </is>
-      </c>
-      <c r="B41" s="14" t="inlineStr">
-        <is>
-          <t>Woodworkers shop closing sale – shop tools &amp; hand tools</t>
-        </is>
-      </c>
-      <c r="C41" s="13" t="inlineStr">
-        <is>
-          <t>woodworking shop closing</t>
-        </is>
-      </c>
-      <c r="D41" s="13" t="inlineStr">
-        <is>
-          <t>Tappan</t>
-        </is>
-      </c>
-      <c r="E41" s="13" t="inlineStr">
+          <t>Ongoing shop-closing sale at 61 Main St, Tappan; many shop and hand tools, schedule a visit. Near the West Nyack body-shop sale (bl-054) for one trip.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — CT / Hudson Valley</t>
+        </is>
+      </c>
+      <c r="B41" s="17" t="inlineStr">
+        <is>
+          <t>8 item(s)</t>
+        </is>
+      </c>
+      <c r="C41" s="18" t="n"/>
+      <c r="D41" s="18" t="n"/>
+      <c r="E41" s="18" t="n"/>
+      <c r="F41" s="18" t="n"/>
+      <c r="G41" s="18" t="n"/>
+      <c r="H41" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="18" t="n"/>
+      <c r="J41" s="18" t="n"/>
+      <c r="K41" s="18" t="n"/>
+      <c r="L41" s="18" t="n"/>
+      <c r="M41" s="18" t="n"/>
+      <c r="N41" s="18" t="n"/>
+      <c r="O41" s="18" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>▸ NYC / Long Island / NJ  (27)</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="n"/>
+      <c r="C42" s="12" t="n"/>
+      <c r="D42" s="12" t="n"/>
+      <c r="E42" s="12" t="n"/>
+      <c r="F42" s="12" t="n"/>
+      <c r="G42" s="12" t="n"/>
+      <c r="H42" s="12" t="n"/>
+      <c r="I42" s="12" t="n"/>
+      <c r="J42" s="12" t="n"/>
+      <c r="K42" s="12" t="n"/>
+      <c r="L42" s="12" t="n"/>
+      <c r="M42" s="12" t="n"/>
+      <c r="N42" s="12" t="n"/>
+      <c r="O42" s="12" t="n"/>
+    </row>
+    <row r="43" outlineLevel="1">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>Met Foodmarkets turnkey grocery liquidation (Grafe Auction)</t>
+        </is>
+      </c>
+      <c r="C43" s="13" t="inlineStr">
+        <is>
+          <t>store closing</t>
+        </is>
+      </c>
+      <c r="D43" s="13" t="inlineStr">
+        <is>
+          <t>Bronx</t>
+        </is>
+      </c>
+      <c r="E43" s="13" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
       </c>
-      <c r="F41" s="13" t="n">
-        <v>179</v>
-      </c>
-      <c r="G41" s="13" t="inlineStr">
-        <is>
-          <t>Priced individually (some free)</t>
-        </is>
-      </c>
-      <c r="H41" s="15" t="n"/>
-      <c r="I41" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-      <c r="J41" s="13" t="inlineStr"/>
-      <c r="K41" s="13" t="inlineStr">
-        <is>
-          <t>Craigslist</t>
-        </is>
-      </c>
-      <c r="L41" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M41" s="13" t="inlineStr"/>
-      <c r="N41" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O41" s="14" t="inlineStr">
-        <is>
-          <t>Ongoing shop-closing sale at 61 Main St, Tappan; many shop and hand tools, schedule a visit. Near the West Nyack body-shop sale (bl-054) for one trip.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — CT / Hudson Valley</t>
-        </is>
-      </c>
-      <c r="B42" s="17" t="inlineStr">
-        <is>
-          <t>9 item(s)</t>
-        </is>
-      </c>
-      <c r="C42" s="18" t="n"/>
-      <c r="D42" s="18" t="n"/>
-      <c r="E42" s="18" t="n"/>
-      <c r="F42" s="18" t="n"/>
-      <c r="G42" s="18" t="n"/>
-      <c r="H42" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I42" s="18" t="n"/>
-      <c r="J42" s="18" t="n"/>
-      <c r="K42" s="18" t="n"/>
-      <c r="L42" s="18" t="n"/>
-      <c r="M42" s="18" t="n"/>
-      <c r="N42" s="18" t="n"/>
-      <c r="O42" s="18" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="11" t="inlineStr">
-        <is>
-          <t>▸ NYC / Long Island / NJ  (26)</t>
-        </is>
-      </c>
-      <c r="B43" s="12" t="n"/>
-      <c r="C43" s="12" t="n"/>
-      <c r="D43" s="12" t="n"/>
-      <c r="E43" s="12" t="n"/>
-      <c r="F43" s="12" t="n"/>
-      <c r="G43" s="12" t="n"/>
-      <c r="H43" s="12" t="n"/>
-      <c r="I43" s="12" t="n"/>
-      <c r="J43" s="12" t="n"/>
-      <c r="K43" s="12" t="n"/>
-      <c r="L43" s="12" t="n"/>
-      <c r="M43" s="12" t="n"/>
-      <c r="N43" s="12" t="n"/>
-      <c r="O43" s="12" t="n"/>
+      <c r="F43" s="13" t="n">
+        <v>181</v>
+      </c>
+      <c r="G43" s="13" t="inlineStr">
+        <is>
+          <t>Online auction</t>
+        </is>
+      </c>
+      <c r="H43" s="15" t="n"/>
+      <c r="I43" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="J43" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-11 01:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K43" s="13" t="inlineStr">
+        <is>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L43" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M43" s="13" t="inlineStr"/>
+      <c r="N43" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O43" s="14" t="inlineStr">
+        <is>
+          <t>2 Hussmann compressor racks, 3-room Amerikooler walk-in cooler/freezer, Hussmann/Hill Phoenix remote cases, 24+ frozen doors, True/Red Bull merchandisers, Hobart mixer-grinder and wrappers, Lyons checkouts, NCR POS, Storflex shelving. Preview Nov 11 9AM-12PM; begins closing Nov 11 1PM EST.</t>
+        </is>
+      </c>
     </row>
     <row r="44" outlineLevel="1">
       <c r="A44" s="13" t="inlineStr">
@@ -22241,7 +22245,7 @@
       </c>
       <c r="B70" s="17" t="inlineStr">
         <is>
-          <t>26 item(s)</t>
+          <t>27 item(s)</t>
         </is>
       </c>
       <c r="C70" s="18" t="n"/>
@@ -23380,7 +23384,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N38" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N39" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N40" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N43" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N44" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N45" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N46" r:id="rId32"/>
@@ -23429,7 +23433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O36"/>
+  <dimension ref="A1:O37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -23591,7 +23595,7 @@
       </c>
       <c r="O2" s="14" t="inlineStr">
         <is>
-          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23654,7 +23658,7 @@
       </c>
       <c r="O3" s="14" t="inlineStr">
         <is>
-          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23784,7 +23788,7 @@
       </c>
       <c r="O5" s="14" t="inlineStr">
         <is>
-          <t>Online auction, closes Thu Oct 22 8:37 PM ET. $12.50 high bid (4 bids) as of 2026-10-18. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Online auction, closes Thu Oct 22 8:37 PM ET. $12.50 high bid (4 bids) as of 2026-10-18. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23989,7 +23993,7 @@
       </c>
       <c r="O8" s="14" t="inlineStr">
         <is>
-          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24054,7 +24058,7 @@
       </c>
       <c r="O9" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24119,7 +24123,7 @@
       </c>
       <c r="O10" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24184,7 +24188,7 @@
       </c>
       <c r="O11" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24314,7 +24318,7 @@
       </c>
       <c r="O13" s="14" t="inlineStr">
         <is>
-          <t>Lots close in sequence from Oct 21 2 PM ET. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Lots close in sequence from Oct 21 2 PM ET. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24379,7 +24383,7 @@
       </c>
       <c r="O14" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24444,7 +24448,7 @@
       </c>
       <c r="O15" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24507,7 +24511,7 @@
       </c>
       <c r="O16" s="14" t="inlineStr">
         <is>
-          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24570,7 +24574,7 @@
       </c>
       <c r="O17" s="14" t="inlineStr">
         <is>
-          <t>Page conflicts: Oct 21 or 22 9 AM (later date used). Closest find. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Page conflicts: Oct 21 or 22 9 AM (later date used). Closest find. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24633,7 +24637,7 @@
       </c>
       <c r="O18" s="14" t="inlineStr">
         <is>
-          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24696,7 +24700,7 @@
       </c>
       <c r="O19" s="14" t="inlineStr">
         <is>
-          <t>Closes Oct 21 10 or 11 AM (later used). Shippable. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Closes Oct 21 10 or 11 AM (later used). Shippable. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24759,7 +24763,7 @@
       </c>
       <c r="O20" s="14" t="inlineStr">
         <is>
-          <t>Oct 21; start time not captured (placeholder 6 PM). [removed 2026-10-21: live webcast auction held Oct 21; listing page now HTTP 503] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Oct 21; start time not captured (placeholder 6 PM). [removed 2026-10-21: live webcast auction held Oct 21; listing page now HTTP 503] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24822,7 +24826,7 @@
       </c>
       <c r="O21" s="14" t="inlineStr">
         <is>
-          <t>Absolute / no reserve. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Absolute / no reserve. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24885,7 +24889,7 @@
       </c>
       <c r="O22" s="14" t="inlineStr">
         <is>
-          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24948,7 +24952,7 @@
       </c>
       <c r="O23" s="14" t="inlineStr">
         <is>
-          <t>Some kitchen gear only. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Some kitchen gear only. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25011,7 +25015,7 @@
       </c>
       <c r="O24" s="14" t="inlineStr">
         <is>
-          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25074,7 +25078,7 @@
       </c>
       <c r="O25" s="14" t="inlineStr">
         <is>
-          <t>Small lot. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Small lot. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25137,7 +25141,7 @@
       </c>
       <c r="O26" s="14" t="inlineStr">
         <is>
-          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25206,7 +25210,7 @@
       </c>
       <c r="O27" s="14" t="inlineStr">
         <is>
-          <t>About 3 days left as of Oct 18 (~Oct 21; exact time not captured). Pickup Sat Oct 24 12–4 PM by appointment. Used, minor wear. eBay asks $200–420; rough resale $150–250. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>About 3 days left as of Oct 18 (~Oct 21; exact time not captured). Pickup Sat Oct 24 12–4 PM by appointment. Used, minor wear. eBay asks $200–420; rough resale $150–250. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25336,7 +25340,7 @@
       </c>
       <c r="O29" s="14" t="inlineStr">
         <is>
-          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25403,7 +25407,7 @@
       </c>
       <c r="O30" s="14" t="inlineStr">
         <is>
-          <t>Wed Oct 21 4 PM. NYC 10013. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Wed Oct 21 4 PM. NYC 10013. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25470,7 +25474,7 @@
       </c>
       <c r="O31" s="14" t="inlineStr">
         <is>
-          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25537,7 +25541,7 @@
       </c>
       <c r="O32" s="14" t="inlineStr">
         <is>
-          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25604,7 +25608,7 @@
       </c>
       <c r="O33" s="14" t="inlineStr">
         <is>
-          <t>Ends Wed Oct 21 8:30 PM EDT. PCI warehouse, 36 Ludlow St, Stamford CT. Page lists preview Oct 28 and removal Thu Oct 29 11-3 (after close). Shipping/delivery available; payment due on pickup day. Items still being added. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Ends Wed Oct 21 8:30 PM EDT. PCI warehouse, 36 Ludlow St, Stamford CT. Page lists preview Oct 28 and removal Thu Oct 29 11-3 (after close). Shipping/delivery available; payment due on pickup day. Items still being added. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25667,7 +25671,7 @@
       </c>
       <c r="O34" s="14" t="inlineStr">
         <is>
-          <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25734,7 +25738,7 @@
       </c>
       <c r="O35" s="14" t="inlineStr">
         <is>
-          <t>Ends Oct 21 7 PM CDT (8 PM ET). 1500 Somerset Ave, Windber PA. Pickups Oct 24-28. Hardware store, not appliance parts. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Ends Oct 21 7 PM CDT (8 PM ET). 1500 Somerset Ave, Windber PA. Pickups Oct 24-28. Hardware store, not appliance parts. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25801,12 +25805,75 @@
       </c>
       <c r="O36" s="14" t="inlineStr">
         <is>
-          <t>Ends Oct 22 7 PM CDT (8 PM ET). Same store as Day 1; pickups Oct 24-28. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+          <t>Ends Oct 22 7 PM CDT (8 PM ET). Same store as Day 1; pickups Oct 24-28. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed]</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>CT / Hudson Valley</t>
+        </is>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>Consignment shop remaining inventory, bulk buyer wanted</t>
+        </is>
+      </c>
+      <c r="C37" s="13" t="inlineStr">
+        <is>
+          <t>store closing</t>
+        </is>
+      </c>
+      <c r="D37" s="13" t="inlineStr">
+        <is>
+          <t>Nyack</t>
+        </is>
+      </c>
+      <c r="E37" s="13" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="F37" s="13" t="n">
+        <v>175</v>
+      </c>
+      <c r="G37" s="13" t="inlineStr">
+        <is>
+          <t>Best offer</t>
+        </is>
+      </c>
+      <c r="H37" s="15" t="n"/>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="J37" s="13" t="inlineStr"/>
+      <c r="K37" s="13" t="inlineStr">
+        <is>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L37" s="13" t="inlineStr">
+        <is>
+          <t>REMOVED</t>
+        </is>
+      </c>
+      <c r="M37" s="13" t="inlineStr"/>
+      <c r="N37" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O37" s="14" t="inlineStr">
+        <is>
+          <t>Assorted secondhand consignment merchandise; one buyer preferred for most/all; pricing negotiable; buyer arranges pickup. [Removed 2026-10-23: CL post flagged for removal]</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O36"/>
+  <autoFilter ref="A1:O37"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
@@ -25843,6 +25910,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N35" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Lot Recon update 2026-10-24 6pm ET
</commit_message>
<xml_diff>
--- a/lot_recon.xlsx
+++ b/lot_recon.xlsx
@@ -21,7 +21,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Wolf Used'!$A$1:$O$188</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Wolf Unclear'!$A$1:$O$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$103</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 2026-10-24 14:02 ET</t>
+          <t>Last updated: 2026-10-24 18:02 ET</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Active listings: 311 · Removed: 38</t>
+          <t>Active listings: 311 · Removed: 39</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9">
@@ -679,7 +679,7 @@
         <v>165</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>612948.6</v>
+        <v>613568.6</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
@@ -714,7 +714,7 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13">
@@ -727,7 +727,7 @@
         <v>311</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>1438809.58</v>
+        <v>1439429.58</v>
       </c>
     </row>
     <row r="15">
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C18" t="n">
         <v>0</v>
@@ -833,7 +833,7 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
@@ -842,7 +842,7 @@
         <v>2</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>6380</v>
+        <v>7375</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C24" t="n">
         <v>1</v>
@@ -1031,7 +1031,7 @@
         <v>7</v>
       </c>
       <c r="E24" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F24" t="n">
         <v>24</v>
@@ -1040,7 +1040,7 @@
         <v>28</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>440366</v>
+        <v>439991</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -5783,7 +5783,7 @@
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>▸ North Shore / Merrimack Valley / S. NH  (3)</t>
+          <t>▸ North Shore / Merrimack Valley / S. NH  (4)</t>
         </is>
       </c>
       <c r="B11" s="12" t="n"/>
@@ -6000,122 +6000,118 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="17" t="inlineStr">
+    <row r="15" outlineLevel="1">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>North Shore / Merrimack Valley / S. NH</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>Wolf CG304P/S/LP 30" gas cooktop (LP), ~3 yrs old, lightly used</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>range/rangetop/oven/cooktop</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Kingston</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="n">
+        <v>57</v>
+      </c>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>$995</t>
+        </is>
+      </c>
+      <c r="H15" s="15" t="n">
+        <v>995</v>
+      </c>
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="J15" s="13" t="inlineStr"/>
+      <c r="K15" s="13" t="inlineStr">
+        <is>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L15" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M15" s="13" t="inlineStr"/>
+      <c r="N15" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O15" s="14" t="inlineStr">
+        <is>
+          <t>By owner. Seller cites current retail $2,410. LP (propane) version, may need conversion kit for natural gas buyers. Moderate margin at $995; negotiate down for a real flip.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Subtotal — North Shore / Merrimack Valley / S. NH</t>
         </is>
       </c>
-      <c r="B15" s="17" t="inlineStr">
-        <is>
-          <t>3 item(s)</t>
-        </is>
-      </c>
-      <c r="C15" s="18" t="n"/>
-      <c r="D15" s="18" t="n"/>
-      <c r="E15" s="18" t="n"/>
-      <c r="F15" s="18" t="n"/>
-      <c r="G15" s="18" t="n"/>
-      <c r="H15" s="19" t="n">
-        <v>380</v>
-      </c>
-      <c r="I15" s="18" t="n"/>
-      <c r="J15" s="18" t="n"/>
-      <c r="K15" s="18" t="n"/>
-      <c r="L15" s="18" t="n"/>
-      <c r="M15" s="18" t="n"/>
-      <c r="N15" s="18" t="n"/>
-      <c r="O15" s="18" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>4 item(s)</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="n"/>
+      <c r="D16" s="18" t="n"/>
+      <c r="E16" s="18" t="n"/>
+      <c r="F16" s="18" t="n"/>
+      <c r="G16" s="18" t="n"/>
+      <c r="H16" s="19" t="n">
+        <v>1375</v>
+      </c>
+      <c r="I16" s="18" t="n"/>
+      <c r="J16" s="18" t="n"/>
+      <c r="K16" s="18" t="n"/>
+      <c r="L16" s="18" t="n"/>
+      <c r="M16" s="18" t="n"/>
+      <c r="N16" s="18" t="n"/>
+      <c r="O16" s="18" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>▸ Cape Cod &amp; Islands  (2)</t>
         </is>
       </c>
-      <c r="B16" s="12" t="n"/>
-      <c r="C16" s="12" t="n"/>
-      <c r="D16" s="12" t="n"/>
-      <c r="E16" s="12" t="n"/>
-      <c r="F16" s="12" t="n"/>
-      <c r="G16" s="12" t="n"/>
-      <c r="H16" s="12" t="n"/>
-      <c r="I16" s="12" t="n"/>
-      <c r="J16" s="12" t="n"/>
-      <c r="K16" s="12" t="n"/>
-      <c r="L16" s="12" t="n"/>
-      <c r="M16" s="12" t="n"/>
-      <c r="N16" s="12" t="n"/>
-      <c r="O16" s="12" t="n"/>
-    </row>
-    <row r="17" outlineLevel="1">
-      <c r="A17" s="13" t="inlineStr">
-        <is>
-          <t>Cape Cod &amp; Islands</t>
-        </is>
-      </c>
-      <c r="B17" s="14" t="inlineStr">
-        <is>
-          <t>WOLF GAS STOVE</t>
-        </is>
-      </c>
-      <c r="C17" s="13" t="inlineStr">
-        <is>
-          <t>range/oven/rangetop</t>
-        </is>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>Dennis</t>
-        </is>
-      </c>
-      <c r="E17" s="13" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="F17" s="13" t="n">
-        <v>41</v>
-      </c>
-      <c r="G17" s="13" t="inlineStr">
-        <is>
-          <t>$300</t>
-        </is>
-      </c>
-      <c r="H17" s="15" t="n">
-        <v>300</v>
-      </c>
-      <c r="I17" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="J17" s="13" t="inlineStr"/>
-      <c r="K17" s="13" t="inlineStr">
-        <is>
-          <t>Craigslist</t>
-        </is>
-      </c>
-      <c r="L17" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M17" s="20" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
-      <c r="N17" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O17" s="14" t="inlineStr">
-        <is>
-          <t>Condition: used. FLIP?: $300 "Wolf gas stove", no details; if working range ~$1.5-3k</t>
-        </is>
-      </c>
+      <c r="B17" s="12" t="n"/>
+      <c r="C17" s="12" t="n"/>
+      <c r="D17" s="12" t="n"/>
+      <c r="E17" s="12" t="n"/>
+      <c r="F17" s="12" t="n"/>
+      <c r="G17" s="12" t="n"/>
+      <c r="H17" s="12" t="n"/>
+      <c r="I17" s="12" t="n"/>
+      <c r="J17" s="12" t="n"/>
+      <c r="K17" s="12" t="n"/>
+      <c r="L17" s="12" t="n"/>
+      <c r="M17" s="12" t="n"/>
+      <c r="N17" s="12" t="n"/>
+      <c r="O17" s="12" t="n"/>
     </row>
     <row r="18" outlineLevel="1">
       <c r="A18" s="13" t="inlineStr">
@@ -6125,7 +6121,7 @@
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>Wolf Gas Range</t>
+          <t>WOLF GAS STOVE</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
@@ -6135,7 +6131,7 @@
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>Harwich Port</t>
+          <t>Dennis</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
@@ -6144,19 +6140,19 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="G18" s="13" t="inlineStr">
         <is>
-          <t>$450</t>
+          <t>$300</t>
         </is>
       </c>
       <c r="H18" s="15" t="n">
-        <v>450</v>
+        <v>300</v>
       </c>
       <c r="I18" s="13" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="J18" s="13" t="inlineStr"/>
@@ -6182,118 +6178,126 @@
       </c>
       <c r="O18" s="14" t="inlineStr">
         <is>
+          <t>Condition: used. FLIP?: $300 "Wolf gas stove", no details; if working range ~$1.5-3k</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" outlineLevel="1">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>Cape Cod &amp; Islands</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>Wolf Gas Range</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>range/oven/rangetop</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>Harwich Port</t>
+        </is>
+      </c>
+      <c r="E19" s="13" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="n">
+        <v>49</v>
+      </c>
+      <c r="G19" s="13" t="inlineStr">
+        <is>
+          <t>$450</t>
+        </is>
+      </c>
+      <c r="H19" s="15" t="n">
+        <v>450</v>
+      </c>
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="J19" s="13" t="inlineStr"/>
+      <c r="K19" s="13" t="inlineStr">
+        <is>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L19" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M19" s="20" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
+      <c r="N19" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O19" s="14" t="inlineStr">
+        <is>
           <t>Condition: used. FLIP: actually 5-burner drop-in cooktop + granite, $450; rough resale $700-950</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="17" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Cape Cod &amp; Islands</t>
         </is>
       </c>
-      <c r="B19" s="17" t="inlineStr">
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>2 item(s)</t>
         </is>
       </c>
-      <c r="C19" s="18" t="n"/>
-      <c r="D19" s="18" t="n"/>
-      <c r="E19" s="18" t="n"/>
-      <c r="F19" s="18" t="n"/>
-      <c r="G19" s="18" t="n"/>
-      <c r="H19" s="19" t="n">
+      <c r="C20" s="18" t="n"/>
+      <c r="D20" s="18" t="n"/>
+      <c r="E20" s="18" t="n"/>
+      <c r="F20" s="18" t="n"/>
+      <c r="G20" s="18" t="n"/>
+      <c r="H20" s="19" t="n">
         <v>750</v>
       </c>
-      <c r="I19" s="18" t="n"/>
-      <c r="J19" s="18" t="n"/>
-      <c r="K19" s="18" t="n"/>
-      <c r="L19" s="18" t="n"/>
-      <c r="M19" s="18" t="n"/>
-      <c r="N19" s="18" t="n"/>
-      <c r="O19" s="18" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="I20" s="18" t="n"/>
+      <c r="J20" s="18" t="n"/>
+      <c r="K20" s="18" t="n"/>
+      <c r="L20" s="18" t="n"/>
+      <c r="M20" s="18" t="n"/>
+      <c r="N20" s="18" t="n"/>
+      <c r="O20" s="18" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>▸ Central / Western MA  (4)</t>
         </is>
       </c>
-      <c r="B20" s="12" t="n"/>
-      <c r="C20" s="12" t="n"/>
-      <c r="D20" s="12" t="n"/>
-      <c r="E20" s="12" t="n"/>
-      <c r="F20" s="12" t="n"/>
-      <c r="G20" s="12" t="n"/>
-      <c r="H20" s="12" t="n"/>
-      <c r="I20" s="12" t="n"/>
-      <c r="J20" s="12" t="n"/>
-      <c r="K20" s="12" t="n"/>
-      <c r="L20" s="12" t="n"/>
-      <c r="M20" s="12" t="n"/>
-      <c r="N20" s="12" t="n"/>
-      <c r="O20" s="12" t="n"/>
-    </row>
-    <row r="21" outlineLevel="1">
-      <c r="A21" s="13" t="inlineStr">
-        <is>
-          <t>Central / Western MA</t>
-        </is>
-      </c>
-      <c r="B21" s="14" t="inlineStr">
-        <is>
-          <t>Wolf stove 36 wide 6 burners exelent condition almos like new</t>
-        </is>
-      </c>
-      <c r="C21" s="13" t="inlineStr">
-        <is>
-          <t>range/oven/rangetop</t>
-        </is>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
-        <is>
-          <t>Worcester</t>
-        </is>
-      </c>
-      <c r="E21" s="13" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="F21" s="13" t="n">
-        <v>52</v>
-      </c>
-      <c r="G21" s="13" t="inlineStr">
-        <is>
-          <t>$5,800</t>
-        </is>
-      </c>
-      <c r="H21" s="15" t="n">
-        <v>5800</v>
-      </c>
-      <c r="I21" s="13" t="inlineStr"/>
-      <c r="J21" s="13" t="inlineStr"/>
-      <c r="K21" s="13" t="inlineStr">
-        <is>
-          <t>OfferUp</t>
-        </is>
-      </c>
-      <c r="L21" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M21" s="13" t="inlineStr"/>
-      <c r="N21" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O21" s="14" t="inlineStr">
-        <is>
-          <t>Condition: used.</t>
-        </is>
-      </c>
+      <c r="B21" s="12" t="n"/>
+      <c r="C21" s="12" t="n"/>
+      <c r="D21" s="12" t="n"/>
+      <c r="E21" s="12" t="n"/>
+      <c r="F21" s="12" t="n"/>
+      <c r="G21" s="12" t="n"/>
+      <c r="H21" s="12" t="n"/>
+      <c r="I21" s="12" t="n"/>
+      <c r="J21" s="12" t="n"/>
+      <c r="K21" s="12" t="n"/>
+      <c r="L21" s="12" t="n"/>
+      <c r="M21" s="12" t="n"/>
+      <c r="N21" s="12" t="n"/>
+      <c r="O21" s="12" t="n"/>
     </row>
     <row r="22" outlineLevel="1">
       <c r="A22" s="13" t="inlineStr">
@@ -6303,7 +6307,7 @@
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>Wolf double oven</t>
+          <t>Wolf stove 36 wide 6 burners exelent condition almos like new</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
@@ -6313,7 +6317,7 @@
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>Palmer</t>
+          <t>Worcester</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
@@ -6322,25 +6326,21 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>78</v>
+        <v>52</v>
       </c>
       <c r="G22" s="13" t="inlineStr">
         <is>
-          <t>$1,900</t>
+          <t>$5,800</t>
         </is>
       </c>
       <c r="H22" s="15" t="n">
-        <v>1900</v>
-      </c>
-      <c r="I22" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
+        <v>5800</v>
+      </c>
+      <c r="I22" s="13" t="inlineStr"/>
       <c r="J22" s="13" t="inlineStr"/>
       <c r="K22" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>OfferUp</t>
         </is>
       </c>
       <c r="L22" s="13" t="inlineStr">
@@ -6348,11 +6348,7 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M22" s="20" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
+      <c r="M22" s="13" t="inlineStr"/>
       <c r="N22" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -6360,7 +6356,7 @@
       </c>
       <c r="O22" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. FLIP: 60"-class 8-burner+griddle at $1,900; 60" Wolf asks $10-11k; rough resale $5-8k</t>
+          <t>Condition: used.</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6368,7 @@
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>36 inch Wolf range with 6 burners</t>
+          <t>Wolf double oven</t>
         </is>
       </c>
       <c r="C23" s="13" t="inlineStr">
@@ -6382,7 +6378,7 @@
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
-          <t>Springfield (Longmeadow)</t>
+          <t>Palmer</t>
         </is>
       </c>
       <c r="E23" s="13" t="inlineStr">
@@ -6391,25 +6387,25 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="G23" s="13" t="inlineStr">
         <is>
-          <t>$2,000</t>
+          <t>$1,900</t>
         </is>
       </c>
       <c r="H23" s="15" t="n">
-        <v>2000</v>
+        <v>1900</v>
       </c>
       <c r="I23" s="13" t="inlineStr">
         <is>
-          <t>posted ~18 days ago</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="J23" s="13" t="inlineStr"/>
       <c r="K23" s="13" t="inlineStr">
         <is>
-          <t>OfferUp</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L23" s="13" t="inlineStr">
@@ -6429,7 +6425,7 @@
       </c>
       <c r="O23" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. FLIP?: 36" dual fuel $2,000; rough resale $3-4k</t>
+          <t>Condition: used. FLIP: 60"-class 8-burner+griddle at $1,900; 60" Wolf asks $10-11k; rough resale $5-8k</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6437,7 @@
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>Wolf 30 Inch Gas Range, Good Condition, Stainless Steel – Northampton, MA</t>
+          <t>36 inch Wolf range with 6 burners</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
@@ -6451,7 +6447,7 @@
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
-          <t>Northampton</t>
+          <t>Springfield (Longmeadow)</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
@@ -6460,19 +6456,19 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="G24" s="13" t="inlineStr">
         <is>
-          <t>$1,925</t>
+          <t>$2,000</t>
         </is>
       </c>
       <c r="H24" s="15" t="n">
-        <v>1925</v>
+        <v>2000</v>
       </c>
       <c r="I24" s="13" t="inlineStr">
         <is>
-          <t>updated ~9 days ago</t>
+          <t>posted ~18 days ago</t>
         </is>
       </c>
       <c r="J24" s="13" t="inlineStr"/>
@@ -6486,7 +6482,11 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M24" s="13" t="inlineStr"/>
+      <c r="M24" s="20" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
       <c r="N24" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -6494,231 +6494,235 @@
       </c>
       <c r="O24" s="14" t="inlineStr">
         <is>
+          <t>Condition: used. FLIP?: 36" dual fuel $2,000; rough resale $3-4k</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" outlineLevel="1">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>Central / Western MA</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>Wolf 30 Inch Gas Range, Good Condition, Stainless Steel – Northampton, MA</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>range/oven/rangetop</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>Northampton</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="n">
+        <v>95</v>
+      </c>
+      <c r="G25" s="13" t="inlineStr">
+        <is>
+          <t>$1,925</t>
+        </is>
+      </c>
+      <c r="H25" s="15" t="n">
+        <v>1925</v>
+      </c>
+      <c r="I25" s="13" t="inlineStr">
+        <is>
+          <t>updated ~9 days ago</t>
+        </is>
+      </c>
+      <c r="J25" s="13" t="inlineStr"/>
+      <c r="K25" s="13" t="inlineStr">
+        <is>
+          <t>OfferUp</t>
+        </is>
+      </c>
+      <c r="L25" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M25" s="13" t="inlineStr"/>
+      <c r="N25" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O25" s="14" t="inlineStr">
+        <is>
           <t>Condition: used.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="17" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Central / Western MA</t>
         </is>
       </c>
-      <c r="B25" s="17" t="inlineStr">
+      <c r="B26" s="17" t="inlineStr">
         <is>
           <t>4 item(s)</t>
         </is>
       </c>
-      <c r="C25" s="18" t="n"/>
-      <c r="D25" s="18" t="n"/>
-      <c r="E25" s="18" t="n"/>
-      <c r="F25" s="18" t="n"/>
-      <c r="G25" s="18" t="n"/>
-      <c r="H25" s="19" t="n">
+      <c r="C26" s="18" t="n"/>
+      <c r="D26" s="18" t="n"/>
+      <c r="E26" s="18" t="n"/>
+      <c r="F26" s="18" t="n"/>
+      <c r="G26" s="18" t="n"/>
+      <c r="H26" s="19" t="n">
         <v>11625</v>
       </c>
-      <c r="I25" s="18" t="n"/>
-      <c r="J25" s="18" t="n"/>
-      <c r="K25" s="18" t="n"/>
-      <c r="L25" s="18" t="n"/>
-      <c r="M25" s="18" t="n"/>
-      <c r="N25" s="18" t="n"/>
-      <c r="O25" s="18" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="I26" s="18" t="n"/>
+      <c r="J26" s="18" t="n"/>
+      <c r="K26" s="18" t="n"/>
+      <c r="L26" s="18" t="n"/>
+      <c r="M26" s="18" t="n"/>
+      <c r="N26" s="18" t="n"/>
+      <c r="O26" s="18" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>▸ Rhode Island  (1)</t>
         </is>
       </c>
-      <c r="B26" s="12" t="n"/>
-      <c r="C26" s="12" t="n"/>
-      <c r="D26" s="12" t="n"/>
-      <c r="E26" s="12" t="n"/>
-      <c r="F26" s="12" t="n"/>
-      <c r="G26" s="12" t="n"/>
-      <c r="H26" s="12" t="n"/>
-      <c r="I26" s="12" t="n"/>
-      <c r="J26" s="12" t="n"/>
-      <c r="K26" s="12" t="n"/>
-      <c r="L26" s="12" t="n"/>
-      <c r="M26" s="12" t="n"/>
-      <c r="N26" s="12" t="n"/>
-      <c r="O26" s="12" t="n"/>
-    </row>
-    <row r="27" outlineLevel="1">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="B27" s="12" t="n"/>
+      <c r="C27" s="12" t="n"/>
+      <c r="D27" s="12" t="n"/>
+      <c r="E27" s="12" t="n"/>
+      <c r="F27" s="12" t="n"/>
+      <c r="G27" s="12" t="n"/>
+      <c r="H27" s="12" t="n"/>
+      <c r="I27" s="12" t="n"/>
+      <c r="J27" s="12" t="n"/>
+      <c r="K27" s="12" t="n"/>
+      <c r="L27" s="12" t="n"/>
+      <c r="M27" s="12" t="n"/>
+      <c r="N27" s="12" t="n"/>
+      <c r="O27" s="12" t="n"/>
+    </row>
+    <row r="28" outlineLevel="1">
+      <c r="A28" s="13" t="inlineStr">
         <is>
           <t>Rhode Island</t>
         </is>
       </c>
-      <c r="B27" s="14" t="inlineStr">
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>Wolf Range</t>
         </is>
       </c>
-      <c r="C27" s="13" t="inlineStr">
+      <c r="C28" s="13" t="inlineStr">
         <is>
           <t>range/oven/rangetop</t>
         </is>
       </c>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>Newport</t>
         </is>
       </c>
-      <c r="E27" s="13" t="inlineStr">
+      <c r="E28" s="13" t="inlineStr">
         <is>
           <t>RI</t>
         </is>
       </c>
-      <c r="F27" s="13" t="n">
+      <c r="F28" s="13" t="n">
         <v>50</v>
       </c>
-      <c r="G27" s="13" t="inlineStr">
+      <c r="G28" s="13" t="inlineStr">
         <is>
           <t>$300</t>
         </is>
       </c>
-      <c r="H27" s="15" t="n">
+      <c r="H28" s="15" t="n">
         <v>300</v>
       </c>
-      <c r="I27" s="13" t="inlineStr"/>
-      <c r="J27" s="13" t="inlineStr"/>
-      <c r="K27" s="13" t="inlineStr">
+      <c r="I28" s="13" t="inlineStr"/>
+      <c r="J28" s="13" t="inlineStr"/>
+      <c r="K28" s="13" t="inlineStr">
         <is>
           <t>OfferUp</t>
         </is>
       </c>
-      <c r="L27" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M27" s="20" t="inlineStr">
+      <c r="L28" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M28" s="20" t="inlineStr">
         <is>
           <t>FLIP</t>
         </is>
       </c>
-      <c r="N27" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O27" s="14" t="inlineStr">
+      <c r="N28" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O28" s="14" t="inlineStr">
         <is>
           <t>Condition: used. FLIP: "Wolf Range" $300 (was $900), all works; verify size/model; ~$1.5k+</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="17" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Rhode Island</t>
         </is>
       </c>
-      <c r="B28" s="17" t="inlineStr">
+      <c r="B29" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C28" s="18" t="n"/>
-      <c r="D28" s="18" t="n"/>
-      <c r="E28" s="18" t="n"/>
-      <c r="F28" s="18" t="n"/>
-      <c r="G28" s="18" t="n"/>
-      <c r="H28" s="19" t="n">
+      <c r="C29" s="18" t="n"/>
+      <c r="D29" s="18" t="n"/>
+      <c r="E29" s="18" t="n"/>
+      <c r="F29" s="18" t="n"/>
+      <c r="G29" s="18" t="n"/>
+      <c r="H29" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I28" s="18" t="n"/>
-      <c r="J28" s="18" t="n"/>
-      <c r="K28" s="18" t="n"/>
-      <c r="L28" s="18" t="n"/>
-      <c r="M28" s="18" t="n"/>
-      <c r="N28" s="18" t="n"/>
-      <c r="O28" s="18" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="11" t="inlineStr">
+      <c r="I29" s="18" t="n"/>
+      <c r="J29" s="18" t="n"/>
+      <c r="K29" s="18" t="n"/>
+      <c r="L29" s="18" t="n"/>
+      <c r="M29" s="18" t="n"/>
+      <c r="N29" s="18" t="n"/>
+      <c r="O29" s="18" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>▸ CT / Hudson Valley  (18)</t>
         </is>
       </c>
-      <c r="B29" s="12" t="n"/>
-      <c r="C29" s="12" t="n"/>
-      <c r="D29" s="12" t="n"/>
-      <c r="E29" s="12" t="n"/>
-      <c r="F29" s="12" t="n"/>
-      <c r="G29" s="12" t="n"/>
-      <c r="H29" s="12" t="n"/>
-      <c r="I29" s="12" t="n"/>
-      <c r="J29" s="12" t="n"/>
-      <c r="K29" s="12" t="n"/>
-      <c r="L29" s="12" t="n"/>
-      <c r="M29" s="12" t="n"/>
-      <c r="N29" s="12" t="n"/>
-      <c r="O29" s="12" t="n"/>
-    </row>
-    <row r="30" outlineLevel="1">
-      <c r="A30" s="13" t="inlineStr">
-        <is>
-          <t>CT / Hudson Valley</t>
-        </is>
-      </c>
-      <c r="B30" s="14" t="inlineStr">
-        <is>
-          <t>Stove wolf 36 inch used good condition</t>
-        </is>
-      </c>
-      <c r="C30" s="13" t="inlineStr">
-        <is>
-          <t>range/oven/rangetop</t>
-        </is>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
-        <is>
-          <t>East Hartford</t>
-        </is>
-      </c>
-      <c r="E30" s="13" t="inlineStr">
-        <is>
-          <t>CT</t>
-        </is>
-      </c>
-      <c r="F30" s="13" t="n">
-        <v>95</v>
-      </c>
-      <c r="G30" s="13" t="inlineStr">
-        <is>
-          <t>$4,450</t>
-        </is>
-      </c>
-      <c r="H30" s="15" t="n">
-        <v>4450</v>
-      </c>
-      <c r="I30" s="13" t="inlineStr"/>
-      <c r="J30" s="13" t="inlineStr"/>
-      <c r="K30" s="13" t="inlineStr">
-        <is>
-          <t>OfferUp</t>
-        </is>
-      </c>
-      <c r="L30" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M30" s="13" t="inlineStr"/>
-      <c r="N30" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O30" s="14" t="inlineStr">
-        <is>
-          <t>Condition: used.</t>
-        </is>
-      </c>
+      <c r="B30" s="12" t="n"/>
+      <c r="C30" s="12" t="n"/>
+      <c r="D30" s="12" t="n"/>
+      <c r="E30" s="12" t="n"/>
+      <c r="F30" s="12" t="n"/>
+      <c r="G30" s="12" t="n"/>
+      <c r="H30" s="12" t="n"/>
+      <c r="I30" s="12" t="n"/>
+      <c r="J30" s="12" t="n"/>
+      <c r="K30" s="12" t="n"/>
+      <c r="L30" s="12" t="n"/>
+      <c r="M30" s="12" t="n"/>
+      <c r="N30" s="12" t="n"/>
+      <c r="O30" s="12" t="n"/>
     </row>
     <row r="31" outlineLevel="1">
       <c r="A31" s="13" t="inlineStr">
@@ -6728,7 +6732,7 @@
       </c>
       <c r="B31" s="14" t="inlineStr">
         <is>
-          <t>Wolf 15” Induction Cooktop</t>
+          <t>Stove wolf 36 inch used good condition</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
@@ -6738,7 +6742,7 @@
       </c>
       <c r="D31" s="13" t="inlineStr">
         <is>
-          <t>Hartford</t>
+          <t>East Hartford</t>
         </is>
       </c>
       <c r="E31" s="13" t="inlineStr">
@@ -6747,15 +6751,15 @@
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="G31" s="13" t="inlineStr">
         <is>
-          <t>$1,200</t>
+          <t>$4,450</t>
         </is>
       </c>
       <c r="H31" s="15" t="n">
-        <v>1200</v>
+        <v>4450</v>
       </c>
       <c r="I31" s="13" t="inlineStr"/>
       <c r="J31" s="13" t="inlineStr"/>
@@ -6789,7 +6793,7 @@
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>Wolfe Electric Stove With Griddle</t>
+          <t>Wolf 15” Induction Cooktop</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
@@ -6799,7 +6803,7 @@
       </c>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>Bridgeport</t>
+          <t>Hartford</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
@@ -6808,15 +6812,15 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>139</v>
+        <v>99</v>
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t>$50</t>
+          <t>$1,200</t>
         </is>
       </c>
       <c r="H32" s="15" t="n">
-        <v>50</v>
+        <v>1200</v>
       </c>
       <c r="I32" s="13" t="inlineStr"/>
       <c r="J32" s="13" t="inlineStr"/>
@@ -6830,11 +6834,7 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M32" s="20" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
+      <c r="M32" s="13" t="inlineStr"/>
       <c r="N32" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -6842,7 +6842,7 @@
       </c>
       <c r="O32" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. FLIP?: "Wolfe" 15" modules $50; likely Wolf integrated modules; confirm brand</t>
+          <t>Condition: used.</t>
         </is>
       </c>
     </row>
@@ -6854,17 +6854,17 @@
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>Wolf Blender</t>
+          <t>Wolfe Electric Stove With Griddle</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>countertop</t>
+          <t>range/oven/rangetop</t>
         </is>
       </c>
       <c r="D33" s="13" t="inlineStr">
         <is>
-          <t>Fairfield</t>
+          <t>Bridgeport</t>
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr">
@@ -6873,15 +6873,15 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="G33" s="13" t="inlineStr">
         <is>
-          <t>$275</t>
+          <t>$50</t>
         </is>
       </c>
       <c r="H33" s="15" t="n">
-        <v>275</v>
+        <v>50</v>
       </c>
       <c r="I33" s="13" t="inlineStr"/>
       <c r="J33" s="13" t="inlineStr"/>
@@ -6895,7 +6895,11 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M33" s="13" t="inlineStr"/>
+      <c r="M33" s="20" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
       <c r="N33" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -6903,7 +6907,7 @@
       </c>
       <c r="O33" s="14" t="inlineStr">
         <is>
-          <t>Condition: used.</t>
+          <t>Condition: used. FLIP?: "Wolfe" 15" modules $50; likely Wolf integrated modules; confirm brand</t>
         </is>
       </c>
     </row>
@@ -6915,44 +6919,40 @@
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>Wolf Restaurant Range LP Gas</t>
+          <t>Wolf Blender</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>range/oven/rangetop</t>
+          <t>countertop</t>
         </is>
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>Pine Plains</t>
+          <t>Fairfield</t>
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>$100</t>
+          <t>$275</t>
         </is>
       </c>
       <c r="H34" s="15" t="n">
-        <v>100</v>
-      </c>
-      <c r="I34" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
+        <v>275</v>
+      </c>
+      <c r="I34" s="13" t="inlineStr"/>
       <c r="J34" s="13" t="inlineStr"/>
       <c r="K34" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>OfferUp</t>
         </is>
       </c>
       <c r="L34" s="13" t="inlineStr">
@@ -6968,7 +6968,7 @@
       </c>
       <c r="O34" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf)</t>
+          <t>Condition: used.</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="B35" s="14" t="inlineStr">
         <is>
-          <t>Wolf 36" Gas Oven - Good - Westport, CT</t>
+          <t>Wolf Restaurant Range LP Gas</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
@@ -6990,34 +6990,34 @@
       </c>
       <c r="D35" s="13" t="inlineStr">
         <is>
-          <t>Westport</t>
+          <t>Pine Plains</t>
         </is>
       </c>
       <c r="E35" s="13" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F35" s="13" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="G35" s="13" t="inlineStr">
         <is>
-          <t>$2,275</t>
+          <t>$100</t>
         </is>
       </c>
       <c r="H35" s="15" t="n">
-        <v>2275</v>
+        <v>100</v>
       </c>
       <c r="I35" s="13" t="inlineStr">
         <is>
-          <t>updated ~9 days ago</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="J35" s="13" t="inlineStr"/>
       <c r="K35" s="13" t="inlineStr">
         <is>
-          <t>OfferUp</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L35" s="13" t="inlineStr">
@@ -7033,7 +7033,7 @@
       </c>
       <c r="O35" s="14" t="inlineStr">
         <is>
-          <t>Condition: used.</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf)</t>
         </is>
       </c>
     </row>
@@ -7045,7 +7045,7 @@
       </c>
       <c r="B36" s="14" t="inlineStr">
         <is>
-          <t>Wolf Gas/Electric Cooktop 5 burner</t>
+          <t>Wolf 36" Gas Oven - Good - Westport, CT</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
@@ -7055,26 +7055,30 @@
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
-          <t>Clifton Park</t>
+          <t>Westport</t>
         </is>
       </c>
       <c r="E36" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="G36" s="13" t="inlineStr">
         <is>
-          <t>$250</t>
+          <t>$2,275</t>
         </is>
       </c>
       <c r="H36" s="15" t="n">
-        <v>250</v>
-      </c>
-      <c r="I36" s="13" t="inlineStr"/>
+        <v>2275</v>
+      </c>
+      <c r="I36" s="13" t="inlineStr">
+        <is>
+          <t>updated ~9 days ago</t>
+        </is>
+      </c>
       <c r="J36" s="13" t="inlineStr"/>
       <c r="K36" s="13" t="inlineStr">
         <is>
@@ -7086,11 +7090,7 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M36" s="20" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
+      <c r="M36" s="13" t="inlineStr"/>
       <c r="N36" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -7098,7 +7098,7 @@
       </c>
       <c r="O36" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. FLIP: 5-burner cooktop $250, excellent; rough resale $600-900</t>
+          <t>Condition: used.</t>
         </is>
       </c>
     </row>
@@ -7110,7 +7110,7 @@
       </c>
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>WOLF Range GE Monogram Fridge Wolf Hood Combo Stainless Steel</t>
+          <t>Wolf Gas/Electric Cooktop 5 burner</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
@@ -7120,12 +7120,12 @@
       </c>
       <c r="D37" s="13" t="inlineStr">
         <is>
-          <t>Stamford</t>
+          <t>Clifton Park</t>
         </is>
       </c>
       <c r="E37" s="13" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F37" s="13" t="n">
@@ -7133,11 +7133,11 @@
       </c>
       <c r="G37" s="13" t="inlineStr">
         <is>
-          <t>$9,000</t>
+          <t>$250</t>
         </is>
       </c>
       <c r="H37" s="15" t="n">
-        <v>9000</v>
+        <v>250</v>
       </c>
       <c r="I37" s="13" t="inlineStr"/>
       <c r="J37" s="13" t="inlineStr"/>
@@ -7151,7 +7151,11 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M37" s="13" t="inlineStr"/>
+      <c r="M37" s="20" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
       <c r="N37" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -7159,7 +7163,7 @@
       </c>
       <c r="O37" s="14" t="inlineStr">
         <is>
-          <t>Condition: used.</t>
+          <t>Condition: used. FLIP: 5-burner cooktop $250, excellent; rough resale $600-900</t>
         </is>
       </c>
     </row>
@@ -7171,7 +7175,7 @@
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>Wolf Range With Convection Oven Stainless Steel 30" 4 Burners</t>
+          <t>WOLF Range GE Monogram Fridge Wolf Hood Combo Stainless Steel</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
@@ -7194,11 +7198,11 @@
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>$1,900</t>
+          <t>$9,000</t>
         </is>
       </c>
       <c r="H38" s="15" t="n">
-        <v>1900</v>
+        <v>9000</v>
       </c>
       <c r="I38" s="13" t="inlineStr"/>
       <c r="J38" s="13" t="inlineStr"/>
@@ -7232,7 +7236,7 @@
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>Wolf 30” Double Oven In Great Condition Gas</t>
+          <t>Wolf Range With Convection Oven Stainless Steel 30" 4 Burners</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
@@ -7255,11 +7259,11 @@
       </c>
       <c r="G39" s="13" t="inlineStr">
         <is>
-          <t>$1,500</t>
+          <t>$1,900</t>
         </is>
       </c>
       <c r="H39" s="15" t="n">
-        <v>1500</v>
+        <v>1900</v>
       </c>
       <c r="I39" s="13" t="inlineStr"/>
       <c r="J39" s="13" t="inlineStr"/>
@@ -7293,7 +7297,7 @@
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>Spectacular Deal - Wolf Gas Range</t>
+          <t>Wolf 30” Double Oven In Great Condition Gas</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
@@ -7303,7 +7307,7 @@
       </c>
       <c r="D40" s="13" t="inlineStr">
         <is>
-          <t>Greenwich</t>
+          <t>Stamford</t>
         </is>
       </c>
       <c r="E40" s="13" t="inlineStr">
@@ -7312,15 +7316,15 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t>$2,000</t>
+          <t>$1,500</t>
         </is>
       </c>
       <c r="H40" s="15" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="I40" s="13" t="inlineStr"/>
       <c r="J40" s="13" t="inlineStr"/>
@@ -7334,11 +7338,7 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M40" s="20" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
+      <c r="M40" s="13" t="inlineStr"/>
       <c r="N40" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -7346,7 +7346,7 @@
       </c>
       <c r="O40" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. FLIP?: DF364C-LP 36" dual fuel $2,000; rough resale $3-4k</t>
+          <t>Condition: used.</t>
         </is>
       </c>
     </row>
@@ -7358,7 +7358,7 @@
       </c>
       <c r="B41" s="14" t="inlineStr">
         <is>
-          <t>WOLF Subzero 30" Gas Range Conventional Stove Stainless Steel</t>
+          <t>Spectacular Deal - Wolf Gas Range</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
@@ -7381,11 +7381,11 @@
       </c>
       <c r="G41" s="13" t="inlineStr">
         <is>
-          <t>$2,300</t>
+          <t>$2,000</t>
         </is>
       </c>
       <c r="H41" s="15" t="n">
-        <v>2300</v>
+        <v>2000</v>
       </c>
       <c r="I41" s="13" t="inlineStr"/>
       <c r="J41" s="13" t="inlineStr"/>
@@ -7399,7 +7399,11 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M41" s="13" t="inlineStr"/>
+      <c r="M41" s="20" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
       <c r="N41" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -7407,7 +7411,7 @@
       </c>
       <c r="O41" s="14" t="inlineStr">
         <is>
-          <t>Condition: used.</t>
+          <t>Condition: used. FLIP?: DF364C-LP 36" dual fuel $2,000; rough resale $3-4k</t>
         </is>
       </c>
     </row>
@@ -7419,7 +7423,7 @@
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>Wolf 36" Electric Stove Range Cooktop 5 Burners</t>
+          <t>WOLF Subzero 30" Gas Range Conventional Stove Stainless Steel</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
@@ -7442,11 +7446,11 @@
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>$1,400</t>
+          <t>$2,300</t>
         </is>
       </c>
       <c r="H42" s="15" t="n">
-        <v>1400</v>
+        <v>2300</v>
       </c>
       <c r="I42" s="13" t="inlineStr"/>
       <c r="J42" s="13" t="inlineStr"/>
@@ -7480,44 +7484,40 @@
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>WOLF Gourmet Elite Countertop Convection Oven (red knob)</t>
+          <t>Wolf 36" Electric Stove Range Cooktop 5 Burners</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
         <is>
-          <t>countertop</t>
+          <t>range/oven/rangetop</t>
         </is>
       </c>
       <c r="D43" s="13" t="inlineStr">
         <is>
-          <t>Armonk</t>
+          <t>Greenwich</t>
         </is>
       </c>
       <c r="E43" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="F43" s="13" t="n">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G43" s="13" t="inlineStr">
         <is>
-          <t>$650</t>
+          <t>$1,400</t>
         </is>
       </c>
       <c r="H43" s="15" t="n">
-        <v>650</v>
-      </c>
-      <c r="I43" s="13" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
+        <v>1400</v>
+      </c>
+      <c r="I43" s="13" t="inlineStr"/>
       <c r="J43" s="13" t="inlineStr"/>
       <c r="K43" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>OfferUp</t>
         </is>
       </c>
       <c r="L43" s="13" t="inlineStr">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="O43" s="14" t="inlineStr">
         <is>
-          <t>Good working condition; orig. $1,800. Updated 2026-10-15.</t>
+          <t>Condition: used.</t>
         </is>
       </c>
     </row>
@@ -7545,7 +7545,7 @@
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>Wolf Gourmet - Programmable Coffee System</t>
+          <t>WOLF Gourmet Elite Countertop Convection Oven (red knob)</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
@@ -7555,7 +7555,7 @@
       </c>
       <c r="D44" s="13" t="inlineStr">
         <is>
-          <t>Rye</t>
+          <t>Armonk</t>
         </is>
       </c>
       <c r="E44" s="13" t="inlineStr">
@@ -7564,21 +7564,25 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>$200</t>
+          <t>$650</t>
         </is>
       </c>
       <c r="H44" s="15" t="n">
-        <v>200</v>
-      </c>
-      <c r="I44" s="13" t="inlineStr"/>
+        <v>650</v>
+      </c>
+      <c r="I44" s="13" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
       <c r="J44" s="13" t="inlineStr"/>
       <c r="K44" s="13" t="inlineStr">
         <is>
-          <t>OfferUp</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L44" s="13" t="inlineStr">
@@ -7594,7 +7598,7 @@
       </c>
       <c r="O44" s="14" t="inlineStr">
         <is>
-          <t>Condition: used.</t>
+          <t>Good working condition; orig. $1,800. Updated 2026-10-15.</t>
         </is>
       </c>
     </row>
@@ -7606,17 +7610,17 @@
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>Wolf 30" E Series Built-In Convection Wall Oven SO30TE/S/TH</t>
+          <t>Wolf Gourmet - Programmable Coffee System</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
         <is>
-          <t>range/rangetop/oven/cooktop</t>
+          <t>countertop</t>
         </is>
       </c>
       <c r="D45" s="13" t="inlineStr">
         <is>
-          <t>Stony Point</t>
+          <t>Rye</t>
         </is>
       </c>
       <c r="E45" s="13" t="inlineStr">
@@ -7625,25 +7629,21 @@
         </is>
       </c>
       <c r="F45" s="13" t="n">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="G45" s="13" t="inlineStr">
         <is>
-          <t>$2,500</t>
+          <t>$200</t>
         </is>
       </c>
       <c r="H45" s="15" t="n">
-        <v>2500</v>
-      </c>
-      <c r="I45" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
+        <v>200</v>
+      </c>
+      <c r="I45" s="13" t="inlineStr"/>
       <c r="J45" s="13" t="inlineStr"/>
       <c r="K45" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>OfferUp</t>
         </is>
       </c>
       <c r="L45" s="13" t="inlineStr">
@@ -7659,7 +7659,7 @@
       </c>
       <c r="O45" s="14" t="inlineStr">
         <is>
-          <t>2017 stainless dual convection Wi-Fi; seller says works perfectly, dusty from reno. Pickup Stony Point NY (Garnerville CL). Mid-market ask; flip=false.</t>
+          <t>Condition: used.</t>
         </is>
       </c>
     </row>
@@ -7671,17 +7671,17 @@
       </c>
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>WOLF 30" Warming Drawer</t>
+          <t>Wolf 30" E Series Built-In Convection Wall Oven SO30TE/S/TH</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>range/oven/rangetop</t>
+          <t>range/rangetop/oven/cooktop</t>
         </is>
       </c>
       <c r="D46" s="13" t="inlineStr">
         <is>
-          <t>Wallkill</t>
+          <t>Stony Point</t>
         </is>
       </c>
       <c r="E46" s="13" t="inlineStr">
@@ -7690,21 +7690,25 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>$500</t>
+          <t>$2,500</t>
         </is>
       </c>
       <c r="H46" s="15" t="n">
-        <v>500</v>
-      </c>
-      <c r="I46" s="13" t="inlineStr"/>
+        <v>2500</v>
+      </c>
+      <c r="I46" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
       <c r="J46" s="13" t="inlineStr"/>
       <c r="K46" s="13" t="inlineStr">
         <is>
-          <t>OfferUp</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L46" s="13" t="inlineStr">
@@ -7720,7 +7724,7 @@
       </c>
       <c r="O46" s="14" t="inlineStr">
         <is>
-          <t>Condition: used.</t>
+          <t>2017 stainless dual convection Wi-Fi; seller says works perfectly, dusty from reno. Pickup Stony Point NY (Garnerville CL). Mid-market ask; flip=false.</t>
         </is>
       </c>
     </row>
@@ -7732,7 +7736,7 @@
       </c>
       <c r="B47" s="14" t="inlineStr">
         <is>
-          <t>Wolf 30inch GR304 natural gas range</t>
+          <t>WOLF 30" Warming Drawer</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
@@ -7742,7 +7746,7 @@
       </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>Wallkill</t>
         </is>
       </c>
       <c r="E47" s="13" t="inlineStr">
@@ -7751,25 +7755,21 @@
         </is>
       </c>
       <c r="F47" s="13" t="n">
-        <v>191</v>
+        <v>177</v>
       </c>
       <c r="G47" s="13" t="inlineStr">
         <is>
-          <t>$2,500</t>
+          <t>$500</t>
         </is>
       </c>
       <c r="H47" s="15" t="n">
-        <v>2500</v>
-      </c>
-      <c r="I47" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
+        <v>500</v>
+      </c>
+      <c r="I47" s="13" t="inlineStr"/>
       <c r="J47" s="13" t="inlineStr"/>
       <c r="K47" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>OfferUp</t>
         </is>
       </c>
       <c r="L47" s="13" t="inlineStr">
@@ -7789,118 +7789,118 @@
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="17" t="inlineStr">
+    <row r="48" outlineLevel="1">
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>CT / Hudson Valley</t>
+        </is>
+      </c>
+      <c r="B48" s="14" t="inlineStr">
+        <is>
+          <t>Wolf 30inch GR304 natural gas range</t>
+        </is>
+      </c>
+      <c r="C48" s="13" t="inlineStr">
+        <is>
+          <t>range/oven/rangetop</t>
+        </is>
+      </c>
+      <c r="D48" s="13" t="inlineStr">
+        <is>
+          <t>Florida</t>
+        </is>
+      </c>
+      <c r="E48" s="13" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="F48" s="13" t="n">
+        <v>191</v>
+      </c>
+      <c r="G48" s="13" t="inlineStr">
+        <is>
+          <t>$2,500</t>
+        </is>
+      </c>
+      <c r="H48" s="15" t="n">
+        <v>2500</v>
+      </c>
+      <c r="I48" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="J48" s="13" t="inlineStr"/>
+      <c r="K48" s="13" t="inlineStr">
+        <is>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L48" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M48" s="13" t="inlineStr"/>
+      <c r="N48" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O48" s="14" t="inlineStr">
+        <is>
+          <t>Condition: used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="17" t="inlineStr">
         <is>
           <t>Subtotal — CT / Hudson Valley</t>
         </is>
       </c>
-      <c r="B48" s="17" t="inlineStr">
+      <c r="B49" s="17" t="inlineStr">
         <is>
           <t>18 item(s)</t>
         </is>
       </c>
-      <c r="C48" s="18" t="n"/>
-      <c r="D48" s="18" t="n"/>
-      <c r="E48" s="18" t="n"/>
-      <c r="F48" s="18" t="n"/>
-      <c r="G48" s="18" t="n"/>
-      <c r="H48" s="19" t="n">
+      <c r="C49" s="18" t="n"/>
+      <c r="D49" s="18" t="n"/>
+      <c r="E49" s="18" t="n"/>
+      <c r="F49" s="18" t="n"/>
+      <c r="G49" s="18" t="n"/>
+      <c r="H49" s="19" t="n">
         <v>33050</v>
       </c>
-      <c r="I48" s="18" t="n"/>
-      <c r="J48" s="18" t="n"/>
-      <c r="K48" s="18" t="n"/>
-      <c r="L48" s="18" t="n"/>
-      <c r="M48" s="18" t="n"/>
-      <c r="N48" s="18" t="n"/>
-      <c r="O48" s="18" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="11" t="inlineStr">
-        <is>
-          <t>▸ NYC / Long Island / NJ  (65)</t>
-        </is>
-      </c>
-      <c r="B49" s="12" t="n"/>
-      <c r="C49" s="12" t="n"/>
-      <c r="D49" s="12" t="n"/>
-      <c r="E49" s="12" t="n"/>
-      <c r="F49" s="12" t="n"/>
-      <c r="G49" s="12" t="n"/>
-      <c r="H49" s="12" t="n"/>
-      <c r="I49" s="12" t="n"/>
-      <c r="J49" s="12" t="n"/>
-      <c r="K49" s="12" t="n"/>
-      <c r="L49" s="12" t="n"/>
-      <c r="M49" s="12" t="n"/>
-      <c r="N49" s="12" t="n"/>
-      <c r="O49" s="12" t="n"/>
-    </row>
-    <row r="50" outlineLevel="1">
-      <c r="A50" s="13" t="inlineStr">
-        <is>
-          <t>NYC / Long Island / NJ</t>
-        </is>
-      </c>
-      <c r="B50" s="14" t="inlineStr">
-        <is>
-          <t>Wolf Electric Insert</t>
-        </is>
-      </c>
-      <c r="C50" s="13" t="inlineStr">
-        <is>
-          <t>range/oven/rangetop</t>
-        </is>
-      </c>
-      <c r="D50" s="13" t="inlineStr">
-        <is>
-          <t>Central Islip</t>
-        </is>
-      </c>
-      <c r="E50" s="13" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="F50" s="13" t="n">
-        <v>154</v>
-      </c>
-      <c r="G50" s="13" t="inlineStr">
-        <is>
-          <t>$100</t>
-        </is>
-      </c>
-      <c r="H50" s="15" t="n">
-        <v>100</v>
-      </c>
-      <c r="I50" s="13" t="inlineStr"/>
-      <c r="J50" s="13" t="inlineStr"/>
-      <c r="K50" s="13" t="inlineStr">
-        <is>
-          <t>OfferUp</t>
-        </is>
-      </c>
-      <c r="L50" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M50" s="20" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
-      <c r="N50" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O50" s="14" t="inlineStr">
-        <is>
-          <t>Condition: used. FLIP?: 30" electric cooktop insert $100; rough resale $300-600</t>
-        </is>
-      </c>
+      <c r="I49" s="18" t="n"/>
+      <c r="J49" s="18" t="n"/>
+      <c r="K49" s="18" t="n"/>
+      <c r="L49" s="18" t="n"/>
+      <c r="M49" s="18" t="n"/>
+      <c r="N49" s="18" t="n"/>
+      <c r="O49" s="18" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="11" t="inlineStr">
+        <is>
+          <t>▸ NYC / Long Island / NJ  (64)</t>
+        </is>
+      </c>
+      <c r="B50" s="12" t="n"/>
+      <c r="C50" s="12" t="n"/>
+      <c r="D50" s="12" t="n"/>
+      <c r="E50" s="12" t="n"/>
+      <c r="F50" s="12" t="n"/>
+      <c r="G50" s="12" t="n"/>
+      <c r="H50" s="12" t="n"/>
+      <c r="I50" s="12" t="n"/>
+      <c r="J50" s="12" t="n"/>
+      <c r="K50" s="12" t="n"/>
+      <c r="L50" s="12" t="n"/>
+      <c r="M50" s="12" t="n"/>
+      <c r="N50" s="12" t="n"/>
+      <c r="O50" s="12" t="n"/>
     </row>
     <row r="51" outlineLevel="1">
       <c r="A51" s="13" t="inlineStr">
@@ -7910,7 +7910,7 @@
       </c>
       <c r="B51" s="14" t="inlineStr">
         <is>
-          <t>WOLF STOVE TOP + STOVE TOP &amp; Grill</t>
+          <t>Wolf Electric Insert</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
@@ -7920,7 +7920,7 @@
       </c>
       <c r="D51" s="13" t="inlineStr">
         <is>
-          <t>Jericho</t>
+          <t>Central Islip</t>
         </is>
       </c>
       <c r="E51" s="13" t="inlineStr">
@@ -7929,15 +7929,15 @@
         </is>
       </c>
       <c r="F51" s="13" t="n">
-        <v>168</v>
+        <v>154</v>
       </c>
       <c r="G51" s="13" t="inlineStr">
         <is>
-          <t>$700</t>
+          <t>$100</t>
         </is>
       </c>
       <c r="H51" s="15" t="n">
-        <v>700</v>
+        <v>100</v>
       </c>
       <c r="I51" s="13" t="inlineStr"/>
       <c r="J51" s="13" t="inlineStr"/>
@@ -7963,7 +7963,7 @@
       </c>
       <c r="O51" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. FLIP: 48" stovetop+grill $700; 48" rangetop ask $2,900; rough resale $1.5-2.5k</t>
+          <t>Condition: used. FLIP?: 30" electric cooktop insert $100; rough resale $300-600</t>
         </is>
       </c>
     </row>
@@ -7975,17 +7975,17 @@
       </c>
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>Wolf Gourmet Toaster Oven</t>
+          <t>WOLF STOVE TOP + STOVE TOP &amp; Grill</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>countertop</t>
+          <t>range/oven/rangetop</t>
         </is>
       </c>
       <c r="D52" s="13" t="inlineStr">
         <is>
-          <t>North Massapequa</t>
+          <t>Jericho</t>
         </is>
       </c>
       <c r="E52" s="13" t="inlineStr">
@@ -7998,11 +7998,11 @@
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>$350</t>
+          <t>$700</t>
         </is>
       </c>
       <c r="H52" s="15" t="n">
-        <v>350</v>
+        <v>700</v>
       </c>
       <c r="I52" s="13" t="inlineStr"/>
       <c r="J52" s="13" t="inlineStr"/>
@@ -8016,7 +8016,11 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M52" s="13" t="inlineStr"/>
+      <c r="M52" s="20" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
       <c r="N52" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -8024,7 +8028,7 @@
       </c>
       <c r="O52" s="14" t="inlineStr">
         <is>
-          <t>Condition: used.</t>
+          <t>Condition: used. FLIP: 48" stovetop+grill $700; 48" rangetop ask $2,900; rough resale $1.5-2.5k</t>
         </is>
       </c>
     </row>
@@ -8036,17 +8040,17 @@
       </c>
       <c r="B53" s="14" t="inlineStr">
         <is>
-          <t>Wolf Oven</t>
+          <t>Wolf Gourmet Toaster Oven</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>range/oven/rangetop</t>
+          <t>countertop</t>
         </is>
       </c>
       <c r="D53" s="13" t="inlineStr">
         <is>
-          <t>Bethpage</t>
+          <t>North Massapequa</t>
         </is>
       </c>
       <c r="E53" s="13" t="inlineStr">
@@ -8059,11 +8063,11 @@
       </c>
       <c r="G53" s="13" t="inlineStr">
         <is>
-          <t>$1,000</t>
+          <t>$350</t>
         </is>
       </c>
       <c r="H53" s="15" t="n">
-        <v>1000</v>
+        <v>350</v>
       </c>
       <c r="I53" s="13" t="inlineStr"/>
       <c r="J53" s="13" t="inlineStr"/>
@@ -8097,7 +8101,7 @@
       </c>
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>Wolf microwave</t>
+          <t>Wolf Oven</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
@@ -8107,7 +8111,7 @@
       </c>
       <c r="D54" s="13" t="inlineStr">
         <is>
-          <t>Massapequa Park</t>
+          <t>Bethpage</t>
         </is>
       </c>
       <c r="E54" s="13" t="inlineStr">
@@ -8116,15 +8120,15 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>$2,000</t>
+          <t>$1,000</t>
         </is>
       </c>
       <c r="H54" s="15" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="I54" s="13" t="inlineStr"/>
       <c r="J54" s="13" t="inlineStr"/>
@@ -8158,7 +8162,7 @@
       </c>
       <c r="B55" s="14" t="inlineStr">
         <is>
-          <t>Cook Top Wolf 36 Inch Gas Plus Griddle Wolf Hood Included</t>
+          <t>Wolf microwave</t>
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr">
@@ -8168,7 +8172,7 @@
       </c>
       <c r="D55" s="13" t="inlineStr">
         <is>
-          <t>Plandome</t>
+          <t>Massapequa Park</t>
         </is>
       </c>
       <c r="E55" s="13" t="inlineStr">
@@ -8177,15 +8181,15 @@
         </is>
       </c>
       <c r="F55" s="13" t="n">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="G55" s="13" t="inlineStr">
         <is>
-          <t>$1,500</t>
+          <t>$2,000</t>
         </is>
       </c>
       <c r="H55" s="15" t="n">
-        <v>1500</v>
+        <v>2000</v>
       </c>
       <c r="I55" s="13" t="inlineStr"/>
       <c r="J55" s="13" t="inlineStr"/>
@@ -8219,7 +8223,7 @@
       </c>
       <c r="B56" s="14" t="inlineStr">
         <is>
-          <t>Wolf Electric Double Oven</t>
+          <t>Cook Top Wolf 36 Inch Gas Plus Griddle Wolf Hood Included</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
@@ -8229,7 +8233,7 @@
       </c>
       <c r="D56" s="13" t="inlineStr">
         <is>
-          <t>Bronx</t>
+          <t>Plandome</t>
         </is>
       </c>
       <c r="E56" s="13" t="inlineStr">
@@ -8238,15 +8242,15 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>$600</t>
+          <t>$1,500</t>
         </is>
       </c>
       <c r="H56" s="15" t="n">
-        <v>600</v>
+        <v>1500</v>
       </c>
       <c r="I56" s="13" t="inlineStr"/>
       <c r="J56" s="13" t="inlineStr"/>
@@ -8260,11 +8264,7 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M56" s="20" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
+      <c r="M56" s="13" t="inlineStr"/>
       <c r="N56" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -8272,7 +8272,7 @@
       </c>
       <c r="O56" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. FLIP: electric double wall oven $600; comp ask $2,800; rough resale $1.5-2.5k</t>
+          <t>Condition: used.</t>
         </is>
       </c>
     </row>
@@ -8284,7 +8284,7 @@
       </c>
       <c r="B57" s="14" t="inlineStr">
         <is>
-          <t>Stove Wolf</t>
+          <t>Wolf Electric Double Oven</t>
         </is>
       </c>
       <c r="C57" s="13" t="inlineStr">
@@ -8307,11 +8307,11 @@
       </c>
       <c r="G57" s="13" t="inlineStr">
         <is>
-          <t>$950</t>
+          <t>$600</t>
         </is>
       </c>
       <c r="H57" s="15" t="n">
-        <v>950</v>
+        <v>600</v>
       </c>
       <c r="I57" s="13" t="inlineStr"/>
       <c r="J57" s="13" t="inlineStr"/>
@@ -8337,7 +8337,7 @@
       </c>
       <c r="O57" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. FLIP?: dealer "Stove Wolf" $950 w/ warranty; size unknown</t>
+          <t>Condition: used. FLIP: electric double wall oven $600; comp ask $2,800; rough resale $1.5-2.5k</t>
         </is>
       </c>
     </row>
@@ -8349,7 +8349,7 @@
       </c>
       <c r="B58" s="14" t="inlineStr">
         <is>
-          <t>Stove Wolf 30 Used</t>
+          <t>Stove Wolf</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
@@ -8372,11 +8372,11 @@
       </c>
       <c r="G58" s="13" t="inlineStr">
         <is>
-          <t>$2,500</t>
+          <t>$950</t>
         </is>
       </c>
       <c r="H58" s="15" t="n">
-        <v>2500</v>
+        <v>950</v>
       </c>
       <c r="I58" s="13" t="inlineStr"/>
       <c r="J58" s="13" t="inlineStr"/>
@@ -8390,7 +8390,11 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M58" s="13" t="inlineStr"/>
+      <c r="M58" s="20" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
       <c r="N58" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -8398,7 +8402,7 @@
       </c>
       <c r="O58" s="14" t="inlineStr">
         <is>
-          <t>Condition: used.</t>
+          <t>Condition: used. FLIP?: dealer "Stove Wolf" $950 w/ warranty; size unknown</t>
         </is>
       </c>
     </row>
@@ -8410,7 +8414,7 @@
       </c>
       <c r="B59" s="14" t="inlineStr">
         <is>
-          <t>Wolf R366 36” 6-Burner Professional Gas Range – $2,500 OBO</t>
+          <t>Stove Wolf 30 Used</t>
         </is>
       </c>
       <c r="C59" s="13" t="inlineStr">
@@ -8420,7 +8424,7 @@
       </c>
       <c r="D59" s="13" t="inlineStr">
         <is>
-          <t>Queens</t>
+          <t>Bronx</t>
         </is>
       </c>
       <c r="E59" s="13" t="inlineStr">
@@ -8429,7 +8433,7 @@
         </is>
       </c>
       <c r="F59" s="13" t="n">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G59" s="13" t="inlineStr">
         <is>
@@ -8439,11 +8443,7 @@
       <c r="H59" s="15" t="n">
         <v>2500</v>
       </c>
-      <c r="I59" s="13" t="inlineStr">
-        <is>
-          <t>posted ~13 days ago</t>
-        </is>
-      </c>
+      <c r="I59" s="13" t="inlineStr"/>
       <c r="J59" s="13" t="inlineStr"/>
       <c r="K59" s="13" t="inlineStr">
         <is>
@@ -8475,7 +8475,7 @@
       </c>
       <c r="B60" s="14" t="inlineStr">
         <is>
-          <t>OVEN WOLF RANGE</t>
+          <t>Wolf R366 36” 6-Burner Professional Gas Range – $2,500 OBO</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
@@ -8498,13 +8498,17 @@
       </c>
       <c r="G60" s="13" t="inlineStr">
         <is>
-          <t>$1,800</t>
+          <t>$2,500</t>
         </is>
       </c>
       <c r="H60" s="15" t="n">
-        <v>1800</v>
-      </c>
-      <c r="I60" s="13" t="inlineStr"/>
+        <v>2500</v>
+      </c>
+      <c r="I60" s="13" t="inlineStr">
+        <is>
+          <t>posted ~13 days ago</t>
+        </is>
+      </c>
       <c r="J60" s="13" t="inlineStr"/>
       <c r="K60" s="13" t="inlineStr">
         <is>
@@ -8536,7 +8540,7 @@
       </c>
       <c r="B61" s="14" t="inlineStr">
         <is>
-          <t>Sub Zero Fridge Wolf Stove and Dishwasher</t>
+          <t>OVEN WOLF RANGE</t>
         </is>
       </c>
       <c r="C61" s="13" t="inlineStr">
@@ -8546,34 +8550,30 @@
       </c>
       <c r="D61" s="13" t="inlineStr">
         <is>
-          <t>Haworth</t>
+          <t>Queens</t>
         </is>
       </c>
       <c r="E61" s="13" t="inlineStr">
         <is>
-          <t>NJ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F61" s="13" t="n">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G61" s="13" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$1,800</t>
         </is>
       </c>
       <c r="H61" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I61" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
+        <v>1800</v>
+      </c>
+      <c r="I61" s="13" t="inlineStr"/>
       <c r="J61" s="13" t="inlineStr"/>
       <c r="K61" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>OfferUp</t>
         </is>
       </c>
       <c r="L61" s="13" t="inlineStr">
@@ -8581,11 +8581,7 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M61" s="20" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
+      <c r="M61" s="13" t="inlineStr"/>
       <c r="N61" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -8593,7 +8589,7 @@
       </c>
       <c r="O61" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. FLIP: FREE Sub-Zero+Wolf stove+DW; posted 9/10, may be gone</t>
+          <t>Condition: used.</t>
         </is>
       </c>
     </row>
@@ -8605,7 +8601,7 @@
       </c>
       <c r="B62" s="14" t="inlineStr">
         <is>
-          <t>Wolf Stove and Sub Zero Fridge</t>
+          <t>Sub Zero Fridge Wolf Stove and Dishwasher</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
@@ -8628,15 +8624,15 @@
       </c>
       <c r="G62" s="13" t="inlineStr">
         <is>
-          <t>$1</t>
+          <t>$0</t>
         </is>
       </c>
       <c r="H62" s="15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I62" s="13" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="J62" s="13" t="inlineStr"/>
@@ -8662,7 +8658,7 @@
       </c>
       <c r="O62" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. FLIP: $1/best offer 30" Wolf + 36" Sub-Zero; posted 9/9, may be stale</t>
+          <t>Condition: used. FLIP: FREE Sub-Zero+Wolf stove+DW; posted 9/10, may be gone</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8670,7 @@
       </c>
       <c r="B63" s="14" t="inlineStr">
         <is>
-          <t>30in Wolf Gas Stove And Hood</t>
+          <t>Wolf Stove and Sub Zero Fridge</t>
         </is>
       </c>
       <c r="C63" s="13" t="inlineStr">
@@ -8684,30 +8680,34 @@
       </c>
       <c r="D63" s="13" t="inlineStr">
         <is>
-          <t>East Atlantic Beach</t>
+          <t>Haworth</t>
         </is>
       </c>
       <c r="E63" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="F63" s="13" t="n">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G63" s="13" t="inlineStr">
         <is>
-          <t>$1,000</t>
+          <t>$1</t>
         </is>
       </c>
       <c r="H63" s="15" t="n">
-        <v>1000</v>
-      </c>
-      <c r="I63" s="13" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="I63" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="J63" s="13" t="inlineStr"/>
       <c r="K63" s="13" t="inlineStr">
         <is>
-          <t>OfferUp</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L63" s="13" t="inlineStr">
@@ -8727,7 +8727,7 @@
       </c>
       <c r="O63" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. FLIP: 30" gas range + hood $1,000, working; rough resale $2-3k</t>
+          <t>Condition: used. FLIP: $1/best offer 30" Wolf + 36" Sub-Zero; posted 9/9, may be stale</t>
         </is>
       </c>
     </row>
@@ -8739,7 +8739,7 @@
       </c>
       <c r="B64" s="14" t="inlineStr">
         <is>
-          <t>Wolf Industrial Stove/griddle Combo</t>
+          <t>30in Wolf Gas Stove And Hood</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
@@ -8749,16 +8749,16 @@
       </c>
       <c r="D64" s="13" t="inlineStr">
         <is>
-          <t>Oradell</t>
+          <t>East Atlantic Beach</t>
         </is>
       </c>
       <c r="E64" s="13" t="inlineStr">
         <is>
-          <t>NJ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F64" s="13" t="n">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G64" s="13" t="inlineStr">
         <is>
@@ -8780,7 +8780,11 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M64" s="13" t="inlineStr"/>
+      <c r="M64" s="20" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
       <c r="N64" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -8788,7 +8792,7 @@
       </c>
       <c r="O64" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf)</t>
+          <t>Condition: used. FLIP: 30" gas range + hood $1,000, working; rough resale $2-3k</t>
         </is>
       </c>
     </row>
@@ -8800,22 +8804,22 @@
       </c>
       <c r="B65" s="14" t="inlineStr">
         <is>
-          <t>Wolf M Series CSO30CM/B/TH 30" convection steam oven (black, tubular handle)</t>
+          <t>Wolf Industrial Stove/griddle Combo</t>
         </is>
       </c>
       <c r="C65" s="13" t="inlineStr">
         <is>
-          <t>range/rangetop/oven/cooktop</t>
+          <t>range/oven/rangetop</t>
         </is>
       </c>
       <c r="D65" s="13" t="inlineStr">
         <is>
-          <t>Jackson Heights</t>
+          <t>Oradell</t>
         </is>
       </c>
       <c r="E65" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="F65" s="13" t="n">
@@ -8823,21 +8827,17 @@
       </c>
       <c r="G65" s="13" t="inlineStr">
         <is>
-          <t>$500</t>
+          <t>$1,000</t>
         </is>
       </c>
       <c r="H65" s="15" t="n">
-        <v>500</v>
-      </c>
-      <c r="I65" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
+        <v>1000</v>
+      </c>
+      <c r="I65" s="13" t="inlineStr"/>
       <c r="J65" s="13" t="inlineStr"/>
       <c r="K65" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>OfferUp</t>
         </is>
       </c>
       <c r="L65" s="13" t="inlineStr">
@@ -8845,11 +8845,7 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M65" s="20" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
+      <c r="M65" s="13" t="inlineStr"/>
       <c r="N65" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -8857,7 +8853,7 @@
       </c>
       <c r="O65" s="14" t="inlineStr">
         <is>
-          <t>Listed "like new", barely used; uninstalled and stored, seller clearing storage. Non-plumbed water tank. Strong flip at $500 for a current M Series built-in steam oven; verify it powers on and the tank/probe are included.</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf)</t>
         </is>
       </c>
     </row>
@@ -8869,17 +8865,17 @@
       </c>
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>Wolf MDD24TE/S/TH 24in E Series drop-down door microwave (2018)</t>
+          <t>Wolf M Series CSO30CM/B/TH 30" convection steam oven (black, tubular handle)</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>built-in microwave</t>
+          <t>range/rangetop/oven/cooktop</t>
         </is>
       </c>
       <c r="D66" s="13" t="inlineStr">
         <is>
-          <t>Astoria (Queens)</t>
+          <t>Jackson Heights</t>
         </is>
       </c>
       <c r="E66" s="13" t="inlineStr">
@@ -8888,19 +8884,19 @@
         </is>
       </c>
       <c r="F66" s="13" t="n">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G66" s="13" t="inlineStr">
         <is>
-          <t>$375</t>
+          <t>$500</t>
         </is>
       </c>
       <c r="H66" s="15" t="n">
-        <v>375</v>
+        <v>500</v>
       </c>
       <c r="I66" s="13" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="J66" s="13" t="inlineStr"/>
@@ -8926,7 +8922,7 @@
       </c>
       <c r="O66" s="14" t="inlineStr">
         <is>
-          <t>Storage-unit clearance, must go by Oct 31; says working (display lit, heating). Built-in, matches E Series ovens. Seller also has Miele G6785 SCVi panel-ready dishwasher; both for $595. Cash/Zelle at pickup.</t>
+          <t>Listed "like new", barely used; uninstalled and stored, seller clearing storage. Non-plumbed water tank. Strong flip at $500 for a current M Series built-in steam oven; verify it powers on and the tank/probe are included.</t>
         </is>
       </c>
     </row>
@@ -12034,7 +12030,7 @@
       </c>
       <c r="B115" s="17" t="inlineStr">
         <is>
-          <t>65 item(s)</t>
+          <t>64 item(s)</t>
         </is>
       </c>
       <c r="C115" s="18" t="n"/>
@@ -12043,7 +12039,7 @@
       <c r="F115" s="18" t="n"/>
       <c r="G115" s="18" t="n"/>
       <c r="H115" s="19" t="n">
-        <v>315576</v>
+        <v>315201</v>
       </c>
       <c r="I115" s="18" t="n"/>
       <c r="J115" s="18" t="n"/>
@@ -16175,14 +16171,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N32" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId21"/>
@@ -16200,7 +16196,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N45" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N46" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N47" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N50" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N48" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N51" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N52" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N53" r:id="rId39"/>
@@ -20341,9 +20337,9 @@
           <t>Hamilton Group via BidSpotter</t>
         </is>
       </c>
-      <c r="L36" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+      <c r="L36" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M36" s="13" t="inlineStr"/>
@@ -22851,9 +22847,9 @@
           <t>HiBid</t>
         </is>
       </c>
-      <c r="L78" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+      <c r="L78" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M78" s="13" t="inlineStr"/>
@@ -23955,7 +23951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O39"/>
+  <dimension ref="A1:O40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -24117,7 +24113,7 @@
       </c>
       <c r="O2" s="14" t="inlineStr">
         <is>
-          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24180,7 +24176,7 @@
       </c>
       <c r="O3" s="14" t="inlineStr">
         <is>
-          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24310,7 +24306,7 @@
       </c>
       <c r="O5" s="14" t="inlineStr">
         <is>
-          <t>Online auction, closes Thu Oct 22 8:37 PM ET. $12.50 high bid (4 bids) as of 2026-10-18. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Online auction, closes Thu Oct 22 8:37 PM ET. $12.50 high bid (4 bids) as of 2026-10-18. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24515,7 +24511,7 @@
       </c>
       <c r="O8" s="14" t="inlineStr">
         <is>
-          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24645,7 +24641,7 @@
       </c>
       <c r="O10" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24710,7 +24706,7 @@
       </c>
       <c r="O11" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24775,7 +24771,7 @@
       </c>
       <c r="O12" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24905,7 +24901,7 @@
       </c>
       <c r="O14" s="14" t="inlineStr">
         <is>
-          <t>Lots close in sequence from Oct 21 2 PM ET. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Lots close in sequence from Oct 21 2 PM ET. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24970,7 +24966,7 @@
       </c>
       <c r="O15" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25035,7 +25031,7 @@
       </c>
       <c r="O16" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25098,7 +25094,7 @@
       </c>
       <c r="O17" s="14" t="inlineStr">
         <is>
-          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25161,7 +25157,7 @@
       </c>
       <c r="O18" s="14" t="inlineStr">
         <is>
-          <t>Page conflicts: Oct 21 or 22 9 AM (later date used). Closest find. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Page conflicts: Oct 21 or 22 9 AM (later date used). Closest find. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25224,7 +25220,7 @@
       </c>
       <c r="O19" s="14" t="inlineStr">
         <is>
-          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25287,7 +25283,7 @@
       </c>
       <c r="O20" s="14" t="inlineStr">
         <is>
-          <t>Closes Oct 21 10 or 11 AM (later used). Shippable. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Closes Oct 21 10 or 11 AM (later used). Shippable. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25350,7 +25346,7 @@
       </c>
       <c r="O21" s="14" t="inlineStr">
         <is>
-          <t>Oct 21; start time not captured (placeholder 6 PM). [removed 2026-10-21: live webcast auction held Oct 21; listing page now HTTP 503] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Oct 21; start time not captured (placeholder 6 PM). [removed 2026-10-21: live webcast auction held Oct 21; listing page now HTTP 503] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25413,7 +25409,7 @@
       </c>
       <c r="O22" s="14" t="inlineStr">
         <is>
-          <t>Absolute / no reserve. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Absolute / no reserve. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25476,7 +25472,7 @@
       </c>
       <c r="O23" s="14" t="inlineStr">
         <is>
-          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25539,7 +25535,7 @@
       </c>
       <c r="O24" s="14" t="inlineStr">
         <is>
-          <t>Some kitchen gear only. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Some kitchen gear only. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25602,7 +25598,7 @@
       </c>
       <c r="O25" s="14" t="inlineStr">
         <is>
-          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25665,7 +25661,7 @@
       </c>
       <c r="O26" s="14" t="inlineStr">
         <is>
-          <t>Small lot. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Small lot. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25728,7 +25724,7 @@
       </c>
       <c r="O27" s="14" t="inlineStr">
         <is>
-          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25797,7 +25793,7 @@
       </c>
       <c r="O28" s="14" t="inlineStr">
         <is>
-          <t>About 3 days left as of Oct 18 (~Oct 21; exact time not captured). Pickup Sat Oct 24 12–4 PM by appointment. Used, minor wear. eBay asks $200–420; rough resale $150–250. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>About 3 days left as of Oct 18 (~Oct 21; exact time not captured). Pickup Sat Oct 24 12–4 PM by appointment. Used, minor wear. eBay asks $200–420; rough resale $150–250. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25927,7 +25923,7 @@
       </c>
       <c r="O30" s="14" t="inlineStr">
         <is>
-          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25994,7 +25990,7 @@
       </c>
       <c r="O31" s="14" t="inlineStr">
         <is>
-          <t>Wed Oct 21 4 PM. NYC 10013. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Wed Oct 21 4 PM. NYC 10013. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26061,7 +26057,7 @@
       </c>
       <c r="O32" s="14" t="inlineStr">
         <is>
-          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26128,7 +26124,7 @@
       </c>
       <c r="O33" s="14" t="inlineStr">
         <is>
-          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26258,7 +26254,7 @@
       </c>
       <c r="O35" s="14" t="inlineStr">
         <is>
-          <t>Ends Wed Oct 21 8:30 PM EDT. PCI warehouse, 36 Ludlow St, Stamford CT. Page lists preview Oct 28 and removal Thu Oct 29 11-3 (after close). Shipping/delivery available; payment due on pickup day. Items still being added. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Ends Wed Oct 21 8:30 PM EDT. PCI warehouse, 36 Ludlow St, Stamford CT. Page lists preview Oct 28 and removal Thu Oct 29 11-3 (after close). Shipping/delivery available; payment due on pickup day. Items still being added. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26321,7 +26317,7 @@
       </c>
       <c r="O36" s="14" t="inlineStr">
         <is>
-          <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26388,7 +26384,7 @@
       </c>
       <c r="O37" s="14" t="inlineStr">
         <is>
-          <t>Ends Oct 21 7 PM CDT (8 PM ET). 1500 Somerset Ave, Windber PA. Pickups Oct 24-28. Hardware store, not appliance parts. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Ends Oct 21 7 PM CDT (8 PM ET). 1500 Somerset Ave, Windber PA. Pickups Oct 24-28. Hardware store, not appliance parts. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26455,7 +26451,7 @@
       </c>
       <c r="O38" s="14" t="inlineStr">
         <is>
-          <t>Ends Oct 22 7 PM CDT (8 PM ET). Same store as Day 1; pickups Oct 24-28. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
+          <t>Ends Oct 22 7 PM CDT (8 PM ET). Same store as Day 1; pickups Oct 24-28. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26522,8 +26518,77 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>Wolf MDD24TE/S/TH 24in E Series drop-down door microwave (2018)</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr">
+        <is>
+          <t>built-in microwave</t>
+        </is>
+      </c>
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>Astoria (Queens)</t>
+        </is>
+      </c>
+      <c r="E40" s="13" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="F40" s="13" t="n">
+        <v>186</v>
+      </c>
+      <c r="G40" s="13" t="inlineStr">
+        <is>
+          <t>$375</t>
+        </is>
+      </c>
+      <c r="H40" s="15" t="n">
+        <v>375</v>
+      </c>
+      <c r="I40" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="J40" s="13" t="inlineStr"/>
+      <c r="K40" s="13" t="inlineStr">
+        <is>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L40" s="13" t="inlineStr">
+        <is>
+          <t>REMOVED</t>
+        </is>
+      </c>
+      <c r="M40" s="20" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
+      <c r="N40" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O40" s="14" t="inlineStr">
+        <is>
+          <t>Storage-unit clearance, must go by Oct 31; says working (display lit, heating). Built-in, matches E Series ovens. Seller also has Miele G6785 SCVi panel-ready dishwasher; both for $595. Cash/Zelle at pickup. | CL posting deleted by author (HTTP 410) 2026-10-24 evening</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O39"/>
+  <autoFilter ref="A1:O40"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
@@ -26563,6 +26628,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N38" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N40" r:id="rId39"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Lot Recon update 2026-10-25 11am ET: +2 Wolf Clifton NJ range bundles
</commit_message>
<xml_diff>
--- a/lot_recon.xlsx
+++ b/lot_recon.xlsx
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Appliance Parts'!$A$1:$O$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wolf New'!$A$1:$O$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Wolf Used'!$A$1:$O$184</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Wolf Used'!$A$1:$O$186</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Wolf Unclear'!$A$1:$O$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$103</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$43</definedName>
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 2026-10-25 07:58 ET</t>
+          <t>Last updated: 2026-10-25 11:07 ET</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Active listings: 309 · Removed: 42</t>
+          <t>Active listings: 311 · Removed: 42</t>
         </is>
       </c>
     </row>
@@ -676,10 +676,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>616860.6</v>
+        <v>635460.6</v>
       </c>
       <c r="D10" t="n">
         <v>2</v>
@@ -714,7 +714,7 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13">
@@ -724,10 +724,10 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>1442721.58</v>
+        <v>1461321.58</v>
       </c>
     </row>
     <row r="15">
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C24" t="n">
         <v>1</v>
@@ -1031,7 +1031,7 @@
         <v>7</v>
       </c>
       <c r="E24" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F24" t="n">
         <v>24</v>
@@ -1040,7 +1040,7 @@
         <v>28</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>444790</v>
+        <v>463390</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -5176,7 +5176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O184"/>
+  <dimension ref="A1:O186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -7884,7 +7884,7 @@
     <row r="50">
       <c r="A50" s="11" t="inlineStr">
         <is>
-          <t>▸ NYC / Long Island / NJ  (64)</t>
+          <t>▸ NYC / Long Island / NJ  (66)</t>
         </is>
       </c>
       <c r="B50" s="12" t="n"/>
@@ -11636,17 +11636,17 @@
       </c>
       <c r="B109" s="14" t="inlineStr">
         <is>
-          <t>36 INCH WOLF RANGE</t>
+          <t>Wolf Stainless 48" Gas Range (Propane) + Sub-Zero 48" Panel Ready Fridge</t>
         </is>
       </c>
       <c r="C109" s="13" t="inlineStr">
         <is>
-          <t>range/oven/rangetop</t>
+          <t>range/rangetop/oven/cooktop</t>
         </is>
       </c>
       <c r="D109" s="13" t="inlineStr">
         <is>
-          <t>Tennent</t>
+          <t>Clifton</t>
         </is>
       </c>
       <c r="E109" s="13" t="inlineStr">
@@ -11655,19 +11655,19 @@
         </is>
       </c>
       <c r="F109" s="13" t="n">
-        <v>221</v>
+        <v>194</v>
       </c>
       <c r="G109" s="13" t="inlineStr">
         <is>
-          <t>$3,500</t>
+          <t>$9,800</t>
         </is>
       </c>
       <c r="H109" s="15" t="n">
-        <v>3500</v>
+        <v>9800</v>
       </c>
       <c r="I109" s="13" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="J109" s="13" t="inlineStr"/>
@@ -11689,7 +11689,7 @@
       </c>
       <c r="O109" s="14" t="inlineStr">
         <is>
-          <t>Condition: used.</t>
+          <t>Clifton NJ dealer-style seller; likely repost of wf-135 (same price/spec). 6 burners w/ grill, LP; fridge water dispenser on front not working. Cash, can deliver. Bundle with fridge, thin margin.</t>
         </is>
       </c>
     </row>
@@ -11701,17 +11701,17 @@
       </c>
       <c r="B110" s="14" t="inlineStr">
         <is>
-          <t>wolf 30" duel fuel range</t>
+          <t>Wolf Stainless 48" Gas Range (Propane) + Sub-Zero 42" Panel Ready Fridge</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
         <is>
-          <t>range/oven/rangetop</t>
+          <t>range/rangetop/oven/cooktop</t>
         </is>
       </c>
       <c r="D110" s="13" t="inlineStr">
         <is>
-          <t>Tennent</t>
+          <t>Clifton</t>
         </is>
       </c>
       <c r="E110" s="13" t="inlineStr">
@@ -11720,19 +11720,19 @@
         </is>
       </c>
       <c r="F110" s="13" t="n">
-        <v>221</v>
+        <v>194</v>
       </c>
       <c r="G110" s="13" t="inlineStr">
         <is>
-          <t>$4,500</t>
+          <t>$8,800</t>
         </is>
       </c>
       <c r="H110" s="15" t="n">
-        <v>4500</v>
+        <v>8800</v>
       </c>
       <c r="I110" s="13" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="J110" s="13" t="inlineStr"/>
@@ -11754,7 +11754,7 @@
       </c>
       <c r="O110" s="14" t="inlineStr">
         <is>
-          <t>Condition: used.</t>
+          <t>Clifton NJ dealer-style seller (same as other Clifton listings). 6 burners w/ grill, LP; Sub-Zero 42in panel-ready built-in w/ ice maker. Cash, can deliver. Bundle, thin margin.</t>
         </is>
       </c>
     </row>
@@ -11766,7 +11766,7 @@
       </c>
       <c r="B111" s="14" t="inlineStr">
         <is>
-          <t>48" WOLF RANGETOP</t>
+          <t>36 INCH WOLF RANGE</t>
         </is>
       </c>
       <c r="C111" s="13" t="inlineStr">
@@ -11789,11 +11789,11 @@
       </c>
       <c r="G111" s="13" t="inlineStr">
         <is>
-          <t>$2,900</t>
+          <t>$3,500</t>
         </is>
       </c>
       <c r="H111" s="15" t="n">
-        <v>2900</v>
+        <v>3500</v>
       </c>
       <c r="I111" s="13" t="inlineStr">
         <is>
@@ -11831,7 +11831,7 @@
       </c>
       <c r="B112" s="14" t="inlineStr">
         <is>
-          <t>48” wolf range</t>
+          <t>wolf 30" duel fuel range</t>
         </is>
       </c>
       <c r="C112" s="13" t="inlineStr">
@@ -11854,11 +11854,11 @@
       </c>
       <c r="G112" s="13" t="inlineStr">
         <is>
-          <t>$5,200</t>
+          <t>$4,500</t>
         </is>
       </c>
       <c r="H112" s="15" t="n">
-        <v>5200</v>
+        <v>4500</v>
       </c>
       <c r="I112" s="13" t="inlineStr">
         <is>
@@ -11896,7 +11896,7 @@
       </c>
       <c r="B113" s="14" t="inlineStr">
         <is>
-          <t>48” wolf</t>
+          <t>48" WOLF RANGETOP</t>
         </is>
       </c>
       <c r="C113" s="13" t="inlineStr">
@@ -11919,11 +11919,11 @@
       </c>
       <c r="G113" s="13" t="inlineStr">
         <is>
-          <t>$5,300</t>
+          <t>$2,900</t>
         </is>
       </c>
       <c r="H113" s="15" t="n">
-        <v>5300</v>
+        <v>2900</v>
       </c>
       <c r="I113" s="13" t="inlineStr">
         <is>
@@ -11961,7 +11961,7 @@
       </c>
       <c r="B114" s="14" t="inlineStr">
         <is>
-          <t>30” wolf duel fuel range</t>
+          <t>48” wolf range</t>
         </is>
       </c>
       <c r="C114" s="13" t="inlineStr">
@@ -11984,11 +11984,11 @@
       </c>
       <c r="G114" s="13" t="inlineStr">
         <is>
-          <t>$4,500</t>
+          <t>$5,200</t>
         </is>
       </c>
       <c r="H114" s="15" t="n">
-        <v>4500</v>
+        <v>5200</v>
       </c>
       <c r="I114" s="13" t="inlineStr">
         <is>
@@ -12018,490 +12018,494 @@
         </is>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" s="17" t="inlineStr">
+    <row r="115" outlineLevel="1">
+      <c r="A115" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B115" s="14" t="inlineStr">
+        <is>
+          <t>48” wolf</t>
+        </is>
+      </c>
+      <c r="C115" s="13" t="inlineStr">
+        <is>
+          <t>range/oven/rangetop</t>
+        </is>
+      </c>
+      <c r="D115" s="13" t="inlineStr">
+        <is>
+          <t>Tennent</t>
+        </is>
+      </c>
+      <c r="E115" s="13" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="F115" s="13" t="n">
+        <v>221</v>
+      </c>
+      <c r="G115" s="13" t="inlineStr">
+        <is>
+          <t>$5,300</t>
+        </is>
+      </c>
+      <c r="H115" s="15" t="n">
+        <v>5300</v>
+      </c>
+      <c r="I115" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="J115" s="13" t="inlineStr"/>
+      <c r="K115" s="13" t="inlineStr">
+        <is>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L115" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M115" s="13" t="inlineStr"/>
+      <c r="N115" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O115" s="14" t="inlineStr">
+        <is>
+          <t>Condition: used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" outlineLevel="1">
+      <c r="A116" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B116" s="14" t="inlineStr">
+        <is>
+          <t>30” wolf duel fuel range</t>
+        </is>
+      </c>
+      <c r="C116" s="13" t="inlineStr">
+        <is>
+          <t>range/oven/rangetop</t>
+        </is>
+      </c>
+      <c r="D116" s="13" t="inlineStr">
+        <is>
+          <t>Tennent</t>
+        </is>
+      </c>
+      <c r="E116" s="13" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="F116" s="13" t="n">
+        <v>221</v>
+      </c>
+      <c r="G116" s="13" t="inlineStr">
+        <is>
+          <t>$4,500</t>
+        </is>
+      </c>
+      <c r="H116" s="15" t="n">
+        <v>4500</v>
+      </c>
+      <c r="I116" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="J116" s="13" t="inlineStr"/>
+      <c r="K116" s="13" t="inlineStr">
+        <is>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L116" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M116" s="13" t="inlineStr"/>
+      <c r="N116" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O116" s="14" t="inlineStr">
+        <is>
+          <t>Condition: used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="17" t="inlineStr">
         <is>
           <t>Subtotal — NYC / Long Island / NJ</t>
         </is>
       </c>
-      <c r="B115" s="17" t="inlineStr">
-        <is>
-          <t>64 item(s)</t>
-        </is>
-      </c>
-      <c r="C115" s="18" t="n"/>
-      <c r="D115" s="18" t="n"/>
-      <c r="E115" s="18" t="n"/>
-      <c r="F115" s="18" t="n"/>
-      <c r="G115" s="18" t="n"/>
-      <c r="H115" s="19" t="n">
-        <v>320000</v>
-      </c>
-      <c r="I115" s="18" t="n"/>
-      <c r="J115" s="18" t="n"/>
-      <c r="K115" s="18" t="n"/>
-      <c r="L115" s="18" t="n"/>
-      <c r="M115" s="18" t="n"/>
-      <c r="N115" s="18" t="n"/>
-      <c r="O115" s="18" t="n"/>
-    </row>
-    <row r="116">
-      <c r="A116" s="11" t="inlineStr">
+      <c r="B117" s="17" t="inlineStr">
+        <is>
+          <t>66 item(s)</t>
+        </is>
+      </c>
+      <c r="C117" s="18" t="n"/>
+      <c r="D117" s="18" t="n"/>
+      <c r="E117" s="18" t="n"/>
+      <c r="F117" s="18" t="n"/>
+      <c r="G117" s="18" t="n"/>
+      <c r="H117" s="19" t="n">
+        <v>338600</v>
+      </c>
+      <c r="I117" s="18" t="n"/>
+      <c r="J117" s="18" t="n"/>
+      <c r="K117" s="18" t="n"/>
+      <c r="L117" s="18" t="n"/>
+      <c r="M117" s="18" t="n"/>
+      <c r="N117" s="18" t="n"/>
+      <c r="O117" s="18" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="11" t="inlineStr">
         <is>
           <t>▸ Eastern PA / Mid-Atlantic  (2)</t>
         </is>
       </c>
-      <c r="B116" s="12" t="n"/>
-      <c r="C116" s="12" t="n"/>
-      <c r="D116" s="12" t="n"/>
-      <c r="E116" s="12" t="n"/>
-      <c r="F116" s="12" t="n"/>
-      <c r="G116" s="12" t="n"/>
-      <c r="H116" s="12" t="n"/>
-      <c r="I116" s="12" t="n"/>
-      <c r="J116" s="12" t="n"/>
-      <c r="K116" s="12" t="n"/>
-      <c r="L116" s="12" t="n"/>
-      <c r="M116" s="12" t="n"/>
-      <c r="N116" s="12" t="n"/>
-      <c r="O116" s="12" t="n"/>
-    </row>
-    <row r="117" outlineLevel="1">
-      <c r="A117" s="13" t="inlineStr">
+      <c r="B118" s="12" t="n"/>
+      <c r="C118" s="12" t="n"/>
+      <c r="D118" s="12" t="n"/>
+      <c r="E118" s="12" t="n"/>
+      <c r="F118" s="12" t="n"/>
+      <c r="G118" s="12" t="n"/>
+      <c r="H118" s="12" t="n"/>
+      <c r="I118" s="12" t="n"/>
+      <c r="J118" s="12" t="n"/>
+      <c r="K118" s="12" t="n"/>
+      <c r="L118" s="12" t="n"/>
+      <c r="M118" s="12" t="n"/>
+      <c r="N118" s="12" t="n"/>
+      <c r="O118" s="12" t="n"/>
+    </row>
+    <row r="119" outlineLevel="1">
+      <c r="A119" s="13" t="inlineStr">
         <is>
           <t>Eastern PA / Mid-Atlantic</t>
         </is>
       </c>
-      <c r="B117" s="14" t="inlineStr">
+      <c r="B119" s="14" t="inlineStr">
         <is>
           <t>Wolf Professional stainless gas range, 4 burners, red knobs (NBM Liquidation as-is appliance auction, lot 327587466)</t>
         </is>
       </c>
-      <c r="C117" s="13" t="inlineStr">
+      <c r="C119" s="13" t="inlineStr">
         <is>
           <t>range</t>
         </is>
       </c>
-      <c r="D117" s="13" t="inlineStr">
+      <c r="D119" s="13" t="inlineStr">
         <is>
           <t>Wilkes-Barre</t>
         </is>
       </c>
-      <c r="E117" s="13" t="inlineStr">
+      <c r="E119" s="13" t="inlineStr">
         <is>
           <t>PA</t>
         </is>
       </c>
-      <c r="F117" s="13" t="n">
+      <c r="F119" s="13" t="n">
         <v>268</v>
       </c>
-      <c r="G117" s="13" t="inlineStr">
+      <c r="G119" s="13" t="inlineStr">
         <is>
           <t>$0 bid (min $10) + BP</t>
         </is>
       </c>
-      <c r="H117" s="15" t="n">
+      <c r="H119" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="I117" s="13" t="inlineStr">
+      <c r="I119" s="13" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="J117" s="13" t="inlineStr">
+      <c r="J119" s="13" t="inlineStr">
         <is>
           <t>2026-10-27 07:11 PM ET</t>
         </is>
       </c>
-      <c r="K117" s="13" t="inlineStr">
+      <c r="K119" s="13" t="inlineStr">
         <is>
           <t>HiBid (NBM Liquidation, Moosic PA)</t>
         </is>
       </c>
-      <c r="L117" s="21" t="inlineStr">
+      <c r="L119" s="21" t="inlineStr">
         <is>
           <t>ENDING SOON</t>
         </is>
       </c>
-      <c r="M117" s="20" t="inlineStr">
+      <c r="M119" s="20" t="inlineStr">
         <is>
           <t>FLIP</t>
         </is>
       </c>
-      <c r="N117" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O117" s="14" t="inlineStr">
+      <c r="N119" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O119" s="14" t="inlineStr">
         <is>
           <t>As-is appliance liquidation auction; width/model not stated in listing, check photos. Closes Oct 27 6:11 PM EST. About 300 mi from 02339.</t>
         </is>
       </c>
     </row>
-    <row r="118" outlineLevel="1">
-      <c r="A118" s="13" t="inlineStr">
+    <row r="120" outlineLevel="1">
+      <c r="A120" s="13" t="inlineStr">
         <is>
           <t>Eastern PA / Mid-Atlantic</t>
         </is>
       </c>
-      <c r="B118" s="14" t="inlineStr">
+      <c r="B120" s="14" t="inlineStr">
         <is>
           <t>Wolf Professional stainless gas range (NBM Liquidation as-is appliance auction, lot 327710355, lot #102)</t>
         </is>
       </c>
-      <c r="C118" s="13" t="inlineStr">
+      <c r="C120" s="13" t="inlineStr">
         <is>
           <t>range</t>
         </is>
       </c>
-      <c r="D118" s="13" t="inlineStr">
+      <c r="D120" s="13" t="inlineStr">
         <is>
           <t>Wilkes-Barre</t>
         </is>
       </c>
-      <c r="E118" s="13" t="inlineStr">
+      <c r="E120" s="13" t="inlineStr">
         <is>
           <t>PA</t>
         </is>
       </c>
-      <c r="F118" s="13" t="n">
+      <c r="F120" s="13" t="n">
         <v>268</v>
       </c>
-      <c r="G118" s="13" t="inlineStr">
+      <c r="G120" s="13" t="inlineStr">
         <is>
           <t>$0 bid (min $1) + BP</t>
         </is>
       </c>
-      <c r="H118" s="15" t="n">
+      <c r="H120" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="I118" s="13" t="inlineStr">
+      <c r="I120" s="13" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="J118" s="13" t="inlineStr">
+      <c r="J120" s="13" t="inlineStr">
         <is>
           <t>2026-10-27 06:45 PM ET</t>
         </is>
       </c>
-      <c r="K118" s="13" t="inlineStr">
+      <c r="K120" s="13" t="inlineStr">
         <is>
           <t>HiBid (NBM Liquidation, Moosic PA)</t>
         </is>
       </c>
-      <c r="L118" s="21" t="inlineStr">
+      <c r="L120" s="21" t="inlineStr">
         <is>
           <t>ENDING SOON</t>
         </is>
       </c>
-      <c r="M118" s="20" t="inlineStr">
+      <c r="M120" s="20" t="inlineStr">
         <is>
           <t>FLIP</t>
         </is>
       </c>
-      <c r="N118" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O118" s="14" t="inlineStr">
+      <c r="N120" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O120" s="14" t="inlineStr">
         <is>
           <t>Second Wolf pro gas range in the same NBM as-is auction as wf-229 (lot 327587466); one pickup covers both. Width/model not stated, check photos. Closes about 6:45 PM ET Oct 27.</t>
         </is>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" s="17" t="inlineStr">
+    <row r="121">
+      <c r="A121" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Eastern PA / Mid-Atlantic</t>
         </is>
       </c>
-      <c r="B119" s="17" t="inlineStr">
+      <c r="B121" s="17" t="inlineStr">
         <is>
           <t>2 item(s)</t>
         </is>
       </c>
-      <c r="C119" s="18" t="n"/>
-      <c r="D119" s="18" t="n"/>
-      <c r="E119" s="18" t="n"/>
-      <c r="F119" s="18" t="n"/>
-      <c r="G119" s="18" t="n"/>
-      <c r="H119" s="19" t="n">
+      <c r="C121" s="18" t="n"/>
+      <c r="D121" s="18" t="n"/>
+      <c r="E121" s="18" t="n"/>
+      <c r="F121" s="18" t="n"/>
+      <c r="G121" s="18" t="n"/>
+      <c r="H121" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I119" s="18" t="n"/>
-      <c r="J119" s="18" t="n"/>
-      <c r="K119" s="18" t="n"/>
-      <c r="L119" s="18" t="n"/>
-      <c r="M119" s="18" t="n"/>
-      <c r="N119" s="18" t="n"/>
-      <c r="O119" s="18" t="n"/>
-    </row>
-    <row r="120">
-      <c r="A120" s="11" t="inlineStr">
+      <c r="I121" s="18" t="n"/>
+      <c r="J121" s="18" t="n"/>
+      <c r="K121" s="18" t="n"/>
+      <c r="L121" s="18" t="n"/>
+      <c r="M121" s="18" t="n"/>
+      <c r="N121" s="18" t="n"/>
+      <c r="O121" s="18" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="11" t="inlineStr">
         <is>
           <t>▸ Upstate / Western NY  (1)</t>
         </is>
       </c>
-      <c r="B120" s="12" t="n"/>
-      <c r="C120" s="12" t="n"/>
-      <c r="D120" s="12" t="n"/>
-      <c r="E120" s="12" t="n"/>
-      <c r="F120" s="12" t="n"/>
-      <c r="G120" s="12" t="n"/>
-      <c r="H120" s="12" t="n"/>
-      <c r="I120" s="12" t="n"/>
-      <c r="J120" s="12" t="n"/>
-      <c r="K120" s="12" t="n"/>
-      <c r="L120" s="12" t="n"/>
-      <c r="M120" s="12" t="n"/>
-      <c r="N120" s="12" t="n"/>
-      <c r="O120" s="12" t="n"/>
-    </row>
-    <row r="121" outlineLevel="1">
-      <c r="A121" s="13" t="inlineStr">
+      <c r="B122" s="12" t="n"/>
+      <c r="C122" s="12" t="n"/>
+      <c r="D122" s="12" t="n"/>
+      <c r="E122" s="12" t="n"/>
+      <c r="F122" s="12" t="n"/>
+      <c r="G122" s="12" t="n"/>
+      <c r="H122" s="12" t="n"/>
+      <c r="I122" s="12" t="n"/>
+      <c r="J122" s="12" t="n"/>
+      <c r="K122" s="12" t="n"/>
+      <c r="L122" s="12" t="n"/>
+      <c r="M122" s="12" t="n"/>
+      <c r="N122" s="12" t="n"/>
+      <c r="O122" s="12" t="n"/>
+    </row>
+    <row r="123" outlineLevel="1">
+      <c r="A123" s="13" t="inlineStr">
         <is>
           <t>Upstate / Western NY</t>
         </is>
       </c>
-      <c r="B121" s="14" t="inlineStr">
+      <c r="B123" s="14" t="inlineStr">
         <is>
           <t>WOLF GAS RANGE 30”</t>
         </is>
       </c>
-      <c r="C121" s="13" t="inlineStr">
+      <c r="C123" s="13" t="inlineStr">
         <is>
           <t>range/oven/rangetop</t>
         </is>
       </c>
-      <c r="D121" s="13" t="inlineStr">
+      <c r="D123" s="13" t="inlineStr">
         <is>
           <t>Binghamton</t>
         </is>
       </c>
-      <c r="E121" s="13" t="inlineStr">
+      <c r="E123" s="13" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
       </c>
-      <c r="F121" s="13" t="n">
+      <c r="F123" s="13" t="n">
         <v>262</v>
       </c>
-      <c r="G121" s="13" t="inlineStr">
+      <c r="G123" s="13" t="inlineStr">
         <is>
           <t>$1,200</t>
         </is>
       </c>
-      <c r="H121" s="15" t="n">
+      <c r="H123" s="15" t="n">
         <v>1200</v>
       </c>
-      <c r="I121" s="13" t="inlineStr">
+      <c r="I123" s="13" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="J121" s="13" t="inlineStr"/>
-      <c r="K121" s="13" t="inlineStr">
+      <c r="J123" s="13" t="inlineStr"/>
+      <c r="K123" s="13" t="inlineStr">
         <is>
           <t>Craigslist</t>
         </is>
       </c>
-      <c r="L121" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M121" s="20" t="inlineStr">
+      <c r="L123" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M123" s="20" t="inlineStr">
         <is>
           <t>FLIP</t>
         </is>
       </c>
-      <c r="N121" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O121" s="14" t="inlineStr">
+      <c r="N123" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O123" s="14" t="inlineStr">
         <is>
           <t>Condition: used. FLIP: 30" gas $1,200, needs ~$300 igniter; repaired 30" ask $1.9-3.5k</t>
         </is>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" s="17" t="inlineStr">
+    <row r="124">
+      <c r="A124" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Upstate / Western NY</t>
         </is>
       </c>
-      <c r="B122" s="17" t="inlineStr">
+      <c r="B124" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C122" s="18" t="n"/>
-      <c r="D122" s="18" t="n"/>
-      <c r="E122" s="18" t="n"/>
-      <c r="F122" s="18" t="n"/>
-      <c r="G122" s="18" t="n"/>
-      <c r="H122" s="19" t="n">
+      <c r="C124" s="18" t="n"/>
+      <c r="D124" s="18" t="n"/>
+      <c r="E124" s="18" t="n"/>
+      <c r="F124" s="18" t="n"/>
+      <c r="G124" s="18" t="n"/>
+      <c r="H124" s="19" t="n">
         <v>1200</v>
       </c>
-      <c r="I122" s="18" t="n"/>
-      <c r="J122" s="18" t="n"/>
-      <c r="K122" s="18" t="n"/>
-      <c r="L122" s="18" t="n"/>
-      <c r="M122" s="18" t="n"/>
-      <c r="N122" s="18" t="n"/>
-      <c r="O122" s="18" t="n"/>
-    </row>
-    <row r="123">
-      <c r="A123" s="11" t="inlineStr">
+      <c r="I124" s="18" t="n"/>
+      <c r="J124" s="18" t="n"/>
+      <c r="K124" s="18" t="n"/>
+      <c r="L124" s="18" t="n"/>
+      <c r="M124" s="18" t="n"/>
+      <c r="N124" s="18" t="n"/>
+      <c r="O124" s="18" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="11" t="inlineStr">
         <is>
           <t>▸ Unknown location  (60)</t>
         </is>
       </c>
-      <c r="B123" s="12" t="n"/>
-      <c r="C123" s="12" t="n"/>
-      <c r="D123" s="12" t="n"/>
-      <c r="E123" s="12" t="n"/>
-      <c r="F123" s="12" t="n"/>
-      <c r="G123" s="12" t="n"/>
-      <c r="H123" s="12" t="n"/>
-      <c r="I123" s="12" t="n"/>
-      <c r="J123" s="12" t="n"/>
-      <c r="K123" s="12" t="n"/>
-      <c r="L123" s="12" t="n"/>
-      <c r="M123" s="12" t="n"/>
-      <c r="N123" s="12" t="n"/>
-      <c r="O123" s="12" t="n"/>
-    </row>
-    <row r="124" outlineLevel="1">
-      <c r="A124" s="13" t="inlineStr">
-        <is>
-          <t>Unknown location</t>
-        </is>
-      </c>
-      <c r="B124" s="14" t="inlineStr">
-        <is>
-          <t>Wolf DF36450C/S/P Dual 36" Fuel Range - 4 Burners, Infrared Charb</t>
-        </is>
-      </c>
-      <c r="C124" s="13" t="inlineStr">
-        <is>
-          <t>range/oven/rangetop</t>
-        </is>
-      </c>
-      <c r="D124" s="13" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="E124" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F124" s="13" t="n"/>
-      <c r="G124" s="13" t="inlineStr">
-        <is>
-          <t>$2,000</t>
-        </is>
-      </c>
-      <c r="H124" s="15" t="n">
-        <v>2000</v>
-      </c>
-      <c r="I124" s="13" t="inlineStr"/>
-      <c r="J124" s="13" t="inlineStr"/>
-      <c r="K124" s="13" t="inlineStr">
-        <is>
-          <t>eBay (pickup only, over 60 mi)</t>
-        </is>
-      </c>
-      <c r="L124" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M124" s="20" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
-      <c r="N124" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O124" s="14" t="inlineStr">
-        <is>
-          <t>Condition: Pre-Owned. FLIP?: DF36450 36" dual fuel $2,000 OBO; rough resale $3-4k (eBay card shows no city; pickup distance in source.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="125" outlineLevel="1">
-      <c r="A125" s="13" t="inlineStr">
-        <is>
-          <t>Unknown location</t>
-        </is>
-      </c>
-      <c r="B125" s="14" t="inlineStr">
-        <is>
-          <t>Wolf 36" Contemporary Gas Cooktop (Model: CG365T/S) – Excellent C</t>
-        </is>
-      </c>
-      <c r="C125" s="13" t="inlineStr">
-        <is>
-          <t>range/oven/rangetop</t>
-        </is>
-      </c>
-      <c r="D125" s="13" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="E125" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F125" s="13" t="n"/>
-      <c r="G125" s="13" t="inlineStr">
-        <is>
-          <t>$500</t>
-        </is>
-      </c>
-      <c r="H125" s="15" t="n">
-        <v>500</v>
-      </c>
-      <c r="I125" s="13" t="inlineStr"/>
-      <c r="J125" s="13" t="inlineStr"/>
-      <c r="K125" s="13" t="inlineStr">
-        <is>
-          <t>eBay (pickup 190 mi)</t>
-        </is>
-      </c>
-      <c r="L125" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M125" s="20" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
-      <c r="N125" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O125" s="14" t="inlineStr">
-        <is>
-          <t>Condition: Pre-Owned. FLIP?: CG365T/S $500 OBO (190 mi); comp ask $950 (eBay card shows no city; pickup distance in source.)</t>
-        </is>
-      </c>
+      <c r="B125" s="12" t="n"/>
+      <c r="C125" s="12" t="n"/>
+      <c r="D125" s="12" t="n"/>
+      <c r="E125" s="12" t="n"/>
+      <c r="F125" s="12" t="n"/>
+      <c r="G125" s="12" t="n"/>
+      <c r="H125" s="12" t="n"/>
+      <c r="I125" s="12" t="n"/>
+      <c r="J125" s="12" t="n"/>
+      <c r="K125" s="12" t="n"/>
+      <c r="L125" s="12" t="n"/>
+      <c r="M125" s="12" t="n"/>
+      <c r="N125" s="12" t="n"/>
+      <c r="O125" s="12" t="n"/>
     </row>
     <row r="126" outlineLevel="1">
       <c r="A126" s="13" t="inlineStr">
@@ -12511,7 +12515,7 @@
       </c>
       <c r="B126" s="14" t="inlineStr">
         <is>
-          <t>Wolf CT36G/S 36” 5 Burner Natural Gas Cooktop Stainles</t>
+          <t>Wolf DF36450C/S/P Dual 36" Fuel Range - 4 Burners, Infrared Charb</t>
         </is>
       </c>
       <c r="C126" s="13" t="inlineStr">
@@ -12532,17 +12536,17 @@
       <c r="F126" s="13" t="n"/>
       <c r="G126" s="13" t="inlineStr">
         <is>
-          <t>$399.99</t>
+          <t>$2,000</t>
         </is>
       </c>
       <c r="H126" s="15" t="n">
-        <v>399.99</v>
+        <v>2000</v>
       </c>
       <c r="I126" s="13" t="inlineStr"/>
       <c r="J126" s="13" t="inlineStr"/>
       <c r="K126" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup 215 mi)</t>
+          <t>eBay (pickup only, over 60 mi)</t>
         </is>
       </c>
       <c r="L126" s="13" t="inlineStr">
@@ -12562,7 +12566,7 @@
       </c>
       <c r="O126" s="14" t="inlineStr">
         <is>
-          <t>Condition: Pre-Owned. FLIP?: CT36G/S 36" cooktop $399.99 (215 mi); rough resale $700-900 (eBay card shows no city; pickup distance in source.)</t>
+          <t>Condition: Pre-Owned. FLIP?: DF36450 36" dual fuel $2,000 OBO; rough resale $3-4k (eBay card shows no city; pickup distance in source.)</t>
         </is>
       </c>
     </row>
@@ -12574,12 +12578,12 @@
       </c>
       <c r="B127" s="14" t="inlineStr">
         <is>
-          <t>Wolf Gourmet Blender Shakes and Smoothies, Red Knob, Stainless (W</t>
+          <t>Wolf 36" Contemporary Gas Cooktop (Model: CG365T/S) – Excellent C</t>
         </is>
       </c>
       <c r="C127" s="13" t="inlineStr">
         <is>
-          <t>countertop</t>
+          <t>range/oven/rangetop</t>
         </is>
       </c>
       <c r="D127" s="13" t="inlineStr">
@@ -12595,11 +12599,11 @@
       <c r="F127" s="13" t="n"/>
       <c r="G127" s="13" t="inlineStr">
         <is>
-          <t>$399</t>
+          <t>$500</t>
         </is>
       </c>
       <c r="H127" s="15" t="n">
-        <v>399</v>
+        <v>500</v>
       </c>
       <c r="I127" s="13" t="inlineStr"/>
       <c r="J127" s="13" t="inlineStr"/>
@@ -12613,7 +12617,11 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M127" s="13" t="inlineStr"/>
+      <c r="M127" s="20" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
       <c r="N127" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -12621,7 +12629,7 @@
       </c>
       <c r="O127" s="14" t="inlineStr">
         <is>
-          <t>Condition: Pre-Owned.  (eBay card shows no city; pickup distance in source.)</t>
+          <t>Condition: Pre-Owned. FLIP?: CG365T/S $500 OBO (190 mi); comp ask $950 (eBay card shows no city; pickup distance in source.)</t>
         </is>
       </c>
     </row>
@@ -12633,12 +12641,12 @@
       </c>
       <c r="B128" s="14" t="inlineStr">
         <is>
-          <t>Wolf Gourmet Countertop Convection Red Knob Oven WGCO100S Tested</t>
+          <t>Wolf CT36G/S 36” 5 Burner Natural Gas Cooktop Stainles</t>
         </is>
       </c>
       <c r="C128" s="13" t="inlineStr">
         <is>
-          <t>countertop</t>
+          <t>range/oven/rangetop</t>
         </is>
       </c>
       <c r="D128" s="13" t="inlineStr">
@@ -12654,17 +12662,17 @@
       <c r="F128" s="13" t="n"/>
       <c r="G128" s="13" t="inlineStr">
         <is>
-          <t>$349.99</t>
+          <t>$399.99</t>
         </is>
       </c>
       <c r="H128" s="15" t="n">
-        <v>349.99</v>
+        <v>399.99</v>
       </c>
       <c r="I128" s="13" t="inlineStr"/>
       <c r="J128" s="13" t="inlineStr"/>
       <c r="K128" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup 210 mi)</t>
+          <t>eBay (pickup 215 mi)</t>
         </is>
       </c>
       <c r="L128" s="13" t="inlineStr">
@@ -12672,7 +12680,11 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M128" s="13" t="inlineStr"/>
+      <c r="M128" s="20" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
       <c r="N128" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -12680,7 +12692,7 @@
       </c>
       <c r="O128" s="14" t="inlineStr">
         <is>
-          <t>Condition: Pre-Owned.  (eBay card shows no city; pickup distance in source.)</t>
+          <t>Condition: Pre-Owned. FLIP?: CT36G/S 36" cooktop $399.99 (215 mi); rough resale $700-900 (eBay card shows no city; pickup distance in source.)</t>
         </is>
       </c>
     </row>
@@ -12692,7 +12704,7 @@
       </c>
       <c r="B129" s="14" t="inlineStr">
         <is>
-          <t>Wolf Gourmet PCSTD-1761 10-Cup Programmable Coffee Maker Red</t>
+          <t>Wolf Gourmet Blender Shakes and Smoothies, Red Knob, Stainless (W</t>
         </is>
       </c>
       <c r="C129" s="13" t="inlineStr">
@@ -12713,17 +12725,17 @@
       <c r="F129" s="13" t="n"/>
       <c r="G129" s="13" t="inlineStr">
         <is>
-          <t>$784.95</t>
+          <t>$399</t>
         </is>
       </c>
       <c r="H129" s="15" t="n">
-        <v>784.95</v>
+        <v>399</v>
       </c>
       <c r="I129" s="13" t="inlineStr"/>
       <c r="J129" s="13" t="inlineStr"/>
       <c r="K129" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup 225 mi)</t>
+          <t>eBay (pickup 190 mi)</t>
         </is>
       </c>
       <c r="L129" s="13" t="inlineStr">
@@ -12751,12 +12763,12 @@
       </c>
       <c r="B130" s="14" t="inlineStr">
         <is>
-          <t>Wolf 36" stainless steel gas rangetop - 4 burners and grill with</t>
+          <t>Wolf Gourmet Countertop Convection Red Knob Oven WGCO100S Tested</t>
         </is>
       </c>
       <c r="C130" s="13" t="inlineStr">
         <is>
-          <t>range/oven/rangetop</t>
+          <t>countertop</t>
         </is>
       </c>
       <c r="D130" s="13" t="inlineStr">
@@ -12772,17 +12784,17 @@
       <c r="F130" s="13" t="n"/>
       <c r="G130" s="13" t="inlineStr">
         <is>
-          <t>$1,500</t>
+          <t>$349.99</t>
         </is>
       </c>
       <c r="H130" s="15" t="n">
-        <v>1500</v>
+        <v>349.99</v>
       </c>
       <c r="I130" s="13" t="inlineStr"/>
       <c r="J130" s="13" t="inlineStr"/>
       <c r="K130" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup 45 mi)</t>
+          <t>eBay (pickup 210 mi)</t>
         </is>
       </c>
       <c r="L130" s="13" t="inlineStr">
@@ -12810,12 +12822,12 @@
       </c>
       <c r="B131" s="14" t="inlineStr">
         <is>
-          <t>60'' Wolf range All Gas (606CG) USED NATURAL GAS</t>
+          <t>Wolf Gourmet PCSTD-1761 10-Cup Programmable Coffee Maker Red</t>
         </is>
       </c>
       <c r="C131" s="13" t="inlineStr">
         <is>
-          <t>range/oven/rangetop</t>
+          <t>countertop</t>
         </is>
       </c>
       <c r="D131" s="13" t="inlineStr">
@@ -12831,17 +12843,17 @@
       <c r="F131" s="13" t="n"/>
       <c r="G131" s="13" t="inlineStr">
         <is>
-          <t>$9,500</t>
+          <t>$784.95</t>
         </is>
       </c>
       <c r="H131" s="15" t="n">
-        <v>9500</v>
+        <v>784.95</v>
       </c>
       <c r="I131" s="13" t="inlineStr"/>
       <c r="J131" s="13" t="inlineStr"/>
       <c r="K131" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup only, over 60 mi)</t>
+          <t>eBay (pickup 225 mi)</t>
         </is>
       </c>
       <c r="L131" s="13" t="inlineStr">
@@ -12869,7 +12881,7 @@
       </c>
       <c r="B132" s="14" t="inlineStr">
         <is>
-          <t>48” Wolf Gas Range R488 (Used &amp; Natural Gas)</t>
+          <t>Wolf 36" stainless steel gas rangetop - 4 burners and grill with</t>
         </is>
       </c>
       <c r="C132" s="13" t="inlineStr">
@@ -12890,17 +12902,17 @@
       <c r="F132" s="13" t="n"/>
       <c r="G132" s="13" t="inlineStr">
         <is>
-          <t>$8,500</t>
+          <t>$1,500</t>
         </is>
       </c>
       <c r="H132" s="15" t="n">
-        <v>8500</v>
+        <v>1500</v>
       </c>
       <c r="I132" s="13" t="inlineStr"/>
       <c r="J132" s="13" t="inlineStr"/>
       <c r="K132" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup 105 mi)</t>
+          <t>eBay (pickup 45 mi)</t>
         </is>
       </c>
       <c r="L132" s="13" t="inlineStr">
@@ -12928,7 +12940,7 @@
       </c>
       <c r="B133" s="14" t="inlineStr">
         <is>
-          <t>48” Wolf Gas Range GR486G (Used)</t>
+          <t>60'' Wolf range All Gas (606CG) USED NATURAL GAS</t>
         </is>
       </c>
       <c r="C133" s="13" t="inlineStr">
@@ -12949,17 +12961,17 @@
       <c r="F133" s="13" t="n"/>
       <c r="G133" s="13" t="inlineStr">
         <is>
-          <t>$11,500</t>
+          <t>$9,500</t>
         </is>
       </c>
       <c r="H133" s="15" t="n">
-        <v>11500</v>
+        <v>9500</v>
       </c>
       <c r="I133" s="13" t="inlineStr"/>
       <c r="J133" s="13" t="inlineStr"/>
       <c r="K133" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup 105 mi)</t>
+          <t>eBay (pickup only, over 60 mi)</t>
         </is>
       </c>
       <c r="L133" s="13" t="inlineStr">
@@ -12987,7 +12999,7 @@
       </c>
       <c r="B134" s="14" t="inlineStr">
         <is>
-          <t>48” Wolf Dual Fuel Range DF484DGLP (Used &amp; Natural Gas)</t>
+          <t>48” Wolf Gas Range R488 (Used &amp; Natural Gas)</t>
         </is>
       </c>
       <c r="C134" s="13" t="inlineStr">
@@ -13008,11 +13020,11 @@
       <c r="F134" s="13" t="n"/>
       <c r="G134" s="13" t="inlineStr">
         <is>
-          <t>$12,500</t>
+          <t>$8,500</t>
         </is>
       </c>
       <c r="H134" s="15" t="n">
-        <v>12500</v>
+        <v>8500</v>
       </c>
       <c r="I134" s="13" t="inlineStr"/>
       <c r="J134" s="13" t="inlineStr"/>
@@ -13046,7 +13058,7 @@
       </c>
       <c r="B135" s="14" t="inlineStr">
         <is>
-          <t>48” Wolf Natural Gas Range GR486G (Used)</t>
+          <t>48” Wolf Gas Range GR486G (Used)</t>
         </is>
       </c>
       <c r="C135" s="13" t="inlineStr">
@@ -13067,11 +13079,11 @@
       <c r="F135" s="13" t="n"/>
       <c r="G135" s="13" t="inlineStr">
         <is>
-          <t>$11,000</t>
+          <t>$11,500</t>
         </is>
       </c>
       <c r="H135" s="15" t="n">
-        <v>11000</v>
+        <v>11500</v>
       </c>
       <c r="I135" s="13" t="inlineStr"/>
       <c r="J135" s="13" t="inlineStr"/>
@@ -13105,7 +13117,7 @@
       </c>
       <c r="B136" s="14" t="inlineStr">
         <is>
-          <t>30” Wolf M Series Double Wall Oven DO30PMSPH (Used)</t>
+          <t>48” Wolf Dual Fuel Range DF484DGLP (Used &amp; Natural Gas)</t>
         </is>
       </c>
       <c r="C136" s="13" t="inlineStr">
@@ -13126,11 +13138,11 @@
       <c r="F136" s="13" t="n"/>
       <c r="G136" s="13" t="inlineStr">
         <is>
-          <t>$7,500</t>
+          <t>$12,500</t>
         </is>
       </c>
       <c r="H136" s="15" t="n">
-        <v>7500</v>
+        <v>12500</v>
       </c>
       <c r="I136" s="13" t="inlineStr"/>
       <c r="J136" s="13" t="inlineStr"/>
@@ -13164,7 +13176,7 @@
       </c>
       <c r="B137" s="14" t="inlineStr">
         <is>
-          <t>30” Wolf M Series Double Wall Oven DO30PMSPH (Used)</t>
+          <t>48” Wolf Natural Gas Range GR486G (Used)</t>
         </is>
       </c>
       <c r="C137" s="13" t="inlineStr">
@@ -13185,11 +13197,11 @@
       <c r="F137" s="13" t="n"/>
       <c r="G137" s="13" t="inlineStr">
         <is>
-          <t>$7,500</t>
+          <t>$11,000</t>
         </is>
       </c>
       <c r="H137" s="15" t="n">
-        <v>7500</v>
+        <v>11000</v>
       </c>
       <c r="I137" s="13" t="inlineStr"/>
       <c r="J137" s="13" t="inlineStr"/>
@@ -13223,7 +13235,7 @@
       </c>
       <c r="B138" s="14" t="inlineStr">
         <is>
-          <t>30” Wolf Double Wall Oven E Series DO30PESPH (Used)</t>
+          <t>30” Wolf M Series Double Wall Oven DO30PMSPH (Used)</t>
         </is>
       </c>
       <c r="C138" s="13" t="inlineStr">
@@ -13244,11 +13256,11 @@
       <c r="F138" s="13" t="n"/>
       <c r="G138" s="13" t="inlineStr">
         <is>
-          <t>$4,500</t>
+          <t>$7,500</t>
         </is>
       </c>
       <c r="H138" s="15" t="n">
-        <v>4500</v>
+        <v>7500</v>
       </c>
       <c r="I138" s="13" t="inlineStr"/>
       <c r="J138" s="13" t="inlineStr"/>
@@ -13282,7 +13294,7 @@
       </c>
       <c r="B139" s="14" t="inlineStr">
         <is>
-          <t>36” Wolf Induction Cooktop CI365TS (Used)</t>
+          <t>30” Wolf M Series Double Wall Oven DO30PMSPH (Used)</t>
         </is>
       </c>
       <c r="C139" s="13" t="inlineStr">
@@ -13303,11 +13315,11 @@
       <c r="F139" s="13" t="n"/>
       <c r="G139" s="13" t="inlineStr">
         <is>
-          <t>$2,700</t>
+          <t>$7,500</t>
         </is>
       </c>
       <c r="H139" s="15" t="n">
-        <v>2700</v>
+        <v>7500</v>
       </c>
       <c r="I139" s="13" t="inlineStr"/>
       <c r="J139" s="13" t="inlineStr"/>
@@ -13341,7 +13353,7 @@
       </c>
       <c r="B140" s="14" t="inlineStr">
         <is>
-          <t>36” Wolf Dual Fuel Range DF366 (Used &amp; Natural gas)</t>
+          <t>30” Wolf Double Wall Oven E Series DO30PESPH (Used)</t>
         </is>
       </c>
       <c r="C140" s="13" t="inlineStr">
@@ -13362,11 +13374,11 @@
       <c r="F140" s="13" t="n"/>
       <c r="G140" s="13" t="inlineStr">
         <is>
-          <t>$8,000</t>
+          <t>$4,500</t>
         </is>
       </c>
       <c r="H140" s="15" t="n">
-        <v>8000</v>
+        <v>4500</v>
       </c>
       <c r="I140" s="13" t="inlineStr"/>
       <c r="J140" s="13" t="inlineStr"/>
@@ -13400,7 +13412,7 @@
       </c>
       <c r="B141" s="14" t="inlineStr">
         <is>
-          <t>48” Wolf Dual Fuel Propane Range DF484CGLP (Used)</t>
+          <t>36” Wolf Induction Cooktop CI365TS (Used)</t>
         </is>
       </c>
       <c r="C141" s="13" t="inlineStr">
@@ -13421,11 +13433,11 @@
       <c r="F141" s="13" t="n"/>
       <c r="G141" s="13" t="inlineStr">
         <is>
-          <t>$10,500</t>
+          <t>$2,700</t>
         </is>
       </c>
       <c r="H141" s="15" t="n">
-        <v>10500</v>
+        <v>2700</v>
       </c>
       <c r="I141" s="13" t="inlineStr"/>
       <c r="J141" s="13" t="inlineStr"/>
@@ -13459,7 +13471,7 @@
       </c>
       <c r="B142" s="14" t="inlineStr">
         <is>
-          <t>48” Wolf LP Range GR486CLP (Used)</t>
+          <t>36” Wolf Dual Fuel Range DF366 (Used &amp; Natural gas)</t>
         </is>
       </c>
       <c r="C142" s="13" t="inlineStr">
@@ -13480,11 +13492,11 @@
       <c r="F142" s="13" t="n"/>
       <c r="G142" s="13" t="inlineStr">
         <is>
-          <t>$10,500</t>
+          <t>$8,000</t>
         </is>
       </c>
       <c r="H142" s="15" t="n">
-        <v>10500</v>
+        <v>8000</v>
       </c>
       <c r="I142" s="13" t="inlineStr"/>
       <c r="J142" s="13" t="inlineStr"/>
@@ -13518,7 +13530,7 @@
       </c>
       <c r="B143" s="14" t="inlineStr">
         <is>
-          <t>36” Wolf Gas Range G366 (Used)</t>
+          <t>48” Wolf Dual Fuel Propane Range DF484CGLP (Used)</t>
         </is>
       </c>
       <c r="C143" s="13" t="inlineStr">
@@ -13539,11 +13551,11 @@
       <c r="F143" s="13" t="n"/>
       <c r="G143" s="13" t="inlineStr">
         <is>
-          <t>$7,000</t>
+          <t>$10,500</t>
         </is>
       </c>
       <c r="H143" s="15" t="n">
-        <v>7000</v>
+        <v>10500</v>
       </c>
       <c r="I143" s="13" t="inlineStr"/>
       <c r="J143" s="13" t="inlineStr"/>
@@ -13577,7 +13589,7 @@
       </c>
       <c r="B144" s="14" t="inlineStr">
         <is>
-          <t>30” Wolf LP Range GR304LP (Used)</t>
+          <t>48” Wolf LP Range GR486CLP (Used)</t>
         </is>
       </c>
       <c r="C144" s="13" t="inlineStr">
@@ -13598,11 +13610,11 @@
       <c r="F144" s="13" t="n"/>
       <c r="G144" s="13" t="inlineStr">
         <is>
-          <t>$5,000</t>
+          <t>$10,500</t>
         </is>
       </c>
       <c r="H144" s="15" t="n">
-        <v>5000</v>
+        <v>10500</v>
       </c>
       <c r="I144" s="13" t="inlineStr"/>
       <c r="J144" s="13" t="inlineStr"/>
@@ -13636,7 +13648,7 @@
       </c>
       <c r="B145" s="14" t="inlineStr">
         <is>
-          <t>48” Wolf Natural Gas Range GR486C (Used)</t>
+          <t>36” Wolf Gas Range G366 (Used)</t>
         </is>
       </c>
       <c r="C145" s="13" t="inlineStr">
@@ -13657,11 +13669,11 @@
       <c r="F145" s="13" t="n"/>
       <c r="G145" s="13" t="inlineStr">
         <is>
-          <t>$9,500</t>
+          <t>$7,000</t>
         </is>
       </c>
       <c r="H145" s="15" t="n">
-        <v>9500</v>
+        <v>7000</v>
       </c>
       <c r="I145" s="13" t="inlineStr"/>
       <c r="J145" s="13" t="inlineStr"/>
@@ -13695,7 +13707,7 @@
       </c>
       <c r="B146" s="14" t="inlineStr">
         <is>
-          <t>30” Wolf M Series Double Wall Oven DO30PMSPH (Slightly Used)</t>
+          <t>30” Wolf LP Range GR304LP (Used)</t>
         </is>
       </c>
       <c r="C146" s="13" t="inlineStr">
@@ -13716,11 +13728,11 @@
       <c r="F146" s="13" t="n"/>
       <c r="G146" s="13" t="inlineStr">
         <is>
-          <t>$7,500</t>
+          <t>$5,000</t>
         </is>
       </c>
       <c r="H146" s="15" t="n">
-        <v>7500</v>
+        <v>5000</v>
       </c>
       <c r="I146" s="13" t="inlineStr"/>
       <c r="J146" s="13" t="inlineStr"/>
@@ -13754,7 +13766,7 @@
       </c>
       <c r="B147" s="14" t="inlineStr">
         <is>
-          <t>36” Wolf Professional Series Gas Cooktop CG365PS (Used)</t>
+          <t>48” Wolf Natural Gas Range GR486C (Used)</t>
         </is>
       </c>
       <c r="C147" s="13" t="inlineStr">
@@ -13775,11 +13787,11 @@
       <c r="F147" s="13" t="n"/>
       <c r="G147" s="13" t="inlineStr">
         <is>
-          <t>$2,000</t>
+          <t>$9,500</t>
         </is>
       </c>
       <c r="H147" s="15" t="n">
-        <v>2000</v>
+        <v>9500</v>
       </c>
       <c r="I147" s="13" t="inlineStr"/>
       <c r="J147" s="13" t="inlineStr"/>
@@ -13813,7 +13825,7 @@
       </c>
       <c r="B148" s="14" t="inlineStr">
         <is>
-          <t>36” Wolf Propane Range G366LP (Used)</t>
+          <t>30” Wolf M Series Double Wall Oven DO30PMSPH (Slightly Used)</t>
         </is>
       </c>
       <c r="C148" s="13" t="inlineStr">
@@ -13834,11 +13846,11 @@
       <c r="F148" s="13" t="n"/>
       <c r="G148" s="13" t="inlineStr">
         <is>
-          <t>$7,000</t>
+          <t>$7,500</t>
         </is>
       </c>
       <c r="H148" s="15" t="n">
-        <v>7000</v>
+        <v>7500</v>
       </c>
       <c r="I148" s="13" t="inlineStr"/>
       <c r="J148" s="13" t="inlineStr"/>
@@ -13872,7 +13884,7 @@
       </c>
       <c r="B149" s="14" t="inlineStr">
         <is>
-          <t>30” Wolf Propane Range GR304LP (Used)</t>
+          <t>36” Wolf Professional Series Gas Cooktop CG365PS (Used)</t>
         </is>
       </c>
       <c r="C149" s="13" t="inlineStr">
@@ -13893,11 +13905,11 @@
       <c r="F149" s="13" t="n"/>
       <c r="G149" s="13" t="inlineStr">
         <is>
-          <t>$5,000</t>
+          <t>$2,000</t>
         </is>
       </c>
       <c r="H149" s="15" t="n">
-        <v>5000</v>
+        <v>2000</v>
       </c>
       <c r="I149" s="13" t="inlineStr"/>
       <c r="J149" s="13" t="inlineStr"/>
@@ -13931,7 +13943,7 @@
       </c>
       <c r="B150" s="14" t="inlineStr">
         <is>
-          <t>Wolf SRT364g -NG 36” Pro Gas Rangetop Griddle Red Knobs w/Hood</t>
+          <t>36” Wolf Propane Range G366LP (Used)</t>
         </is>
       </c>
       <c r="C150" s="13" t="inlineStr">
@@ -13952,17 +13964,17 @@
       <c r="F150" s="13" t="n"/>
       <c r="G150" s="13" t="inlineStr">
         <is>
-          <t>$3,500</t>
+          <t>$7,000</t>
         </is>
       </c>
       <c r="H150" s="15" t="n">
-        <v>3500</v>
+        <v>7000</v>
       </c>
       <c r="I150" s="13" t="inlineStr"/>
       <c r="J150" s="13" t="inlineStr"/>
       <c r="K150" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup 120 mi)</t>
+          <t>eBay (pickup 105 mi)</t>
         </is>
       </c>
       <c r="L150" s="13" t="inlineStr">
@@ -13990,7 +14002,7 @@
       </c>
       <c r="B151" s="14" t="inlineStr">
         <is>
-          <t>Wolf 5 Burner 36" Professional Natural Gas Cooktop with 5 Burners</t>
+          <t>30” Wolf Propane Range GR304LP (Used)</t>
         </is>
       </c>
       <c r="C151" s="13" t="inlineStr">
@@ -14011,17 +14023,17 @@
       <c r="F151" s="13" t="n"/>
       <c r="G151" s="13" t="inlineStr">
         <is>
-          <t>$1,399</t>
+          <t>$5,000</t>
         </is>
       </c>
       <c r="H151" s="15" t="n">
-        <v>1399</v>
+        <v>5000</v>
       </c>
       <c r="I151" s="13" t="inlineStr"/>
       <c r="J151" s="13" t="inlineStr"/>
       <c r="K151" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup 120 mi)</t>
+          <t>eBay (pickup 105 mi)</t>
         </is>
       </c>
       <c r="L151" s="13" t="inlineStr">
@@ -14049,7 +14061,7 @@
       </c>
       <c r="B152" s="14" t="inlineStr">
         <is>
-          <t>Wolf 48” 8-Burner Freestanding Double Oven Range with Griddle- GA</t>
+          <t>Wolf SRT364g -NG 36” Pro Gas Rangetop Griddle Red Knobs w/Hood</t>
         </is>
       </c>
       <c r="C152" s="13" t="inlineStr">
@@ -14070,17 +14082,17 @@
       <c r="F152" s="13" t="n"/>
       <c r="G152" s="13" t="inlineStr">
         <is>
-          <t>$6,500</t>
+          <t>$3,500</t>
         </is>
       </c>
       <c r="H152" s="15" t="n">
-        <v>6500</v>
+        <v>3500</v>
       </c>
       <c r="I152" s="13" t="inlineStr"/>
       <c r="J152" s="13" t="inlineStr"/>
       <c r="K152" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup only, over 60 mi)</t>
+          <t>eBay (pickup 120 mi)</t>
         </is>
       </c>
       <c r="L152" s="13" t="inlineStr">
@@ -14108,7 +14120,7 @@
       </c>
       <c r="B153" s="14" t="inlineStr">
         <is>
-          <t>Wolf 36" Gas Range Top - SRT364C - 4 Burners + Charbroiler (Grill</t>
+          <t>Wolf 5 Burner 36" Professional Natural Gas Cooktop with 5 Burners</t>
         </is>
       </c>
       <c r="C153" s="13" t="inlineStr">
@@ -14129,17 +14141,17 @@
       <c r="F153" s="13" t="n"/>
       <c r="G153" s="13" t="inlineStr">
         <is>
-          <t>$2,899</t>
+          <t>$1,399</t>
         </is>
       </c>
       <c r="H153" s="15" t="n">
-        <v>2899</v>
+        <v>1399</v>
       </c>
       <c r="I153" s="13" t="inlineStr"/>
       <c r="J153" s="13" t="inlineStr"/>
       <c r="K153" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup 150 mi)</t>
+          <t>eBay (pickup 120 mi)</t>
         </is>
       </c>
       <c r="L153" s="13" t="inlineStr">
@@ -14167,7 +14179,7 @@
       </c>
       <c r="B154" s="14" t="inlineStr">
         <is>
-          <t>WOLF range top - model 36 - 6 gas</t>
+          <t>Wolf 48” 8-Burner Freestanding Double Oven Range with Griddle- GA</t>
         </is>
       </c>
       <c r="C154" s="13" t="inlineStr">
@@ -14188,11 +14200,11 @@
       <c r="F154" s="13" t="n"/>
       <c r="G154" s="13" t="inlineStr">
         <is>
-          <t>$1,400</t>
+          <t>$6,500</t>
         </is>
       </c>
       <c r="H154" s="15" t="n">
-        <v>1400</v>
+        <v>6500</v>
       </c>
       <c r="I154" s="13" t="inlineStr"/>
       <c r="J154" s="13" t="inlineStr"/>
@@ -14226,7 +14238,7 @@
       </c>
       <c r="B155" s="14" t="inlineStr">
         <is>
-          <t>Wolf 30in Rangetop Natural Gas</t>
+          <t>Wolf 36" Gas Range Top - SRT364C - 4 Burners + Charbroiler (Grill</t>
         </is>
       </c>
       <c r="C155" s="13" t="inlineStr">
@@ -14247,17 +14259,17 @@
       <c r="F155" s="13" t="n"/>
       <c r="G155" s="13" t="inlineStr">
         <is>
-          <t>$3,200</t>
+          <t>$2,899</t>
         </is>
       </c>
       <c r="H155" s="15" t="n">
-        <v>3200</v>
+        <v>2899</v>
       </c>
       <c r="I155" s="13" t="inlineStr"/>
       <c r="J155" s="13" t="inlineStr"/>
       <c r="K155" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup only, over 60 mi)</t>
+          <t>eBay (pickup 150 mi)</t>
         </is>
       </c>
       <c r="L155" s="13" t="inlineStr">
@@ -14285,7 +14297,7 @@
       </c>
       <c r="B156" s="14" t="inlineStr">
         <is>
-          <t>30in Wolf Rangetop SRT304</t>
+          <t>WOLF range top - model 36 - 6 gas</t>
         </is>
       </c>
       <c r="C156" s="13" t="inlineStr">
@@ -14306,11 +14318,11 @@
       <c r="F156" s="13" t="n"/>
       <c r="G156" s="13" t="inlineStr">
         <is>
-          <t>$3,200</t>
+          <t>$1,400</t>
         </is>
       </c>
       <c r="H156" s="15" t="n">
-        <v>3200</v>
+        <v>1400</v>
       </c>
       <c r="I156" s="13" t="inlineStr"/>
       <c r="J156" s="13" t="inlineStr"/>
@@ -14344,7 +14356,7 @@
       </c>
       <c r="B157" s="14" t="inlineStr">
         <is>
-          <t>oven wolf steam oven oven oven steam oven</t>
+          <t>Wolf 30in Rangetop Natural Gas</t>
         </is>
       </c>
       <c r="C157" s="13" t="inlineStr">
@@ -14365,11 +14377,11 @@
       <c r="F157" s="13" t="n"/>
       <c r="G157" s="13" t="inlineStr">
         <is>
-          <t>$899</t>
+          <t>$3,200</t>
         </is>
       </c>
       <c r="H157" s="15" t="n">
-        <v>899</v>
+        <v>3200</v>
       </c>
       <c r="I157" s="13" t="inlineStr"/>
       <c r="J157" s="13" t="inlineStr"/>
@@ -14403,7 +14415,7 @@
       </c>
       <c r="B158" s="14" t="inlineStr">
         <is>
-          <t>Wolf 6 Burner Commercial Range - Challenger XL36 - Good Condition</t>
+          <t>30in Wolf Rangetop SRT304</t>
         </is>
       </c>
       <c r="C158" s="13" t="inlineStr">
@@ -14424,11 +14436,11 @@
       <c r="F158" s="13" t="n"/>
       <c r="G158" s="13" t="inlineStr">
         <is>
-          <t>$800</t>
+          <t>$3,200</t>
         </is>
       </c>
       <c r="H158" s="15" t="n">
-        <v>800</v>
+        <v>3200</v>
       </c>
       <c r="I158" s="13" t="inlineStr"/>
       <c r="J158" s="13" t="inlineStr"/>
@@ -14450,7 +14462,7 @@
       </c>
       <c r="O158" s="14" t="inlineStr">
         <is>
-          <t>Condition: Pre-Owned. commercial Wolf (not Sub-Zero Wolf) (eBay card shows no city; pickup distance in source.)</t>
+          <t>Condition: Pre-Owned.  (eBay card shows no city; pickup distance in source.)</t>
         </is>
       </c>
     </row>
@@ -14462,7 +14474,7 @@
       </c>
       <c r="B159" s="14" t="inlineStr">
         <is>
-          <t>60in Wolf Range Dual Fuel 6 Burners Grill and Griddle PROPANE</t>
+          <t>oven wolf steam oven oven oven steam oven</t>
         </is>
       </c>
       <c r="C159" s="13" t="inlineStr">
@@ -14483,11 +14495,11 @@
       <c r="F159" s="13" t="n"/>
       <c r="G159" s="13" t="inlineStr">
         <is>
-          <t>$8,900</t>
+          <t>$899</t>
         </is>
       </c>
       <c r="H159" s="15" t="n">
-        <v>8900</v>
+        <v>899</v>
       </c>
       <c r="I159" s="13" t="inlineStr"/>
       <c r="J159" s="13" t="inlineStr"/>
@@ -14521,7 +14533,7 @@
       </c>
       <c r="B160" s="14" t="inlineStr">
         <is>
-          <t>Wolf RT486C 48-inch Gas Rangetop Propane Set Up w/ Cha</t>
+          <t>Wolf 6 Burner Commercial Range - Challenger XL36 - Good Condition</t>
         </is>
       </c>
       <c r="C160" s="13" t="inlineStr">
@@ -14542,11 +14554,11 @@
       <c r="F160" s="13" t="n"/>
       <c r="G160" s="13" t="inlineStr">
         <is>
-          <t>$2,650</t>
+          <t>$800</t>
         </is>
       </c>
       <c r="H160" s="15" t="n">
-        <v>2650</v>
+        <v>800</v>
       </c>
       <c r="I160" s="13" t="inlineStr"/>
       <c r="J160" s="13" t="inlineStr"/>
@@ -14568,7 +14580,7 @@
       </c>
       <c r="O160" s="14" t="inlineStr">
         <is>
-          <t>Condition: Pre-Owned.  (eBay card shows no city; pickup distance in source.)</t>
+          <t>Condition: Pre-Owned. commercial Wolf (not Sub-Zero Wolf) (eBay card shows no city; pickup distance in source.)</t>
         </is>
       </c>
     </row>
@@ -14580,7 +14592,7 @@
       </c>
       <c r="B161" s="14" t="inlineStr">
         <is>
-          <t>wolf 36 gas rangetop</t>
+          <t>60in Wolf Range Dual Fuel 6 Burners Grill and Griddle PROPANE</t>
         </is>
       </c>
       <c r="C161" s="13" t="inlineStr">
@@ -14601,11 +14613,11 @@
       <c r="F161" s="13" t="n"/>
       <c r="G161" s="13" t="inlineStr">
         <is>
-          <t>$2,500</t>
+          <t>$8,900</t>
         </is>
       </c>
       <c r="H161" s="15" t="n">
-        <v>2500</v>
+        <v>8900</v>
       </c>
       <c r="I161" s="13" t="inlineStr"/>
       <c r="J161" s="13" t="inlineStr"/>
@@ -14639,7 +14651,7 @@
       </c>
       <c r="B162" s="14" t="inlineStr">
         <is>
-          <t>Wolf 36" 5 Burner Gas Cooktop Stainless Steel model CT36G/S</t>
+          <t>Wolf RT486C 48-inch Gas Rangetop Propane Set Up w/ Cha</t>
         </is>
       </c>
       <c r="C162" s="13" t="inlineStr">
@@ -14660,17 +14672,17 @@
       <c r="F162" s="13" t="n"/>
       <c r="G162" s="13" t="inlineStr">
         <is>
-          <t>$999.99</t>
+          <t>$2,650</t>
         </is>
       </c>
       <c r="H162" s="15" t="n">
-        <v>999.99</v>
+        <v>2650</v>
       </c>
       <c r="I162" s="13" t="inlineStr"/>
       <c r="J162" s="13" t="inlineStr"/>
       <c r="K162" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup 175 mi)</t>
+          <t>eBay (pickup only, over 60 mi)</t>
         </is>
       </c>
       <c r="L162" s="13" t="inlineStr">
@@ -14698,7 +14710,7 @@
       </c>
       <c r="B163" s="14" t="inlineStr">
         <is>
-          <t>Wolf Gas Cooktop CG304P/S 30"W Professional 4-Burner Stainless St</t>
+          <t>wolf 36 gas rangetop</t>
         </is>
       </c>
       <c r="C163" s="13" t="inlineStr">
@@ -14719,11 +14731,11 @@
       <c r="F163" s="13" t="n"/>
       <c r="G163" s="13" t="inlineStr">
         <is>
-          <t>$655</t>
+          <t>$2,500</t>
         </is>
       </c>
       <c r="H163" s="15" t="n">
-        <v>655</v>
+        <v>2500</v>
       </c>
       <c r="I163" s="13" t="inlineStr"/>
       <c r="J163" s="13" t="inlineStr"/>
@@ -14757,7 +14769,7 @@
       </c>
       <c r="B164" s="14" t="inlineStr">
         <is>
-          <t>Wolf DF486C 48" Professional Dual Fuel Range 6-Burners + Charbrio</t>
+          <t>Wolf 36" 5 Burner Gas Cooktop Stainless Steel model CT36G/S</t>
         </is>
       </c>
       <c r="C164" s="13" t="inlineStr">
@@ -14778,17 +14790,17 @@
       <c r="F164" s="13" t="n"/>
       <c r="G164" s="13" t="inlineStr">
         <is>
-          <t>$9,425</t>
+          <t>$999.99</t>
         </is>
       </c>
       <c r="H164" s="15" t="n">
-        <v>9425</v>
+        <v>999.99</v>
       </c>
       <c r="I164" s="13" t="inlineStr"/>
       <c r="J164" s="13" t="inlineStr"/>
       <c r="K164" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup only, over 60 mi)</t>
+          <t>eBay (pickup 175 mi)</t>
         </is>
       </c>
       <c r="L164" s="13" t="inlineStr">
@@ -14816,7 +14828,7 @@
       </c>
       <c r="B165" s="14" t="inlineStr">
         <is>
-          <t>Wolf L Series 30" Double Electric Wall Oven</t>
+          <t>Wolf Gas Cooktop CG304P/S 30"W Professional 4-Burner Stainless St</t>
         </is>
       </c>
       <c r="C165" s="13" t="inlineStr">
@@ -14837,11 +14849,11 @@
       <c r="F165" s="13" t="n"/>
       <c r="G165" s="13" t="inlineStr">
         <is>
-          <t>$4,750</t>
+          <t>$655</t>
         </is>
       </c>
       <c r="H165" s="15" t="n">
-        <v>4750</v>
+        <v>655</v>
       </c>
       <c r="I165" s="13" t="inlineStr"/>
       <c r="J165" s="13" t="inlineStr"/>
@@ -14875,7 +14887,7 @@
       </c>
       <c r="B166" s="14" t="inlineStr">
         <is>
-          <t>Wolf SO30FS 30 inch Single Electric Wall Oven</t>
+          <t>Wolf DF486C 48" Professional Dual Fuel Range 6-Burners + Charbrio</t>
         </is>
       </c>
       <c r="C166" s="13" t="inlineStr">
@@ -14896,11 +14908,11 @@
       <c r="F166" s="13" t="n"/>
       <c r="G166" s="13" t="inlineStr">
         <is>
-          <t>$1,600</t>
+          <t>$9,425</t>
         </is>
       </c>
       <c r="H166" s="15" t="n">
-        <v>1600</v>
+        <v>9425</v>
       </c>
       <c r="I166" s="13" t="inlineStr"/>
       <c r="J166" s="13" t="inlineStr"/>
@@ -14934,7 +14946,7 @@
       </c>
       <c r="B167" s="14" t="inlineStr">
         <is>
-          <t>30” Wolf Double Wall Oven E Series DO30PESPH (Used)</t>
+          <t>Wolf L Series 30" Double Electric Wall Oven</t>
         </is>
       </c>
       <c r="C167" s="13" t="inlineStr">
@@ -14955,11 +14967,11 @@
       <c r="F167" s="13" t="n"/>
       <c r="G167" s="13" t="inlineStr">
         <is>
-          <t>$2,500</t>
+          <t>$4,750</t>
         </is>
       </c>
       <c r="H167" s="15" t="n">
-        <v>2500</v>
+        <v>4750</v>
       </c>
       <c r="I167" s="13" t="inlineStr"/>
       <c r="J167" s="13" t="inlineStr"/>
@@ -14993,7 +15005,7 @@
       </c>
       <c r="B168" s="14" t="inlineStr">
         <is>
-          <t>wolf oven 030U/S</t>
+          <t>Wolf SO30FS 30 inch Single Electric Wall Oven</t>
         </is>
       </c>
       <c r="C168" s="13" t="inlineStr">
@@ -15014,17 +15026,17 @@
       <c r="F168" s="13" t="n"/>
       <c r="G168" s="13" t="inlineStr">
         <is>
-          <t>$1,200</t>
+          <t>$1,600</t>
         </is>
       </c>
       <c r="H168" s="15" t="n">
-        <v>1200</v>
+        <v>1600</v>
       </c>
       <c r="I168" s="13" t="inlineStr"/>
       <c r="J168" s="13" t="inlineStr"/>
       <c r="K168" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup 185 mi)</t>
+          <t>eBay (pickup only, over 60 mi)</t>
         </is>
       </c>
       <c r="L168" s="13" t="inlineStr">
@@ -15052,7 +15064,7 @@
       </c>
       <c r="B169" s="14" t="inlineStr">
         <is>
-          <t>Wolf Wall Oven &amp; Warming Drawer-Series E-Offers Accepted-Excellen</t>
+          <t>30” Wolf Double Wall Oven E Series DO30PESPH (Used)</t>
         </is>
       </c>
       <c r="C169" s="13" t="inlineStr">
@@ -15073,11 +15085,11 @@
       <c r="F169" s="13" t="n"/>
       <c r="G169" s="13" t="inlineStr">
         <is>
-          <t>$1,100</t>
+          <t>$2,500</t>
         </is>
       </c>
       <c r="H169" s="15" t="n">
-        <v>1100</v>
+        <v>2500</v>
       </c>
       <c r="I169" s="13" t="inlineStr"/>
       <c r="J169" s="13" t="inlineStr"/>
@@ -15111,7 +15123,7 @@
       </c>
       <c r="B170" s="14" t="inlineStr">
         <is>
-          <t>wolf 36 inch gas cooktop</t>
+          <t>wolf oven 030U/S</t>
         </is>
       </c>
       <c r="C170" s="13" t="inlineStr">
@@ -15132,17 +15144,17 @@
       <c r="F170" s="13" t="n"/>
       <c r="G170" s="13" t="inlineStr">
         <is>
-          <t>$650</t>
+          <t>$1,200</t>
         </is>
       </c>
       <c r="H170" s="15" t="n">
-        <v>650</v>
+        <v>1200</v>
       </c>
       <c r="I170" s="13" t="inlineStr"/>
       <c r="J170" s="13" t="inlineStr"/>
       <c r="K170" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup 190 mi)</t>
+          <t>eBay (pickup 185 mi)</t>
         </is>
       </c>
       <c r="L170" s="13" t="inlineStr">
@@ -15170,7 +15182,7 @@
       </c>
       <c r="B171" s="14" t="inlineStr">
         <is>
-          <t>Wolf 36” Natural Gas Rangetop Cooktop RT366 , 6 Burner 💎💎💎 Red Kn</t>
+          <t>Wolf Wall Oven &amp; Warming Drawer-Series E-Offers Accepted-Excellen</t>
         </is>
       </c>
       <c r="C171" s="13" t="inlineStr">
@@ -15191,17 +15203,17 @@
       <c r="F171" s="13" t="n"/>
       <c r="G171" s="13" t="inlineStr">
         <is>
-          <t>$2,700</t>
+          <t>$1,100</t>
         </is>
       </c>
       <c r="H171" s="15" t="n">
-        <v>2700</v>
+        <v>1100</v>
       </c>
       <c r="I171" s="13" t="inlineStr"/>
       <c r="J171" s="13" t="inlineStr"/>
       <c r="K171" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup 190 mi)</t>
+          <t>eBay (pickup only, over 60 mi)</t>
         </is>
       </c>
       <c r="L171" s="13" t="inlineStr">
@@ -15229,7 +15241,7 @@
       </c>
       <c r="B172" s="14" t="inlineStr">
         <is>
-          <t>Wolf SO24TESTH Electric Convection Oven</t>
+          <t>wolf 36 inch gas cooktop</t>
         </is>
       </c>
       <c r="C172" s="13" t="inlineStr">
@@ -15250,17 +15262,17 @@
       <c r="F172" s="13" t="n"/>
       <c r="G172" s="13" t="inlineStr">
         <is>
-          <t>$1,020</t>
+          <t>$650</t>
         </is>
       </c>
       <c r="H172" s="15" t="n">
-        <v>1020</v>
+        <v>650</v>
       </c>
       <c r="I172" s="13" t="inlineStr"/>
       <c r="J172" s="13" t="inlineStr"/>
       <c r="K172" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup only, over 60 mi)</t>
+          <t>eBay (pickup 190 mi)</t>
         </is>
       </c>
       <c r="L172" s="13" t="inlineStr">
@@ -15288,7 +15300,7 @@
       </c>
       <c r="B173" s="14" t="inlineStr">
         <is>
-          <t>Wolf Electric Cooktop CT30E/B 30" Radiant 4 Burner Black Glass To</t>
+          <t>Wolf 36” Natural Gas Rangetop Cooktop RT366 , 6 Burner 💎💎💎 Red Kn</t>
         </is>
       </c>
       <c r="C173" s="13" t="inlineStr">
@@ -15309,17 +15321,17 @@
       <c r="F173" s="13" t="n"/>
       <c r="G173" s="13" t="inlineStr">
         <is>
-          <t>$684.99</t>
+          <t>$2,700</t>
         </is>
       </c>
       <c r="H173" s="15" t="n">
-        <v>684.99</v>
+        <v>2700</v>
       </c>
       <c r="I173" s="13" t="inlineStr"/>
       <c r="J173" s="13" t="inlineStr"/>
       <c r="K173" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup 210 mi)</t>
+          <t>eBay (pickup 190 mi)</t>
         </is>
       </c>
       <c r="L173" s="13" t="inlineStr">
@@ -15347,7 +15359,7 @@
       </c>
       <c r="B174" s="14" t="inlineStr">
         <is>
-          <t>Wolf IM15/S 15" Stainless Steel Multi-Function Gas Cooktop</t>
+          <t>Wolf SO24TESTH Electric Convection Oven</t>
         </is>
       </c>
       <c r="C174" s="13" t="inlineStr">
@@ -15368,17 +15380,17 @@
       <c r="F174" s="13" t="n"/>
       <c r="G174" s="13" t="inlineStr">
         <is>
-          <t>$779</t>
+          <t>$1,020</t>
         </is>
       </c>
       <c r="H174" s="15" t="n">
-        <v>779</v>
+        <v>1020</v>
       </c>
       <c r="I174" s="13" t="inlineStr"/>
       <c r="J174" s="13" t="inlineStr"/>
       <c r="K174" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup 210 mi)</t>
+          <t>eBay (pickup only, over 60 mi)</t>
         </is>
       </c>
       <c r="L174" s="13" t="inlineStr">
@@ -15406,7 +15418,7 @@
       </c>
       <c r="B175" s="14" t="inlineStr">
         <is>
-          <t>Wolf RT488 48" Stainless Steel Pro-Style Gas Rangetop</t>
+          <t>Wolf Electric Cooktop CT30E/B 30" Radiant 4 Burner Black Glass To</t>
         </is>
       </c>
       <c r="C175" s="13" t="inlineStr">
@@ -15427,11 +15439,11 @@
       <c r="F175" s="13" t="n"/>
       <c r="G175" s="13" t="inlineStr">
         <is>
-          <t>$2,999</t>
+          <t>$684.99</t>
         </is>
       </c>
       <c r="H175" s="15" t="n">
-        <v>2999</v>
+        <v>684.99</v>
       </c>
       <c r="I175" s="13" t="inlineStr"/>
       <c r="J175" s="13" t="inlineStr"/>
@@ -15465,7 +15477,7 @@
       </c>
       <c r="B176" s="14" t="inlineStr">
         <is>
-          <t>Wolf DO30U/S 30" Stainless Steel Electric Double Wall Oven</t>
+          <t>Wolf IM15/S 15" Stainless Steel Multi-Function Gas Cooktop</t>
         </is>
       </c>
       <c r="C176" s="13" t="inlineStr">
@@ -15486,11 +15498,11 @@
       <c r="F176" s="13" t="n"/>
       <c r="G176" s="13" t="inlineStr">
         <is>
-          <t>$3,469</t>
+          <t>$779</t>
         </is>
       </c>
       <c r="H176" s="15" t="n">
-        <v>3469</v>
+        <v>779</v>
       </c>
       <c r="I176" s="13" t="inlineStr"/>
       <c r="J176" s="13" t="inlineStr"/>
@@ -15524,7 +15536,7 @@
       </c>
       <c r="B177" s="14" t="inlineStr">
         <is>
-          <t>Wolf 48" Range Top - SRT486C 6 Burners Infrared Charbroiler</t>
+          <t>Wolf RT488 48" Stainless Steel Pro-Style Gas Rangetop</t>
         </is>
       </c>
       <c r="C177" s="13" t="inlineStr">
@@ -15545,17 +15557,17 @@
       <c r="F177" s="13" t="n"/>
       <c r="G177" s="13" t="inlineStr">
         <is>
-          <t>$2,700</t>
+          <t>$2,999</t>
         </is>
       </c>
       <c r="H177" s="15" t="n">
-        <v>2700</v>
+        <v>2999</v>
       </c>
       <c r="I177" s="13" t="inlineStr"/>
       <c r="J177" s="13" t="inlineStr"/>
       <c r="K177" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup only, over 60 mi)</t>
+          <t>eBay (pickup 210 mi)</t>
         </is>
       </c>
       <c r="L177" s="13" t="inlineStr">
@@ -15583,7 +15595,7 @@
       </c>
       <c r="B178" s="14" t="inlineStr">
         <is>
-          <t>36" Wolf Natural Gas Range 4 Burner with Griddle have vent sold s</t>
+          <t>Wolf DO30U/S 30" Stainless Steel Electric Double Wall Oven</t>
         </is>
       </c>
       <c r="C178" s="13" t="inlineStr">
@@ -15604,17 +15616,17 @@
       <c r="F178" s="13" t="n"/>
       <c r="G178" s="13" t="inlineStr">
         <is>
-          <t>$3,899</t>
+          <t>$3,469</t>
         </is>
       </c>
       <c r="H178" s="15" t="n">
-        <v>3899</v>
+        <v>3469</v>
       </c>
       <c r="I178" s="13" t="inlineStr"/>
       <c r="J178" s="13" t="inlineStr"/>
       <c r="K178" s="13" t="inlineStr">
         <is>
-          <t>eBay (pickup only, over 60 mi)</t>
+          <t>eBay (pickup 210 mi)</t>
         </is>
       </c>
       <c r="L178" s="13" t="inlineStr">
@@ -15642,7 +15654,7 @@
       </c>
       <c r="B179" s="14" t="inlineStr">
         <is>
-          <t>Used Wolf SO30F/S 30" 30" Built-In L Series Electric Oven - Frame</t>
+          <t>Wolf 48" Range Top - SRT486C 6 Burners Infrared Charbroiler</t>
         </is>
       </c>
       <c r="C179" s="13" t="inlineStr">
@@ -15663,11 +15675,11 @@
       <c r="F179" s="13" t="n"/>
       <c r="G179" s="13" t="inlineStr">
         <is>
-          <t>$1,200</t>
+          <t>$2,700</t>
         </is>
       </c>
       <c r="H179" s="15" t="n">
-        <v>1200</v>
+        <v>2700</v>
       </c>
       <c r="I179" s="13" t="inlineStr"/>
       <c r="J179" s="13" t="inlineStr"/>
@@ -15701,12 +15713,12 @@
       </c>
       <c r="B180" s="14" t="inlineStr">
         <is>
-          <t>Wolf Gourmet 10" skillet</t>
+          <t>36" Wolf Natural Gas Range 4 Burner with Griddle have vent sold s</t>
         </is>
       </c>
       <c r="C180" s="13" t="inlineStr">
         <is>
-          <t>countertop</t>
+          <t>range/oven/rangetop</t>
         </is>
       </c>
       <c r="D180" s="13" t="inlineStr">
@@ -15716,27 +15728,23 @@
       </c>
       <c r="E180" s="13" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F180" s="13" t="n"/>
       <c r="G180" s="13" t="inlineStr">
         <is>
-          <t>$300</t>
+          <t>$3,899</t>
         </is>
       </c>
       <c r="H180" s="15" t="n">
-        <v>300</v>
-      </c>
-      <c r="I180" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
+        <v>3899</v>
+      </c>
+      <c r="I180" s="13" t="inlineStr"/>
       <c r="J180" s="13" t="inlineStr"/>
       <c r="K180" s="13" t="inlineStr">
         <is>
-          <t>Mercari</t>
+          <t>eBay (pickup only, over 60 mi)</t>
         </is>
       </c>
       <c r="L180" s="13" t="inlineStr">
@@ -15752,7 +15760,7 @@
       </c>
       <c r="O180" s="14" t="inlineStr">
         <is>
-          <t>Not a flip: ask at/above resale. Ships from MA (city not shown). Mercari blocks automated rechecks.</t>
+          <t>Condition: Pre-Owned.  (eBay card shows no city; pickup distance in source.)</t>
         </is>
       </c>
     </row>
@@ -15764,12 +15772,12 @@
       </c>
       <c r="B181" s="14" t="inlineStr">
         <is>
-          <t>Wolf Gourmet stainless 6-qt Dutch oven with lid</t>
+          <t>Used Wolf SO30F/S 30" 30" Built-In L Series Electric Oven - Frame</t>
         </is>
       </c>
       <c r="C181" s="13" t="inlineStr">
         <is>
-          <t>countertop</t>
+          <t>range/oven/rangetop</t>
         </is>
       </c>
       <c r="D181" s="13" t="inlineStr">
@@ -15779,27 +15787,23 @@
       </c>
       <c r="E181" s="13" t="inlineStr">
         <is>
-          <t>NJ</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F181" s="13" t="n"/>
       <c r="G181" s="13" t="inlineStr">
         <is>
-          <t>$450</t>
+          <t>$1,200</t>
         </is>
       </c>
       <c r="H181" s="15" t="n">
-        <v>450</v>
-      </c>
-      <c r="I181" s="13" t="inlineStr">
-        <is>
-          <t>2026-02-16</t>
-        </is>
-      </c>
+        <v>1200</v>
+      </c>
+      <c r="I181" s="13" t="inlineStr"/>
       <c r="J181" s="13" t="inlineStr"/>
       <c r="K181" s="13" t="inlineStr">
         <is>
-          <t>Mercari</t>
+          <t>eBay (pickup only, over 60 mi)</t>
         </is>
       </c>
       <c r="L181" s="13" t="inlineStr">
@@ -15815,7 +15819,7 @@
       </c>
       <c r="O181" s="14" t="inlineStr">
         <is>
-          <t>Not a flip: ask at/above market; 8-month-old listing. Ships from NJ. Mercari blocks automated rechecks.</t>
+          <t>Condition: Pre-Owned.  (eBay card shows no city; pickup distance in source.)</t>
         </is>
       </c>
     </row>
@@ -15827,7 +15831,7 @@
       </c>
       <c r="B182" s="14" t="inlineStr">
         <is>
-          <t>Wolf Gourmet saucepan with lid</t>
+          <t>Wolf Gourmet 10" skillet</t>
         </is>
       </c>
       <c r="C182" s="13" t="inlineStr">
@@ -15848,15 +15852,15 @@
       <c r="F182" s="13" t="n"/>
       <c r="G182" s="13" t="inlineStr">
         <is>
-          <t>$340</t>
+          <t>$300</t>
         </is>
       </c>
       <c r="H182" s="15" t="n">
-        <v>340</v>
+        <v>300</v>
       </c>
       <c r="I182" s="13" t="inlineStr">
         <is>
-          <t>2025-04-27</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="J182" s="13" t="inlineStr"/>
@@ -15878,7 +15882,7 @@
       </c>
       <c r="O182" s="14" t="inlineStr">
         <is>
-          <t>Not a flip: stale listing (Apr 2025). Ships from MA. Mercari blocks automated rechecks.</t>
+          <t>Not a flip: ask at/above resale. Ships from MA (city not shown). Mercari blocks automated rechecks.</t>
         </is>
       </c>
     </row>
@@ -15890,7 +15894,7 @@
       </c>
       <c r="B183" s="14" t="inlineStr">
         <is>
-          <t>Wolf Gourmet 3.5-qt sauté pan with lid</t>
+          <t>Wolf Gourmet stainless 6-qt Dutch oven with lid</t>
         </is>
       </c>
       <c r="C183" s="13" t="inlineStr">
@@ -15905,21 +15909,21 @@
       </c>
       <c r="E183" s="13" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="F183" s="13" t="n"/>
       <c r="G183" s="13" t="inlineStr">
         <is>
-          <t>$480</t>
+          <t>$450</t>
         </is>
       </c>
       <c r="H183" s="15" t="n">
-        <v>480</v>
+        <v>450</v>
       </c>
       <c r="I183" s="13" t="inlineStr">
         <is>
-          <t>2025-04-27</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="J183" s="13" t="inlineStr"/>
@@ -15941,39 +15945,165 @@
       </c>
       <c r="O183" s="14" t="inlineStr">
         <is>
+          <t>Not a flip: ask at/above market; 8-month-old listing. Ships from NJ. Mercari blocks automated rechecks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="184" outlineLevel="1">
+      <c r="A184" s="13" t="inlineStr">
+        <is>
+          <t>Unknown location</t>
+        </is>
+      </c>
+      <c r="B184" s="14" t="inlineStr">
+        <is>
+          <t>Wolf Gourmet saucepan with lid</t>
+        </is>
+      </c>
+      <c r="C184" s="13" t="inlineStr">
+        <is>
+          <t>countertop</t>
+        </is>
+      </c>
+      <c r="D184" s="13" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E184" s="13" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F184" s="13" t="n"/>
+      <c r="G184" s="13" t="inlineStr">
+        <is>
+          <t>$340</t>
+        </is>
+      </c>
+      <c r="H184" s="15" t="n">
+        <v>340</v>
+      </c>
+      <c r="I184" s="13" t="inlineStr">
+        <is>
+          <t>2025-04-27</t>
+        </is>
+      </c>
+      <c r="J184" s="13" t="inlineStr"/>
+      <c r="K184" s="13" t="inlineStr">
+        <is>
+          <t>Mercari</t>
+        </is>
+      </c>
+      <c r="L184" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M184" s="13" t="inlineStr"/>
+      <c r="N184" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O184" s="14" t="inlineStr">
+        <is>
+          <t>Not a flip: stale listing (Apr 2025). Ships from MA. Mercari blocks automated rechecks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185" outlineLevel="1">
+      <c r="A185" s="13" t="inlineStr">
+        <is>
+          <t>Unknown location</t>
+        </is>
+      </c>
+      <c r="B185" s="14" t="inlineStr">
+        <is>
+          <t>Wolf Gourmet 3.5-qt sauté pan with lid</t>
+        </is>
+      </c>
+      <c r="C185" s="13" t="inlineStr">
+        <is>
+          <t>countertop</t>
+        </is>
+      </c>
+      <c r="D185" s="13" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E185" s="13" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="F185" s="13" t="n"/>
+      <c r="G185" s="13" t="inlineStr">
+        <is>
+          <t>$480</t>
+        </is>
+      </c>
+      <c r="H185" s="15" t="n">
+        <v>480</v>
+      </c>
+      <c r="I185" s="13" t="inlineStr">
+        <is>
+          <t>2025-04-27</t>
+        </is>
+      </c>
+      <c r="J185" s="13" t="inlineStr"/>
+      <c r="K185" s="13" t="inlineStr">
+        <is>
+          <t>Mercari</t>
+        </is>
+      </c>
+      <c r="L185" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M185" s="13" t="inlineStr"/>
+      <c r="N185" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O185" s="14" t="inlineStr">
+        <is>
           <t>Not a flip: stale listing; likely same MA seller as the saucepan. Mercari blocks automated rechecks.</t>
         </is>
       </c>
     </row>
-    <row r="184">
-      <c r="A184" s="17" t="inlineStr">
+    <row r="186">
+      <c r="A186" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Unknown location</t>
         </is>
       </c>
-      <c r="B184" s="17" t="inlineStr">
+      <c r="B186" s="17" t="inlineStr">
         <is>
           <t>60 item(s)</t>
         </is>
       </c>
-      <c r="C184" s="18" t="n"/>
-      <c r="D184" s="18" t="n"/>
-      <c r="E184" s="18" t="n"/>
-      <c r="F184" s="18" t="n"/>
-      <c r="G184" s="18" t="n"/>
-      <c r="H184" s="19" t="n">
+      <c r="C186" s="18" t="n"/>
+      <c r="D186" s="18" t="n"/>
+      <c r="E186" s="18" t="n"/>
+      <c r="F186" s="18" t="n"/>
+      <c r="G186" s="18" t="n"/>
+      <c r="H186" s="19" t="n">
         <v>234881.91</v>
       </c>
-      <c r="I184" s="18" t="n"/>
-      <c r="J184" s="18" t="n"/>
-      <c r="K184" s="18" t="n"/>
-      <c r="L184" s="18" t="n"/>
-      <c r="M184" s="18" t="n"/>
-      <c r="N184" s="18" t="n"/>
-      <c r="O184" s="18" t="n"/>
+      <c r="I186" s="18" t="n"/>
+      <c r="J186" s="18" t="n"/>
+      <c r="K186" s="18" t="n"/>
+      <c r="L186" s="18" t="n"/>
+      <c r="M186" s="18" t="n"/>
+      <c r="N186" s="18" t="n"/>
+      <c r="O186" s="18" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O184"/>
+  <autoFilter ref="A1:O186"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId2"/>
@@ -16075,11 +16205,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N112" r:id="rId98"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N113" r:id="rId99"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N114" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N117" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N118" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N121" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N124" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N125" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N115" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N116" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N119" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N120" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N123" r:id="rId105"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N126" r:id="rId106"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N127" r:id="rId107"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N128" r:id="rId108"/>
@@ -16138,6 +16268,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N181" r:id="rId161"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N182" r:id="rId162"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N183" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N184" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N185" r:id="rId165"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -19975,9 +20107,9 @@
           <t>THC Auction</t>
         </is>
       </c>
-      <c r="L32" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+      <c r="L32" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M32" s="13" t="inlineStr"/>
@@ -21902,9 +22034,9 @@
           <t>HiBid (Ideal Trading Corp)</t>
         </is>
       </c>
-      <c r="L65" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+      <c r="L65" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M65" s="13" t="inlineStr"/>
@@ -23237,9 +23369,9 @@
           <t>PPL Group</t>
         </is>
       </c>
-      <c r="L92" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+      <c r="L92" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M92" s="13" t="inlineStr"/>
@@ -23925,7 +24057,7 @@
       </c>
       <c r="O2" s="14" t="inlineStr">
         <is>
-          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23988,7 +24120,7 @@
       </c>
       <c r="O3" s="14" t="inlineStr">
         <is>
-          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24118,7 +24250,7 @@
       </c>
       <c r="O5" s="14" t="inlineStr">
         <is>
-          <t>Online auction, closes Thu Oct 22 8:37 PM ET. $12.50 high bid (4 bids) as of 2026-10-18. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Online auction, closes Thu Oct 22 8:37 PM ET. $12.50 high bid (4 bids) as of 2026-10-18. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24392,7 +24524,7 @@
       </c>
       <c r="O9" s="14" t="inlineStr">
         <is>
-          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24461,7 +24593,7 @@
       </c>
       <c r="O10" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. FLIP?: Wolf Gourmet blender, bid $0; resale $150-250 but ~800 mi away | HiBid lot closed 2026-10-24 2026-10-25 [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Condition: used. FLIP?: Wolf Gourmet blender, bid $0; resale $150-250 but ~800 mi away | HiBid lot closed 2026-10-24 2026-10-25 [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24656,7 +24788,7 @@
       </c>
       <c r="O13" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24721,7 +24853,7 @@
       </c>
       <c r="O14" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24786,7 +24918,7 @@
       </c>
       <c r="O15" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24916,7 +25048,7 @@
       </c>
       <c r="O17" s="14" t="inlineStr">
         <is>
-          <t>Lots close in sequence from Oct 21 2 PM ET. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Lots close in sequence from Oct 21 2 PM ET. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24981,7 +25113,7 @@
       </c>
       <c r="O18" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25046,7 +25178,7 @@
       </c>
       <c r="O19" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25109,7 +25241,7 @@
       </c>
       <c r="O20" s="14" t="inlineStr">
         <is>
-          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25172,7 +25304,7 @@
       </c>
       <c r="O21" s="14" t="inlineStr">
         <is>
-          <t>Page conflicts: Oct 21 or 22 9 AM (later date used). Closest find. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Page conflicts: Oct 21 or 22 9 AM (later date used). Closest find. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25235,7 +25367,7 @@
       </c>
       <c r="O22" s="14" t="inlineStr">
         <is>
-          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25298,7 +25430,7 @@
       </c>
       <c r="O23" s="14" t="inlineStr">
         <is>
-          <t>Closes Oct 21 10 or 11 AM (later used). Shippable. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Closes Oct 21 10 or 11 AM (later used). Shippable. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25361,7 +25493,7 @@
       </c>
       <c r="O24" s="14" t="inlineStr">
         <is>
-          <t>Oct 21; start time not captured (placeholder 6 PM). [removed 2026-10-21: live webcast auction held Oct 21; listing page now HTTP 503] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Oct 21; start time not captured (placeholder 6 PM). [removed 2026-10-21: live webcast auction held Oct 21; listing page now HTTP 503] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25424,7 +25556,7 @@
       </c>
       <c r="O25" s="14" t="inlineStr">
         <is>
-          <t>Absolute / no reserve. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Absolute / no reserve. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25487,7 +25619,7 @@
       </c>
       <c r="O26" s="14" t="inlineStr">
         <is>
-          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25550,7 +25682,7 @@
       </c>
       <c r="O27" s="14" t="inlineStr">
         <is>
-          <t>Some kitchen gear only. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Some kitchen gear only. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25613,7 +25745,7 @@
       </c>
       <c r="O28" s="14" t="inlineStr">
         <is>
-          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25676,7 +25808,7 @@
       </c>
       <c r="O29" s="14" t="inlineStr">
         <is>
-          <t>Small lot. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Small lot. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25739,7 +25871,7 @@
       </c>
       <c r="O30" s="14" t="inlineStr">
         <is>
-          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25808,7 +25940,7 @@
       </c>
       <c r="O31" s="14" t="inlineStr">
         <is>
-          <t>About 3 days left as of Oct 18 (~Oct 21; exact time not captured). Pickup Sat Oct 24 12–4 PM by appointment. Used, minor wear. eBay asks $200–420; rough resale $150–250. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>About 3 days left as of Oct 18 (~Oct 21; exact time not captured). Pickup Sat Oct 24 12–4 PM by appointment. Used, minor wear. eBay asks $200–420; rough resale $150–250. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25938,7 +26070,7 @@
       </c>
       <c r="O33" s="14" t="inlineStr">
         <is>
-          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26005,7 +26137,7 @@
       </c>
       <c r="O34" s="14" t="inlineStr">
         <is>
-          <t>Wed Oct 21 4 PM. NYC 10013. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Wed Oct 21 4 PM. NYC 10013. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26072,7 +26204,7 @@
       </c>
       <c r="O35" s="14" t="inlineStr">
         <is>
-          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26139,7 +26271,7 @@
       </c>
       <c r="O36" s="14" t="inlineStr">
         <is>
-          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26269,7 +26401,7 @@
       </c>
       <c r="O38" s="14" t="inlineStr">
         <is>
-          <t>Ends Wed Oct 21 8:30 PM EDT. PCI warehouse, 36 Ludlow St, Stamford CT. Page lists preview Oct 28 and removal Thu Oct 29 11-3 (after close). Shipping/delivery available; payment due on pickup day. Items still being added. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Ends Wed Oct 21 8:30 PM EDT. PCI warehouse, 36 Ludlow St, Stamford CT. Page lists preview Oct 28 and removal Thu Oct 29 11-3 (after close). Shipping/delivery available; payment due on pickup day. Items still being added. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26332,7 +26464,7 @@
       </c>
       <c r="O39" s="14" t="inlineStr">
         <is>
-          <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26399,7 +26531,7 @@
       </c>
       <c r="O40" s="14" t="inlineStr">
         <is>
-          <t>Ends Oct 21 7 PM CDT (8 PM ET). 1500 Somerset Ave, Windber PA. Pickups Oct 24-28. Hardware store, not appliance parts. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Ends Oct 21 7 PM CDT (8 PM ET). 1500 Somerset Ave, Windber PA. Pickups Oct 24-28. Hardware store, not appliance parts. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26466,7 +26598,7 @@
       </c>
       <c r="O41" s="14" t="inlineStr">
         <is>
-          <t>Ends Oct 22 7 PM CDT (8 PM ET). Same store as Day 1; pickups Oct 24-28. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Ends Oct 22 7 PM CDT (8 PM ET). Same store as Day 1; pickups Oct 24-28. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lot Recon update 2026-10-25 night: +bl-096 Vernon MI Hardware-Napa auction, bl-090 Bristol dates Nov 6-8, recheck bl-043 (deleted)
</commit_message>
<xml_diff>
--- a/lot_recon.xlsx
+++ b/lot_recon.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wolf New'!$A$1:$O$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Wolf Used'!$A$1:$O$186</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Wolf Unclear'!$A$1:$O$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$105</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 2026-10-25 17:58 ET</t>
+          <t>Last updated: 2026-10-25 17:59 ET</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Active listings: 309 · Removed: 45</t>
+          <t>Active listings: 310 · Removed: 45</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
         <v>30</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>137825</v>
+        <v>137830</v>
       </c>
       <c r="D11" t="n">
         <v>2</v>
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>0</v>
@@ -724,10 +724,10 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>1461321.58</v>
+        <v>1461326.58</v>
       </c>
     </row>
     <row r="15">
@@ -1205,7 +1205,7 @@
         <v>1</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>36005</v>
+        <v>36010</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C30" t="n">
         <v>1</v>
@@ -1235,14 +1235,14 @@
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H30" s="6" t="n">
         <v>5</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>735–1124</t>
+          <t>675–1124</t>
         </is>
       </c>
     </row>
@@ -18202,7 +18202,7 @@
       </c>
       <c r="O35" s="14" t="inlineStr">
         <is>
-          <t>Condition: unknown.</t>
+          <t>Condition: unknown. Checked 2026-10-25 ~6pm ET: still open, closes 7:43 PM ET (soft close).</t>
         </is>
       </c>
     </row>
@@ -18237,11 +18237,11 @@
       </c>
       <c r="G36" s="13" t="inlineStr">
         <is>
-          <t>$0 high bid</t>
+          <t>$5 high bid (2 bids)</t>
         </is>
       </c>
       <c r="H36" s="15" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I36" s="13" t="inlineStr"/>
       <c r="J36" s="13" t="inlineStr">
@@ -18267,7 +18267,7 @@
       </c>
       <c r="O36" s="14" t="inlineStr">
         <is>
-          <t>Condition: unknown.</t>
+          <t>Condition: unknown. Checked 2026-10-25 ~6pm ET: still open, closes 7:43 PM ET (soft close).</t>
         </is>
       </c>
     </row>
@@ -18288,7 +18288,7 @@
       <c r="F37" s="18" t="n"/>
       <c r="G37" s="18" t="n"/>
       <c r="H37" s="19" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="I37" s="18" t="n"/>
       <c r="J37" s="18" t="n"/>
@@ -18342,7 +18342,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O104"/>
+  <dimension ref="A1:O105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -22514,7 +22514,11 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="J75" s="13" t="inlineStr"/>
+      <c r="J75" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-08 05:00 PM ET</t>
+        </is>
+      </c>
       <c r="K75" s="13" t="inlineStr">
         <is>
           <t>Craigslist</t>
@@ -22533,7 +22537,7 @@
       </c>
       <c r="O75" s="14" t="inlineStr">
         <is>
-          <t>Sale 8am-5pm daily, no end date; industrial shelving and lab equipment, not appliances</t>
+          <t>Sale Nov 6-8 ONLY, 8 AM-5 PM (updated 2026-10-25; was 'daily'). 806 Beaver St near Rt 13. Industrial shelving and lab equipment, not appliances; bulk offer invited. Email to schedule viewing.</t>
         </is>
       </c>
     </row>
@@ -23208,7 +23212,7 @@
     <row r="92">
       <c r="A92" s="11" t="inlineStr">
         <is>
-          <t>▸ Midwest  (2)</t>
+          <t>▸ Midwest  (3)</t>
         </is>
       </c>
       <c r="B92" s="12" t="n"/>
@@ -23234,42 +23238,42 @@
       </c>
       <c r="B93" s="14" t="inlineStr">
         <is>
-          <t>American Sale – total liquidation, all 7 stores (pools, hot tubs, grills, holiday decor)</t>
+          <t>Vernon Hardware-Napa inventory liquidation (hardware + NAPA auto parts store closing after 87 yrs): tools, hardware, plumbing, electrical, auto parts</t>
         </is>
       </c>
       <c r="C93" s="13" t="inlineStr">
         <is>
-          <t>retail GOB</t>
+          <t>store closing auction</t>
         </is>
       </c>
       <c r="D93" s="13" t="inlineStr">
         <is>
-          <t>Chicagoland</t>
+          <t>Vernon</t>
         </is>
       </c>
       <c r="E93" s="13" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>MI</t>
         </is>
       </c>
       <c r="F93" s="13" t="n">
-        <v>876</v>
+        <v>675</v>
       </c>
       <c r="G93" s="13" t="inlineStr">
         <is>
-          <t>Retail GOB, up to 70% off</t>
+          <t>No-reserve online auction (Xyz Auction Service), BP 10% cash/cert. check, 13% card</t>
         </is>
       </c>
       <c r="H93" s="15" t="n"/>
-      <c r="I93" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="J93" s="13" t="inlineStr"/>
+      <c r="I93" s="13" t="inlineStr"/>
+      <c r="J93" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-05 07:00 PM ET</t>
+        </is>
+      </c>
       <c r="K93" s="13" t="inlineStr">
         <is>
-          <t>Tiger Group (PR Newswire)</t>
+          <t>EstateSales.net</t>
         </is>
       </c>
       <c r="L93" s="13" t="inlineStr">
@@ -23285,7 +23289,7 @@
       </c>
       <c r="O93" s="14" t="inlineStr">
         <is>
-          <t>Posted Oct 15. Watch for a bulk/fixture auction.</t>
+          <t>Bidding opens Mon Nov 2 7 AM; lots begin closing Thu Nov 5 7 PM (bid on auctioneer's site, (989) 288-4600). Far from MA: only worth it for bulk lots that justify the trip. URL verified live 2026-10-25.</t>
         </is>
       </c>
     </row>
@@ -23297,47 +23301,47 @@
       </c>
       <c r="B94" s="14" t="inlineStr">
         <is>
-          <t>Restaurant, Bar &amp; DJ Equipment Liquidation: Alto-Shaam combi, Southbend/Blodgett ovens, True refrigeration, Manitowoc, Hobart saw, DJ/AV gear</t>
+          <t>American Sale – total liquidation, all 7 stores (pools, hot tubs, grills, holiday decor)</t>
         </is>
       </c>
       <c r="C94" s="13" t="inlineStr">
         <is>
-          <t>restaurant liquidation auction</t>
+          <t>retail GOB</t>
         </is>
       </c>
       <c r="D94" s="13" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Chicagoland</t>
         </is>
       </c>
       <c r="E94" s="13" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="F94" s="13" t="n">
-        <v>1124</v>
+        <v>876</v>
       </c>
       <c r="G94" s="13" t="inlineStr">
         <is>
-          <t>Timed online auction</t>
+          <t>Retail GOB, up to 70% off</t>
         </is>
       </c>
       <c r="H94" s="15" t="n"/>
-      <c r="I94" s="13" t="inlineStr"/>
-      <c r="J94" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26 02:00 PM ET</t>
-        </is>
-      </c>
+      <c r="I94" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="J94" s="13" t="inlineStr"/>
       <c r="K94" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
-        </is>
-      </c>
-      <c r="L94" s="21" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>Tiger Group (PR Newswire)</t>
+        </is>
+      </c>
+      <c r="L94" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M94" s="13" t="inlineStr"/>
@@ -23348,370 +23352,433 @@
       </c>
       <c r="O94" s="14" t="inlineStr">
         <is>
+          <t>Posted Oct 15. Watch for a bulk/fixture auction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" outlineLevel="1">
+      <c r="A95" s="13" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="B95" s="14" t="inlineStr">
+        <is>
+          <t>Restaurant, Bar &amp; DJ Equipment Liquidation: Alto-Shaam combi, Southbend/Blodgett ovens, True refrigeration, Manitowoc, Hobart saw, DJ/AV gear</t>
+        </is>
+      </c>
+      <c r="C95" s="13" t="inlineStr">
+        <is>
+          <t>restaurant liquidation auction</t>
+        </is>
+      </c>
+      <c r="D95" s="13" t="inlineStr">
+        <is>
+          <t>Austin</t>
+        </is>
+      </c>
+      <c r="E95" s="13" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="F95" s="13" t="n">
+        <v>1124</v>
+      </c>
+      <c r="G95" s="13" t="inlineStr">
+        <is>
+          <t>Timed online auction</t>
+        </is>
+      </c>
+      <c r="H95" s="15" t="n"/>
+      <c r="I95" s="13" t="inlineStr"/>
+      <c r="J95" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-26 02:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K95" s="13" t="inlineStr">
+        <is>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L95" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M95" s="13" t="inlineStr"/>
+      <c r="N95" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O95" s="14" t="inlineStr">
+        <is>
           <t>Begins closing Oct 26 1 PM CDT.</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="17" t="inlineStr">
+    <row r="96">
+      <c r="A96" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Midwest</t>
         </is>
       </c>
-      <c r="B95" s="17" t="inlineStr">
-        <is>
-          <t>2 item(s)</t>
-        </is>
-      </c>
-      <c r="C95" s="18" t="n"/>
-      <c r="D95" s="18" t="n"/>
-      <c r="E95" s="18" t="n"/>
-      <c r="F95" s="18" t="n"/>
-      <c r="G95" s="18" t="n"/>
-      <c r="H95" s="19" t="n">
+      <c r="B96" s="17" t="inlineStr">
+        <is>
+          <t>3 item(s)</t>
+        </is>
+      </c>
+      <c r="C96" s="18" t="n"/>
+      <c r="D96" s="18" t="n"/>
+      <c r="E96" s="18" t="n"/>
+      <c r="F96" s="18" t="n"/>
+      <c r="G96" s="18" t="n"/>
+      <c r="H96" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I95" s="18" t="n"/>
-      <c r="J95" s="18" t="n"/>
-      <c r="K95" s="18" t="n"/>
-      <c r="L95" s="18" t="n"/>
-      <c r="M95" s="18" t="n"/>
-      <c r="N95" s="18" t="n"/>
-      <c r="O95" s="18" t="n"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="11" t="inlineStr">
+      <c r="I96" s="18" t="n"/>
+      <c r="J96" s="18" t="n"/>
+      <c r="K96" s="18" t="n"/>
+      <c r="L96" s="18" t="n"/>
+      <c r="M96" s="18" t="n"/>
+      <c r="N96" s="18" t="n"/>
+      <c r="O96" s="18" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="11" t="inlineStr">
         <is>
           <t>▸ Texas / South Central  (1)</t>
         </is>
       </c>
-      <c r="B96" s="12" t="n"/>
-      <c r="C96" s="12" t="n"/>
-      <c r="D96" s="12" t="n"/>
-      <c r="E96" s="12" t="n"/>
-      <c r="F96" s="12" t="n"/>
-      <c r="G96" s="12" t="n"/>
-      <c r="H96" s="12" t="n"/>
-      <c r="I96" s="12" t="n"/>
-      <c r="J96" s="12" t="n"/>
-      <c r="K96" s="12" t="n"/>
-      <c r="L96" s="12" t="n"/>
-      <c r="M96" s="12" t="n"/>
-      <c r="N96" s="12" t="n"/>
-      <c r="O96" s="12" t="n"/>
-    </row>
-    <row r="97" outlineLevel="1">
-      <c r="A97" s="13" t="inlineStr">
+      <c r="B97" s="12" t="n"/>
+      <c r="C97" s="12" t="n"/>
+      <c r="D97" s="12" t="n"/>
+      <c r="E97" s="12" t="n"/>
+      <c r="F97" s="12" t="n"/>
+      <c r="G97" s="12" t="n"/>
+      <c r="H97" s="12" t="n"/>
+      <c r="I97" s="12" t="n"/>
+      <c r="J97" s="12" t="n"/>
+      <c r="K97" s="12" t="n"/>
+      <c r="L97" s="12" t="n"/>
+      <c r="M97" s="12" t="n"/>
+      <c r="N97" s="12" t="n"/>
+      <c r="O97" s="12" t="n"/>
+    </row>
+    <row r="98" outlineLevel="1">
+      <c r="A98" s="13" t="inlineStr">
         <is>
           <t>Texas / South Central</t>
         </is>
       </c>
-      <c r="B97" s="14" t="inlineStr">
+      <c r="B98" s="14" t="inlineStr">
         <is>
           <t>Southwest beverage distributor surplus – mostly unused: 16 True merchandisers, 75 Bunn brewers, 100+ micro-market kiosks</t>
         </is>
       </c>
-      <c r="C97" s="13" t="inlineStr">
+      <c r="C98" s="13" t="inlineStr">
         <is>
           <t>distributor surplus</t>
         </is>
       </c>
-      <c r="D97" s="13" t="inlineStr">
+      <c r="D98" s="13" t="inlineStr">
         <is>
           <t>Mesquite</t>
         </is>
       </c>
-      <c r="E97" s="13" t="inlineStr">
+      <c r="E98" s="13" t="inlineStr">
         <is>
           <t>TX</t>
         </is>
       </c>
-      <c r="F97" s="13" t="n">
+      <c r="F98" s="13" t="n">
         <v>1547</v>
       </c>
-      <c r="G97" s="13" t="inlineStr">
+      <c r="G98" s="13" t="inlineStr">
         <is>
           <t>Online auction</t>
         </is>
       </c>
-      <c r="H97" s="15" t="n"/>
-      <c r="I97" s="13" t="inlineStr"/>
-      <c r="J97" s="13" t="inlineStr">
+      <c r="H98" s="15" t="n"/>
+      <c r="I98" s="13" t="inlineStr"/>
+      <c r="J98" s="13" t="inlineStr">
         <is>
           <t>2026-11-13 11:00 AM ET</t>
         </is>
       </c>
-      <c r="K97" s="13" t="inlineStr">
+      <c r="K98" s="13" t="inlineStr">
         <is>
           <t>Heritage Global Partners</t>
         </is>
       </c>
-      <c r="L97" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M97" s="13" t="inlineStr"/>
-      <c r="N97" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O97" s="14" t="inlineStr">
+      <c r="L98" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M98" s="13" t="inlineStr"/>
+      <c r="N98" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O98" s="14" t="inlineStr">
         <is>
           <t>Near-new appliances, resell by unit. Nov 13 10 AM CST.</t>
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="17" t="inlineStr">
+    <row r="99">
+      <c r="A99" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Texas / South Central</t>
         </is>
       </c>
-      <c r="B98" s="17" t="inlineStr">
+      <c r="B99" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C98" s="18" t="n"/>
-      <c r="D98" s="18" t="n"/>
-      <c r="E98" s="18" t="n"/>
-      <c r="F98" s="18" t="n"/>
-      <c r="G98" s="18" t="n"/>
-      <c r="H98" s="19" t="n">
+      <c r="C99" s="18" t="n"/>
+      <c r="D99" s="18" t="n"/>
+      <c r="E99" s="18" t="n"/>
+      <c r="F99" s="18" t="n"/>
+      <c r="G99" s="18" t="n"/>
+      <c r="H99" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I98" s="18" t="n"/>
-      <c r="J98" s="18" t="n"/>
-      <c r="K98" s="18" t="n"/>
-      <c r="L98" s="18" t="n"/>
-      <c r="M98" s="18" t="n"/>
-      <c r="N98" s="18" t="n"/>
-      <c r="O98" s="18" t="n"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="11" t="inlineStr">
+      <c r="I99" s="18" t="n"/>
+      <c r="J99" s="18" t="n"/>
+      <c r="K99" s="18" t="n"/>
+      <c r="L99" s="18" t="n"/>
+      <c r="M99" s="18" t="n"/>
+      <c r="N99" s="18" t="n"/>
+      <c r="O99" s="18" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="11" t="inlineStr">
         <is>
           <t>▸ West / Other  (1)</t>
         </is>
       </c>
-      <c r="B99" s="12" t="n"/>
-      <c r="C99" s="12" t="n"/>
-      <c r="D99" s="12" t="n"/>
-      <c r="E99" s="12" t="n"/>
-      <c r="F99" s="12" t="n"/>
-      <c r="G99" s="12" t="n"/>
-      <c r="H99" s="12" t="n"/>
-      <c r="I99" s="12" t="n"/>
-      <c r="J99" s="12" t="n"/>
-      <c r="K99" s="12" t="n"/>
-      <c r="L99" s="12" t="n"/>
-      <c r="M99" s="12" t="n"/>
-      <c r="N99" s="12" t="n"/>
-      <c r="O99" s="12" t="n"/>
-    </row>
-    <row r="100" outlineLevel="1">
-      <c r="A100" s="13" t="inlineStr">
+      <c r="B100" s="12" t="n"/>
+      <c r="C100" s="12" t="n"/>
+      <c r="D100" s="12" t="n"/>
+      <c r="E100" s="12" t="n"/>
+      <c r="F100" s="12" t="n"/>
+      <c r="G100" s="12" t="n"/>
+      <c r="H100" s="12" t="n"/>
+      <c r="I100" s="12" t="n"/>
+      <c r="J100" s="12" t="n"/>
+      <c r="K100" s="12" t="n"/>
+      <c r="L100" s="12" t="n"/>
+      <c r="M100" s="12" t="n"/>
+      <c r="N100" s="12" t="n"/>
+      <c r="O100" s="12" t="n"/>
+    </row>
+    <row r="101" outlineLevel="1">
+      <c r="A101" s="13" t="inlineStr">
         <is>
           <t>West / Other</t>
         </is>
       </c>
-      <c r="B100" s="14" t="inlineStr">
+      <c r="B101" s="14" t="inlineStr">
         <is>
           <t>National salad concept liquidation – full contents of 63 fast-casual restaurants (AZ/TX/OK/NV)</t>
         </is>
       </c>
-      <c r="C100" s="13" t="inlineStr">
+      <c r="C101" s="13" t="inlineStr">
         <is>
           <t>restaurant chain liquidation</t>
         </is>
       </c>
-      <c r="D100" s="13" t="inlineStr">
+      <c r="D101" s="13" t="inlineStr">
         <is>
           <t>Phoenix</t>
         </is>
       </c>
-      <c r="E100" s="13" t="inlineStr">
+      <c r="E101" s="13" t="inlineStr">
         <is>
           <t>AZ</t>
         </is>
       </c>
-      <c r="F100" s="13" t="n">
+      <c r="F101" s="13" t="n">
         <v>2307</v>
       </c>
-      <c r="G100" s="13" t="inlineStr">
+      <c r="G101" s="13" t="inlineStr">
         <is>
           <t>Online auctions, dates TBD</t>
         </is>
       </c>
-      <c r="H100" s="15" t="n"/>
-      <c r="I100" s="13" t="inlineStr">
+      <c r="H101" s="15" t="n"/>
+      <c r="I101" s="13" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="J100" s="13" t="inlineStr"/>
-      <c r="K100" s="13" t="inlineStr">
+      <c r="J101" s="13" t="inlineStr"/>
+      <c r="K101" s="13" t="inlineStr">
         <is>
           <t>RestaurantEquipment.bid (TAGeX)</t>
         </is>
       </c>
-      <c r="L100" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M100" s="13" t="inlineStr"/>
-      <c r="N100" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O100" s="14" t="inlineStr">
+      <c r="L101" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M101" s="13" t="inlineStr"/>
+      <c r="N101" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O101" s="14" t="inlineStr">
         <is>
           <t>Rolling market-by-market auctions, none live yet (Phoenix metro 30 locations, DFW 14, Tucson 6, Houston 5, plus OK/NV). Pickup on site at each restaurant. Pinned at Phoenix.</t>
         </is>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="17" t="inlineStr">
+    <row r="102">
+      <c r="A102" s="17" t="inlineStr">
         <is>
           <t>Subtotal — West / Other</t>
         </is>
       </c>
-      <c r="B101" s="17" t="inlineStr">
+      <c r="B102" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C101" s="18" t="n"/>
-      <c r="D101" s="18" t="n"/>
-      <c r="E101" s="18" t="n"/>
-      <c r="F101" s="18" t="n"/>
-      <c r="G101" s="18" t="n"/>
-      <c r="H101" s="19" t="n">
+      <c r="C102" s="18" t="n"/>
+      <c r="D102" s="18" t="n"/>
+      <c r="E102" s="18" t="n"/>
+      <c r="F102" s="18" t="n"/>
+      <c r="G102" s="18" t="n"/>
+      <c r="H102" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I101" s="18" t="n"/>
-      <c r="J101" s="18" t="n"/>
-      <c r="K101" s="18" t="n"/>
-      <c r="L101" s="18" t="n"/>
-      <c r="M101" s="18" t="n"/>
-      <c r="N101" s="18" t="n"/>
-      <c r="O101" s="18" t="n"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="11" t="inlineStr">
+      <c r="I102" s="18" t="n"/>
+      <c r="J102" s="18" t="n"/>
+      <c r="K102" s="18" t="n"/>
+      <c r="L102" s="18" t="n"/>
+      <c r="M102" s="18" t="n"/>
+      <c r="N102" s="18" t="n"/>
+      <c r="O102" s="18" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="11" t="inlineStr">
         <is>
           <t>▸ Unknown location  (1)</t>
         </is>
       </c>
-      <c r="B102" s="12" t="n"/>
-      <c r="C102" s="12" t="n"/>
-      <c r="D102" s="12" t="n"/>
-      <c r="E102" s="12" t="n"/>
-      <c r="F102" s="12" t="n"/>
-      <c r="G102" s="12" t="n"/>
-      <c r="H102" s="12" t="n"/>
-      <c r="I102" s="12" t="n"/>
-      <c r="J102" s="12" t="n"/>
-      <c r="K102" s="12" t="n"/>
-      <c r="L102" s="12" t="n"/>
-      <c r="M102" s="12" t="n"/>
-      <c r="N102" s="12" t="n"/>
-      <c r="O102" s="12" t="n"/>
-    </row>
-    <row r="103" outlineLevel="1">
-      <c r="A103" s="13" t="inlineStr">
+      <c r="B103" s="12" t="n"/>
+      <c r="C103" s="12" t="n"/>
+      <c r="D103" s="12" t="n"/>
+      <c r="E103" s="12" t="n"/>
+      <c r="F103" s="12" t="n"/>
+      <c r="G103" s="12" t="n"/>
+      <c r="H103" s="12" t="n"/>
+      <c r="I103" s="12" t="n"/>
+      <c r="J103" s="12" t="n"/>
+      <c r="K103" s="12" t="n"/>
+      <c r="L103" s="12" t="n"/>
+      <c r="M103" s="12" t="n"/>
+      <c r="N103" s="12" t="n"/>
+      <c r="O103" s="12" t="n"/>
+    </row>
+    <row r="104" outlineLevel="1">
+      <c r="A104" s="13" t="inlineStr">
         <is>
           <t>Unknown location</t>
         </is>
       </c>
-      <c r="B103" s="14" t="inlineStr">
+      <c r="B104" s="14" t="inlineStr">
         <is>
           <t>Retail furniture store auction: living room sets, sofas, dining/bedroom sets, recliners, dinettes, chandeliers, lamps, rugs, decor, store fixtures</t>
         </is>
       </c>
-      <c r="C103" s="13" t="inlineStr">
+      <c r="C104" s="13" t="inlineStr">
         <is>
           <t>store closing auction</t>
         </is>
       </c>
-      <c r="D103" s="13" t="inlineStr">
+      <c r="D104" s="13" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="E103" s="13" t="inlineStr">
+      <c r="E104" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F103" s="13" t="n"/>
-      <c r="G103" s="13" t="inlineStr">
+      <c r="F104" s="13" t="n"/>
+      <c r="G104" s="13" t="inlineStr">
         <is>
           <t>Online-only auction (BidSpotter), 18% BP</t>
         </is>
       </c>
-      <c r="H103" s="15" t="n"/>
-      <c r="I103" s="13" t="inlineStr"/>
-      <c r="J103" s="13" t="inlineStr">
+      <c r="H104" s="15" t="n"/>
+      <c r="I104" s="13" t="inlineStr"/>
+      <c r="J104" s="13" t="inlineStr">
         <is>
           <t>2026-10-29 10:00 AM ET</t>
         </is>
       </c>
-      <c r="K103" s="13" t="inlineStr">
+      <c r="K104" s="13" t="inlineStr">
         <is>
           <t>Paul E. Saperstein (PESCO)</t>
         </is>
       </c>
-      <c r="L103" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M103" s="13" t="inlineStr"/>
-      <c r="N103" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O103" s="14" t="inlineStr">
+      <c r="L104" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M104" s="13" t="inlineStr"/>
+      <c r="N104" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O104" s="14" t="inlineStr">
         <is>
           <t>Location TBD (not yet released; PESCO licensed MA/NH/RI/VT, terms cite MA sales tax). Showroom display items, as-is. Inspection Wed Oct 28 12-6 PM; pickup Oct 30, Oct 31, Nov 2.</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="17" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Unknown location</t>
         </is>
       </c>
-      <c r="B104" s="17" t="inlineStr">
+      <c r="B105" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C104" s="18" t="n"/>
-      <c r="D104" s="18" t="n"/>
-      <c r="E104" s="18" t="n"/>
-      <c r="F104" s="18" t="n"/>
-      <c r="G104" s="18" t="n"/>
-      <c r="H104" s="19" t="n">
+      <c r="C105" s="18" t="n"/>
+      <c r="D105" s="18" t="n"/>
+      <c r="E105" s="18" t="n"/>
+      <c r="F105" s="18" t="n"/>
+      <c r="G105" s="18" t="n"/>
+      <c r="H105" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I104" s="18" t="n"/>
-      <c r="J104" s="18" t="n"/>
-      <c r="K104" s="18" t="n"/>
-      <c r="L104" s="18" t="n"/>
-      <c r="M104" s="18" t="n"/>
-      <c r="N104" s="18" t="n"/>
-      <c r="O104" s="18" t="n"/>
+      <c r="I105" s="18" t="n"/>
+      <c r="J105" s="18" t="n"/>
+      <c r="K105" s="18" t="n"/>
+      <c r="L105" s="18" t="n"/>
+      <c r="M105" s="18" t="n"/>
+      <c r="N105" s="18" t="n"/>
+      <c r="O105" s="18" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O104"/>
+  <autoFilter ref="A1:O105"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId2"/>
@@ -23781,9 +23848,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N90" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N93" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N94" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N97" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N100" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N103" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N95" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N98" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N101" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N104" r:id="rId72"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -23957,7 +24025,7 @@
       </c>
       <c r="O2" s="14" t="inlineStr">
         <is>
-          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24020,7 +24088,7 @@
       </c>
       <c r="O3" s="14" t="inlineStr">
         <is>
-          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24150,7 +24218,7 @@
       </c>
       <c r="O5" s="14" t="inlineStr">
         <is>
-          <t>Online auction, closes Thu Oct 22 8:37 PM ET. $12.50 high bid (4 bids) as of 2026-10-18. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Online auction, closes Thu Oct 22 8:37 PM ET. $12.50 high bid (4 bids) as of 2026-10-18. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24493,7 +24561,7 @@
       </c>
       <c r="O10" s="14" t="inlineStr">
         <is>
-          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24562,7 +24630,7 @@
       </c>
       <c r="O11" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. FLIP?: Wolf Gourmet blender, bid $0; resale $150-250 but ~800 mi away | HiBid lot closed 2026-10-24 2026-10-25 [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Condition: used. FLIP?: Wolf Gourmet blender, bid $0; resale $150-250 but ~800 mi away | HiBid lot closed 2026-10-24 2026-10-25 [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24757,7 +24825,7 @@
       </c>
       <c r="O14" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24822,7 +24890,7 @@
       </c>
       <c r="O15" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24887,7 +24955,7 @@
       </c>
       <c r="O16" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25017,7 +25085,7 @@
       </c>
       <c r="O18" s="14" t="inlineStr">
         <is>
-          <t>Lots close in sequence from Oct 21 2 PM ET. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Lots close in sequence from Oct 21 2 PM ET. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25082,7 +25150,7 @@
       </c>
       <c r="O19" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25147,7 +25215,7 @@
       </c>
       <c r="O20" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25210,7 +25278,7 @@
       </c>
       <c r="O21" s="14" t="inlineStr">
         <is>
-          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25273,7 +25341,7 @@
       </c>
       <c r="O22" s="14" t="inlineStr">
         <is>
-          <t>Page conflicts: Oct 21 or 22 9 AM (later date used). Closest find. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Page conflicts: Oct 21 or 22 9 AM (later date used). Closest find. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25336,7 +25404,7 @@
       </c>
       <c r="O23" s="14" t="inlineStr">
         <is>
-          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25399,7 +25467,7 @@
       </c>
       <c r="O24" s="14" t="inlineStr">
         <is>
-          <t>Closes Oct 21 10 or 11 AM (later used). Shippable. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Closes Oct 21 10 or 11 AM (later used). Shippable. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25462,7 +25530,7 @@
       </c>
       <c r="O25" s="14" t="inlineStr">
         <is>
-          <t>Oct 21; start time not captured (placeholder 6 PM). [removed 2026-10-21: live webcast auction held Oct 21; listing page now HTTP 503] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Oct 21; start time not captured (placeholder 6 PM). [removed 2026-10-21: live webcast auction held Oct 21; listing page now HTTP 503] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25525,7 +25593,7 @@
       </c>
       <c r="O26" s="14" t="inlineStr">
         <is>
-          <t>Absolute / no reserve. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Absolute / no reserve. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25588,7 +25656,7 @@
       </c>
       <c r="O27" s="14" t="inlineStr">
         <is>
-          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25651,7 +25719,7 @@
       </c>
       <c r="O28" s="14" t="inlineStr">
         <is>
-          <t>Some kitchen gear only. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Some kitchen gear only. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25714,7 +25782,7 @@
       </c>
       <c r="O29" s="14" t="inlineStr">
         <is>
-          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25777,7 +25845,7 @@
       </c>
       <c r="O30" s="14" t="inlineStr">
         <is>
-          <t>Small lot. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Small lot. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25840,7 +25908,7 @@
       </c>
       <c r="O31" s="14" t="inlineStr">
         <is>
-          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25909,7 +25977,7 @@
       </c>
       <c r="O32" s="14" t="inlineStr">
         <is>
-          <t>About 3 days left as of Oct 18 (~Oct 21; exact time not captured). Pickup Sat Oct 24 12–4 PM by appointment. Used, minor wear. eBay asks $200–420; rough resale $150–250. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>About 3 days left as of Oct 18 (~Oct 21; exact time not captured). Pickup Sat Oct 24 12–4 PM by appointment. Used, minor wear. eBay asks $200–420; rough resale $150–250. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25980,7 +26048,7 @@
       </c>
       <c r="O33" s="14" t="inlineStr">
         <is>
-          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale. [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale. [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26110,7 +26178,7 @@
       </c>
       <c r="O35" s="14" t="inlineStr">
         <is>
-          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26177,7 +26245,7 @@
       </c>
       <c r="O36" s="14" t="inlineStr">
         <is>
-          <t>Wed Oct 21 4 PM. NYC 10013. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Wed Oct 21 4 PM. NYC 10013. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26244,7 +26312,7 @@
       </c>
       <c r="O37" s="14" t="inlineStr">
         <is>
-          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26311,7 +26379,7 @@
       </c>
       <c r="O38" s="14" t="inlineStr">
         <is>
-          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26374,7 +26442,7 @@
       </c>
       <c r="O39" s="14" t="inlineStr">
         <is>
-          <t>Small off-category FYI; seller says resell individually. Same $250 / 10-tool lot, reposted under new CL URLs repeatedly (latest 2026-10-22 4:24 PM). | CL repost 6Z43nD92 deleted by author 2026-10-24 | Reposted 2026-10-25 11:25 AM (xxm7mDLa), now $225; reactivated. | CL posting deleted 2026-10-25</t>
+          <t>Small off-category FYI; seller says resell individually. Same $250 / 10-tool lot, reposted under new CL URLs repeatedly (latest 2026-10-22 4:24 PM). | CL repost 6Z43nD92 deleted by author 2026-10-24 | Reposted 2026-10-25 11:25 AM (xxm7mDLa), now $225; reactivated. | CL posting deleted 2026-10-25 | Re-verified 2026-10-25 6pm ET: HTTP 410, 'This posting has been deleted by its author'; stays REMOVED.</t>
         </is>
       </c>
     </row>
@@ -26441,7 +26509,7 @@
       </c>
       <c r="O40" s="14" t="inlineStr">
         <is>
-          <t>Ends Wed Oct 21 8:30 PM EDT. PCI warehouse, 36 Ludlow St, Stamford CT. Page lists preview Oct 28 and removal Thu Oct 29 11-3 (after close). Shipping/delivery available; payment due on pickup day. Items still being added. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Ends Wed Oct 21 8:30 PM EDT. PCI warehouse, 36 Ludlow St, Stamford CT. Page lists preview Oct 28 and removal Thu Oct 29 11-3 (after close). Shipping/delivery available; payment due on pickup day. Items still being added. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26504,7 +26572,7 @@
       </c>
       <c r="O41" s="14" t="inlineStr">
         <is>
-          <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26571,7 +26639,7 @@
       </c>
       <c r="O42" s="14" t="inlineStr">
         <is>
-          <t>Ends Oct 21 7 PM CDT (8 PM ET). 1500 Somerset Ave, Windber PA. Pickups Oct 24-28. Hardware store, not appliance parts. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Ends Oct 21 7 PM CDT (8 PM ET). 1500 Somerset Ave, Windber PA. Pickups Oct 24-28. Hardware store, not appliance parts. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26638,7 +26706,7 @@
       </c>
       <c r="O43" s="14" t="inlineStr">
         <is>
-          <t>Ends Oct 22 7 PM CDT (8 PM ET). Same store as Day 1; pickups Oct 24-28. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
+          <t>Ends Oct 22 7 PM CDT (8 PM ET). Same store as Day 1; pickups Oct 24-28. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26837,7 +26905,7 @@
       </c>
       <c r="O46" s="14" t="inlineStr">
         <is>
-          <t>864 S Undermountain Rd. Event Barn + Stagecoach Tavern contents, furniture, lamps, rugs, restaurant supplies. Oct 24 10-6 and Oct 25 12-3 only. [auto-removed 2026-10-25: closing date passed]</t>
+          <t>864 S Undermountain Rd. Event Barn + Stagecoach Tavern contents, furniture, lamps, rugs, restaurant supplies. Oct 24 10-6 and Oct 25 12-3 only. [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lot Recon update 2026-10-26 pm: +bl-097 Pete's Famous Bakery (PCI Ewing NJ, ends Nov 8), +bl-098 The Mill Restaurant & Cafe (PCI Ewing NJ, ends Nov 1); restore bl-045 Outlaw Grill Stamford CT (still live, ends Oct 28 8:30 PM EDT)
</commit_message>
<xml_diff>
--- a/lot_recon.xlsx
+++ b/lot_recon.xlsx
@@ -20,8 +20,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wolf New'!$A$1:$O$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Wolf Used'!$A$1:$O$184</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Wolf Unclear'!$A$1:$O$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$103</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 2026-10-26 08:07 ET</t>
+          <t>Last updated: 2026-10-26 10:41 ET</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Active listings: 306 · Removed: 49</t>
+          <t>Active listings: 309 · Removed: 48</t>
         </is>
       </c>
     </row>
@@ -708,13 +708,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13">
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="C13" s="7" t="n">
         <v>1453577.58</v>
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C23" t="n">
         <v>1</v>
@@ -1004,7 +1004,7 @@
         <v>4</v>
       </c>
       <c r="G23" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H23" s="6" t="n">
         <v>64650</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C24" t="n">
         <v>1</v>
@@ -1037,7 +1037,7 @@
         <v>24</v>
       </c>
       <c r="G24" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H24" s="6" t="n">
         <v>455590</v>
@@ -18026,7 +18026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O103"/>
+  <dimension ref="A1:O106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -19764,7 +19764,7 @@
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>▸ CT / Hudson Valley  (9)</t>
+          <t>▸ CT / Hudson Valley  (10)</t>
         </is>
       </c>
       <c r="B34" s="12" t="n"/>
@@ -20105,47 +20105,51 @@
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>BJ's Wholesale closeout – racking, forklifts, Hobart</t>
+          <t>The Outlaw Grill Steakhouse – used restaurant equipment auction (PCI Auctions CT, e.g. Vulcan EV60 Endurance 60" range)</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>restaurant auction</t>
         </is>
       </c>
       <c r="D40" s="13" t="inlineStr">
         <is>
-          <t>Rotterdam</t>
+          <t>Stamford</t>
         </is>
       </c>
       <c r="E40" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Online auction, current bids (Vulcan EV60 range now $175, list $21,895)</t>
         </is>
       </c>
       <c r="H40" s="15" t="n"/>
-      <c r="I40" s="13" t="inlineStr"/>
+      <c r="I40" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
       <c r="J40" s="13" t="inlineStr">
         <is>
-          <t>2026-11-10 10:00 AM ET</t>
+          <t>2026-10-28 08:30 PM ET</t>
         </is>
       </c>
       <c r="K40" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
-        </is>
-      </c>
-      <c r="L40" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>PCI Auctions</t>
+        </is>
+      </c>
+      <c r="L40" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M40" s="13" t="inlineStr"/>
@@ -20156,7 +20160,7 @@
       </c>
       <c r="O40" s="14" t="inlineStr">
         <is>
-          <t>Closes from Nov 10 10 AM.</t>
+          <t>Ends Wed Oct 28 8:30 PM EDT (corrected: earlier Oct 21 date was wrong; still live 2026-10-26). PCI warehouse, 36 Ludlow St, Stamford CT. Preview Oct 28 11-2; removal Thu Oct 29 11-3. Vulcan EV60 electric range ($21,895 list, now $175) plus Hobart equipment. Shipping/delivery available; payment due on pickup day.</t>
         </is>
       </c>
     </row>
@@ -20168,17 +20172,17 @@
       </c>
       <c r="B41" s="14" t="inlineStr">
         <is>
-          <t>Retiring horse tack shop (25 yrs online + retail) – remaining inventory: new English &amp; Western tack, saddles, apparel, equipment, plus shelving/displays</t>
+          <t>BJ's Wholesale closeout – racking, forklifts, Hobart</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
-          <t>retirement</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D41" s="13" t="inlineStr">
         <is>
-          <t>Gardiner</t>
+          <t>Rotterdam</t>
         </is>
       </c>
       <c r="E41" s="13" t="inlineStr">
@@ -20187,23 +20191,23 @@
         </is>
       </c>
       <c r="F41" s="13" t="n">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="G41" s="13" t="inlineStr">
         <is>
-          <t>$80,000 (seller cites $200K+ retail)</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H41" s="15" t="n"/>
-      <c r="I41" s="13" t="inlineStr">
-        <is>
-          <t>2026-05-16</t>
-        </is>
-      </c>
-      <c r="J41" s="13" t="inlineStr"/>
+      <c r="I41" s="13" t="inlineStr"/>
+      <c r="J41" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-10 10:00 AM ET</t>
+        </is>
+      </c>
       <c r="K41" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>Grafe Auction</t>
         </is>
       </c>
       <c r="L41" s="13" t="inlineStr">
@@ -20219,7 +20223,7 @@
       </c>
       <c r="O41" s="14" t="inlineStr">
         <is>
-          <t>Old post (May) but still live 2026-10-24; whole-inventory buyout, call for details. Large capital outlay; niche (equestrian).</t>
+          <t>Closes from Nov 10 10 AM.</t>
         </is>
       </c>
     </row>
@@ -20231,17 +20235,17 @@
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>Body shop closing after 50 years – tools, welder, generators, plasma</t>
+          <t>Retiring horse tack shop (25 yrs online + retail) – remaining inventory: new English &amp; Western tack, saddles, apparel, equipment, plus shelving/displays</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>tools liquidation</t>
+          <t>retirement</t>
         </is>
       </c>
       <c r="D42" s="13" t="inlineStr">
         <is>
-          <t>West Nyack</t>
+          <t>Gardiner</t>
         </is>
       </c>
       <c r="E42" s="13" t="inlineStr">
@@ -20250,17 +20254,17 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>Make offer / lot</t>
+          <t>$80,000 (seller cites $200K+ retail)</t>
         </is>
       </c>
       <c r="H42" s="15" t="n"/>
       <c r="I42" s="13" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="J42" s="13" t="inlineStr"/>
@@ -20282,7 +20286,7 @@
       </c>
       <c r="O42" s="14" t="inlineStr">
         <is>
-          <t>One-man auto body shop closing/retirement (Park Ridge / West Nyack NY-NJ border). Heat lamps, Kansas jack pullers, Miller 200 welder, generators, sheet-metal brake, hydraulic press, plasma cutter, engine hoist. Posted Aug 16; still open 2026-10-19.</t>
+          <t>Old post (May) but still live 2026-10-24; whole-inventory buyout, call for details. Large capital outlay; niche (equestrian).</t>
         </is>
       </c>
     </row>
@@ -20294,17 +20298,17 @@
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>Woodworkers shop closing sale – shop tools &amp; hand tools</t>
+          <t>Body shop closing after 50 years – tools, welder, generators, plasma</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
         <is>
-          <t>woodworking shop closing</t>
+          <t>tools liquidation</t>
         </is>
       </c>
       <c r="D43" s="13" t="inlineStr">
         <is>
-          <t>Tappan</t>
+          <t>West Nyack</t>
         </is>
       </c>
       <c r="E43" s="13" t="inlineStr">
@@ -20313,17 +20317,17 @@
         </is>
       </c>
       <c r="F43" s="13" t="n">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G43" s="13" t="inlineStr">
         <is>
-          <t>Priced individually (some free)</t>
+          <t>Make offer / lot</t>
         </is>
       </c>
       <c r="H43" s="15" t="n"/>
       <c r="I43" s="13" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="J43" s="13" t="inlineStr"/>
@@ -20345,124 +20349,120 @@
       </c>
       <c r="O43" s="14" t="inlineStr">
         <is>
+          <t>One-man auto body shop closing/retirement (Park Ridge / West Nyack NY-NJ border). Heat lamps, Kansas jack pullers, Miller 200 welder, generators, sheet-metal brake, hydraulic press, plasma cutter, engine hoist. Posted Aug 16; still open 2026-10-19.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" outlineLevel="1">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
+          <t>CT / Hudson Valley</t>
+        </is>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>Woodworkers shop closing sale – shop tools &amp; hand tools</t>
+        </is>
+      </c>
+      <c r="C44" s="13" t="inlineStr">
+        <is>
+          <t>woodworking shop closing</t>
+        </is>
+      </c>
+      <c r="D44" s="13" t="inlineStr">
+        <is>
+          <t>Tappan</t>
+        </is>
+      </c>
+      <c r="E44" s="13" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="F44" s="13" t="n">
+        <v>179</v>
+      </c>
+      <c r="G44" s="13" t="inlineStr">
+        <is>
+          <t>Priced individually (some free)</t>
+        </is>
+      </c>
+      <c r="H44" s="15" t="n"/>
+      <c r="I44" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="J44" s="13" t="inlineStr"/>
+      <c r="K44" s="13" t="inlineStr">
+        <is>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L44" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M44" s="13" t="inlineStr"/>
+      <c r="N44" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O44" s="14" t="inlineStr">
+        <is>
           <t>Ongoing shop-closing sale at 61 Main St, Tappan; many shop and hand tools, schedule a visit. Near the West Nyack body-shop sale (bl-054) for one trip.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="17" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="17" t="inlineStr">
         <is>
           <t>Subtotal — CT / Hudson Valley</t>
         </is>
       </c>
-      <c r="B44" s="17" t="inlineStr">
-        <is>
-          <t>9 item(s)</t>
-        </is>
-      </c>
-      <c r="C44" s="18" t="n"/>
-      <c r="D44" s="18" t="n"/>
-      <c r="E44" s="18" t="n"/>
-      <c r="F44" s="18" t="n"/>
-      <c r="G44" s="18" t="n"/>
-      <c r="H44" s="19" t="n">
+      <c r="B45" s="17" t="inlineStr">
+        <is>
+          <t>10 item(s)</t>
+        </is>
+      </c>
+      <c r="C45" s="18" t="n"/>
+      <c r="D45" s="18" t="n"/>
+      <c r="E45" s="18" t="n"/>
+      <c r="F45" s="18" t="n"/>
+      <c r="G45" s="18" t="n"/>
+      <c r="H45" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I44" s="18" t="n"/>
-      <c r="J44" s="18" t="n"/>
-      <c r="K44" s="18" t="n"/>
-      <c r="L44" s="18" t="n"/>
-      <c r="M44" s="18" t="n"/>
-      <c r="N44" s="18" t="n"/>
-      <c r="O44" s="18" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="11" t="inlineStr">
-        <is>
-          <t>▸ NYC / Long Island / NJ  (27)</t>
-        </is>
-      </c>
-      <c r="B45" s="12" t="n"/>
-      <c r="C45" s="12" t="n"/>
-      <c r="D45" s="12" t="n"/>
-      <c r="E45" s="12" t="n"/>
-      <c r="F45" s="12" t="n"/>
-      <c r="G45" s="12" t="n"/>
-      <c r="H45" s="12" t="n"/>
-      <c r="I45" s="12" t="n"/>
-      <c r="J45" s="12" t="n"/>
-      <c r="K45" s="12" t="n"/>
-      <c r="L45" s="12" t="n"/>
-      <c r="M45" s="12" t="n"/>
-      <c r="N45" s="12" t="n"/>
-      <c r="O45" s="12" t="n"/>
-    </row>
-    <row r="46" outlineLevel="1">
-      <c r="A46" s="13" t="inlineStr">
-        <is>
-          <t>NYC / Long Island / NJ</t>
-        </is>
-      </c>
-      <c r="B46" s="14" t="inlineStr">
-        <is>
-          <t>Met Foodmarkets turnkey grocery liquidation (Grafe Auction)</t>
-        </is>
-      </c>
-      <c r="C46" s="13" t="inlineStr">
-        <is>
-          <t>store closing</t>
-        </is>
-      </c>
-      <c r="D46" s="13" t="inlineStr">
-        <is>
-          <t>Bronx</t>
-        </is>
-      </c>
-      <c r="E46" s="13" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="F46" s="13" t="n">
-        <v>181</v>
-      </c>
-      <c r="G46" s="13" t="inlineStr">
-        <is>
-          <t>Online auction</t>
-        </is>
-      </c>
-      <c r="H46" s="15" t="n"/>
-      <c r="I46" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="J46" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-11 01:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K46" s="13" t="inlineStr">
-        <is>
-          <t>Grafe Auction</t>
-        </is>
-      </c>
-      <c r="L46" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M46" s="13" t="inlineStr"/>
-      <c r="N46" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O46" s="14" t="inlineStr">
-        <is>
-          <t>2 Hussmann compressor racks, 3-room Amerikooler walk-in cooler/freezer, Hussmann/Hill Phoenix remote cases, 24+ frozen doors, True/Red Bull merchandisers, Hobart mixer-grinder and wrappers, Lyons checkouts, NCR POS, Storflex shelving. Preview Nov 11 9AM-12PM; begins closing Nov 11 1PM EST.</t>
-        </is>
-      </c>
+      <c r="I45" s="18" t="n"/>
+      <c r="J45" s="18" t="n"/>
+      <c r="K45" s="18" t="n"/>
+      <c r="L45" s="18" t="n"/>
+      <c r="M45" s="18" t="n"/>
+      <c r="N45" s="18" t="n"/>
+      <c r="O45" s="18" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>▸ NYC / Long Island / NJ  (29)</t>
+        </is>
+      </c>
+      <c r="B46" s="12" t="n"/>
+      <c r="C46" s="12" t="n"/>
+      <c r="D46" s="12" t="n"/>
+      <c r="E46" s="12" t="n"/>
+      <c r="F46" s="12" t="n"/>
+      <c r="G46" s="12" t="n"/>
+      <c r="H46" s="12" t="n"/>
+      <c r="I46" s="12" t="n"/>
+      <c r="J46" s="12" t="n"/>
+      <c r="K46" s="12" t="n"/>
+      <c r="L46" s="12" t="n"/>
+      <c r="M46" s="12" t="n"/>
+      <c r="N46" s="12" t="n"/>
+      <c r="O46" s="12" t="n"/>
     </row>
     <row r="47" outlineLevel="1">
       <c r="A47" s="13" t="inlineStr">
@@ -20472,42 +20472,46 @@
       </c>
       <c r="B47" s="14" t="inlineStr">
         <is>
-          <t>Viva Margherita restaurant complete contents (building torn down)</t>
+          <t>Met Foodmarkets turnkey grocery liquidation (Grafe Auction)</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
         <is>
-          <t>restaurant closing</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>Edgewater</t>
+          <t>Bronx</t>
         </is>
       </c>
       <c r="E47" s="13" t="inlineStr">
         <is>
-          <t>NJ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F47" s="13" t="n">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="G47" s="13" t="inlineStr">
         <is>
-          <t>Complete contents / make offer</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H47" s="15" t="n"/>
       <c r="I47" s="13" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-      <c r="J47" s="13" t="inlineStr"/>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="J47" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-11 01:00 PM ET</t>
+        </is>
+      </c>
       <c r="K47" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>Grafe Auction</t>
         </is>
       </c>
       <c r="L47" s="13" t="inlineStr">
@@ -20523,7 +20527,7 @@
       </c>
       <c r="O47" s="14" t="inlineStr">
         <is>
-          <t>Address 163 Old River Road, Edgewater NJ. Building being torn down; complete restaurant contents for sale / make offer.</t>
+          <t>2 Hussmann compressor racks, 3-room Amerikooler walk-in cooler/freezer, Hussmann/Hill Phoenix remote cases, 24+ frozen doors, True/Red Bull merchandisers, Hobart mixer-grinder and wrappers, Lyons checkouts, NCR POS, Storflex shelving. Preview Nov 11 9AM-12PM; begins closing Nov 11 1PM EST.</t>
         </is>
       </c>
     </row>
@@ -20535,7 +20539,7 @@
       </c>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>Gourmet Deli/Caterer, 100-yr Madison Ave deli liquidation (51 lots: Alto-Shaam ovens, Globe slicer, refrigerated deli cases/merchandisers, walk-in box, Metro racking)</t>
+          <t>Viva Margherita restaurant complete contents (building torn down)</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
@@ -20545,41 +20549,37 @@
       </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Edgewater</t>
         </is>
       </c>
       <c r="E48" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>Live/online auction, prebidding open; 18% BP online</t>
+          <t>Complete contents / make offer</t>
         </is>
       </c>
       <c r="H48" s="15" t="n"/>
       <c r="I48" s="13" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="J48" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-27 02:00 PM ET</t>
-        </is>
-      </c>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="J48" s="13" t="inlineStr"/>
       <c r="K48" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
-        </is>
-      </c>
-      <c r="L48" s="21" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L48" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M48" s="13" t="inlineStr"/>
@@ -20590,7 +20590,7 @@
       </c>
       <c r="O48" s="14" t="inlineStr">
         <is>
-          <t>Live webcast starts Tue Oct 27 2 PM ET; preview Oct 27 11 AM; checkout Wed Oct 28 10-5. Address released before auction. Shipping can be arranged at buyer's cost.</t>
+          <t>Address 163 Old River Road, Edgewater NJ. Building being torn down; complete restaurant contents for sale / make offer.</t>
         </is>
       </c>
     </row>
@@ -20602,17 +20602,17 @@
       </c>
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>Daycare/preschool closing: entire inventory of 4 classrooms (tables, cubbies, indoor playground, toys; $40K invested)</t>
+          <t>Gourmet Deli/Caterer, 100-yr Madison Ave deli liquidation (51 lots: Alto-Shaam ovens, Globe slicer, refrigerated deli cases/merchandisers, walk-in box, Metro racking)</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
         <is>
-          <t>business closing</t>
+          <t>restaurant closing</t>
         </is>
       </c>
       <c r="D49" s="13" t="inlineStr">
         <is>
-          <t>Long Island City</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="E49" s="13" t="inlineStr">
@@ -20621,28 +20621,32 @@
         </is>
       </c>
       <c r="F49" s="13" t="n">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="G49" s="13" t="inlineStr">
         <is>
-          <t>$8,000 all</t>
+          <t>Live/online auction, prebidding open; 18% BP online</t>
         </is>
       </c>
       <c r="H49" s="15" t="n"/>
       <c r="I49" s="13" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="J49" s="13" t="inlineStr"/>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J49" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-27 02:00 PM ET</t>
+        </is>
+      </c>
       <c r="K49" s="13" t="inlineStr">
         <is>
-          <t>Craigslist (by owner)</t>
-        </is>
-      </c>
-      <c r="L49" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
+        </is>
+      </c>
+      <c r="L49" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M49" s="13" t="inlineStr"/>
@@ -20653,7 +20657,7 @@
       </c>
       <c r="O49" s="14" t="inlineStr">
         <is>
-          <t>Off-category FYI; bulky, needs a truck.</t>
+          <t>Live webcast starts Tue Oct 27 2 PM ET; preview Oct 27 11 AM; checkout Wed Oct 28 10-5. Address released before auction. Shipping can be arranged at buyer's cost.</t>
         </is>
       </c>
     </row>
@@ -20665,17 +20669,17 @@
       </c>
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>Kitchen store closing: sinks, faucets, hoods, vanities, counters, office stuff (mostly new in box)</t>
+          <t>Daycare/preschool closing: entire inventory of 4 classrooms (tables, cubbies, indoor playground, toys; $40K invested)</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>business closing</t>
         </is>
       </c>
       <c r="D50" s="13" t="inlineStr">
         <is>
-          <t>Brooklyn</t>
+          <t>Long Island City</t>
         </is>
       </c>
       <c r="E50" s="13" t="inlineStr">
@@ -20684,11 +20688,11 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>$8,000 all</t>
         </is>
       </c>
       <c r="H50" s="15" t="n"/>
@@ -20716,7 +20720,7 @@
       </c>
       <c r="O50" s="14" t="inlineStr">
         <is>
-          <t>Sheepshead Bay. Mostly new-in-box kitchen/bath fixtures; delivery available for large purchases. No prices posted.</t>
+          <t>Off-category FYI; bulky, needs a truck.</t>
         </is>
       </c>
     </row>
@@ -20728,17 +20732,17 @@
       </c>
       <c r="B51" s="14" t="inlineStr">
         <is>
-          <t>Flooring company closed – pro tool package</t>
+          <t>Kitchen store closing: sinks, faucets, hoods, vanities, counters, office stuff (mostly new in box)</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
-          <t>tools liquidation</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D51" s="13" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Brooklyn</t>
         </is>
       </c>
       <c r="E51" s="13" t="inlineStr">
@@ -20747,23 +20751,23 @@
         </is>
       </c>
       <c r="F51" s="13" t="n">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="G51" s="13" t="inlineStr">
         <is>
-          <t>$1,000</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H51" s="15" t="n"/>
       <c r="I51" s="13" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J51" s="13" t="inlineStr"/>
       <c r="K51" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>Craigslist (by owner)</t>
         </is>
       </c>
       <c r="L51" s="13" t="inlineStr">
@@ -20779,7 +20783,7 @@
       </c>
       <c r="O51" s="14" t="inlineStr">
         <is>
-          <t>Flooring/construction company closed; pro tool package $1,000.</t>
+          <t>Sheepshead Bay. Mostly new-in-box kitchen/bath fixtures; delivery available for large purchases. No prices posted.</t>
         </is>
       </c>
     </row>
@@ -20791,12 +20795,12 @@
       </c>
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>New-in-box commercial refrigeration lot – 10 Beverage-Air &amp; Perlick units (bar never opened)</t>
+          <t>Flooring company closed – pro tool package</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>commercial refrigeration lot</t>
+          <t>tools liquidation</t>
         </is>
       </c>
       <c r="D52" s="13" t="inlineStr">
@@ -20814,13 +20818,13 @@
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>$27,500 all 10 (or per unit $2,800–$4,150)</t>
+          <t>$1,000</t>
         </is>
       </c>
       <c r="H52" s="15" t="n"/>
       <c r="I52" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="J52" s="13" t="inlineStr"/>
@@ -20842,7 +20846,7 @@
       </c>
       <c r="O52" s="14" t="inlineStr">
         <is>
-          <t>Financial District. Never installed, factory packaging: 2 Beverage-Air HBF23HC-1-HS reach-in freezers ($4,150 ea), 3 HBR23HC-1-HS reach-in fridges ($3,550 ea), 1 UCR48AHC 48" undercounter ($2,800), 3 Perlick HC24FS4 glass frosters + 1 HC24RS4 beverage fridge ($2,850 ea). Seller says full retail $47,463 (about 42% off as a bundle). Updated Oct 14.</t>
+          <t>Flooring/construction company closed; pro tool package $1,000.</t>
         </is>
       </c>
     </row>
@@ -20854,46 +20858,42 @@
       </c>
       <c r="B53" s="14" t="inlineStr">
         <is>
-          <t>Corporate caterer – Alto-Shaam, new boxed Avantco rice cookers &amp; Cadco oven, Perlick, MerryChef</t>
+          <t>New-in-box commercial refrigeration lot – 10 Beverage-Air &amp; Perlick units (bar never opened)</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>commercial refrigeration lot</t>
         </is>
       </c>
       <c r="D53" s="13" t="inlineStr">
         <is>
-          <t>Jersey City</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="E53" s="13" t="inlineStr">
         <is>
-          <t>NJ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F53" s="13" t="n">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G53" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>$27,500 all 10 (or per unit $2,800–$4,150)</t>
         </is>
       </c>
       <c r="H53" s="15" t="n"/>
       <c r="I53" s="13" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="J53" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-05 07:00 PM ET</t>
-        </is>
-      </c>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="J53" s="13" t="inlineStr"/>
       <c r="K53" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L53" s="13" t="inlineStr">
@@ -20909,7 +20909,7 @@
       </c>
       <c r="O53" s="14" t="inlineStr">
         <is>
-          <t>Thu Oct 22 2 PM. [auto-removed 2026-10-22: closing date passed] | Rescheduled: live &amp; online Nov 5 (preview 11 AM, bidding closes 7 PM ET), 19 lots.</t>
+          <t>Financial District. Never installed, factory packaging: 2 Beverage-Air HBF23HC-1-HS reach-in freezers ($4,150 ea), 3 HBR23HC-1-HS reach-in fridges ($3,550 ea), 1 UCR48AHC 48" undercounter ($2,800), 3 Perlick HC24FS4 glass frosters + 1 HC24RS4 beverage fridge ($2,850 ea). Seller says full retail $47,463 (about 42% off as a bundle). Updated Oct 14.</t>
         </is>
       </c>
     </row>
@@ -20921,12 +20921,12 @@
       </c>
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>Lighting store closing – lease ended, up to 70% off showroom</t>
+          <t>Corporate caterer – Alto-Shaam, new boxed Avantco rice cookers &amp; Cadco oven, Perlick, MerryChef</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D54" s="13" t="inlineStr">
@@ -20944,19 +20944,23 @@
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>up to 70% off</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H54" s="15" t="n"/>
       <c r="I54" s="13" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="J54" s="13" t="inlineStr"/>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="J54" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-05 07:00 PM ET</t>
+        </is>
+      </c>
       <c r="K54" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
       <c r="L54" s="13" t="inlineStr">
@@ -20972,7 +20976,7 @@
       </c>
       <c r="O54" s="14" t="inlineStr">
         <is>
-          <t>Lighting store closing, lease ended. Showroom inventory up to 70% off.</t>
+          <t>Thu Oct 22 2 PM. [auto-removed 2026-10-22: closing date passed] | Rescheduled: live &amp; online Nov 5 (preview 11 AM, bidding closes 7 PM ET), 19 lots.</t>
         </is>
       </c>
     </row>
@@ -20984,12 +20988,12 @@
       </c>
       <c r="B55" s="14" t="inlineStr">
         <is>
-          <t>Baonanas LLC ABC sale: turnkey ice cream / gelato / dessert shop equipment</t>
+          <t>Lighting store closing – lease ended, up to 70% off showroom</t>
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr">
         <is>
-          <t>restaurant / commercial kitchen contents</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D55" s="13" t="inlineStr">
@@ -21007,15 +21011,19 @@
       </c>
       <c r="G55" s="13" t="inlineStr">
         <is>
-          <t>Accepting offers</t>
+          <t>up to 70% off</t>
         </is>
       </c>
       <c r="H55" s="15" t="n"/>
-      <c r="I55" s="13" t="inlineStr"/>
+      <c r="I55" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
       <c r="J55" s="13" t="inlineStr"/>
       <c r="K55" s="13" t="inlineStr">
         <is>
-          <t>AuctionAdvisors</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L55" s="13" t="inlineStr">
@@ -21031,7 +21039,7 @@
       </c>
       <c r="O55" s="14" t="inlineStr">
         <is>
-          <t>181 Monticello Ave. Assignment for the benefit of creditors. IFI Panorama gelato display cases, refrigerated topping stations, commercial mixers, refrigerators/freezers, stainless worktables, ice machine, POS, smallwares, gelato carts, catering gear, FF&amp;E.</t>
+          <t>Lighting store closing, lease ended. Showroom inventory up to 70% off.</t>
         </is>
       </c>
     </row>
@@ -21043,17 +21051,17 @@
       </c>
       <c r="B56" s="14" t="inlineStr">
         <is>
-          <t>Tools / plumbing / MRO supply inventory – Hilti/DeWalt/Milwaukee, fittings, heat pumps</t>
+          <t>Baonanas LLC ABC sale: turnkey ice cream / gelato / dessert shop equipment</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>restaurant / commercial kitchen contents</t>
         </is>
       </c>
       <c r="D56" s="13" t="inlineStr">
         <is>
-          <t>Riverdale</t>
+          <t>Jersey City</t>
         </is>
       </c>
       <c r="E56" s="13" t="inlineStr">
@@ -21062,23 +21070,19 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Accepting offers</t>
         </is>
       </c>
       <c r="H56" s="15" t="n"/>
       <c r="I56" s="13" t="inlineStr"/>
-      <c r="J56" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-30 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="J56" s="13" t="inlineStr"/>
       <c r="K56" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
+          <t>AuctionAdvisors</t>
         </is>
       </c>
       <c r="L56" s="13" t="inlineStr">
@@ -21094,7 +21098,7 @@
       </c>
       <c r="O56" s="14" t="inlineStr">
         <is>
-          <t>Bulk resale inventory.</t>
+          <t>181 Monticello Ave. Assignment for the benefit of creditors. IFI Panorama gelato display cases, refrigerated topping stations, commercial mixers, refrigerators/freezers, stainless worktables, ice machine, POS, smallwares, gelato carts, catering gear, FF&amp;E.</t>
         </is>
       </c>
     </row>
@@ -21106,12 +21110,12 @@
       </c>
       <c r="B57" s="14" t="inlineStr">
         <is>
-          <t>Ice cream + cookie franchise equipment – Taylor soft-serve, Atosa, Blodgett</t>
+          <t>Tools / plumbing / MRO supply inventory – Hilti/DeWalt/Milwaukee, fittings, heat pumps</t>
         </is>
       </c>
       <c r="C57" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>inventory</t>
         </is>
       </c>
       <c r="D57" s="13" t="inlineStr">
@@ -21136,7 +21140,7 @@
       <c r="I57" s="13" t="inlineStr"/>
       <c r="J57" s="13" t="inlineStr">
         <is>
-          <t>2026-11-05 11:00 AM ET</t>
+          <t>2026-10-30 11:00 AM ET</t>
         </is>
       </c>
       <c r="K57" s="13" t="inlineStr">
@@ -21157,7 +21161,7 @@
       </c>
       <c r="O57" s="14" t="inlineStr">
         <is>
-          <t>Resellable units.</t>
+          <t>Bulk resale inventory.</t>
         </is>
       </c>
     </row>
@@ -21169,17 +21173,17 @@
       </c>
       <c r="B58" s="14" t="inlineStr">
         <is>
-          <t>U.S. Vision court-ordered liquidation: ~70,000 designer eyeglass/sunglass frames + optical/optometry equipment at ~80 former stores + IP</t>
+          <t>Ice cream + cookie franchise equipment – Taylor soft-serve, Atosa, Blodgett</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>court-ordered retail chain liquidation</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D58" s="13" t="inlineStr">
         <is>
-          <t>Montclair</t>
+          <t>Riverdale</t>
         </is>
       </c>
       <c r="E58" s="13" t="inlineStr">
@@ -21188,19 +21192,23 @@
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G58" s="13" t="inlineStr">
         <is>
-          <t>Accepting offers (terms in offering memo, NDA required)</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H58" s="15" t="n"/>
       <c r="I58" s="13" t="inlineStr"/>
-      <c r="J58" s="13" t="inlineStr"/>
+      <c r="J58" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-05 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K58" s="13" t="inlineStr">
         <is>
-          <t>AuctionAdvisors</t>
+          <t>A.J. Willner</t>
         </is>
       </c>
       <c r="L58" s="13" t="inlineStr">
@@ -21216,7 +21224,7 @@
       </c>
       <c r="O58" s="14" t="inlineStr">
         <is>
-          <t>Three-lot sale pursuant to court order; bids accepted for individual lots, combinations, or substantially all assets. Equipment is spread across ~80 former store locations. Not appliance-related; big-ticket bulk inventory play.</t>
+          <t>Resellable units.</t>
         </is>
       </c>
     </row>
@@ -21228,17 +21236,17 @@
       </c>
       <c r="B59" s="14" t="inlineStr">
         <is>
-          <t>Wascomat commercial washers liquidation (22× W105, 6× W185, dryer panels)</t>
+          <t>U.S. Vision court-ordered liquidation: ~70,000 designer eyeglass/sunglass frames + optical/optometry equipment at ~80 former stores + IP</t>
         </is>
       </c>
       <c r="C59" s="13" t="inlineStr">
         <is>
-          <t>commercial laundry</t>
+          <t>court-ordered retail chain liquidation</t>
         </is>
       </c>
       <c r="D59" s="13" t="inlineStr">
         <is>
-          <t>Newark</t>
+          <t>Montclair</t>
         </is>
       </c>
       <c r="E59" s="13" t="inlineStr">
@@ -21247,23 +21255,19 @@
         </is>
       </c>
       <c r="F59" s="13" t="n">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G59" s="13" t="inlineStr">
         <is>
-          <t>$500–$800 each / panels $150</t>
+          <t>Accepting offers (terms in offering memo, NDA required)</t>
         </is>
       </c>
       <c r="H59" s="15" t="n"/>
-      <c r="I59" s="13" t="inlineStr">
-        <is>
-          <t>2026-07-12</t>
-        </is>
-      </c>
+      <c r="I59" s="13" t="inlineStr"/>
       <c r="J59" s="13" t="inlineStr"/>
       <c r="K59" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>AuctionAdvisors</t>
         </is>
       </c>
       <c r="L59" s="13" t="inlineStr">
@@ -21279,7 +21283,7 @@
       </c>
       <c r="O59" s="14" t="inlineStr">
         <is>
-          <t>22× W105 @ $500, 6× W185 @ $800, 20 dryer panels $150. Commercial laundry liquidation.</t>
+          <t>Three-lot sale pursuant to court order; bids accepted for individual lots, combinations, or substantially all assets. Equipment is spread across ~80 former store locations. Not appliance-related; big-ticket bulk inventory play.</t>
         </is>
       </c>
     </row>
@@ -21291,17 +21295,17 @@
       </c>
       <c r="B60" s="14" t="inlineStr">
         <is>
-          <t>Major food-service caterer – new-in-box True reach-ins, Beverage-Air, TurboChef, Resfab ventless fryer</t>
+          <t>Wascomat commercial washers liquidation (22× W105, 6× W185, dryer panels)</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>commercial laundry</t>
         </is>
       </c>
       <c r="D60" s="13" t="inlineStr">
         <is>
-          <t>Parsippany</t>
+          <t>Newark</t>
         </is>
       </c>
       <c r="E60" s="13" t="inlineStr">
@@ -21310,27 +21314,23 @@
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="G60" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>$500–$800 each / panels $150</t>
         </is>
       </c>
       <c r="H60" s="15" t="n"/>
       <c r="I60" s="13" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="J60" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-03 02:00 PM ET</t>
-        </is>
-      </c>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="J60" s="13" t="inlineStr"/>
       <c r="K60" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L60" s="13" t="inlineStr">
@@ -21346,7 +21346,7 @@
       </c>
       <c r="O60" s="14" t="inlineStr">
         <is>
-          <t>Tue Nov 3 2 PM, checkout Nov 4.</t>
+          <t>22× W105 @ $500, 6× W185 @ $800, 20 dryer panels $150. Commercial laundry liquidation.</t>
         </is>
       </c>
     </row>
@@ -21358,17 +21358,17 @@
       </c>
       <c r="B61" s="14" t="inlineStr">
         <is>
-          <t>Business closing – 160 new Carnes exhaust fans</t>
+          <t>Major food-service caterer – new-in-box True reach-ins, Beverage-Air, TurboChef, Resfab ventless fryer</t>
         </is>
       </c>
       <c r="C61" s="13" t="inlineStr">
         <is>
-          <t>HVAC inventory</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D61" s="13" t="inlineStr">
         <is>
-          <t>Kenilworth</t>
+          <t>Parsippany</t>
         </is>
       </c>
       <c r="E61" s="13" t="inlineStr">
@@ -21381,19 +21381,23 @@
       </c>
       <c r="G61" s="13" t="inlineStr">
         <is>
-          <t>$40 each or $5,000 all OBO</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H61" s="15" t="n"/>
       <c r="I61" s="13" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="J61" s="13" t="inlineStr"/>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="J61" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-03 02:00 PM ET</t>
+        </is>
+      </c>
       <c r="K61" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
       <c r="L61" s="13" t="inlineStr">
@@ -21409,7 +21413,7 @@
       </c>
       <c r="O61" s="14" t="inlineStr">
         <is>
-          <t>160 new Carnes 80CFM 1.0 sone exhaust fans. $40 each or $5,000 for all OBO. Business closing HVAC inventory.</t>
+          <t>Tue Nov 3 2 PM, checkout Nov 4.</t>
         </is>
       </c>
     </row>
@@ -21421,12 +21425,12 @@
       </c>
       <c r="B62" s="14" t="inlineStr">
         <is>
-          <t>Air Systems Inc – sheet metal / HVAC fabrication shop liquidation</t>
+          <t>Business closing – 160 new Carnes exhaust fans</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>HVAC shop liquidation</t>
+          <t>HVAC inventory</t>
         </is>
       </c>
       <c r="D62" s="13" t="inlineStr">
@@ -21444,19 +21448,19 @@
       </c>
       <c r="G62" s="13" t="inlineStr">
         <is>
-          <t>Timed online (15% BP)</t>
+          <t>$40 each or $5,000 all OBO</t>
         </is>
       </c>
       <c r="H62" s="15" t="n"/>
-      <c r="I62" s="13" t="inlineStr"/>
-      <c r="J62" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-29 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="I62" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="J62" s="13" t="inlineStr"/>
       <c r="K62" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner Auctions</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L62" s="13" t="inlineStr">
@@ -21472,7 +21476,7 @@
       </c>
       <c r="O62" s="14" t="inlineStr">
         <is>
-          <t>Vicon HVAC plasma; Flagler/Lockformer/Roto-Die/Engel fab; welders; Clark forklift; Genie Superlift; Ridgid/Milwaukee/DeWalt/Bosch/Hilti/Makita tools; AeroVent/Carnes exhaust fans; racking/scaffolding. Preview Oct 28–29 AM; pickup Oct 29 PM–Nov 4. Same town as Carnes fan CL lot.</t>
+          <t>160 new Carnes 80CFM 1.0 sone exhaust fans. $40 each or $5,000 for all OBO. Business closing HVAC inventory.</t>
         </is>
       </c>
     </row>
@@ -21484,17 +21488,17 @@
       </c>
       <c r="B63" s="14" t="inlineStr">
         <is>
-          <t>Former Rush Bowls franchise ABC sale: commercial refrigeration, Vitamix blenders, ice &amp; beverage equipment</t>
+          <t>Air Systems Inc – sheet metal / HVAC fabrication shop liquidation</t>
         </is>
       </c>
       <c r="C63" s="13" t="inlineStr">
         <is>
-          <t>restaurant / commercial kitchen contents</t>
+          <t>HVAC shop liquidation</t>
         </is>
       </c>
       <c r="D63" s="13" t="inlineStr">
         <is>
-          <t>Westfield</t>
+          <t>Kenilworth</t>
         </is>
       </c>
       <c r="E63" s="13" t="inlineStr">
@@ -21503,19 +21507,23 @@
         </is>
       </c>
       <c r="F63" s="13" t="n">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="G63" s="13" t="inlineStr">
         <is>
-          <t>Accepting offers</t>
+          <t>Timed online (15% BP)</t>
         </is>
       </c>
       <c r="H63" s="15" t="n"/>
       <c r="I63" s="13" t="inlineStr"/>
-      <c r="J63" s="13" t="inlineStr"/>
+      <c r="J63" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-29 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K63" s="13" t="inlineStr">
         <is>
-          <t>AuctionAdvisors</t>
+          <t>A.J. Willner Auctions</t>
         </is>
       </c>
       <c r="L63" s="13" t="inlineStr">
@@ -21531,7 +21539,7 @@
       </c>
       <c r="O63" s="14" t="inlineStr">
         <is>
-          <t>27 East Broad St. Assignment for the benefit of creditors of 333 Star Enterprises (d/b/a Rush Bowls). Commercial refrigeration/freezers, Vitamix blenders, stainless workstations/sinks, ice and beverage equipment, POS, shelving. Inspection by contacting the auctioneer.</t>
+          <t>Vicon HVAC plasma; Flagler/Lockformer/Roto-Die/Engel fab; welders; Clark forklift; Genie Superlift; Ridgid/Milwaukee/DeWalt/Bosch/Hilti/Makita tools; AeroVent/Carnes exhaust fans; racking/scaffolding. Preview Oct 28–29 AM; pickup Oct 29 PM–Nov 4. Same town as Carnes fan CL lot.</t>
         </is>
       </c>
     </row>
@@ -21543,17 +21551,17 @@
       </c>
       <c r="B64" s="14" t="inlineStr">
         <is>
-          <t>Bimmer Clinic business liquidation (BMW repair shop): vehicle lifts, forklift, skid steer, refrigerant recovery, shop tools &amp; equipment</t>
+          <t>Former Rush Bowls franchise ABC sale: commercial refrigeration, Vitamix blenders, ice &amp; beverage equipment</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>business liquidation auction</t>
+          <t>restaurant / commercial kitchen contents</t>
         </is>
       </c>
       <c r="D64" s="13" t="inlineStr">
         <is>
-          <t>South Amboy</t>
+          <t>Westfield</t>
         </is>
       </c>
       <c r="E64" s="13" t="inlineStr">
@@ -21562,23 +21570,19 @@
         </is>
       </c>
       <c r="F64" s="13" t="n">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="G64" s="13" t="inlineStr">
         <is>
-          <t>Timed online auction</t>
+          <t>Accepting offers</t>
         </is>
       </c>
       <c r="H64" s="15" t="n"/>
       <c r="I64" s="13" t="inlineStr"/>
-      <c r="J64" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-12 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="J64" s="13" t="inlineStr"/>
       <c r="K64" s="13" t="inlineStr">
         <is>
-          <t>AJ Willner Auctions</t>
+          <t>AuctionAdvisors</t>
         </is>
       </c>
       <c r="L64" s="13" t="inlineStr">
@@ -21594,7 +21598,7 @@
       </c>
       <c r="O64" s="14" t="inlineStr">
         <is>
-          <t>Ends Nov 12 11 AM EST.</t>
+          <t>27 East Broad St. Assignment for the benefit of creditors of 333 Star Enterprises (d/b/a Rush Bowls). Commercial refrigeration/freezers, Vitamix blenders, stainless workstations/sinks, ice and beverage equipment, POS, shelving. Inspection by contacting the auctioneer.</t>
         </is>
       </c>
     </row>
@@ -21606,17 +21610,17 @@
       </c>
       <c r="B65" s="14" t="inlineStr">
         <is>
-          <t>Drywall &amp; Acoustical Contractor 2: Hilti tools, material handling, supplies (Ideal Trading Corp)</t>
+          <t>Bimmer Clinic business liquidation (BMW repair shop): vehicle lifts, forklift, skid steer, refrigerant recovery, shop tools &amp; equipment</t>
         </is>
       </c>
       <c r="C65" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>business liquidation auction</t>
         </is>
       </c>
       <c r="D65" s="13" t="inlineStr">
         <is>
-          <t>Randolph</t>
+          <t>South Amboy</t>
         </is>
       </c>
       <c r="E65" s="13" t="inlineStr">
@@ -21625,28 +21629,28 @@
         </is>
       </c>
       <c r="F65" s="13" t="n">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G65" s="13" t="inlineStr">
         <is>
-          <t>Online auction (HiBid terms)</t>
+          <t>Timed online auction</t>
         </is>
       </c>
       <c r="H65" s="15" t="n"/>
       <c r="I65" s="13" t="inlineStr"/>
       <c r="J65" s="13" t="inlineStr">
         <is>
-          <t>2026-10-28 11:00 AM ET</t>
+          <t>2026-11-12 11:00 AM ET</t>
         </is>
       </c>
       <c r="K65" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Ideal Trading Corp)</t>
-        </is>
-      </c>
-      <c r="L65" s="21" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>AJ Willner Auctions</t>
+        </is>
+      </c>
+      <c r="L65" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M65" s="13" t="inlineStr"/>
@@ -21657,7 +21661,7 @@
       </c>
       <c r="O65" s="14" t="inlineStr">
         <is>
-          <t>Contractor contents; closes Oct 28 11 AM. Hilti tools resell well on eBay.</t>
+          <t>Ends Nov 12 11 AM EST.</t>
         </is>
       </c>
     </row>
@@ -21669,17 +21673,17 @@
       </c>
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>New modular concession kitchens (warehouseman's lien) – 5 units, CaptiveAire hoods, new Ovention/Turbo Air</t>
+          <t>Drywall &amp; Acoustical Contractor 2: Hilti tools, material handling, supplies (Ideal Trading Corp)</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>lien sale</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D66" s="13" t="inlineStr">
         <is>
-          <t>Edison</t>
+          <t>Randolph</t>
         </is>
       </c>
       <c r="E66" s="13" t="inlineStr">
@@ -21688,24 +21692,28 @@
         </is>
       </c>
       <c r="F66" s="13" t="n">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="G66" s="13" t="inlineStr">
         <is>
-          <t>Online auction, $2K load-out fee</t>
+          <t>Online auction (HiBid terms)</t>
         </is>
       </c>
       <c r="H66" s="15" t="n"/>
       <c r="I66" s="13" t="inlineStr"/>
-      <c r="J66" s="13" t="inlineStr"/>
+      <c r="J66" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-28 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K66" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
-        </is>
-      </c>
-      <c r="L66" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>HiBid (Ideal Trading Corp)</t>
+        </is>
+      </c>
+      <c r="L66" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M66" s="13" t="inlineStr"/>
@@ -21716,7 +21724,7 @@
       </c>
       <c r="O66" s="14" t="inlineStr">
         <is>
-          <t>&gt;$100K new. Close date not captured.</t>
+          <t>Contractor contents; closes Oct 28 11 AM. Hilti tools resell well on eBay.</t>
         </is>
       </c>
     </row>
@@ -21728,17 +21736,17 @@
       </c>
       <c r="B67" s="14" t="inlineStr">
         <is>
-          <t>Party City (Ch. 11) store – fixtures + party merchandise inventory</t>
+          <t>New modular concession kitchens (warehouseman's lien) – 5 units, CaptiveAire hoods, new Ovention/Turbo Air</t>
         </is>
       </c>
       <c r="C67" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>lien sale</t>
         </is>
       </c>
       <c r="D67" s="13" t="inlineStr">
         <is>
-          <t>East Brunswick</t>
+          <t>Edison</t>
         </is>
       </c>
       <c r="E67" s="13" t="inlineStr">
@@ -21747,20 +21755,16 @@
         </is>
       </c>
       <c r="F67" s="13" t="n">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="G67" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Online auction, $2K load-out fee</t>
         </is>
       </c>
       <c r="H67" s="15" t="n"/>
       <c r="I67" s="13" t="inlineStr"/>
-      <c r="J67" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-03 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="J67" s="13" t="inlineStr"/>
       <c r="K67" s="13" t="inlineStr">
         <is>
           <t>A.J. Willner</t>
@@ -21779,7 +21783,7 @@
       </c>
       <c r="O67" s="14" t="inlineStr">
         <is>
-          <t>Store inventory.</t>
+          <t>&gt;$100K new. Close date not captured.</t>
         </is>
       </c>
     </row>
@@ -21791,17 +21795,17 @@
       </c>
       <c r="B68" s="14" t="inlineStr">
         <is>
-          <t>Bakery/Cafe Somerville NJ – rack ovens, La Marzocco, food truck (~76 lots)</t>
+          <t>Party City (Ch. 11) store – fixtures + party merchandise inventory</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D68" s="13" t="inlineStr">
         <is>
-          <t>Somerville</t>
+          <t>East Brunswick</t>
         </is>
       </c>
       <c r="E68" s="13" t="inlineStr">
@@ -21810,32 +21814,28 @@
         </is>
       </c>
       <c r="F68" s="13" t="n">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="G68" s="13" t="inlineStr">
         <is>
-          <t>Live webcast + online (18% BP online)</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H68" s="15" t="n"/>
-      <c r="I68" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
+      <c r="I68" s="13" t="inlineStr"/>
       <c r="J68" s="13" t="inlineStr">
         <is>
-          <t>2026-10-26 02:00 PM ET</t>
+          <t>2026-11-03 11:00 AM ET</t>
         </is>
       </c>
       <c r="K68" s="13" t="inlineStr">
         <is>
-          <t>HiBid / Best Buy Auctioneers</t>
-        </is>
-      </c>
-      <c r="L68" s="21" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>A.J. Willner</t>
+        </is>
+      </c>
+      <c r="L68" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M68" s="13" t="inlineStr"/>
@@ -21846,7 +21846,7 @@
       </c>
       <c r="O68" s="14" t="inlineStr">
         <is>
-          <t>Full bakery/cafe commercial kitchen: food truck w/ pizza oven, La Marzocco espresso, Mazzer, Baxter + Empire Logiudice rack ovens, dough depositor, Globe floor mixer, Artic Air / SS refrigeration, fryers, Vitamix, Robot Coupe, display cases, dining furniture. Preview 11 AM sale day; checkout Tue 10/27. | 2026-10-26 8am ET: HiBid shows auction open (absentee bidding), 84 open lots; live webcast starts 2 PM ET today.</t>
+          <t>Store inventory.</t>
         </is>
       </c>
     </row>
@@ -21858,7 +21858,7 @@
       </c>
       <c r="B69" s="14" t="inlineStr">
         <is>
-          <t>Ability to Work kitchen and store – commercial kitchen + store fixtures (~135 lots)</t>
+          <t>Bakery/Cafe Somerville NJ – rack ovens, La Marzocco, food truck (~76 lots)</t>
         </is>
       </c>
       <c r="C69" s="13" t="inlineStr">
@@ -21868,7 +21868,7 @@
       </c>
       <c r="D69" s="13" t="inlineStr">
         <is>
-          <t>Flemington</t>
+          <t>Somerville</t>
         </is>
       </c>
       <c r="E69" s="13" t="inlineStr">
@@ -21877,23 +21877,27 @@
         </is>
       </c>
       <c r="F69" s="13" t="n">
-        <v>237</v>
+        <v>224</v>
       </c>
       <c r="G69" s="13" t="inlineStr">
         <is>
-          <t>Timed online (15% BP)</t>
+          <t>Live webcast + online (18% BP online)</t>
         </is>
       </c>
       <c r="H69" s="15" t="n"/>
-      <c r="I69" s="13" t="inlineStr"/>
+      <c r="I69" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
       <c r="J69" s="13" t="inlineStr">
         <is>
-          <t>2026-10-27 11:02 AM ET</t>
+          <t>2026-10-26 02:00 PM ET</t>
         </is>
       </c>
       <c r="K69" s="13" t="inlineStr">
         <is>
-          <t>HiBid</t>
+          <t>HiBid / Best Buy Auctioneers</t>
         </is>
       </c>
       <c r="L69" s="21" t="inlineStr">
@@ -21909,7 +21913,7 @@
       </c>
       <c r="O69" s="14" t="inlineStr">
         <is>
-          <t>Apprentice/hospitality training cafe-kitchen and store dispersal. Preview 9–11 AM sale day; removal Oct 27 noon–Oct 29.</t>
+          <t>Full bakery/cafe commercial kitchen: food truck w/ pizza oven, La Marzocco espresso, Mazzer, Baxter + Empire Logiudice rack ovens, dough depositor, Globe floor mixer, Artic Air / SS refrigeration, fryers, Vitamix, Robot Coupe, display cases, dining furniture. Preview 11 AM sale day; checkout Tue 10/27. | 2026-10-26 8am ET: HiBid shows auction open (absentee bidding), 84 open lots; live webcast starts 2 PM ET today.</t>
         </is>
       </c>
     </row>
@@ -21921,17 +21925,17 @@
       </c>
       <c r="B70" s="14" t="inlineStr">
         <is>
-          <t>Wren Kitchens showroom closing – JennAir/Café/KitchenAid/GE Profile appliances + display kitchens</t>
+          <t>Ability to Work kitchen and store – commercial kitchen + store fixtures (~135 lots)</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>showroom closing</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D70" s="13" t="inlineStr">
         <is>
-          <t>Lawrenceville</t>
+          <t>Flemington</t>
         </is>
       </c>
       <c r="E70" s="13" t="inlineStr">
@@ -21940,23 +21944,23 @@
         </is>
       </c>
       <c r="F70" s="13" t="n">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="G70" s="13" t="inlineStr">
         <is>
-          <t>Online auction, 18% BP</t>
+          <t>Timed online (15% BP)</t>
         </is>
       </c>
       <c r="H70" s="15" t="n"/>
       <c r="I70" s="13" t="inlineStr"/>
       <c r="J70" s="13" t="inlineStr">
         <is>
-          <t>2026-10-27 09:00 AM ET</t>
+          <t>2026-10-27 11:02 AM ET</t>
         </is>
       </c>
       <c r="K70" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
+          <t>HiBid</t>
         </is>
       </c>
       <c r="L70" s="21" t="inlineStr">
@@ -21972,7 +21976,7 @@
       </c>
       <c r="O70" s="14" t="inlineStr">
         <is>
-          <t>Premium floor-model appliances; lots close from Oct 27 9 AM.</t>
+          <t>Apprentice/hospitality training cafe-kitchen and store dispersal. Preview 9–11 AM sale day; removal Oct 27 noon–Oct 29.</t>
         </is>
       </c>
     </row>
@@ -21984,17 +21988,17 @@
       </c>
       <c r="B71" s="14" t="inlineStr">
         <is>
-          <t>50+ yr antique business liquidation – entire 30x60 warehouse full of antiques, wrought iron, collectibles, furniture, lighting (no reasonable offer refused)</t>
+          <t>Wren Kitchens showroom closing – JennAir/Café/KitchenAid/GE Profile appliances + display kitchens</t>
         </is>
       </c>
       <c r="C71" s="13" t="inlineStr">
         <is>
-          <t>business liquidation</t>
+          <t>showroom closing</t>
         </is>
       </c>
       <c r="D71" s="13" t="inlineStr">
         <is>
-          <t>Pennington</t>
+          <t>Lawrenceville</t>
         </is>
       </c>
       <c r="E71" s="13" t="inlineStr">
@@ -22003,35 +22007,31 @@
         </is>
       </c>
       <c r="F71" s="13" t="n">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="G71" s="13" t="inlineStr">
         <is>
-          <t>Best offer (cash &amp; carry)</t>
+          <t>Online auction, 18% BP</t>
         </is>
       </c>
       <c r="H71" s="15" t="n"/>
-      <c r="I71" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="J71" s="13" t="inlineStr"/>
+      <c r="I71" s="13" t="inlineStr"/>
+      <c r="J71" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-27 09:00 AM ET</t>
+        </is>
+      </c>
       <c r="K71" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
-        </is>
-      </c>
-      <c r="L71" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M71" s="20" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L71" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M71" s="13" t="inlineStr"/>
       <c r="N71" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -22039,7 +22039,7 @@
       </c>
       <c r="O71" s="14" t="inlineStr">
         <is>
-          <t>By appointment; bring truck/flashlight/boxes. Seller reposts the same sale under many CL URLs (e.g. gsHWPrsC9miNrtazkuhXoD, oBMFsC2ADf3YjgMSngPdpy, 15uS5HaHeQBJ2rEBQNFK8n). Not appliances – bulk resale stock.</t>
+          <t>Premium floor-model appliances; lots close from Oct 27 9 AM.</t>
         </is>
       </c>
     </row>
@@ -22051,17 +22051,17 @@
       </c>
       <c r="B72" s="14" t="inlineStr">
         <is>
-          <t>Wren Kitchens showroom closing – GE/Whirlpool/KitchenAid/Café incl. NIB Café range + 35 kitchens</t>
+          <t>50+ yr antique business liquidation – entire 30x60 warehouse full of antiques, wrought iron, collectibles, furniture, lighting (no reasonable offer refused)</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>showroom closing</t>
+          <t>business liquidation</t>
         </is>
       </c>
       <c r="D72" s="13" t="inlineStr">
         <is>
-          <t>Cherry Hill</t>
+          <t>Pennington</t>
         </is>
       </c>
       <c r="E72" s="13" t="inlineStr">
@@ -22070,23 +22070,23 @@
         </is>
       </c>
       <c r="F72" s="13" t="n">
-        <v>266</v>
+        <v>241</v>
       </c>
       <c r="G72" s="13" t="inlineStr">
         <is>
-          <t>Online auction, openers ~$0.50</t>
+          <t>Best offer (cash &amp; carry)</t>
         </is>
       </c>
       <c r="H72" s="15" t="n"/>
-      <c r="I72" s="13" t="inlineStr"/>
-      <c r="J72" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-02 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="I72" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="J72" s="13" t="inlineStr"/>
       <c r="K72" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L72" s="13" t="inlineStr">
@@ -22094,7 +22094,11 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M72" s="13" t="inlineStr"/>
+      <c r="M72" s="20" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
       <c r="N72" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -22102,106 +22106,188 @@
       </c>
       <c r="O72" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Nov 2 11 AM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — NYC / Long Island / NJ</t>
-        </is>
-      </c>
-      <c r="B73" s="17" t="inlineStr">
-        <is>
-          <t>27 item(s)</t>
-        </is>
-      </c>
-      <c r="C73" s="18" t="n"/>
-      <c r="D73" s="18" t="n"/>
-      <c r="E73" s="18" t="n"/>
-      <c r="F73" s="18" t="n"/>
-      <c r="G73" s="18" t="n"/>
-      <c r="H73" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I73" s="18" t="n"/>
-      <c r="J73" s="18" t="n"/>
-      <c r="K73" s="18" t="n"/>
-      <c r="L73" s="18" t="n"/>
-      <c r="M73" s="18" t="n"/>
-      <c r="N73" s="18" t="n"/>
-      <c r="O73" s="18" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="11" t="inlineStr">
-        <is>
-          <t>▸ Eastern PA / Mid-Atlantic  (5)</t>
-        </is>
-      </c>
-      <c r="B74" s="12" t="n"/>
-      <c r="C74" s="12" t="n"/>
-      <c r="D74" s="12" t="n"/>
-      <c r="E74" s="12" t="n"/>
-      <c r="F74" s="12" t="n"/>
-      <c r="G74" s="12" t="n"/>
-      <c r="H74" s="12" t="n"/>
-      <c r="I74" s="12" t="n"/>
-      <c r="J74" s="12" t="n"/>
-      <c r="K74" s="12" t="n"/>
-      <c r="L74" s="12" t="n"/>
-      <c r="M74" s="12" t="n"/>
-      <c r="N74" s="12" t="n"/>
-      <c r="O74" s="12" t="n"/>
+          <t>By appointment; bring truck/flashlight/boxes. Seller reposts the same sale under many CL URLs (e.g. gsHWPrsC9miNrtazkuhXoD, oBMFsC2ADf3YjgMSngPdpy, 15uS5HaHeQBJ2rEBQNFK8n). Not appliances – bulk resale stock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" outlineLevel="1">
+      <c r="A73" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B73" s="14" t="inlineStr">
+        <is>
+          <t>Pete's Famous Bakery equipment auction (Trima K2 bun divider-rounder, Bloemhof dough sheeter, Empire spiral mixer, JAC bread slicer, Groen 60-gal tilting kettle, Hoshizaki, Pitco fryer)</t>
+        </is>
+      </c>
+      <c r="C73" s="13" t="inlineStr">
+        <is>
+          <t>restaurant auction</t>
+        </is>
+      </c>
+      <c r="D73" s="13" t="inlineStr">
+        <is>
+          <t>Ewing</t>
+        </is>
+      </c>
+      <c r="E73" s="13" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="F73" s="13" t="n">
+        <v>244</v>
+      </c>
+      <c r="G73" s="13" t="inlineStr">
+        <is>
+          <t>Online auction, first lot ~$850</t>
+        </is>
+      </c>
+      <c r="H73" s="15" t="n"/>
+      <c r="I73" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="J73" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-08 08:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K73" s="13" t="inlineStr">
+        <is>
+          <t>PCI Auctions</t>
+        </is>
+      </c>
+      <c r="L73" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M73" s="13" t="inlineStr"/>
+      <c r="N73" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O73" s="14" t="inlineStr">
+        <is>
+          <t>Ends Sun Nov 8 8 PM EST. PCI NY/NJ warehouse, 200 Kelsey Ave, Ewing NJ 08638. Preview Nov 5-6; removal Nov 9. Also Hoshizaki pizza prep table + 2-door reach-in. PCI offers shipping. Page doesn't say outright the bakery closed. URL verified live 2026-10-26.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" outlineLevel="1">
+      <c r="A74" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B74" s="14" t="inlineStr">
+        <is>
+          <t>The Mill Restaurant &amp; Cafe equipment auction (dual turbo combi oven, double-deck 6-pie pizza oven, 3-bay pasta cooker, more)</t>
+        </is>
+      </c>
+      <c r="C74" s="13" t="inlineStr">
+        <is>
+          <t>restaurant auction</t>
+        </is>
+      </c>
+      <c r="D74" s="13" t="inlineStr">
+        <is>
+          <t>Ewing</t>
+        </is>
+      </c>
+      <c r="E74" s="13" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="F74" s="13" t="n">
+        <v>244</v>
+      </c>
+      <c r="G74" s="13" t="inlineStr">
+        <is>
+          <t>Online auction, current bids</t>
+        </is>
+      </c>
+      <c r="H74" s="15" t="n"/>
+      <c r="I74" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="J74" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-01 08:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K74" s="13" t="inlineStr">
+        <is>
+          <t>PCI Auctions</t>
+        </is>
+      </c>
+      <c r="L74" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M74" s="13" t="inlineStr"/>
+      <c r="N74" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O74" s="14" t="inlineStr">
+        <is>
+          <t>Ends Sun Nov 1 8 PM EST. PCI NY/NJ warehouse, 200 Kelsey Ave, Ewing NJ 08638. Preview Oct 29-30; removal Nov 2. Full restaurant cooking line. Shipping/delivery available. URL verified live 2026-10-26.</t>
+        </is>
+      </c>
     </row>
     <row r="75" outlineLevel="1">
       <c r="A75" s="13" t="inlineStr">
         <is>
-          <t>Eastern PA / Mid-Atlantic</t>
+          <t>NYC / Long Island / NJ</t>
         </is>
       </c>
       <c r="B75" s="14" t="inlineStr">
         <is>
-          <t>Piscitello's Home Center closing after 68 years: storewide 20% off liquidation (hardware, lumber, doors, windows, kitchen/bath)</t>
+          <t>Wren Kitchens showroom closing – GE/Whirlpool/KitchenAid/Café incl. NIB Café range + 35 kitchens</t>
         </is>
       </c>
       <c r="C75" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>showroom closing</t>
         </is>
       </c>
       <c r="D75" s="13" t="inlineStr">
         <is>
-          <t>Wilson</t>
+          <t>Cherry Hill</t>
         </is>
       </c>
       <c r="E75" s="13" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="F75" s="13" t="n">
-        <v>250</v>
+        <v>266</v>
       </c>
       <c r="G75" s="13" t="inlineStr">
         <is>
-          <t>20% off storewide (all sales final)</t>
+          <t>Online auction, openers ~$0.50</t>
         </is>
       </c>
       <c r="H75" s="15" t="n"/>
-      <c r="I75" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
+      <c r="I75" s="13" t="inlineStr"/>
       <c r="J75" s="13" t="inlineStr">
         <is>
-          <t>2026-10-30 06:00 PM ET</t>
+          <t>2026-11-02 11:00 AM ET</t>
         </is>
       </c>
       <c r="K75" s="13" t="inlineStr">
         <is>
-          <t>LehighValley.com article</t>
+          <t>Grafe Auction</t>
         </is>
       </c>
       <c r="L75" s="13" t="inlineStr">
@@ -22217,139 +22303,57 @@
       </c>
       <c r="O75" s="14" t="inlineStr">
         <is>
-          <t>2300 Wood Ave, Wilson Borough (Easton area). Final day Oct 30. Retail-floor sale, not a bulk lot; ask in person about buying remaining stock outright.</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" outlineLevel="1">
-      <c r="A76" s="13" t="inlineStr">
-        <is>
-          <t>Eastern PA / Mid-Atlantic</t>
-        </is>
-      </c>
-      <c r="B76" s="14" t="inlineStr">
-        <is>
-          <t>Hearing aid manufacturing facility inventory liquidation (shelving, 3D printers/scanners, laser engravers, Porta-Vac, sound booths, office; bulk offer invited)</t>
-        </is>
-      </c>
-      <c r="C76" s="13" t="inlineStr">
-        <is>
-          <t>facility liquidation</t>
-        </is>
-      </c>
-      <c r="D76" s="13" t="inlineStr">
-        <is>
-          <t>Bristol</t>
-        </is>
-      </c>
-      <c r="E76" s="13" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="F76" s="13" t="n">
-        <v>252</v>
-      </c>
-      <c r="G76" s="13" t="inlineStr">
-        <is>
-          <t>Best offer / bulk offer for complete lot</t>
-        </is>
-      </c>
-      <c r="H76" s="15" t="n"/>
-      <c r="I76" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="J76" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-08 05:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K76" s="13" t="inlineStr">
-        <is>
-          <t>Craigslist</t>
-        </is>
-      </c>
-      <c r="L76" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M76" s="13" t="inlineStr"/>
-      <c r="N76" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O76" s="14" t="inlineStr">
-        <is>
-          <t>Sale Nov 6-8 ONLY, 8 AM-5 PM (updated 2026-10-25; was 'daily'). 806 Beaver St near Rt 13. Industrial shelving and lab equipment, not appliances; bulk offer invited. Email to schedule viewing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" outlineLevel="1">
-      <c r="A77" s="13" t="inlineStr">
-        <is>
-          <t>Eastern PA / Mid-Atlantic</t>
-        </is>
-      </c>
-      <c r="B77" s="14" t="inlineStr">
-        <is>
-          <t>NBM Liquidation as-is/damaged appliance &amp; more auction (357 lots)</t>
-        </is>
-      </c>
-      <c r="C77" s="13" t="inlineStr">
-        <is>
-          <t>auction pallet</t>
-        </is>
-      </c>
-      <c r="D77" s="13" t="inlineStr">
-        <is>
-          <t>Scranton</t>
-        </is>
-      </c>
-      <c r="E77" s="13" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="F77" s="13" t="n">
-        <v>255</v>
-      </c>
-      <c r="G77" s="13" t="inlineStr">
-        <is>
-          <t>Online auction</t>
-        </is>
-      </c>
-      <c r="H77" s="15" t="n"/>
-      <c r="I77" s="13" t="inlineStr"/>
-      <c r="J77" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-27 06:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K77" s="13" t="inlineStr">
-        <is>
-          <t>HiBid</t>
-        </is>
-      </c>
-      <c r="L77" s="21" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
-        </is>
-      </c>
-      <c r="M77" s="13" t="inlineStr"/>
-      <c r="N77" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O77" s="14" t="inlineStr">
-        <is>
-          <t>Recurring reseller auction (not a closing): as-is/damaged whole appliances and more. Pickup 733 Davis St Scranton PA. Same seller as the two Wolf range lots wf-229/wf-230.</t>
-        </is>
-      </c>
+          <t>Lots close from Nov 2 11 AM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B76" s="17" t="inlineStr">
+        <is>
+          <t>29 item(s)</t>
+        </is>
+      </c>
+      <c r="C76" s="18" t="n"/>
+      <c r="D76" s="18" t="n"/>
+      <c r="E76" s="18" t="n"/>
+      <c r="F76" s="18" t="n"/>
+      <c r="G76" s="18" t="n"/>
+      <c r="H76" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I76" s="18" t="n"/>
+      <c r="J76" s="18" t="n"/>
+      <c r="K76" s="18" t="n"/>
+      <c r="L76" s="18" t="n"/>
+      <c r="M76" s="18" t="n"/>
+      <c r="N76" s="18" t="n"/>
+      <c r="O76" s="18" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="11" t="inlineStr">
+        <is>
+          <t>▸ Eastern PA / Mid-Atlantic  (5)</t>
+        </is>
+      </c>
+      <c r="B77" s="12" t="n"/>
+      <c r="C77" s="12" t="n"/>
+      <c r="D77" s="12" t="n"/>
+      <c r="E77" s="12" t="n"/>
+      <c r="F77" s="12" t="n"/>
+      <c r="G77" s="12" t="n"/>
+      <c r="H77" s="12" t="n"/>
+      <c r="I77" s="12" t="n"/>
+      <c r="J77" s="12" t="n"/>
+      <c r="K77" s="12" t="n"/>
+      <c r="L77" s="12" t="n"/>
+      <c r="M77" s="12" t="n"/>
+      <c r="N77" s="12" t="n"/>
+      <c r="O77" s="12" t="n"/>
     </row>
     <row r="78" outlineLevel="1">
       <c r="A78" s="13" t="inlineStr">
@@ -22359,7 +22363,7 @@
       </c>
       <c r="B78" s="14" t="inlineStr">
         <is>
-          <t>Limerick Hardware inventory liquidation (Alderfer, online-only)</t>
+          <t>Piscitello's Home Center closing after 68 years: storewide 20% off liquidation (hardware, lumber, doors, windows, kitchen/bath)</t>
         </is>
       </c>
       <c r="C78" s="13" t="inlineStr">
@@ -22369,7 +22373,7 @@
       </c>
       <c r="D78" s="13" t="inlineStr">
         <is>
-          <t>Limerick</t>
+          <t>Wilson</t>
         </is>
       </c>
       <c r="E78" s="13" t="inlineStr">
@@ -22378,27 +22382,27 @@
         </is>
       </c>
       <c r="F78" s="13" t="n">
-        <v>277</v>
+        <v>250</v>
       </c>
       <c r="G78" s="13" t="inlineStr">
         <is>
-          <t>Online auction, no reserve info</t>
+          <t>20% off storewide (all sales final)</t>
         </is>
       </c>
       <c r="H78" s="15" t="n"/>
       <c r="I78" s="13" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="J78" s="13" t="inlineStr">
         <is>
-          <t>2026-11-02 08:00 PM ET</t>
+          <t>2026-10-30 06:00 PM ET</t>
         </is>
       </c>
       <c r="K78" s="13" t="inlineStr">
         <is>
-          <t>Alderfer Auction</t>
+          <t>LehighValley.com article</t>
         </is>
       </c>
       <c r="L78" s="13" t="inlineStr">
@@ -22414,7 +22418,7 @@
       </c>
       <c r="O78" s="14" t="inlineStr">
         <is>
-          <t>Hardware store inventory: Hillman fasteners/cabinets, DeWalt/Paslode tools, plumbing/electrical (Moen, Watts), Traeger/Weber/Broil King grills, Toro TimeCutter zero-turn, Wesco pallet jack, Lozier shelving, checkouts. Preview by appointment Fri Oct 30 1-3PM. Begins closing Nov 2 8PM EST.</t>
+          <t>2300 Wood Ave, Wilson Borough (Easton area). Final day Oct 30. Retail-floor sale, not a bulk lot; ask in person about buying remaining stock outright.</t>
         </is>
       </c>
     </row>
@@ -22426,17 +22430,17 @@
       </c>
       <c r="B79" s="14" t="inlineStr">
         <is>
-          <t>Victorino's Pizzeria + Subway sub shop + brand-new scratch &amp; dent restaurant equipment (Marsal pizza oven, True merchandisers, Vulcan/Migali fryers, Stoelting soft-serve)</t>
+          <t>Hearing aid manufacturing facility inventory liquidation (shelving, 3D printers/scanners, laser engravers, Porta-Vac, sound booths, office; bulk offer invited)</t>
         </is>
       </c>
       <c r="C79" s="13" t="inlineStr">
         <is>
-          <t>restaurant closing</t>
+          <t>facility liquidation</t>
         </is>
       </c>
       <c r="D79" s="13" t="inlineStr">
         <is>
-          <t>Manheim</t>
+          <t>Bristol</t>
         </is>
       </c>
       <c r="E79" s="13" t="inlineStr">
@@ -22445,27 +22449,27 @@
         </is>
       </c>
       <c r="F79" s="13" t="n">
-        <v>320</v>
+        <v>252</v>
       </c>
       <c r="G79" s="13" t="inlineStr">
         <is>
-          <t>Online auction, items being added</t>
+          <t>Best offer / bulk offer for complete lot</t>
         </is>
       </c>
       <c r="H79" s="15" t="n"/>
       <c r="I79" s="13" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="J79" s="13" t="inlineStr">
         <is>
-          <t>2026-11-05 08:00 PM ET</t>
+          <t>2026-11-08 05:00 PM ET</t>
         </is>
       </c>
       <c r="K79" s="13" t="inlineStr">
         <is>
-          <t>PCI Auctions East Coast</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L79" s="13" t="inlineStr">
@@ -22481,107 +22485,193 @@
       </c>
       <c r="O79" s="14" t="inlineStr">
         <is>
-          <t>Ends Thu Nov 5 8 PM EST. PCI East Coast warehouse, 141 W End Dr, Manheim PA. Preview Wed Nov 4 10-2; removal Fri Nov 6 10-4. Shipping/delivery available.</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Eastern PA / Mid-Atlantic</t>
-        </is>
-      </c>
-      <c r="B80" s="17" t="inlineStr">
-        <is>
-          <t>5 item(s)</t>
-        </is>
-      </c>
-      <c r="C80" s="18" t="n"/>
-      <c r="D80" s="18" t="n"/>
-      <c r="E80" s="18" t="n"/>
-      <c r="F80" s="18" t="n"/>
-      <c r="G80" s="18" t="n"/>
-      <c r="H80" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I80" s="18" t="n"/>
-      <c r="J80" s="18" t="n"/>
-      <c r="K80" s="18" t="n"/>
-      <c r="L80" s="18" t="n"/>
-      <c r="M80" s="18" t="n"/>
-      <c r="N80" s="18" t="n"/>
-      <c r="O80" s="18" t="n"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="11" t="inlineStr">
-        <is>
-          <t>▸ Upstate / Western NY  (1)</t>
-        </is>
-      </c>
-      <c r="B81" s="12" t="n"/>
-      <c r="C81" s="12" t="n"/>
-      <c r="D81" s="12" t="n"/>
-      <c r="E81" s="12" t="n"/>
-      <c r="F81" s="12" t="n"/>
-      <c r="G81" s="12" t="n"/>
-      <c r="H81" s="12" t="n"/>
-      <c r="I81" s="12" t="n"/>
-      <c r="J81" s="12" t="n"/>
-      <c r="K81" s="12" t="n"/>
-      <c r="L81" s="12" t="n"/>
-      <c r="M81" s="12" t="n"/>
-      <c r="N81" s="12" t="n"/>
-      <c r="O81" s="12" t="n"/>
+          <t>Sale Nov 6-8 ONLY, 8 AM-5 PM (updated 2026-10-25; was 'daily'). 806 Beaver St near Rt 13. Industrial shelving and lab equipment, not appliances; bulk offer invited. Email to schedule viewing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" outlineLevel="1">
+      <c r="A80" s="13" t="inlineStr">
+        <is>
+          <t>Eastern PA / Mid-Atlantic</t>
+        </is>
+      </c>
+      <c r="B80" s="14" t="inlineStr">
+        <is>
+          <t>NBM Liquidation as-is/damaged appliance &amp; more auction (357 lots)</t>
+        </is>
+      </c>
+      <c r="C80" s="13" t="inlineStr">
+        <is>
+          <t>auction pallet</t>
+        </is>
+      </c>
+      <c r="D80" s="13" t="inlineStr">
+        <is>
+          <t>Scranton</t>
+        </is>
+      </c>
+      <c r="E80" s="13" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="F80" s="13" t="n">
+        <v>255</v>
+      </c>
+      <c r="G80" s="13" t="inlineStr">
+        <is>
+          <t>Online auction</t>
+        </is>
+      </c>
+      <c r="H80" s="15" t="n"/>
+      <c r="I80" s="13" t="inlineStr"/>
+      <c r="J80" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-27 06:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K80" s="13" t="inlineStr">
+        <is>
+          <t>HiBid</t>
+        </is>
+      </c>
+      <c r="L80" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M80" s="13" t="inlineStr"/>
+      <c r="N80" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O80" s="14" t="inlineStr">
+        <is>
+          <t>Recurring reseller auction (not a closing): as-is/damaged whole appliances and more. Pickup 733 Davis St Scranton PA. Same seller as the two Wolf range lots wf-229/wf-230.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" outlineLevel="1">
+      <c r="A81" s="13" t="inlineStr">
+        <is>
+          <t>Eastern PA / Mid-Atlantic</t>
+        </is>
+      </c>
+      <c r="B81" s="14" t="inlineStr">
+        <is>
+          <t>Limerick Hardware inventory liquidation (Alderfer, online-only)</t>
+        </is>
+      </c>
+      <c r="C81" s="13" t="inlineStr">
+        <is>
+          <t>store closing</t>
+        </is>
+      </c>
+      <c r="D81" s="13" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="E81" s="13" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="F81" s="13" t="n">
+        <v>277</v>
+      </c>
+      <c r="G81" s="13" t="inlineStr">
+        <is>
+          <t>Online auction, no reserve info</t>
+        </is>
+      </c>
+      <c r="H81" s="15" t="n"/>
+      <c r="I81" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="J81" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-02 08:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K81" s="13" t="inlineStr">
+        <is>
+          <t>Alderfer Auction</t>
+        </is>
+      </c>
+      <c r="L81" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M81" s="13" t="inlineStr"/>
+      <c r="N81" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O81" s="14" t="inlineStr">
+        <is>
+          <t>Hardware store inventory: Hillman fasteners/cabinets, DeWalt/Paslode tools, plumbing/electrical (Moen, Watts), Traeger/Weber/Broil King grills, Toro TimeCutter zero-turn, Wesco pallet jack, Lozier shelving, checkouts. Preview by appointment Fri Oct 30 1-3PM. Begins closing Nov 2 8PM EST.</t>
+        </is>
+      </c>
     </row>
     <row r="82" outlineLevel="1">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>Upstate / Western NY</t>
+          <t>Eastern PA / Mid-Atlantic</t>
         </is>
       </c>
       <c r="B82" s="14" t="inlineStr">
         <is>
-          <t>Restaurant &amp; fitness equipment</t>
+          <t>Victorino's Pizzeria + Subway sub shop + brand-new scratch &amp; dent restaurant equipment (Marsal pizza oven, True merchandisers, Vulcan/Migali fryers, Stoelting soft-serve)</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>restaurant closing</t>
         </is>
       </c>
       <c r="D82" s="13" t="inlineStr">
         <is>
-          <t>Williamsville</t>
+          <t>Manheim</t>
         </is>
       </c>
       <c r="E82" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="F82" s="13" t="n">
-        <v>408</v>
+        <v>320</v>
       </c>
       <c r="G82" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Online auction, items being added</t>
         </is>
       </c>
       <c r="H82" s="15" t="n"/>
-      <c r="I82" s="13" t="inlineStr"/>
+      <c r="I82" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
       <c r="J82" s="13" t="inlineStr">
         <is>
-          <t>2026-10-26 07:30 PM ET</t>
+          <t>2026-11-05 08:00 PM ET</t>
         </is>
       </c>
       <c r="K82" s="13" t="inlineStr">
         <is>
-          <t>Cash Auctions</t>
-        </is>
-      </c>
-      <c r="L82" s="21" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>PCI Auctions East Coast</t>
+        </is>
+      </c>
+      <c r="L82" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M82" s="13" t="inlineStr"/>
@@ -22592,19 +22682,19 @@
       </c>
       <c r="O82" s="14" t="inlineStr">
         <is>
-          <t>Lots not reviewed.</t>
+          <t>Ends Thu Nov 5 8 PM EST. PCI East Coast warehouse, 141 W End Dr, Manheim PA. Preview Wed Nov 4 10-2; removal Fri Nov 6 10-4. Shipping/delivery available.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="17" t="inlineStr">
         <is>
-          <t>Subtotal — Upstate / Western NY</t>
+          <t>Subtotal — Eastern PA / Mid-Atlantic</t>
         </is>
       </c>
       <c r="B83" s="17" t="inlineStr">
         <is>
-          <t>1 item(s)</t>
+          <t>5 item(s)</t>
         </is>
       </c>
       <c r="C83" s="18" t="n"/>
@@ -22626,7 +22716,7 @@
     <row r="84">
       <c r="A84" s="11" t="inlineStr">
         <is>
-          <t>▸ Virginia  (1)</t>
+          <t>▸ Upstate / Western NY  (1)</t>
         </is>
       </c>
       <c r="B84" s="12" t="n"/>
@@ -22647,52 +22737,52 @@
     <row r="85" outlineLevel="1">
       <c r="A85" s="13" t="inlineStr">
         <is>
-          <t>Virginia</t>
+          <t>Upstate / Western NY</t>
         </is>
       </c>
       <c r="B85" s="14" t="inlineStr">
         <is>
-          <t>Haynes Furniture / The Dump – 12 stores closing (furniture, mattresses)</t>
+          <t>Restaurant &amp; fitness equipment</t>
         </is>
       </c>
       <c r="C85" s="13" t="inlineStr">
         <is>
-          <t>retail GOB</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D85" s="13" t="inlineStr">
         <is>
-          <t>Virginia Beach</t>
+          <t>Williamsville</t>
         </is>
       </c>
       <c r="E85" s="13" t="inlineStr">
         <is>
-          <t>VA</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F85" s="13" t="n">
-        <v>456</v>
+        <v>408</v>
       </c>
       <c r="G85" s="13" t="inlineStr">
         <is>
-          <t>Retail GOB markdowns</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H85" s="15" t="n"/>
-      <c r="I85" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="J85" s="13" t="inlineStr"/>
+      <c r="I85" s="13" t="inlineStr"/>
+      <c r="J85" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-26 07:30 PM ET</t>
+        </is>
+      </c>
       <c r="K85" s="13" t="inlineStr">
         <is>
-          <t>SB360 (PR Newswire)</t>
-        </is>
-      </c>
-      <c r="L85" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>Cash Auctions</t>
+        </is>
+      </c>
+      <c r="L85" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M85" s="13" t="inlineStr"/>
@@ -22703,14 +22793,14 @@
       </c>
       <c r="O85" s="14" t="inlineStr">
         <is>
-          <t>Posted Oct 8. Multi-state (VA/AZ/GA/IL/TX); pinned at Virginia Beach. Home goods only.</t>
+          <t>Lots not reviewed.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="17" t="inlineStr">
         <is>
-          <t>Subtotal — Virginia</t>
+          <t>Subtotal — Upstate / Western NY</t>
         </is>
       </c>
       <c r="B86" s="17" t="inlineStr">
@@ -22737,7 +22827,7 @@
     <row r="87">
       <c r="A87" s="11" t="inlineStr">
         <is>
-          <t>▸ Southeast  (1)</t>
+          <t>▸ Virginia  (1)</t>
         </is>
       </c>
       <c r="B87" s="12" t="n"/>
@@ -22758,52 +22848,52 @@
     <row r="88" outlineLevel="1">
       <c r="A88" s="13" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Virginia</t>
         </is>
       </c>
       <c r="B88" s="14" t="inlineStr">
         <is>
-          <t>Carter Control Systems Inc. bankruptcy Day 2: fabrication equipment + $5MM+ inventory (conveyor systems maker)</t>
+          <t>Haynes Furniture / The Dump – 12 stores closing (furniture, mattresses)</t>
         </is>
       </c>
       <c r="C88" s="13" t="inlineStr">
         <is>
-          <t>bankruptcy auction</t>
+          <t>retail GOB</t>
         </is>
       </c>
       <c r="D88" s="13" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Virginia Beach</t>
         </is>
       </c>
       <c r="E88" s="13" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>VA</t>
         </is>
       </c>
       <c r="F88" s="13" t="n">
-        <v>894</v>
+        <v>456</v>
       </c>
       <c r="G88" s="13" t="inlineStr">
         <is>
-          <t>Timed online auction</t>
+          <t>Retail GOB markdowns</t>
         </is>
       </c>
       <c r="H88" s="15" t="n"/>
-      <c r="I88" s="13" t="inlineStr"/>
-      <c r="J88" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-28 10:00 AM ET</t>
-        </is>
-      </c>
+      <c r="I88" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="J88" s="13" t="inlineStr"/>
       <c r="K88" s="13" t="inlineStr">
         <is>
-          <t>PPL Group</t>
-        </is>
-      </c>
-      <c r="L88" s="21" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>SB360 (PR Newswire)</t>
+        </is>
+      </c>
+      <c r="L88" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M88" s="13" t="inlineStr"/>
@@ -22814,14 +22904,14 @@
       </c>
       <c r="O88" s="14" t="inlineStr">
         <is>
-          <t>Ends Oct 28 10 AM ET; preview Oct 26-27; removal Oct 29-Nov 13.</t>
+          <t>Posted Oct 8. Multi-state (VA/AZ/GA/IL/TX); pinned at Virginia Beach. Home goods only.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="17" t="inlineStr">
         <is>
-          <t>Subtotal — Southeast</t>
+          <t>Subtotal — Virginia</t>
         </is>
       </c>
       <c r="B89" s="17" t="inlineStr">
@@ -22848,7 +22938,7 @@
     <row r="90">
       <c r="A90" s="11" t="inlineStr">
         <is>
-          <t>▸ Midwest  (3)</t>
+          <t>▸ Southeast  (1)</t>
         </is>
       </c>
       <c r="B90" s="12" t="n"/>
@@ -22869,52 +22959,52 @@
     <row r="91" outlineLevel="1">
       <c r="A91" s="13" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="B91" s="14" t="inlineStr">
         <is>
-          <t>Vernon Hardware-Napa inventory liquidation (hardware + NAPA auto parts store closing after 87 yrs): tools, hardware, plumbing, electrical, auto parts</t>
+          <t>Carter Control Systems Inc. bankruptcy Day 2: fabrication equipment + $5MM+ inventory (conveyor systems maker)</t>
         </is>
       </c>
       <c r="C91" s="13" t="inlineStr">
         <is>
-          <t>store closing auction</t>
+          <t>bankruptcy auction</t>
         </is>
       </c>
       <c r="D91" s="13" t="inlineStr">
         <is>
-          <t>Vernon</t>
+          <t>Savannah</t>
         </is>
       </c>
       <c r="E91" s="13" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="F91" s="13" t="n">
-        <v>675</v>
+        <v>894</v>
       </c>
       <c r="G91" s="13" t="inlineStr">
         <is>
-          <t>No-reserve online auction (Xyz Auction Service), BP 10% cash/cert. check, 13% card</t>
+          <t>Timed online auction</t>
         </is>
       </c>
       <c r="H91" s="15" t="n"/>
       <c r="I91" s="13" t="inlineStr"/>
       <c r="J91" s="13" t="inlineStr">
         <is>
-          <t>2026-11-05 07:00 PM ET</t>
+          <t>2026-10-28 10:00 AM ET</t>
         </is>
       </c>
       <c r="K91" s="13" t="inlineStr">
         <is>
-          <t>EstateSales.net</t>
-        </is>
-      </c>
-      <c r="L91" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>PPL Group</t>
+        </is>
+      </c>
+      <c r="L91" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M91" s="13" t="inlineStr"/>
@@ -22925,233 +23015,233 @@
       </c>
       <c r="O91" s="14" t="inlineStr">
         <is>
+          <t>Ends Oct 28 10 AM ET; preview Oct 26-27; removal Oct 29-Nov 13.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Southeast</t>
+        </is>
+      </c>
+      <c r="B92" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C92" s="18" t="n"/>
+      <c r="D92" s="18" t="n"/>
+      <c r="E92" s="18" t="n"/>
+      <c r="F92" s="18" t="n"/>
+      <c r="G92" s="18" t="n"/>
+      <c r="H92" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I92" s="18" t="n"/>
+      <c r="J92" s="18" t="n"/>
+      <c r="K92" s="18" t="n"/>
+      <c r="L92" s="18" t="n"/>
+      <c r="M92" s="18" t="n"/>
+      <c r="N92" s="18" t="n"/>
+      <c r="O92" s="18" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="11" t="inlineStr">
+        <is>
+          <t>▸ Midwest  (3)</t>
+        </is>
+      </c>
+      <c r="B93" s="12" t="n"/>
+      <c r="C93" s="12" t="n"/>
+      <c r="D93" s="12" t="n"/>
+      <c r="E93" s="12" t="n"/>
+      <c r="F93" s="12" t="n"/>
+      <c r="G93" s="12" t="n"/>
+      <c r="H93" s="12" t="n"/>
+      <c r="I93" s="12" t="n"/>
+      <c r="J93" s="12" t="n"/>
+      <c r="K93" s="12" t="n"/>
+      <c r="L93" s="12" t="n"/>
+      <c r="M93" s="12" t="n"/>
+      <c r="N93" s="12" t="n"/>
+      <c r="O93" s="12" t="n"/>
+    </row>
+    <row r="94" outlineLevel="1">
+      <c r="A94" s="13" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="B94" s="14" t="inlineStr">
+        <is>
+          <t>Vernon Hardware-Napa inventory liquidation (hardware + NAPA auto parts store closing after 87 yrs): tools, hardware, plumbing, electrical, auto parts</t>
+        </is>
+      </c>
+      <c r="C94" s="13" t="inlineStr">
+        <is>
+          <t>store closing auction</t>
+        </is>
+      </c>
+      <c r="D94" s="13" t="inlineStr">
+        <is>
+          <t>Vernon</t>
+        </is>
+      </c>
+      <c r="E94" s="13" t="inlineStr">
+        <is>
+          <t>MI</t>
+        </is>
+      </c>
+      <c r="F94" s="13" t="n">
+        <v>675</v>
+      </c>
+      <c r="G94" s="13" t="inlineStr">
+        <is>
+          <t>No-reserve online auction (Xyz Auction Service), BP 10% cash/cert. check, 13% card</t>
+        </is>
+      </c>
+      <c r="H94" s="15" t="n"/>
+      <c r="I94" s="13" t="inlineStr"/>
+      <c r="J94" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-05 07:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K94" s="13" t="inlineStr">
+        <is>
+          <t>EstateSales.net</t>
+        </is>
+      </c>
+      <c r="L94" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M94" s="13" t="inlineStr"/>
+      <c r="N94" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O94" s="14" t="inlineStr">
+        <is>
           <t>Bidding opens Mon Nov 2 7 AM; lots begin closing Thu Nov 5 7 PM (bid on auctioneer's site, (989) 288-4600). Far from MA: only worth it for bulk lots that justify the trip. URL verified live 2026-10-25.</t>
         </is>
       </c>
     </row>
-    <row r="92" outlineLevel="1">
-      <c r="A92" s="13" t="inlineStr">
+    <row r="95" outlineLevel="1">
+      <c r="A95" s="13" t="inlineStr">
         <is>
           <t>Midwest</t>
         </is>
       </c>
-      <c r="B92" s="14" t="inlineStr">
+      <c r="B95" s="14" t="inlineStr">
         <is>
           <t>American Sale – total liquidation, all 7 stores (pools, hot tubs, grills, holiday decor)</t>
         </is>
       </c>
-      <c r="C92" s="13" t="inlineStr">
+      <c r="C95" s="13" t="inlineStr">
         <is>
           <t>retail GOB</t>
         </is>
       </c>
-      <c r="D92" s="13" t="inlineStr">
+      <c r="D95" s="13" t="inlineStr">
         <is>
           <t>Chicagoland</t>
         </is>
       </c>
-      <c r="E92" s="13" t="inlineStr">
+      <c r="E95" s="13" t="inlineStr">
         <is>
           <t>IL</t>
         </is>
       </c>
-      <c r="F92" s="13" t="n">
+      <c r="F95" s="13" t="n">
         <v>876</v>
       </c>
-      <c r="G92" s="13" t="inlineStr">
+      <c r="G95" s="13" t="inlineStr">
         <is>
           <t>Retail GOB, up to 70% off</t>
         </is>
       </c>
-      <c r="H92" s="15" t="n"/>
-      <c r="I92" s="13" t="inlineStr">
+      <c r="H95" s="15" t="n"/>
+      <c r="I95" s="13" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="J92" s="13" t="inlineStr"/>
-      <c r="K92" s="13" t="inlineStr">
+      <c r="J95" s="13" t="inlineStr"/>
+      <c r="K95" s="13" t="inlineStr">
         <is>
           <t>Tiger Group (PR Newswire)</t>
         </is>
       </c>
-      <c r="L92" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M92" s="13" t="inlineStr"/>
-      <c r="N92" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O92" s="14" t="inlineStr">
+      <c r="L95" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M95" s="13" t="inlineStr"/>
+      <c r="N95" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O95" s="14" t="inlineStr">
         <is>
           <t>Posted Oct 15. Watch for a bulk/fixture auction.</t>
         </is>
       </c>
-    </row>
-    <row r="93" outlineLevel="1">
-      <c r="A93" s="13" t="inlineStr">
-        <is>
-          <t>Midwest</t>
-        </is>
-      </c>
-      <c r="B93" s="14" t="inlineStr">
-        <is>
-          <t>Restaurant, Bar &amp; DJ Equipment Liquidation: Alto-Shaam combi, Southbend/Blodgett ovens, True refrigeration, Manitowoc, Hobart saw, DJ/AV gear</t>
-        </is>
-      </c>
-      <c r="C93" s="13" t="inlineStr">
-        <is>
-          <t>restaurant liquidation auction</t>
-        </is>
-      </c>
-      <c r="D93" s="13" t="inlineStr">
-        <is>
-          <t>Austin</t>
-        </is>
-      </c>
-      <c r="E93" s="13" t="inlineStr">
-        <is>
-          <t>MN</t>
-        </is>
-      </c>
-      <c r="F93" s="13" t="n">
-        <v>1124</v>
-      </c>
-      <c r="G93" s="13" t="inlineStr">
-        <is>
-          <t>Timed online auction</t>
-        </is>
-      </c>
-      <c r="H93" s="15" t="n"/>
-      <c r="I93" s="13" t="inlineStr"/>
-      <c r="J93" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26 02:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K93" s="13" t="inlineStr">
-        <is>
-          <t>Grafe Auction</t>
-        </is>
-      </c>
-      <c r="L93" s="21" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
-        </is>
-      </c>
-      <c r="M93" s="13" t="inlineStr"/>
-      <c r="N93" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O93" s="14" t="inlineStr">
-        <is>
-          <t>Begins closing Oct 26 1 PM CDT.</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="17" t="inlineStr">
-        <is>
-          <t>Subtotal — Midwest</t>
-        </is>
-      </c>
-      <c r="B94" s="17" t="inlineStr">
-        <is>
-          <t>3 item(s)</t>
-        </is>
-      </c>
-      <c r="C94" s="18" t="n"/>
-      <c r="D94" s="18" t="n"/>
-      <c r="E94" s="18" t="n"/>
-      <c r="F94" s="18" t="n"/>
-      <c r="G94" s="18" t="n"/>
-      <c r="H94" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I94" s="18" t="n"/>
-      <c r="J94" s="18" t="n"/>
-      <c r="K94" s="18" t="n"/>
-      <c r="L94" s="18" t="n"/>
-      <c r="M94" s="18" t="n"/>
-      <c r="N94" s="18" t="n"/>
-      <c r="O94" s="18" t="n"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="11" t="inlineStr">
-        <is>
-          <t>▸ Texas / South Central  (1)</t>
-        </is>
-      </c>
-      <c r="B95" s="12" t="n"/>
-      <c r="C95" s="12" t="n"/>
-      <c r="D95" s="12" t="n"/>
-      <c r="E95" s="12" t="n"/>
-      <c r="F95" s="12" t="n"/>
-      <c r="G95" s="12" t="n"/>
-      <c r="H95" s="12" t="n"/>
-      <c r="I95" s="12" t="n"/>
-      <c r="J95" s="12" t="n"/>
-      <c r="K95" s="12" t="n"/>
-      <c r="L95" s="12" t="n"/>
-      <c r="M95" s="12" t="n"/>
-      <c r="N95" s="12" t="n"/>
-      <c r="O95" s="12" t="n"/>
     </row>
     <row r="96" outlineLevel="1">
       <c r="A96" s="13" t="inlineStr">
         <is>
-          <t>Texas / South Central</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="B96" s="14" t="inlineStr">
         <is>
-          <t>Southwest beverage distributor surplus – mostly unused: 16 True merchandisers, 75 Bunn brewers, 100+ micro-market kiosks</t>
+          <t>Restaurant, Bar &amp; DJ Equipment Liquidation: Alto-Shaam combi, Southbend/Blodgett ovens, True refrigeration, Manitowoc, Hobart saw, DJ/AV gear</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
         <is>
-          <t>distributor surplus</t>
+          <t>restaurant liquidation auction</t>
         </is>
       </c>
       <c r="D96" s="13" t="inlineStr">
         <is>
-          <t>Mesquite</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E96" s="13" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="F96" s="13" t="n">
-        <v>1547</v>
+        <v>1124</v>
       </c>
       <c r="G96" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Timed online auction</t>
         </is>
       </c>
       <c r="H96" s="15" t="n"/>
       <c r="I96" s="13" t="inlineStr"/>
       <c r="J96" s="13" t="inlineStr">
         <is>
-          <t>2026-11-13 11:00 AM ET</t>
+          <t>2026-10-26 02:00 PM ET</t>
         </is>
       </c>
       <c r="K96" s="13" t="inlineStr">
         <is>
-          <t>Heritage Global Partners</t>
-        </is>
-      </c>
-      <c r="L96" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L96" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M96" s="13" t="inlineStr"/>
@@ -23162,19 +23252,19 @@
       </c>
       <c r="O96" s="14" t="inlineStr">
         <is>
-          <t>Near-new appliances, resell by unit. Nov 13 10 AM CST.</t>
+          <t>Begins closing Oct 26 1 PM CDT.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="17" t="inlineStr">
         <is>
-          <t>Subtotal — Texas / South Central</t>
+          <t>Subtotal — Midwest</t>
         </is>
       </c>
       <c r="B97" s="17" t="inlineStr">
         <is>
-          <t>1 item(s)</t>
+          <t>3 item(s)</t>
         </is>
       </c>
       <c r="C97" s="18" t="n"/>
@@ -23196,7 +23286,7 @@
     <row r="98">
       <c r="A98" s="11" t="inlineStr">
         <is>
-          <t>▸ West / Other  (1)</t>
+          <t>▸ Texas / South Central  (1)</t>
         </is>
       </c>
       <c r="B98" s="12" t="n"/>
@@ -23217,47 +23307,47 @@
     <row r="99" outlineLevel="1">
       <c r="A99" s="13" t="inlineStr">
         <is>
-          <t>West / Other</t>
+          <t>Texas / South Central</t>
         </is>
       </c>
       <c r="B99" s="14" t="inlineStr">
         <is>
-          <t>National salad concept liquidation – full contents of 63 fast-casual restaurants (AZ/TX/OK/NV)</t>
+          <t>Southwest beverage distributor surplus – mostly unused: 16 True merchandisers, 75 Bunn brewers, 100+ micro-market kiosks</t>
         </is>
       </c>
       <c r="C99" s="13" t="inlineStr">
         <is>
-          <t>restaurant chain liquidation</t>
+          <t>distributor surplus</t>
         </is>
       </c>
       <c r="D99" s="13" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Mesquite</t>
         </is>
       </c>
       <c r="E99" s="13" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="F99" s="13" t="n">
-        <v>2307</v>
+        <v>1547</v>
       </c>
       <c r="G99" s="13" t="inlineStr">
         <is>
-          <t>Online auctions, dates TBD</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H99" s="15" t="n"/>
-      <c r="I99" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="J99" s="13" t="inlineStr"/>
+      <c r="I99" s="13" t="inlineStr"/>
+      <c r="J99" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-13 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K99" s="13" t="inlineStr">
         <is>
-          <t>RestaurantEquipment.bid (TAGeX)</t>
+          <t>Heritage Global Partners</t>
         </is>
       </c>
       <c r="L99" s="13" t="inlineStr">
@@ -23273,14 +23363,14 @@
       </c>
       <c r="O99" s="14" t="inlineStr">
         <is>
-          <t>Rolling market-by-market auctions, none live yet (Phoenix metro 30 locations, DFW 14, Tucson 6, Houston 5, plus OK/NV). Pickup on site at each restaurant. Pinned at Phoenix.</t>
+          <t>Near-new appliances, resell by unit. Nov 13 10 AM CST.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="17" t="inlineStr">
         <is>
-          <t>Subtotal — West / Other</t>
+          <t>Subtotal — Texas / South Central</t>
         </is>
       </c>
       <c r="B100" s="17" t="inlineStr">
@@ -23307,7 +23397,7 @@
     <row r="101">
       <c r="A101" s="11" t="inlineStr">
         <is>
-          <t>▸ Unknown location  (1)</t>
+          <t>▸ West / Other  (1)</t>
         </is>
       </c>
       <c r="B101" s="12" t="n"/>
@@ -23328,45 +23418,47 @@
     <row r="102" outlineLevel="1">
       <c r="A102" s="13" t="inlineStr">
         <is>
-          <t>Unknown location</t>
+          <t>West / Other</t>
         </is>
       </c>
       <c r="B102" s="14" t="inlineStr">
         <is>
-          <t>Retail furniture store auction: living room sets, sofas, dining/bedroom sets, recliners, dinettes, chandeliers, lamps, rugs, decor, store fixtures</t>
+          <t>National salad concept liquidation – full contents of 63 fast-casual restaurants (AZ/TX/OK/NV)</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
         <is>
-          <t>store closing auction</t>
+          <t>restaurant chain liquidation</t>
         </is>
       </c>
       <c r="D102" s="13" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="E102" s="13" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F102" s="13" t="n"/>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="F102" s="13" t="n">
+        <v>2307</v>
+      </c>
       <c r="G102" s="13" t="inlineStr">
         <is>
-          <t>Online-only auction (BidSpotter), 18% BP</t>
+          <t>Online auctions, dates TBD</t>
         </is>
       </c>
       <c r="H102" s="15" t="n"/>
-      <c r="I102" s="13" t="inlineStr"/>
-      <c r="J102" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-29 10:00 AM ET</t>
-        </is>
-      </c>
+      <c r="I102" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="J102" s="13" t="inlineStr"/>
       <c r="K102" s="13" t="inlineStr">
         <is>
-          <t>Paul E. Saperstein (PESCO)</t>
+          <t>RestaurantEquipment.bid (TAGeX)</t>
         </is>
       </c>
       <c r="L102" s="13" t="inlineStr">
@@ -23382,14 +23474,14 @@
       </c>
       <c r="O102" s="14" t="inlineStr">
         <is>
-          <t>Location TBD (not yet released; PESCO licensed MA/NH/RI/VT, terms cite MA sales tax). Showroom display items, as-is. Inspection Wed Oct 28 12-6 PM; pickup Oct 30, Oct 31, Nov 2.</t>
+          <t>Rolling market-by-market auctions, none live yet (Phoenix metro 30 locations, DFW 14, Tucson 6, Houston 5, plus OK/NV). Pickup on site at each restaurant. Pinned at Phoenix.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="17" t="inlineStr">
         <is>
-          <t>Subtotal — Unknown location</t>
+          <t>Subtotal — West / Other</t>
         </is>
       </c>
       <c r="B103" s="17" t="inlineStr">
@@ -23413,8 +23505,117 @@
       <c r="N103" s="18" t="n"/>
       <c r="O103" s="18" t="n"/>
     </row>
+    <row r="104">
+      <c r="A104" s="11" t="inlineStr">
+        <is>
+          <t>▸ Unknown location  (1)</t>
+        </is>
+      </c>
+      <c r="B104" s="12" t="n"/>
+      <c r="C104" s="12" t="n"/>
+      <c r="D104" s="12" t="n"/>
+      <c r="E104" s="12" t="n"/>
+      <c r="F104" s="12" t="n"/>
+      <c r="G104" s="12" t="n"/>
+      <c r="H104" s="12" t="n"/>
+      <c r="I104" s="12" t="n"/>
+      <c r="J104" s="12" t="n"/>
+      <c r="K104" s="12" t="n"/>
+      <c r="L104" s="12" t="n"/>
+      <c r="M104" s="12" t="n"/>
+      <c r="N104" s="12" t="n"/>
+      <c r="O104" s="12" t="n"/>
+    </row>
+    <row r="105" outlineLevel="1">
+      <c r="A105" s="13" t="inlineStr">
+        <is>
+          <t>Unknown location</t>
+        </is>
+      </c>
+      <c r="B105" s="14" t="inlineStr">
+        <is>
+          <t>Retail furniture store auction: living room sets, sofas, dining/bedroom sets, recliners, dinettes, chandeliers, lamps, rugs, decor, store fixtures</t>
+        </is>
+      </c>
+      <c r="C105" s="13" t="inlineStr">
+        <is>
+          <t>store closing auction</t>
+        </is>
+      </c>
+      <c r="D105" s="13" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E105" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F105" s="13" t="n"/>
+      <c r="G105" s="13" t="inlineStr">
+        <is>
+          <t>Online-only auction (BidSpotter), 18% BP</t>
+        </is>
+      </c>
+      <c r="H105" s="15" t="n"/>
+      <c r="I105" s="13" t="inlineStr"/>
+      <c r="J105" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K105" s="13" t="inlineStr">
+        <is>
+          <t>Paul E. Saperstein (PESCO)</t>
+        </is>
+      </c>
+      <c r="L105" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M105" s="13" t="inlineStr"/>
+      <c r="N105" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O105" s="14" t="inlineStr">
+        <is>
+          <t>Location TBD (not yet released; PESCO licensed MA/NH/RI/VT, terms cite MA sales tax). Showroom display items, as-is. Inspection Wed Oct 28 12-6 PM; pickup Oct 30, Oct 31, Nov 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="17" t="inlineStr">
+        <is>
+          <t>Subtotal — Unknown location</t>
+        </is>
+      </c>
+      <c r="B106" s="17" t="inlineStr">
+        <is>
+          <t>1 item(s)</t>
+        </is>
+      </c>
+      <c r="C106" s="18" t="n"/>
+      <c r="D106" s="18" t="n"/>
+      <c r="E106" s="18" t="n"/>
+      <c r="F106" s="18" t="n"/>
+      <c r="G106" s="18" t="n"/>
+      <c r="H106" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I106" s="18" t="n"/>
+      <c r="J106" s="18" t="n"/>
+      <c r="K106" s="18" t="n"/>
+      <c r="L106" s="18" t="n"/>
+      <c r="M106" s="18" t="n"/>
+      <c r="N106" s="18" t="n"/>
+      <c r="O106" s="18" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O103"/>
+  <autoFilter ref="A1:O106"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId2"/>
@@ -23447,7 +23648,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N43" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N46" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N44" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N47" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N48" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N49" r:id="rId35"/>
@@ -23474,20 +23675,23 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N70" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N71" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N72" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N75" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N76" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N77" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N73" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N74" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N75" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N78" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N79" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N82" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N85" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N88" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N91" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N92" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N93" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N96" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N99" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N102" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N80" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N81" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N82" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N85" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N88" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N91" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N94" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N95" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N96" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N99" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N102" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N105" r:id="rId75"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -23499,7 +23703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O50"/>
+  <dimension ref="A1:O49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -23661,7 +23865,7 @@
       </c>
       <c r="O2" s="14" t="inlineStr">
         <is>
-          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23724,7 +23928,7 @@
       </c>
       <c r="O3" s="14" t="inlineStr">
         <is>
-          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23854,7 +24058,7 @@
       </c>
       <c r="O5" s="14" t="inlineStr">
         <is>
-          <t>Online auction, closes Thu Oct 22 8:37 PM ET. $12.50 high bid (4 bids) as of 2026-10-18. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Online auction, closes Thu Oct 22 8:37 PM ET. $12.50 high bid (4 bids) as of 2026-10-18. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23923,7 +24127,7 @@
       </c>
       <c r="O6" s="14" t="inlineStr">
         <is>
-          <t>Condition: new. FLIP: SPO24TE speed oven NIB, bid $0; flip if under ~$1k; rough resale $1.5-2k | HiBid lot closed/SOLD Oct 25 (high bid $2,000). [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: new. FLIP: SPO24TE speed oven NIB, bid $0; flip if under ~$1k; rough resale $1.5-2k | HiBid lot closed/SOLD Oct 25 (high bid $2,000). [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24266,7 +24470,7 @@
       </c>
       <c r="O11" s="14" t="inlineStr">
         <is>
-          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24335,7 +24539,7 @@
       </c>
       <c r="O12" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. FLIP?: Wolf Gourmet blender, bid $0; resale $150-250 but ~800 mi away | HiBid lot closed 2026-10-24 2026-10-25 [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: used. FLIP?: Wolf Gourmet blender, bid $0; resale $150-250 but ~800 mi away | HiBid lot closed 2026-10-24 2026-10-25 [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24400,7 +24604,7 @@
       </c>
       <c r="O13" s="14" t="inlineStr">
         <is>
-          <t>Condition: unknown. Checked 2026-10-25 ~6pm ET: still open, closes 7:43 PM ET (soft close). | 2026-10-26: HiBid lot closed Oct 25. [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: unknown. Checked 2026-10-25 ~6pm ET: still open, closes 7:43 PM ET (soft close). | 2026-10-26: HiBid lot closed Oct 25. [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24465,7 +24669,7 @@
       </c>
       <c r="O14" s="14" t="inlineStr">
         <is>
-          <t>Condition: unknown. Checked 2026-10-25 ~6pm ET: still open, closes 7:43 PM ET (soft close). | 2026-10-26: HiBid lot closed Oct 25. [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: unknown. Checked 2026-10-25 ~6pm ET: still open, closes 7:43 PM ET (soft close). | 2026-10-26: HiBid lot closed Oct 25. [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24725,7 +24929,7 @@
       </c>
       <c r="O18" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24790,7 +24994,7 @@
       </c>
       <c r="O19" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24855,7 +25059,7 @@
       </c>
       <c r="O20" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24985,7 +25189,7 @@
       </c>
       <c r="O22" s="14" t="inlineStr">
         <is>
-          <t>Lots close in sequence from Oct 21 2 PM ET. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Lots close in sequence from Oct 21 2 PM ET. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25050,7 +25254,7 @@
       </c>
       <c r="O23" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25115,7 +25319,7 @@
       </c>
       <c r="O24" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25178,7 +25382,7 @@
       </c>
       <c r="O25" s="14" t="inlineStr">
         <is>
-          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25241,7 +25445,7 @@
       </c>
       <c r="O26" s="14" t="inlineStr">
         <is>
-          <t>Page conflicts: Oct 21 or 22 9 AM (later date used). Closest find. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Page conflicts: Oct 21 or 22 9 AM (later date used). Closest find. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25304,7 +25508,7 @@
       </c>
       <c r="O27" s="14" t="inlineStr">
         <is>
-          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25367,7 +25571,7 @@
       </c>
       <c r="O28" s="14" t="inlineStr">
         <is>
-          <t>Closes Oct 21 10 or 11 AM (later used). Shippable. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Closes Oct 21 10 or 11 AM (later used). Shippable. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25430,7 +25634,7 @@
       </c>
       <c r="O29" s="14" t="inlineStr">
         <is>
-          <t>Oct 21; start time not captured (placeholder 6 PM). [removed 2026-10-21: live webcast auction held Oct 21; listing page now HTTP 503] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Oct 21; start time not captured (placeholder 6 PM). [removed 2026-10-21: live webcast auction held Oct 21; listing page now HTTP 503] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25493,7 +25697,7 @@
       </c>
       <c r="O30" s="14" t="inlineStr">
         <is>
-          <t>Absolute / no reserve. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Absolute / no reserve. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25556,7 +25760,7 @@
       </c>
       <c r="O31" s="14" t="inlineStr">
         <is>
-          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25619,7 +25823,7 @@
       </c>
       <c r="O32" s="14" t="inlineStr">
         <is>
-          <t>Some kitchen gear only. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Some kitchen gear only. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25682,7 +25886,7 @@
       </c>
       <c r="O33" s="14" t="inlineStr">
         <is>
-          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25745,7 +25949,7 @@
       </c>
       <c r="O34" s="14" t="inlineStr">
         <is>
-          <t>Small lot. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Small lot. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25808,7 +26012,7 @@
       </c>
       <c r="O35" s="14" t="inlineStr">
         <is>
-          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25877,7 +26081,7 @@
       </c>
       <c r="O36" s="14" t="inlineStr">
         <is>
-          <t>About 3 days left as of Oct 18 (~Oct 21; exact time not captured). Pickup Sat Oct 24 12–4 PM by appointment. Used, minor wear. eBay asks $200–420; rough resale $150–250. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>About 3 days left as of Oct 18 (~Oct 21; exact time not captured). Pickup Sat Oct 24 12–4 PM by appointment. Used, minor wear. eBay asks $200–420; rough resale $150–250. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25948,7 +26152,7 @@
       </c>
       <c r="O37" s="14" t="inlineStr">
         <is>
-          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale. [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] | 2026-10-26: verified HiBid auction 785156 ARCHIVED (0 open lots). [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale. [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] | 2026-10-26: verified HiBid auction 785156 ARCHIVED (0 open lots). [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26078,7 +26282,7 @@
       </c>
       <c r="O39" s="14" t="inlineStr">
         <is>
-          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26145,7 +26349,7 @@
       </c>
       <c r="O40" s="14" t="inlineStr">
         <is>
-          <t>Wed Oct 21 4 PM. NYC 10013. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Wed Oct 21 4 PM. NYC 10013. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26212,7 +26416,7 @@
       </c>
       <c r="O41" s="14" t="inlineStr">
         <is>
-          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26279,63 +26483,59 @@
       </c>
       <c r="O42" s="14" t="inlineStr">
         <is>
-          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>CT / Hudson Valley</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>The Outlaw Grill Steakhouse – used restaurant equipment auction (PCI Auctions CT, e.g. Vulcan EV60 Endurance 60" range)</t>
+          <t>Straub's Fine Foods store equipment – bakery, kitchen, meat room, Hussmann refrigeration</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
         <is>
-          <t>restaurant auction</t>
+          <t>grocery/restaurant</t>
         </is>
       </c>
       <c r="D43" s="13" t="inlineStr">
         <is>
-          <t>Stamford</t>
+          <t>St. Louis</t>
         </is>
       </c>
       <c r="E43" s="13" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="F43" s="13" t="n">
-        <v>159</v>
+        <v>1046</v>
       </c>
       <c r="G43" s="13" t="inlineStr">
         <is>
-          <t>Online auction, current bids</t>
+          <t>Online auction (18% BP)</t>
         </is>
       </c>
       <c r="H43" s="15" t="n"/>
-      <c r="I43" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
+      <c r="I43" s="13" t="inlineStr"/>
       <c r="J43" s="13" t="inlineStr">
         <is>
-          <t>2026-10-21 08:30 PM ET</t>
+          <t>2026-10-21 11:00 AM ET</t>
         </is>
       </c>
       <c r="K43" s="13" t="inlineStr">
         <is>
-          <t>PCI Auctions</t>
+          <t>Grafe Auction</t>
         </is>
       </c>
       <c r="L43" s="13" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-10-21 08:30 PM ET)</t>
+          <t>EXPIRED (2026-10-21 11:00 AM ET)</t>
         </is>
       </c>
       <c r="M43" s="13" t="inlineStr"/>
@@ -26346,59 +26546,59 @@
       </c>
       <c r="O43" s="14" t="inlineStr">
         <is>
-          <t>Ends Wed Oct 21 8:30 PM EDT. PCI warehouse, 36 Ludlow St, Stamford CT. Page lists preview Oct 28 and removal Thu Oct 29 11-3 (after close). Shipping/delivery available; payment due on pickup day. Items still being added. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>Western PA / Ohio Valley</t>
         </is>
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>Straub's Fine Foods store equipment – bakery, kitchen, meat room, Hussmann refrigeration</t>
+          <t>Millers Pizza &amp; More – pizza business, commercial kitchen &amp; event space contents (362 lots)</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>grocery/restaurant</t>
+          <t>restaurant / commercial kitchen contents</t>
         </is>
       </c>
       <c r="D44" s="13" t="inlineStr">
         <is>
-          <t>St. Louis</t>
+          <t>Everson</t>
         </is>
       </c>
       <c r="E44" s="13" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>1046</v>
+        <v>478</v>
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>Online auction (18% BP)</t>
+          <t>Online auction, 15% buyer premium</t>
         </is>
       </c>
       <c r="H44" s="15" t="n"/>
       <c r="I44" s="13" t="inlineStr"/>
       <c r="J44" s="13" t="inlineStr">
         <is>
-          <t>2026-10-21 11:00 AM ET</t>
+          <t>2026-10-25 07:00 PM ET</t>
         </is>
       </c>
       <c r="K44" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
+          <t>HiBid (Bid Local LLC)</t>
         </is>
       </c>
       <c r="L44" s="13" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-10-21 11:00 AM ET)</t>
+          <t>EXPIRED (2026-10-25 07:00 PM ET)</t>
         </is>
       </c>
       <c r="M44" s="13" t="inlineStr"/>
@@ -26409,7 +26609,7 @@
       </c>
       <c r="O44" s="14" t="inlineStr">
         <is>
-          <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Property of Millers Pizza and More LLC; online-only, 362 lots, lots begin closing Oct 25 7 PM. Pickup Everson PA by appointment Tue 10/27 and Wed 10/28. Building (4,500 sq ft) to be auctioned separately. [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26421,17 +26621,17 @@
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>Millers Pizza &amp; More – pizza business, commercial kitchen &amp; event space contents (362 lots)</t>
+          <t>Petrunak's Hardware Store liquidation Day 1 (530 lots: doors, hardware, tools, building supplies)</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
         <is>
-          <t>restaurant / commercial kitchen contents</t>
+          <t>store closing auction</t>
         </is>
       </c>
       <c r="D45" s="13" t="inlineStr">
         <is>
-          <t>Everson</t>
+          <t>Windber</t>
         </is>
       </c>
       <c r="E45" s="13" t="inlineStr">
@@ -26440,28 +26640,32 @@
         </is>
       </c>
       <c r="F45" s="13" t="n">
-        <v>478</v>
+        <v>437</v>
       </c>
       <c r="G45" s="13" t="inlineStr">
         <is>
-          <t>Online auction, 15% buyer premium</t>
+          <t>Timed online auction (530 lots)</t>
         </is>
       </c>
       <c r="H45" s="15" t="n"/>
-      <c r="I45" s="13" t="inlineStr"/>
+      <c r="I45" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
       <c r="J45" s="13" t="inlineStr">
         <is>
-          <t>2026-10-25 07:00 PM ET</t>
+          <t>2026-10-21 08:00 PM ET</t>
         </is>
       </c>
       <c r="K45" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Bid Local LLC)</t>
+          <t>Carey Auctions</t>
         </is>
       </c>
       <c r="L45" s="13" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-10-25 07:00 PM ET)</t>
+          <t>EXPIRED (2026-10-21 08:00 PM ET)</t>
         </is>
       </c>
       <c r="M45" s="13" t="inlineStr"/>
@@ -26472,7 +26676,7 @@
       </c>
       <c r="O45" s="14" t="inlineStr">
         <is>
-          <t>Property of Millers Pizza and More LLC; online-only, 362 lots, lots begin closing Oct 25 7 PM. Pickup Everson PA by appointment Tue 10/27 and Wed 10/28. Building (4,500 sq ft) to be auctioned separately. [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Ends Oct 21 7 PM CDT (8 PM ET). 1500 Somerset Ave, Windber PA. Pickups Oct 24-28. Hardware store, not appliance parts. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26484,7 +26688,7 @@
       </c>
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>Petrunak's Hardware Store liquidation Day 1 (530 lots: doors, hardware, tools, building supplies)</t>
+          <t>Petrunak's Hardware Store liquidation Day 2 (433 lots)</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
@@ -26507,7 +26711,7 @@
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>Timed online auction (530 lots)</t>
+          <t>Timed online auction (433 lots)</t>
         </is>
       </c>
       <c r="H46" s="15" t="n"/>
@@ -26518,7 +26722,7 @@
       </c>
       <c r="J46" s="13" t="inlineStr">
         <is>
-          <t>2026-10-21 08:00 PM ET</t>
+          <t>2026-10-22 08:00 PM ET</t>
         </is>
       </c>
       <c r="K46" s="13" t="inlineStr">
@@ -26528,7 +26732,7 @@
       </c>
       <c r="L46" s="13" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-10-21 08:00 PM ET)</t>
+          <t>EXPIRED (2026-10-22 08:00 PM ET)</t>
         </is>
       </c>
       <c r="M46" s="13" t="inlineStr"/>
@@ -26539,63 +26743,59 @@
       </c>
       <c r="O46" s="14" t="inlineStr">
         <is>
-          <t>Ends Oct 21 7 PM CDT (8 PM ET). 1500 Somerset Ave, Windber PA. Pickups Oct 24-28. Hardware store, not appliance parts. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Ends Oct 22 7 PM CDT (8 PM ET). Same store as Day 1; pickups Oct 24-28. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>Western PA / Ohio Valley</t>
+          <t>CT / Hudson Valley</t>
         </is>
       </c>
       <c r="B47" s="14" t="inlineStr">
         <is>
-          <t>Petrunak's Hardware Store liquidation Day 2 (433 lots)</t>
+          <t>Consignment shop remaining inventory, bulk buyer wanted</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
         <is>
-          <t>store closing auction</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>Windber</t>
+          <t>Nyack</t>
         </is>
       </c>
       <c r="E47" s="13" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F47" s="13" t="n">
-        <v>437</v>
+        <v>175</v>
       </c>
       <c r="G47" s="13" t="inlineStr">
         <is>
-          <t>Timed online auction (433 lots)</t>
+          <t>Best offer</t>
         </is>
       </c>
       <c r="H47" s="15" t="n"/>
       <c r="I47" s="13" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="J47" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-22 08:00 PM ET</t>
-        </is>
-      </c>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="J47" s="13" t="inlineStr"/>
       <c r="K47" s="13" t="inlineStr">
         <is>
-          <t>Carey Auctions</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L47" s="13" t="inlineStr">
         <is>
-          <t>EXPIRED (2026-10-22 08:00 PM ET)</t>
+          <t>REMOVED</t>
         </is>
       </c>
       <c r="M47" s="13" t="inlineStr"/>
@@ -26606,29 +26806,29 @@
       </c>
       <c r="O47" s="14" t="inlineStr">
         <is>
-          <t>Ends Oct 22 7 PM CDT (8 PM ET). Same store as Day 1; pickups Oct 24-28. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Assorted secondhand consignment merchandise; one buyer preferred for most/all; pricing negotiable; buyer arranges pickup. [Removed 2026-10-23: CL post flagged for removal]</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>CT / Hudson Valley</t>
+          <t>NYC / Long Island / NJ</t>
         </is>
       </c>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>Consignment shop remaining inventory, bulk buyer wanted</t>
+          <t>Wolf MDD24TE/S/TH 24in E Series drop-down door microwave (2018)</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>built-in microwave</t>
         </is>
       </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>Nyack</t>
+          <t>Astoria (Queens)</t>
         </is>
       </c>
       <c r="E48" s="13" t="inlineStr">
@@ -26637,17 +26837,19 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>175</v>
+        <v>186</v>
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>Best offer</t>
-        </is>
-      </c>
-      <c r="H48" s="15" t="n"/>
+          <t>$375</t>
+        </is>
+      </c>
+      <c r="H48" s="15" t="n">
+        <v>375</v>
+      </c>
       <c r="I48" s="13" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="J48" s="13" t="inlineStr"/>
@@ -26661,7 +26863,11 @@
           <t>REMOVED</t>
         </is>
       </c>
-      <c r="M48" s="13" t="inlineStr"/>
+      <c r="M48" s="20" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
       <c r="N48" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -26669,68 +26875,66 @@
       </c>
       <c r="O48" s="14" t="inlineStr">
         <is>
-          <t>Assorted secondhand consignment merchandise; one buyer preferred for most/all; pricing negotiable; buyer arranges pickup. [Removed 2026-10-23: CL post flagged for removal]</t>
+          <t>Storage-unit clearance, must go by Oct 31; says working (display lit, heating). Built-in, matches E Series ovens. Seller also has Miele G6785 SCVi panel-ready dishwasher; both for $595. Cash/Zelle at pickup. | CL posting deleted by author (HTTP 410) 2026-10-24 evening</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>NYC / Long Island / NJ</t>
+          <t>Central / Western MA</t>
         </is>
       </c>
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>Wolf MDD24TE/S/TH 24in E Series drop-down door microwave (2018)</t>
+          <t>Race Brook Lodge business-closing tag sale (30-yr inn/event venue contents)</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
         <is>
-          <t>built-in microwave</t>
+          <t>business closing tag sale</t>
         </is>
       </c>
       <c r="D49" s="13" t="inlineStr">
         <is>
-          <t>Astoria (Queens)</t>
+          <t>Sheffield</t>
         </is>
       </c>
       <c r="E49" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="F49" s="13" t="n">
-        <v>186</v>
+        <v>130</v>
       </c>
       <c r="G49" s="13" t="inlineStr">
         <is>
-          <t>$375</t>
-        </is>
-      </c>
-      <c r="H49" s="15" t="n">
-        <v>375</v>
-      </c>
+          <t>Tag sale</t>
+        </is>
+      </c>
+      <c r="H49" s="15" t="n"/>
       <c r="I49" s="13" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="J49" s="13" t="inlineStr"/>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="J49" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-25 03:00 PM ET</t>
+        </is>
+      </c>
       <c r="K49" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>EstateSales.net</t>
         </is>
       </c>
       <c r="L49" s="13" t="inlineStr">
         <is>
-          <t>REMOVED</t>
-        </is>
-      </c>
-      <c r="M49" s="20" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
+          <t>EXPIRED (2026-10-25 03:00 PM ET)</t>
+        </is>
+      </c>
+      <c r="M49" s="13" t="inlineStr"/>
       <c r="N49" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -26738,79 +26942,12 @@
       </c>
       <c r="O49" s="14" t="inlineStr">
         <is>
-          <t>Storage-unit clearance, must go by Oct 31; says working (display lit, heating). Built-in, matches E Series ovens. Seller also has Miele G6785 SCVi panel-ready dishwasher; both for $595. Cash/Zelle at pickup. | CL posting deleted by author (HTTP 410) 2026-10-24 evening</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="13" t="inlineStr">
-        <is>
-          <t>Central / Western MA</t>
-        </is>
-      </c>
-      <c r="B50" s="14" t="inlineStr">
-        <is>
-          <t>Race Brook Lodge business-closing tag sale (30-yr inn/event venue contents)</t>
-        </is>
-      </c>
-      <c r="C50" s="13" t="inlineStr">
-        <is>
-          <t>business closing tag sale</t>
-        </is>
-      </c>
-      <c r="D50" s="13" t="inlineStr">
-        <is>
-          <t>Sheffield</t>
-        </is>
-      </c>
-      <c r="E50" s="13" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="F50" s="13" t="n">
-        <v>130</v>
-      </c>
-      <c r="G50" s="13" t="inlineStr">
-        <is>
-          <t>Tag sale</t>
-        </is>
-      </c>
-      <c r="H50" s="15" t="n"/>
-      <c r="I50" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="J50" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-25 03:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K50" s="13" t="inlineStr">
-        <is>
-          <t>EstateSales.net</t>
-        </is>
-      </c>
-      <c r="L50" s="13" t="inlineStr">
-        <is>
-          <t>EXPIRED (2026-10-25 03:00 PM ET)</t>
-        </is>
-      </c>
-      <c r="M50" s="13" t="inlineStr"/>
-      <c r="N50" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O50" s="14" t="inlineStr">
-        <is>
-          <t>864 S Undermountain Rd. Event Barn + Stagecoach Tavern contents, furniture, lamps, rugs, restaurant supplies. Oct 24 10-6 and Oct 25 12-3 only. [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>864 S Undermountain Rd. Event Barn + Stagecoach Tavern contents, furniture, lamps, rugs, restaurant supplies. Oct 24 10-6 and Oct 25 12-3 only. [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O50"/>
+  <autoFilter ref="A1:O49"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
@@ -26860,7 +26997,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N47" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N48" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N50" r:id="rId49"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Lot Recon update 2026-10-26 11am ET: recheck, no changes (309 active)
</commit_message>
<xml_diff>
--- a/lot_recon.xlsx
+++ b/lot_recon.xlsx
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 2026-10-26 10:41 ET</t>
+          <t>Last updated: 2026-10-26 11:01 ET</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13">
@@ -21526,9 +21526,9 @@
           <t>A.J. Willner Auctions</t>
         </is>
       </c>
-      <c r="L63" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+      <c r="L63" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M63" s="13" t="inlineStr"/>
@@ -23865,7 +23865,7 @@
       </c>
       <c r="O2" s="14" t="inlineStr">
         <is>
-          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -23928,7 +23928,7 @@
       </c>
       <c r="O3" s="14" t="inlineStr">
         <is>
-          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24058,7 +24058,7 @@
       </c>
       <c r="O5" s="14" t="inlineStr">
         <is>
-          <t>Online auction, closes Thu Oct 22 8:37 PM ET. $12.50 high bid (4 bids) as of 2026-10-18. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Online auction, closes Thu Oct 22 8:37 PM ET. $12.50 high bid (4 bids) as of 2026-10-18. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24127,7 +24127,7 @@
       </c>
       <c r="O6" s="14" t="inlineStr">
         <is>
-          <t>Condition: new. FLIP: SPO24TE speed oven NIB, bid $0; flip if under ~$1k; rough resale $1.5-2k | HiBid lot closed/SOLD Oct 25 (high bid $2,000). [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: new. FLIP: SPO24TE speed oven NIB, bid $0; flip if under ~$1k; rough resale $1.5-2k | HiBid lot closed/SOLD Oct 25 (high bid $2,000). [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24470,7 +24470,7 @@
       </c>
       <c r="O11" s="14" t="inlineStr">
         <is>
-          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24539,7 +24539,7 @@
       </c>
       <c r="O12" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. FLIP?: Wolf Gourmet blender, bid $0; resale $150-250 but ~800 mi away | HiBid lot closed 2026-10-24 2026-10-25 [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: used. FLIP?: Wolf Gourmet blender, bid $0; resale $150-250 but ~800 mi away | HiBid lot closed 2026-10-24 2026-10-25 [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24604,7 +24604,7 @@
       </c>
       <c r="O13" s="14" t="inlineStr">
         <is>
-          <t>Condition: unknown. Checked 2026-10-25 ~6pm ET: still open, closes 7:43 PM ET (soft close). | 2026-10-26: HiBid lot closed Oct 25. [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: unknown. Checked 2026-10-25 ~6pm ET: still open, closes 7:43 PM ET (soft close). | 2026-10-26: HiBid lot closed Oct 25. [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24669,7 +24669,7 @@
       </c>
       <c r="O14" s="14" t="inlineStr">
         <is>
-          <t>Condition: unknown. Checked 2026-10-25 ~6pm ET: still open, closes 7:43 PM ET (soft close). | 2026-10-26: HiBid lot closed Oct 25. [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: unknown. Checked 2026-10-25 ~6pm ET: still open, closes 7:43 PM ET (soft close). | 2026-10-26: HiBid lot closed Oct 25. [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24929,7 +24929,7 @@
       </c>
       <c r="O18" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24994,7 +24994,7 @@
       </c>
       <c r="O19" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25059,7 +25059,7 @@
       </c>
       <c r="O20" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25189,7 +25189,7 @@
       </c>
       <c r="O22" s="14" t="inlineStr">
         <is>
-          <t>Lots close in sequence from Oct 21 2 PM ET. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Lots close in sequence from Oct 21 2 PM ET. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25254,7 +25254,7 @@
       </c>
       <c r="O23" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25319,7 +25319,7 @@
       </c>
       <c r="O24" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25382,7 +25382,7 @@
       </c>
       <c r="O25" s="14" t="inlineStr">
         <is>
-          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25445,7 +25445,7 @@
       </c>
       <c r="O26" s="14" t="inlineStr">
         <is>
-          <t>Page conflicts: Oct 21 or 22 9 AM (later date used). Closest find. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Page conflicts: Oct 21 or 22 9 AM (later date used). Closest find. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25508,7 +25508,7 @@
       </c>
       <c r="O27" s="14" t="inlineStr">
         <is>
-          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25571,7 +25571,7 @@
       </c>
       <c r="O28" s="14" t="inlineStr">
         <is>
-          <t>Closes Oct 21 10 or 11 AM (later used). Shippable. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Closes Oct 21 10 or 11 AM (later used). Shippable. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25634,7 +25634,7 @@
       </c>
       <c r="O29" s="14" t="inlineStr">
         <is>
-          <t>Oct 21; start time not captured (placeholder 6 PM). [removed 2026-10-21: live webcast auction held Oct 21; listing page now HTTP 503] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Oct 21; start time not captured (placeholder 6 PM). [removed 2026-10-21: live webcast auction held Oct 21; listing page now HTTP 503] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25697,7 +25697,7 @@
       </c>
       <c r="O30" s="14" t="inlineStr">
         <is>
-          <t>Absolute / no reserve. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Absolute / no reserve. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25760,7 +25760,7 @@
       </c>
       <c r="O31" s="14" t="inlineStr">
         <is>
-          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25823,7 +25823,7 @@
       </c>
       <c r="O32" s="14" t="inlineStr">
         <is>
-          <t>Some kitchen gear only. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Some kitchen gear only. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25886,7 +25886,7 @@
       </c>
       <c r="O33" s="14" t="inlineStr">
         <is>
-          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25949,7 +25949,7 @@
       </c>
       <c r="O34" s="14" t="inlineStr">
         <is>
-          <t>Small lot. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Small lot. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26012,7 +26012,7 @@
       </c>
       <c r="O35" s="14" t="inlineStr">
         <is>
-          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26081,7 +26081,7 @@
       </c>
       <c r="O36" s="14" t="inlineStr">
         <is>
-          <t>About 3 days left as of Oct 18 (~Oct 21; exact time not captured). Pickup Sat Oct 24 12–4 PM by appointment. Used, minor wear. eBay asks $200–420; rough resale $150–250. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>About 3 days left as of Oct 18 (~Oct 21; exact time not captured). Pickup Sat Oct 24 12–4 PM by appointment. Used, minor wear. eBay asks $200–420; rough resale $150–250. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26152,7 +26152,7 @@
       </c>
       <c r="O37" s="14" t="inlineStr">
         <is>
-          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale. [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] | 2026-10-26: verified HiBid auction 785156 ARCHIVED (0 open lots). [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale. [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] | 2026-10-26: verified HiBid auction 785156 ARCHIVED (0 open lots). [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26282,7 +26282,7 @@
       </c>
       <c r="O39" s="14" t="inlineStr">
         <is>
-          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26349,7 +26349,7 @@
       </c>
       <c r="O40" s="14" t="inlineStr">
         <is>
-          <t>Wed Oct 21 4 PM. NYC 10013. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Wed Oct 21 4 PM. NYC 10013. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26416,7 +26416,7 @@
       </c>
       <c r="O41" s="14" t="inlineStr">
         <is>
-          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26483,7 +26483,7 @@
       </c>
       <c r="O42" s="14" t="inlineStr">
         <is>
-          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26546,7 +26546,7 @@
       </c>
       <c r="O43" s="14" t="inlineStr">
         <is>
-          <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26609,7 +26609,7 @@
       </c>
       <c r="O44" s="14" t="inlineStr">
         <is>
-          <t>Property of Millers Pizza and More LLC; online-only, 362 lots, lots begin closing Oct 25 7 PM. Pickup Everson PA by appointment Tue 10/27 and Wed 10/28. Building (4,500 sq ft) to be auctioned separately. [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Property of Millers Pizza and More LLC; online-only, 362 lots, lots begin closing Oct 25 7 PM. Pickup Everson PA by appointment Tue 10/27 and Wed 10/28. Building (4,500 sq ft) to be auctioned separately. [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26676,7 +26676,7 @@
       </c>
       <c r="O45" s="14" t="inlineStr">
         <is>
-          <t>Ends Oct 21 7 PM CDT (8 PM ET). 1500 Somerset Ave, Windber PA. Pickups Oct 24-28. Hardware store, not appliance parts. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Ends Oct 21 7 PM CDT (8 PM ET). 1500 Somerset Ave, Windber PA. Pickups Oct 24-28. Hardware store, not appliance parts. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26743,7 +26743,7 @@
       </c>
       <c r="O46" s="14" t="inlineStr">
         <is>
-          <t>Ends Oct 22 7 PM CDT (8 PM ET). Same store as Day 1; pickups Oct 24-28. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Ends Oct 22 7 PM CDT (8 PM ET). Same store as Day 1; pickups Oct 24-28. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26942,7 +26942,7 @@
       </c>
       <c r="O49" s="14" t="inlineStr">
         <is>
-          <t>864 S Undermountain Rd. Event Barn + Stagecoach Tavern contents, furniture, lamps, rugs, restaurant supplies. Oct 24 10-6 and Oct 25 12-3 only. [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>864 S Undermountain Rd. Event Barn + Stagecoach Tavern contents, furniture, lamps, rugs, restaurant supplies. Oct 24 10-6 and Oct 25 12-3 only. [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lot Recon update 2026-10-26 2pm ET: recheck, no changes (312 active)
</commit_message>
<xml_diff>
--- a/lot_recon.xlsx
+++ b/lot_recon.xlsx
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 2026-10-26 13:40 ET</t>
+          <t>Last updated: 2026-10-26 13:57 ET</t>
         </is>
       </c>
     </row>
@@ -24019,7 +24019,7 @@
       </c>
       <c r="O2" s="14" t="inlineStr">
         <is>
-          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Integrity Auction House. Internet bidding closes Mon Oct 19 9:18 PM ET. $50 high bid (1 bid) as of 2026-10-18. [Closed Oct 19; HiBid price realized $50.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24082,7 +24082,7 @@
       </c>
       <c r="O3" s="14" t="inlineStr">
         <is>
-          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Live auction Mon Oct 19 4 PM, 3457 Wilmington Rd. Few bulk parts. [Live auction held Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24212,7 +24212,7 @@
       </c>
       <c r="O5" s="14" t="inlineStr">
         <is>
-          <t>Online auction, closes Thu Oct 22 8:37 PM ET. $12.50 high bid (4 bids) as of 2026-10-18. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Online auction, closes Thu Oct 22 8:37 PM ET. $12.50 high bid (4 bids) as of 2026-10-18. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24281,7 +24281,7 @@
       </c>
       <c r="O6" s="14" t="inlineStr">
         <is>
-          <t>Condition: new. FLIP: SPO24TE speed oven NIB, bid $0; flip if under ~$1k; rough resale $1.5-2k | HiBid lot closed/SOLD Oct 25 (high bid $2,000). [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: new. FLIP: SPO24TE speed oven NIB, bid $0; flip if under ~$1k; rough resale $1.5-2k | HiBid lot closed/SOLD Oct 25 (high bid $2,000). [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24624,7 +24624,7 @@
       </c>
       <c r="O11" s="14" t="inlineStr">
         <is>
-          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: Pre-Owned. FLIP: SO36U/S tested, auction $99/0 bids, pickup only; rough resale $600-1k (eBay card shows no city; pickup distance in source.) Ends Oct 18 ~2:19 PM per eBay card (time zone uncertain; could be earlier). [auto-removed 2026-10-18: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24693,7 +24693,7 @@
       </c>
       <c r="O12" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. FLIP?: Wolf Gourmet blender, bid $0; resale $150-250 but ~800 mi away | HiBid lot closed 2026-10-24 2026-10-25 [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: used. FLIP?: Wolf Gourmet blender, bid $0; resale $150-250 but ~800 mi away | HiBid lot closed 2026-10-24 2026-10-25 [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24758,7 +24758,7 @@
       </c>
       <c r="O13" s="14" t="inlineStr">
         <is>
-          <t>Condition: unknown. Checked 2026-10-25 ~6pm ET: still open, closes 7:43 PM ET (soft close). | 2026-10-26: HiBid lot closed Oct 25. [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: unknown. Checked 2026-10-25 ~6pm ET: still open, closes 7:43 PM ET (soft close). | 2026-10-26: HiBid lot closed Oct 25. [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -24823,7 +24823,7 @@
       </c>
       <c r="O14" s="14" t="inlineStr">
         <is>
-          <t>Condition: unknown. Checked 2026-10-25 ~6pm ET: still open, closes 7:43 PM ET (soft close). | 2026-10-26: HiBid lot closed Oct 25. [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: unknown. Checked 2026-10-25 ~6pm ET: still open, closes 7:43 PM ET (soft close). | 2026-10-26: HiBid lot closed Oct 25. [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25083,7 +25083,7 @@
       </c>
       <c r="O18" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25148,7 +25148,7 @@
       </c>
       <c r="O19" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25213,7 +25213,7 @@
       </c>
       <c r="O20" s="14" t="inlineStr">
         <is>
-          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Condition: used. commercial Wolf (not Sub-Zero Wolf) HiBid lot closed/sold ~$37.50 on 2026-10-18. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25343,7 +25343,7 @@
       </c>
       <c r="O22" s="14" t="inlineStr">
         <is>
-          <t>Lots close in sequence from Oct 21 2 PM ET. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Lots close in sequence from Oct 21 2 PM ET. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25408,7 +25408,7 @@
       </c>
       <c r="O23" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Lots close from Oct 19 2 PM ET. [HiBid catalog closed 2 PM ET Oct 19.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25473,7 +25473,7 @@
       </c>
       <c r="O24" s="14" t="inlineStr">
         <is>
-          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Lots close from Oct 20 2 PM ET. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25536,7 +25536,7 @@
       </c>
       <c r="O25" s="14" t="inlineStr">
         <is>
-          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Tested and new units. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25599,7 +25599,7 @@
       </c>
       <c r="O26" s="14" t="inlineStr">
         <is>
-          <t>Page conflicts: Oct 21 or 22 9 AM (later date used). Closest find. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Page conflicts: Oct 21 or 22 9 AM (later date used). Closest find. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25662,7 +25662,7 @@
       </c>
       <c r="O27" s="14" t="inlineStr">
         <is>
-          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Pickup Oct 21 only. [Lots began closing 1 PM ET Oct 19; ended.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25725,7 +25725,7 @@
       </c>
       <c r="O28" s="14" t="inlineStr">
         <is>
-          <t>Closes Oct 21 10 or 11 AM (later used). Shippable. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Closes Oct 21 10 or 11 AM (later used). Shippable. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25788,7 +25788,7 @@
       </c>
       <c r="O29" s="14" t="inlineStr">
         <is>
-          <t>Oct 21; start time not captured (placeholder 6 PM). [removed 2026-10-21: live webcast auction held Oct 21; listing page now HTTP 503] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Oct 21; start time not captured (placeholder 6 PM). [removed 2026-10-21: live webcast auction held Oct 21; listing page now HTTP 503] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25851,7 +25851,7 @@
       </c>
       <c r="O30" s="14" t="inlineStr">
         <is>
-          <t>Absolute / no reserve. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Absolute / no reserve. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25914,7 +25914,7 @@
       </c>
       <c r="O31" s="14" t="inlineStr">
         <is>
-          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Close Oct 18 or 19 6 PM (later used). [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -25977,7 +25977,7 @@
       </c>
       <c r="O32" s="14" t="inlineStr">
         <is>
-          <t>Some kitchen gear only. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Some kitchen gear only. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26040,7 +26040,7 @@
       </c>
       <c r="O33" s="14" t="inlineStr">
         <is>
-          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>No new out-of-state bidders. Small. [Ended Oct 19 7 PM.] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26103,7 +26103,7 @@
       </c>
       <c r="O34" s="14" t="inlineStr">
         <is>
-          <t>Small lot. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Small lot. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26166,7 +26166,7 @@
       </c>
       <c r="O35" s="14" t="inlineStr">
         <is>
-          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Closes from Oct 20 10 AM CDT. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26235,7 +26235,7 @@
       </c>
       <c r="O36" s="14" t="inlineStr">
         <is>
-          <t>About 3 days left as of Oct 18 (~Oct 21; exact time not captured). Pickup Sat Oct 24 12–4 PM by appointment. Used, minor wear. eBay asks $200–420; rough resale $150–250. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>About 3 days left as of Oct 18 (~Oct 21; exact time not captured). Pickup Sat Oct 24 12–4 PM by appointment. Used, minor wear. eBay asks $200–420; rough resale $150–250. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26306,7 +26306,7 @@
       </c>
       <c r="O37" s="14" t="inlineStr">
         <is>
-          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale. [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] | 2026-10-26: verified HiBid auction 785156 ARCHIVED (0 open lots). [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Sun Oct 25 1 PM (preview 11 AM), checkout Oct 26. Many lots in box. Recurring appliance sale; the Wolf SPO24TE speed oven lot already on the map is likely from this sale. [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] | 2026-10-26: verified HiBid auction 785156 ARCHIVED (0 open lots). [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26436,7 +26436,7 @@
       </c>
       <c r="O39" s="14" t="inlineStr">
         <is>
-          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>"Short notice" auction Mon Oct 19 1 PM. [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26503,7 +26503,7 @@
       </c>
       <c r="O40" s="14" t="inlineStr">
         <is>
-          <t>Wed Oct 21 4 PM. NYC 10013. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Wed Oct 21 4 PM. NYC 10013. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26570,7 +26570,7 @@
       </c>
       <c r="O41" s="14" t="inlineStr">
         <is>
-          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Tue Oct 20 2 PM. No item description on page. [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26637,7 +26637,7 @@
       </c>
       <c r="O42" s="14" t="inlineStr">
         <is>
-          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Mon Oct 19 4 PM. No item description on page. [HiBid shows Bidding Closed, Oct 19 4 PM.] [auto-removed 2026-10-19: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-20: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26700,7 +26700,7 @@
       </c>
       <c r="O43" s="14" t="inlineStr">
         <is>
-          <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Kingshighway store: Revent double-rack oven + proofer, Reed revolving oven, Vulcan convection, Groen kettle, Southbend 6-burner, Pitco fryer, Stero dishwasher, Hobart saw/grinders, Berkel slicers, Hussmann cases + compressor racks, walk-ins, Hoshizaki/Scotsman ice machines, Crown pallet jack. Preview Oct 20 3–6 PM CDT; pickup in St. Louis. [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-21: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26763,7 +26763,7 @@
       </c>
       <c r="O44" s="14" t="inlineStr">
         <is>
-          <t>Property of Millers Pizza and More LLC; online-only, 362 lots, lots begin closing Oct 25 7 PM. Pickup Everson PA by appointment Tue 10/27 and Wed 10/28. Building (4,500 sq ft) to be auctioned separately. [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Property of Millers Pizza and More LLC; online-only, 362 lots, lots begin closing Oct 25 7 PM. Pickup Everson PA by appointment Tue 10/27 and Wed 10/28. Building (4,500 sq ft) to be auctioned separately. [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26830,7 +26830,7 @@
       </c>
       <c r="O45" s="14" t="inlineStr">
         <is>
-          <t>Ends Oct 21 7 PM CDT (8 PM ET). 1500 Somerset Ave, Windber PA. Pickups Oct 24-28. Hardware store, not appliance parts. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Ends Oct 21 7 PM CDT (8 PM ET). 1500 Somerset Ave, Windber PA. Pickups Oct 24-28. Hardware store, not appliance parts. [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-22: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -26897,7 +26897,7 @@
       </c>
       <c r="O46" s="14" t="inlineStr">
         <is>
-          <t>Ends Oct 22 7 PM CDT (8 PM ET). Same store as Day 1; pickups Oct 24-28. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>Ends Oct 22 7 PM CDT (8 PM ET). Same store as Day 1; pickups Oct 24-28. [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-23: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-24: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>
@@ -27096,7 +27096,7 @@
       </c>
       <c r="O49" s="14" t="inlineStr">
         <is>
-          <t>864 S Undermountain Rd. Event Barn + Stagecoach Tavern contents, furniture, lamps, rugs, restaurant supplies. Oct 24 10-6 and Oct 25 12-3 only. [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
+          <t>864 S Undermountain Rd. Event Barn + Stagecoach Tavern contents, furniture, lamps, rugs, restaurant supplies. Oct 24 10-6 and Oct 25 12-3 only. [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-25: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed] [auto-removed 2026-10-26: closing date passed]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lot Recon update 2026-10-26 night Liquidation Scout: add TGI Fridays Westbury NY HiBid auction (bl-100); bl-043 Waltham tools new CL repost h2V6YLfs; restore bl-051 Somerville NJ (HiBid open, closes 7 PM ET) (311 active)
</commit_message>
<xml_diff>
--- a/lot_recon.xlsx
+++ b/lot_recon.xlsx
@@ -20,8 +20,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wolf New'!$A$1:$O$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Wolf Used'!$A$1:$O$185</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Wolf Unclear'!$A$1:$O$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$103</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Business Liquidation'!$A$1:$O$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Removed'!$A$1:$O$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 2026-10-26 17:39 ET</t>
+          <t>Last updated: 2026-10-26 17:46 ET</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Active listings: 309 · Removed: 51</t>
+          <t>Active listings: 311 · Removed: 50</t>
         </is>
       </c>
     </row>
@@ -708,13 +708,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13">
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C13" s="7" t="n">
         <v>1462977.58</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C24" t="n">
         <v>1</v>
@@ -1037,7 +1037,7 @@
         <v>24</v>
       </c>
       <c r="G24" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H24" s="6" t="n">
         <v>461790</v>
@@ -18096,7 +18096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O103"/>
+  <dimension ref="A1:O105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -18466,7 +18466,7 @@
       </c>
       <c r="O6" s="14" t="inlineStr">
         <is>
-          <t>Small off-category FYI; seller says resell individually. Same $250 / 10-tool lot, reposted under new CL URLs repeatedly (latest 2026-10-22 4:24 PM). | CL repost 6Z43nD92 deleted by author 2026-10-24 | Reposted 2026-10-25 11:25 AM (xxm7mDLa), now $225; reactivated. | CL posting deleted 2026-10-25 | Re-verified 2026-10-25 6pm ET: HTTP 410, 'This posting has been deleted by its author'; stays REMOVED. | Reposted 2026-10-25 5:59 PM (iM4jce2X, post id 7989822312), $225 for all 10 tools; verified live 2026-10-26 8am ET (HTTP 200); reactivated.</t>
+          <t>Small off-category FYI; seller says resell individually. Same $250 / 10-tool lot, reposted under new CL URLs repeatedly (latest 2026-10-22 4:24 PM). | CL repost 6Z43nD92 deleted by author 2026-10-24 | Reposted 2026-10-25 11:25 AM (xxm7mDLa), now $225; reactivated. | CL posting deleted 2026-10-25 | Re-verified 2026-10-25 6pm ET: HTTP 410, 'This posting has been deleted by its author'; stays REMOVED. | Reposted 2026-10-25 5:59 PM (iM4jce2X, post id 7989822312), $225 for all 10 tools; verified live 2026-10-26 8am ET (HTTP 200); reactivated. | iM4jce2Xk9HFJAsVZ1CdK3 link now HTTP 410 (deleted). Reposted 2026-10-26 3:03 PM (h2V6YLfs, post id 7990278777), still $225 for 10 tools; verified live 2026-10-26 5:45pm ET (HTTP 200).</t>
         </is>
       </c>
     </row>
@@ -20646,7 +20646,7 @@
     <row r="48">
       <c r="A48" s="11" t="inlineStr">
         <is>
-          <t>▸ NYC / Long Island / NJ  (28)</t>
+          <t>▸ NYC / Long Island / NJ  (30)</t>
         </is>
       </c>
       <c r="B48" s="12" t="n"/>
@@ -20672,17 +20672,17 @@
       </c>
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>Met Foodmarkets turnkey grocery liquidation (Grafe Auction)</t>
+          <t>TGI Fridays Westbury restaurant contents auction (105 lots) – Glastender bar sink/ice-bin stations, RSI stainless table, glycol beer system, furnishings</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D49" s="13" t="inlineStr">
         <is>
-          <t>Bronx</t>
+          <t>Westbury</t>
         </is>
       </c>
       <c r="E49" s="13" t="inlineStr">
@@ -20691,27 +20691,27 @@
         </is>
       </c>
       <c r="F49" s="13" t="n">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="G49" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Timed online auction (HiBid)</t>
         </is>
       </c>
       <c r="H49" s="15" t="n"/>
       <c r="I49" s="13" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="J49" s="13" t="inlineStr">
         <is>
-          <t>2026-11-11 01:00 PM ET</t>
+          <t>2026-11-10 11:00 AM ET</t>
         </is>
       </c>
       <c r="K49" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
+          <t>HiBid / Tri State Auctions</t>
         </is>
       </c>
       <c r="L49" s="13" t="inlineStr">
@@ -20727,7 +20727,7 @@
       </c>
       <c r="O49" s="14" t="inlineStr">
         <is>
-          <t>2 Hussmann compressor racks, 3-room Amerikooler walk-in cooler/freezer, Hussmann/Hill Phoenix remote cases, 24+ frozen doors, True/Red Bull merchandisers, Hobart mixer-grinder and wrappers, Lyons checkouts, NCR POS, Storflex shelving. Preview Nov 11 9AM-12PM; begins closing Nov 11 1PM EST.</t>
+          <t>829 Merrick Ave, Westbury NY. Full contents of a chain restaurant on Long Island (~3-4 hrs from 02339); bar stations and stainless tables resell well. Also glycol beer system, red leather chairs, other furnishings. Opened Oct 25; closes Nov 10 11 AM ET. Verified 2026-10-26 5:45pm ET: HiBid OPEN_ABSENTEE, 105 lots.</t>
         </is>
       </c>
     </row>
@@ -20739,42 +20739,46 @@
       </c>
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>Viva Margherita restaurant complete contents (building torn down)</t>
+          <t>Met Foodmarkets turnkey grocery liquidation (Grafe Auction)</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>restaurant closing</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D50" s="13" t="inlineStr">
         <is>
-          <t>Edgewater</t>
+          <t>Bronx</t>
         </is>
       </c>
       <c r="E50" s="13" t="inlineStr">
         <is>
-          <t>NJ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>Complete contents / make offer</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H50" s="15" t="n"/>
       <c r="I50" s="13" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-      <c r="J50" s="13" t="inlineStr"/>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="J50" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-11 01:00 PM ET</t>
+        </is>
+      </c>
       <c r="K50" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>Grafe Auction</t>
         </is>
       </c>
       <c r="L50" s="13" t="inlineStr">
@@ -20790,7 +20794,7 @@
       </c>
       <c r="O50" s="14" t="inlineStr">
         <is>
-          <t>Address 163 Old River Road, Edgewater NJ. Building being torn down; complete restaurant contents for sale / make offer.</t>
+          <t>2 Hussmann compressor racks, 3-room Amerikooler walk-in cooler/freezer, Hussmann/Hill Phoenix remote cases, 24+ frozen doors, True/Red Bull merchandisers, Hobart mixer-grinder and wrappers, Lyons checkouts, NCR POS, Storflex shelving. Preview Nov 11 9AM-12PM; begins closing Nov 11 1PM EST.</t>
         </is>
       </c>
     </row>
@@ -20802,7 +20806,7 @@
       </c>
       <c r="B51" s="14" t="inlineStr">
         <is>
-          <t>Gourmet Deli/Caterer, 100-yr Madison Ave deli liquidation (51 lots: Alto-Shaam ovens, Globe slicer, refrigerated deli cases/merchandisers, walk-in box, Metro racking)</t>
+          <t>Viva Margherita restaurant complete contents (building torn down)</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
@@ -20812,41 +20816,37 @@
       </c>
       <c r="D51" s="13" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Edgewater</t>
         </is>
       </c>
       <c r="E51" s="13" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="F51" s="13" t="n">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="G51" s="13" t="inlineStr">
         <is>
-          <t>Live/online auction, prebidding open; 18% BP online</t>
+          <t>Complete contents / make offer</t>
         </is>
       </c>
       <c r="H51" s="15" t="n"/>
       <c r="I51" s="13" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="J51" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-27 02:00 PM ET</t>
-        </is>
-      </c>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="J51" s="13" t="inlineStr"/>
       <c r="K51" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
-        </is>
-      </c>
-      <c r="L51" s="21" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L51" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M51" s="13" t="inlineStr"/>
@@ -20857,7 +20857,7 @@
       </c>
       <c r="O51" s="14" t="inlineStr">
         <is>
-          <t>Live webcast starts Tue Oct 27 2 PM ET; preview Oct 27 11 AM; checkout Wed Oct 28 10-5. Address released before auction. Shipping can be arranged at buyer's cost.</t>
+          <t>Address 163 Old River Road, Edgewater NJ. Building being torn down; complete restaurant contents for sale / make offer.</t>
         </is>
       </c>
     </row>
@@ -20869,17 +20869,17 @@
       </c>
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>Daycare/preschool closing: entire inventory of 4 classrooms (tables, cubbies, indoor playground, toys; $40K invested)</t>
+          <t>Gourmet Deli/Caterer, 100-yr Madison Ave deli liquidation (51 lots: Alto-Shaam ovens, Globe slicer, refrigerated deli cases/merchandisers, walk-in box, Metro racking)</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>business closing</t>
+          <t>restaurant closing</t>
         </is>
       </c>
       <c r="D52" s="13" t="inlineStr">
         <is>
-          <t>Long Island City</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="E52" s="13" t="inlineStr">
@@ -20888,28 +20888,32 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>$8,000 all</t>
+          <t>Live/online auction, prebidding open; 18% BP online</t>
         </is>
       </c>
       <c r="H52" s="15" t="n"/>
       <c r="I52" s="13" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="J52" s="13" t="inlineStr"/>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J52" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-27 02:00 PM ET</t>
+        </is>
+      </c>
       <c r="K52" s="13" t="inlineStr">
         <is>
-          <t>Craigslist (by owner)</t>
-        </is>
-      </c>
-      <c r="L52" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
+        </is>
+      </c>
+      <c r="L52" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M52" s="13" t="inlineStr"/>
@@ -20920,7 +20924,7 @@
       </c>
       <c r="O52" s="14" t="inlineStr">
         <is>
-          <t>Off-category FYI; bulky, needs a truck.</t>
+          <t>Live webcast starts Tue Oct 27 2 PM ET; preview Oct 27 11 AM; checkout Wed Oct 28 10-5. Address released before auction. Shipping can be arranged at buyer's cost.</t>
         </is>
       </c>
     </row>
@@ -20932,17 +20936,17 @@
       </c>
       <c r="B53" s="14" t="inlineStr">
         <is>
-          <t>Kitchen store closing: sinks, faucets, hoods, vanities, counters, office stuff (mostly new in box)</t>
+          <t>Daycare/preschool closing: entire inventory of 4 classrooms (tables, cubbies, indoor playground, toys; $40K invested)</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>business closing</t>
         </is>
       </c>
       <c r="D53" s="13" t="inlineStr">
         <is>
-          <t>Brooklyn</t>
+          <t>Long Island City</t>
         </is>
       </c>
       <c r="E53" s="13" t="inlineStr">
@@ -20951,11 +20955,11 @@
         </is>
       </c>
       <c r="F53" s="13" t="n">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="G53" s="13" t="inlineStr">
         <is>
-          <t>Not listed</t>
+          <t>$8,000 all</t>
         </is>
       </c>
       <c r="H53" s="15" t="n"/>
@@ -20983,7 +20987,7 @@
       </c>
       <c r="O53" s="14" t="inlineStr">
         <is>
-          <t>Sheepshead Bay. Mostly new-in-box kitchen/bath fixtures; delivery available for large purchases. No prices posted.</t>
+          <t>Off-category FYI; bulky, needs a truck.</t>
         </is>
       </c>
     </row>
@@ -20995,17 +20999,17 @@
       </c>
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>Flooring company closed – pro tool package</t>
+          <t>Kitchen store closing: sinks, faucets, hoods, vanities, counters, office stuff (mostly new in box)</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>tools liquidation</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D54" s="13" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Brooklyn</t>
         </is>
       </c>
       <c r="E54" s="13" t="inlineStr">
@@ -21014,23 +21018,23 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>$1,000</t>
+          <t>Not listed</t>
         </is>
       </c>
       <c r="H54" s="15" t="n"/>
       <c r="I54" s="13" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J54" s="13" t="inlineStr"/>
       <c r="K54" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>Craigslist (by owner)</t>
         </is>
       </c>
       <c r="L54" s="13" t="inlineStr">
@@ -21046,7 +21050,7 @@
       </c>
       <c r="O54" s="14" t="inlineStr">
         <is>
-          <t>Flooring/construction company closed; pro tool package $1,000.</t>
+          <t>Sheepshead Bay. Mostly new-in-box kitchen/bath fixtures; delivery available for large purchases. No prices posted.</t>
         </is>
       </c>
     </row>
@@ -21058,12 +21062,12 @@
       </c>
       <c r="B55" s="14" t="inlineStr">
         <is>
-          <t>New-in-box commercial refrigeration lot – 10 Beverage-Air &amp; Perlick units (bar never opened)</t>
+          <t>Flooring company closed – pro tool package</t>
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr">
         <is>
-          <t>commercial refrigeration lot</t>
+          <t>tools liquidation</t>
         </is>
       </c>
       <c r="D55" s="13" t="inlineStr">
@@ -21081,13 +21085,13 @@
       </c>
       <c r="G55" s="13" t="inlineStr">
         <is>
-          <t>$27,500 all 10 (or per unit $2,800–$4,150)</t>
+          <t>$1,000</t>
         </is>
       </c>
       <c r="H55" s="15" t="n"/>
       <c r="I55" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="J55" s="13" t="inlineStr"/>
@@ -21109,7 +21113,7 @@
       </c>
       <c r="O55" s="14" t="inlineStr">
         <is>
-          <t>Financial District. Never installed, factory packaging: 2 Beverage-Air HBF23HC-1-HS reach-in freezers ($4,150 ea), 3 HBR23HC-1-HS reach-in fridges ($3,550 ea), 1 UCR48AHC 48" undercounter ($2,800), 3 Perlick HC24FS4 glass frosters + 1 HC24RS4 beverage fridge ($2,850 ea). Seller says full retail $47,463 (about 42% off as a bundle). Updated Oct 14.</t>
+          <t>Flooring/construction company closed; pro tool package $1,000.</t>
         </is>
       </c>
     </row>
@@ -21121,46 +21125,42 @@
       </c>
       <c r="B56" s="14" t="inlineStr">
         <is>
-          <t>Corporate caterer – Alto-Shaam, new boxed Avantco rice cookers &amp; Cadco oven, Perlick, MerryChef</t>
+          <t>New-in-box commercial refrigeration lot – 10 Beverage-Air &amp; Perlick units (bar never opened)</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>commercial refrigeration lot</t>
         </is>
       </c>
       <c r="D56" s="13" t="inlineStr">
         <is>
-          <t>Jersey City</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="E56" s="13" t="inlineStr">
         <is>
-          <t>NJ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>$27,500 all 10 (or per unit $2,800–$4,150)</t>
         </is>
       </c>
       <c r="H56" s="15" t="n"/>
       <c r="I56" s="13" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="J56" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-05 07:00 PM ET</t>
-        </is>
-      </c>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="J56" s="13" t="inlineStr"/>
       <c r="K56" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L56" s="13" t="inlineStr">
@@ -21176,7 +21176,7 @@
       </c>
       <c r="O56" s="14" t="inlineStr">
         <is>
-          <t>Thu Oct 22 2 PM. [auto-removed 2026-10-22: closing date passed] | Rescheduled: live &amp; online Nov 5 (preview 11 AM, bidding closes 7 PM ET), 19 lots.</t>
+          <t>Financial District. Never installed, factory packaging: 2 Beverage-Air HBF23HC-1-HS reach-in freezers ($4,150 ea), 3 HBR23HC-1-HS reach-in fridges ($3,550 ea), 1 UCR48AHC 48" undercounter ($2,800), 3 Perlick HC24FS4 glass frosters + 1 HC24RS4 beverage fridge ($2,850 ea). Seller says full retail $47,463 (about 42% off as a bundle). Updated Oct 14.</t>
         </is>
       </c>
     </row>
@@ -21188,12 +21188,12 @@
       </c>
       <c r="B57" s="14" t="inlineStr">
         <is>
-          <t>Lighting store closing – lease ended, up to 70% off showroom</t>
+          <t>Corporate caterer – Alto-Shaam, new boxed Avantco rice cookers &amp; Cadco oven, Perlick, MerryChef</t>
         </is>
       </c>
       <c r="C57" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D57" s="13" t="inlineStr">
@@ -21211,19 +21211,23 @@
       </c>
       <c r="G57" s="13" t="inlineStr">
         <is>
-          <t>up to 70% off</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H57" s="15" t="n"/>
       <c r="I57" s="13" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="J57" s="13" t="inlineStr"/>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="J57" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-05 07:00 PM ET</t>
+        </is>
+      </c>
       <c r="K57" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
       <c r="L57" s="13" t="inlineStr">
@@ -21239,7 +21243,7 @@
       </c>
       <c r="O57" s="14" t="inlineStr">
         <is>
-          <t>Lighting store closing, lease ended. Showroom inventory up to 70% off.</t>
+          <t>Thu Oct 22 2 PM. [auto-removed 2026-10-22: closing date passed] | Rescheduled: live &amp; online Nov 5 (preview 11 AM, bidding closes 7 PM ET), 19 lots.</t>
         </is>
       </c>
     </row>
@@ -21251,12 +21255,12 @@
       </c>
       <c r="B58" s="14" t="inlineStr">
         <is>
-          <t>Baonanas LLC ABC sale: turnkey ice cream / gelato / dessert shop equipment</t>
+          <t>Lighting store closing – lease ended, up to 70% off showroom</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>restaurant / commercial kitchen contents</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D58" s="13" t="inlineStr">
@@ -21274,15 +21278,19 @@
       </c>
       <c r="G58" s="13" t="inlineStr">
         <is>
-          <t>Accepting offers</t>
+          <t>up to 70% off</t>
         </is>
       </c>
       <c r="H58" s="15" t="n"/>
-      <c r="I58" s="13" t="inlineStr"/>
+      <c r="I58" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
       <c r="J58" s="13" t="inlineStr"/>
       <c r="K58" s="13" t="inlineStr">
         <is>
-          <t>AuctionAdvisors</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L58" s="13" t="inlineStr">
@@ -21298,7 +21306,7 @@
       </c>
       <c r="O58" s="14" t="inlineStr">
         <is>
-          <t>181 Monticello Ave. Assignment for the benefit of creditors. IFI Panorama gelato display cases, refrigerated topping stations, commercial mixers, refrigerators/freezers, stainless worktables, ice machine, POS, smallwares, gelato carts, catering gear, FF&amp;E.</t>
+          <t>Lighting store closing, lease ended. Showroom inventory up to 70% off.</t>
         </is>
       </c>
     </row>
@@ -21310,17 +21318,17 @@
       </c>
       <c r="B59" s="14" t="inlineStr">
         <is>
-          <t>Tools / plumbing / MRO supply inventory – Hilti/DeWalt/Milwaukee, fittings, heat pumps</t>
+          <t>Baonanas LLC ABC sale: turnkey ice cream / gelato / dessert shop equipment</t>
         </is>
       </c>
       <c r="C59" s="13" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>restaurant / commercial kitchen contents</t>
         </is>
       </c>
       <c r="D59" s="13" t="inlineStr">
         <is>
-          <t>Riverdale</t>
+          <t>Jersey City</t>
         </is>
       </c>
       <c r="E59" s="13" t="inlineStr">
@@ -21329,23 +21337,19 @@
         </is>
       </c>
       <c r="F59" s="13" t="n">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="G59" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Accepting offers</t>
         </is>
       </c>
       <c r="H59" s="15" t="n"/>
       <c r="I59" s="13" t="inlineStr"/>
-      <c r="J59" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-30 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="J59" s="13" t="inlineStr"/>
       <c r="K59" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
+          <t>AuctionAdvisors</t>
         </is>
       </c>
       <c r="L59" s="13" t="inlineStr">
@@ -21361,7 +21365,7 @@
       </c>
       <c r="O59" s="14" t="inlineStr">
         <is>
-          <t>Bulk resale inventory.</t>
+          <t>181 Monticello Ave. Assignment for the benefit of creditors. IFI Panorama gelato display cases, refrigerated topping stations, commercial mixers, refrigerators/freezers, stainless worktables, ice machine, POS, smallwares, gelato carts, catering gear, FF&amp;E.</t>
         </is>
       </c>
     </row>
@@ -21373,12 +21377,12 @@
       </c>
       <c r="B60" s="14" t="inlineStr">
         <is>
-          <t>Ice cream + cookie franchise equipment – Taylor soft-serve, Atosa, Blodgett</t>
+          <t>Tools / plumbing / MRO supply inventory – Hilti/DeWalt/Milwaukee, fittings, heat pumps</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>inventory</t>
         </is>
       </c>
       <c r="D60" s="13" t="inlineStr">
@@ -21403,7 +21407,7 @@
       <c r="I60" s="13" t="inlineStr"/>
       <c r="J60" s="13" t="inlineStr">
         <is>
-          <t>2026-11-05 11:00 AM ET</t>
+          <t>2026-10-30 11:00 AM ET</t>
         </is>
       </c>
       <c r="K60" s="13" t="inlineStr">
@@ -21424,7 +21428,7 @@
       </c>
       <c r="O60" s="14" t="inlineStr">
         <is>
-          <t>Resellable units.</t>
+          <t>Bulk resale inventory.</t>
         </is>
       </c>
     </row>
@@ -21436,17 +21440,17 @@
       </c>
       <c r="B61" s="14" t="inlineStr">
         <is>
-          <t>U.S. Vision court-ordered liquidation: ~70,000 designer eyeglass/sunglass frames + optical/optometry equipment at ~80 former stores + IP</t>
+          <t>Ice cream + cookie franchise equipment – Taylor soft-serve, Atosa, Blodgett</t>
         </is>
       </c>
       <c r="C61" s="13" t="inlineStr">
         <is>
-          <t>court-ordered retail chain liquidation</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D61" s="13" t="inlineStr">
         <is>
-          <t>Montclair</t>
+          <t>Riverdale</t>
         </is>
       </c>
       <c r="E61" s="13" t="inlineStr">
@@ -21455,19 +21459,23 @@
         </is>
       </c>
       <c r="F61" s="13" t="n">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G61" s="13" t="inlineStr">
         <is>
-          <t>Accepting offers (terms in offering memo, NDA required)</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H61" s="15" t="n"/>
       <c r="I61" s="13" t="inlineStr"/>
-      <c r="J61" s="13" t="inlineStr"/>
+      <c r="J61" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-05 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K61" s="13" t="inlineStr">
         <is>
-          <t>AuctionAdvisors</t>
+          <t>A.J. Willner</t>
         </is>
       </c>
       <c r="L61" s="13" t="inlineStr">
@@ -21483,7 +21491,7 @@
       </c>
       <c r="O61" s="14" t="inlineStr">
         <is>
-          <t>Three-lot sale pursuant to court order; bids accepted for individual lots, combinations, or substantially all assets. Equipment is spread across ~80 former store locations. Not appliance-related; big-ticket bulk inventory play.</t>
+          <t>Resellable units.</t>
         </is>
       </c>
     </row>
@@ -21495,17 +21503,17 @@
       </c>
       <c r="B62" s="14" t="inlineStr">
         <is>
-          <t>Wascomat commercial washers liquidation (22× W105, 6× W185, dryer panels)</t>
+          <t>U.S. Vision court-ordered liquidation: ~70,000 designer eyeglass/sunglass frames + optical/optometry equipment at ~80 former stores + IP</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>commercial laundry</t>
+          <t>court-ordered retail chain liquidation</t>
         </is>
       </c>
       <c r="D62" s="13" t="inlineStr">
         <is>
-          <t>Newark</t>
+          <t>Montclair</t>
         </is>
       </c>
       <c r="E62" s="13" t="inlineStr">
@@ -21514,23 +21522,19 @@
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G62" s="13" t="inlineStr">
         <is>
-          <t>$500–$800 each / panels $150</t>
+          <t>Accepting offers (terms in offering memo, NDA required)</t>
         </is>
       </c>
       <c r="H62" s="15" t="n"/>
-      <c r="I62" s="13" t="inlineStr">
-        <is>
-          <t>2026-07-12</t>
-        </is>
-      </c>
+      <c r="I62" s="13" t="inlineStr"/>
       <c r="J62" s="13" t="inlineStr"/>
       <c r="K62" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>AuctionAdvisors</t>
         </is>
       </c>
       <c r="L62" s="13" t="inlineStr">
@@ -21546,7 +21550,7 @@
       </c>
       <c r="O62" s="14" t="inlineStr">
         <is>
-          <t>22× W105 @ $500, 6× W185 @ $800, 20 dryer panels $150. Commercial laundry liquidation.</t>
+          <t>Three-lot sale pursuant to court order; bids accepted for individual lots, combinations, or substantially all assets. Equipment is spread across ~80 former store locations. Not appliance-related; big-ticket bulk inventory play.</t>
         </is>
       </c>
     </row>
@@ -21558,17 +21562,17 @@
       </c>
       <c r="B63" s="14" t="inlineStr">
         <is>
-          <t>Major food-service caterer – new-in-box True reach-ins, Beverage-Air, TurboChef, Resfab ventless fryer</t>
+          <t>Wascomat commercial washers liquidation (22× W105, 6× W185, dryer panels)</t>
         </is>
       </c>
       <c r="C63" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>commercial laundry</t>
         </is>
       </c>
       <c r="D63" s="13" t="inlineStr">
         <is>
-          <t>Parsippany</t>
+          <t>Newark</t>
         </is>
       </c>
       <c r="E63" s="13" t="inlineStr">
@@ -21577,27 +21581,23 @@
         </is>
       </c>
       <c r="F63" s="13" t="n">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="G63" s="13" t="inlineStr">
         <is>
-          <t>Live + webcast, 18% BP + 3%</t>
+          <t>$500–$800 each / panels $150</t>
         </is>
       </c>
       <c r="H63" s="15" t="n"/>
       <c r="I63" s="13" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="J63" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-03 02:00 PM ET</t>
-        </is>
-      </c>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="J63" s="13" t="inlineStr"/>
       <c r="K63" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Best Buy Auctioneers)</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L63" s="13" t="inlineStr">
@@ -21613,7 +21613,7 @@
       </c>
       <c r="O63" s="14" t="inlineStr">
         <is>
-          <t>Tue Nov 3 2 PM, checkout Nov 4.</t>
+          <t>22× W105 @ $500, 6× W185 @ $800, 20 dryer panels $150. Commercial laundry liquidation.</t>
         </is>
       </c>
     </row>
@@ -21625,17 +21625,17 @@
       </c>
       <c r="B64" s="14" t="inlineStr">
         <is>
-          <t>Business closing – 160 new Carnes exhaust fans</t>
+          <t>Major food-service caterer – new-in-box True reach-ins, Beverage-Air, TurboChef, Resfab ventless fryer</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>HVAC inventory</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D64" s="13" t="inlineStr">
         <is>
-          <t>Kenilworth</t>
+          <t>Parsippany</t>
         </is>
       </c>
       <c r="E64" s="13" t="inlineStr">
@@ -21648,19 +21648,23 @@
       </c>
       <c r="G64" s="13" t="inlineStr">
         <is>
-          <t>$40 each or $5,000 all OBO</t>
+          <t>Live + webcast, 18% BP + 3%</t>
         </is>
       </c>
       <c r="H64" s="15" t="n"/>
       <c r="I64" s="13" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="J64" s="13" t="inlineStr"/>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="J64" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-03 02:00 PM ET</t>
+        </is>
+      </c>
       <c r="K64" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>HiBid (Best Buy Auctioneers)</t>
         </is>
       </c>
       <c r="L64" s="13" t="inlineStr">
@@ -21676,7 +21680,7 @@
       </c>
       <c r="O64" s="14" t="inlineStr">
         <is>
-          <t>160 new Carnes 80CFM 1.0 sone exhaust fans. $40 each or $5,000 for all OBO. Business closing HVAC inventory.</t>
+          <t>Tue Nov 3 2 PM, checkout Nov 4.</t>
         </is>
       </c>
     </row>
@@ -21688,12 +21692,12 @@
       </c>
       <c r="B65" s="14" t="inlineStr">
         <is>
-          <t>Air Systems Inc – sheet metal / HVAC fabrication shop liquidation</t>
+          <t>Business closing – 160 new Carnes exhaust fans</t>
         </is>
       </c>
       <c r="C65" s="13" t="inlineStr">
         <is>
-          <t>HVAC shop liquidation</t>
+          <t>HVAC inventory</t>
         </is>
       </c>
       <c r="D65" s="13" t="inlineStr">
@@ -21711,24 +21715,24 @@
       </c>
       <c r="G65" s="13" t="inlineStr">
         <is>
-          <t>Timed online (15% BP)</t>
+          <t>$40 each or $5,000 all OBO</t>
         </is>
       </c>
       <c r="H65" s="15" t="n"/>
-      <c r="I65" s="13" t="inlineStr"/>
-      <c r="J65" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-29 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="I65" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="J65" s="13" t="inlineStr"/>
       <c r="K65" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner Auctions</t>
-        </is>
-      </c>
-      <c r="L65" s="21" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>Craigslist</t>
+        </is>
+      </c>
+      <c r="L65" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M65" s="13" t="inlineStr"/>
@@ -21739,7 +21743,7 @@
       </c>
       <c r="O65" s="14" t="inlineStr">
         <is>
-          <t>Vicon HVAC plasma; Flagler/Lockformer/Roto-Die/Engel fab; welders; Clark forklift; Genie Superlift; Ridgid/Milwaukee/DeWalt/Bosch/Hilti/Makita tools; AeroVent/Carnes exhaust fans; racking/scaffolding. Preview Oct 28–29 AM; pickup Oct 29 PM–Nov 4. Same town as Carnes fan CL lot.</t>
+          <t>160 new Carnes 80CFM 1.0 sone exhaust fans. $40 each or $5,000 for all OBO. Business closing HVAC inventory.</t>
         </is>
       </c>
     </row>
@@ -21751,17 +21755,17 @@
       </c>
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>Former Rush Bowls franchise ABC sale: commercial refrigeration, Vitamix blenders, ice &amp; beverage equipment</t>
+          <t>Air Systems Inc – sheet metal / HVAC fabrication shop liquidation</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>restaurant / commercial kitchen contents</t>
+          <t>HVAC shop liquidation</t>
         </is>
       </c>
       <c r="D66" s="13" t="inlineStr">
         <is>
-          <t>Westfield</t>
+          <t>Kenilworth</t>
         </is>
       </c>
       <c r="E66" s="13" t="inlineStr">
@@ -21770,24 +21774,28 @@
         </is>
       </c>
       <c r="F66" s="13" t="n">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="G66" s="13" t="inlineStr">
         <is>
-          <t>Accepting offers</t>
+          <t>Timed online (15% BP)</t>
         </is>
       </c>
       <c r="H66" s="15" t="n"/>
       <c r="I66" s="13" t="inlineStr"/>
-      <c r="J66" s="13" t="inlineStr"/>
+      <c r="J66" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-29 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K66" s="13" t="inlineStr">
         <is>
-          <t>AuctionAdvisors</t>
-        </is>
-      </c>
-      <c r="L66" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>A.J. Willner Auctions</t>
+        </is>
+      </c>
+      <c r="L66" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M66" s="13" t="inlineStr"/>
@@ -21798,7 +21806,7 @@
       </c>
       <c r="O66" s="14" t="inlineStr">
         <is>
-          <t>27 East Broad St. Assignment for the benefit of creditors of 333 Star Enterprises (d/b/a Rush Bowls). Commercial refrigeration/freezers, Vitamix blenders, stainless workstations/sinks, ice and beverage equipment, POS, shelving. Inspection by contacting the auctioneer.</t>
+          <t>Vicon HVAC plasma; Flagler/Lockformer/Roto-Die/Engel fab; welders; Clark forklift; Genie Superlift; Ridgid/Milwaukee/DeWalt/Bosch/Hilti/Makita tools; AeroVent/Carnes exhaust fans; racking/scaffolding. Preview Oct 28–29 AM; pickup Oct 29 PM–Nov 4. Same town as Carnes fan CL lot.</t>
         </is>
       </c>
     </row>
@@ -21810,17 +21818,17 @@
       </c>
       <c r="B67" s="14" t="inlineStr">
         <is>
-          <t>Bimmer Clinic business liquidation (BMW repair shop): vehicle lifts, forklift, skid steer, refrigerant recovery, shop tools &amp; equipment</t>
+          <t>Former Rush Bowls franchise ABC sale: commercial refrigeration, Vitamix blenders, ice &amp; beverage equipment</t>
         </is>
       </c>
       <c r="C67" s="13" t="inlineStr">
         <is>
-          <t>business liquidation auction</t>
+          <t>restaurant / commercial kitchen contents</t>
         </is>
       </c>
       <c r="D67" s="13" t="inlineStr">
         <is>
-          <t>South Amboy</t>
+          <t>Westfield</t>
         </is>
       </c>
       <c r="E67" s="13" t="inlineStr">
@@ -21829,23 +21837,19 @@
         </is>
       </c>
       <c r="F67" s="13" t="n">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="G67" s="13" t="inlineStr">
         <is>
-          <t>Timed online auction</t>
+          <t>Accepting offers</t>
         </is>
       </c>
       <c r="H67" s="15" t="n"/>
       <c r="I67" s="13" t="inlineStr"/>
-      <c r="J67" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-12 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="J67" s="13" t="inlineStr"/>
       <c r="K67" s="13" t="inlineStr">
         <is>
-          <t>AJ Willner Auctions</t>
+          <t>AuctionAdvisors</t>
         </is>
       </c>
       <c r="L67" s="13" t="inlineStr">
@@ -21861,7 +21865,7 @@
       </c>
       <c r="O67" s="14" t="inlineStr">
         <is>
-          <t>Ends Nov 12 11 AM EST.</t>
+          <t>27 East Broad St. Assignment for the benefit of creditors of 333 Star Enterprises (d/b/a Rush Bowls). Commercial refrigeration/freezers, Vitamix blenders, stainless workstations/sinks, ice and beverage equipment, POS, shelving. Inspection by contacting the auctioneer.</t>
         </is>
       </c>
     </row>
@@ -21873,17 +21877,17 @@
       </c>
       <c r="B68" s="14" t="inlineStr">
         <is>
-          <t>Drywall &amp; Acoustical Contractor 2: Hilti tools, material handling, supplies (Ideal Trading Corp)</t>
+          <t>Bimmer Clinic business liquidation (BMW repair shop): vehicle lifts, forklift, skid steer, refrigerant recovery, shop tools &amp; equipment</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>auction</t>
+          <t>business liquidation auction</t>
         </is>
       </c>
       <c r="D68" s="13" t="inlineStr">
         <is>
-          <t>Randolph</t>
+          <t>South Amboy</t>
         </is>
       </c>
       <c r="E68" s="13" t="inlineStr">
@@ -21892,28 +21896,28 @@
         </is>
       </c>
       <c r="F68" s="13" t="n">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G68" s="13" t="inlineStr">
         <is>
-          <t>Online auction (HiBid terms)</t>
+          <t>Timed online auction</t>
         </is>
       </c>
       <c r="H68" s="15" t="n"/>
       <c r="I68" s="13" t="inlineStr"/>
       <c r="J68" s="13" t="inlineStr">
         <is>
-          <t>2026-10-28 11:00 AM ET</t>
+          <t>2026-11-12 11:00 AM ET</t>
         </is>
       </c>
       <c r="K68" s="13" t="inlineStr">
         <is>
-          <t>HiBid (Ideal Trading Corp)</t>
-        </is>
-      </c>
-      <c r="L68" s="21" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>AJ Willner Auctions</t>
+        </is>
+      </c>
+      <c r="L68" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M68" s="13" t="inlineStr"/>
@@ -21924,7 +21928,7 @@
       </c>
       <c r="O68" s="14" t="inlineStr">
         <is>
-          <t>Contractor contents; closes Oct 28 11 AM. Hilti tools resell well on eBay.</t>
+          <t>Ends Nov 12 11 AM EST.</t>
         </is>
       </c>
     </row>
@@ -21936,17 +21940,17 @@
       </c>
       <c r="B69" s="14" t="inlineStr">
         <is>
-          <t>New modular concession kitchens (warehouseman's lien) – 5 units, CaptiveAire hoods, new Ovention/Turbo Air</t>
+          <t>Drywall &amp; Acoustical Contractor 2: Hilti tools, material handling, supplies (Ideal Trading Corp)</t>
         </is>
       </c>
       <c r="C69" s="13" t="inlineStr">
         <is>
-          <t>lien sale</t>
+          <t>auction</t>
         </is>
       </c>
       <c r="D69" s="13" t="inlineStr">
         <is>
-          <t>Edison</t>
+          <t>Randolph</t>
         </is>
       </c>
       <c r="E69" s="13" t="inlineStr">
@@ -21955,24 +21959,28 @@
         </is>
       </c>
       <c r="F69" s="13" t="n">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="G69" s="13" t="inlineStr">
         <is>
-          <t>Online auction, $2K load-out fee</t>
+          <t>Online auction (HiBid terms)</t>
         </is>
       </c>
       <c r="H69" s="15" t="n"/>
       <c r="I69" s="13" t="inlineStr"/>
-      <c r="J69" s="13" t="inlineStr"/>
+      <c r="J69" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-28 11:00 AM ET</t>
+        </is>
+      </c>
       <c r="K69" s="13" t="inlineStr">
         <is>
-          <t>A.J. Willner</t>
-        </is>
-      </c>
-      <c r="L69" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>HiBid (Ideal Trading Corp)</t>
+        </is>
+      </c>
+      <c r="L69" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M69" s="13" t="inlineStr"/>
@@ -21983,7 +21991,7 @@
       </c>
       <c r="O69" s="14" t="inlineStr">
         <is>
-          <t>&gt;$100K new. Close date not captured.</t>
+          <t>Contractor contents; closes Oct 28 11 AM. Hilti tools resell well on eBay.</t>
         </is>
       </c>
     </row>
@@ -21995,17 +22003,17 @@
       </c>
       <c r="B70" s="14" t="inlineStr">
         <is>
-          <t>Party City (Ch. 11) store – fixtures + party merchandise inventory</t>
+          <t>New modular concession kitchens (warehouseman's lien) – 5 units, CaptiveAire hoods, new Ovention/Turbo Air</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>lien sale</t>
         </is>
       </c>
       <c r="D70" s="13" t="inlineStr">
         <is>
-          <t>East Brunswick</t>
+          <t>Edison</t>
         </is>
       </c>
       <c r="E70" s="13" t="inlineStr">
@@ -22014,20 +22022,16 @@
         </is>
       </c>
       <c r="F70" s="13" t="n">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="G70" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>Online auction, $2K load-out fee</t>
         </is>
       </c>
       <c r="H70" s="15" t="n"/>
       <c r="I70" s="13" t="inlineStr"/>
-      <c r="J70" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-03 11:00 AM ET</t>
-        </is>
-      </c>
+      <c r="J70" s="13" t="inlineStr"/>
       <c r="K70" s="13" t="inlineStr">
         <is>
           <t>A.J. Willner</t>
@@ -22046,7 +22050,7 @@
       </c>
       <c r="O70" s="14" t="inlineStr">
         <is>
-          <t>Store inventory.</t>
+          <t>&gt;$100K new. Close date not captured.</t>
         </is>
       </c>
     </row>
@@ -22058,17 +22062,17 @@
       </c>
       <c r="B71" s="14" t="inlineStr">
         <is>
-          <t>Ability to Work kitchen and store – commercial kitchen + store fixtures (~135 lots)</t>
+          <t>Party City (Ch. 11) store – fixtures + party merchandise inventory</t>
         </is>
       </c>
       <c r="C71" s="13" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D71" s="13" t="inlineStr">
         <is>
-          <t>Flemington</t>
+          <t>East Brunswick</t>
         </is>
       </c>
       <c r="E71" s="13" t="inlineStr">
@@ -22077,28 +22081,28 @@
         </is>
       </c>
       <c r="F71" s="13" t="n">
-        <v>237</v>
+        <v>220</v>
       </c>
       <c r="G71" s="13" t="inlineStr">
         <is>
-          <t>Timed online (15% BP)</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H71" s="15" t="n"/>
       <c r="I71" s="13" t="inlineStr"/>
       <c r="J71" s="13" t="inlineStr">
         <is>
-          <t>2026-10-27 11:02 AM ET</t>
+          <t>2026-11-03 11:00 AM ET</t>
         </is>
       </c>
       <c r="K71" s="13" t="inlineStr">
         <is>
-          <t>HiBid</t>
-        </is>
-      </c>
-      <c r="L71" s="21" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>A.J. Willner</t>
+        </is>
+      </c>
+      <c r="L71" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M71" s="13" t="inlineStr"/>
@@ -22109,7 +22113,7 @@
       </c>
       <c r="O71" s="14" t="inlineStr">
         <is>
-          <t>Apprentice/hospitality training cafe-kitchen and store dispersal. Preview 9–11 AM sale day; removal Oct 27 noon–Oct 29.</t>
+          <t>Store inventory.</t>
         </is>
       </c>
     </row>
@@ -22121,17 +22125,17 @@
       </c>
       <c r="B72" s="14" t="inlineStr">
         <is>
-          <t>Wren Kitchens showroom closing – JennAir/Café/KitchenAid/GE Profile appliances + display kitchens</t>
+          <t>Bakery/Cafe Somerville NJ – rack ovens, La Marzocco, food truck (~76 lots)</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>showroom closing</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D72" s="13" t="inlineStr">
         <is>
-          <t>Lawrenceville</t>
+          <t>Somerville</t>
         </is>
       </c>
       <c r="E72" s="13" t="inlineStr">
@@ -22140,23 +22144,27 @@
         </is>
       </c>
       <c r="F72" s="13" t="n">
-        <v>239</v>
+        <v>224</v>
       </c>
       <c r="G72" s="13" t="inlineStr">
         <is>
-          <t>Online auction, 18% BP</t>
+          <t>Live webcast + online (18% BP online)</t>
         </is>
       </c>
       <c r="H72" s="15" t="n"/>
-      <c r="I72" s="13" t="inlineStr"/>
+      <c r="I72" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
       <c r="J72" s="13" t="inlineStr">
         <is>
-          <t>2026-10-27 09:00 AM ET</t>
+          <t>2026-10-26 07:00 PM ET</t>
         </is>
       </c>
       <c r="K72" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
+          <t>HiBid / Best Buy Auctioneers</t>
         </is>
       </c>
       <c r="L72" s="21" t="inlineStr">
@@ -22172,7 +22180,7 @@
       </c>
       <c r="O72" s="14" t="inlineStr">
         <is>
-          <t>Premium floor-model appliances; lots close from Oct 27 9 AM.</t>
+          <t>Full bakery/cafe commercial kitchen: food truck w/ pizza oven, La Marzocco espresso, Mazzer, Baxter + Empire Logiudice rack ovens, dough depositor, Globe floor mixer, Artic Air / SS refrigeration, fryers, Vitamix, Robot Coupe, display cases, dining furniture. Preview 11 AM sale day; checkout Tue 10/27. | 2026-10-26 8am ET: HiBid shows auction open (absentee bidding), 84 open lots; live webcast starts 2 PM ET today. | Restored 2026-10-26 5:45pm ET: HiBid shows OPEN_WEBCAST (live webcast in progress), bid close 7 PM ET tonight; only 1 of 144 lots still open.</t>
         </is>
       </c>
     </row>
@@ -22184,17 +22192,17 @@
       </c>
       <c r="B73" s="14" t="inlineStr">
         <is>
-          <t>50+ yr antique business liquidation – entire 30x60 warehouse full of antiques, wrought iron, collectibles, furniture, lighting (no reasonable offer refused)</t>
+          <t>Ability to Work kitchen and store – commercial kitchen + store fixtures (~135 lots)</t>
         </is>
       </c>
       <c r="C73" s="13" t="inlineStr">
         <is>
-          <t>business liquidation</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D73" s="13" t="inlineStr">
         <is>
-          <t>Pennington</t>
+          <t>Flemington</t>
         </is>
       </c>
       <c r="E73" s="13" t="inlineStr">
@@ -22203,35 +22211,31 @@
         </is>
       </c>
       <c r="F73" s="13" t="n">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="G73" s="13" t="inlineStr">
         <is>
-          <t>Best offer (cash &amp; carry)</t>
+          <t>Timed online (15% BP)</t>
         </is>
       </c>
       <c r="H73" s="15" t="n"/>
-      <c r="I73" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="J73" s="13" t="inlineStr"/>
+      <c r="I73" s="13" t="inlineStr"/>
+      <c r="J73" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-27 11:02 AM ET</t>
+        </is>
+      </c>
       <c r="K73" s="13" t="inlineStr">
         <is>
-          <t>Craigslist</t>
-        </is>
-      </c>
-      <c r="L73" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M73" s="20" t="inlineStr">
-        <is>
-          <t>FLIP</t>
-        </is>
-      </c>
+          <t>HiBid</t>
+        </is>
+      </c>
+      <c r="L73" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
+        </is>
+      </c>
+      <c r="M73" s="13" t="inlineStr"/>
       <c r="N73" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -22239,7 +22243,7 @@
       </c>
       <c r="O73" s="14" t="inlineStr">
         <is>
-          <t>By appointment; bring truck/flashlight/boxes. Seller reposts the same sale under many CL URLs (e.g. gsHWPrsC9miNrtazkuhXoD, oBMFsC2ADf3YjgMSngPdpy, 15uS5HaHeQBJ2rEBQNFK8n). Not appliances – bulk resale stock.</t>
+          <t>Apprentice/hospitality training cafe-kitchen and store dispersal. Preview 9–11 AM sale day; removal Oct 27 noon–Oct 29.</t>
         </is>
       </c>
     </row>
@@ -22251,17 +22255,17 @@
       </c>
       <c r="B74" s="14" t="inlineStr">
         <is>
-          <t>Pete's Famous Bakery equipment auction (Trima K2 bun divider-rounder, Bloemhof dough sheeter, Empire spiral mixer, JAC bread slicer, Groen 60-gal tilting kettle, Hoshizaki, Pitco fryer)</t>
+          <t>Wren Kitchens showroom closing – JennAir/Café/KitchenAid/GE Profile appliances + display kitchens</t>
         </is>
       </c>
       <c r="C74" s="13" t="inlineStr">
         <is>
-          <t>restaurant auction</t>
+          <t>showroom closing</t>
         </is>
       </c>
       <c r="D74" s="13" t="inlineStr">
         <is>
-          <t>Ewing</t>
+          <t>Lawrenceville</t>
         </is>
       </c>
       <c r="E74" s="13" t="inlineStr">
@@ -22270,32 +22274,28 @@
         </is>
       </c>
       <c r="F74" s="13" t="n">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="G74" s="13" t="inlineStr">
         <is>
-          <t>Online auction, first lot ~$850</t>
+          <t>Online auction, 18% BP</t>
         </is>
       </c>
       <c r="H74" s="15" t="n"/>
-      <c r="I74" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
+      <c r="I74" s="13" t="inlineStr"/>
       <c r="J74" s="13" t="inlineStr">
         <is>
-          <t>2026-11-08 08:00 PM ET</t>
+          <t>2026-10-27 09:00 AM ET</t>
         </is>
       </c>
       <c r="K74" s="13" t="inlineStr">
         <is>
-          <t>PCI Auctions</t>
-        </is>
-      </c>
-      <c r="L74" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L74" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M74" s="13" t="inlineStr"/>
@@ -22306,7 +22306,7 @@
       </c>
       <c r="O74" s="14" t="inlineStr">
         <is>
-          <t>Ends Sun Nov 8 8 PM EST. PCI NY/NJ warehouse, 200 Kelsey Ave, Ewing NJ 08638. Preview Nov 5-6; removal Nov 9. Also Hoshizaki pizza prep table + 2-door reach-in. PCI offers shipping. Page doesn't say outright the bakery closed. URL verified live 2026-10-26.</t>
+          <t>Premium floor-model appliances; lots close from Oct 27 9 AM.</t>
         </is>
       </c>
     </row>
@@ -22318,17 +22318,17 @@
       </c>
       <c r="B75" s="14" t="inlineStr">
         <is>
-          <t>The Mill Restaurant &amp; Cafe equipment auction (dual turbo combi oven, double-deck 6-pie pizza oven, 3-bay pasta cooker, more)</t>
+          <t>50+ yr antique business liquidation – entire 30x60 warehouse full of antiques, wrought iron, collectibles, furniture, lighting (no reasonable offer refused)</t>
         </is>
       </c>
       <c r="C75" s="13" t="inlineStr">
         <is>
-          <t>restaurant auction</t>
+          <t>business liquidation</t>
         </is>
       </c>
       <c r="D75" s="13" t="inlineStr">
         <is>
-          <t>Ewing</t>
+          <t>Pennington</t>
         </is>
       </c>
       <c r="E75" s="13" t="inlineStr">
@@ -22337,27 +22337,23 @@
         </is>
       </c>
       <c r="F75" s="13" t="n">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="G75" s="13" t="inlineStr">
         <is>
-          <t>Online auction, current bids</t>
+          <t>Best offer (cash &amp; carry)</t>
         </is>
       </c>
       <c r="H75" s="15" t="n"/>
       <c r="I75" s="13" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="J75" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-01 08:00 PM ET</t>
-        </is>
-      </c>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="J75" s="13" t="inlineStr"/>
       <c r="K75" s="13" t="inlineStr">
         <is>
-          <t>PCI Auctions</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L75" s="13" t="inlineStr">
@@ -22365,7 +22361,11 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M75" s="13" t="inlineStr"/>
+      <c r="M75" s="20" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
       <c r="N75" s="16" t="inlineStr">
         <is>
           <t>Open</t>
@@ -22373,7 +22373,7 @@
       </c>
       <c r="O75" s="14" t="inlineStr">
         <is>
-          <t>Ends Sun Nov 1 8 PM EST. PCI NY/NJ warehouse, 200 Kelsey Ave, Ewing NJ 08638. Preview Oct 29-30; removal Nov 2. Full restaurant cooking line. Shipping/delivery available. URL verified live 2026-10-26.</t>
+          <t>By appointment; bring truck/flashlight/boxes. Seller reposts the same sale under many CL URLs (e.g. gsHWPrsC9miNrtazkuhXoD, oBMFsC2ADf3YjgMSngPdpy, 15uS5HaHeQBJ2rEBQNFK8n). Not appliances – bulk resale stock.</t>
         </is>
       </c>
     </row>
@@ -22385,17 +22385,17 @@
       </c>
       <c r="B76" s="14" t="inlineStr">
         <is>
-          <t>Wren Kitchens showroom closing – GE/Whirlpool/KitchenAid/Café incl. NIB Café range + 35 kitchens</t>
+          <t>Pete's Famous Bakery equipment auction (Trima K2 bun divider-rounder, Bloemhof dough sheeter, Empire spiral mixer, JAC bread slicer, Groen 60-gal tilting kettle, Hoshizaki, Pitco fryer)</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
-          <t>showroom closing</t>
+          <t>restaurant auction</t>
         </is>
       </c>
       <c r="D76" s="13" t="inlineStr">
         <is>
-          <t>Cherry Hill</t>
+          <t>Ewing</t>
         </is>
       </c>
       <c r="E76" s="13" t="inlineStr">
@@ -22404,23 +22404,27 @@
         </is>
       </c>
       <c r="F76" s="13" t="n">
-        <v>266</v>
+        <v>244</v>
       </c>
       <c r="G76" s="13" t="inlineStr">
         <is>
-          <t>Online auction, openers ~$0.50</t>
+          <t>Online auction, first lot ~$850</t>
         </is>
       </c>
       <c r="H76" s="15" t="n"/>
-      <c r="I76" s="13" t="inlineStr"/>
+      <c r="I76" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
       <c r="J76" s="13" t="inlineStr">
         <is>
-          <t>2026-11-02 11:00 AM ET</t>
+          <t>2026-11-08 08:00 PM ET</t>
         </is>
       </c>
       <c r="K76" s="13" t="inlineStr">
         <is>
-          <t>Grafe Auction</t>
+          <t>PCI Auctions</t>
         </is>
       </c>
       <c r="L76" s="13" t="inlineStr">
@@ -22436,191 +22440,187 @@
       </c>
       <c r="O76" s="14" t="inlineStr">
         <is>
+          <t>Ends Sun Nov 8 8 PM EST. PCI NY/NJ warehouse, 200 Kelsey Ave, Ewing NJ 08638. Preview Nov 5-6; removal Nov 9. Also Hoshizaki pizza prep table + 2-door reach-in. PCI offers shipping. Page doesn't say outright the bakery closed. URL verified live 2026-10-26.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" outlineLevel="1">
+      <c r="A77" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B77" s="14" t="inlineStr">
+        <is>
+          <t>The Mill Restaurant &amp; Cafe equipment auction (dual turbo combi oven, double-deck 6-pie pizza oven, 3-bay pasta cooker, more)</t>
+        </is>
+      </c>
+      <c r="C77" s="13" t="inlineStr">
+        <is>
+          <t>restaurant auction</t>
+        </is>
+      </c>
+      <c r="D77" s="13" t="inlineStr">
+        <is>
+          <t>Ewing</t>
+        </is>
+      </c>
+      <c r="E77" s="13" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="F77" s="13" t="n">
+        <v>244</v>
+      </c>
+      <c r="G77" s="13" t="inlineStr">
+        <is>
+          <t>Online auction, current bids</t>
+        </is>
+      </c>
+      <c r="H77" s="15" t="n"/>
+      <c r="I77" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="J77" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-01 08:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K77" s="13" t="inlineStr">
+        <is>
+          <t>PCI Auctions</t>
+        </is>
+      </c>
+      <c r="L77" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M77" s="13" t="inlineStr"/>
+      <c r="N77" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O77" s="14" t="inlineStr">
+        <is>
+          <t>Ends Sun Nov 1 8 PM EST. PCI NY/NJ warehouse, 200 Kelsey Ave, Ewing NJ 08638. Preview Oct 29-30; removal Nov 2. Full restaurant cooking line. Shipping/delivery available. URL verified live 2026-10-26.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" outlineLevel="1">
+      <c r="A78" s="13" t="inlineStr">
+        <is>
+          <t>NYC / Long Island / NJ</t>
+        </is>
+      </c>
+      <c r="B78" s="14" t="inlineStr">
+        <is>
+          <t>Wren Kitchens showroom closing – GE/Whirlpool/KitchenAid/Café incl. NIB Café range + 35 kitchens</t>
+        </is>
+      </c>
+      <c r="C78" s="13" t="inlineStr">
+        <is>
+          <t>showroom closing</t>
+        </is>
+      </c>
+      <c r="D78" s="13" t="inlineStr">
+        <is>
+          <t>Cherry Hill</t>
+        </is>
+      </c>
+      <c r="E78" s="13" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="F78" s="13" t="n">
+        <v>266</v>
+      </c>
+      <c r="G78" s="13" t="inlineStr">
+        <is>
+          <t>Online auction, openers ~$0.50</t>
+        </is>
+      </c>
+      <c r="H78" s="15" t="n"/>
+      <c r="I78" s="13" t="inlineStr"/>
+      <c r="J78" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-02 11:00 AM ET</t>
+        </is>
+      </c>
+      <c r="K78" s="13" t="inlineStr">
+        <is>
+          <t>Grafe Auction</t>
+        </is>
+      </c>
+      <c r="L78" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M78" s="13" t="inlineStr"/>
+      <c r="N78" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O78" s="14" t="inlineStr">
+        <is>
           <t>Lots close from Nov 2 11 AM.</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="17" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="17" t="inlineStr">
         <is>
           <t>Subtotal — NYC / Long Island / NJ</t>
         </is>
       </c>
-      <c r="B77" s="17" t="inlineStr">
-        <is>
-          <t>28 item(s)</t>
-        </is>
-      </c>
-      <c r="C77" s="18" t="n"/>
-      <c r="D77" s="18" t="n"/>
-      <c r="E77" s="18" t="n"/>
-      <c r="F77" s="18" t="n"/>
-      <c r="G77" s="18" t="n"/>
-      <c r="H77" s="19" t="n">
+      <c r="B79" s="17" t="inlineStr">
+        <is>
+          <t>30 item(s)</t>
+        </is>
+      </c>
+      <c r="C79" s="18" t="n"/>
+      <c r="D79" s="18" t="n"/>
+      <c r="E79" s="18" t="n"/>
+      <c r="F79" s="18" t="n"/>
+      <c r="G79" s="18" t="n"/>
+      <c r="H79" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I77" s="18" t="n"/>
-      <c r="J77" s="18" t="n"/>
-      <c r="K77" s="18" t="n"/>
-      <c r="L77" s="18" t="n"/>
-      <c r="M77" s="18" t="n"/>
-      <c r="N77" s="18" t="n"/>
-      <c r="O77" s="18" t="n"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="11" t="inlineStr">
+      <c r="I79" s="18" t="n"/>
+      <c r="J79" s="18" t="n"/>
+      <c r="K79" s="18" t="n"/>
+      <c r="L79" s="18" t="n"/>
+      <c r="M79" s="18" t="n"/>
+      <c r="N79" s="18" t="n"/>
+      <c r="O79" s="18" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="inlineStr">
         <is>
           <t>▸ Eastern PA / Mid-Atlantic  (5)</t>
         </is>
       </c>
-      <c r="B78" s="12" t="n"/>
-      <c r="C78" s="12" t="n"/>
-      <c r="D78" s="12" t="n"/>
-      <c r="E78" s="12" t="n"/>
-      <c r="F78" s="12" t="n"/>
-      <c r="G78" s="12" t="n"/>
-      <c r="H78" s="12" t="n"/>
-      <c r="I78" s="12" t="n"/>
-      <c r="J78" s="12" t="n"/>
-      <c r="K78" s="12" t="n"/>
-      <c r="L78" s="12" t="n"/>
-      <c r="M78" s="12" t="n"/>
-      <c r="N78" s="12" t="n"/>
-      <c r="O78" s="12" t="n"/>
-    </row>
-    <row r="79" outlineLevel="1">
-      <c r="A79" s="13" t="inlineStr">
-        <is>
-          <t>Eastern PA / Mid-Atlantic</t>
-        </is>
-      </c>
-      <c r="B79" s="14" t="inlineStr">
-        <is>
-          <t>Piscitello's Home Center closing after 68 years: storewide 20% off liquidation (hardware, lumber, doors, windows, kitchen/bath)</t>
-        </is>
-      </c>
-      <c r="C79" s="13" t="inlineStr">
-        <is>
-          <t>store closing</t>
-        </is>
-      </c>
-      <c r="D79" s="13" t="inlineStr">
-        <is>
-          <t>Wilson</t>
-        </is>
-      </c>
-      <c r="E79" s="13" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="F79" s="13" t="n">
-        <v>250</v>
-      </c>
-      <c r="G79" s="13" t="inlineStr">
-        <is>
-          <t>20% off storewide (all sales final)</t>
-        </is>
-      </c>
-      <c r="H79" s="15" t="n"/>
-      <c r="I79" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="J79" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-30 06:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K79" s="13" t="inlineStr">
-        <is>
-          <t>LehighValley.com article</t>
-        </is>
-      </c>
-      <c r="L79" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M79" s="13" t="inlineStr"/>
-      <c r="N79" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O79" s="14" t="inlineStr">
-        <is>
-          <t>2300 Wood Ave, Wilson Borough (Easton area). Final day Oct 30. Retail-floor sale, not a bulk lot; ask in person about buying remaining stock outright.</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" outlineLevel="1">
-      <c r="A80" s="13" t="inlineStr">
-        <is>
-          <t>Eastern PA / Mid-Atlantic</t>
-        </is>
-      </c>
-      <c r="B80" s="14" t="inlineStr">
-        <is>
-          <t>Hearing aid manufacturing facility inventory liquidation (shelving, 3D printers/scanners, laser engravers, Porta-Vac, sound booths, office; bulk offer invited)</t>
-        </is>
-      </c>
-      <c r="C80" s="13" t="inlineStr">
-        <is>
-          <t>facility liquidation</t>
-        </is>
-      </c>
-      <c r="D80" s="13" t="inlineStr">
-        <is>
-          <t>Bristol</t>
-        </is>
-      </c>
-      <c r="E80" s="13" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="F80" s="13" t="n">
-        <v>252</v>
-      </c>
-      <c r="G80" s="13" t="inlineStr">
-        <is>
-          <t>Best offer / bulk offer for complete lot</t>
-        </is>
-      </c>
-      <c r="H80" s="15" t="n"/>
-      <c r="I80" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="J80" s="13" t="inlineStr">
-        <is>
-          <t>2026-11-08 05:00 PM ET</t>
-        </is>
-      </c>
-      <c r="K80" s="13" t="inlineStr">
-        <is>
-          <t>Craigslist</t>
-        </is>
-      </c>
-      <c r="L80" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M80" s="13" t="inlineStr"/>
-      <c r="N80" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O80" s="14" t="inlineStr">
-        <is>
-          <t>Sale Nov 6-8 ONLY, 8 AM-5 PM (updated 2026-10-25; was 'daily'). 806 Beaver St near Rt 13. Industrial shelving and lab equipment, not appliances; bulk offer invited. Email to schedule viewing.</t>
-        </is>
-      </c>
+      <c r="B80" s="12" t="n"/>
+      <c r="C80" s="12" t="n"/>
+      <c r="D80" s="12" t="n"/>
+      <c r="E80" s="12" t="n"/>
+      <c r="F80" s="12" t="n"/>
+      <c r="G80" s="12" t="n"/>
+      <c r="H80" s="12" t="n"/>
+      <c r="I80" s="12" t="n"/>
+      <c r="J80" s="12" t="n"/>
+      <c r="K80" s="12" t="n"/>
+      <c r="L80" s="12" t="n"/>
+      <c r="M80" s="12" t="n"/>
+      <c r="N80" s="12" t="n"/>
+      <c r="O80" s="12" t="n"/>
     </row>
     <row r="81" outlineLevel="1">
       <c r="A81" s="13" t="inlineStr">
@@ -22630,17 +22630,17 @@
       </c>
       <c r="B81" s="14" t="inlineStr">
         <is>
-          <t>NBM Liquidation as-is/damaged appliance &amp; more auction (357 lots)</t>
+          <t>Piscitello's Home Center closing after 68 years: storewide 20% off liquidation (hardware, lumber, doors, windows, kitchen/bath)</t>
         </is>
       </c>
       <c r="C81" s="13" t="inlineStr">
         <is>
-          <t>auction pallet</t>
+          <t>store closing</t>
         </is>
       </c>
       <c r="D81" s="13" t="inlineStr">
         <is>
-          <t>Scranton</t>
+          <t>Wilson</t>
         </is>
       </c>
       <c r="E81" s="13" t="inlineStr">
@@ -22649,28 +22649,32 @@
         </is>
       </c>
       <c r="F81" s="13" t="n">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="G81" s="13" t="inlineStr">
         <is>
-          <t>Online auction</t>
+          <t>20% off storewide (all sales final)</t>
         </is>
       </c>
       <c r="H81" s="15" t="n"/>
-      <c r="I81" s="13" t="inlineStr"/>
+      <c r="I81" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
       <c r="J81" s="13" t="inlineStr">
         <is>
-          <t>2026-10-27 06:00 PM ET</t>
+          <t>2026-10-30 06:00 PM ET</t>
         </is>
       </c>
       <c r="K81" s="13" t="inlineStr">
         <is>
-          <t>HiBid</t>
-        </is>
-      </c>
-      <c r="L81" s="21" t="inlineStr">
-        <is>
-          <t>ENDING SOON</t>
+          <t>LehighValley.com article</t>
+        </is>
+      </c>
+      <c r="L81" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M81" s="13" t="inlineStr"/>
@@ -22681,7 +22685,7 @@
       </c>
       <c r="O81" s="14" t="inlineStr">
         <is>
-          <t>Recurring reseller auction (not a closing): as-is/damaged whole appliances and more. Pickup 733 Davis St Scranton PA. Same seller as the two Wolf range lots wf-229/wf-230.</t>
+          <t>2300 Wood Ave, Wilson Borough (Easton area). Final day Oct 30. Retail-floor sale, not a bulk lot; ask in person about buying remaining stock outright.</t>
         </is>
       </c>
     </row>
@@ -22693,17 +22697,17 @@
       </c>
       <c r="B82" s="14" t="inlineStr">
         <is>
-          <t>Limerick Hardware inventory liquidation (Alderfer, online-only)</t>
+          <t>Hearing aid manufacturing facility inventory liquidation (shelving, 3D printers/scanners, laser engravers, Porta-Vac, sound booths, office; bulk offer invited)</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>store closing</t>
+          <t>facility liquidation</t>
         </is>
       </c>
       <c r="D82" s="13" t="inlineStr">
         <is>
-          <t>Limerick</t>
+          <t>Bristol</t>
         </is>
       </c>
       <c r="E82" s="13" t="inlineStr">
@@ -22712,27 +22716,27 @@
         </is>
       </c>
       <c r="F82" s="13" t="n">
-        <v>277</v>
+        <v>252</v>
       </c>
       <c r="G82" s="13" t="inlineStr">
         <is>
-          <t>Online auction, no reserve info</t>
+          <t>Best offer / bulk offer for complete lot</t>
         </is>
       </c>
       <c r="H82" s="15" t="n"/>
       <c r="I82" s="13" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="J82" s="13" t="inlineStr">
         <is>
-          <t>2026-11-02 08:00 PM ET</t>
+          <t>2026-11-08 05:00 PM ET</t>
         </is>
       </c>
       <c r="K82" s="13" t="inlineStr">
         <is>
-          <t>Alderfer Auction</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="L82" s="13" t="inlineStr">
@@ -22748,7 +22752,7 @@
       </c>
       <c r="O82" s="14" t="inlineStr">
         <is>
-          <t>Hardware store inventory: Hillman fasteners/cabinets, DeWalt/Paslode tools, plumbing/electrical (Moen, Watts), Traeger/Weber/Broil King grills, Toro TimeCutter zero-turn, Wesco pallet jack, Lozier shelving, checkouts. Preview by appointment Fri Oct 30 1-3PM. Begins closing Nov 2 8PM EST.</t>
+          <t>Sale Nov 6-8 ONLY, 8 AM-5 PM (updated 2026-10-25; was 'daily'). 806 Beaver St near Rt 13. Industrial shelving and lab equipment, not appliances; bulk offer invited. Email to schedule viewing.</t>
         </is>
       </c>
     </row>
@@ -22760,17 +22764,17 @@
       </c>
       <c r="B83" s="14" t="inlineStr">
         <is>
-          <t>Victorino's Pizzeria + Subway sub shop + brand-new scratch &amp; dent restaurant equipment (Marsal pizza oven, True merchandisers, Vulcan/Migali fryers, Stoelting soft-serve)</t>
+          <t>NBM Liquidation as-is/damaged appliance &amp; more auction (357 lots)</t>
         </is>
       </c>
       <c r="C83" s="13" t="inlineStr">
         <is>
-          <t>restaurant closing</t>
+          <t>auction pallet</t>
         </is>
       </c>
       <c r="D83" s="13" t="inlineStr">
         <is>
-          <t>Manheim</t>
+          <t>Scranton</t>
         </is>
       </c>
       <c r="E83" s="13" t="inlineStr">
@@ -22779,32 +22783,28 @@
         </is>
       </c>
       <c r="F83" s="13" t="n">
-        <v>320</v>
+        <v>255</v>
       </c>
       <c r="G83" s="13" t="inlineStr">
         <is>
-          <t>Online auction, items being added</t>
+          <t>Online auction</t>
         </is>
       </c>
       <c r="H83" s="15" t="n"/>
-      <c r="I83" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
+      <c r="I83" s="13" t="inlineStr"/>
       <c r="J83" s="13" t="inlineStr">
         <is>
-          <t>2026-11-05 08:00 PM ET</t>
+          <t>2026-10-27 06:00 PM ET</t>
         </is>
       </c>
       <c r="K83" s="13" t="inlineStr">
         <is>
-          <t>PCI Auctions East Coast</t>
-        </is>
-      </c>
-      <c r="L83" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>HiBid</t>
+        </is>
+      </c>
+      <c r="L83" s="21" t="inlineStr">
+        <is>
+          <t>ENDING SOON</t>
         </is>
       </c>
       <c r="M83" s="13" t="inlineStr"/>
@@ -22815,768 +22815,902 @@
       </c>
       <c r="O83" s="14" t="inlineStr">
         <is>
+          <t>Recurring reseller auction (not a closing): as-is/damaged whole appliances and more. Pickup 733 Davis St Scranton PA. Same seller as the two Wolf range lots wf-229/wf-230.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" outlineLevel="1">
+      <c r="A84" s="13" t="inlineStr">
+        <is>
+          <t>Eastern PA / Mid-Atlantic</t>
+        </is>
+      </c>
+      <c r="B84" s="14" t="inlineStr">
+        <is>
+          <t>Limerick Hardware inventory liquidation (Alderfer, online-only)</t>
+        </is>
+      </c>
+      <c r="C84" s="13" t="inlineStr">
+        <is>
+          <t>store closing</t>
+        </is>
+      </c>
+      <c r="D84" s="13" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="E84" s="13" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="F84" s="13" t="n">
+        <v>277</v>
+      </c>
+      <c r="G84" s="13" t="inlineStr">
+        <is>
+          <t>Online auction, no reserve info</t>
+        </is>
+      </c>
+      <c r="H84" s="15" t="n"/>
+      <c r="I84" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="J84" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-02 08:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K84" s="13" t="inlineStr">
+        <is>
+          <t>Alderfer Auction</t>
+        </is>
+      </c>
+      <c r="L84" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M84" s="13" t="inlineStr"/>
+      <c r="N84" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O84" s="14" t="inlineStr">
+        <is>
+          <t>Hardware store inventory: Hillman fasteners/cabinets, DeWalt/Paslode tools, plumbing/electrical (Moen, Watts), Traeger/Weber/Broil King grills, Toro TimeCutter zero-turn, Wesco pallet jack, Lozier shelving, checkouts. Preview by appointment Fri Oct 30 1-3PM. Begins closing Nov 2 8PM EST.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" outlineLevel="1">
+      <c r="A85" s="13" t="inlineStr">
+        <is>
+          <t>Eastern PA / Mid-Atlantic</t>
+        </is>
+      </c>
+      <c r="B85" s="14" t="inlineStr">
+        <is>
+          <t>Victorino's Pizzeria + Subway sub shop + brand-new scratch &amp; dent restaurant equipment (Marsal pizza oven, True merchandisers, Vulcan/Migali fryers, Stoelting soft-serve)</t>
+        </is>
+      </c>
+      <c r="C85" s="13" t="inlineStr">
+        <is>
+          <t>restaurant closing</t>
+        </is>
+      </c>
+      <c r="D85" s="13" t="inlineStr">
+        <is>
+          <t>Manheim</t>
+        </is>
+      </c>
+      <c r="E85" s="13" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="F85" s="13" t="n">
+        <v>320</v>
+      </c>
+      <c r="G85" s="13" t="inlineStr">
+        <is>
+          <t>Online auction, items being added</t>
+        </is>
+      </c>
+      <c r="H85" s="15" t="n"/>
+      <c r="I85" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="J85" s="13" t="inlineStr">
+        <is>
+          <t>2026-11-05 08:00 PM ET</t>
+        </is>
+      </c>
+      <c r="K85" s="13" t="inlineStr">
+        <is>
+          <t>PCI Auctions East Coast</t>
+        </is>
+      </c>
+      <c r="L85" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M85" s="13" t="inlineStr"/>
+      <c r="N85" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O85" s="14" t="inlineStr">
+        <is>
           <t>Ends Thu Nov 5 8 PM EST. PCI East Coast warehouse, 141 W End Dr, Manheim PA. Preview Wed Nov 4 10-2; removal Fri Nov 6 10-4. Shipping/delivery available.</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="17" t="inlineStr">
+    <row r="86">
+      <c r="A86" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Eastern PA / Mid-Atlantic</t>
         </is>
       </c>
-      <c r="B84" s="17" t="inlineStr">
+      <c r="B86" s="17" t="inlineStr">
         <is>
           <t>5 item(s)</t>
         </is>
       </c>
-      <c r="C84" s="18" t="n"/>
-      <c r="D84" s="18" t="n"/>
-      <c r="E84" s="18" t="n"/>
-      <c r="F84" s="18" t="n"/>
-      <c r="G84" s="18" t="n"/>
-      <c r="H84" s="19" t="n">
+      <c r="C86" s="18" t="n"/>
+      <c r="D86" s="18" t="n"/>
+      <c r="E86" s="18" t="n"/>
+      <c r="F86" s="18" t="n"/>
+      <c r="G86" s="18" t="n"/>
+      <c r="H86" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I84" s="18" t="n"/>
-      <c r="J84" s="18" t="n"/>
-      <c r="K84" s="18" t="n"/>
-      <c r="L84" s="18" t="n"/>
-      <c r="M84" s="18" t="n"/>
-      <c r="N84" s="18" t="n"/>
-      <c r="O84" s="18" t="n"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="11" t="inlineStr">
+      <c r="I86" s="18" t="n"/>
+      <c r="J86" s="18" t="n"/>
+      <c r="K86" s="18" t="n"/>
+      <c r="L86" s="18" t="n"/>
+      <c r="M86" s="18" t="n"/>
+      <c r="N86" s="18" t="n"/>
+      <c r="O86" s="18" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="11" t="inlineStr">
         <is>
           <t>▸ Upstate / Western NY  (1)</t>
         </is>
       </c>
-      <c r="B85" s="12" t="n"/>
-      <c r="C85" s="12" t="n"/>
-      <c r="D85" s="12" t="n"/>
-      <c r="E85" s="12" t="n"/>
-      <c r="F85" s="12" t="n"/>
-      <c r="G85" s="12" t="n"/>
-      <c r="H85" s="12" t="n"/>
-      <c r="I85" s="12" t="n"/>
-      <c r="J85" s="12" t="n"/>
-      <c r="K85" s="12" t="n"/>
-      <c r="L85" s="12" t="n"/>
-      <c r="M85" s="12" t="n"/>
-      <c r="N85" s="12" t="n"/>
-      <c r="O85" s="12" t="n"/>
-    </row>
-    <row r="86" outlineLevel="1">
-      <c r="A86" s="13" t="inlineStr">
+      <c r="B87" s="12" t="n"/>
+      <c r="C87" s="12" t="n"/>
+      <c r="D87" s="12" t="n"/>
+      <c r="E87" s="12" t="n"/>
+      <c r="F87" s="12" t="n"/>
+      <c r="G87" s="12" t="n"/>
+      <c r="H87" s="12" t="n"/>
+      <c r="I87" s="12" t="n"/>
+      <c r="J87" s="12" t="n"/>
+      <c r="K87" s="12" t="n"/>
+      <c r="L87" s="12" t="n"/>
+      <c r="M87" s="12" t="n"/>
+      <c r="N87" s="12" t="n"/>
+      <c r="O87" s="12" t="n"/>
+    </row>
+    <row r="88" outlineLevel="1">
+      <c r="A88" s="13" t="inlineStr">
         <is>
           <t>Upstate / Western NY</t>
         </is>
       </c>
-      <c r="B86" s="14" t="inlineStr">
+      <c r="B88" s="14" t="inlineStr">
         <is>
           <t>Restaurant &amp; fitness equipment</t>
         </is>
       </c>
-      <c r="C86" s="13" t="inlineStr">
+      <c r="C88" s="13" t="inlineStr">
         <is>
           <t>restaurant</t>
         </is>
       </c>
-      <c r="D86" s="13" t="inlineStr">
+      <c r="D88" s="13" t="inlineStr">
         <is>
           <t>Williamsville</t>
         </is>
       </c>
-      <c r="E86" s="13" t="inlineStr">
+      <c r="E88" s="13" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
       </c>
-      <c r="F86" s="13" t="n">
+      <c r="F88" s="13" t="n">
         <v>408</v>
       </c>
-      <c r="G86" s="13" t="inlineStr">
+      <c r="G88" s="13" t="inlineStr">
         <is>
           <t>Online auction</t>
         </is>
       </c>
-      <c r="H86" s="15" t="n"/>
-      <c r="I86" s="13" t="inlineStr"/>
-      <c r="J86" s="13" t="inlineStr">
+      <c r="H88" s="15" t="n"/>
+      <c r="I88" s="13" t="inlineStr"/>
+      <c r="J88" s="13" t="inlineStr">
         <is>
           <t>2026-10-26 07:30 PM ET</t>
         </is>
       </c>
-      <c r="K86" s="13" t="inlineStr">
+      <c r="K88" s="13" t="inlineStr">
         <is>
           <t>Cash Auctions</t>
         </is>
       </c>
-      <c r="L86" s="21" t="inlineStr">
+      <c r="L88" s="21" t="inlineStr">
         <is>
           <t>ENDING SOON</t>
         </is>
       </c>
-      <c r="M86" s="13" t="inlineStr"/>
-      <c r="N86" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O86" s="14" t="inlineStr">
+      <c r="M88" s="13" t="inlineStr"/>
+      <c r="N88" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O88" s="14" t="inlineStr">
         <is>
           <t>Lots not reviewed.</t>
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="17" t="inlineStr">
+    <row r="89">
+      <c r="A89" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Upstate / Western NY</t>
         </is>
       </c>
-      <c r="B87" s="17" t="inlineStr">
+      <c r="B89" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C87" s="18" t="n"/>
-      <c r="D87" s="18" t="n"/>
-      <c r="E87" s="18" t="n"/>
-      <c r="F87" s="18" t="n"/>
-      <c r="G87" s="18" t="n"/>
-      <c r="H87" s="19" t="n">
+      <c r="C89" s="18" t="n"/>
+      <c r="D89" s="18" t="n"/>
+      <c r="E89" s="18" t="n"/>
+      <c r="F89" s="18" t="n"/>
+      <c r="G89" s="18" t="n"/>
+      <c r="H89" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I87" s="18" t="n"/>
-      <c r="J87" s="18" t="n"/>
-      <c r="K87" s="18" t="n"/>
-      <c r="L87" s="18" t="n"/>
-      <c r="M87" s="18" t="n"/>
-      <c r="N87" s="18" t="n"/>
-      <c r="O87" s="18" t="n"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="11" t="inlineStr">
+      <c r="I89" s="18" t="n"/>
+      <c r="J89" s="18" t="n"/>
+      <c r="K89" s="18" t="n"/>
+      <c r="L89" s="18" t="n"/>
+      <c r="M89" s="18" t="n"/>
+      <c r="N89" s="18" t="n"/>
+      <c r="O89" s="18" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="11" t="inlineStr">
         <is>
           <t>▸ Virginia  (1)</t>
         </is>
       </c>
-      <c r="B88" s="12" t="n"/>
-      <c r="C88" s="12" t="n"/>
-      <c r="D88" s="12" t="n"/>
-      <c r="E88" s="12" t="n"/>
-      <c r="F88" s="12" t="n"/>
-      <c r="G88" s="12" t="n"/>
-      <c r="H88" s="12" t="n"/>
-      <c r="I88" s="12" t="n"/>
-      <c r="J88" s="12" t="n"/>
-      <c r="K88" s="12" t="n"/>
-      <c r="L88" s="12" t="n"/>
-      <c r="M88" s="12" t="n"/>
-      <c r="N88" s="12" t="n"/>
-      <c r="O88" s="12" t="n"/>
-    </row>
-    <row r="89" outlineLevel="1">
-      <c r="A89" s="13" t="inlineStr">
+      <c r="B90" s="12" t="n"/>
+      <c r="C90" s="12" t="n"/>
+      <c r="D90" s="12" t="n"/>
+      <c r="E90" s="12" t="n"/>
+      <c r="F90" s="12" t="n"/>
+      <c r="G90" s="12" t="n"/>
+      <c r="H90" s="12" t="n"/>
+      <c r="I90" s="12" t="n"/>
+      <c r="J90" s="12" t="n"/>
+      <c r="K90" s="12" t="n"/>
+      <c r="L90" s="12" t="n"/>
+      <c r="M90" s="12" t="n"/>
+      <c r="N90" s="12" t="n"/>
+      <c r="O90" s="12" t="n"/>
+    </row>
+    <row r="91" outlineLevel="1">
+      <c r="A91" s="13" t="inlineStr">
         <is>
           <t>Virginia</t>
         </is>
       </c>
-      <c r="B89" s="14" t="inlineStr">
+      <c r="B91" s="14" t="inlineStr">
         <is>
           <t>Haynes Furniture / The Dump – 12 stores closing (furniture, mattresses)</t>
         </is>
       </c>
-      <c r="C89" s="13" t="inlineStr">
+      <c r="C91" s="13" t="inlineStr">
         <is>
           <t>retail GOB</t>
         </is>
       </c>
-      <c r="D89" s="13" t="inlineStr">
+      <c r="D91" s="13" t="inlineStr">
         <is>
           <t>Virginia Beach</t>
         </is>
       </c>
-      <c r="E89" s="13" t="inlineStr">
+      <c r="E91" s="13" t="inlineStr">
         <is>
           <t>VA</t>
         </is>
       </c>
-      <c r="F89" s="13" t="n">
+      <c r="F91" s="13" t="n">
         <v>456</v>
       </c>
-      <c r="G89" s="13" t="inlineStr">
+      <c r="G91" s="13" t="inlineStr">
         <is>
           <t>Retail GOB markdowns</t>
         </is>
       </c>
-      <c r="H89" s="15" t="n"/>
-      <c r="I89" s="13" t="inlineStr">
+      <c r="H91" s="15" t="n"/>
+      <c r="I91" s="13" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>
       </c>
-      <c r="J89" s="13" t="inlineStr"/>
-      <c r="K89" s="13" t="inlineStr">
+      <c r="J91" s="13" t="inlineStr"/>
+      <c r="K91" s="13" t="inlineStr">
         <is>
           <t>SB360 (PR Newswire)</t>
         </is>
       </c>
-      <c r="L89" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M89" s="13" t="inlineStr"/>
-      <c r="N89" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O89" s="14" t="inlineStr">
+      <c r="L91" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M91" s="13" t="inlineStr"/>
+      <c r="N91" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O91" s="14" t="inlineStr">
         <is>
           <t>Posted Oct 8. Multi-state (VA/AZ/GA/IL/TX); pinned at Virginia Beach. Home goods only.</t>
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="17" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Virginia</t>
         </is>
       </c>
-      <c r="B90" s="17" t="inlineStr">
+      <c r="B92" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C90" s="18" t="n"/>
-      <c r="D90" s="18" t="n"/>
-      <c r="E90" s="18" t="n"/>
-      <c r="F90" s="18" t="n"/>
-      <c r="G90" s="18" t="n"/>
-      <c r="H90" s="19" t="n">
+      <c r="C92" s="18" t="n"/>
+      <c r="D92" s="18" t="n"/>
+      <c r="E92" s="18" t="n"/>
+      <c r="F92" s="18" t="n"/>
+      <c r="G92" s="18" t="n"/>
+      <c r="H92" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I90" s="18" t="n"/>
-      <c r="J90" s="18" t="n"/>
-      <c r="K90" s="18" t="n"/>
-      <c r="L90" s="18" t="n"/>
-      <c r="M90" s="18" t="n"/>
-      <c r="N90" s="18" t="n"/>
-      <c r="O90" s="18" t="n"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="11" t="inlineStr">
+      <c r="I92" s="18" t="n"/>
+      <c r="J92" s="18" t="n"/>
+      <c r="K92" s="18" t="n"/>
+      <c r="L92" s="18" t="n"/>
+      <c r="M92" s="18" t="n"/>
+      <c r="N92" s="18" t="n"/>
+      <c r="O92" s="18" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="11" t="inlineStr">
         <is>
           <t>▸ Southeast  (1)</t>
         </is>
       </c>
-      <c r="B91" s="12" t="n"/>
-      <c r="C91" s="12" t="n"/>
-      <c r="D91" s="12" t="n"/>
-      <c r="E91" s="12" t="n"/>
-      <c r="F91" s="12" t="n"/>
-      <c r="G91" s="12" t="n"/>
-      <c r="H91" s="12" t="n"/>
-      <c r="I91" s="12" t="n"/>
-      <c r="J91" s="12" t="n"/>
-      <c r="K91" s="12" t="n"/>
-      <c r="L91" s="12" t="n"/>
-      <c r="M91" s="12" t="n"/>
-      <c r="N91" s="12" t="n"/>
-      <c r="O91" s="12" t="n"/>
-    </row>
-    <row r="92" outlineLevel="1">
-      <c r="A92" s="13" t="inlineStr">
+      <c r="B93" s="12" t="n"/>
+      <c r="C93" s="12" t="n"/>
+      <c r="D93" s="12" t="n"/>
+      <c r="E93" s="12" t="n"/>
+      <c r="F93" s="12" t="n"/>
+      <c r="G93" s="12" t="n"/>
+      <c r="H93" s="12" t="n"/>
+      <c r="I93" s="12" t="n"/>
+      <c r="J93" s="12" t="n"/>
+      <c r="K93" s="12" t="n"/>
+      <c r="L93" s="12" t="n"/>
+      <c r="M93" s="12" t="n"/>
+      <c r="N93" s="12" t="n"/>
+      <c r="O93" s="12" t="n"/>
+    </row>
+    <row r="94" outlineLevel="1">
+      <c r="A94" s="13" t="inlineStr">
         <is>
           <t>Southeast</t>
         </is>
       </c>
-      <c r="B92" s="14" t="inlineStr">
+      <c r="B94" s="14" t="inlineStr">
         <is>
           <t>Carter Control Systems Inc. bankruptcy Day 2: fabrication equipment + $5MM+ inventory (conveyor systems maker)</t>
         </is>
       </c>
-      <c r="C92" s="13" t="inlineStr">
+      <c r="C94" s="13" t="inlineStr">
         <is>
           <t>bankruptcy auction</t>
         </is>
       </c>
-      <c r="D92" s="13" t="inlineStr">
+      <c r="D94" s="13" t="inlineStr">
         <is>
           <t>Savannah</t>
         </is>
       </c>
-      <c r="E92" s="13" t="inlineStr">
+      <c r="E94" s="13" t="inlineStr">
         <is>
           <t>GA</t>
         </is>
       </c>
-      <c r="F92" s="13" t="n">
+      <c r="F94" s="13" t="n">
         <v>894</v>
       </c>
-      <c r="G92" s="13" t="inlineStr">
+      <c r="G94" s="13" t="inlineStr">
         <is>
           <t>Timed online auction</t>
         </is>
       </c>
-      <c r="H92" s="15" t="n"/>
-      <c r="I92" s="13" t="inlineStr"/>
-      <c r="J92" s="13" t="inlineStr">
+      <c r="H94" s="15" t="n"/>
+      <c r="I94" s="13" t="inlineStr"/>
+      <c r="J94" s="13" t="inlineStr">
         <is>
           <t>2026-10-28 10:00 AM ET</t>
         </is>
       </c>
-      <c r="K92" s="13" t="inlineStr">
+      <c r="K94" s="13" t="inlineStr">
         <is>
           <t>PPL Group</t>
         </is>
       </c>
-      <c r="L92" s="21" t="inlineStr">
+      <c r="L94" s="21" t="inlineStr">
         <is>
           <t>ENDING SOON</t>
         </is>
       </c>
-      <c r="M92" s="13" t="inlineStr"/>
-      <c r="N92" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O92" s="14" t="inlineStr">
+      <c r="M94" s="13" t="inlineStr"/>
+      <c r="N94" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O94" s="14" t="inlineStr">
         <is>
           <t>Ends Oct 28 10 AM ET; preview Oct 26-27; removal Oct 29-Nov 13.</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="17" t="inlineStr">
+    <row r="95">
+      <c r="A95" s="17" t="inlineStr">
         <is>
           <t>Subtotal — Southeast</t>
         </is>
       </c>
-      <c r="B93" s="17" t="inlineStr">
+      <c r="B95" s="17" t="inlineStr">
         <is>
           <t>1 item(s)</t>
         </is>
       </c>
-      <c r="C93" s="18" t="n"/>
-      <c r="D93" s="18" t="n"/>
-      <c r="E93" s="18" t="n"/>
-      <c r="F93" s="18" t="n"/>
-      <c r="G93" s="18" t="n"/>
-      <c r="H93" s="19" t="n">
+      <c r="C95" s="18" t="n"/>
+      <c r="D95" s="18" t="n"/>
+      <c r="E95" s="18" t="n"/>
+      <c r="F95" s="18" t="n"/>
+      <c r="G95" s="18" t="n"/>
+      <c r="H95" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I93" s="18" t="n"/>
-      <c r="J93" s="18" t="n"/>
-      <c r="K93" s="18" t="n"/>
-      <c r="L93" s="18" t="n"/>
-      <c r="M93" s="18" t="n"/>
-      <c r="N93" s="18" t="n"/>
-      <c r="O93" s="18" t="n"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="11" t="inlineStr">
+      <c r="I95" s="18" t="n"/>
+      <c r="J95" s="18" t="n"/>
+      <c r="K95" s="18" t="n"/>
+      <c r="L95" s="18" t="n"/>
+      <c r="M95" s="18" t="n"/>
+      <c r="N95" s="18" t="n"/>
+      <c r="O95" s="18" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="11" t="inlineStr">
         <is>
           <t>▸ Midwest  (2)</t>
         </is>
       </c>
-      <c r="B94" s="12" t="n"/>
-      <c r="C94" s="12" t="n"/>
-      <c r="D94" s="12" t="n"/>
-      <c r="E94" s="12" t="n"/>
-      <c r="F94" s="12" t="n"/>
-      <c r="G94" s="12" t="n"/>
-      <c r="H94" s="12" t="n"/>
-      <c r="I94" s="12" t="n"/>
-      <c r="J94" s="12" t="n"/>
-      <c r="K94" s="12" t="n"/>
-      <c r="L94" s="12" t="n"/>
-      <c r="M94" s="12" t="n"/>
-      <c r="N94" s="12" t="n"/>
-      <c r="O94" s="12" t="n"/>
-    </row>
-    <row r="95" outlineLevel="1">
-      <c r="A95" s="13" t="inlineStr">
+      <c r="B96" s="12" t="n"/>
+      <c r="C96" s="12" t="n"/>
+      <c r="D96" s="12" t="n"/>
+      <c r="E96" s="12" t="n"/>
+      <c r="F96" s="12" t="n"/>
+      <c r="G96" s="12" t="n"/>
+      <c r="H96" s="12" t="n"/>
+      <c r="I96" s="12" t="n"/>
+      <c r="J96" s="12" t="n"/>
+      <c r="K96" s="12" t="n"/>
+      <c r="L96" s="12" t="n"/>
+      <c r="M96" s="12" t="n"/>
+      <c r="N96" s="12" t="n"/>
+      <c r="O96" s="12" t="n"/>
+    </row>
+    <row r="97" outlineLevel="1">
+      <c r="A97" s="13" t="inlineStr">
         <is>
           <t>Midwest</t>
         </is>
       </c>
-      <c r="B95" s="14" t="inlineStr">
+      <c r="B97" s="14" t="inlineStr">
         <is>
           <t>Vernon Hardware-Napa inventory liquidation (hardware + NAPA auto parts store closing after 87 yrs): tools, hardware, plumbing, electrical, auto parts</t>
         </is>
       </c>
-      <c r="C95" s="13" t="inlineStr">
+      <c r="C97" s="13" t="inlineStr">
         <is>
           <t>store closing auction</t>
         </is>
       </c>
-      <c r="D95" s="13" t="inlineStr">
+      <c r="D97" s="13" t="inlineStr">
         <is>
           <t>Vernon</t>
         </is>
       </c>
-      <c r="E95" s="13" t="inlineStr">
+      <c r="E97" s="13" t="inlineStr">
         <is>
           <t>MI</t>
         </is>
       </c>
-      <c r="F95" s="13" t="n">
+      <c r="F97" s="13" t="n">
         <v>675</v>
       </c>
-      <c r="G95" s="13" t="inlineStr">
+      <c r="G97" s="13" t="inlineStr">
         <is>
           <t>No-reserve online auction (Xyz Auction Service), BP 10% cash/cert. check, 13% card</t>
         </is>
       </c>
-      <c r="H95" s="15" t="n"/>
-      <c r="I95" s="13" t="inlineStr"/>
-      <c r="J95" s="13" t="inlineStr">
+      <c r="H97" s="15" t="n"/>
+      <c r="I97" s="13" t="inlineStr"/>
+      <c r="J97" s="13" t="inlineStr">
         <is>
           <t>2026-11-05 07:00 PM ET</t>
         </is>
       </c>
-      <c r="K95" s="13" t="inlineStr">
+      <c r="K97" s="13" t="inlineStr">
         <is>
           <t>EstateSales.net</t>
         </is>
       </c>
-      <c r="L95" s="13" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M95" s="13" t="inlineStr"/>
-      <c r="N95" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="O95" s="14" t="inlineStr">
+      <c r="L97" s="13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M97" s="13" t="inlineStr"/>
+      <c r="N97" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="O97" s="14" t="inlineStr">
         <is>
           <t>Bidding opens Mon Nov 2 7 AM; lots begin closing Thu Nov 5 7 PM (bid on auctioneer's site, (989) 288-4600). Far from MA: only worth it for bulk lots that justify the trip. URL verified live 2026-10-25.</t>
         </is>
       </c>
     </row>
-    <row r="96" outlineLevel="1">
-      <c r="A96" s="13" t="inlineStr">
+    <row r="98" outlineLevel="1">
+      <c r="A98" s="13" t="inlineStr">
         <is>
           <t>Midwest</t>
         </is>
       </c>
-      <c r="B96" s="14" t="inlineStr">
+      <c r="B98" s="14" t="inlineStr">
         <is>
           <t>American Sale – total liquidation, all 7 stores (pools, hot tubs, grills, holiday decor)</t>
         </is>
       </c>
-      <c r="C96" s="13" t="inlineStr">
+      <c r="C98" s="13" t="inlineStr">
         <is>
           <t>retail GOB</t>
         </is>
       </c>
-      <c r="D96" s="13" t="inlineStr">
+      <c r="D98" s="13" t="inlineStr">
         <is>
           <t>Chicagoland</t>
         </is>
       </c>
-      <c r="E96" s="13" t="inlineStr">
+      <c r="E98" s="13" t="inlineStr">
         <is>
           <t>IL</t>
         </is>
       </c>
-      <c r="F96" s="13" t="n">
+      <c r="F98" s="13" t="n">
         <v>876</v>
       </c>
-      <c r="G96" s="13" t="inlineS